<commit_message>
Data update — 2026-10-06 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_oct2026.xlsx
+++ b/results/strategy_pnl_oct2026.xlsx
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trade Log'!$A$3:$O$503</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1079,8 +1079,12 @@
       <c r="F4" s="26" t="n">
         <v>1752</v>
       </c>
-      <c r="G4" s="24" t="inlineStr"/>
-      <c r="H4" s="25" t="inlineStr"/>
+      <c r="G4" s="24" t="n">
+        <v>46301</v>
+      </c>
+      <c r="H4" s="25" t="n">
+        <v>85.81999999999999</v>
+      </c>
       <c r="I4" s="21">
         <f>IF(OR($B4="",$H4=""),"",IF($C4="LONG",($H4-$E4)*$F4,($E4-$H4)*$F4))</f>
         <v/>
@@ -1090,7 +1094,7 @@
         <v/>
       </c>
       <c r="K4" s="4" t="n">
-        <v>14.75</v>
+        <v>193.24</v>
       </c>
       <c r="L4" s="21">
         <f>IF(OR($B4="",$I4=""),"",$I4-IF($K4="",0,$K4))</f>
@@ -1113,12 +1117,12 @@
     <row r="5">
       <c r="A5" s="23" t="inlineStr">
         <is>
-          <t>DHAN-34126100566209+321261005656309+34126100566409+321261005657009+23126100565509+23126100565609+34126100566609+34126100566709+221261005674009+321261005658809+221261005675209+23126100566009+321261005659709+34126100567409+221261005676309+34126100567709</t>
+          <t>DHAN-23126100565309+34126100566309+23126100565409+34126100566509+221261005673109+23126100565709+221261005673609+34126100566809+23126100565809+23126100565909+34126100567109+34126100567209+34126100567309</t>
         </is>
       </c>
       <c r="B5" s="23" t="inlineStr">
         <is>
-          <t>DPABHUSHAN</t>
+          <t>SGFIN</t>
         </is>
       </c>
       <c r="C5" s="23" t="inlineStr">
@@ -1130,13 +1134,17 @@
         <v>46300</v>
       </c>
       <c r="E5" s="25" t="n">
-        <v>2108.8394</v>
+        <v>679.0067</v>
       </c>
       <c r="F5" s="26" t="n">
-        <v>71</v>
-      </c>
-      <c r="G5" s="24" t="inlineStr"/>
-      <c r="H5" s="25" t="inlineStr"/>
+        <v>442</v>
+      </c>
+      <c r="G5" s="24" t="n">
+        <v>46301</v>
+      </c>
+      <c r="H5" s="25" t="n">
+        <v>660.0599999999999</v>
+      </c>
       <c r="I5" s="21">
         <f>IF(OR($B5="",$H5=""),"",IF($C5="LONG",($H5-$E5)*$F5,($E5-$H5)*$F5))</f>
         <v/>
@@ -1146,7 +1154,7 @@
         <v/>
       </c>
       <c r="K5" s="4" t="n">
-        <v>14.75</v>
+        <v>574.35</v>
       </c>
       <c r="L5" s="21">
         <f>IF(OR($B5="",$I5=""),"",$I5-IF($K5="",0,$K5))</f>
@@ -1162,19 +1170,19 @@
       </c>
       <c r="O5" s="23" t="inlineStr">
         <is>
-          <t>10-15</t>
+          <t>5-10</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="23" t="inlineStr">
         <is>
-          <t>DHAN-23126100565309+34126100566309+23126100565409+34126100566509+221261005673109+23126100565709+221261005673609+34126100566809+23126100565809+23126100565909+34126100567109+34126100567209+34126100567309</t>
+          <t>DHAN-221261005679509</t>
         </is>
       </c>
       <c r="B6" s="23" t="inlineStr">
         <is>
-          <t>SGFIN</t>
+          <t>SMCGLOBAL</t>
         </is>
       </c>
       <c r="C6" s="23" t="inlineStr">
@@ -1186,13 +1194,17 @@
         <v>46300</v>
       </c>
       <c r="E6" s="25" t="n">
-        <v>679.0067</v>
+        <v>113.9808</v>
       </c>
       <c r="F6" s="26" t="n">
-        <v>442</v>
-      </c>
-      <c r="G6" s="24" t="inlineStr"/>
-      <c r="H6" s="25" t="inlineStr"/>
+        <v>2624</v>
+      </c>
+      <c r="G6" s="24" t="n">
+        <v>46301</v>
+      </c>
+      <c r="H6" s="25" t="n">
+        <v>109.23</v>
+      </c>
       <c r="I6" s="21">
         <f>IF(OR($B6="",$H6=""),"",IF($C6="LONG",($H6-$E6)*$F6,($E6-$H6)*$F6))</f>
         <v/>
@@ -1202,7 +1214,7 @@
         <v/>
       </c>
       <c r="K6" s="4" t="n">
-        <v>50.15</v>
+        <v>479.89</v>
       </c>
       <c r="L6" s="21">
         <f>IF(OR($B6="",$I6=""),"",$I6-IF($K6="",0,$K6))</f>
@@ -1218,19 +1230,19 @@
       </c>
       <c r="O6" s="23" t="inlineStr">
         <is>
-          <t>5-10</t>
+          <t>15-20</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261005679509</t>
+          <t>DHAN-34126100566209+321261005656309+34126100566409+321261005657009+23126100565509+23126100565609+34126100566609+34126100566709+221261005674009+321261005658809+221261005675209+23126100566009+321261005659709+34126100567409+221261005676309+34126100567709</t>
         </is>
       </c>
       <c r="B7" s="23" t="inlineStr">
         <is>
-          <t>SMCGLOBAL</t>
+          <t>DPABHUSHAN</t>
         </is>
       </c>
       <c r="C7" s="23" t="inlineStr">
@@ -1242,10 +1254,10 @@
         <v>46300</v>
       </c>
       <c r="E7" s="25" t="n">
-        <v>113.9808</v>
+        <v>2108.8394</v>
       </c>
       <c r="F7" s="26" t="n">
-        <v>2624</v>
+        <v>71</v>
       </c>
       <c r="G7" s="24" t="inlineStr"/>
       <c r="H7" s="25" t="inlineStr"/>
@@ -1258,7 +1270,7 @@
         <v/>
       </c>
       <c r="K7" s="4" t="n">
-        <v>50.15</v>
+        <v>192.54</v>
       </c>
       <c r="L7" s="21">
         <f>IF(OR($B7="",$I7=""),"",$I7-IF($K7="",0,$K7))</f>
@@ -1274,19 +1286,37 @@
       </c>
       <c r="O7" s="23" t="inlineStr">
         <is>
-          <t>15-20</t>
+          <t>10-15</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="n"/>
-      <c r="B8" s="23" t="n"/>
-      <c r="C8" s="23" t="n"/>
-      <c r="D8" s="24" t="n"/>
-      <c r="E8" s="25" t="n"/>
-      <c r="F8" s="26" t="n"/>
-      <c r="G8" s="24" t="n"/>
-      <c r="H8" s="25" t="n"/>
+      <c r="A8" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261006605709</t>
+        </is>
+      </c>
+      <c r="B8" s="23" t="inlineStr">
+        <is>
+          <t>KRISHNADEF</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D8" s="24" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E8" s="25" t="n">
+        <v>1297.2208</v>
+      </c>
+      <c r="F8" s="26" t="n">
+        <v>231</v>
+      </c>
+      <c r="G8" s="24" t="inlineStr"/>
+      <c r="H8" s="25" t="inlineStr"/>
       <c r="I8" s="21">
         <f>IF(OR($B8="",$H8=""),"",IF($C8="LONG",($H8-$E8)*$F8,($E8-$H8)*$F8))</f>
         <v/>
@@ -1295,7 +1325,9 @@
         <f>IF(OR($B8="",$I8="",$E8=0,$F8=0),"",$I8/($E8*$F8))</f>
         <v/>
       </c>
-      <c r="K8" s="4" t="n"/>
+      <c r="K8" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($K8="",0,$K8))</f>
         <v/>
@@ -1308,17 +1340,39 @@
         <f>IF($B8="","",IF($H8="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O8" s="23" t="n"/>
+      <c r="O8" s="23" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="n"/>
-      <c r="B9" s="23" t="n"/>
-      <c r="C9" s="23" t="n"/>
-      <c r="D9" s="24" t="n"/>
-      <c r="E9" s="25" t="n"/>
-      <c r="F9" s="26" t="n"/>
-      <c r="G9" s="24" t="n"/>
-      <c r="H9" s="25" t="n"/>
+      <c r="A9" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126100671709+23126100663009+23126100663109+321261006600309+321261006600609+321261006600809+23126100663309+221261006573809+221261006574009+23126100663509+23126100663709+23126100663809+34126100672309+221261006576409+221261006576709</t>
+        </is>
+      </c>
+      <c r="B9" s="23" t="inlineStr">
+        <is>
+          <t>SATIN</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D9" s="24" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E9" s="25" t="n">
+        <v>228.9869</v>
+      </c>
+      <c r="F9" s="26" t="n">
+        <v>1307</v>
+      </c>
+      <c r="G9" s="24" t="inlineStr"/>
+      <c r="H9" s="25" t="inlineStr"/>
       <c r="I9" s="21">
         <f>IF(OR($B9="",$H9=""),"",IF($C9="LONG",($H9-$E9)*$F9,($E9-$H9)*$F9))</f>
         <v/>
@@ -1327,7 +1381,9 @@
         <f>IF(OR($B9="",$I9="",$E9=0,$F9=0),"",$I9/($E9*$F9))</f>
         <v/>
       </c>
-      <c r="K9" s="4" t="n"/>
+      <c r="K9" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L9" s="21">
         <f>IF(OR($B9="",$I9=""),"",$I9-IF($K9="",0,$K9))</f>
         <v/>
@@ -1340,17 +1396,39 @@
         <f>IF($B9="","",IF($H9="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O9" s="23" t="n"/>
+      <c r="O9" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="n"/>
-      <c r="B10" s="23" t="n"/>
-      <c r="C10" s="23" t="n"/>
-      <c r="D10" s="24" t="n"/>
-      <c r="E10" s="25" t="n"/>
-      <c r="F10" s="26" t="n"/>
-      <c r="G10" s="24" t="n"/>
-      <c r="H10" s="25" t="n"/>
+      <c r="A10" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261006571909+221261006572109+34126100671809+23126100663209+34126100672009+23126100663409+321261006601809+34126100672209+23126100663909+23126100664109+23126100664209+34126100672409+23126100664309+221261006577209+34126100672509</t>
+        </is>
+      </c>
+      <c r="B10" s="23" t="inlineStr">
+        <is>
+          <t>YUKEN</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D10" s="24" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E10" s="25" t="n">
+        <v>1238.3789</v>
+      </c>
+      <c r="F10" s="26" t="n">
+        <v>242</v>
+      </c>
+      <c r="G10" s="24" t="inlineStr"/>
+      <c r="H10" s="25" t="inlineStr"/>
       <c r="I10" s="21">
         <f>IF(OR($B10="",$H10=""),"",IF($C10="LONG",($H10-$E10)*$F10,($E10-$H10)*$F10))</f>
         <v/>
@@ -1359,7 +1437,9 @@
         <f>IF(OR($B10="",$I10="",$E10=0,$F10=0),"",$I10/($E10*$F10))</f>
         <v/>
       </c>
-      <c r="K10" s="4" t="n"/>
+      <c r="K10" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L10" s="21">
         <f>IF(OR($B10="",$I10=""),"",$I10-IF($K10="",0,$K10))</f>
         <v/>
@@ -1372,7 +1452,11 @@
         <f>IF($B10="","",IF($H10="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O10" s="23" t="n"/>
+      <c r="O10" s="23" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="23" t="n"/>
@@ -29825,7 +29909,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29995,7 +30079,7 @@
     <row r="6">
       <c r="A6" s="27" t="inlineStr">
         <is>
-          <t>SGFIN</t>
+          <t>KRISHNADEF</t>
         </is>
       </c>
       <c r="B6" s="20">
@@ -30038,78 +30122,207 @@
     <row r="7">
       <c r="A7" s="27" t="inlineStr">
         <is>
+          <t>SATIN</t>
+        </is>
+      </c>
+      <c r="B7" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A7)</f>
+        <v/>
+      </c>
+      <c r="C7" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A7,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D7" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A7,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E7" s="22">
+        <f>IFERROR($C7/$B7,"")</f>
+        <v/>
+      </c>
+      <c r="F7" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A7,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G7" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A7,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H7" s="21">
+        <f>IFERROR($G7/$B7,"")</f>
+        <v/>
+      </c>
+      <c r="I7" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A7),"")</f>
+        <v/>
+      </c>
+      <c r="J7" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A7),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="27" t="inlineStr">
+        <is>
+          <t>SGFIN</t>
+        </is>
+      </c>
+      <c r="B8" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A8)</f>
+        <v/>
+      </c>
+      <c r="C8" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A8,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D8" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A8,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E8" s="22">
+        <f>IFERROR($C8/$B8,"")</f>
+        <v/>
+      </c>
+      <c r="F8" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A8,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G8" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A8,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H8" s="21">
+        <f>IFERROR($G8/$B8,"")</f>
+        <v/>
+      </c>
+      <c r="I8" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A8),"")</f>
+        <v/>
+      </c>
+      <c r="J8" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A8),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="27" t="inlineStr">
+        <is>
           <t>SMCGLOBAL</t>
         </is>
       </c>
-      <c r="B7" s="20">
-        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A7)</f>
-        <v/>
-      </c>
-      <c r="C7" s="20">
-        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A7,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
-        <v/>
-      </c>
-      <c r="D7" s="20">
-        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A7,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
-        <v/>
-      </c>
-      <c r="E7" s="22">
-        <f>IFERROR($C7/$B7,"")</f>
-        <v/>
-      </c>
-      <c r="F7" s="21">
-        <f>SUMIF('Trade Log'!$B$4:$B$503,$A7,'Trade Log'!$I$4:$I$503)</f>
-        <v/>
-      </c>
-      <c r="G7" s="21">
-        <f>SUMIF('Trade Log'!$B$4:$B$503,$A7,'Trade Log'!$L$4:$L$503)</f>
-        <v/>
-      </c>
-      <c r="H7" s="21">
-        <f>IFERROR($G7/$B7,"")</f>
-        <v/>
-      </c>
-      <c r="I7" s="21">
-        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A7),"")</f>
-        <v/>
-      </c>
-      <c r="J7" s="21">
-        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A7),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="B9" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A9)</f>
+        <v/>
+      </c>
+      <c r="C9" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A9,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D9" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A9,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E9" s="22">
+        <f>IFERROR($C9/$B9,"")</f>
+        <v/>
+      </c>
+      <c r="F9" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A9,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G9" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A9,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H9" s="21">
+        <f>IFERROR($G9/$B9,"")</f>
+        <v/>
+      </c>
+      <c r="I9" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A9),"")</f>
+        <v/>
+      </c>
+      <c r="J9" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A9),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="27" t="inlineStr">
+        <is>
+          <t>YUKEN</t>
+        </is>
+      </c>
+      <c r="B10" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A10)</f>
+        <v/>
+      </c>
+      <c r="C10" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A10,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D10" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A10,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E10" s="22">
+        <f>IFERROR($C10/$B10,"")</f>
+        <v/>
+      </c>
+      <c r="F10" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A10,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G10" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A10,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H10" s="21">
+        <f>IFERROR($G10/$B10,"")</f>
+        <v/>
+      </c>
+      <c r="I10" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A10),"")</f>
+        <v/>
+      </c>
+      <c r="J10" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A10),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B8" s="30">
-        <f>SUM(B4:B7)</f>
-        <v/>
-      </c>
-      <c r="C8" s="30">
-        <f>SUM(C4:C7)</f>
-        <v/>
-      </c>
-      <c r="D8" s="30">
-        <f>SUM(D4:D7)</f>
-        <v/>
-      </c>
-      <c r="E8" s="31">
-        <f>IFERROR(C8/B8,"")</f>
-        <v/>
-      </c>
-      <c r="F8" s="32">
-        <f>SUM(F4:F7)</f>
-        <v/>
-      </c>
-      <c r="G8" s="32">
-        <f>SUM(G4:G7)</f>
-        <v/>
-      </c>
-      <c r="H8" s="32">
-        <f>IFERROR(G8/B8,"")</f>
+      <c r="B11" s="30">
+        <f>SUM(B4:B10)</f>
+        <v/>
+      </c>
+      <c r="C11" s="30">
+        <f>SUM(C4:C10)</f>
+        <v/>
+      </c>
+      <c r="D11" s="30">
+        <f>SUM(D4:D10)</f>
+        <v/>
+      </c>
+      <c r="E11" s="31">
+        <f>IFERROR(C11/B11,"")</f>
+        <v/>
+      </c>
+      <c r="F11" s="32">
+        <f>SUM(F4:F10)</f>
+        <v/>
+      </c>
+      <c r="G11" s="32">
+        <f>SUM(G4:G10)</f>
+        <v/>
+      </c>
+      <c r="H11" s="32">
+        <f>IFERROR(G11/B11,"")</f>
         <v/>
       </c>
     </row>
@@ -30128,7 +30341,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -30249,24 +30462,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D4" s="24" t="inlineStr"/>
+      <c r="D4" s="24" t="n">
+        <v>46301</v>
+      </c>
       <c r="E4" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>0</v>
+        <v>150.32</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0</v>
+        <v>4.61</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>0</v>
+        <v>22.55</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>0</v>
+        <v>0.86</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>14.75</v>
@@ -30285,12 +30500,12 @@
     <row r="5">
       <c r="A5" s="23" t="inlineStr">
         <is>
-          <t>DHAN-34126100566209+321261005656309+34126100566409+321261005657009+23126100565509+23126100565609+34126100566609+34126100566709+221261005674009+321261005658809+221261005675209+23126100566009+321261005659709+34126100567409+221261005676309+34126100567709</t>
+          <t>DHAN-23126100565309+34126100566309+23126100565409+34126100566509+221261005673109+23126100565709+221261005673609+34126100566809+23126100565809+23126100565909+34126100567109+34126100567209+34126100567309</t>
         </is>
       </c>
       <c r="B5" s="23" t="inlineStr">
         <is>
-          <t>DPABHUSHAN</t>
+          <t>SGFIN</t>
         </is>
       </c>
       <c r="C5" s="23" t="inlineStr">
@@ -30298,33 +30513,35 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D5" s="24" t="inlineStr"/>
+      <c r="D5" s="24" t="n">
+        <v>46301</v>
+      </c>
       <c r="E5" s="4" t="n">
-        <v>0</v>
+        <v>90.04000000000001</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>0</v>
+        <v>300.12</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>0</v>
+        <v>45.02</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>0</v>
+        <v>17.92</v>
       </c>
       <c r="K5" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L5" s="4" t="n">
-        <v>0</v>
+        <v>35.4</v>
       </c>
       <c r="M5" s="4" t="n">
-        <v>0</v>
+        <v>61.58</v>
       </c>
       <c r="N5" s="21">
         <f>SUM(E5:M5)</f>
@@ -30334,12 +30551,12 @@
     <row r="6">
       <c r="A6" s="23" t="inlineStr">
         <is>
-          <t>DHAN-23126100565309+34126100566309+23126100565409+34126100566509+221261005673109+23126100565709+221261005673609+34126100566809+23126100565809+23126100565909+34126100567109+34126100567209+34126100567309</t>
+          <t>DHAN-221261005679509</t>
         </is>
       </c>
       <c r="B6" s="23" t="inlineStr">
         <is>
-          <t>SGFIN</t>
+          <t>SMCGLOBAL</t>
         </is>
       </c>
       <c r="C6" s="23" t="inlineStr">
@@ -30347,24 +30564,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D6" s="24" t="inlineStr"/>
+      <c r="D6" s="24" t="n">
+        <v>46301</v>
+      </c>
       <c r="E6" s="4" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>0</v>
+        <v>298.83</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0</v>
+        <v>9.19</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>0</v>
+        <v>44.97</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>0</v>
+        <v>5.31</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>14.75</v>
@@ -30373,7 +30592,7 @@
         <v>35.4</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>0</v>
+        <v>51.14</v>
       </c>
       <c r="N6" s="21">
         <f>SUM(E6:M6)</f>
@@ -30383,12 +30602,12 @@
     <row r="7">
       <c r="A7" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261005679509</t>
+          <t>DHAN-34126100566209+321261005656309+34126100566409+321261005657009+23126100565509+23126100565609+34126100566609+34126100566709+221261005674009+321261005658809+221261005675209+23126100566009+321261005659709+34126100567409+221261005676309+34126100567709</t>
         </is>
       </c>
       <c r="B7" s="23" t="inlineStr">
         <is>
-          <t>SMCGLOBAL</t>
+          <t>DPABHUSHAN</t>
         </is>
       </c>
       <c r="C7" s="23" t="inlineStr">
@@ -30401,25 +30620,25 @@
         <v>0</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>0</v>
+        <v>149.73</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>0</v>
+        <v>4.6</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>0</v>
+        <v>22.46</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>0</v>
+        <v>0.85</v>
       </c>
       <c r="K7" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L7" s="4" t="n">
-        <v>35.4</v>
+        <v>0</v>
       </c>
       <c r="M7" s="4" t="n">
         <v>0</v>
@@ -30430,54 +30649,201 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261006605709</t>
+        </is>
+      </c>
+      <c r="B8" s="23" t="inlineStr">
+        <is>
+          <t>KRISHNADEF</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D8" s="24" t="inlineStr"/>
+      <c r="E8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="21">
+        <f>SUM(E8:M8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126100671709+23126100663009+23126100663109+321261006600309+321261006600609+321261006600809+23126100663309+221261006573809+221261006574009+23126100663509+23126100663709+23126100663809+34126100672309+221261006576409+221261006576709</t>
+        </is>
+      </c>
+      <c r="B9" s="23" t="inlineStr">
+        <is>
+          <t>SATIN</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D9" s="24" t="inlineStr"/>
+      <c r="E9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L9" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="21">
+        <f>SUM(E9:M9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261006571909+221261006572109+34126100671809+23126100663209+34126100672009+23126100663409+321261006601809+34126100672209+23126100663909+23126100664109+23126100664209+34126100672409+23126100664309+221261006577209+34126100672509</t>
+        </is>
+      </c>
+      <c r="B10" s="23" t="inlineStr">
+        <is>
+          <t>YUKEN</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D10" s="24" t="inlineStr"/>
+      <c r="E10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="21">
+        <f>SUM(E10:M10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E8" s="32">
-        <f>SUM(E4:E7)</f>
-        <v/>
-      </c>
-      <c r="F8" s="32">
-        <f>SUM(F4:F7)</f>
-        <v/>
-      </c>
-      <c r="G8" s="32">
-        <f>SUM(G4:G7)</f>
-        <v/>
-      </c>
-      <c r="H8" s="32">
-        <f>SUM(H4:H7)</f>
-        <v/>
-      </c>
-      <c r="I8" s="32">
-        <f>SUM(I4:I7)</f>
-        <v/>
-      </c>
-      <c r="J8" s="32">
-        <f>SUM(J4:J7)</f>
-        <v/>
-      </c>
-      <c r="K8" s="32">
-        <f>SUM(K4:K7)</f>
-        <v/>
-      </c>
-      <c r="L8" s="32">
-        <f>SUM(L4:L7)</f>
-        <v/>
-      </c>
-      <c r="M8" s="32">
-        <f>SUM(M4:M7)</f>
-        <v/>
-      </c>
-      <c r="N8" s="32">
-        <f>SUM(N4:N7)</f>
+      <c r="E11" s="32">
+        <f>SUM(E4:E10)</f>
+        <v/>
+      </c>
+      <c r="F11" s="32">
+        <f>SUM(F4:F10)</f>
+        <v/>
+      </c>
+      <c r="G11" s="32">
+        <f>SUM(G4:G10)</f>
+        <v/>
+      </c>
+      <c r="H11" s="32">
+        <f>SUM(H4:H10)</f>
+        <v/>
+      </c>
+      <c r="I11" s="32">
+        <f>SUM(I4:I10)</f>
+        <v/>
+      </c>
+      <c r="J11" s="32">
+        <f>SUM(J4:J10)</f>
+        <v/>
+      </c>
+      <c r="K11" s="32">
+        <f>SUM(K4:K10)</f>
+        <v/>
+      </c>
+      <c r="L11" s="32">
+        <f>SUM(L4:L10)</f>
+        <v/>
+      </c>
+      <c r="M11" s="32">
+        <f>SUM(M4:M10)</f>
+        <v/>
+      </c>
+      <c r="N11" s="32">
+        <f>SUM(N4:N10)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:N7"/>
+  <autoFilter ref="A3:N10"/>
   <mergeCells count="2">
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>
@@ -30492,7 +30858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -30586,68 +30952,238 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="27" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B5" s="20">
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,1),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
+      <c r="C5" s="20">
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,1),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,11,1),'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D5" s="20">
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,1),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,11,1),'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E5" s="22">
+        <f>IFERROR($C5/$B5,"")</f>
+        <v/>
+      </c>
+      <c r="F5" s="21">
+        <f>SUMIFS('Trade Log'!$I$4:$I$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,1),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
+      <c r="G5" s="21">
+        <f>SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,1),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
+      <c r="H5" s="21">
+        <f>IFERROR($G5/$B5,"")</f>
+        <v/>
+      </c>
+      <c r="I5" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,1),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,11,1)),"")</f>
+        <v/>
+      </c>
+      <c r="J5" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,1),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,11,1)),"")</f>
+        <v/>
+      </c>
+      <c r="K5" s="29">
+        <f>IFERROR(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,1),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,11,1),'Trade Log'!$L$4:$L$503,"&gt;0")/ABS(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,1),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,11,1),'Trade Log'!$L$4:$L$503,"&lt;0")),"")</f>
+        <v/>
+      </c>
+    </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B6" s="30">
+        <f>SUM(B5:B5)</f>
+        <v/>
+      </c>
+      <c r="C6" s="30">
+        <f>SUM(C5:C5)</f>
+        <v/>
+      </c>
+      <c r="D6" s="30">
+        <f>SUM(D5:D5)</f>
+        <v/>
+      </c>
+      <c r="E6" s="31">
+        <f>IFERROR(C6/B6,"")</f>
+        <v/>
+      </c>
+      <c r="F6" s="32">
+        <f>SUM(F5:F5)</f>
+        <v/>
+      </c>
+      <c r="G6" s="32">
+        <f>SUM(G5:G5)</f>
+        <v/>
+      </c>
+      <c r="H6" s="32">
+        <f>IFERROR(G6/B6,"")</f>
+        <v/>
+      </c>
+      <c r="K6" s="33">
+        <f>IFERROR(SUMIF('Trade Log'!$L$4:$L$503,"&gt;0")/ABS(SUMIF('Trade Log'!$L$4:$L$503,"&lt;0")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
           <t>WEEKLY PnL</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="19" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>Period</t>
         </is>
       </c>
-      <c r="B7" s="19" t="inlineStr">
+      <c r="B9" s="19" t="inlineStr">
         <is>
           <t>Trades</t>
         </is>
       </c>
-      <c r="C7" s="19" t="inlineStr">
+      <c r="C9" s="19" t="inlineStr">
         <is>
           <t>Wins</t>
         </is>
       </c>
-      <c r="D7" s="19" t="inlineStr">
+      <c r="D9" s="19" t="inlineStr">
         <is>
           <t>Losses</t>
         </is>
       </c>
-      <c r="E7" s="19" t="inlineStr">
+      <c r="E9" s="19" t="inlineStr">
         <is>
           <t>Win Rate</t>
         </is>
       </c>
-      <c r="F7" s="19" t="inlineStr">
+      <c r="F9" s="19" t="inlineStr">
         <is>
           <t>Gross P&amp;L</t>
         </is>
       </c>
-      <c r="G7" s="19" t="inlineStr">
+      <c r="G9" s="19" t="inlineStr">
         <is>
           <t>Net P&amp;L</t>
         </is>
       </c>
-      <c r="H7" s="19" t="inlineStr">
+      <c r="H9" s="19" t="inlineStr">
         <is>
           <t>Avg Net P&amp;L / Trade</t>
         </is>
       </c>
-      <c r="I7" s="19" t="inlineStr">
+      <c r="I9" s="19" t="inlineStr">
         <is>
           <t>Best Trade</t>
         </is>
       </c>
-      <c r="J7" s="19" t="inlineStr">
+      <c r="J9" s="19" t="inlineStr">
         <is>
           <t>Worst Trade</t>
         </is>
       </c>
-      <c r="K7" s="19" t="inlineStr">
+      <c r="K9" s="19" t="inlineStr">
         <is>
           <t>Profit Factor</t>
         </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="28" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B10" s="20">
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,5),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,12))</f>
+        <v/>
+      </c>
+      <c r="C10" s="20">
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,5),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,12),'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D10" s="20">
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,5),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,12),'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E10" s="22">
+        <f>IFERROR($C10/$B10,"")</f>
+        <v/>
+      </c>
+      <c r="F10" s="21">
+        <f>SUMIFS('Trade Log'!$I$4:$I$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,5),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,12))</f>
+        <v/>
+      </c>
+      <c r="G10" s="21">
+        <f>SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,5),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,12))</f>
+        <v/>
+      </c>
+      <c r="H10" s="21">
+        <f>IFERROR($G10/$B10,"")</f>
+        <v/>
+      </c>
+      <c r="I10" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,5),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,12)),"")</f>
+        <v/>
+      </c>
+      <c r="J10" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,5),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,12)),"")</f>
+        <v/>
+      </c>
+      <c r="K10" s="29">
+        <f>IFERROR(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,5),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,12),'Trade Log'!$L$4:$L$503,"&gt;0")/ABS(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,5),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,12),'Trade Log'!$L$4:$L$503,"&lt;0")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B11" s="30">
+        <f>SUM(B10:B10)</f>
+        <v/>
+      </c>
+      <c r="C11" s="30">
+        <f>SUM(C10:C10)</f>
+        <v/>
+      </c>
+      <c r="D11" s="30">
+        <f>SUM(D10:D10)</f>
+        <v/>
+      </c>
+      <c r="E11" s="31">
+        <f>IFERROR(C11/B11,"")</f>
+        <v/>
+      </c>
+      <c r="F11" s="32">
+        <f>SUM(F10:F10)</f>
+        <v/>
+      </c>
+      <c r="G11" s="32">
+        <f>SUM(G10:G10)</f>
+        <v/>
+      </c>
+      <c r="H11" s="32">
+        <f>IFERROR(G11/B11,"")</f>
+        <v/>
+      </c>
+      <c r="K11" s="33">
+        <f>IFERROR(SUMIF('Trade Log'!$L$4:$L$503,"&gt;0")/ABS(SUMIF('Trade Log'!$L$4:$L$503,"&lt;0")),"")</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Data update — 2026-10-07 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_oct2026.xlsx
+++ b/results/strategy_pnl_oct2026.xlsx
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trade Log'!$A$3:$O$503</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1094,7 +1094,7 @@
         <v/>
       </c>
       <c r="K4" s="4" t="n">
-        <v>193.24</v>
+        <v>349.23</v>
       </c>
       <c r="L4" s="21">
         <f>IF(OR($B4="",$I4=""),"",$I4-IF($K4="",0,$K4))</f>
@@ -1154,7 +1154,7 @@
         <v/>
       </c>
       <c r="K5" s="4" t="n">
-        <v>574.35</v>
+        <v>900.61</v>
       </c>
       <c r="L5" s="21">
         <f>IF(OR($B5="",$I5=""),"",$I5-IF($K5="",0,$K5))</f>
@@ -1214,7 +1214,7 @@
         <v/>
       </c>
       <c r="K6" s="4" t="n">
-        <v>479.89</v>
+        <v>800.83</v>
       </c>
       <c r="L6" s="21">
         <f>IF(OR($B6="",$I6=""),"",$I6-IF($K6="",0,$K6))</f>
@@ -1237,12 +1237,12 @@
     <row r="7">
       <c r="A7" s="23" t="inlineStr">
         <is>
-          <t>DHAN-34126100566209+321261005656309+34126100566409+321261005657009+23126100565509+23126100565609+34126100566609+34126100566709+221261005674009+321261005658809+221261005675209+23126100566009+321261005659709+34126100567409+221261005676309+34126100567709</t>
+          <t>DHAN-321261006605709</t>
         </is>
       </c>
       <c r="B7" s="23" t="inlineStr">
         <is>
-          <t>DPABHUSHAN</t>
+          <t>KRISHNADEF</t>
         </is>
       </c>
       <c r="C7" s="23" t="inlineStr">
@@ -1251,16 +1251,20 @@
         </is>
       </c>
       <c r="D7" s="24" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="E7" s="25" t="n">
-        <v>2108.8394</v>
+        <v>1297.2208</v>
       </c>
       <c r="F7" s="26" t="n">
-        <v>71</v>
-      </c>
-      <c r="G7" s="24" t="inlineStr"/>
-      <c r="H7" s="25" t="inlineStr"/>
+        <v>231</v>
+      </c>
+      <c r="G7" s="24" t="n">
+        <v>46302</v>
+      </c>
+      <c r="H7" s="25" t="n">
+        <v>1280.57</v>
+      </c>
       <c r="I7" s="21">
         <f>IF(OR($B7="",$H7=""),"",IF($C7="LONG",($H7-$E7)*$F7,($E7-$H7)*$F7))</f>
         <v/>
@@ -1270,7 +1274,7 @@
         <v/>
       </c>
       <c r="K7" s="4" t="n">
-        <v>192.54</v>
+        <v>481.53</v>
       </c>
       <c r="L7" s="21">
         <f>IF(OR($B7="",$I7=""),"",$I7-IF($K7="",0,$K7))</f>
@@ -1293,12 +1297,12 @@
     <row r="8">
       <c r="A8" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261006605709</t>
+          <t>DHAN-34126100671709+23126100663009+23126100663109+321261006600309+321261006600609+321261006600809+23126100663309+221261006573809+221261006574009+23126100663509+23126100663709+23126100663809+34126100672309+221261006576409+221261006576709</t>
         </is>
       </c>
       <c r="B8" s="23" t="inlineStr">
         <is>
-          <t>KRISHNADEF</t>
+          <t>SATIN</t>
         </is>
       </c>
       <c r="C8" s="23" t="inlineStr">
@@ -1310,13 +1314,17 @@
         <v>46301</v>
       </c>
       <c r="E8" s="25" t="n">
-        <v>1297.2208</v>
+        <v>228.9869</v>
       </c>
       <c r="F8" s="26" t="n">
-        <v>231</v>
-      </c>
-      <c r="G8" s="24" t="inlineStr"/>
-      <c r="H8" s="25" t="inlineStr"/>
+        <v>1307</v>
+      </c>
+      <c r="G8" s="24" t="n">
+        <v>46302</v>
+      </c>
+      <c r="H8" s="25" t="n">
+        <v>235.36</v>
+      </c>
       <c r="I8" s="21">
         <f>IF(OR($B8="",$H8=""),"",IF($C8="LONG",($H8-$E8)*$F8,($E8-$H8)*$F8))</f>
         <v/>
@@ -1326,7 +1334,7 @@
         <v/>
       </c>
       <c r="K8" s="4" t="n">
-        <v>50.15</v>
+        <v>572.87</v>
       </c>
       <c r="L8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($K8="",0,$K8))</f>
@@ -1342,19 +1350,19 @@
       </c>
       <c r="O8" s="23" t="inlineStr">
         <is>
-          <t>10-15</t>
+          <t>5-10</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="23" t="inlineStr">
         <is>
-          <t>DHAN-34126100671709+23126100663009+23126100663109+321261006600309+321261006600609+321261006600809+23126100663309+221261006573809+221261006574009+23126100663509+23126100663709+23126100663809+34126100672309+221261006576409+221261006576709</t>
+          <t>DHAN-34126100786209</t>
         </is>
       </c>
       <c r="B9" s="23" t="inlineStr">
         <is>
-          <t>SATIN</t>
+          <t>ARFIN</t>
         </is>
       </c>
       <c r="C9" s="23" t="inlineStr">
@@ -1363,13 +1371,13 @@
         </is>
       </c>
       <c r="D9" s="24" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E9" s="25" t="n">
-        <v>228.9869</v>
+        <v>103.743</v>
       </c>
       <c r="F9" s="26" t="n">
-        <v>1307</v>
+        <v>2316</v>
       </c>
       <c r="G9" s="24" t="inlineStr"/>
       <c r="H9" s="25" t="inlineStr"/>
@@ -1405,12 +1413,12 @@
     <row r="10">
       <c r="A10" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261006571909+221261006572109+34126100671809+23126100663209+34126100672009+23126100663409+321261006601809+34126100672209+23126100663909+23126100664109+23126100664209+34126100672409+23126100664309+221261006577209+34126100672509</t>
+          <t>DHAN-34126100566209+321261005656309+34126100566409+321261005657009+23126100565509+23126100565609+34126100566609+34126100566709+221261005674009+321261005658809+221261005675209+23126100566009+321261005659709+34126100567409+221261005676309+34126100567709</t>
         </is>
       </c>
       <c r="B10" s="23" t="inlineStr">
         <is>
-          <t>YUKEN</t>
+          <t>DPABHUSHAN</t>
         </is>
       </c>
       <c r="C10" s="23" t="inlineStr">
@@ -1419,13 +1427,13 @@
         </is>
       </c>
       <c r="D10" s="24" t="n">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="E10" s="25" t="n">
-        <v>1238.3789</v>
+        <v>2108.8394</v>
       </c>
       <c r="F10" s="26" t="n">
-        <v>242</v>
+        <v>71</v>
       </c>
       <c r="G10" s="24" t="inlineStr"/>
       <c r="H10" s="25" t="inlineStr"/>
@@ -1438,7 +1446,7 @@
         <v/>
       </c>
       <c r="K10" s="4" t="n">
-        <v>50.15</v>
+        <v>192.54</v>
       </c>
       <c r="L10" s="21">
         <f>IF(OR($B10="",$I10=""),"",$I10-IF($K10="",0,$K10))</f>
@@ -1459,14 +1467,32 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="n"/>
-      <c r="B11" s="23" t="n"/>
-      <c r="C11" s="23" t="n"/>
-      <c r="D11" s="24" t="n"/>
-      <c r="E11" s="25" t="n"/>
-      <c r="F11" s="26" t="n"/>
-      <c r="G11" s="24" t="n"/>
-      <c r="H11" s="25" t="n"/>
+      <c r="A11" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261007626809+321261007628809+34126100785209+34126100785309+23126100782509+34126100785409+221261007628809+321261007630509+34126100785509+23126100782909+34126100785609+34126100785709+23126100783209+221261007631209+34126100785809+321261007631609+321261007632109</t>
+        </is>
+      </c>
+      <c r="B11" s="23" t="inlineStr">
+        <is>
+          <t>GPTINFRA</t>
+        </is>
+      </c>
+      <c r="C11" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D11" s="24" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E11" s="25" t="n">
+        <v>129.8444</v>
+      </c>
+      <c r="F11" s="26" t="n">
+        <v>1848</v>
+      </c>
+      <c r="G11" s="24" t="inlineStr"/>
+      <c r="H11" s="25" t="inlineStr"/>
       <c r="I11" s="21">
         <f>IF(OR($B11="",$H11=""),"",IF($C11="LONG",($H11-$E11)*$F11,($E11-$H11)*$F11))</f>
         <v/>
@@ -1475,7 +1501,9 @@
         <f>IF(OR($B11="",$I11="",$E11=0,$F11=0),"",$I11/($E11*$F11))</f>
         <v/>
       </c>
-      <c r="K11" s="4" t="n"/>
+      <c r="K11" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L11" s="21">
         <f>IF(OR($B11="",$I11=""),"",$I11-IF($K11="",0,$K11))</f>
         <v/>
@@ -1488,17 +1516,39 @@
         <f>IF($B11="","",IF($H11="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O11" s="23" t="n"/>
+      <c r="O11" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="n"/>
-      <c r="B12" s="23" t="n"/>
-      <c r="C12" s="23" t="n"/>
-      <c r="D12" s="24" t="n"/>
-      <c r="E12" s="25" t="n"/>
-      <c r="F12" s="26" t="n"/>
-      <c r="G12" s="24" t="n"/>
-      <c r="H12" s="25" t="n"/>
+      <c r="A12" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261007633409</t>
+        </is>
+      </c>
+      <c r="B12" s="23" t="inlineStr">
+        <is>
+          <t>MOBIKWIK</t>
+        </is>
+      </c>
+      <c r="C12" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D12" s="24" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E12" s="25" t="n">
+        <v>257.0405</v>
+      </c>
+      <c r="F12" s="26" t="n">
+        <v>936</v>
+      </c>
+      <c r="G12" s="24" t="inlineStr"/>
+      <c r="H12" s="25" t="inlineStr"/>
       <c r="I12" s="21">
         <f>IF(OR($B12="",$H12=""),"",IF($C12="LONG",($H12-$E12)*$F12,($E12-$H12)*$F12))</f>
         <v/>
@@ -1507,7 +1557,9 @@
         <f>IF(OR($B12="",$I12="",$E12=0,$F12=0),"",$I12/($E12*$F12))</f>
         <v/>
       </c>
-      <c r="K12" s="4" t="n"/>
+      <c r="K12" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L12" s="21">
         <f>IF(OR($B12="",$I12=""),"",$I12-IF($K12="",0,$K12))</f>
         <v/>
@@ -1520,17 +1572,39 @@
         <f>IF($B12="","",IF($H12="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O12" s="23" t="n"/>
+      <c r="O12" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="n"/>
-      <c r="B13" s="23" t="n"/>
-      <c r="C13" s="23" t="n"/>
-      <c r="D13" s="24" t="n"/>
-      <c r="E13" s="25" t="n"/>
-      <c r="F13" s="26" t="n"/>
-      <c r="G13" s="24" t="n"/>
-      <c r="H13" s="25" t="n"/>
+      <c r="A13" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126100785009+34126100785109+221261007627809+221261007628109+321261007629509+23126100782809+321261007629709+221261007629309+221261007629609+221261007629909+23126100783009</t>
+        </is>
+      </c>
+      <c r="B13" s="23" t="inlineStr">
+        <is>
+          <t>PNGSREVA</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D13" s="24" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E13" s="25" t="n">
+        <v>622.1242</v>
+      </c>
+      <c r="F13" s="26" t="n">
+        <v>385</v>
+      </c>
+      <c r="G13" s="24" t="inlineStr"/>
+      <c r="H13" s="25" t="inlineStr"/>
       <c r="I13" s="21">
         <f>IF(OR($B13="",$H13=""),"",IF($C13="LONG",($H13-$E13)*$F13,($E13-$H13)*$F13))</f>
         <v/>
@@ -1539,7 +1613,9 @@
         <f>IF(OR($B13="",$I13="",$E13=0,$F13=0),"",$I13/($E13*$F13))</f>
         <v/>
       </c>
-      <c r="K13" s="4" t="n"/>
+      <c r="K13" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($K13="",0,$K13))</f>
         <v/>
@@ -1552,17 +1628,39 @@
         <f>IF($B13="","",IF($H13="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O13" s="23" t="n"/>
+      <c r="O13" s="23" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="23" t="n"/>
-      <c r="B14" s="23" t="n"/>
-      <c r="C14" s="23" t="n"/>
-      <c r="D14" s="24" t="n"/>
-      <c r="E14" s="25" t="n"/>
-      <c r="F14" s="26" t="n"/>
-      <c r="G14" s="24" t="n"/>
-      <c r="H14" s="25" t="n"/>
+      <c r="A14" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261006571909+221261006572109+34126100671809+23126100663209+34126100672009+23126100663409+321261006601809+34126100672209+23126100663909+23126100664109+23126100664209+34126100672409+23126100664309+221261006577209+34126100672509</t>
+        </is>
+      </c>
+      <c r="B14" s="23" t="inlineStr">
+        <is>
+          <t>YUKEN</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D14" s="24" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E14" s="25" t="n">
+        <v>1238.3789</v>
+      </c>
+      <c r="F14" s="26" t="n">
+        <v>242</v>
+      </c>
+      <c r="G14" s="24" t="inlineStr"/>
+      <c r="H14" s="25" t="inlineStr"/>
       <c r="I14" s="21">
         <f>IF(OR($B14="",$H14=""),"",IF($C14="LONG",($H14-$E14)*$F14,($E14-$H14)*$F14))</f>
         <v/>
@@ -1571,7 +1669,9 @@
         <f>IF(OR($B14="",$I14="",$E14=0,$F14=0),"",$I14/($E14*$F14))</f>
         <v/>
       </c>
-      <c r="K14" s="4" t="n"/>
+      <c r="K14" s="4" t="n">
+        <v>563.34</v>
+      </c>
       <c r="L14" s="21">
         <f>IF(OR($B14="",$I14=""),"",$I14-IF($K14="",0,$K14))</f>
         <v/>
@@ -1584,7 +1684,11 @@
         <f>IF($B14="","",IF($H14="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O14" s="23" t="n"/>
+      <c r="O14" s="23" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="23" t="n"/>
@@ -29909,7 +30013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29993,7 +30097,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>DELTACORP</t>
+          <t>ARFIN</t>
         </is>
       </c>
       <c r="B4" s="20">
@@ -30036,7 +30140,7 @@
     <row r="5">
       <c r="A5" s="27" t="inlineStr">
         <is>
-          <t>DPABHUSHAN</t>
+          <t>DELTACORP</t>
         </is>
       </c>
       <c r="B5" s="20">
@@ -30079,7 +30183,7 @@
     <row r="6">
       <c r="A6" s="27" t="inlineStr">
         <is>
-          <t>KRISHNADEF</t>
+          <t>DPABHUSHAN</t>
         </is>
       </c>
       <c r="B6" s="20">
@@ -30122,7 +30226,7 @@
     <row r="7">
       <c r="A7" s="27" t="inlineStr">
         <is>
-          <t>SATIN</t>
+          <t>GPTINFRA</t>
         </is>
       </c>
       <c r="B7" s="20">
@@ -30165,7 +30269,7 @@
     <row r="8">
       <c r="A8" s="27" t="inlineStr">
         <is>
-          <t>SGFIN</t>
+          <t>KRISHNADEF</t>
         </is>
       </c>
       <c r="B8" s="20">
@@ -30208,7 +30312,7 @@
     <row r="9">
       <c r="A9" s="27" t="inlineStr">
         <is>
-          <t>SMCGLOBAL</t>
+          <t>MOBIKWIK</t>
         </is>
       </c>
       <c r="B9" s="20">
@@ -30251,78 +30355,250 @@
     <row r="10">
       <c r="A10" s="27" t="inlineStr">
         <is>
+          <t>PNGSREVA</t>
+        </is>
+      </c>
+      <c r="B10" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A10)</f>
+        <v/>
+      </c>
+      <c r="C10" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A10,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D10" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A10,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E10" s="22">
+        <f>IFERROR($C10/$B10,"")</f>
+        <v/>
+      </c>
+      <c r="F10" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A10,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G10" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A10,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H10" s="21">
+        <f>IFERROR($G10/$B10,"")</f>
+        <v/>
+      </c>
+      <c r="I10" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A10),"")</f>
+        <v/>
+      </c>
+      <c r="J10" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A10),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="27" t="inlineStr">
+        <is>
+          <t>SATIN</t>
+        </is>
+      </c>
+      <c r="B11" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A11)</f>
+        <v/>
+      </c>
+      <c r="C11" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A11,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D11" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A11,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E11" s="22">
+        <f>IFERROR($C11/$B11,"")</f>
+        <v/>
+      </c>
+      <c r="F11" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A11,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G11" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A11,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H11" s="21">
+        <f>IFERROR($G11/$B11,"")</f>
+        <v/>
+      </c>
+      <c r="I11" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A11),"")</f>
+        <v/>
+      </c>
+      <c r="J11" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A11),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="27" t="inlineStr">
+        <is>
+          <t>SGFIN</t>
+        </is>
+      </c>
+      <c r="B12" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A12)</f>
+        <v/>
+      </c>
+      <c r="C12" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A12,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D12" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A12,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E12" s="22">
+        <f>IFERROR($C12/$B12,"")</f>
+        <v/>
+      </c>
+      <c r="F12" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A12,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G12" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A12,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H12" s="21">
+        <f>IFERROR($G12/$B12,"")</f>
+        <v/>
+      </c>
+      <c r="I12" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A12),"")</f>
+        <v/>
+      </c>
+      <c r="J12" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A12),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="27" t="inlineStr">
+        <is>
+          <t>SMCGLOBAL</t>
+        </is>
+      </c>
+      <c r="B13" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A13)</f>
+        <v/>
+      </c>
+      <c r="C13" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A13,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D13" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A13,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E13" s="22">
+        <f>IFERROR($C13/$B13,"")</f>
+        <v/>
+      </c>
+      <c r="F13" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A13,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G13" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A13,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H13" s="21">
+        <f>IFERROR($G13/$B13,"")</f>
+        <v/>
+      </c>
+      <c r="I13" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A13),"")</f>
+        <v/>
+      </c>
+      <c r="J13" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A13),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="27" t="inlineStr">
+        <is>
           <t>YUKEN</t>
         </is>
       </c>
-      <c r="B10" s="20">
-        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A10)</f>
-        <v/>
-      </c>
-      <c r="C10" s="20">
-        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A10,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
-        <v/>
-      </c>
-      <c r="D10" s="20">
-        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A10,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
-        <v/>
-      </c>
-      <c r="E10" s="22">
-        <f>IFERROR($C10/$B10,"")</f>
-        <v/>
-      </c>
-      <c r="F10" s="21">
-        <f>SUMIF('Trade Log'!$B$4:$B$503,$A10,'Trade Log'!$I$4:$I$503)</f>
-        <v/>
-      </c>
-      <c r="G10" s="21">
-        <f>SUMIF('Trade Log'!$B$4:$B$503,$A10,'Trade Log'!$L$4:$L$503)</f>
-        <v/>
-      </c>
-      <c r="H10" s="21">
-        <f>IFERROR($G10/$B10,"")</f>
-        <v/>
-      </c>
-      <c r="I10" s="21">
-        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A10),"")</f>
-        <v/>
-      </c>
-      <c r="J10" s="21">
-        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A10),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="B14" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A14)</f>
+        <v/>
+      </c>
+      <c r="C14" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A14,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D14" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A14,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E14" s="22">
+        <f>IFERROR($C14/$B14,"")</f>
+        <v/>
+      </c>
+      <c r="F14" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A14,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G14" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A14,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H14" s="21">
+        <f>IFERROR($G14/$B14,"")</f>
+        <v/>
+      </c>
+      <c r="I14" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A14),"")</f>
+        <v/>
+      </c>
+      <c r="J14" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A14),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B11" s="30">
-        <f>SUM(B4:B10)</f>
-        <v/>
-      </c>
-      <c r="C11" s="30">
-        <f>SUM(C4:C10)</f>
-        <v/>
-      </c>
-      <c r="D11" s="30">
-        <f>SUM(D4:D10)</f>
-        <v/>
-      </c>
-      <c r="E11" s="31">
-        <f>IFERROR(C11/B11,"")</f>
-        <v/>
-      </c>
-      <c r="F11" s="32">
-        <f>SUM(F4:F10)</f>
-        <v/>
-      </c>
-      <c r="G11" s="32">
-        <f>SUM(G4:G10)</f>
-        <v/>
-      </c>
-      <c r="H11" s="32">
-        <f>IFERROR(G11/B11,"")</f>
+      <c r="B15" s="30">
+        <f>SUM(B4:B14)</f>
+        <v/>
+      </c>
+      <c r="C15" s="30">
+        <f>SUM(C4:C14)</f>
+        <v/>
+      </c>
+      <c r="D15" s="30">
+        <f>SUM(D4:D14)</f>
+        <v/>
+      </c>
+      <c r="E15" s="31">
+        <f>IFERROR(C15/B15,"")</f>
+        <v/>
+      </c>
+      <c r="F15" s="32">
+        <f>SUM(F4:F14)</f>
+        <v/>
+      </c>
+      <c r="G15" s="32">
+        <f>SUM(G4:G14)</f>
+        <v/>
+      </c>
+      <c r="H15" s="32">
+        <f>IFERROR(G15/B15,"")</f>
         <v/>
       </c>
     </row>
@@ -30341,7 +30617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -30469,19 +30745,19 @@
         <v>0</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>150.32</v>
+        <v>300.68</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>4.61</v>
+        <v>9.23</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>0.15</v>
+        <v>0.3</v>
       </c>
       <c r="I4" s="4" t="n">
         <v>22.55</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>0.86</v>
+        <v>1.72</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>14.75</v>
@@ -30517,22 +30793,22 @@
         <v>46301</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>90.04000000000001</v>
+        <v>110.04</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>300.12</v>
+        <v>591.87</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>9.210000000000001</v>
+        <v>18.17</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>0.3</v>
+        <v>0.59</v>
       </c>
       <c r="I5" s="4" t="n">
         <v>45.02</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>17.92</v>
+        <v>23.18</v>
       </c>
       <c r="K5" s="4" t="n">
         <v>14.75</v>
@@ -30568,22 +30844,22 @@
         <v>46301</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>298.83</v>
+        <v>585.45</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>9.19</v>
+        <v>17.98</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>0.3</v>
+        <v>0.59</v>
       </c>
       <c r="I6" s="4" t="n">
         <v>44.97</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>5.31</v>
+        <v>10.54</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>14.75</v>
@@ -30602,12 +30878,12 @@
     <row r="7">
       <c r="A7" s="23" t="inlineStr">
         <is>
-          <t>DHAN-34126100566209+321261005656309+34126100566409+321261005657009+23126100565509+23126100565609+34126100566609+34126100566709+221261005674009+321261005658809+221261005675209+23126100566009+321261005659709+34126100567409+221261005676309+34126100567709</t>
+          <t>DHAN-321261006605709</t>
         </is>
       </c>
       <c r="B7" s="23" t="inlineStr">
         <is>
-          <t>DPABHUSHAN</t>
+          <t>KRISHNADEF</t>
         </is>
       </c>
       <c r="C7" s="23" t="inlineStr">
@@ -30615,33 +30891,35 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D7" s="24" t="inlineStr"/>
+      <c r="D7" s="24" t="n">
+        <v>46302</v>
+      </c>
       <c r="E7" s="4" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>149.73</v>
+        <v>300.16</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>4.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>0.15</v>
+        <v>0.3</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>22.46</v>
+        <v>45.16</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>0.85</v>
+        <v>5.31</v>
       </c>
       <c r="K7" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L7" s="4" t="n">
-        <v>0</v>
+        <v>35.4</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>0</v>
+        <v>51.24</v>
       </c>
       <c r="N7" s="21">
         <f>SUM(E7:M7)</f>
@@ -30651,12 +30929,12 @@
     <row r="8">
       <c r="A8" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261006605709</t>
+          <t>DHAN-34126100671709+23126100663009+23126100663109+321261006600309+321261006600609+321261006600809+23126100663309+221261006573809+221261006574009+23126100663509+23126100663709+23126100663809+34126100672309+221261006576409+221261006576709</t>
         </is>
       </c>
       <c r="B8" s="23" t="inlineStr">
         <is>
-          <t>KRISHNADEF</t>
+          <t>SATIN</t>
         </is>
       </c>
       <c r="C8" s="23" t="inlineStr">
@@ -30664,24 +30942,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D8" s="24" t="inlineStr"/>
+      <c r="D8" s="24" t="n">
+        <v>46302</v>
+      </c>
       <c r="E8" s="4" t="n">
-        <v>0</v>
+        <v>89.77</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>0</v>
+        <v>299.29</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>0</v>
+        <v>9.19</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>0</v>
+        <v>44.89</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>0</v>
+        <v>17.87</v>
       </c>
       <c r="K8" s="4" t="n">
         <v>14.75</v>
@@ -30690,7 +30970,7 @@
         <v>35.4</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>0</v>
+        <v>61.41</v>
       </c>
       <c r="N8" s="21">
         <f>SUM(E8:M8)</f>
@@ -30700,12 +30980,12 @@
     <row r="9">
       <c r="A9" s="23" t="inlineStr">
         <is>
-          <t>DHAN-34126100671709+23126100663009+23126100663109+321261006600309+321261006600609+321261006600809+23126100663309+221261006573809+221261006574009+23126100663509+23126100663709+23126100663809+34126100672309+221261006576409+221261006576709</t>
+          <t>DHAN-34126100786209</t>
         </is>
       </c>
       <c r="B9" s="23" t="inlineStr">
         <is>
-          <t>SATIN</t>
+          <t>ARFIN</t>
         </is>
       </c>
       <c r="C9" s="23" t="inlineStr">
@@ -30749,12 +31029,12 @@
     <row r="10">
       <c r="A10" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261006571909+221261006572109+34126100671809+23126100663209+34126100672009+23126100663409+321261006601809+34126100672209+23126100663909+23126100664109+23126100664209+34126100672409+23126100664309+221261006577209+34126100672509</t>
+          <t>DHAN-34126100566209+321261005656309+34126100566409+321261005657009+23126100565509+23126100565609+34126100566609+34126100566709+221261005674009+321261005658809+221261005675209+23126100566009+321261005659709+34126100567409+221261005676309+34126100567709</t>
         </is>
       </c>
       <c r="B10" s="23" t="inlineStr">
         <is>
-          <t>YUKEN</t>
+          <t>DPABHUSHAN</t>
         </is>
       </c>
       <c r="C10" s="23" t="inlineStr">
@@ -30767,25 +31047,25 @@
         <v>0</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>0</v>
+        <v>149.73</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0</v>
+        <v>4.6</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>0</v>
+        <v>22.46</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>0</v>
+        <v>0.85</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>35.4</v>
+        <v>0</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>0</v>
@@ -30796,54 +31076,250 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261007626809+321261007628809+34126100785209+34126100785309+23126100782509+34126100785409+221261007628809+321261007630509+34126100785509+23126100782909+34126100785609+34126100785709+23126100783209+221261007631209+34126100785809+321261007631609+321261007632109</t>
+        </is>
+      </c>
+      <c r="B11" s="23" t="inlineStr">
+        <is>
+          <t>GPTINFRA</t>
+        </is>
+      </c>
+      <c r="C11" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D11" s="24" t="inlineStr"/>
+      <c r="E11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L11" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="21">
+        <f>SUM(E11:M11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261007633409</t>
+        </is>
+      </c>
+      <c r="B12" s="23" t="inlineStr">
+        <is>
+          <t>MOBIKWIK</t>
+        </is>
+      </c>
+      <c r="C12" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D12" s="24" t="inlineStr"/>
+      <c r="E12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="21">
+        <f>SUM(E12:M12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126100785009+34126100785109+221261007627809+221261007628109+321261007629509+23126100782809+321261007629709+221261007629309+221261007629609+221261007629909+23126100783009</t>
+        </is>
+      </c>
+      <c r="B13" s="23" t="inlineStr">
+        <is>
+          <t>PNGSREVA</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D13" s="24" t="inlineStr"/>
+      <c r="E13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L13" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="21">
+        <f>SUM(E13:M13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261006571909+221261006572109+34126100671809+23126100663209+34126100672009+23126100663409+321261006601809+34126100672209+23126100663909+23126100664109+23126100664209+34126100672409+23126100664309+221261006577209+34126100672509</t>
+        </is>
+      </c>
+      <c r="B14" s="23" t="inlineStr">
+        <is>
+          <t>YUKEN</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D14" s="24" t="inlineStr"/>
+      <c r="E14" s="4" t="n">
+        <v>89.91</v>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>299.69</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="H14" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="I14" s="4" t="n">
+        <v>44.95</v>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>17.89</v>
+      </c>
+      <c r="K14" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L14" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M14" s="4" t="n">
+        <v>51.25</v>
+      </c>
+      <c r="N14" s="21">
+        <f>SUM(E14:M14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E11" s="32">
-        <f>SUM(E4:E10)</f>
-        <v/>
-      </c>
-      <c r="F11" s="32">
-        <f>SUM(F4:F10)</f>
-        <v/>
-      </c>
-      <c r="G11" s="32">
-        <f>SUM(G4:G10)</f>
-        <v/>
-      </c>
-      <c r="H11" s="32">
-        <f>SUM(H4:H10)</f>
-        <v/>
-      </c>
-      <c r="I11" s="32">
-        <f>SUM(I4:I10)</f>
-        <v/>
-      </c>
-      <c r="J11" s="32">
-        <f>SUM(J4:J10)</f>
-        <v/>
-      </c>
-      <c r="K11" s="32">
-        <f>SUM(K4:K10)</f>
-        <v/>
-      </c>
-      <c r="L11" s="32">
-        <f>SUM(L4:L10)</f>
-        <v/>
-      </c>
-      <c r="M11" s="32">
-        <f>SUM(M4:M10)</f>
-        <v/>
-      </c>
-      <c r="N11" s="32">
-        <f>SUM(N4:N10)</f>
+      <c r="E15" s="32">
+        <f>SUM(E4:E14)</f>
+        <v/>
+      </c>
+      <c r="F15" s="32">
+        <f>SUM(F4:F14)</f>
+        <v/>
+      </c>
+      <c r="G15" s="32">
+        <f>SUM(G4:G14)</f>
+        <v/>
+      </c>
+      <c r="H15" s="32">
+        <f>SUM(H4:H14)</f>
+        <v/>
+      </c>
+      <c r="I15" s="32">
+        <f>SUM(I4:I14)</f>
+        <v/>
+      </c>
+      <c r="J15" s="32">
+        <f>SUM(J4:J14)</f>
+        <v/>
+      </c>
+      <c r="K15" s="32">
+        <f>SUM(K4:K14)</f>
+        <v/>
+      </c>
+      <c r="L15" s="32">
+        <f>SUM(L4:L14)</f>
+        <v/>
+      </c>
+      <c r="M15" s="32">
+        <f>SUM(M4:M14)</f>
+        <v/>
+      </c>
+      <c r="N15" s="32">
+        <f>SUM(N4:N14)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:N10"/>
+  <autoFilter ref="A3:N14"/>
   <mergeCells count="2">
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>

</xml_diff>

<commit_message>
Data update — 2026-10-08 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_oct2026.xlsx
+++ b/results/strategy_pnl_oct2026.xlsx
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trade Log'!$A$3:$O$503</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1117,12 +1117,12 @@
     <row r="5">
       <c r="A5" s="23" t="inlineStr">
         <is>
-          <t>DHAN-23126100565309+34126100566309+23126100565409+34126100566509+221261005673109+23126100565709+221261005673609+34126100566809+23126100565809+23126100565909+34126100567109+34126100567209+34126100567309</t>
+          <t>DHAN-34126100566209+321261005656309+34126100566409+321261005657009+23126100565509+23126100565609+34126100566609+34126100566709+221261005674009+321261005658809+221261005675209+23126100566009+321261005659709+34126100567409+221261005676309+34126100567709</t>
         </is>
       </c>
       <c r="B5" s="23" t="inlineStr">
         <is>
-          <t>SGFIN</t>
+          <t>DPABHUSHAN</t>
         </is>
       </c>
       <c r="C5" s="23" t="inlineStr">
@@ -1134,16 +1134,16 @@
         <v>46300</v>
       </c>
       <c r="E5" s="25" t="n">
-        <v>679.0067</v>
+        <v>2108.8394</v>
       </c>
       <c r="F5" s="26" t="n">
-        <v>442</v>
+        <v>71</v>
       </c>
       <c r="G5" s="24" t="n">
         <v>46301</v>
       </c>
       <c r="H5" s="25" t="n">
-        <v>660.0599999999999</v>
+        <v>1945.5</v>
       </c>
       <c r="I5" s="21">
         <f>IF(OR($B5="",$H5=""),"",IF($C5="LONG",($H5-$E5)*$F5,($E5-$H5)*$F5))</f>
@@ -1154,7 +1154,7 @@
         <v/>
       </c>
       <c r="K5" s="4" t="n">
-        <v>900.61</v>
+        <v>192.54</v>
       </c>
       <c r="L5" s="21">
         <f>IF(OR($B5="",$I5=""),"",$I5-IF($K5="",0,$K5))</f>
@@ -1170,19 +1170,19 @@
       </c>
       <c r="O5" s="23" t="inlineStr">
         <is>
-          <t>5-10</t>
+          <t>10-15</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261005679509</t>
+          <t>DHAN-23126100565309+34126100566309+23126100565409+34126100566509+221261005673109+23126100565709+221261005673609+34126100566809+23126100565809+23126100565909+34126100567109+34126100567209+34126100567309</t>
         </is>
       </c>
       <c r="B6" s="23" t="inlineStr">
         <is>
-          <t>SMCGLOBAL</t>
+          <t>SGFIN</t>
         </is>
       </c>
       <c r="C6" s="23" t="inlineStr">
@@ -1194,16 +1194,16 @@
         <v>46300</v>
       </c>
       <c r="E6" s="25" t="n">
-        <v>113.9808</v>
+        <v>679.0067</v>
       </c>
       <c r="F6" s="26" t="n">
-        <v>2624</v>
+        <v>442</v>
       </c>
       <c r="G6" s="24" t="n">
         <v>46301</v>
       </c>
       <c r="H6" s="25" t="n">
-        <v>109.23</v>
+        <v>660.0599999999999</v>
       </c>
       <c r="I6" s="21">
         <f>IF(OR($B6="",$H6=""),"",IF($C6="LONG",($H6-$E6)*$F6,($E6-$H6)*$F6))</f>
@@ -1214,7 +1214,7 @@
         <v/>
       </c>
       <c r="K6" s="4" t="n">
-        <v>800.83</v>
+        <v>900.61</v>
       </c>
       <c r="L6" s="21">
         <f>IF(OR($B6="",$I6=""),"",$I6-IF($K6="",0,$K6))</f>
@@ -1230,19 +1230,19 @@
       </c>
       <c r="O6" s="23" t="inlineStr">
         <is>
-          <t>15-20</t>
+          <t>5-10</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261006605709</t>
+          <t>DHAN-221261005679509</t>
         </is>
       </c>
       <c r="B7" s="23" t="inlineStr">
         <is>
-          <t>KRISHNADEF</t>
+          <t>SMCGLOBAL</t>
         </is>
       </c>
       <c r="C7" s="23" t="inlineStr">
@@ -1251,19 +1251,19 @@
         </is>
       </c>
       <c r="D7" s="24" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E7" s="25" t="n">
+        <v>113.9808</v>
+      </c>
+      <c r="F7" s="26" t="n">
+        <v>2624</v>
+      </c>
+      <c r="G7" s="24" t="n">
         <v>46301</v>
       </c>
-      <c r="E7" s="25" t="n">
-        <v>1297.2208</v>
-      </c>
-      <c r="F7" s="26" t="n">
-        <v>231</v>
-      </c>
-      <c r="G7" s="24" t="n">
-        <v>46302</v>
-      </c>
       <c r="H7" s="25" t="n">
-        <v>1280.57</v>
+        <v>109.23</v>
       </c>
       <c r="I7" s="21">
         <f>IF(OR($B7="",$H7=""),"",IF($C7="LONG",($H7-$E7)*$F7,($E7-$H7)*$F7))</f>
@@ -1274,7 +1274,7 @@
         <v/>
       </c>
       <c r="K7" s="4" t="n">
-        <v>481.53</v>
+        <v>786.51</v>
       </c>
       <c r="L7" s="21">
         <f>IF(OR($B7="",$I7=""),"",$I7-IF($K7="",0,$K7))</f>
@@ -1290,19 +1290,19 @@
       </c>
       <c r="O7" s="23" t="inlineStr">
         <is>
-          <t>10-15</t>
+          <t>15-20</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="23" t="inlineStr">
         <is>
-          <t>DHAN-34126100671709+23126100663009+23126100663109+321261006600309+321261006600609+321261006600809+23126100663309+221261006573809+221261006574009+23126100663509+23126100663709+23126100663809+34126100672309+221261006576409+221261006576709</t>
+          <t>DHAN-321261006605709</t>
         </is>
       </c>
       <c r="B8" s="23" t="inlineStr">
         <is>
-          <t>SATIN</t>
+          <t>KRISHNADEF</t>
         </is>
       </c>
       <c r="C8" s="23" t="inlineStr">
@@ -1314,16 +1314,16 @@
         <v>46301</v>
       </c>
       <c r="E8" s="25" t="n">
-        <v>228.9869</v>
+        <v>1297.2208</v>
       </c>
       <c r="F8" s="26" t="n">
-        <v>1307</v>
+        <v>231</v>
       </c>
       <c r="G8" s="24" t="n">
         <v>46302</v>
       </c>
       <c r="H8" s="25" t="n">
-        <v>235.36</v>
+        <v>1280.57</v>
       </c>
       <c r="I8" s="21">
         <f>IF(OR($B8="",$H8=""),"",IF($C8="LONG",($H8-$E8)*$F8,($E8-$H8)*$F8))</f>
@@ -1334,7 +1334,7 @@
         <v/>
       </c>
       <c r="K8" s="4" t="n">
-        <v>572.87</v>
+        <v>812</v>
       </c>
       <c r="L8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($K8="",0,$K8))</f>
@@ -1350,19 +1350,19 @@
       </c>
       <c r="O8" s="23" t="inlineStr">
         <is>
-          <t>5-10</t>
+          <t>10-15</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="23" t="inlineStr">
         <is>
-          <t>DHAN-34126100786209</t>
+          <t>DHAN-34126100671709+23126100663009+23126100663109+321261006600309+321261006600609+321261006600809+23126100663309+221261006573809+221261006574009+23126100663509+23126100663709+23126100663809+34126100672309+221261006576409+221261006576709</t>
         </is>
       </c>
       <c r="B9" s="23" t="inlineStr">
         <is>
-          <t>ARFIN</t>
+          <t>SATIN</t>
         </is>
       </c>
       <c r="C9" s="23" t="inlineStr">
@@ -1371,16 +1371,20 @@
         </is>
       </c>
       <c r="D9" s="24" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E9" s="25" t="n">
+        <v>228.9869</v>
+      </c>
+      <c r="F9" s="26" t="n">
+        <v>1307</v>
+      </c>
+      <c r="G9" s="24" t="n">
         <v>46302</v>
       </c>
-      <c r="E9" s="25" t="n">
-        <v>103.743</v>
-      </c>
-      <c r="F9" s="26" t="n">
-        <v>2316</v>
-      </c>
-      <c r="G9" s="24" t="inlineStr"/>
-      <c r="H9" s="25" t="inlineStr"/>
+      <c r="H9" s="25" t="n">
+        <v>235.36</v>
+      </c>
       <c r="I9" s="21">
         <f>IF(OR($B9="",$H9=""),"",IF($C9="LONG",($H9-$E9)*$F9,($E9-$H9)*$F9))</f>
         <v/>
@@ -1390,7 +1394,7 @@
         <v/>
       </c>
       <c r="K9" s="4" t="n">
-        <v>50.15</v>
+        <v>915.22</v>
       </c>
       <c r="L9" s="21">
         <f>IF(OR($B9="",$I9=""),"",$I9-IF($K9="",0,$K9))</f>
@@ -1413,12 +1417,12 @@
     <row r="10">
       <c r="A10" s="23" t="inlineStr">
         <is>
-          <t>DHAN-34126100566209+321261005656309+34126100566409+321261005657009+23126100565509+23126100565609+34126100566609+34126100566709+221261005674009+321261005658809+221261005675209+23126100566009+321261005659709+34126100567409+221261005676309+34126100567709</t>
+          <t>DHAN-221261006571909+221261006572109+34126100671809+23126100663209+34126100672009+23126100663409+321261006601809+34126100672209+23126100663909+23126100664109+23126100664209+34126100672409+23126100664309+221261006577209+34126100672509</t>
         </is>
       </c>
       <c r="B10" s="23" t="inlineStr">
         <is>
-          <t>DPABHUSHAN</t>
+          <t>YUKEN</t>
         </is>
       </c>
       <c r="C10" s="23" t="inlineStr">
@@ -1427,16 +1431,20 @@
         </is>
       </c>
       <c r="D10" s="24" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="E10" s="25" t="n">
-        <v>2108.8394</v>
+        <v>1238.3789</v>
       </c>
       <c r="F10" s="26" t="n">
-        <v>71</v>
-      </c>
-      <c r="G10" s="24" t="inlineStr"/>
-      <c r="H10" s="25" t="inlineStr"/>
+        <v>242</v>
+      </c>
+      <c r="G10" s="24" t="n">
+        <v>46302</v>
+      </c>
+      <c r="H10" s="25" t="n">
+        <v>1238.1025</v>
+      </c>
       <c r="I10" s="21">
         <f>IF(OR($B10="",$H10=""),"",IF($C10="LONG",($H10-$E10)*$F10,($E10-$H10)*$F10))</f>
         <v/>
@@ -1446,7 +1454,7 @@
         <v/>
       </c>
       <c r="K10" s="4" t="n">
-        <v>192.54</v>
+        <v>897.77</v>
       </c>
       <c r="L10" s="21">
         <f>IF(OR($B10="",$I10=""),"",$I10-IF($K10="",0,$K10))</f>
@@ -1469,12 +1477,12 @@
     <row r="11">
       <c r="A11" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261007626809+321261007628809+34126100785209+34126100785309+23126100782509+34126100785409+221261007628809+321261007630509+34126100785509+23126100782909+34126100785609+34126100785709+23126100783209+221261007631209+34126100785809+321261007631609+321261007632109</t>
+          <t>DHAN-34126100786209</t>
         </is>
       </c>
       <c r="B11" s="23" t="inlineStr">
         <is>
-          <t>GPTINFRA</t>
+          <t>ARFIN</t>
         </is>
       </c>
       <c r="C11" s="23" t="inlineStr">
@@ -1486,13 +1494,17 @@
         <v>46302</v>
       </c>
       <c r="E11" s="25" t="n">
-        <v>129.8444</v>
+        <v>103.743</v>
       </c>
       <c r="F11" s="26" t="n">
-        <v>1848</v>
-      </c>
-      <c r="G11" s="24" t="inlineStr"/>
-      <c r="H11" s="25" t="inlineStr"/>
+        <v>2316</v>
+      </c>
+      <c r="G11" s="24" t="n">
+        <v>46303</v>
+      </c>
+      <c r="H11" s="25" t="n">
+        <v>103.7</v>
+      </c>
       <c r="I11" s="21">
         <f>IF(OR($B11="",$H11=""),"",IF($C11="LONG",($H11-$E11)*$F11,($E11-$H11)*$F11))</f>
         <v/>
@@ -1502,7 +1514,7 @@
         <v/>
       </c>
       <c r="K11" s="4" t="n">
-        <v>50.15</v>
+        <v>400.07</v>
       </c>
       <c r="L11" s="21">
         <f>IF(OR($B11="",$I11=""),"",$I11-IF($K11="",0,$K11))</f>
@@ -1525,12 +1537,12 @@
     <row r="12">
       <c r="A12" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261007633409</t>
+          <t>DHAN-221261007626809+321261007628809+34126100785209+34126100785309+23126100782509+34126100785409+221261007628809+321261007630509+34126100785509+23126100782909+34126100785609+34126100785709+23126100783209+221261007631209+34126100785809+321261007631609+321261007632109</t>
         </is>
       </c>
       <c r="B12" s="23" t="inlineStr">
         <is>
-          <t>MOBIKWIK</t>
+          <t>GPTINFRA</t>
         </is>
       </c>
       <c r="C12" s="23" t="inlineStr">
@@ -1542,13 +1554,17 @@
         <v>46302</v>
       </c>
       <c r="E12" s="25" t="n">
-        <v>257.0405</v>
+        <v>129.8444</v>
       </c>
       <c r="F12" s="26" t="n">
-        <v>936</v>
-      </c>
-      <c r="G12" s="24" t="inlineStr"/>
-      <c r="H12" s="25" t="inlineStr"/>
+        <v>1848</v>
+      </c>
+      <c r="G12" s="24" t="n">
+        <v>46303</v>
+      </c>
+      <c r="H12" s="25" t="n">
+        <v>125.94</v>
+      </c>
       <c r="I12" s="21">
         <f>IF(OR($B12="",$H12=""),"",IF($C12="LONG",($H12-$E12)*$F12,($E12-$H12)*$F12))</f>
         <v/>
@@ -1558,7 +1574,7 @@
         <v/>
       </c>
       <c r="K12" s="4" t="n">
-        <v>50.15</v>
+        <v>469.24</v>
       </c>
       <c r="L12" s="21">
         <f>IF(OR($B12="",$I12=""),"",$I12-IF($K12="",0,$K12))</f>
@@ -1581,12 +1597,12 @@
     <row r="13">
       <c r="A13" s="23" t="inlineStr">
         <is>
-          <t>DHAN-34126100785009+34126100785109+221261007627809+221261007628109+321261007629509+23126100782809+321261007629709+221261007629309+221261007629609+221261007629909+23126100783009</t>
+          <t>DHAN-321261007633409</t>
         </is>
       </c>
       <c r="B13" s="23" t="inlineStr">
         <is>
-          <t>PNGSREVA</t>
+          <t>MOBIKWIK</t>
         </is>
       </c>
       <c r="C13" s="23" t="inlineStr">
@@ -1598,13 +1614,17 @@
         <v>46302</v>
       </c>
       <c r="E13" s="25" t="n">
-        <v>622.1242</v>
+        <v>257.0405</v>
       </c>
       <c r="F13" s="26" t="n">
-        <v>385</v>
-      </c>
-      <c r="G13" s="24" t="inlineStr"/>
-      <c r="H13" s="25" t="inlineStr"/>
+        <v>936</v>
+      </c>
+      <c r="G13" s="24" t="n">
+        <v>46303</v>
+      </c>
+      <c r="H13" s="25" t="n">
+        <v>238.86</v>
+      </c>
       <c r="I13" s="21">
         <f>IF(OR($B13="",$H13=""),"",IF($C13="LONG",($H13-$E13)*$F13,($E13-$H13)*$F13))</f>
         <v/>
@@ -1614,7 +1634,7 @@
         <v/>
       </c>
       <c r="K13" s="4" t="n">
-        <v>50.15</v>
+        <v>409.68</v>
       </c>
       <c r="L13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($K13="",0,$K13))</f>
@@ -1630,19 +1650,19 @@
       </c>
       <c r="O13" s="23" t="inlineStr">
         <is>
-          <t>10-15</t>
+          <t>5-10</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261006571909+221261006572109+34126100671809+23126100663209+34126100672009+23126100663409+321261006601809+34126100672209+23126100663909+23126100664109+23126100664209+34126100672409+23126100664309+221261006577209+34126100672509</t>
+          <t>DHAN-34126100785009+34126100785109+221261007627809+221261007628109+321261007629509+23126100782809+321261007629709+221261007629309+221261007629609+221261007629909+23126100783009</t>
         </is>
       </c>
       <c r="B14" s="23" t="inlineStr">
         <is>
-          <t>YUKEN</t>
+          <t>PNGSREVA</t>
         </is>
       </c>
       <c r="C14" s="23" t="inlineStr">
@@ -1651,16 +1671,20 @@
         </is>
       </c>
       <c r="D14" s="24" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E14" s="25" t="n">
-        <v>1238.3789</v>
+        <v>622.1242</v>
       </c>
       <c r="F14" s="26" t="n">
-        <v>242</v>
-      </c>
-      <c r="G14" s="24" t="inlineStr"/>
-      <c r="H14" s="25" t="inlineStr"/>
+        <v>385</v>
+      </c>
+      <c r="G14" s="24" t="n">
+        <v>46303</v>
+      </c>
+      <c r="H14" s="25" t="n">
+        <v>636</v>
+      </c>
       <c r="I14" s="21">
         <f>IF(OR($B14="",$H14=""),"",IF($C14="LONG",($H14-$E14)*$F14,($E14-$H14)*$F14))</f>
         <v/>
@@ -1670,7 +1694,7 @@
         <v/>
       </c>
       <c r="K14" s="4" t="n">
-        <v>563.34</v>
+        <v>460.32</v>
       </c>
       <c r="L14" s="21">
         <f>IF(OR($B14="",$I14=""),"",$I14-IF($K14="",0,$K14))</f>
@@ -1691,14 +1715,32 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="n"/>
-      <c r="B15" s="23" t="n"/>
-      <c r="C15" s="23" t="n"/>
-      <c r="D15" s="24" t="n"/>
-      <c r="E15" s="25" t="n"/>
-      <c r="F15" s="26" t="n"/>
-      <c r="G15" s="24" t="n"/>
-      <c r="H15" s="25" t="n"/>
+      <c r="A15" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126100860109+221261008541409+34126100865109+34126100865209+23126100860209+321261008684009+221261008543809+34126100865509+34126100865709+321261008684809+321261008685109+321261008685409+34126100865909+34126100866009+221261008545809+221261008545909+34126100866109+23126100860509</t>
+        </is>
+      </c>
+      <c r="B15" s="23" t="inlineStr">
+        <is>
+          <t>KOTIC</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D15" s="24" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E15" s="25" t="n">
+        <v>157.0151</v>
+      </c>
+      <c r="F15" s="26" t="n">
+        <v>858</v>
+      </c>
+      <c r="G15" s="24" t="inlineStr"/>
+      <c r="H15" s="25" t="inlineStr"/>
       <c r="I15" s="21">
         <f>IF(OR($B15="",$H15=""),"",IF($C15="LONG",($H15-$E15)*$F15,($E15-$H15)*$F15))</f>
         <v/>
@@ -1707,7 +1749,9 @@
         <f>IF(OR($B15="",$I15="",$E15=0,$F15=0),"",$I15/($E15*$F15))</f>
         <v/>
       </c>
-      <c r="K15" s="4" t="n"/>
+      <c r="K15" s="4" t="n">
+        <v>14.75</v>
+      </c>
       <c r="L15" s="21">
         <f>IF(OR($B15="",$I15=""),"",$I15-IF($K15="",0,$K15))</f>
         <v/>
@@ -1720,17 +1764,39 @@
         <f>IF($B15="","",IF($H15="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O15" s="23" t="n"/>
+      <c r="O15" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="23" t="n"/>
-      <c r="B16" s="23" t="n"/>
-      <c r="C16" s="23" t="n"/>
-      <c r="D16" s="24" t="n"/>
-      <c r="E16" s="25" t="n"/>
-      <c r="F16" s="26" t="n"/>
-      <c r="G16" s="24" t="n"/>
-      <c r="H16" s="25" t="n"/>
+      <c r="A16" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261008541309+221261008541509+321261008683209+221261008542109+34126100865309+34126100865409+221261008543409+221261008543909+221261008544309+34126100865609+221261008545009+23126100860309+34126100865809+23126100860409</t>
+        </is>
+      </c>
+      <c r="B16" s="23" t="inlineStr">
+        <is>
+          <t>PNGSREVA</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D16" s="24" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E16" s="25" t="n">
+        <v>705.2641</v>
+      </c>
+      <c r="F16" s="26" t="n">
+        <v>213</v>
+      </c>
+      <c r="G16" s="24" t="inlineStr"/>
+      <c r="H16" s="25" t="inlineStr"/>
       <c r="I16" s="21">
         <f>IF(OR($B16="",$H16=""),"",IF($C16="LONG",($H16-$E16)*$F16,($E16-$H16)*$F16))</f>
         <v/>
@@ -1739,7 +1805,9 @@
         <f>IF(OR($B16="",$I16="",$E16=0,$F16=0),"",$I16/($E16*$F16))</f>
         <v/>
       </c>
-      <c r="K16" s="4" t="n"/>
+      <c r="K16" s="4" t="n">
+        <v>14.75</v>
+      </c>
       <c r="L16" s="21">
         <f>IF(OR($B16="",$I16=""),"",$I16-IF($K16="",0,$K16))</f>
         <v/>
@@ -1752,7 +1820,11 @@
         <f>IF($B16="","",IF($H16="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O16" s="23" t="n"/>
+      <c r="O16" s="23" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="23" t="n"/>
@@ -30013,7 +30085,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30269,7 +30341,7 @@
     <row r="8">
       <c r="A8" s="27" t="inlineStr">
         <is>
-          <t>KRISHNADEF</t>
+          <t>KOTIC</t>
         </is>
       </c>
       <c r="B8" s="20">
@@ -30312,7 +30384,7 @@
     <row r="9">
       <c r="A9" s="27" t="inlineStr">
         <is>
-          <t>MOBIKWIK</t>
+          <t>KRISHNADEF</t>
         </is>
       </c>
       <c r="B9" s="20">
@@ -30355,7 +30427,7 @@
     <row r="10">
       <c r="A10" s="27" t="inlineStr">
         <is>
-          <t>PNGSREVA</t>
+          <t>MOBIKWIK</t>
         </is>
       </c>
       <c r="B10" s="20">
@@ -30398,7 +30470,7 @@
     <row r="11">
       <c r="A11" s="27" t="inlineStr">
         <is>
-          <t>SATIN</t>
+          <t>PNGSREVA</t>
         </is>
       </c>
       <c r="B11" s="20">
@@ -30441,7 +30513,7 @@
     <row r="12">
       <c r="A12" s="27" t="inlineStr">
         <is>
-          <t>SGFIN</t>
+          <t>SATIN</t>
         </is>
       </c>
       <c r="B12" s="20">
@@ -30484,7 +30556,7 @@
     <row r="13">
       <c r="A13" s="27" t="inlineStr">
         <is>
-          <t>SMCGLOBAL</t>
+          <t>SGFIN</t>
         </is>
       </c>
       <c r="B13" s="20">
@@ -30527,78 +30599,121 @@
     <row r="14">
       <c r="A14" s="27" t="inlineStr">
         <is>
+          <t>SMCGLOBAL</t>
+        </is>
+      </c>
+      <c r="B14" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A14)</f>
+        <v/>
+      </c>
+      <c r="C14" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A14,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D14" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A14,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E14" s="22">
+        <f>IFERROR($C14/$B14,"")</f>
+        <v/>
+      </c>
+      <c r="F14" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A14,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G14" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A14,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H14" s="21">
+        <f>IFERROR($G14/$B14,"")</f>
+        <v/>
+      </c>
+      <c r="I14" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A14),"")</f>
+        <v/>
+      </c>
+      <c r="J14" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A14),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="27" t="inlineStr">
+        <is>
           <t>YUKEN</t>
         </is>
       </c>
-      <c r="B14" s="20">
-        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A14)</f>
-        <v/>
-      </c>
-      <c r="C14" s="20">
-        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A14,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
-        <v/>
-      </c>
-      <c r="D14" s="20">
-        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A14,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
-        <v/>
-      </c>
-      <c r="E14" s="22">
-        <f>IFERROR($C14/$B14,"")</f>
-        <v/>
-      </c>
-      <c r="F14" s="21">
-        <f>SUMIF('Trade Log'!$B$4:$B$503,$A14,'Trade Log'!$I$4:$I$503)</f>
-        <v/>
-      </c>
-      <c r="G14" s="21">
-        <f>SUMIF('Trade Log'!$B$4:$B$503,$A14,'Trade Log'!$L$4:$L$503)</f>
-        <v/>
-      </c>
-      <c r="H14" s="21">
-        <f>IFERROR($G14/$B14,"")</f>
-        <v/>
-      </c>
-      <c r="I14" s="21">
-        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A14),"")</f>
-        <v/>
-      </c>
-      <c r="J14" s="21">
-        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A14),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="B15" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A15)</f>
+        <v/>
+      </c>
+      <c r="C15" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A15,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D15" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A15,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E15" s="22">
+        <f>IFERROR($C15/$B15,"")</f>
+        <v/>
+      </c>
+      <c r="F15" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A15,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G15" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A15,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H15" s="21">
+        <f>IFERROR($G15/$B15,"")</f>
+        <v/>
+      </c>
+      <c r="I15" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A15),"")</f>
+        <v/>
+      </c>
+      <c r="J15" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A15),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B15" s="30">
-        <f>SUM(B4:B14)</f>
-        <v/>
-      </c>
-      <c r="C15" s="30">
-        <f>SUM(C4:C14)</f>
-        <v/>
-      </c>
-      <c r="D15" s="30">
-        <f>SUM(D4:D14)</f>
-        <v/>
-      </c>
-      <c r="E15" s="31">
-        <f>IFERROR(C15/B15,"")</f>
-        <v/>
-      </c>
-      <c r="F15" s="32">
-        <f>SUM(F4:F14)</f>
-        <v/>
-      </c>
-      <c r="G15" s="32">
-        <f>SUM(G4:G14)</f>
-        <v/>
-      </c>
-      <c r="H15" s="32">
-        <f>IFERROR(G15/B15,"")</f>
+      <c r="B16" s="30">
+        <f>SUM(B4:B15)</f>
+        <v/>
+      </c>
+      <c r="C16" s="30">
+        <f>SUM(C4:C15)</f>
+        <v/>
+      </c>
+      <c r="D16" s="30">
+        <f>SUM(D4:D15)</f>
+        <v/>
+      </c>
+      <c r="E16" s="31">
+        <f>IFERROR(C16/B16,"")</f>
+        <v/>
+      </c>
+      <c r="F16" s="32">
+        <f>SUM(F4:F15)</f>
+        <v/>
+      </c>
+      <c r="G16" s="32">
+        <f>SUM(G4:G15)</f>
+        <v/>
+      </c>
+      <c r="H16" s="32">
+        <f>IFERROR(G16/B16,"")</f>
         <v/>
       </c>
     </row>
@@ -30617,7 +30732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -30776,12 +30891,12 @@
     <row r="5">
       <c r="A5" s="23" t="inlineStr">
         <is>
-          <t>DHAN-23126100565309+34126100566309+23126100565409+34126100566509+221261005673109+23126100565709+221261005673609+34126100566809+23126100565809+23126100565909+34126100567109+34126100567209+34126100567309</t>
+          <t>DHAN-34126100566209+321261005656309+34126100566409+321261005657009+23126100565509+23126100565609+34126100566609+34126100566709+221261005674009+321261005658809+221261005675209+23126100566009+321261005659709+34126100567409+221261005676309+34126100567709</t>
         </is>
       </c>
       <c r="B5" s="23" t="inlineStr">
         <is>
-          <t>SGFIN</t>
+          <t>DPABHUSHAN</t>
         </is>
       </c>
       <c r="C5" s="23" t="inlineStr">
@@ -30793,31 +30908,31 @@
         <v>46301</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>110.04</v>
+        <v>0</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>591.87</v>
+        <v>149.73</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>18.17</v>
+        <v>4.6</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>0.59</v>
+        <v>0.15</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>45.02</v>
+        <v>22.46</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>23.18</v>
+        <v>0.85</v>
       </c>
       <c r="K5" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L5" s="4" t="n">
-        <v>35.4</v>
+        <v>0</v>
       </c>
       <c r="M5" s="4" t="n">
-        <v>61.58</v>
+        <v>0</v>
       </c>
       <c r="N5" s="21">
         <f>SUM(E5:M5)</f>
@@ -30827,12 +30942,12 @@
     <row r="6">
       <c r="A6" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261005679509</t>
+          <t>DHAN-23126100565309+34126100566309+23126100565409+34126100566509+221261005673109+23126100565709+221261005673609+34126100566809+23126100565809+23126100565909+34126100567109+34126100567209+34126100567309</t>
         </is>
       </c>
       <c r="B6" s="23" t="inlineStr">
         <is>
-          <t>SMCGLOBAL</t>
+          <t>SGFIN</t>
         </is>
       </c>
       <c r="C6" s="23" t="inlineStr">
@@ -30844,22 +30959,22 @@
         <v>46301</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>40</v>
+        <v>110.04</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>585.45</v>
+        <v>591.87</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>17.98</v>
+        <v>18.17</v>
       </c>
       <c r="H6" s="4" t="n">
         <v>0.59</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>44.97</v>
+        <v>45.02</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>10.54</v>
+        <v>23.18</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>14.75</v>
@@ -30868,7 +30983,7 @@
         <v>35.4</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>51.14</v>
+        <v>61.58</v>
       </c>
       <c r="N6" s="21">
         <f>SUM(E6:M6)</f>
@@ -30878,12 +30993,12 @@
     <row r="7">
       <c r="A7" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261006605709</t>
+          <t>DHAN-221261005679509</t>
         </is>
       </c>
       <c r="B7" s="23" t="inlineStr">
         <is>
-          <t>KRISHNADEF</t>
+          <t>SMCGLOBAL</t>
         </is>
       </c>
       <c r="C7" s="23" t="inlineStr">
@@ -30892,25 +31007,25 @@
         </is>
       </c>
       <c r="D7" s="24" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>300.16</v>
+        <v>585.45</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>9.199999999999999</v>
+        <v>17.98</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>0.3</v>
+        <v>0.59</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>45.16</v>
+        <v>44.97</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>5.31</v>
+        <v>10.54</v>
       </c>
       <c r="K7" s="4" t="n">
         <v>14.75</v>
@@ -30919,7 +31034,7 @@
         <v>35.4</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>51.24</v>
+        <v>36.82</v>
       </c>
       <c r="N7" s="21">
         <f>SUM(E7:M7)</f>
@@ -30929,12 +31044,12 @@
     <row r="8">
       <c r="A8" s="23" t="inlineStr">
         <is>
-          <t>DHAN-34126100671709+23126100663009+23126100663109+321261006600309+321261006600609+321261006600809+23126100663309+221261006573809+221261006574009+23126100663509+23126100663709+23126100663809+34126100672309+221261006576409+221261006576709</t>
+          <t>DHAN-321261006605709</t>
         </is>
       </c>
       <c r="B8" s="23" t="inlineStr">
         <is>
-          <t>SATIN</t>
+          <t>KRISHNADEF</t>
         </is>
       </c>
       <c r="C8" s="23" t="inlineStr">
@@ -30946,22 +31061,22 @@
         <v>46302</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>89.77</v>
+        <v>40</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>299.29</v>
+        <v>595.97</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>9.19</v>
+        <v>18.28</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>44.89</v>
+        <v>45.16</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>17.87</v>
+        <v>10.6</v>
       </c>
       <c r="K8" s="4" t="n">
         <v>14.75</v>
@@ -30970,7 +31085,7 @@
         <v>35.4</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>61.41</v>
+        <v>51.24</v>
       </c>
       <c r="N8" s="21">
         <f>SUM(E8:M8)</f>
@@ -30980,12 +31095,12 @@
     <row r="9">
       <c r="A9" s="23" t="inlineStr">
         <is>
-          <t>DHAN-34126100786209</t>
+          <t>DHAN-34126100671709+23126100663009+23126100663109+321261006600309+321261006600609+321261006600809+23126100663309+221261006573809+221261006574009+23126100663509+23126100663709+23126100663809+34126100672309+221261006576409+221261006576709</t>
         </is>
       </c>
       <c r="B9" s="23" t="inlineStr">
         <is>
-          <t>ARFIN</t>
+          <t>SATIN</t>
         </is>
       </c>
       <c r="C9" s="23" t="inlineStr">
@@ -30993,24 +31108,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D9" s="24" t="inlineStr"/>
+      <c r="D9" s="24" t="n">
+        <v>46302</v>
+      </c>
       <c r="E9" s="4" t="n">
-        <v>0</v>
+        <v>109.77</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>0</v>
+        <v>606.55</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0</v>
+        <v>18.63</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="I9" s="4" t="n">
-        <v>0</v>
+        <v>44.89</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>0</v>
+        <v>23.22</v>
       </c>
       <c r="K9" s="4" t="n">
         <v>14.75</v>
@@ -31019,7 +31136,7 @@
         <v>35.4</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>0</v>
+        <v>61.41</v>
       </c>
       <c r="N9" s="21">
         <f>SUM(E9:M9)</f>
@@ -31029,12 +31146,12 @@
     <row r="10">
       <c r="A10" s="23" t="inlineStr">
         <is>
-          <t>DHAN-34126100566209+321261005656309+34126100566409+321261005657009+23126100565509+23126100565609+34126100566609+34126100566709+221261005674009+321261005658809+221261005675209+23126100566009+321261005659709+34126100567409+221261005676309+34126100567709</t>
+          <t>DHAN-221261006571909+221261006572109+34126100671809+23126100663209+34126100672009+23126100663409+321261006601809+34126100672209+23126100663909+23126100664109+23126100664209+34126100672409+23126100664309+221261006577209+34126100672509</t>
         </is>
       </c>
       <c r="B10" s="23" t="inlineStr">
         <is>
-          <t>DPABHUSHAN</t>
+          <t>YUKEN</t>
         </is>
       </c>
       <c r="C10" s="23" t="inlineStr">
@@ -31042,33 +31159,35 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D10" s="24" t="inlineStr"/>
+      <c r="D10" s="24" t="n">
+        <v>46302</v>
+      </c>
       <c r="E10" s="4" t="n">
-        <v>0</v>
+        <v>109.91</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>149.73</v>
+        <v>599.3099999999999</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>4.6</v>
+        <v>18.4</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>0.15</v>
+        <v>0.6</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>22.46</v>
+        <v>44.95</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>0.85</v>
+        <v>23.2</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>0</v>
+        <v>35.4</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>0</v>
+        <v>51.25</v>
       </c>
       <c r="N10" s="21">
         <f>SUM(E10:M10)</f>
@@ -31078,12 +31197,12 @@
     <row r="11">
       <c r="A11" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261007626809+321261007628809+34126100785209+34126100785309+23126100782509+34126100785409+221261007628809+321261007630509+34126100785509+23126100782909+34126100785609+34126100785709+23126100783209+221261007631209+34126100785809+321261007631609+321261007632109</t>
+          <t>DHAN-34126100786209</t>
         </is>
       </c>
       <c r="B11" s="23" t="inlineStr">
         <is>
-          <t>GPTINFRA</t>
+          <t>ARFIN</t>
         </is>
       </c>
       <c r="C11" s="23" t="inlineStr">
@@ -31091,24 +31210,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D11" s="24" t="inlineStr"/>
+      <c r="D11" s="24" t="n">
+        <v>46303</v>
+      </c>
       <c r="E11" s="4" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>0</v>
+        <v>240.26</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>0</v>
+        <v>7.38</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>0</v>
+        <v>0.24</v>
       </c>
       <c r="I11" s="4" t="n">
-        <v>0</v>
+        <v>35.99</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>0</v>
+        <v>4.97</v>
       </c>
       <c r="K11" s="4" t="n">
         <v>14.75</v>
@@ -31117,7 +31238,7 @@
         <v>35.4</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>0</v>
+        <v>41.09</v>
       </c>
       <c r="N11" s="21">
         <f>SUM(E11:M11)</f>
@@ -31127,12 +31248,12 @@
     <row r="12">
       <c r="A12" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261007633409</t>
+          <t>DHAN-221261007626809+321261007628809+34126100785209+34126100785309+23126100782509+34126100785409+221261007628809+321261007630509+34126100785509+23126100782909+34126100785609+34126100785709+23126100783209+221261007631209+34126100785809+321261007631609+321261007632109</t>
         </is>
       </c>
       <c r="B12" s="23" t="inlineStr">
         <is>
-          <t>MOBIKWIK</t>
+          <t>GPTINFRA</t>
         </is>
       </c>
       <c r="C12" s="23" t="inlineStr">
@@ -31140,24 +31261,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D12" s="24" t="inlineStr"/>
+      <c r="D12" s="24" t="n">
+        <v>46303</v>
+      </c>
       <c r="E12" s="4" t="n">
-        <v>0</v>
+        <v>71.98999999999999</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>0</v>
+        <v>239.94</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0</v>
+        <v>7.37</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>0</v>
+        <v>0.24</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>0</v>
+        <v>35.99</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>0</v>
+        <v>14.33</v>
       </c>
       <c r="K12" s="4" t="n">
         <v>14.75</v>
@@ -31166,7 +31289,7 @@
         <v>35.4</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>0</v>
+        <v>49.24</v>
       </c>
       <c r="N12" s="21">
         <f>SUM(E12:M12)</f>
@@ -31176,12 +31299,12 @@
     <row r="13">
       <c r="A13" s="23" t="inlineStr">
         <is>
-          <t>DHAN-34126100785009+34126100785109+221261007627809+221261007628109+321261007629509+23126100782809+321261007629709+221261007629309+221261007629609+221261007629909+23126100783009</t>
+          <t>DHAN-321261007633409</t>
         </is>
       </c>
       <c r="B13" s="23" t="inlineStr">
         <is>
-          <t>PNGSREVA</t>
+          <t>MOBIKWIK</t>
         </is>
       </c>
       <c r="C13" s="23" t="inlineStr">
@@ -31189,24 +31312,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D13" s="24" t="inlineStr"/>
+      <c r="D13" s="24" t="n">
+        <v>46303</v>
+      </c>
       <c r="E13" s="4" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>0</v>
+        <v>240.59</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0</v>
+        <v>7.39</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>0</v>
+        <v>0.24</v>
       </c>
       <c r="I13" s="4" t="n">
-        <v>0</v>
+        <v>36.09</v>
       </c>
       <c r="J13" s="4" t="n">
-        <v>0</v>
+        <v>4.97</v>
       </c>
       <c r="K13" s="4" t="n">
         <v>14.75</v>
@@ -31215,7 +31340,7 @@
         <v>35.4</v>
       </c>
       <c r="M13" s="4" t="n">
-        <v>0</v>
+        <v>50.25</v>
       </c>
       <c r="N13" s="21">
         <f>SUM(E13:M13)</f>
@@ -31225,12 +31350,12 @@
     <row r="14">
       <c r="A14" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261006571909+221261006572109+34126100671809+23126100663209+34126100672009+23126100663409+321261006601809+34126100672209+23126100663909+23126100664109+23126100664209+34126100672409+23126100664309+221261006577209+34126100672509</t>
+          <t>DHAN-34126100785009+34126100785109+221261007627809+221261007628109+321261007629509+23126100782809+321261007629709+221261007629309+221261007629609+221261007629909+23126100783009</t>
         </is>
       </c>
       <c r="B14" s="23" t="inlineStr">
         <is>
-          <t>YUKEN</t>
+          <t>PNGSREVA</t>
         </is>
       </c>
       <c r="C14" s="23" t="inlineStr">
@@ -31238,24 +31363,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D14" s="24" t="inlineStr"/>
+      <c r="D14" s="24" t="n">
+        <v>46303</v>
+      </c>
       <c r="E14" s="4" t="n">
-        <v>89.91</v>
+        <v>71.87</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>299.69</v>
+        <v>239.52</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>9.199999999999999</v>
+        <v>7.35</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>0.3</v>
+        <v>0.24</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>44.95</v>
+        <v>35.93</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>17.89</v>
+        <v>14.3</v>
       </c>
       <c r="K14" s="4" t="n">
         <v>14.75</v>
@@ -31264,7 +31391,7 @@
         <v>35.4</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>51.25</v>
+        <v>40.96</v>
       </c>
       <c r="N14" s="21">
         <f>SUM(E14:M14)</f>
@@ -31272,54 +31399,152 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126100860109+221261008541409+34126100865109+34126100865209+23126100860209+321261008684009+221261008543809+34126100865509+34126100865709+321261008684809+321261008685109+321261008685409+34126100865909+34126100866009+221261008545809+221261008545909+34126100866109+23126100860509</t>
+        </is>
+      </c>
+      <c r="B15" s="23" t="inlineStr">
+        <is>
+          <t>KOTIC</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D15" s="24" t="inlineStr"/>
+      <c r="E15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="21">
+        <f>SUM(E15:M15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261008541309+221261008541509+321261008683209+221261008542109+34126100865309+34126100865409+221261008543409+221261008543909+221261008544309+34126100865609+221261008545009+23126100860309+34126100865809+23126100860409</t>
+        </is>
+      </c>
+      <c r="B16" s="23" t="inlineStr">
+        <is>
+          <t>PNGSREVA</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D16" s="24" t="inlineStr"/>
+      <c r="E16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="21">
+        <f>SUM(E16:M16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E15" s="32">
-        <f>SUM(E4:E14)</f>
-        <v/>
-      </c>
-      <c r="F15" s="32">
-        <f>SUM(F4:F14)</f>
-        <v/>
-      </c>
-      <c r="G15" s="32">
-        <f>SUM(G4:G14)</f>
-        <v/>
-      </c>
-      <c r="H15" s="32">
-        <f>SUM(H4:H14)</f>
-        <v/>
-      </c>
-      <c r="I15" s="32">
-        <f>SUM(I4:I14)</f>
-        <v/>
-      </c>
-      <c r="J15" s="32">
-        <f>SUM(J4:J14)</f>
-        <v/>
-      </c>
-      <c r="K15" s="32">
-        <f>SUM(K4:K14)</f>
-        <v/>
-      </c>
-      <c r="L15" s="32">
-        <f>SUM(L4:L14)</f>
-        <v/>
-      </c>
-      <c r="M15" s="32">
-        <f>SUM(M4:M14)</f>
-        <v/>
-      </c>
-      <c r="N15" s="32">
-        <f>SUM(N4:N14)</f>
+      <c r="E17" s="32">
+        <f>SUM(E4:E16)</f>
+        <v/>
+      </c>
+      <c r="F17" s="32">
+        <f>SUM(F4:F16)</f>
+        <v/>
+      </c>
+      <c r="G17" s="32">
+        <f>SUM(G4:G16)</f>
+        <v/>
+      </c>
+      <c r="H17" s="32">
+        <f>SUM(H4:H16)</f>
+        <v/>
+      </c>
+      <c r="I17" s="32">
+        <f>SUM(I4:I16)</f>
+        <v/>
+      </c>
+      <c r="J17" s="32">
+        <f>SUM(J4:J16)</f>
+        <v/>
+      </c>
+      <c r="K17" s="32">
+        <f>SUM(K4:K16)</f>
+        <v/>
+      </c>
+      <c r="L17" s="32">
+        <f>SUM(L4:L16)</f>
+        <v/>
+      </c>
+      <c r="M17" s="32">
+        <f>SUM(M4:M16)</f>
+        <v/>
+      </c>
+      <c r="N17" s="32">
+        <f>SUM(N4:N16)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:N14"/>
+  <autoFilter ref="A3:N16"/>
   <mergeCells count="2">
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>

</xml_diff>

<commit_message>
Data update — 2026-10-09 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_oct2026.xlsx
+++ b/results/strategy_pnl_oct2026.xlsx
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trade Log'!$A$3:$O$503</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1214,7 +1214,7 @@
         <v/>
       </c>
       <c r="K6" s="4" t="n">
-        <v>900.61</v>
+        <v>959.4400000000001</v>
       </c>
       <c r="L6" s="21">
         <f>IF(OR($B6="",$I6=""),"",$I6-IF($K6="",0,$K6))</f>
@@ -1274,7 +1274,7 @@
         <v/>
       </c>
       <c r="K7" s="4" t="n">
-        <v>786.51</v>
+        <v>821.6799999999999</v>
       </c>
       <c r="L7" s="21">
         <f>IF(OR($B7="",$I7=""),"",$I7-IF($K7="",0,$K7))</f>
@@ -1334,7 +1334,7 @@
         <v/>
       </c>
       <c r="K8" s="4" t="n">
-        <v>812</v>
+        <v>832.9</v>
       </c>
       <c r="L8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($K8="",0,$K8))</f>
@@ -1394,7 +1394,7 @@
         <v/>
       </c>
       <c r="K9" s="4" t="n">
-        <v>915.22</v>
+        <v>973.89</v>
       </c>
       <c r="L9" s="21">
         <f>IF(OR($B9="",$I9=""),"",$I9-IF($K9="",0,$K9))</f>
@@ -1454,7 +1454,7 @@
         <v/>
       </c>
       <c r="K10" s="4" t="n">
-        <v>897.77</v>
+        <v>946.72</v>
       </c>
       <c r="L10" s="21">
         <f>IF(OR($B10="",$I10=""),"",$I10-IF($K10="",0,$K10))</f>
@@ -1514,7 +1514,7 @@
         <v/>
       </c>
       <c r="K11" s="4" t="n">
-        <v>400.07</v>
+        <v>671.91</v>
       </c>
       <c r="L11" s="21">
         <f>IF(OR($B11="",$I11=""),"",$I11-IF($K11="",0,$K11))</f>
@@ -1574,7 +1574,7 @@
         <v/>
       </c>
       <c r="K12" s="4" t="n">
-        <v>469.24</v>
+        <v>733.1900000000001</v>
       </c>
       <c r="L12" s="21">
         <f>IF(OR($B12="",$I12=""),"",$I12-IF($K12="",0,$K12))</f>
@@ -1634,7 +1634,7 @@
         <v/>
       </c>
       <c r="K13" s="4" t="n">
-        <v>409.68</v>
+        <v>664.04</v>
       </c>
       <c r="L13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($K13="",0,$K13))</f>
@@ -1694,7 +1694,7 @@
         <v/>
       </c>
       <c r="K14" s="4" t="n">
-        <v>460.32</v>
+        <v>664.58</v>
       </c>
       <c r="L14" s="21">
         <f>IF(OR($B14="",$I14=""),"",$I14-IF($K14="",0,$K14))</f>
@@ -1717,12 +1717,12 @@
     <row r="15">
       <c r="A15" s="23" t="inlineStr">
         <is>
-          <t>DHAN-23126100860109+221261008541409+34126100865109+34126100865209+23126100860209+321261008684009+221261008543809+34126100865509+34126100865709+321261008684809+321261008685109+321261008685409+34126100865909+34126100866009+221261008545809+221261008545909+34126100866109+23126100860509</t>
+          <t>DHAN-221261008541309+221261008541509+321261008683209+221261008542109+34126100865309+34126100865409+221261008543409+221261008543909+221261008544309+34126100865609+221261008545009+23126100860309+34126100865809+23126100860409</t>
         </is>
       </c>
       <c r="B15" s="23" t="inlineStr">
         <is>
-          <t>KOTIC</t>
+          <t>PNGSREVA</t>
         </is>
       </c>
       <c r="C15" s="23" t="inlineStr">
@@ -1734,13 +1734,17 @@
         <v>46303</v>
       </c>
       <c r="E15" s="25" t="n">
-        <v>157.0151</v>
+        <v>705.2641</v>
       </c>
       <c r="F15" s="26" t="n">
-        <v>858</v>
-      </c>
-      <c r="G15" s="24" t="inlineStr"/>
-      <c r="H15" s="25" t="inlineStr"/>
+        <v>213</v>
+      </c>
+      <c r="G15" s="24" t="n">
+        <v>46304</v>
+      </c>
+      <c r="H15" s="25" t="n">
+        <v>693.37</v>
+      </c>
       <c r="I15" s="21">
         <f>IF(OR($B15="",$H15=""),"",IF($C15="LONG",($H15-$E15)*$F15,($E15-$H15)*$F15))</f>
         <v/>
@@ -1750,7 +1754,7 @@
         <v/>
       </c>
       <c r="K15" s="4" t="n">
-        <v>14.75</v>
+        <v>78.05</v>
       </c>
       <c r="L15" s="21">
         <f>IF(OR($B15="",$I15=""),"",$I15-IF($K15="",0,$K15))</f>
@@ -1766,19 +1770,19 @@
       </c>
       <c r="O15" s="23" t="inlineStr">
         <is>
-          <t>5-10</t>
+          <t>10-15</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261008541309+221261008541509+321261008683209+221261008542109+34126100865309+34126100865409+221261008543409+221261008543909+221261008544309+34126100865609+221261008545009+23126100860309+34126100865809+23126100860409</t>
+          <t>DHAN-231261009113209+231261009113709+231261009113909+321261009657809+321261009658409+321261009658709+231261009115309+321261009659409+321261009660109+231261009116109+231261009116309+231261009116509+231261009117109</t>
         </is>
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>PNGSREVA</t>
+          <t>INOXGREEN</t>
         </is>
       </c>
       <c r="C16" s="23" t="inlineStr">
@@ -1787,13 +1791,13 @@
         </is>
       </c>
       <c r="D16" s="24" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E16" s="25" t="n">
-        <v>705.2641</v>
+        <v>129.4349</v>
       </c>
       <c r="F16" s="26" t="n">
-        <v>213</v>
+        <v>1547</v>
       </c>
       <c r="G16" s="24" t="inlineStr"/>
       <c r="H16" s="25" t="inlineStr"/>
@@ -1806,7 +1810,7 @@
         <v/>
       </c>
       <c r="K16" s="4" t="n">
-        <v>14.75</v>
+        <v>50.15</v>
       </c>
       <c r="L16" s="21">
         <f>IF(OR($B16="",$I16=""),"",$I16-IF($K16="",0,$K16))</f>
@@ -1827,14 +1831,32 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="23" t="n"/>
-      <c r="B17" s="23" t="n"/>
-      <c r="C17" s="23" t="n"/>
-      <c r="D17" s="24" t="n"/>
-      <c r="E17" s="25" t="n"/>
-      <c r="F17" s="26" t="n"/>
-      <c r="G17" s="24" t="n"/>
-      <c r="H17" s="25" t="n"/>
+      <c r="A17" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126100860109+221261008541409+34126100865109+34126100865209+23126100860209+321261008684009+221261008543809+34126100865509+34126100865709+321261008684809+321261008685109+321261008685409+34126100865909+34126100866009+221261008545809+221261008545909+34126100866109+23126100860509</t>
+        </is>
+      </c>
+      <c r="B17" s="23" t="inlineStr">
+        <is>
+          <t>KOTIC</t>
+        </is>
+      </c>
+      <c r="C17" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D17" s="24" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E17" s="25" t="n">
+        <v>157.0151</v>
+      </c>
+      <c r="F17" s="26" t="n">
+        <v>858</v>
+      </c>
+      <c r="G17" s="24" t="inlineStr"/>
+      <c r="H17" s="25" t="inlineStr"/>
       <c r="I17" s="21">
         <f>IF(OR($B17="",$H17=""),"",IF($C17="LONG",($H17-$E17)*$F17,($E17-$H17)*$F17))</f>
         <v/>
@@ -1843,7 +1865,9 @@
         <f>IF(OR($B17="",$I17="",$E17=0,$F17=0),"",$I17/($E17*$F17))</f>
         <v/>
       </c>
-      <c r="K17" s="4" t="n"/>
+      <c r="K17" s="4" t="n">
+        <v>175</v>
+      </c>
       <c r="L17" s="21">
         <f>IF(OR($B17="",$I17=""),"",$I17-IF($K17="",0,$K17))</f>
         <v/>
@@ -1856,17 +1880,39 @@
         <f>IF($B17="","",IF($H17="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O17" s="23" t="n"/>
+      <c r="O17" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="23" t="n"/>
-      <c r="B18" s="23" t="n"/>
-      <c r="C18" s="23" t="n"/>
-      <c r="D18" s="24" t="n"/>
-      <c r="E18" s="25" t="n"/>
-      <c r="F18" s="26" t="n"/>
-      <c r="G18" s="24" t="n"/>
-      <c r="H18" s="25" t="n"/>
+      <c r="A18" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261009656409+231261009113609+231261009114009+321261009657909+231261009114709+231261009115009+321261009659009+231261009115809+321261009660609+321261009660809+321261009661309+231261009117309+321261009662609+321261009663009+231261009117809+321261009663809+231261009118209</t>
+        </is>
+      </c>
+      <c r="B18" s="23" t="inlineStr">
+        <is>
+          <t>MMWL</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D18" s="24" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E18" s="25" t="n">
+        <v>20.9882</v>
+      </c>
+      <c r="F18" s="26" t="n">
+        <v>3589</v>
+      </c>
+      <c r="G18" s="24" t="inlineStr"/>
+      <c r="H18" s="25" t="inlineStr"/>
       <c r="I18" s="21">
         <f>IF(OR($B18="",$H18=""),"",IF($C18="LONG",($H18-$E18)*$F18,($E18-$H18)*$F18))</f>
         <v/>
@@ -1875,7 +1921,9 @@
         <f>IF(OR($B18="",$I18="",$E18=0,$F18=0),"",$I18/($E18*$F18))</f>
         <v/>
       </c>
-      <c r="K18" s="4" t="n"/>
+      <c r="K18" s="4" t="n">
+        <v>14.75</v>
+      </c>
       <c r="L18" s="21">
         <f>IF(OR($B18="",$I18=""),"",$I18-IF($K18="",0,$K18))</f>
         <v/>
@@ -1888,17 +1936,39 @@
         <f>IF($B18="","",IF($H18="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O18" s="23" t="n"/>
+      <c r="O18" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="23" t="n"/>
-      <c r="B19" s="23" t="n"/>
-      <c r="C19" s="23" t="n"/>
-      <c r="D19" s="24" t="n"/>
-      <c r="E19" s="25" t="n"/>
-      <c r="F19" s="26" t="n"/>
-      <c r="G19" s="24" t="n"/>
-      <c r="H19" s="25" t="n"/>
+      <c r="A19" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261009656509+321261009657209+231261009114209+231261009114409+231261009114609+321261009658609+321261009659109+321261009659509+231261009115709+321261009660509+231261009116209</t>
+        </is>
+      </c>
+      <c r="B19" s="23" t="inlineStr">
+        <is>
+          <t>RSYSTEMS</t>
+        </is>
+      </c>
+      <c r="C19" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D19" s="24" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E19" s="25" t="n">
+        <v>274.9019</v>
+      </c>
+      <c r="F19" s="26" t="n">
+        <v>727</v>
+      </c>
+      <c r="G19" s="24" t="inlineStr"/>
+      <c r="H19" s="25" t="inlineStr"/>
       <c r="I19" s="21">
         <f>IF(OR($B19="",$H19=""),"",IF($C19="LONG",($H19-$E19)*$F19,($E19-$H19)*$F19))</f>
         <v/>
@@ -1907,7 +1977,9 @@
         <f>IF(OR($B19="",$I19="",$E19=0,$F19=0),"",$I19/($E19*$F19))</f>
         <v/>
       </c>
-      <c r="K19" s="4" t="n"/>
+      <c r="K19" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L19" s="21">
         <f>IF(OR($B19="",$I19=""),"",$I19-IF($K19="",0,$K19))</f>
         <v/>
@@ -1920,17 +1992,39 @@
         <f>IF($B19="","",IF($H19="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O19" s="23" t="n"/>
+      <c r="O19" s="23" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="23" t="n"/>
-      <c r="B20" s="23" t="n"/>
-      <c r="C20" s="23" t="n"/>
-      <c r="D20" s="24" t="n"/>
-      <c r="E20" s="25" t="n"/>
-      <c r="F20" s="26" t="n"/>
-      <c r="G20" s="24" t="n"/>
-      <c r="H20" s="25" t="n"/>
+      <c r="A20" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-231261009113309+231261009113509+231261009114309+231261009114509+231261009114809+321261009658809+321261009659609+231261009115609+231261009116009+321261009660909+231261009116609+321261009661609+321261009662209+231261009117509+321261009662909+231261009117909</t>
+        </is>
+      </c>
+      <c r="B20" s="23" t="inlineStr">
+        <is>
+          <t>SAKSOFT</t>
+        </is>
+      </c>
+      <c r="C20" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D20" s="24" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E20" s="25" t="n">
+        <v>138.9161</v>
+      </c>
+      <c r="F20" s="26" t="n">
+        <v>1443</v>
+      </c>
+      <c r="G20" s="24" t="inlineStr"/>
+      <c r="H20" s="25" t="inlineStr"/>
       <c r="I20" s="21">
         <f>IF(OR($B20="",$H20=""),"",IF($C20="LONG",($H20-$E20)*$F20,($E20-$H20)*$F20))</f>
         <v/>
@@ -1939,7 +2033,9 @@
         <f>IF(OR($B20="",$I20="",$E20=0,$F20=0),"",$I20/($E20*$F20))</f>
         <v/>
       </c>
-      <c r="K20" s="4" t="n"/>
+      <c r="K20" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L20" s="21">
         <f>IF(OR($B20="",$I20=""),"",$I20-IF($K20="",0,$K20))</f>
         <v/>
@@ -1952,17 +2048,39 @@
         <f>IF($B20="","",IF($H20="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O20" s="23" t="n"/>
+      <c r="O20" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="23" t="n"/>
-      <c r="B21" s="23" t="n"/>
-      <c r="C21" s="23" t="n"/>
-      <c r="D21" s="24" t="n"/>
-      <c r="E21" s="25" t="n"/>
-      <c r="F21" s="26" t="n"/>
-      <c r="G21" s="24" t="n"/>
-      <c r="H21" s="25" t="n"/>
+      <c r="A21" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-231261009113409+321261009657109+321261009657509+321261009658009+231261009114909+231261009115109+231261009115209+231261009115409+321261009660209+321261009660409+321261009661009+231261009116709+321261009661709+321261009662109+321261009662509</t>
+        </is>
+      </c>
+      <c r="B21" s="23" t="inlineStr">
+        <is>
+          <t>SMCGLOBAL</t>
+        </is>
+      </c>
+      <c r="C21" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D21" s="24" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E21" s="25" t="n">
+        <v>115.2011</v>
+      </c>
+      <c r="F21" s="26" t="n">
+        <v>864</v>
+      </c>
+      <c r="G21" s="24" t="inlineStr"/>
+      <c r="H21" s="25" t="inlineStr"/>
       <c r="I21" s="21">
         <f>IF(OR($B21="",$H21=""),"",IF($C21="LONG",($H21-$E21)*$F21,($E21-$H21)*$F21))</f>
         <v/>
@@ -1971,7 +2089,9 @@
         <f>IF(OR($B21="",$I21="",$E21=0,$F21=0),"",$I21/($E21*$F21))</f>
         <v/>
       </c>
-      <c r="K21" s="4" t="n"/>
+      <c r="K21" s="4" t="n">
+        <v>14.75</v>
+      </c>
       <c r="L21" s="21">
         <f>IF(OR($B21="",$I21=""),"",$I21-IF($K21="",0,$K21))</f>
         <v/>
@@ -1984,17 +2104,39 @@
         <f>IF($B21="","",IF($H21="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O21" s="23" t="n"/>
+      <c r="O21" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="23" t="n"/>
-      <c r="B22" s="23" t="n"/>
-      <c r="C22" s="23" t="n"/>
-      <c r="D22" s="24" t="n"/>
-      <c r="E22" s="25" t="n"/>
-      <c r="F22" s="26" t="n"/>
-      <c r="G22" s="24" t="n"/>
-      <c r="H22" s="25" t="n"/>
+      <c r="A22" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261009656609+231261009113809+231261009114109+321261009658109+231261009115509+231261009116409+231261009116809+231261009117009+231261009117209+231261009117609+231261009117709+231261009118009+231261009118109</t>
+        </is>
+      </c>
+      <c r="B22" s="23" t="inlineStr">
+        <is>
+          <t>SUNCLAY</t>
+        </is>
+      </c>
+      <c r="C22" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D22" s="24" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E22" s="25" t="n">
+        <v>1228.0927</v>
+      </c>
+      <c r="F22" s="26" t="n">
+        <v>164</v>
+      </c>
+      <c r="G22" s="24" t="inlineStr"/>
+      <c r="H22" s="25" t="inlineStr"/>
       <c r="I22" s="21">
         <f>IF(OR($B22="",$H22=""),"",IF($C22="LONG",($H22-$E22)*$F22,($E22-$H22)*$F22))</f>
         <v/>
@@ -2003,7 +2145,9 @@
         <f>IF(OR($B22="",$I22="",$E22=0,$F22=0),"",$I22/($E22*$F22))</f>
         <v/>
       </c>
-      <c r="K22" s="4" t="n"/>
+      <c r="K22" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L22" s="21">
         <f>IF(OR($B22="",$I22=""),"",$I22-IF($K22="",0,$K22))</f>
         <v/>
@@ -2016,7 +2160,11 @@
         <f>IF($B22="","",IF($H22="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O22" s="23" t="n"/>
+      <c r="O22" s="23" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="23" t="n"/>
@@ -30085,7 +30233,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30341,7 +30489,7 @@
     <row r="8">
       <c r="A8" s="27" t="inlineStr">
         <is>
-          <t>KOTIC</t>
+          <t>INOXGREEN</t>
         </is>
       </c>
       <c r="B8" s="20">
@@ -30384,7 +30532,7 @@
     <row r="9">
       <c r="A9" s="27" t="inlineStr">
         <is>
-          <t>KRISHNADEF</t>
+          <t>KOTIC</t>
         </is>
       </c>
       <c r="B9" s="20">
@@ -30427,7 +30575,7 @@
     <row r="10">
       <c r="A10" s="27" t="inlineStr">
         <is>
-          <t>MOBIKWIK</t>
+          <t>KRISHNADEF</t>
         </is>
       </c>
       <c r="B10" s="20">
@@ -30470,7 +30618,7 @@
     <row r="11">
       <c r="A11" s="27" t="inlineStr">
         <is>
-          <t>PNGSREVA</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="B11" s="20">
@@ -30513,7 +30661,7 @@
     <row r="12">
       <c r="A12" s="27" t="inlineStr">
         <is>
-          <t>SATIN</t>
+          <t>MOBIKWIK</t>
         </is>
       </c>
       <c r="B12" s="20">
@@ -30556,7 +30704,7 @@
     <row r="13">
       <c r="A13" s="27" t="inlineStr">
         <is>
-          <t>SGFIN</t>
+          <t>PNGSREVA</t>
         </is>
       </c>
       <c r="B13" s="20">
@@ -30599,7 +30747,7 @@
     <row r="14">
       <c r="A14" s="27" t="inlineStr">
         <is>
-          <t>SMCGLOBAL</t>
+          <t>RSYSTEMS</t>
         </is>
       </c>
       <c r="B14" s="20">
@@ -30642,78 +30790,293 @@
     <row r="15">
       <c r="A15" s="27" t="inlineStr">
         <is>
+          <t>SAKSOFT</t>
+        </is>
+      </c>
+      <c r="B15" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A15)</f>
+        <v/>
+      </c>
+      <c r="C15" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A15,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D15" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A15,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E15" s="22">
+        <f>IFERROR($C15/$B15,"")</f>
+        <v/>
+      </c>
+      <c r="F15" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A15,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G15" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A15,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H15" s="21">
+        <f>IFERROR($G15/$B15,"")</f>
+        <v/>
+      </c>
+      <c r="I15" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A15),"")</f>
+        <v/>
+      </c>
+      <c r="J15" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A15),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="27" t="inlineStr">
+        <is>
+          <t>SATIN</t>
+        </is>
+      </c>
+      <c r="B16" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A16)</f>
+        <v/>
+      </c>
+      <c r="C16" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A16,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D16" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A16,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E16" s="22">
+        <f>IFERROR($C16/$B16,"")</f>
+        <v/>
+      </c>
+      <c r="F16" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A16,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G16" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A16,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H16" s="21">
+        <f>IFERROR($G16/$B16,"")</f>
+        <v/>
+      </c>
+      <c r="I16" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A16),"")</f>
+        <v/>
+      </c>
+      <c r="J16" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A16),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="27" t="inlineStr">
+        <is>
+          <t>SGFIN</t>
+        </is>
+      </c>
+      <c r="B17" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A17)</f>
+        <v/>
+      </c>
+      <c r="C17" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A17,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D17" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A17,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E17" s="22">
+        <f>IFERROR($C17/$B17,"")</f>
+        <v/>
+      </c>
+      <c r="F17" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A17,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G17" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A17,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H17" s="21">
+        <f>IFERROR($G17/$B17,"")</f>
+        <v/>
+      </c>
+      <c r="I17" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A17),"")</f>
+        <v/>
+      </c>
+      <c r="J17" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A17),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="27" t="inlineStr">
+        <is>
+          <t>SMCGLOBAL</t>
+        </is>
+      </c>
+      <c r="B18" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A18)</f>
+        <v/>
+      </c>
+      <c r="C18" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A18,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D18" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A18,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E18" s="22">
+        <f>IFERROR($C18/$B18,"")</f>
+        <v/>
+      </c>
+      <c r="F18" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A18,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G18" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A18,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H18" s="21">
+        <f>IFERROR($G18/$B18,"")</f>
+        <v/>
+      </c>
+      <c r="I18" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A18),"")</f>
+        <v/>
+      </c>
+      <c r="J18" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A18),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="27" t="inlineStr">
+        <is>
+          <t>SUNCLAY</t>
+        </is>
+      </c>
+      <c r="B19" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A19)</f>
+        <v/>
+      </c>
+      <c r="C19" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A19,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D19" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A19,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E19" s="22">
+        <f>IFERROR($C19/$B19,"")</f>
+        <v/>
+      </c>
+      <c r="F19" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A19,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G19" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A19,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H19" s="21">
+        <f>IFERROR($G19/$B19,"")</f>
+        <v/>
+      </c>
+      <c r="I19" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A19),"")</f>
+        <v/>
+      </c>
+      <c r="J19" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A19),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="27" t="inlineStr">
+        <is>
           <t>YUKEN</t>
         </is>
       </c>
-      <c r="B15" s="20">
-        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A15)</f>
-        <v/>
-      </c>
-      <c r="C15" s="20">
-        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A15,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
-        <v/>
-      </c>
-      <c r="D15" s="20">
-        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A15,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
-        <v/>
-      </c>
-      <c r="E15" s="22">
-        <f>IFERROR($C15/$B15,"")</f>
-        <v/>
-      </c>
-      <c r="F15" s="21">
-        <f>SUMIF('Trade Log'!$B$4:$B$503,$A15,'Trade Log'!$I$4:$I$503)</f>
-        <v/>
-      </c>
-      <c r="G15" s="21">
-        <f>SUMIF('Trade Log'!$B$4:$B$503,$A15,'Trade Log'!$L$4:$L$503)</f>
-        <v/>
-      </c>
-      <c r="H15" s="21">
-        <f>IFERROR($G15/$B15,"")</f>
-        <v/>
-      </c>
-      <c r="I15" s="21">
-        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A15),"")</f>
-        <v/>
-      </c>
-      <c r="J15" s="21">
-        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A15),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="B20" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A20)</f>
+        <v/>
+      </c>
+      <c r="C20" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A20,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D20" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A20,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E20" s="22">
+        <f>IFERROR($C20/$B20,"")</f>
+        <v/>
+      </c>
+      <c r="F20" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A20,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G20" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A20,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H20" s="21">
+        <f>IFERROR($G20/$B20,"")</f>
+        <v/>
+      </c>
+      <c r="I20" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A20),"")</f>
+        <v/>
+      </c>
+      <c r="J20" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A20),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B16" s="30">
-        <f>SUM(B4:B15)</f>
-        <v/>
-      </c>
-      <c r="C16" s="30">
-        <f>SUM(C4:C15)</f>
-        <v/>
-      </c>
-      <c r="D16" s="30">
-        <f>SUM(D4:D15)</f>
-        <v/>
-      </c>
-      <c r="E16" s="31">
-        <f>IFERROR(C16/B16,"")</f>
-        <v/>
-      </c>
-      <c r="F16" s="32">
-        <f>SUM(F4:F15)</f>
-        <v/>
-      </c>
-      <c r="G16" s="32">
-        <f>SUM(G4:G15)</f>
-        <v/>
-      </c>
-      <c r="H16" s="32">
-        <f>IFERROR(G16/B16,"")</f>
+      <c r="B21" s="30">
+        <f>SUM(B4:B20)</f>
+        <v/>
+      </c>
+      <c r="C21" s="30">
+        <f>SUM(C4:C20)</f>
+        <v/>
+      </c>
+      <c r="D21" s="30">
+        <f>SUM(D4:D20)</f>
+        <v/>
+      </c>
+      <c r="E21" s="31">
+        <f>IFERROR(C21/B21,"")</f>
+        <v/>
+      </c>
+      <c r="F21" s="32">
+        <f>SUM(F4:F20)</f>
+        <v/>
+      </c>
+      <c r="G21" s="32">
+        <f>SUM(G4:G20)</f>
+        <v/>
+      </c>
+      <c r="H21" s="32">
+        <f>IFERROR(G21/B21,"")</f>
         <v/>
       </c>
     </row>
@@ -30732,7 +31095,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -30983,7 +31346,7 @@
         <v>35.4</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>61.58</v>
+        <v>120.42</v>
       </c>
       <c r="N6" s="21">
         <f>SUM(E6:M6)</f>
@@ -31034,7 +31397,7 @@
         <v>35.4</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>36.82</v>
+        <v>72</v>
       </c>
       <c r="N7" s="21">
         <f>SUM(E7:M7)</f>
@@ -31085,7 +31448,7 @@
         <v>35.4</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>51.24</v>
+        <v>72.14</v>
       </c>
       <c r="N8" s="21">
         <f>SUM(E8:M8)</f>
@@ -31136,7 +31499,7 @@
         <v>35.4</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>61.41</v>
+        <v>120.08</v>
       </c>
       <c r="N9" s="21">
         <f>SUM(E9:M9)</f>
@@ -31187,7 +31550,7 @@
         <v>35.4</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>51.25</v>
+        <v>100.2</v>
       </c>
       <c r="N10" s="21">
         <f>SUM(E10:M10)</f>
@@ -31214,22 +31577,22 @@
         <v>46303</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>240.26</v>
+        <v>480.43</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>7.38</v>
+        <v>14.75</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>0.24</v>
+        <v>0.48</v>
       </c>
       <c r="I11" s="4" t="n">
         <v>35.99</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>4.97</v>
+        <v>9.94</v>
       </c>
       <c r="K11" s="4" t="n">
         <v>14.75</v>
@@ -31238,7 +31601,7 @@
         <v>35.4</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>41.09</v>
+        <v>40.17</v>
       </c>
       <c r="N11" s="21">
         <f>SUM(E11:M11)</f>
@@ -31265,22 +31628,22 @@
         <v>46303</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>71.98999999999999</v>
+        <v>91.98999999999999</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>239.94</v>
+        <v>472.68</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>7.37</v>
+        <v>14.51</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>0.24</v>
+        <v>0.47</v>
       </c>
       <c r="I12" s="4" t="n">
         <v>35.99</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>14.33</v>
+        <v>19.26</v>
       </c>
       <c r="K12" s="4" t="n">
         <v>14.75</v>
@@ -31289,7 +31652,7 @@
         <v>35.4</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>49.24</v>
+        <v>48.14</v>
       </c>
       <c r="N12" s="21">
         <f>SUM(E12:M12)</f>
@@ -31316,22 +31679,22 @@
         <v>46303</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>240.59</v>
+        <v>464.16</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>7.39</v>
+        <v>14.25</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>0.24</v>
+        <v>0.46</v>
       </c>
       <c r="I13" s="4" t="n">
         <v>36.09</v>
       </c>
       <c r="J13" s="4" t="n">
-        <v>4.97</v>
+        <v>9.85</v>
       </c>
       <c r="K13" s="4" t="n">
         <v>14.75</v>
@@ -31340,7 +31703,7 @@
         <v>35.4</v>
       </c>
       <c r="M13" s="4" t="n">
-        <v>50.25</v>
+        <v>49.08</v>
       </c>
       <c r="N13" s="21">
         <f>SUM(E13:M13)</f>
@@ -31367,22 +31730,22 @@
         <v>46303</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>71.87</v>
+        <v>111.87</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>239.52</v>
+        <v>388.32</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>7.35</v>
+        <v>14.87</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>0.24</v>
+        <v>0.49</v>
       </c>
       <c r="I14" s="4" t="n">
         <v>35.93</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>14.3</v>
+        <v>22.9</v>
       </c>
       <c r="K14" s="4" t="n">
         <v>14.75</v>
@@ -31391,7 +31754,7 @@
         <v>35.4</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>40.96</v>
+        <v>40.04</v>
       </c>
       <c r="N14" s="21">
         <f>SUM(E14:M14)</f>
@@ -31401,12 +31764,12 @@
     <row r="15">
       <c r="A15" s="23" t="inlineStr">
         <is>
-          <t>DHAN-23126100860109+221261008541409+34126100865109+34126100865209+23126100860209+321261008684009+221261008543809+34126100865509+34126100865709+321261008684809+321261008685109+321261008685409+34126100865909+34126100866009+221261008545809+221261008545909+34126100866109+23126100860509</t>
+          <t>DHAN-221261008541309+221261008541509+321261008683209+221261008542109+34126100865309+34126100865409+221261008543409+221261008543909+221261008544309+34126100865609+221261008545009+23126100860309+34126100865809+23126100860409</t>
         </is>
       </c>
       <c r="B15" s="23" t="inlineStr">
         <is>
-          <t>KOTIC</t>
+          <t>PNGSREVA</t>
         </is>
       </c>
       <c r="C15" s="23" t="inlineStr">
@@ -31414,24 +31777,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D15" s="24" t="inlineStr"/>
+      <c r="D15" s="24" t="n">
+        <v>46304</v>
+      </c>
       <c r="E15" s="4" t="n">
-        <v>0</v>
+        <v>45.06</v>
       </c>
       <c r="F15" s="4" t="n">
         <v>0</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0</v>
+        <v>4.61</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="I15" s="4" t="n">
-        <v>0</v>
+        <v>4.51</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>0</v>
+        <v>8.970000000000001</v>
       </c>
       <c r="K15" s="4" t="n">
         <v>14.75</v>
@@ -31450,12 +31815,12 @@
     <row r="16">
       <c r="A16" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261008541309+221261008541509+321261008683209+221261008542109+34126100865309+34126100865409+221261008543409+221261008543909+221261008544309+34126100865609+221261008545009+23126100860309+34126100865809+23126100860409</t>
+          <t>DHAN-231261009113209+231261009113709+231261009113909+321261009657809+321261009658409+321261009658709+231261009115309+321261009659409+321261009660109+231261009116109+231261009116309+231261009116509+231261009117109</t>
         </is>
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>PNGSREVA</t>
+          <t>INOXGREEN</t>
         </is>
       </c>
       <c r="C16" s="23" t="inlineStr">
@@ -31486,7 +31851,7 @@
         <v>14.75</v>
       </c>
       <c r="L16" s="4" t="n">
-        <v>0</v>
+        <v>35.4</v>
       </c>
       <c r="M16" s="4" t="n">
         <v>0</v>
@@ -31497,54 +31862,348 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126100860109+221261008541409+34126100865109+34126100865209+23126100860209+321261008684009+221261008543809+34126100865509+34126100865709+321261008684809+321261008685109+321261008685409+34126100865909+34126100866009+221261008545809+221261008545909+34126100866109+23126100860509</t>
+        </is>
+      </c>
+      <c r="B17" s="23" t="inlineStr">
+        <is>
+          <t>KOTIC</t>
+        </is>
+      </c>
+      <c r="C17" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D17" s="24" t="inlineStr"/>
+      <c r="E17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>134.72</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>4.14</v>
+      </c>
+      <c r="H17" s="4" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="I17" s="4" t="n">
+        <v>20.49</v>
+      </c>
+      <c r="J17" s="4" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="K17" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" s="21">
+        <f>SUM(E17:M17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261009656409+231261009113609+231261009114009+321261009657909+231261009114709+231261009115009+321261009659009+231261009115809+321261009660609+321261009660809+321261009661309+231261009117309+321261009662609+321261009663009+231261009117809+321261009663809+231261009118209</t>
+        </is>
+      </c>
+      <c r="B18" s="23" t="inlineStr">
+        <is>
+          <t>MMWL</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D18" s="24" t="inlineStr"/>
+      <c r="E18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" s="21">
+        <f>SUM(E18:M18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261009656509+321261009657209+231261009114209+231261009114409+231261009114609+321261009658609+321261009659109+321261009659509+231261009115709+321261009660509+231261009116209</t>
+        </is>
+      </c>
+      <c r="B19" s="23" t="inlineStr">
+        <is>
+          <t>RSYSTEMS</t>
+        </is>
+      </c>
+      <c r="C19" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D19" s="24" t="inlineStr"/>
+      <c r="E19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L19" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" s="21">
+        <f>SUM(E19:M19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-231261009113309+231261009113509+231261009114309+231261009114509+231261009114809+321261009658809+321261009659609+231261009115609+231261009116009+321261009660909+231261009116609+321261009661609+321261009662209+231261009117509+321261009662909+231261009117909</t>
+        </is>
+      </c>
+      <c r="B20" s="23" t="inlineStr">
+        <is>
+          <t>SAKSOFT</t>
+        </is>
+      </c>
+      <c r="C20" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D20" s="24" t="inlineStr"/>
+      <c r="E20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L20" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" s="21">
+        <f>SUM(E20:M20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-231261009113409+321261009657109+321261009657509+321261009658009+231261009114909+231261009115109+231261009115209+231261009115409+321261009660209+321261009660409+321261009661009+231261009116709+321261009661709+321261009662109+321261009662509</t>
+        </is>
+      </c>
+      <c r="B21" s="23" t="inlineStr">
+        <is>
+          <t>SMCGLOBAL</t>
+        </is>
+      </c>
+      <c r="C21" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D21" s="24" t="inlineStr"/>
+      <c r="E21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" s="21">
+        <f>SUM(E21:M21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261009656609+231261009113809+231261009114109+321261009658109+231261009115509+231261009116409+231261009116809+231261009117009+231261009117209+231261009117609+231261009117709+231261009118009+231261009118109</t>
+        </is>
+      </c>
+      <c r="B22" s="23" t="inlineStr">
+        <is>
+          <t>SUNCLAY</t>
+        </is>
+      </c>
+      <c r="C22" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D22" s="24" t="inlineStr"/>
+      <c r="E22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L22" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" s="21">
+        <f>SUM(E22:M22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E17" s="32">
-        <f>SUM(E4:E16)</f>
-        <v/>
-      </c>
-      <c r="F17" s="32">
-        <f>SUM(F4:F16)</f>
-        <v/>
-      </c>
-      <c r="G17" s="32">
-        <f>SUM(G4:G16)</f>
-        <v/>
-      </c>
-      <c r="H17" s="32">
-        <f>SUM(H4:H16)</f>
-        <v/>
-      </c>
-      <c r="I17" s="32">
-        <f>SUM(I4:I16)</f>
-        <v/>
-      </c>
-      <c r="J17" s="32">
-        <f>SUM(J4:J16)</f>
-        <v/>
-      </c>
-      <c r="K17" s="32">
-        <f>SUM(K4:K16)</f>
-        <v/>
-      </c>
-      <c r="L17" s="32">
-        <f>SUM(L4:L16)</f>
-        <v/>
-      </c>
-      <c r="M17" s="32">
-        <f>SUM(M4:M16)</f>
-        <v/>
-      </c>
-      <c r="N17" s="32">
-        <f>SUM(N4:N16)</f>
+      <c r="E23" s="32">
+        <f>SUM(E4:E22)</f>
+        <v/>
+      </c>
+      <c r="F23" s="32">
+        <f>SUM(F4:F22)</f>
+        <v/>
+      </c>
+      <c r="G23" s="32">
+        <f>SUM(G4:G22)</f>
+        <v/>
+      </c>
+      <c r="H23" s="32">
+        <f>SUM(H4:H22)</f>
+        <v/>
+      </c>
+      <c r="I23" s="32">
+        <f>SUM(I4:I22)</f>
+        <v/>
+      </c>
+      <c r="J23" s="32">
+        <f>SUM(J4:J22)</f>
+        <v/>
+      </c>
+      <c r="K23" s="32">
+        <f>SUM(K4:K22)</f>
+        <v/>
+      </c>
+      <c r="L23" s="32">
+        <f>SUM(L4:L22)</f>
+        <v/>
+      </c>
+      <c r="M23" s="32">
+        <f>SUM(M4:M22)</f>
+        <v/>
+      </c>
+      <c r="N23" s="32">
+        <f>SUM(N4:N22)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:N16"/>
+  <autoFilter ref="A3:N22"/>
   <mergeCells count="2">
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>

</xml_diff>

<commit_message>
Data update — 2026-10-12 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_oct2026.xlsx
+++ b/results/strategy_pnl_oct2026.xlsx
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trade Log'!$A$3:$O$503</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$27</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1214,7 +1214,7 @@
         <v/>
       </c>
       <c r="K6" s="4" t="n">
-        <v>959.4400000000001</v>
+        <v>962.8200000000001</v>
       </c>
       <c r="L6" s="21">
         <f>IF(OR($B6="",$I6=""),"",$I6-IF($K6="",0,$K6))</f>
@@ -1274,7 +1274,7 @@
         <v/>
       </c>
       <c r="K7" s="4" t="n">
-        <v>821.6799999999999</v>
+        <v>823.7</v>
       </c>
       <c r="L7" s="21">
         <f>IF(OR($B7="",$I7=""),"",$I7-IF($K7="",0,$K7))</f>
@@ -1334,7 +1334,7 @@
         <v/>
       </c>
       <c r="K8" s="4" t="n">
-        <v>832.9</v>
+        <v>834.92</v>
       </c>
       <c r="L8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($K8="",0,$K8))</f>
@@ -1394,7 +1394,7 @@
         <v/>
       </c>
       <c r="K9" s="4" t="n">
-        <v>973.89</v>
+        <v>977.26</v>
       </c>
       <c r="L9" s="21">
         <f>IF(OR($B9="",$I9=""),"",$I9-IF($K9="",0,$K9))</f>
@@ -1454,7 +1454,7 @@
         <v/>
       </c>
       <c r="K10" s="4" t="n">
-        <v>946.72</v>
+        <v>949.53</v>
       </c>
       <c r="L10" s="21">
         <f>IF(OR($B10="",$I10=""),"",$I10-IF($K10="",0,$K10))</f>
@@ -1514,7 +1514,7 @@
         <v/>
       </c>
       <c r="K11" s="4" t="n">
-        <v>671.91</v>
+        <v>673.03</v>
       </c>
       <c r="L11" s="21">
         <f>IF(OR($B11="",$I11=""),"",$I11-IF($K11="",0,$K11))</f>
@@ -1574,7 +1574,7 @@
         <v/>
       </c>
       <c r="K12" s="4" t="n">
-        <v>733.1900000000001</v>
+        <v>734.54</v>
       </c>
       <c r="L12" s="21">
         <f>IF(OR($B12="",$I12=""),"",$I12-IF($K12="",0,$K12))</f>
@@ -1634,7 +1634,7 @@
         <v/>
       </c>
       <c r="K13" s="4" t="n">
-        <v>664.04</v>
+        <v>644.73</v>
       </c>
       <c r="L13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($K13="",0,$K13))</f>
@@ -1694,7 +1694,7 @@
         <v/>
       </c>
       <c r="K14" s="4" t="n">
-        <v>664.58</v>
+        <v>665.7</v>
       </c>
       <c r="L14" s="21">
         <f>IF(OR($B14="",$I14=""),"",$I14-IF($K14="",0,$K14))</f>
@@ -1754,7 +1754,7 @@
         <v/>
       </c>
       <c r="K15" s="4" t="n">
-        <v>78.05</v>
+        <v>254.86</v>
       </c>
       <c r="L15" s="21">
         <f>IF(OR($B15="",$I15=""),"",$I15-IF($K15="",0,$K15))</f>
@@ -1799,8 +1799,12 @@
       <c r="F16" s="26" t="n">
         <v>1547</v>
       </c>
-      <c r="G16" s="24" t="inlineStr"/>
-      <c r="H16" s="25" t="inlineStr"/>
+      <c r="G16" s="24" t="n">
+        <v>46307</v>
+      </c>
+      <c r="H16" s="25" t="n">
+        <v>121.63</v>
+      </c>
       <c r="I16" s="21">
         <f>IF(OR($B16="",$H16=""),"",IF($C16="LONG",($H16-$E16)*$F16,($E16-$H16)*$F16))</f>
         <v/>
@@ -1810,7 +1814,7 @@
         <v/>
       </c>
       <c r="K16" s="4" t="n">
-        <v>50.15</v>
+        <v>482.09</v>
       </c>
       <c r="L16" s="21">
         <f>IF(OR($B16="",$I16=""),"",$I16-IF($K16="",0,$K16))</f>
@@ -1833,12 +1837,12 @@
     <row r="17">
       <c r="A17" s="23" t="inlineStr">
         <is>
-          <t>DHAN-23126100860109+221261008541409+34126100865109+34126100865209+23126100860209+321261008684009+221261008543809+34126100865509+34126100865709+321261008684809+321261008685109+321261008685409+34126100865909+34126100866009+221261008545809+221261008545909+34126100866109+23126100860509</t>
+          <t>DHAN-321261009656509+321261009657209+231261009114209+231261009114409+231261009114609+321261009658609+321261009659109+321261009659509+231261009115709+321261009660509+231261009116209</t>
         </is>
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>KOTIC</t>
+          <t>RSYSTEMS</t>
         </is>
       </c>
       <c r="C17" s="23" t="inlineStr">
@@ -1847,16 +1851,20 @@
         </is>
       </c>
       <c r="D17" s="24" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E17" s="25" t="n">
-        <v>157.0151</v>
+        <v>274.9019</v>
       </c>
       <c r="F17" s="26" t="n">
-        <v>858</v>
-      </c>
-      <c r="G17" s="24" t="inlineStr"/>
-      <c r="H17" s="25" t="inlineStr"/>
+        <v>727</v>
+      </c>
+      <c r="G17" s="24" t="n">
+        <v>46307</v>
+      </c>
+      <c r="H17" s="25" t="n">
+        <v>263</v>
+      </c>
       <c r="I17" s="21">
         <f>IF(OR($B17="",$H17=""),"",IF($C17="LONG",($H17-$E17)*$F17,($E17-$H17)*$F17))</f>
         <v/>
@@ -1866,7 +1874,7 @@
         <v/>
       </c>
       <c r="K17" s="4" t="n">
-        <v>175</v>
+        <v>485.75</v>
       </c>
       <c r="L17" s="21">
         <f>IF(OR($B17="",$I17=""),"",$I17-IF($K17="",0,$K17))</f>
@@ -1882,19 +1890,19 @@
       </c>
       <c r="O17" s="23" t="inlineStr">
         <is>
-          <t>5-10</t>
+          <t>10-15</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261009656409+231261009113609+231261009114009+321261009657909+231261009114709+231261009115009+321261009659009+231261009115809+321261009660609+321261009660809+321261009661309+231261009117309+321261009662609+321261009663009+231261009117809+321261009663809+231261009118209</t>
+          <t>DHAN-231261009113309+231261009113509+231261009114309+231261009114509+231261009114809+321261009658809+321261009659609+231261009115609+231261009116009+321261009660909+231261009116609+321261009661609+321261009662209+231261009117509+321261009662909+231261009117909</t>
         </is>
       </c>
       <c r="B18" s="23" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>SAKSOFT</t>
         </is>
       </c>
       <c r="C18" s="23" t="inlineStr">
@@ -1906,13 +1914,17 @@
         <v>46304</v>
       </c>
       <c r="E18" s="25" t="n">
-        <v>20.9882</v>
+        <v>138.9161</v>
       </c>
       <c r="F18" s="26" t="n">
-        <v>3589</v>
-      </c>
-      <c r="G18" s="24" t="inlineStr"/>
-      <c r="H18" s="25" t="inlineStr"/>
+        <v>1443</v>
+      </c>
+      <c r="G18" s="24" t="n">
+        <v>46307</v>
+      </c>
+      <c r="H18" s="25" t="n">
+        <v>140.87</v>
+      </c>
       <c r="I18" s="21">
         <f>IF(OR($B18="",$H18=""),"",IF($C18="LONG",($H18-$E18)*$F18,($E18-$H18)*$F18))</f>
         <v/>
@@ -1922,7 +1934,7 @@
         <v/>
       </c>
       <c r="K18" s="4" t="n">
-        <v>14.75</v>
+        <v>482.51</v>
       </c>
       <c r="L18" s="21">
         <f>IF(OR($B18="",$I18=""),"",$I18-IF($K18="",0,$K18))</f>
@@ -1945,12 +1957,12 @@
     <row r="19">
       <c r="A19" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261009656509+321261009657209+231261009114209+231261009114409+231261009114609+321261009658609+321261009659109+321261009659509+231261009115709+321261009660509+231261009116209</t>
+          <t>DHAN-231261009113409+321261009657109+321261009657509+321261009658009+231261009114909+231261009115109+231261009115209+231261009115409+321261009660209+321261009660409+321261009661009+231261009116709+321261009661709+321261009662109+321261009662509</t>
         </is>
       </c>
       <c r="B19" s="23" t="inlineStr">
         <is>
-          <t>RSYSTEMS</t>
+          <t>SMCGLOBAL</t>
         </is>
       </c>
       <c r="C19" s="23" t="inlineStr">
@@ -1962,13 +1974,17 @@
         <v>46304</v>
       </c>
       <c r="E19" s="25" t="n">
-        <v>274.9019</v>
+        <v>115.2011</v>
       </c>
       <c r="F19" s="26" t="n">
-        <v>727</v>
-      </c>
-      <c r="G19" s="24" t="inlineStr"/>
-      <c r="H19" s="25" t="inlineStr"/>
+        <v>864</v>
+      </c>
+      <c r="G19" s="24" t="n">
+        <v>46307</v>
+      </c>
+      <c r="H19" s="25" t="n">
+        <v>115.68</v>
+      </c>
       <c r="I19" s="21">
         <f>IF(OR($B19="",$H19=""),"",IF($C19="LONG",($H19-$E19)*$F19,($E19-$H19)*$F19))</f>
         <v/>
@@ -1978,7 +1994,7 @@
         <v/>
       </c>
       <c r="K19" s="4" t="n">
-        <v>50.15</v>
+        <v>132.93</v>
       </c>
       <c r="L19" s="21">
         <f>IF(OR($B19="",$I19=""),"",$I19-IF($K19="",0,$K19))</f>
@@ -1994,19 +2010,19 @@
       </c>
       <c r="O19" s="23" t="inlineStr">
         <is>
-          <t>10-15</t>
+          <t>5-10</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="23" t="inlineStr">
         <is>
-          <t>DHAN-231261009113309+231261009113509+231261009114309+231261009114509+231261009114809+321261009658809+321261009659609+231261009115609+231261009116009+321261009660909+231261009116609+321261009661609+321261009662209+231261009117509+321261009662909+231261009117909</t>
+          <t>DHAN-221261012636809+23126101284009+221261012637709+34126101276009+23126101284709+23126101285909+23126101286009+34126101277509+34126101277709+23126101286509+34126101278209+321261012631509+34126101278309+321261012632109+321261012632509</t>
         </is>
       </c>
       <c r="B20" s="23" t="inlineStr">
         <is>
-          <t>SAKSOFT</t>
+          <t>BLUSPRING</t>
         </is>
       </c>
       <c r="C20" s="23" t="inlineStr">
@@ -2015,13 +2031,13 @@
         </is>
       </c>
       <c r="D20" s="24" t="n">
-        <v>46304</v>
+        <v>46307</v>
       </c>
       <c r="E20" s="25" t="n">
-        <v>138.9161</v>
+        <v>157.2127</v>
       </c>
       <c r="F20" s="26" t="n">
-        <v>1443</v>
+        <v>1095</v>
       </c>
       <c r="G20" s="24" t="inlineStr"/>
       <c r="H20" s="25" t="inlineStr"/>
@@ -2057,12 +2073,12 @@
     <row r="21">
       <c r="A21" s="23" t="inlineStr">
         <is>
-          <t>DHAN-231261009113409+321261009657109+321261009657509+321261009658009+231261009114909+231261009115109+231261009115209+231261009115409+321261009660209+321261009660409+321261009661009+231261009116709+321261009661709+321261009662109+321261009662509</t>
+          <t>DHAN-221261012636709+221261012637509+321261012626709+221261012638409+23126101284609+34126101276109+221261012640409+34126101277309+34126101277409+221261012641109+321261012630109</t>
         </is>
       </c>
       <c r="B21" s="23" t="inlineStr">
         <is>
-          <t>SMCGLOBAL</t>
+          <t>GOODLUCK</t>
         </is>
       </c>
       <c r="C21" s="23" t="inlineStr">
@@ -2071,13 +2087,13 @@
         </is>
       </c>
       <c r="D21" s="24" t="n">
-        <v>46304</v>
+        <v>46307</v>
       </c>
       <c r="E21" s="25" t="n">
-        <v>115.2011</v>
+        <v>564.8409</v>
       </c>
       <c r="F21" s="26" t="n">
-        <v>864</v>
+        <v>303</v>
       </c>
       <c r="G21" s="24" t="inlineStr"/>
       <c r="H21" s="25" t="inlineStr"/>
@@ -2090,7 +2106,7 @@
         <v/>
       </c>
       <c r="K21" s="4" t="n">
-        <v>14.75</v>
+        <v>50.15</v>
       </c>
       <c r="L21" s="21">
         <f>IF(OR($B21="",$I21=""),"",$I21-IF($K21="",0,$K21))</f>
@@ -2106,19 +2122,19 @@
       </c>
       <c r="O21" s="23" t="inlineStr">
         <is>
-          <t>5-10</t>
+          <t>10-15</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261009656609+231261009113809+231261009114109+321261009658109+231261009115509+231261009116409+231261009116809+231261009117009+231261009117209+231261009117609+231261009117709+231261009118009+231261009118109</t>
+          <t>DHAN-23126100860109+221261008541409+34126100865109+34126100865209+23126100860209+321261008684009+221261008543809+34126100865509+34126100865709+321261008684809+321261008685109+321261008685409+34126100865909+34126100866009+221261008545809+221261008545909+34126100866109+23126100860509</t>
         </is>
       </c>
       <c r="B22" s="23" t="inlineStr">
         <is>
-          <t>SUNCLAY</t>
+          <t>KOTIC</t>
         </is>
       </c>
       <c r="C22" s="23" t="inlineStr">
@@ -2127,13 +2143,13 @@
         </is>
       </c>
       <c r="D22" s="24" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="E22" s="25" t="n">
-        <v>1228.0927</v>
+        <v>157.0151</v>
       </c>
       <c r="F22" s="26" t="n">
-        <v>164</v>
+        <v>858</v>
       </c>
       <c r="G22" s="24" t="inlineStr"/>
       <c r="H22" s="25" t="inlineStr"/>
@@ -2146,7 +2162,7 @@
         <v/>
       </c>
       <c r="K22" s="4" t="n">
-        <v>50.15</v>
+        <v>175</v>
       </c>
       <c r="L22" s="21">
         <f>IF(OR($B22="",$I22=""),"",$I22-IF($K22="",0,$K22))</f>
@@ -2161,148 +2177,262 @@
         <v/>
       </c>
       <c r="O22" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261009656409+231261009113609+231261009114009+321261009657909+231261009114709+231261009115009+321261009659009+231261009115809+321261009660609+321261009660809+321261009661309+231261009117309+321261009662609+321261009663009+231261009117809+321261009663809+231261009118209</t>
+        </is>
+      </c>
+      <c r="B23" s="23" t="inlineStr">
+        <is>
+          <t>MMWL</t>
+        </is>
+      </c>
+      <c r="C23" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D23" s="24" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E23" s="25" t="n">
+        <v>20.9882</v>
+      </c>
+      <c r="F23" s="26" t="n">
+        <v>3589</v>
+      </c>
+      <c r="G23" s="24" t="inlineStr"/>
+      <c r="H23" s="25" t="inlineStr"/>
+      <c r="I23" s="21">
+        <f>IF(OR($B23="",$H23=""),"",IF($C23="LONG",($H23-$E23)*$F23,($E23-$H23)*$F23))</f>
+        <v/>
+      </c>
+      <c r="J23" s="22">
+        <f>IF(OR($B23="",$I23="",$E23=0,$F23=0),"",$I23/($E23*$F23))</f>
+        <v/>
+      </c>
+      <c r="K23" s="4" t="n">
+        <v>104.2</v>
+      </c>
+      <c r="L23" s="21">
+        <f>IF(OR($B23="",$I23=""),"",$I23-IF($K23="",0,$K23))</f>
+        <v/>
+      </c>
+      <c r="M23" s="22">
+        <f>IF(OR($B23="",$L23="",$E23=0,$F23=0),"",$L23/($E23*$F23))</f>
+        <v/>
+      </c>
+      <c r="N23" s="27">
+        <f>IF($B23="","",IF($H23="","Open","Closed"))</f>
+        <v/>
+      </c>
+      <c r="O23" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261012625809+321261012626209+23126101284209+23126101284309+321261012626909+34126101276209+34126101277109+321261012628809+221261012640809+23126101286309+34126101278009+321261012630809+221261012643209</t>
+        </is>
+      </c>
+      <c r="B24" s="23" t="inlineStr">
+        <is>
+          <t>MMWL</t>
+        </is>
+      </c>
+      <c r="C24" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D24" s="24" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E24" s="25" t="n">
+        <v>22.8999</v>
+      </c>
+      <c r="F24" s="26" t="n">
+        <v>3742</v>
+      </c>
+      <c r="G24" s="24" t="inlineStr"/>
+      <c r="H24" s="25" t="inlineStr"/>
+      <c r="I24" s="21">
+        <f>IF(OR($B24="",$H24=""),"",IF($C24="LONG",($H24-$E24)*$F24,($E24-$H24)*$F24))</f>
+        <v/>
+      </c>
+      <c r="J24" s="22">
+        <f>IF(OR($B24="",$I24="",$E24=0,$F24=0),"",$I24/($E24*$F24))</f>
+        <v/>
+      </c>
+      <c r="K24" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L24" s="21">
+        <f>IF(OR($B24="",$I24=""),"",$I24-IF($K24="",0,$K24))</f>
+        <v/>
+      </c>
+      <c r="M24" s="22">
+        <f>IF(OR($B24="",$L24="",$E24=0,$F24=0),"",$L24/($E24*$F24))</f>
+        <v/>
+      </c>
+      <c r="N24" s="27">
+        <f>IF($B24="","",IF($H24="","Open","Closed"))</f>
+        <v/>
+      </c>
+      <c r="O24" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126101275609+321261012626309+221261012637809+34126101275809+23126101284509+321261012627209+34126101277009+34126101277209+34126101277609+221261012641209+321261012630309+23126101287209+321261012631409+321261012631709+321261012632009</t>
+        </is>
+      </c>
+      <c r="B25" s="23" t="inlineStr">
+        <is>
+          <t>PRINCEPIPE</t>
+        </is>
+      </c>
+      <c r="C25" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D25" s="24" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E25" s="25" t="n">
+        <v>267.6149</v>
+      </c>
+      <c r="F25" s="26" t="n">
+        <v>641</v>
+      </c>
+      <c r="G25" s="24" t="inlineStr"/>
+      <c r="H25" s="25" t="inlineStr"/>
+      <c r="I25" s="21">
+        <f>IF(OR($B25="",$H25=""),"",IF($C25="LONG",($H25-$E25)*$F25,($E25-$H25)*$F25))</f>
+        <v/>
+      </c>
+      <c r="J25" s="22">
+        <f>IF(OR($B25="",$I25="",$E25=0,$F25=0),"",$I25/($E25*$F25))</f>
+        <v/>
+      </c>
+      <c r="K25" s="4" t="n">
+        <v>50.15</v>
+      </c>
+      <c r="L25" s="21">
+        <f>IF(OR($B25="",$I25=""),"",$I25-IF($K25="",0,$K25))</f>
+        <v/>
+      </c>
+      <c r="M25" s="22">
+        <f>IF(OR($B25="",$L25="",$E25=0,$F25=0),"",$L25/($E25*$F25))</f>
+        <v/>
+      </c>
+      <c r="N25" s="27">
+        <f>IF($B25="","",IF($H25="","Open","Closed"))</f>
+        <v/>
+      </c>
+      <c r="O25" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261009656609+231261009113809+231261009114109+321261009658109+231261009115509+231261009116409+231261009116809+231261009117009+231261009117209+231261009117609+231261009117709+231261009118009+231261009118109</t>
+        </is>
+      </c>
+      <c r="B26" s="23" t="inlineStr">
+        <is>
+          <t>SUNCLAY</t>
+        </is>
+      </c>
+      <c r="C26" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D26" s="24" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E26" s="25" t="n">
+        <v>1228.0927</v>
+      </c>
+      <c r="F26" s="26" t="n">
+        <v>164</v>
+      </c>
+      <c r="G26" s="24" t="inlineStr"/>
+      <c r="H26" s="25" t="inlineStr"/>
+      <c r="I26" s="21">
+        <f>IF(OR($B26="",$H26=""),"",IF($C26="LONG",($H26-$E26)*$F26,($E26-$H26)*$F26))</f>
+        <v/>
+      </c>
+      <c r="J26" s="22">
+        <f>IF(OR($B26="",$I26="",$E26=0,$F26=0),"",$I26/($E26*$F26))</f>
+        <v/>
+      </c>
+      <c r="K26" s="4" t="n">
+        <v>471.71</v>
+      </c>
+      <c r="L26" s="21">
+        <f>IF(OR($B26="",$I26=""),"",$I26-IF($K26="",0,$K26))</f>
+        <v/>
+      </c>
+      <c r="M26" s="22">
+        <f>IF(OR($B26="",$L26="",$E26=0,$F26=0),"",$L26/($E26*$F26))</f>
+        <v/>
+      </c>
+      <c r="N26" s="27">
+        <f>IF($B26="","",IF($H26="","Open","Closed"))</f>
+        <v/>
+      </c>
+      <c r="O26" s="23" t="inlineStr">
         <is>
           <t>10-15</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="23" t="n"/>
-      <c r="B23" s="23" t="n"/>
-      <c r="C23" s="23" t="n"/>
-      <c r="D23" s="24" t="n"/>
-      <c r="E23" s="25" t="n"/>
-      <c r="F23" s="26" t="n"/>
-      <c r="G23" s="24" t="n"/>
-      <c r="H23" s="25" t="n"/>
-      <c r="I23" s="21">
-        <f>IF(OR($B23="",$H23=""),"",IF($C23="LONG",($H23-$E23)*$F23,($E23-$H23)*$F23))</f>
-        <v/>
-      </c>
-      <c r="J23" s="22">
-        <f>IF(OR($B23="",$I23="",$E23=0,$F23=0),"",$I23/($E23*$F23))</f>
-        <v/>
-      </c>
-      <c r="K23" s="4" t="n"/>
-      <c r="L23" s="21">
-        <f>IF(OR($B23="",$I23=""),"",$I23-IF($K23="",0,$K23))</f>
-        <v/>
-      </c>
-      <c r="M23" s="22">
-        <f>IF(OR($B23="",$L23="",$E23=0,$F23=0),"",$L23/($E23*$F23))</f>
-        <v/>
-      </c>
-      <c r="N23" s="27">
-        <f>IF($B23="","",IF($H23="","Open","Closed"))</f>
-        <v/>
-      </c>
-      <c r="O23" s="23" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="23" t="n"/>
-      <c r="B24" s="23" t="n"/>
-      <c r="C24" s="23" t="n"/>
-      <c r="D24" s="24" t="n"/>
-      <c r="E24" s="25" t="n"/>
-      <c r="F24" s="26" t="n"/>
-      <c r="G24" s="24" t="n"/>
-      <c r="H24" s="25" t="n"/>
-      <c r="I24" s="21">
-        <f>IF(OR($B24="",$H24=""),"",IF($C24="LONG",($H24-$E24)*$F24,($E24-$H24)*$F24))</f>
-        <v/>
-      </c>
-      <c r="J24" s="22">
-        <f>IF(OR($B24="",$I24="",$E24=0,$F24=0),"",$I24/($E24*$F24))</f>
-        <v/>
-      </c>
-      <c r="K24" s="4" t="n"/>
-      <c r="L24" s="21">
-        <f>IF(OR($B24="",$I24=""),"",$I24-IF($K24="",0,$K24))</f>
-        <v/>
-      </c>
-      <c r="M24" s="22">
-        <f>IF(OR($B24="",$L24="",$E24=0,$F24=0),"",$L24/($E24*$F24))</f>
-        <v/>
-      </c>
-      <c r="N24" s="27">
-        <f>IF($B24="","",IF($H24="","Open","Closed"))</f>
-        <v/>
-      </c>
-      <c r="O24" s="23" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="23" t="n"/>
-      <c r="B25" s="23" t="n"/>
-      <c r="C25" s="23" t="n"/>
-      <c r="D25" s="24" t="n"/>
-      <c r="E25" s="25" t="n"/>
-      <c r="F25" s="26" t="n"/>
-      <c r="G25" s="24" t="n"/>
-      <c r="H25" s="25" t="n"/>
-      <c r="I25" s="21">
-        <f>IF(OR($B25="",$H25=""),"",IF($C25="LONG",($H25-$E25)*$F25,($E25-$H25)*$F25))</f>
-        <v/>
-      </c>
-      <c r="J25" s="22">
-        <f>IF(OR($B25="",$I25="",$E25=0,$F25=0),"",$I25/($E25*$F25))</f>
-        <v/>
-      </c>
-      <c r="K25" s="4" t="n"/>
-      <c r="L25" s="21">
-        <f>IF(OR($B25="",$I25=""),"",$I25-IF($K25="",0,$K25))</f>
-        <v/>
-      </c>
-      <c r="M25" s="22">
-        <f>IF(OR($B25="",$L25="",$E25=0,$F25=0),"",$L25/($E25*$F25))</f>
-        <v/>
-      </c>
-      <c r="N25" s="27">
-        <f>IF($B25="","",IF($H25="","Open","Closed"))</f>
-        <v/>
-      </c>
-      <c r="O25" s="23" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="23" t="n"/>
-      <c r="B26" s="23" t="n"/>
-      <c r="C26" s="23" t="n"/>
-      <c r="D26" s="24" t="n"/>
-      <c r="E26" s="25" t="n"/>
-      <c r="F26" s="26" t="n"/>
-      <c r="G26" s="24" t="n"/>
-      <c r="H26" s="25" t="n"/>
-      <c r="I26" s="21">
-        <f>IF(OR($B26="",$H26=""),"",IF($C26="LONG",($H26-$E26)*$F26,($E26-$H26)*$F26))</f>
-        <v/>
-      </c>
-      <c r="J26" s="22">
-        <f>IF(OR($B26="",$I26="",$E26=0,$F26=0),"",$I26/($E26*$F26))</f>
-        <v/>
-      </c>
-      <c r="K26" s="4" t="n"/>
-      <c r="L26" s="21">
-        <f>IF(OR($B26="",$I26=""),"",$I26-IF($K26="",0,$K26))</f>
-        <v/>
-      </c>
-      <c r="M26" s="22">
-        <f>IF(OR($B26="",$L26="",$E26=0,$F26=0),"",$L26/($E26*$F26))</f>
-        <v/>
-      </c>
-      <c r="N26" s="27">
-        <f>IF($B26="","",IF($H26="","Open","Closed"))</f>
-        <v/>
-      </c>
-      <c r="O26" s="23" t="n"/>
-    </row>
     <row r="27">
-      <c r="A27" s="23" t="n"/>
-      <c r="B27" s="23" t="n"/>
-      <c r="C27" s="23" t="n"/>
-      <c r="D27" s="24" t="n"/>
-      <c r="E27" s="25" t="n"/>
-      <c r="F27" s="26" t="n"/>
-      <c r="G27" s="24" t="n"/>
-      <c r="H27" s="25" t="n"/>
+      <c r="A27" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126101283509+23126101284109+34126101275709+221261012638509+34126101275909+23126101284809+321261012628509+321261012628709+23126101286109+321261012629509+221261012641909+221261012642709+23126101287309+221261012643409+34126101278409</t>
+        </is>
+      </c>
+      <c r="B27" s="23" t="inlineStr">
+        <is>
+          <t>SWARAJENG</t>
+        </is>
+      </c>
+      <c r="C27" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D27" s="24" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E27" s="25" t="n">
+        <v>3741.3844</v>
+      </c>
+      <c r="F27" s="26" t="n">
+        <v>45</v>
+      </c>
+      <c r="G27" s="24" t="inlineStr"/>
+      <c r="H27" s="25" t="inlineStr"/>
       <c r="I27" s="21">
         <f>IF(OR($B27="",$H27=""),"",IF($C27="LONG",($H27-$E27)*$F27,($E27-$H27)*$F27))</f>
         <v/>
@@ -2311,7 +2441,9 @@
         <f>IF(OR($B27="",$I27="",$E27=0,$F27=0),"",$I27/($E27*$F27))</f>
         <v/>
       </c>
-      <c r="K27" s="4" t="n"/>
+      <c r="K27" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L27" s="21">
         <f>IF(OR($B27="",$I27=""),"",$I27-IF($K27="",0,$K27))</f>
         <v/>
@@ -2324,7 +2456,11 @@
         <f>IF($B27="","",IF($H27="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O27" s="23" t="n"/>
+      <c r="O27" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="23" t="n"/>
@@ -30233,7 +30369,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30360,7 +30496,7 @@
     <row r="5">
       <c r="A5" s="27" t="inlineStr">
         <is>
-          <t>DELTACORP</t>
+          <t>BLUSPRING</t>
         </is>
       </c>
       <c r="B5" s="20">
@@ -30403,7 +30539,7 @@
     <row r="6">
       <c r="A6" s="27" t="inlineStr">
         <is>
-          <t>DPABHUSHAN</t>
+          <t>DELTACORP</t>
         </is>
       </c>
       <c r="B6" s="20">
@@ -30446,7 +30582,7 @@
     <row r="7">
       <c r="A7" s="27" t="inlineStr">
         <is>
-          <t>GPTINFRA</t>
+          <t>DPABHUSHAN</t>
         </is>
       </c>
       <c r="B7" s="20">
@@ -30489,7 +30625,7 @@
     <row r="8">
       <c r="A8" s="27" t="inlineStr">
         <is>
-          <t>INOXGREEN</t>
+          <t>GOODLUCK</t>
         </is>
       </c>
       <c r="B8" s="20">
@@ -30532,7 +30668,7 @@
     <row r="9">
       <c r="A9" s="27" t="inlineStr">
         <is>
-          <t>KOTIC</t>
+          <t>GPTINFRA</t>
         </is>
       </c>
       <c r="B9" s="20">
@@ -30575,7 +30711,7 @@
     <row r="10">
       <c r="A10" s="27" t="inlineStr">
         <is>
-          <t>KRISHNADEF</t>
+          <t>INOXGREEN</t>
         </is>
       </c>
       <c r="B10" s="20">
@@ -30618,7 +30754,7 @@
     <row r="11">
       <c r="A11" s="27" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>KOTIC</t>
         </is>
       </c>
       <c r="B11" s="20">
@@ -30661,7 +30797,7 @@
     <row r="12">
       <c r="A12" s="27" t="inlineStr">
         <is>
-          <t>MOBIKWIK</t>
+          <t>KRISHNADEF</t>
         </is>
       </c>
       <c r="B12" s="20">
@@ -30704,7 +30840,7 @@
     <row r="13">
       <c r="A13" s="27" t="inlineStr">
         <is>
-          <t>PNGSREVA</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="B13" s="20">
@@ -30747,7 +30883,7 @@
     <row r="14">
       <c r="A14" s="27" t="inlineStr">
         <is>
-          <t>RSYSTEMS</t>
+          <t>MOBIKWIK</t>
         </is>
       </c>
       <c r="B14" s="20">
@@ -30790,7 +30926,7 @@
     <row r="15">
       <c r="A15" s="27" t="inlineStr">
         <is>
-          <t>SAKSOFT</t>
+          <t>PNGSREVA</t>
         </is>
       </c>
       <c r="B15" s="20">
@@ -30833,7 +30969,7 @@
     <row r="16">
       <c r="A16" s="27" t="inlineStr">
         <is>
-          <t>SATIN</t>
+          <t>PRINCEPIPE</t>
         </is>
       </c>
       <c r="B16" s="20">
@@ -30876,7 +31012,7 @@
     <row r="17">
       <c r="A17" s="27" t="inlineStr">
         <is>
-          <t>SGFIN</t>
+          <t>RSYSTEMS</t>
         </is>
       </c>
       <c r="B17" s="20">
@@ -30919,7 +31055,7 @@
     <row r="18">
       <c r="A18" s="27" t="inlineStr">
         <is>
-          <t>SMCGLOBAL</t>
+          <t>SAKSOFT</t>
         </is>
       </c>
       <c r="B18" s="20">
@@ -30962,7 +31098,7 @@
     <row r="19">
       <c r="A19" s="27" t="inlineStr">
         <is>
-          <t>SUNCLAY</t>
+          <t>SATIN</t>
         </is>
       </c>
       <c r="B19" s="20">
@@ -31005,78 +31141,250 @@
     <row r="20">
       <c r="A20" s="27" t="inlineStr">
         <is>
+          <t>SGFIN</t>
+        </is>
+      </c>
+      <c r="B20" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A20)</f>
+        <v/>
+      </c>
+      <c r="C20" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A20,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D20" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A20,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E20" s="22">
+        <f>IFERROR($C20/$B20,"")</f>
+        <v/>
+      </c>
+      <c r="F20" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A20,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G20" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A20,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H20" s="21">
+        <f>IFERROR($G20/$B20,"")</f>
+        <v/>
+      </c>
+      <c r="I20" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A20),"")</f>
+        <v/>
+      </c>
+      <c r="J20" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A20),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="27" t="inlineStr">
+        <is>
+          <t>SMCGLOBAL</t>
+        </is>
+      </c>
+      <c r="B21" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A21)</f>
+        <v/>
+      </c>
+      <c r="C21" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A21,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D21" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A21,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E21" s="22">
+        <f>IFERROR($C21/$B21,"")</f>
+        <v/>
+      </c>
+      <c r="F21" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A21,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G21" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A21,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H21" s="21">
+        <f>IFERROR($G21/$B21,"")</f>
+        <v/>
+      </c>
+      <c r="I21" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A21),"")</f>
+        <v/>
+      </c>
+      <c r="J21" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A21),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="27" t="inlineStr">
+        <is>
+          <t>SUNCLAY</t>
+        </is>
+      </c>
+      <c r="B22" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A22)</f>
+        <v/>
+      </c>
+      <c r="C22" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A22,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D22" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A22,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E22" s="22">
+        <f>IFERROR($C22/$B22,"")</f>
+        <v/>
+      </c>
+      <c r="F22" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A22,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G22" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A22,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H22" s="21">
+        <f>IFERROR($G22/$B22,"")</f>
+        <v/>
+      </c>
+      <c r="I22" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A22),"")</f>
+        <v/>
+      </c>
+      <c r="J22" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A22),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="27" t="inlineStr">
+        <is>
+          <t>SWARAJENG</t>
+        </is>
+      </c>
+      <c r="B23" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A23)</f>
+        <v/>
+      </c>
+      <c r="C23" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A23,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D23" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A23,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E23" s="22">
+        <f>IFERROR($C23/$B23,"")</f>
+        <v/>
+      </c>
+      <c r="F23" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A23,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G23" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A23,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H23" s="21">
+        <f>IFERROR($G23/$B23,"")</f>
+        <v/>
+      </c>
+      <c r="I23" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A23),"")</f>
+        <v/>
+      </c>
+      <c r="J23" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A23),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="27" t="inlineStr">
+        <is>
           <t>YUKEN</t>
         </is>
       </c>
-      <c r="B20" s="20">
-        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A20)</f>
-        <v/>
-      </c>
-      <c r="C20" s="20">
-        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A20,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
-        <v/>
-      </c>
-      <c r="D20" s="20">
-        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A20,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
-        <v/>
-      </c>
-      <c r="E20" s="22">
-        <f>IFERROR($C20/$B20,"")</f>
-        <v/>
-      </c>
-      <c r="F20" s="21">
-        <f>SUMIF('Trade Log'!$B$4:$B$503,$A20,'Trade Log'!$I$4:$I$503)</f>
-        <v/>
-      </c>
-      <c r="G20" s="21">
-        <f>SUMIF('Trade Log'!$B$4:$B$503,$A20,'Trade Log'!$L$4:$L$503)</f>
-        <v/>
-      </c>
-      <c r="H20" s="21">
-        <f>IFERROR($G20/$B20,"")</f>
-        <v/>
-      </c>
-      <c r="I20" s="21">
-        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A20),"")</f>
-        <v/>
-      </c>
-      <c r="J20" s="21">
-        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A20),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="B24" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A24)</f>
+        <v/>
+      </c>
+      <c r="C24" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A24,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D24" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A24,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E24" s="22">
+        <f>IFERROR($C24/$B24,"")</f>
+        <v/>
+      </c>
+      <c r="F24" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A24,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G24" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A24,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H24" s="21">
+        <f>IFERROR($G24/$B24,"")</f>
+        <v/>
+      </c>
+      <c r="I24" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A24),"")</f>
+        <v/>
+      </c>
+      <c r="J24" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A24),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B21" s="30">
-        <f>SUM(B4:B20)</f>
-        <v/>
-      </c>
-      <c r="C21" s="30">
-        <f>SUM(C4:C20)</f>
-        <v/>
-      </c>
-      <c r="D21" s="30">
-        <f>SUM(D4:D20)</f>
-        <v/>
-      </c>
-      <c r="E21" s="31">
-        <f>IFERROR(C21/B21,"")</f>
-        <v/>
-      </c>
-      <c r="F21" s="32">
-        <f>SUM(F4:F20)</f>
-        <v/>
-      </c>
-      <c r="G21" s="32">
-        <f>SUM(G4:G20)</f>
-        <v/>
-      </c>
-      <c r="H21" s="32">
-        <f>IFERROR(G21/B21,"")</f>
+      <c r="B25" s="30">
+        <f>SUM(B4:B24)</f>
+        <v/>
+      </c>
+      <c r="C25" s="30">
+        <f>SUM(C4:C24)</f>
+        <v/>
+      </c>
+      <c r="D25" s="30">
+        <f>SUM(D4:D24)</f>
+        <v/>
+      </c>
+      <c r="E25" s="31">
+        <f>IFERROR(C25/B25,"")</f>
+        <v/>
+      </c>
+      <c r="F25" s="32">
+        <f>SUM(F4:F24)</f>
+        <v/>
+      </c>
+      <c r="G25" s="32">
+        <f>SUM(G4:G24)</f>
+        <v/>
+      </c>
+      <c r="H25" s="32">
+        <f>IFERROR(G25/B25,"")</f>
         <v/>
       </c>
     </row>
@@ -31095,7 +31403,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N23"/>
+  <dimension ref="A1:N28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -31346,7 +31654,7 @@
         <v>35.4</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>120.42</v>
+        <v>123.79</v>
       </c>
       <c r="N6" s="21">
         <f>SUM(E6:M6)</f>
@@ -31397,7 +31705,7 @@
         <v>35.4</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>72</v>
+        <v>74.02</v>
       </c>
       <c r="N7" s="21">
         <f>SUM(E7:M7)</f>
@@ -31448,7 +31756,7 @@
         <v>35.4</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>72.14</v>
+        <v>74.16</v>
       </c>
       <c r="N8" s="21">
         <f>SUM(E8:M8)</f>
@@ -31499,7 +31807,7 @@
         <v>35.4</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>120.08</v>
+        <v>123.45</v>
       </c>
       <c r="N9" s="21">
         <f>SUM(E9:M9)</f>
@@ -31550,7 +31858,7 @@
         <v>35.4</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>100.2</v>
+        <v>103.01</v>
       </c>
       <c r="N10" s="21">
         <f>SUM(E10:M10)</f>
@@ -31601,7 +31909,7 @@
         <v>35.4</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>40.17</v>
+        <v>41.29</v>
       </c>
       <c r="N11" s="21">
         <f>SUM(E11:M11)</f>
@@ -31652,7 +31960,7 @@
         <v>35.4</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>48.14</v>
+        <v>49.49</v>
       </c>
       <c r="N12" s="21">
         <f>SUM(E12:M12)</f>
@@ -31703,7 +32011,7 @@
         <v>35.4</v>
       </c>
       <c r="M13" s="4" t="n">
-        <v>49.08</v>
+        <v>29.77</v>
       </c>
       <c r="N13" s="21">
         <f>SUM(E13:M13)</f>
@@ -31754,7 +32062,7 @@
         <v>35.4</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>40.04</v>
+        <v>41.17</v>
       </c>
       <c r="N14" s="21">
         <f>SUM(E14:M14)</f>
@@ -31781,22 +32089,22 @@
         <v>46304</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>45.06</v>
+        <v>65.06</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>0</v>
+        <v>147.69</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>4.61</v>
+        <v>9.15</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>0.15</v>
+        <v>0.3</v>
       </c>
       <c r="I15" s="4" t="n">
         <v>4.51</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>8.970000000000001</v>
+        <v>13.41</v>
       </c>
       <c r="K15" s="4" t="n">
         <v>14.75</v>
@@ -31828,24 +32136,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D16" s="24" t="inlineStr"/>
+      <c r="D16" s="24" t="n">
+        <v>46307</v>
+      </c>
       <c r="E16" s="4" t="n">
-        <v>0</v>
+        <v>60.1</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>0</v>
+        <v>200.23</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0</v>
+        <v>6.15</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="I16" s="4" t="n">
-        <v>0</v>
+        <v>30.04</v>
       </c>
       <c r="J16" s="4" t="n">
-        <v>0</v>
+        <v>11.96</v>
       </c>
       <c r="K16" s="4" t="n">
         <v>14.75</v>
@@ -31854,7 +32164,7 @@
         <v>35.4</v>
       </c>
       <c r="M16" s="4" t="n">
-        <v>0</v>
+        <v>123.27</v>
       </c>
       <c r="N16" s="21">
         <f>SUM(E16:M16)</f>
@@ -31864,12 +32174,12 @@
     <row r="17">
       <c r="A17" s="23" t="inlineStr">
         <is>
-          <t>DHAN-23126100860109+221261008541409+34126100865109+34126100865209+23126100860209+321261008684009+221261008543809+34126100865509+34126100865709+321261008684809+321261008685109+321261008685409+34126100865909+34126100866009+221261008545809+221261008545909+34126100866109+23126100860509</t>
+          <t>DHAN-321261009656509+321261009657209+231261009114209+231261009114409+231261009114609+321261009658609+321261009659109+321261009659509+231261009115709+321261009660509+231261009116209</t>
         </is>
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>KOTIC</t>
+          <t>RSYSTEMS</t>
         </is>
       </c>
       <c r="C17" s="23" t="inlineStr">
@@ -31877,33 +32187,35 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D17" s="24" t="inlineStr"/>
+      <c r="D17" s="24" t="n">
+        <v>46307</v>
+      </c>
       <c r="E17" s="4" t="n">
-        <v>0</v>
+        <v>59.98</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>134.72</v>
+        <v>199.85</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>4.14</v>
+        <v>6.14</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>0.13</v>
+        <v>0.2</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>20.49</v>
+        <v>29.98</v>
       </c>
       <c r="J17" s="4" t="n">
-        <v>0.77</v>
+        <v>11.94</v>
       </c>
       <c r="K17" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L17" s="4" t="n">
-        <v>0</v>
+        <v>35.4</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>0</v>
+        <v>127.52</v>
       </c>
       <c r="N17" s="21">
         <f>SUM(E17:M17)</f>
@@ -31913,12 +32225,12 @@
     <row r="18">
       <c r="A18" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261009656409+231261009113609+231261009114009+321261009657909+231261009114709+231261009115009+321261009659009+231261009115809+321261009660609+321261009660809+321261009661309+231261009117309+321261009662609+321261009663009+231261009117809+321261009663809+231261009118209</t>
+          <t>DHAN-231261009113309+231261009113509+231261009114309+231261009114509+231261009114809+321261009658809+321261009659609+231261009115609+231261009116009+321261009660909+231261009116609+321261009661609+321261009662209+231261009117509+321261009662909+231261009117909</t>
         </is>
       </c>
       <c r="B18" s="23" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>SAKSOFT</t>
         </is>
       </c>
       <c r="C18" s="23" t="inlineStr">
@@ -31926,33 +32238,35 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D18" s="24" t="inlineStr"/>
+      <c r="D18" s="24" t="n">
+        <v>46307</v>
+      </c>
       <c r="E18" s="4" t="n">
-        <v>0</v>
+        <v>60.11</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>0</v>
+        <v>200.46</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0</v>
+        <v>6.15</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="I18" s="4" t="n">
-        <v>0</v>
+        <v>30.07</v>
       </c>
       <c r="J18" s="4" t="n">
-        <v>0</v>
+        <v>11.96</v>
       </c>
       <c r="K18" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L18" s="4" t="n">
-        <v>0</v>
+        <v>35.4</v>
       </c>
       <c r="M18" s="4" t="n">
-        <v>0</v>
+        <v>123.4</v>
       </c>
       <c r="N18" s="21">
         <f>SUM(E18:M18)</f>
@@ -31962,12 +32276,12 @@
     <row r="19">
       <c r="A19" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261009656509+321261009657209+231261009114209+231261009114409+231261009114609+321261009658609+321261009659109+321261009659509+231261009115709+321261009660509+231261009116209</t>
+          <t>DHAN-231261009113409+321261009657109+321261009657509+321261009658009+231261009114909+231261009115109+231261009115209+231261009115409+321261009660209+321261009660409+321261009661009+231261009116709+321261009661709+321261009662109+321261009662509</t>
         </is>
       </c>
       <c r="B19" s="23" t="inlineStr">
         <is>
-          <t>RSYSTEMS</t>
+          <t>SMCGLOBAL</t>
         </is>
       </c>
       <c r="C19" s="23" t="inlineStr">
@@ -31975,30 +32289,32 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D19" s="24" t="inlineStr"/>
+      <c r="D19" s="24" t="n">
+        <v>46307</v>
+      </c>
       <c r="E19" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>0</v>
+        <v>99.53</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>0</v>
+        <v>3.06</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="I19" s="4" t="n">
-        <v>0</v>
+        <v>14.93</v>
       </c>
       <c r="J19" s="4" t="n">
-        <v>0</v>
+        <v>0.57</v>
       </c>
       <c r="K19" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L19" s="4" t="n">
-        <v>35.4</v>
+        <v>0</v>
       </c>
       <c r="M19" s="4" t="n">
         <v>0</v>
@@ -32011,12 +32327,12 @@
     <row r="20">
       <c r="A20" s="23" t="inlineStr">
         <is>
-          <t>DHAN-231261009113309+231261009113509+231261009114309+231261009114509+231261009114809+321261009658809+321261009659609+231261009115609+231261009116009+321261009660909+231261009116609+321261009661609+321261009662209+231261009117509+321261009662909+231261009117909</t>
+          <t>DHAN-221261012636809+23126101284009+221261012637709+34126101276009+23126101284709+23126101285909+23126101286009+34126101277509+34126101277709+23126101286509+34126101278209+321261012631509+34126101278309+321261012632109+321261012632509</t>
         </is>
       </c>
       <c r="B20" s="23" t="inlineStr">
         <is>
-          <t>SAKSOFT</t>
+          <t>BLUSPRING</t>
         </is>
       </c>
       <c r="C20" s="23" t="inlineStr">
@@ -32060,12 +32376,12 @@
     <row r="21">
       <c r="A21" s="23" t="inlineStr">
         <is>
-          <t>DHAN-231261009113409+321261009657109+321261009657509+321261009658009+231261009114909+231261009115109+231261009115209+231261009115409+321261009660209+321261009660409+321261009661009+231261009116709+321261009661709+321261009662109+321261009662509</t>
+          <t>DHAN-221261012636709+221261012637509+321261012626709+221261012638409+23126101284609+34126101276109+221261012640409+34126101277309+34126101277409+221261012641109+321261012630109</t>
         </is>
       </c>
       <c r="B21" s="23" t="inlineStr">
         <is>
-          <t>SMCGLOBAL</t>
+          <t>GOODLUCK</t>
         </is>
       </c>
       <c r="C21" s="23" t="inlineStr">
@@ -32096,7 +32412,7 @@
         <v>14.75</v>
       </c>
       <c r="L21" s="4" t="n">
-        <v>0</v>
+        <v>35.4</v>
       </c>
       <c r="M21" s="4" t="n">
         <v>0</v>
@@ -32109,12 +32425,12 @@
     <row r="22">
       <c r="A22" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261009656609+231261009113809+231261009114109+321261009658109+231261009115509+231261009116409+231261009116809+231261009117009+231261009117209+231261009117609+231261009117709+231261009118009+231261009118109</t>
+          <t>DHAN-23126100860109+221261008541409+34126100865109+34126100865209+23126100860209+321261008684009+221261008543809+34126100865509+34126100865709+321261008684809+321261008685109+321261008685409+34126100865909+34126100866009+221261008545809+221261008545909+34126100866109+23126100860509</t>
         </is>
       </c>
       <c r="B22" s="23" t="inlineStr">
         <is>
-          <t>SUNCLAY</t>
+          <t>KOTIC</t>
         </is>
       </c>
       <c r="C22" s="23" t="inlineStr">
@@ -32127,25 +32443,25 @@
         <v>0</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>0</v>
+        <v>134.72</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>0</v>
+        <v>4.14</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>0</v>
+        <v>0.13</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>0</v>
+        <v>20.49</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>0</v>
+        <v>0.77</v>
       </c>
       <c r="K22" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L22" s="4" t="n">
-        <v>35.4</v>
+        <v>0</v>
       </c>
       <c r="M22" s="4" t="n">
         <v>0</v>
@@ -32156,54 +32472,299 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="A23" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261009656409+231261009113609+231261009114009+321261009657909+231261009114709+231261009115009+321261009659009+231261009115809+321261009660609+321261009660809+321261009661309+231261009117309+321261009662609+321261009663009+231261009117809+321261009663809+231261009118209</t>
+        </is>
+      </c>
+      <c r="B23" s="23" t="inlineStr">
+        <is>
+          <t>MMWL</t>
+        </is>
+      </c>
+      <c r="C23" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D23" s="24" t="inlineStr"/>
+      <c r="E23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>75.33</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="H23" s="4" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="I23" s="4" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="J23" s="4" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="K23" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" s="21">
+        <f>SUM(E23:M23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261012625809+321261012626209+23126101284209+23126101284309+321261012626909+34126101276209+34126101277109+321261012628809+221261012640809+23126101286309+34126101278009+321261012630809+221261012643209</t>
+        </is>
+      </c>
+      <c r="B24" s="23" t="inlineStr">
+        <is>
+          <t>MMWL</t>
+        </is>
+      </c>
+      <c r="C24" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D24" s="24" t="inlineStr"/>
+      <c r="E24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" s="21">
+        <f>SUM(E24:M24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126101275609+321261012626309+221261012637809+34126101275809+23126101284509+321261012627209+34126101277009+34126101277209+34126101277609+221261012641209+321261012630309+23126101287209+321261012631409+321261012631709+321261012632009</t>
+        </is>
+      </c>
+      <c r="B25" s="23" t="inlineStr">
+        <is>
+          <t>PRINCEPIPE</t>
+        </is>
+      </c>
+      <c r="C25" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D25" s="24" t="inlineStr"/>
+      <c r="E25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L25" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" s="21">
+        <f>SUM(E25:M25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261009656609+231261009113809+231261009114109+321261009658109+231261009115509+231261009116409+231261009116809+231261009117009+231261009117209+231261009117609+231261009117709+231261009118009+231261009118109</t>
+        </is>
+      </c>
+      <c r="B26" s="23" t="inlineStr">
+        <is>
+          <t>SUNCLAY</t>
+        </is>
+      </c>
+      <c r="C26" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D26" s="24" t="inlineStr"/>
+      <c r="E26" s="4" t="n">
+        <v>49.11</v>
+      </c>
+      <c r="F26" s="4" t="n">
+        <v>201.41</v>
+      </c>
+      <c r="G26" s="4" t="n">
+        <v>6.18</v>
+      </c>
+      <c r="H26" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I26" s="4" t="n">
+        <v>30.68</v>
+      </c>
+      <c r="J26" s="4" t="n">
+        <v>9.99</v>
+      </c>
+      <c r="K26" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L26" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M26" s="4" t="n">
+        <v>123.99</v>
+      </c>
+      <c r="N26" s="21">
+        <f>SUM(E26:M26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126101283509+23126101284109+34126101275709+221261012638509+34126101275909+23126101284809+321261012628509+321261012628709+23126101286109+321261012629509+221261012641909+221261012642709+23126101287309+221261012643409+34126101278409</t>
+        </is>
+      </c>
+      <c r="B27" s="23" t="inlineStr">
+        <is>
+          <t>SWARAJENG</t>
+        </is>
+      </c>
+      <c r="C27" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D27" s="24" t="inlineStr"/>
+      <c r="E27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L27" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" s="21">
+        <f>SUM(E27:M27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E23" s="32">
-        <f>SUM(E4:E22)</f>
-        <v/>
-      </c>
-      <c r="F23" s="32">
-        <f>SUM(F4:F22)</f>
-        <v/>
-      </c>
-      <c r="G23" s="32">
-        <f>SUM(G4:G22)</f>
-        <v/>
-      </c>
-      <c r="H23" s="32">
-        <f>SUM(H4:H22)</f>
-        <v/>
-      </c>
-      <c r="I23" s="32">
-        <f>SUM(I4:I22)</f>
-        <v/>
-      </c>
-      <c r="J23" s="32">
-        <f>SUM(J4:J22)</f>
-        <v/>
-      </c>
-      <c r="K23" s="32">
-        <f>SUM(K4:K22)</f>
-        <v/>
-      </c>
-      <c r="L23" s="32">
-        <f>SUM(L4:L22)</f>
-        <v/>
-      </c>
-      <c r="M23" s="32">
-        <f>SUM(M4:M22)</f>
-        <v/>
-      </c>
-      <c r="N23" s="32">
-        <f>SUM(N4:N22)</f>
+      <c r="E28" s="32">
+        <f>SUM(E4:E27)</f>
+        <v/>
+      </c>
+      <c r="F28" s="32">
+        <f>SUM(F4:F27)</f>
+        <v/>
+      </c>
+      <c r="G28" s="32">
+        <f>SUM(G4:G27)</f>
+        <v/>
+      </c>
+      <c r="H28" s="32">
+        <f>SUM(H4:H27)</f>
+        <v/>
+      </c>
+      <c r="I28" s="32">
+        <f>SUM(I4:I27)</f>
+        <v/>
+      </c>
+      <c r="J28" s="32">
+        <f>SUM(J4:J27)</f>
+        <v/>
+      </c>
+      <c r="K28" s="32">
+        <f>SUM(K4:K27)</f>
+        <v/>
+      </c>
+      <c r="L28" s="32">
+        <f>SUM(L4:L27)</f>
+        <v/>
+      </c>
+      <c r="M28" s="32">
+        <f>SUM(M4:M27)</f>
+        <v/>
+      </c>
+      <c r="N28" s="32">
+        <f>SUM(N4:N27)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:N22"/>
+  <autoFilter ref="A3:N27"/>
   <mergeCells count="2">
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>
@@ -32218,7 +32779,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -32508,40 +33069,85 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="28" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B11" s="20">
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,12),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,19))</f>
+        <v/>
+      </c>
+      <c r="C11" s="20">
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,12),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,19),'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D11" s="20">
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,12),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,19),'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E11" s="22">
+        <f>IFERROR($C11/$B11,"")</f>
+        <v/>
+      </c>
+      <c r="F11" s="21">
+        <f>SUMIFS('Trade Log'!$I$4:$I$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,12),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,19))</f>
+        <v/>
+      </c>
+      <c r="G11" s="21">
+        <f>SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,12),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,19))</f>
+        <v/>
+      </c>
+      <c r="H11" s="21">
+        <f>IFERROR($G11/$B11,"")</f>
+        <v/>
+      </c>
+      <c r="I11" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,12),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,19)),"")</f>
+        <v/>
+      </c>
+      <c r="J11" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,12),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,19)),"")</f>
+        <v/>
+      </c>
+      <c r="K11" s="29">
+        <f>IFERROR(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,12),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,19),'Trade Log'!$L$4:$L$503,"&gt;0")/ABS(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,12),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,19),'Trade Log'!$L$4:$L$503,"&lt;0")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B11" s="30">
-        <f>SUM(B10:B10)</f>
-        <v/>
-      </c>
-      <c r="C11" s="30">
-        <f>SUM(C10:C10)</f>
-        <v/>
-      </c>
-      <c r="D11" s="30">
-        <f>SUM(D10:D10)</f>
-        <v/>
-      </c>
-      <c r="E11" s="31">
-        <f>IFERROR(C11/B11,"")</f>
-        <v/>
-      </c>
-      <c r="F11" s="32">
-        <f>SUM(F10:F10)</f>
-        <v/>
-      </c>
-      <c r="G11" s="32">
-        <f>SUM(G10:G10)</f>
-        <v/>
-      </c>
-      <c r="H11" s="32">
-        <f>IFERROR(G11/B11,"")</f>
-        <v/>
-      </c>
-      <c r="K11" s="33">
+      <c r="B12" s="30">
+        <f>SUM(B10:B11)</f>
+        <v/>
+      </c>
+      <c r="C12" s="30">
+        <f>SUM(C10:C11)</f>
+        <v/>
+      </c>
+      <c r="D12" s="30">
+        <f>SUM(D10:D11)</f>
+        <v/>
+      </c>
+      <c r="E12" s="31">
+        <f>IFERROR(C12/B12,"")</f>
+        <v/>
+      </c>
+      <c r="F12" s="32">
+        <f>SUM(F10:F11)</f>
+        <v/>
+      </c>
+      <c r="G12" s="32">
+        <f>SUM(G10:G11)</f>
+        <v/>
+      </c>
+      <c r="H12" s="32">
+        <f>IFERROR(G12/B12,"")</f>
+        <v/>
+      </c>
+      <c r="K12" s="33">
         <f>IFERROR(SUMIF('Trade Log'!$L$4:$L$503,"&gt;0")/ABS(SUMIF('Trade Log'!$L$4:$L$503,"&lt;0")),"")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Reconcile KOTIC, MMWL (10-09 entry), and SUNCLAY stuck at status=open
Same recurring bug as YUKEN (2026-10-07): a bot-placed exit sell partially
fills within the 12s confirmation poll, times out, then fully fills on its
own with nothing ever reconciling it. All three confirmed NOT manual
trades -- every exit order traces back to a real "[trade] Order placed"
log entry from this bot, verified via Dhan's /trades API and the
order-update-feed cache:

- KOTIC (entered 10-08): exited 10-09 09:16:57 @ 158.01, +853.62
- MMWL (entered 10-09): exited 10-12 09:16:47 @ 21.55, +2016.30
  (first real exit chance was 10-12 -- weekend in between, nothing wrong
  there)
- SUNCLAY (entered 10-09): exited 10-12 12:03:30 @ 1195.11, -5409.16
  (took ~4 minutes to fill, not seconds -- the code's own "rejected"
  wording here is a misnomer, same root cause as the other two)

Workbooks regenerated via --sync-pnl to reflect the fix.
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_oct2026.xlsx
+++ b/results/strategy_pnl_oct2026.xlsx
@@ -1717,12 +1717,12 @@
     <row r="15">
       <c r="A15" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261008541309+221261008541509+321261008683209+221261008542109+34126100865309+34126100865409+221261008543409+221261008543909+221261008544309+34126100865609+221261008545009+23126100860309+34126100865809+23126100860409</t>
+          <t>DHAN-23126100860109+221261008541409+34126100865109+34126100865209+23126100860209+321261008684009+221261008543809+34126100865509+34126100865709+321261008684809+321261008685109+321261008685409+34126100865909+34126100866009+221261008545809+221261008545909+34126100866109+23126100860509</t>
         </is>
       </c>
       <c r="B15" s="23" t="inlineStr">
         <is>
-          <t>PNGSREVA</t>
+          <t>KOTIC</t>
         </is>
       </c>
       <c r="C15" s="23" t="inlineStr">
@@ -1734,16 +1734,16 @@
         <v>46303</v>
       </c>
       <c r="E15" s="25" t="n">
-        <v>705.2641</v>
+        <v>157.0151</v>
       </c>
       <c r="F15" s="26" t="n">
-        <v>213</v>
+        <v>858</v>
       </c>
       <c r="G15" s="24" t="n">
         <v>46304</v>
       </c>
       <c r="H15" s="25" t="n">
-        <v>693.37</v>
+        <v>158.01</v>
       </c>
       <c r="I15" s="21">
         <f>IF(OR($B15="",$H15=""),"",IF($C15="LONG",($H15-$E15)*$F15,($E15-$H15)*$F15))</f>
@@ -1754,7 +1754,7 @@
         <v/>
       </c>
       <c r="K15" s="4" t="n">
-        <v>254.86</v>
+        <v>315.57</v>
       </c>
       <c r="L15" s="21">
         <f>IF(OR($B15="",$I15=""),"",$I15-IF($K15="",0,$K15))</f>
@@ -1770,19 +1770,19 @@
       </c>
       <c r="O15" s="23" t="inlineStr">
         <is>
-          <t>10-15</t>
+          <t>5-10</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="23" t="inlineStr">
         <is>
-          <t>DHAN-231261009113209+231261009113709+231261009113909+321261009657809+321261009658409+321261009658709+231261009115309+321261009659409+321261009660109+231261009116109+231261009116309+231261009116509+231261009117109</t>
+          <t>DHAN-221261008541309+221261008541509+321261008683209+221261008542109+34126100865309+34126100865409+221261008543409+221261008543909+221261008544309+34126100865609+221261008545009+23126100860309+34126100865809+23126100860409</t>
         </is>
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>INOXGREEN</t>
+          <t>PNGSREVA</t>
         </is>
       </c>
       <c r="C16" s="23" t="inlineStr">
@@ -1791,19 +1791,19 @@
         </is>
       </c>
       <c r="D16" s="24" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E16" s="25" t="n">
+        <v>705.2641</v>
+      </c>
+      <c r="F16" s="26" t="n">
+        <v>213</v>
+      </c>
+      <c r="G16" s="24" t="n">
         <v>46304</v>
       </c>
-      <c r="E16" s="25" t="n">
-        <v>129.4349</v>
-      </c>
-      <c r="F16" s="26" t="n">
-        <v>1547</v>
-      </c>
-      <c r="G16" s="24" t="n">
-        <v>46307</v>
-      </c>
       <c r="H16" s="25" t="n">
-        <v>121.63</v>
+        <v>693.37</v>
       </c>
       <c r="I16" s="21">
         <f>IF(OR($B16="",$H16=""),"",IF($C16="LONG",($H16-$E16)*$F16,($E16-$H16)*$F16))</f>
@@ -1814,7 +1814,7 @@
         <v/>
       </c>
       <c r="K16" s="4" t="n">
-        <v>482.09</v>
+        <v>254.86</v>
       </c>
       <c r="L16" s="21">
         <f>IF(OR($B16="",$I16=""),"",$I16-IF($K16="",0,$K16))</f>
@@ -1837,12 +1837,12 @@
     <row r="17">
       <c r="A17" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261009656509+321261009657209+231261009114209+231261009114409+231261009114609+321261009658609+321261009659109+321261009659509+231261009115709+321261009660509+231261009116209</t>
+          <t>DHAN-231261009113209+231261009113709+231261009113909+321261009657809+321261009658409+321261009658709+231261009115309+321261009659409+321261009660109+231261009116109+231261009116309+231261009116509+231261009117109</t>
         </is>
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>RSYSTEMS</t>
+          <t>INOXGREEN</t>
         </is>
       </c>
       <c r="C17" s="23" t="inlineStr">
@@ -1854,16 +1854,16 @@
         <v>46304</v>
       </c>
       <c r="E17" s="25" t="n">
-        <v>274.9019</v>
+        <v>129.4349</v>
       </c>
       <c r="F17" s="26" t="n">
-        <v>727</v>
+        <v>1547</v>
       </c>
       <c r="G17" s="24" t="n">
         <v>46307</v>
       </c>
       <c r="H17" s="25" t="n">
-        <v>263</v>
+        <v>121.63</v>
       </c>
       <c r="I17" s="21">
         <f>IF(OR($B17="",$H17=""),"",IF($C17="LONG",($H17-$E17)*$F17,($E17-$H17)*$F17))</f>
@@ -1874,7 +1874,7 @@
         <v/>
       </c>
       <c r="K17" s="4" t="n">
-        <v>485.75</v>
+        <v>482.09</v>
       </c>
       <c r="L17" s="21">
         <f>IF(OR($B17="",$I17=""),"",$I17-IF($K17="",0,$K17))</f>
@@ -1897,12 +1897,12 @@
     <row r="18">
       <c r="A18" s="23" t="inlineStr">
         <is>
-          <t>DHAN-231261009113309+231261009113509+231261009114309+231261009114509+231261009114809+321261009658809+321261009659609+231261009115609+231261009116009+321261009660909+231261009116609+321261009661609+321261009662209+231261009117509+321261009662909+231261009117909</t>
+          <t>DHAN-321261009656409+231261009113609+231261009114009+321261009657909+231261009114709+231261009115009+321261009659009+231261009115809+321261009660609+321261009660809+321261009661309+231261009117309+321261009662609+321261009663009+231261009117809+321261009663809+231261009118209</t>
         </is>
       </c>
       <c r="B18" s="23" t="inlineStr">
         <is>
-          <t>SAKSOFT</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="C18" s="23" t="inlineStr">
@@ -1914,16 +1914,16 @@
         <v>46304</v>
       </c>
       <c r="E18" s="25" t="n">
-        <v>138.9161</v>
+        <v>20.9882</v>
       </c>
       <c r="F18" s="26" t="n">
-        <v>1443</v>
+        <v>3589</v>
       </c>
       <c r="G18" s="24" t="n">
         <v>46307</v>
       </c>
       <c r="H18" s="25" t="n">
-        <v>140.87</v>
+        <v>21.55</v>
       </c>
       <c r="I18" s="21">
         <f>IF(OR($B18="",$H18=""),"",IF($C18="LONG",($H18-$E18)*$F18,($E18-$H18)*$F18))</f>
@@ -1934,7 +1934,7 @@
         <v/>
       </c>
       <c r="K18" s="4" t="n">
-        <v>482.51</v>
+        <v>104.2</v>
       </c>
       <c r="L18" s="21">
         <f>IF(OR($B18="",$I18=""),"",$I18-IF($K18="",0,$K18))</f>
@@ -1957,12 +1957,12 @@
     <row r="19">
       <c r="A19" s="23" t="inlineStr">
         <is>
-          <t>DHAN-231261009113409+321261009657109+321261009657509+321261009658009+231261009114909+231261009115109+231261009115209+231261009115409+321261009660209+321261009660409+321261009661009+231261009116709+321261009661709+321261009662109+321261009662509</t>
+          <t>DHAN-321261009656509+321261009657209+231261009114209+231261009114409+231261009114609+321261009658609+321261009659109+321261009659509+231261009115709+321261009660509+231261009116209</t>
         </is>
       </c>
       <c r="B19" s="23" t="inlineStr">
         <is>
-          <t>SMCGLOBAL</t>
+          <t>RSYSTEMS</t>
         </is>
       </c>
       <c r="C19" s="23" t="inlineStr">
@@ -1974,16 +1974,16 @@
         <v>46304</v>
       </c>
       <c r="E19" s="25" t="n">
-        <v>115.2011</v>
+        <v>274.9019</v>
       </c>
       <c r="F19" s="26" t="n">
-        <v>864</v>
+        <v>727</v>
       </c>
       <c r="G19" s="24" t="n">
         <v>46307</v>
       </c>
       <c r="H19" s="25" t="n">
-        <v>115.68</v>
+        <v>263</v>
       </c>
       <c r="I19" s="21">
         <f>IF(OR($B19="",$H19=""),"",IF($C19="LONG",($H19-$E19)*$F19,($E19-$H19)*$F19))</f>
@@ -1994,7 +1994,7 @@
         <v/>
       </c>
       <c r="K19" s="4" t="n">
-        <v>132.93</v>
+        <v>485.75</v>
       </c>
       <c r="L19" s="21">
         <f>IF(OR($B19="",$I19=""),"",$I19-IF($K19="",0,$K19))</f>
@@ -2010,19 +2010,19 @@
       </c>
       <c r="O19" s="23" t="inlineStr">
         <is>
-          <t>5-10</t>
+          <t>10-15</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261012636809+23126101284009+221261012637709+34126101276009+23126101284709+23126101285909+23126101286009+34126101277509+34126101277709+23126101286509+34126101278209+321261012631509+34126101278309+321261012632109+321261012632509</t>
+          <t>DHAN-231261009113309+231261009113509+231261009114309+231261009114509+231261009114809+321261009658809+321261009659609+231261009115609+231261009116009+321261009660909+231261009116609+321261009661609+321261009662209+231261009117509+321261009662909+231261009117909</t>
         </is>
       </c>
       <c r="B20" s="23" t="inlineStr">
         <is>
-          <t>BLUSPRING</t>
+          <t>SAKSOFT</t>
         </is>
       </c>
       <c r="C20" s="23" t="inlineStr">
@@ -2031,16 +2031,20 @@
         </is>
       </c>
       <c r="D20" s="24" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E20" s="25" t="n">
+        <v>138.9161</v>
+      </c>
+      <c r="F20" s="26" t="n">
+        <v>1443</v>
+      </c>
+      <c r="G20" s="24" t="n">
         <v>46307</v>
       </c>
-      <c r="E20" s="25" t="n">
-        <v>157.2127</v>
-      </c>
-      <c r="F20" s="26" t="n">
-        <v>1095</v>
-      </c>
-      <c r="G20" s="24" t="inlineStr"/>
-      <c r="H20" s="25" t="inlineStr"/>
+      <c r="H20" s="25" t="n">
+        <v>140.87</v>
+      </c>
       <c r="I20" s="21">
         <f>IF(OR($B20="",$H20=""),"",IF($C20="LONG",($H20-$E20)*$F20,($E20-$H20)*$F20))</f>
         <v/>
@@ -2050,7 +2054,7 @@
         <v/>
       </c>
       <c r="K20" s="4" t="n">
-        <v>50.15</v>
+        <v>482.51</v>
       </c>
       <c r="L20" s="21">
         <f>IF(OR($B20="",$I20=""),"",$I20-IF($K20="",0,$K20))</f>
@@ -2073,12 +2077,12 @@
     <row r="21">
       <c r="A21" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261012636709+221261012637509+321261012626709+221261012638409+23126101284609+34126101276109+221261012640409+34126101277309+34126101277409+221261012641109+321261012630109</t>
+          <t>DHAN-231261009113409+321261009657109+321261009657509+321261009658009+231261009114909+231261009115109+231261009115209+231261009115409+321261009660209+321261009660409+321261009661009+231261009116709+321261009661709+321261009662109+321261009662509</t>
         </is>
       </c>
       <c r="B21" s="23" t="inlineStr">
         <is>
-          <t>GOODLUCK</t>
+          <t>SMCGLOBAL</t>
         </is>
       </c>
       <c r="C21" s="23" t="inlineStr">
@@ -2087,16 +2091,20 @@
         </is>
       </c>
       <c r="D21" s="24" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E21" s="25" t="n">
+        <v>115.2011</v>
+      </c>
+      <c r="F21" s="26" t="n">
+        <v>864</v>
+      </c>
+      <c r="G21" s="24" t="n">
         <v>46307</v>
       </c>
-      <c r="E21" s="25" t="n">
-        <v>564.8409</v>
-      </c>
-      <c r="F21" s="26" t="n">
-        <v>303</v>
-      </c>
-      <c r="G21" s="24" t="inlineStr"/>
-      <c r="H21" s="25" t="inlineStr"/>
+      <c r="H21" s="25" t="n">
+        <v>115.68</v>
+      </c>
       <c r="I21" s="21">
         <f>IF(OR($B21="",$H21=""),"",IF($C21="LONG",($H21-$E21)*$F21,($E21-$H21)*$F21))</f>
         <v/>
@@ -2106,7 +2114,7 @@
         <v/>
       </c>
       <c r="K21" s="4" t="n">
-        <v>50.15</v>
+        <v>132.93</v>
       </c>
       <c r="L21" s="21">
         <f>IF(OR($B21="",$I21=""),"",$I21-IF($K21="",0,$K21))</f>
@@ -2122,19 +2130,19 @@
       </c>
       <c r="O21" s="23" t="inlineStr">
         <is>
-          <t>10-15</t>
+          <t>5-10</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="23" t="inlineStr">
         <is>
-          <t>DHAN-23126100860109+221261008541409+34126100865109+34126100865209+23126100860209+321261008684009+221261008543809+34126100865509+34126100865709+321261008684809+321261008685109+321261008685409+34126100865909+34126100866009+221261008545809+221261008545909+34126100866109+23126100860509</t>
+          <t>DHAN-321261009656609+231261009113809+231261009114109+321261009658109+231261009115509+231261009116409+231261009116809+231261009117009+231261009117209+231261009117609+231261009117709+231261009118009+231261009118109</t>
         </is>
       </c>
       <c r="B22" s="23" t="inlineStr">
         <is>
-          <t>KOTIC</t>
+          <t>SUNCLAY</t>
         </is>
       </c>
       <c r="C22" s="23" t="inlineStr">
@@ -2143,16 +2151,20 @@
         </is>
       </c>
       <c r="D22" s="24" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E22" s="25" t="n">
-        <v>157.0151</v>
+        <v>1228.0927</v>
       </c>
       <c r="F22" s="26" t="n">
-        <v>858</v>
-      </c>
-      <c r="G22" s="24" t="inlineStr"/>
-      <c r="H22" s="25" t="inlineStr"/>
+        <v>164</v>
+      </c>
+      <c r="G22" s="24" t="n">
+        <v>46307</v>
+      </c>
+      <c r="H22" s="25" t="n">
+        <v>1195.11</v>
+      </c>
       <c r="I22" s="21">
         <f>IF(OR($B22="",$H22=""),"",IF($C22="LONG",($H22-$E22)*$F22,($E22-$H22)*$F22))</f>
         <v/>
@@ -2162,7 +2174,7 @@
         <v/>
       </c>
       <c r="K22" s="4" t="n">
-        <v>175</v>
+        <v>471.71</v>
       </c>
       <c r="L22" s="21">
         <f>IF(OR($B22="",$I22=""),"",$I22-IF($K22="",0,$K22))</f>
@@ -2178,19 +2190,19 @@
       </c>
       <c r="O22" s="23" t="inlineStr">
         <is>
-          <t>5-10</t>
+          <t>10-15</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261009656409+231261009113609+231261009114009+321261009657909+231261009114709+231261009115009+321261009659009+231261009115809+321261009660609+321261009660809+321261009661309+231261009117309+321261009662609+321261009663009+231261009117809+321261009663809+231261009118209</t>
+          <t>DHAN-221261012636809+23126101284009+221261012637709+34126101276009+23126101284709+23126101285909+23126101286009+34126101277509+34126101277709+23126101286509+34126101278209+321261012631509+34126101278309+321261012632109+321261012632509</t>
         </is>
       </c>
       <c r="B23" s="23" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>BLUSPRING</t>
         </is>
       </c>
       <c r="C23" s="23" t="inlineStr">
@@ -2199,13 +2211,13 @@
         </is>
       </c>
       <c r="D23" s="24" t="n">
-        <v>46304</v>
+        <v>46307</v>
       </c>
       <c r="E23" s="25" t="n">
-        <v>20.9882</v>
+        <v>157.2127</v>
       </c>
       <c r="F23" s="26" t="n">
-        <v>3589</v>
+        <v>1095</v>
       </c>
       <c r="G23" s="24" t="inlineStr"/>
       <c r="H23" s="25" t="inlineStr"/>
@@ -2218,7 +2230,7 @@
         <v/>
       </c>
       <c r="K23" s="4" t="n">
-        <v>104.2</v>
+        <v>50.15</v>
       </c>
       <c r="L23" s="21">
         <f>IF(OR($B23="",$I23=""),"",$I23-IF($K23="",0,$K23))</f>
@@ -2241,12 +2253,12 @@
     <row r="24">
       <c r="A24" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261012625809+321261012626209+23126101284209+23126101284309+321261012626909+34126101276209+34126101277109+321261012628809+221261012640809+23126101286309+34126101278009+321261012630809+221261012643209</t>
+          <t>DHAN-221261012636709+221261012637509+321261012626709+221261012638409+23126101284609+34126101276109+221261012640409+34126101277309+34126101277409+221261012641109+321261012630109</t>
         </is>
       </c>
       <c r="B24" s="23" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>GOODLUCK</t>
         </is>
       </c>
       <c r="C24" s="23" t="inlineStr">
@@ -2258,10 +2270,10 @@
         <v>46307</v>
       </c>
       <c r="E24" s="25" t="n">
-        <v>22.8999</v>
+        <v>564.8409</v>
       </c>
       <c r="F24" s="26" t="n">
-        <v>3742</v>
+        <v>303</v>
       </c>
       <c r="G24" s="24" t="inlineStr"/>
       <c r="H24" s="25" t="inlineStr"/>
@@ -2274,7 +2286,7 @@
         <v/>
       </c>
       <c r="K24" s="4" t="n">
-        <v>14.75</v>
+        <v>50.15</v>
       </c>
       <c r="L24" s="21">
         <f>IF(OR($B24="",$I24=""),"",$I24-IF($K24="",0,$K24))</f>
@@ -2290,19 +2302,19 @@
       </c>
       <c r="O24" s="23" t="inlineStr">
         <is>
-          <t>5-10</t>
+          <t>10-15</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="23" t="inlineStr">
         <is>
-          <t>DHAN-34126101275609+321261012626309+221261012637809+34126101275809+23126101284509+321261012627209+34126101277009+34126101277209+34126101277609+221261012641209+321261012630309+23126101287209+321261012631409+321261012631709+321261012632009</t>
+          <t>DHAN-321261012625809+321261012626209+23126101284209+23126101284309+321261012626909+34126101276209+34126101277109+321261012628809+221261012640809+23126101286309+34126101278009+321261012630809+221261012643209</t>
         </is>
       </c>
       <c r="B25" s="23" t="inlineStr">
         <is>
-          <t>PRINCEPIPE</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="C25" s="23" t="inlineStr">
@@ -2314,10 +2326,10 @@
         <v>46307</v>
       </c>
       <c r="E25" s="25" t="n">
-        <v>267.6149</v>
+        <v>22.8999</v>
       </c>
       <c r="F25" s="26" t="n">
-        <v>641</v>
+        <v>3742</v>
       </c>
       <c r="G25" s="24" t="inlineStr"/>
       <c r="H25" s="25" t="inlineStr"/>
@@ -2330,7 +2342,7 @@
         <v/>
       </c>
       <c r="K25" s="4" t="n">
-        <v>50.15</v>
+        <v>14.75</v>
       </c>
       <c r="L25" s="21">
         <f>IF(OR($B25="",$I25=""),"",$I25-IF($K25="",0,$K25))</f>
@@ -2353,12 +2365,12 @@
     <row r="26">
       <c r="A26" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261009656609+231261009113809+231261009114109+321261009658109+231261009115509+231261009116409+231261009116809+231261009117009+231261009117209+231261009117609+231261009117709+231261009118009+231261009118109</t>
+          <t>DHAN-34126101275609+321261012626309+221261012637809+34126101275809+23126101284509+321261012627209+34126101277009+34126101277209+34126101277609+221261012641209+321261012630309+23126101287209+321261012631409+321261012631709+321261012632009</t>
         </is>
       </c>
       <c r="B26" s="23" t="inlineStr">
         <is>
-          <t>SUNCLAY</t>
+          <t>PRINCEPIPE</t>
         </is>
       </c>
       <c r="C26" s="23" t="inlineStr">
@@ -2367,13 +2379,13 @@
         </is>
       </c>
       <c r="D26" s="24" t="n">
-        <v>46304</v>
+        <v>46307</v>
       </c>
       <c r="E26" s="25" t="n">
-        <v>1228.0927</v>
+        <v>267.6149</v>
       </c>
       <c r="F26" s="26" t="n">
-        <v>164</v>
+        <v>641</v>
       </c>
       <c r="G26" s="24" t="inlineStr"/>
       <c r="H26" s="25" t="inlineStr"/>
@@ -2386,7 +2398,7 @@
         <v/>
       </c>
       <c r="K26" s="4" t="n">
-        <v>471.71</v>
+        <v>50.15</v>
       </c>
       <c r="L26" s="21">
         <f>IF(OR($B26="",$I26=""),"",$I26-IF($K26="",0,$K26))</f>
@@ -2402,7 +2414,7 @@
       </c>
       <c r="O26" s="23" t="inlineStr">
         <is>
-          <t>10-15</t>
+          <t>5-10</t>
         </is>
       </c>
     </row>
@@ -32072,12 +32084,12 @@
     <row r="15">
       <c r="A15" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261008541309+221261008541509+321261008683209+221261008542109+34126100865309+34126100865409+221261008543409+221261008543909+221261008544309+34126100865609+221261008545009+23126100860309+34126100865809+23126100860409</t>
+          <t>DHAN-23126100860109+221261008541409+34126100865109+34126100865209+23126100860209+321261008684009+221261008543809+34126100865509+34126100865709+321261008684809+321261008685109+321261008685409+34126100865909+34126100866009+221261008545809+221261008545909+34126100866109+23126100860509</t>
         </is>
       </c>
       <c r="B15" s="23" t="inlineStr">
         <is>
-          <t>PNGSREVA</t>
+          <t>KOTIC</t>
         </is>
       </c>
       <c r="C15" s="23" t="inlineStr">
@@ -32089,22 +32101,22 @@
         <v>46304</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>65.06</v>
+        <v>0</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>147.69</v>
+        <v>270.22</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>9.15</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>0.3</v>
+        <v>0.27</v>
       </c>
       <c r="I15" s="4" t="n">
-        <v>4.51</v>
+        <v>20.49</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>13.41</v>
+        <v>1.54</v>
       </c>
       <c r="K15" s="4" t="n">
         <v>14.75</v>
@@ -32123,12 +32135,12 @@
     <row r="16">
       <c r="A16" s="23" t="inlineStr">
         <is>
-          <t>DHAN-231261009113209+231261009113709+231261009113909+321261009657809+321261009658409+321261009658709+231261009115309+321261009659409+321261009660109+231261009116109+231261009116309+231261009116509+231261009117109</t>
+          <t>DHAN-221261008541309+221261008541509+321261008683209+221261008542109+34126100865309+34126100865409+221261008543409+221261008543909+221261008544309+34126100865609+221261008545009+23126100860309+34126100865809+23126100860409</t>
         </is>
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>INOXGREEN</t>
+          <t>PNGSREVA</t>
         </is>
       </c>
       <c r="C16" s="23" t="inlineStr">
@@ -32137,34 +32149,34 @@
         </is>
       </c>
       <c r="D16" s="24" t="n">
-        <v>46307</v>
+        <v>46304</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>60.1</v>
+        <v>65.06</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>200.23</v>
+        <v>147.69</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>6.15</v>
+        <v>9.15</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="I16" s="4" t="n">
-        <v>30.04</v>
+        <v>4.51</v>
       </c>
       <c r="J16" s="4" t="n">
-        <v>11.96</v>
+        <v>13.41</v>
       </c>
       <c r="K16" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L16" s="4" t="n">
-        <v>35.4</v>
+        <v>0</v>
       </c>
       <c r="M16" s="4" t="n">
-        <v>123.27</v>
+        <v>0</v>
       </c>
       <c r="N16" s="21">
         <f>SUM(E16:M16)</f>
@@ -32174,12 +32186,12 @@
     <row r="17">
       <c r="A17" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261009656509+321261009657209+231261009114209+231261009114409+231261009114609+321261009658609+321261009659109+321261009659509+231261009115709+321261009660509+231261009116209</t>
+          <t>DHAN-231261009113209+231261009113709+231261009113909+321261009657809+321261009658409+321261009658709+231261009115309+321261009659409+321261009660109+231261009116109+231261009116309+231261009116509+231261009117109</t>
         </is>
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>RSYSTEMS</t>
+          <t>INOXGREEN</t>
         </is>
       </c>
       <c r="C17" s="23" t="inlineStr">
@@ -32191,22 +32203,22 @@
         <v>46307</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>59.98</v>
+        <v>60.1</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>199.85</v>
+        <v>200.23</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>6.14</v>
+        <v>6.15</v>
       </c>
       <c r="H17" s="4" t="n">
         <v>0.2</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>29.98</v>
+        <v>30.04</v>
       </c>
       <c r="J17" s="4" t="n">
-        <v>11.94</v>
+        <v>11.96</v>
       </c>
       <c r="K17" s="4" t="n">
         <v>14.75</v>
@@ -32215,7 +32227,7 @@
         <v>35.4</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>127.52</v>
+        <v>123.27</v>
       </c>
       <c r="N17" s="21">
         <f>SUM(E17:M17)</f>
@@ -32225,12 +32237,12 @@
     <row r="18">
       <c r="A18" s="23" t="inlineStr">
         <is>
-          <t>DHAN-231261009113309+231261009113509+231261009114309+231261009114509+231261009114809+321261009658809+321261009659609+231261009115609+231261009116009+321261009660909+231261009116609+321261009661609+321261009662209+231261009117509+321261009662909+231261009117909</t>
+          <t>DHAN-321261009656409+231261009113609+231261009114009+321261009657909+231261009114709+231261009115009+321261009659009+231261009115809+321261009660609+321261009660809+321261009661309+231261009117309+321261009662609+321261009663009+231261009117809+321261009663809+231261009118209</t>
         </is>
       </c>
       <c r="B18" s="23" t="inlineStr">
         <is>
-          <t>SAKSOFT</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="C18" s="23" t="inlineStr">
@@ -32242,31 +32254,31 @@
         <v>46307</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>60.11</v>
+        <v>0</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>200.46</v>
+        <v>75.33</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>6.15</v>
+        <v>2.31</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>0.2</v>
+        <v>0.08</v>
       </c>
       <c r="I18" s="4" t="n">
-        <v>30.07</v>
+        <v>11.3</v>
       </c>
       <c r="J18" s="4" t="n">
-        <v>11.96</v>
+        <v>0.43</v>
       </c>
       <c r="K18" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L18" s="4" t="n">
-        <v>35.4</v>
+        <v>0</v>
       </c>
       <c r="M18" s="4" t="n">
-        <v>123.4</v>
+        <v>0</v>
       </c>
       <c r="N18" s="21">
         <f>SUM(E18:M18)</f>
@@ -32276,12 +32288,12 @@
     <row r="19">
       <c r="A19" s="23" t="inlineStr">
         <is>
-          <t>DHAN-231261009113409+321261009657109+321261009657509+321261009658009+231261009114909+231261009115109+231261009115209+231261009115409+321261009660209+321261009660409+321261009661009+231261009116709+321261009661709+321261009662109+321261009662509</t>
+          <t>DHAN-321261009656509+321261009657209+231261009114209+231261009114409+231261009114609+321261009658609+321261009659109+321261009659509+231261009115709+321261009660509+231261009116209</t>
         </is>
       </c>
       <c r="B19" s="23" t="inlineStr">
         <is>
-          <t>SMCGLOBAL</t>
+          <t>RSYSTEMS</t>
         </is>
       </c>
       <c r="C19" s="23" t="inlineStr">
@@ -32293,31 +32305,31 @@
         <v>46307</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>0</v>
+        <v>59.98</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>99.53</v>
+        <v>199.85</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>3.06</v>
+        <v>6.14</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I19" s="4" t="n">
-        <v>14.93</v>
+        <v>29.98</v>
       </c>
       <c r="J19" s="4" t="n">
-        <v>0.57</v>
+        <v>11.94</v>
       </c>
       <c r="K19" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L19" s="4" t="n">
-        <v>0</v>
+        <v>35.4</v>
       </c>
       <c r="M19" s="4" t="n">
-        <v>0</v>
+        <v>127.52</v>
       </c>
       <c r="N19" s="21">
         <f>SUM(E19:M19)</f>
@@ -32327,12 +32339,12 @@
     <row r="20">
       <c r="A20" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261012636809+23126101284009+221261012637709+34126101276009+23126101284709+23126101285909+23126101286009+34126101277509+34126101277709+23126101286509+34126101278209+321261012631509+34126101278309+321261012632109+321261012632509</t>
+          <t>DHAN-231261009113309+231261009113509+231261009114309+231261009114509+231261009114809+321261009658809+321261009659609+231261009115609+231261009116009+321261009660909+231261009116609+321261009661609+321261009662209+231261009117509+321261009662909+231261009117909</t>
         </is>
       </c>
       <c r="B20" s="23" t="inlineStr">
         <is>
-          <t>BLUSPRING</t>
+          <t>SAKSOFT</t>
         </is>
       </c>
       <c r="C20" s="23" t="inlineStr">
@@ -32340,24 +32352,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D20" s="24" t="inlineStr"/>
+      <c r="D20" s="24" t="n">
+        <v>46307</v>
+      </c>
       <c r="E20" s="4" t="n">
-        <v>0</v>
+        <v>60.11</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>0</v>
+        <v>200.46</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0</v>
+        <v>6.15</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>0</v>
+        <v>30.07</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>0</v>
+        <v>11.96</v>
       </c>
       <c r="K20" s="4" t="n">
         <v>14.75</v>
@@ -32366,7 +32380,7 @@
         <v>35.4</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>0</v>
+        <v>123.4</v>
       </c>
       <c r="N20" s="21">
         <f>SUM(E20:M20)</f>
@@ -32376,12 +32390,12 @@
     <row r="21">
       <c r="A21" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261012636709+221261012637509+321261012626709+221261012638409+23126101284609+34126101276109+221261012640409+34126101277309+34126101277409+221261012641109+321261012630109</t>
+          <t>DHAN-231261009113409+321261009657109+321261009657509+321261009658009+231261009114909+231261009115109+231261009115209+231261009115409+321261009660209+321261009660409+321261009661009+231261009116709+321261009661709+321261009662109+321261009662509</t>
         </is>
       </c>
       <c r="B21" s="23" t="inlineStr">
         <is>
-          <t>GOODLUCK</t>
+          <t>SMCGLOBAL</t>
         </is>
       </c>
       <c r="C21" s="23" t="inlineStr">
@@ -32389,30 +32403,32 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D21" s="24" t="inlineStr"/>
+      <c r="D21" s="24" t="n">
+        <v>46307</v>
+      </c>
       <c r="E21" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>0</v>
+        <v>99.53</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>0</v>
+        <v>3.06</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="I21" s="4" t="n">
-        <v>0</v>
+        <v>14.93</v>
       </c>
       <c r="J21" s="4" t="n">
-        <v>0</v>
+        <v>0.57</v>
       </c>
       <c r="K21" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L21" s="4" t="n">
-        <v>35.4</v>
+        <v>0</v>
       </c>
       <c r="M21" s="4" t="n">
         <v>0</v>
@@ -32425,12 +32441,12 @@
     <row r="22">
       <c r="A22" s="23" t="inlineStr">
         <is>
-          <t>DHAN-23126100860109+221261008541409+34126100865109+34126100865209+23126100860209+321261008684009+221261008543809+34126100865509+34126100865709+321261008684809+321261008685109+321261008685409+34126100865909+34126100866009+221261008545809+221261008545909+34126100866109+23126100860509</t>
+          <t>DHAN-321261009656609+231261009113809+231261009114109+321261009658109+231261009115509+231261009116409+231261009116809+231261009117009+231261009117209+231261009117609+231261009117709+231261009118009+231261009118109</t>
         </is>
       </c>
       <c r="B22" s="23" t="inlineStr">
         <is>
-          <t>KOTIC</t>
+          <t>SUNCLAY</t>
         </is>
       </c>
       <c r="C22" s="23" t="inlineStr">
@@ -32438,33 +32454,35 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D22" s="24" t="inlineStr"/>
+      <c r="D22" s="24" t="n">
+        <v>46307</v>
+      </c>
       <c r="E22" s="4" t="n">
-        <v>0</v>
+        <v>49.11</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>134.72</v>
+        <v>201.41</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>4.14</v>
+        <v>6.18</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>0.13</v>
+        <v>0.2</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>20.49</v>
+        <v>30.68</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>0.77</v>
+        <v>9.99</v>
       </c>
       <c r="K22" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L22" s="4" t="n">
-        <v>0</v>
+        <v>35.4</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>0</v>
+        <v>123.99</v>
       </c>
       <c r="N22" s="21">
         <f>SUM(E22:M22)</f>
@@ -32474,12 +32492,12 @@
     <row r="23">
       <c r="A23" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261009656409+231261009113609+231261009114009+321261009657909+231261009114709+231261009115009+321261009659009+231261009115809+321261009660609+321261009660809+321261009661309+231261009117309+321261009662609+321261009663009+231261009117809+321261009663809+231261009118209</t>
+          <t>DHAN-221261012636809+23126101284009+221261012637709+34126101276009+23126101284709+23126101285909+23126101286009+34126101277509+34126101277709+23126101286509+34126101278209+321261012631509+34126101278309+321261012632109+321261012632509</t>
         </is>
       </c>
       <c r="B23" s="23" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>BLUSPRING</t>
         </is>
       </c>
       <c r="C23" s="23" t="inlineStr">
@@ -32492,25 +32510,25 @@
         <v>0</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>75.33</v>
+        <v>0</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>2.31</v>
+        <v>0</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>0.08</v>
+        <v>0</v>
       </c>
       <c r="I23" s="4" t="n">
-        <v>11.3</v>
+        <v>0</v>
       </c>
       <c r="J23" s="4" t="n">
-        <v>0.43</v>
+        <v>0</v>
       </c>
       <c r="K23" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L23" s="4" t="n">
-        <v>0</v>
+        <v>35.4</v>
       </c>
       <c r="M23" s="4" t="n">
         <v>0</v>
@@ -32523,12 +32541,12 @@
     <row r="24">
       <c r="A24" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261012625809+321261012626209+23126101284209+23126101284309+321261012626909+34126101276209+34126101277109+321261012628809+221261012640809+23126101286309+34126101278009+321261012630809+221261012643209</t>
+          <t>DHAN-221261012636709+221261012637509+321261012626709+221261012638409+23126101284609+34126101276109+221261012640409+34126101277309+34126101277409+221261012641109+321261012630109</t>
         </is>
       </c>
       <c r="B24" s="23" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>GOODLUCK</t>
         </is>
       </c>
       <c r="C24" s="23" t="inlineStr">
@@ -32559,7 +32577,7 @@
         <v>14.75</v>
       </c>
       <c r="L24" s="4" t="n">
-        <v>0</v>
+        <v>35.4</v>
       </c>
       <c r="M24" s="4" t="n">
         <v>0</v>
@@ -32572,12 +32590,12 @@
     <row r="25">
       <c r="A25" s="23" t="inlineStr">
         <is>
-          <t>DHAN-34126101275609+321261012626309+221261012637809+34126101275809+23126101284509+321261012627209+34126101277009+34126101277209+34126101277609+221261012641209+321261012630309+23126101287209+321261012631409+321261012631709+321261012632009</t>
+          <t>DHAN-321261012625809+321261012626209+23126101284209+23126101284309+321261012626909+34126101276209+34126101277109+321261012628809+221261012640809+23126101286309+34126101278009+321261012630809+221261012643209</t>
         </is>
       </c>
       <c r="B25" s="23" t="inlineStr">
         <is>
-          <t>PRINCEPIPE</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="C25" s="23" t="inlineStr">
@@ -32608,7 +32626,7 @@
         <v>14.75</v>
       </c>
       <c r="L25" s="4" t="n">
-        <v>35.4</v>
+        <v>0</v>
       </c>
       <c r="M25" s="4" t="n">
         <v>0</v>
@@ -32621,12 +32639,12 @@
     <row r="26">
       <c r="A26" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261009656609+231261009113809+231261009114109+321261009658109+231261009115509+231261009116409+231261009116809+231261009117009+231261009117209+231261009117609+231261009117709+231261009118009+231261009118109</t>
+          <t>DHAN-34126101275609+321261012626309+221261012637809+34126101275809+23126101284509+321261012627209+34126101277009+34126101277209+34126101277609+221261012641209+321261012630309+23126101287209+321261012631409+321261012631709+321261012632009</t>
         </is>
       </c>
       <c r="B26" s="23" t="inlineStr">
         <is>
-          <t>SUNCLAY</t>
+          <t>PRINCEPIPE</t>
         </is>
       </c>
       <c r="C26" s="23" t="inlineStr">
@@ -32636,22 +32654,22 @@
       </c>
       <c r="D26" s="24" t="inlineStr"/>
       <c r="E26" s="4" t="n">
-        <v>49.11</v>
+        <v>0</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>201.41</v>
+        <v>0</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>6.18</v>
+        <v>0</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="I26" s="4" t="n">
-        <v>30.68</v>
+        <v>0</v>
       </c>
       <c r="J26" s="4" t="n">
-        <v>9.99</v>
+        <v>0</v>
       </c>
       <c r="K26" s="4" t="n">
         <v>14.75</v>
@@ -32660,7 +32678,7 @@
         <v>35.4</v>
       </c>
       <c r="M26" s="4" t="n">
-        <v>123.99</v>
+        <v>0</v>
       </c>
       <c r="N26" s="21">
         <f>SUM(E26:M26)</f>

</xml_diff>

<commit_message>
Data update — 2026-10-13 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_oct2026.xlsx
+++ b/results/strategy_pnl_oct2026.xlsx
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trade Log'!$A$3:$O$503</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1214,7 +1214,7 @@
         <v/>
       </c>
       <c r="K6" s="4" t="n">
-        <v>962.8200000000001</v>
+        <v>964.78</v>
       </c>
       <c r="L6" s="21">
         <f>IF(OR($B6="",$I6=""),"",$I6-IF($K6="",0,$K6))</f>
@@ -1274,7 +1274,7 @@
         <v/>
       </c>
       <c r="K7" s="4" t="n">
-        <v>823.7</v>
+        <v>824.88</v>
       </c>
       <c r="L7" s="21">
         <f>IF(OR($B7="",$I7=""),"",$I7-IF($K7="",0,$K7))</f>
@@ -1334,7 +1334,7 @@
         <v/>
       </c>
       <c r="K8" s="4" t="n">
-        <v>834.92</v>
+        <v>836.1</v>
       </c>
       <c r="L8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($K8="",0,$K8))</f>
@@ -1394,7 +1394,7 @@
         <v/>
       </c>
       <c r="K9" s="4" t="n">
-        <v>977.26</v>
+        <v>979.22</v>
       </c>
       <c r="L9" s="21">
         <f>IF(OR($B9="",$I9=""),"",$I9-IF($K9="",0,$K9))</f>
@@ -1454,7 +1454,7 @@
         <v/>
       </c>
       <c r="K10" s="4" t="n">
-        <v>949.53</v>
+        <v>951.17</v>
       </c>
       <c r="L10" s="21">
         <f>IF(OR($B10="",$I10=""),"",$I10-IF($K10="",0,$K10))</f>
@@ -1514,7 +1514,7 @@
         <v/>
       </c>
       <c r="K11" s="4" t="n">
-        <v>673.03</v>
+        <v>673.6900000000001</v>
       </c>
       <c r="L11" s="21">
         <f>IF(OR($B11="",$I11=""),"",$I11-IF($K11="",0,$K11))</f>
@@ -1574,7 +1574,7 @@
         <v/>
       </c>
       <c r="K12" s="4" t="n">
-        <v>734.54</v>
+        <v>735.3200000000001</v>
       </c>
       <c r="L12" s="21">
         <f>IF(OR($B12="",$I12=""),"",$I12-IF($K12="",0,$K12))</f>
@@ -1634,7 +1634,7 @@
         <v/>
       </c>
       <c r="K13" s="4" t="n">
-        <v>644.73</v>
+        <v>645.21</v>
       </c>
       <c r="L13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($K13="",0,$K13))</f>
@@ -1694,7 +1694,7 @@
         <v/>
       </c>
       <c r="K14" s="4" t="n">
-        <v>665.7</v>
+        <v>654.64</v>
       </c>
       <c r="L14" s="21">
         <f>IF(OR($B14="",$I14=""),"",$I14-IF($K14="",0,$K14))</f>
@@ -1874,7 +1874,7 @@
         <v/>
       </c>
       <c r="K17" s="4" t="n">
-        <v>482.09</v>
+        <v>651.58</v>
       </c>
       <c r="L17" s="21">
         <f>IF(OR($B17="",$I17=""),"",$I17-IF($K17="",0,$K17))</f>
@@ -1934,7 +1934,7 @@
         <v/>
       </c>
       <c r="K18" s="4" t="n">
-        <v>104.2</v>
+        <v>150.64</v>
       </c>
       <c r="L18" s="21">
         <f>IF(OR($B18="",$I18=""),"",$I18-IF($K18="",0,$K18))</f>
@@ -1994,7 +1994,7 @@
         <v/>
       </c>
       <c r="K19" s="4" t="n">
-        <v>485.75</v>
+        <v>707.5</v>
       </c>
       <c r="L19" s="21">
         <f>IF(OR($B19="",$I19=""),"",$I19-IF($K19="",0,$K19))</f>
@@ -2054,7 +2054,7 @@
         <v/>
       </c>
       <c r="K20" s="4" t="n">
-        <v>482.51</v>
+        <v>716.86</v>
       </c>
       <c r="L20" s="21">
         <f>IF(OR($B20="",$I20=""),"",$I20-IF($K20="",0,$K20))</f>
@@ -2114,7 +2114,7 @@
         <v/>
       </c>
       <c r="K21" s="4" t="n">
-        <v>132.93</v>
+        <v>236.62</v>
       </c>
       <c r="L21" s="21">
         <f>IF(OR($B21="",$I21=""),"",$I21-IF($K21="",0,$K21))</f>
@@ -2174,7 +2174,7 @@
         <v/>
       </c>
       <c r="K22" s="4" t="n">
-        <v>471.71</v>
+        <v>698.64</v>
       </c>
       <c r="L22" s="21">
         <f>IF(OR($B22="",$I22=""),"",$I22-IF($K22="",0,$K22))</f>
@@ -2219,8 +2219,12 @@
       <c r="F23" s="26" t="n">
         <v>1095</v>
       </c>
-      <c r="G23" s="24" t="inlineStr"/>
-      <c r="H23" s="25" t="inlineStr"/>
+      <c r="G23" s="24" t="n">
+        <v>46308</v>
+      </c>
+      <c r="H23" s="25" t="n">
+        <v>162.33</v>
+      </c>
       <c r="I23" s="21">
         <f>IF(OR($B23="",$H23=""),"",IF($C23="LONG",($H23-$E23)*$F23,($E23-$H23)*$F23))</f>
         <v/>
@@ -2230,7 +2234,7 @@
         <v/>
       </c>
       <c r="K23" s="4" t="n">
-        <v>50.15</v>
+        <v>344.89</v>
       </c>
       <c r="L23" s="21">
         <f>IF(OR($B23="",$I23=""),"",$I23-IF($K23="",0,$K23))</f>
@@ -2253,30 +2257,34 @@
     <row r="24">
       <c r="A24" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261012636709+221261012637509+321261012626709+221261012638409+23126101284609+34126101276109+221261012640409+34126101277309+34126101277409+221261012641109+321261012630109</t>
+          <t>DHAN-321261013231409</t>
         </is>
       </c>
       <c r="B24" s="23" t="inlineStr">
         <is>
-          <t>GOODLUCK</t>
+          <t>BLUSPRING</t>
         </is>
       </c>
       <c r="C24" s="23" t="inlineStr">
         <is>
-          <t>LONG</t>
+          <t>SHORT</t>
         </is>
       </c>
       <c r="D24" s="24" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="E24" s="25" t="n">
-        <v>564.8409</v>
+        <v>162.42</v>
       </c>
       <c r="F24" s="26" t="n">
-        <v>303</v>
-      </c>
-      <c r="G24" s="24" t="inlineStr"/>
-      <c r="H24" s="25" t="inlineStr"/>
+        <v>1095</v>
+      </c>
+      <c r="G24" s="24" t="n">
+        <v>46308</v>
+      </c>
+      <c r="H24" s="25" t="n">
+        <v>158.62</v>
+      </c>
       <c r="I24" s="21">
         <f>IF(OR($B24="",$H24=""),"",IF($C24="LONG",($H24-$E24)*$F24,($E24-$H24)*$F24))</f>
         <v/>
@@ -2286,7 +2294,7 @@
         <v/>
       </c>
       <c r="K24" s="4" t="n">
-        <v>50.15</v>
+        <v>0</v>
       </c>
       <c r="L24" s="21">
         <f>IF(OR($B24="",$I24=""),"",$I24-IF($K24="",0,$K24))</f>
@@ -2302,19 +2310,19 @@
       </c>
       <c r="O24" s="23" t="inlineStr">
         <is>
-          <t>10-15</t>
+          <t>5-10</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261012625809+321261012626209+23126101284209+23126101284309+321261012626909+34126101276209+34126101277109+321261012628809+221261012640809+23126101286309+34126101278009+321261012630809+221261012643209</t>
+          <t>DHAN-221261012636709+221261012637509+321261012626709+221261012638409+23126101284609+34126101276109+221261012640409+34126101277309+34126101277409+221261012641109+321261012630109</t>
         </is>
       </c>
       <c r="B25" s="23" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>GOODLUCK</t>
         </is>
       </c>
       <c r="C25" s="23" t="inlineStr">
@@ -2326,13 +2334,17 @@
         <v>46307</v>
       </c>
       <c r="E25" s="25" t="n">
-        <v>22.8999</v>
+        <v>564.8409</v>
       </c>
       <c r="F25" s="26" t="n">
-        <v>3742</v>
-      </c>
-      <c r="G25" s="24" t="inlineStr"/>
-      <c r="H25" s="25" t="inlineStr"/>
+        <v>303</v>
+      </c>
+      <c r="G25" s="24" t="n">
+        <v>46308</v>
+      </c>
+      <c r="H25" s="25" t="n">
+        <v>581.02</v>
+      </c>
       <c r="I25" s="21">
         <f>IF(OR($B25="",$H25=""),"",IF($C25="LONG",($H25-$E25)*$F25,($E25-$H25)*$F25))</f>
         <v/>
@@ -2342,7 +2354,7 @@
         <v/>
       </c>
       <c r="K25" s="4" t="n">
-        <v>14.75</v>
+        <v>350.52</v>
       </c>
       <c r="L25" s="21">
         <f>IF(OR($B25="",$I25=""),"",$I25-IF($K25="",0,$K25))</f>
@@ -2358,7 +2370,7 @@
       </c>
       <c r="O25" s="23" t="inlineStr">
         <is>
-          <t>5-10</t>
+          <t>10-15</t>
         </is>
       </c>
     </row>
@@ -2387,8 +2399,12 @@
       <c r="F26" s="26" t="n">
         <v>641</v>
       </c>
-      <c r="G26" s="24" t="inlineStr"/>
-      <c r="H26" s="25" t="inlineStr"/>
+      <c r="G26" s="24" t="n">
+        <v>46308</v>
+      </c>
+      <c r="H26" s="25" t="n">
+        <v>262</v>
+      </c>
       <c r="I26" s="21">
         <f>IF(OR($B26="",$H26=""),"",IF($C26="LONG",($H26-$E26)*$F26,($E26-$H26)*$F26))</f>
         <v/>
@@ -2398,7 +2414,7 @@
         <v/>
       </c>
       <c r="K26" s="4" t="n">
-        <v>50.15</v>
+        <v>349.27</v>
       </c>
       <c r="L26" s="21">
         <f>IF(OR($B26="",$I26=""),"",$I26-IF($K26="",0,$K26))</f>
@@ -2443,8 +2459,12 @@
       <c r="F27" s="26" t="n">
         <v>45</v>
       </c>
-      <c r="G27" s="24" t="inlineStr"/>
-      <c r="H27" s="25" t="inlineStr"/>
+      <c r="G27" s="24" t="n">
+        <v>46308</v>
+      </c>
+      <c r="H27" s="25" t="n">
+        <v>3721.09</v>
+      </c>
       <c r="I27" s="21">
         <f>IF(OR($B27="",$H27=""),"",IF($C27="LONG",($H27-$E27)*$F27,($E27-$H27)*$F27))</f>
         <v/>
@@ -2454,7 +2474,7 @@
         <v/>
       </c>
       <c r="K27" s="4" t="n">
-        <v>50.15</v>
+        <v>349.97</v>
       </c>
       <c r="L27" s="21">
         <f>IF(OR($B27="",$I27=""),"",$I27-IF($K27="",0,$K27))</f>
@@ -2475,14 +2495,32 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="23" t="n"/>
-      <c r="B28" s="23" t="n"/>
-      <c r="C28" s="23" t="n"/>
-      <c r="D28" s="24" t="n"/>
-      <c r="E28" s="25" t="n"/>
-      <c r="F28" s="26" t="n"/>
-      <c r="G28" s="24" t="n"/>
-      <c r="H28" s="25" t="n"/>
+      <c r="A28" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126101377709+221261013593709+321261013572009+23126101376509+221261013594809+34126101378609+221261013595609+23126101377609+321261013574409+321261013575009+23126101378109+23126101378209</t>
+        </is>
+      </c>
+      <c r="B28" s="23" t="inlineStr">
+        <is>
+          <t>CMLL</t>
+        </is>
+      </c>
+      <c r="C28" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D28" s="24" t="n">
+        <v>46308</v>
+      </c>
+      <c r="E28" s="25" t="n">
+        <v>617.1578</v>
+      </c>
+      <c r="F28" s="26" t="n">
+        <v>277</v>
+      </c>
+      <c r="G28" s="24" t="inlineStr"/>
+      <c r="H28" s="25" t="inlineStr"/>
       <c r="I28" s="21">
         <f>IF(OR($B28="",$H28=""),"",IF($C28="LONG",($H28-$E28)*$F28,($E28-$H28)*$F28))</f>
         <v/>
@@ -2491,7 +2529,9 @@
         <f>IF(OR($B28="",$I28="",$E28=0,$F28=0),"",$I28/($E28*$F28))</f>
         <v/>
       </c>
-      <c r="K28" s="4" t="n"/>
+      <c r="K28" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($K28="",0,$K28))</f>
         <v/>
@@ -2504,17 +2544,39 @@
         <f>IF($B28="","",IF($H28="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O28" s="23" t="n"/>
+      <c r="O28" s="23" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="23" t="n"/>
-      <c r="B29" s="23" t="n"/>
-      <c r="C29" s="23" t="n"/>
-      <c r="D29" s="24" t="n"/>
-      <c r="E29" s="25" t="n"/>
-      <c r="F29" s="26" t="n"/>
-      <c r="G29" s="24" t="n"/>
-      <c r="H29" s="25" t="n"/>
+      <c r="A29" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261013592809+34126101377809+321261013572109+23126101376309+34126101378309+321261013573109+34126101378709+221261013596309+23126101377709+221261013597309+321261013575409+321261013575609</t>
+        </is>
+      </c>
+      <c r="B29" s="23" t="inlineStr">
+        <is>
+          <t>HATHWAY</t>
+        </is>
+      </c>
+      <c r="C29" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D29" s="24" t="n">
+        <v>46308</v>
+      </c>
+      <c r="E29" s="25" t="n">
+        <v>11.158</v>
+      </c>
+      <c r="F29" s="26" t="n">
+        <v>15360</v>
+      </c>
+      <c r="G29" s="24" t="inlineStr"/>
+      <c r="H29" s="25" t="inlineStr"/>
       <c r="I29" s="21">
         <f>IF(OR($B29="",$H29=""),"",IF($C29="LONG",($H29-$E29)*$F29,($E29-$H29)*$F29))</f>
         <v/>
@@ -2523,7 +2585,9 @@
         <f>IF(OR($B29="",$I29="",$E29=0,$F29=0),"",$I29/($E29*$F29))</f>
         <v/>
       </c>
-      <c r="K29" s="4" t="n"/>
+      <c r="K29" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L29" s="21">
         <f>IF(OR($B29="",$I29=""),"",$I29-IF($K29="",0,$K29))</f>
         <v/>
@@ -2536,17 +2600,39 @@
         <f>IF($B29="","",IF($H29="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O29" s="23" t="n"/>
+      <c r="O29" s="23" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="23" t="n"/>
-      <c r="B30" s="23" t="n"/>
-      <c r="C30" s="23" t="n"/>
-      <c r="D30" s="24" t="n"/>
-      <c r="E30" s="25" t="n"/>
-      <c r="F30" s="26" t="n"/>
-      <c r="G30" s="24" t="n"/>
-      <c r="H30" s="25" t="n"/>
+      <c r="A30" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126101375909+221261013593509+221261013594309+34126101378209+321261013572509+23126101377109+321261013573709+23126101377509+34126101379009+321261013575109+221261013597709+221261013598409+34126101379609</t>
+        </is>
+      </c>
+      <c r="B30" s="23" t="inlineStr">
+        <is>
+          <t>INDIAGLYCO</t>
+        </is>
+      </c>
+      <c r="C30" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D30" s="24" t="n">
+        <v>46308</v>
+      </c>
+      <c r="E30" s="25" t="n">
+        <v>352.906</v>
+      </c>
+      <c r="F30" s="26" t="n">
+        <v>243</v>
+      </c>
+      <c r="G30" s="24" t="inlineStr"/>
+      <c r="H30" s="25" t="inlineStr"/>
       <c r="I30" s="21">
         <f>IF(OR($B30="",$H30=""),"",IF($C30="LONG",($H30-$E30)*$F30,($E30-$H30)*$F30))</f>
         <v/>
@@ -2555,7 +2641,9 @@
         <f>IF(OR($B30="",$I30="",$E30=0,$F30=0),"",$I30/($E30*$F30))</f>
         <v/>
       </c>
-      <c r="K30" s="4" t="n"/>
+      <c r="K30" s="4" t="n">
+        <v>14.75</v>
+      </c>
       <c r="L30" s="21">
         <f>IF(OR($B30="",$I30=""),"",$I30-IF($K30="",0,$K30))</f>
         <v/>
@@ -2568,17 +2656,39 @@
         <f>IF($B30="","",IF($H30="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O30" s="23" t="n"/>
+      <c r="O30" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="23" t="n"/>
-      <c r="B31" s="23" t="n"/>
-      <c r="C31" s="23" t="n"/>
-      <c r="D31" s="24" t="n"/>
-      <c r="E31" s="25" t="n"/>
-      <c r="F31" s="26" t="n"/>
-      <c r="G31" s="24" t="n"/>
-      <c r="H31" s="25" t="n"/>
+      <c r="A31" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126101377609+221261013593609+34126101378109+23126101376709+34126101378409+23126101377009+221261013595709+221261013596109+221261013596609+23126101377809+34126101379309+34126101379709+23126101378409+34126101379809+221261013599309+321261013576809</t>
+        </is>
+      </c>
+      <c r="B31" s="23" t="inlineStr">
+        <is>
+          <t>INDOKEM</t>
+        </is>
+      </c>
+      <c r="C31" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D31" s="24" t="n">
+        <v>46308</v>
+      </c>
+      <c r="E31" s="25" t="n">
+        <v>677.9853000000001</v>
+      </c>
+      <c r="F31" s="26" t="n">
+        <v>126</v>
+      </c>
+      <c r="G31" s="24" t="inlineStr"/>
+      <c r="H31" s="25" t="inlineStr"/>
       <c r="I31" s="21">
         <f>IF(OR($B31="",$H31=""),"",IF($C31="LONG",($H31-$E31)*$F31,($E31-$H31)*$F31))</f>
         <v/>
@@ -2587,7 +2697,9 @@
         <f>IF(OR($B31="",$I31="",$E31=0,$F31=0),"",$I31/($E31*$F31))</f>
         <v/>
       </c>
-      <c r="K31" s="4" t="n"/>
+      <c r="K31" s="4" t="n">
+        <v>14.75</v>
+      </c>
       <c r="L31" s="21">
         <f>IF(OR($B31="",$I31=""),"",$I31-IF($K31="",0,$K31))</f>
         <v/>
@@ -2600,17 +2712,39 @@
         <f>IF($B31="","",IF($H31="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O31" s="23" t="n"/>
+      <c r="O31" s="23" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="23" t="n"/>
-      <c r="B32" s="23" t="n"/>
-      <c r="C32" s="23" t="n"/>
-      <c r="D32" s="24" t="n"/>
-      <c r="E32" s="25" t="n"/>
-      <c r="F32" s="26" t="n"/>
-      <c r="G32" s="24" t="n"/>
-      <c r="H32" s="25" t="n"/>
+      <c r="A32" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261012625809+321261012626209+23126101284209+23126101284309+321261012626909+34126101276209+34126101277109+321261012628809+221261012640809+23126101286309+34126101278009+321261012630809+221261012643209</t>
+        </is>
+      </c>
+      <c r="B32" s="23" t="inlineStr">
+        <is>
+          <t>MMWL</t>
+        </is>
+      </c>
+      <c r="C32" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D32" s="24" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E32" s="25" t="n">
+        <v>22.8999</v>
+      </c>
+      <c r="F32" s="26" t="n">
+        <v>3742</v>
+      </c>
+      <c r="G32" s="24" t="inlineStr"/>
+      <c r="H32" s="25" t="inlineStr"/>
       <c r="I32" s="21">
         <f>IF(OR($B32="",$H32=""),"",IF($C32="LONG",($H32-$E32)*$F32,($E32-$H32)*$F32))</f>
         <v/>
@@ -2619,7 +2753,9 @@
         <f>IF(OR($B32="",$I32="",$E32=0,$F32=0),"",$I32/($E32*$F32))</f>
         <v/>
       </c>
-      <c r="K32" s="4" t="n"/>
+      <c r="K32" s="4" t="n">
+        <v>53.57</v>
+      </c>
       <c r="L32" s="21">
         <f>IF(OR($B32="",$I32=""),"",$I32-IF($K32="",0,$K32))</f>
         <v/>
@@ -2632,17 +2768,39 @@
         <f>IF($B32="","",IF($H32="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O32" s="23" t="n"/>
+      <c r="O32" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="23" t="n"/>
-      <c r="B33" s="23" t="n"/>
-      <c r="C33" s="23" t="n"/>
-      <c r="D33" s="24" t="n"/>
-      <c r="E33" s="25" t="n"/>
-      <c r="F33" s="26" t="n"/>
-      <c r="G33" s="24" t="n"/>
-      <c r="H33" s="25" t="n"/>
+      <c r="A33" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261013593009+23126101376209+34126101378009+221261013594409+23126101376909+23126101377209+23126101377309+321261013574209+321261013574509+23126101377909+34126101379509+321261013575709</t>
+        </is>
+      </c>
+      <c r="B33" s="23" t="inlineStr">
+        <is>
+          <t>PIXTRANS</t>
+        </is>
+      </c>
+      <c r="C33" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D33" s="24" t="n">
+        <v>46308</v>
+      </c>
+      <c r="E33" s="25" t="n">
+        <v>1889.5856</v>
+      </c>
+      <c r="F33" s="26" t="n">
+        <v>90</v>
+      </c>
+      <c r="G33" s="24" t="inlineStr"/>
+      <c r="H33" s="25" t="inlineStr"/>
       <c r="I33" s="21">
         <f>IF(OR($B33="",$H33=""),"",IF($C33="LONG",($H33-$E33)*$F33,($E33-$H33)*$F33))</f>
         <v/>
@@ -2651,7 +2809,9 @@
         <f>IF(OR($B33="",$I33="",$E33=0,$F33=0),"",$I33/($E33*$F33))</f>
         <v/>
       </c>
-      <c r="K33" s="4" t="n"/>
+      <c r="K33" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L33" s="21">
         <f>IF(OR($B33="",$I33=""),"",$I33-IF($K33="",0,$K33))</f>
         <v/>
@@ -2664,17 +2824,39 @@
         <f>IF($B33="","",IF($H33="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O33" s="23" t="n"/>
+      <c r="O33" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="23" t="n"/>
-      <c r="B34" s="23" t="n"/>
-      <c r="C34" s="23" t="n"/>
-      <c r="D34" s="24" t="n"/>
-      <c r="E34" s="25" t="n"/>
-      <c r="F34" s="26" t="n"/>
-      <c r="G34" s="24" t="n"/>
-      <c r="H34" s="25" t="n"/>
+      <c r="A34" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261013571309+221261013593809+221261013594209+23126101376409+34126101378509+321261013573309+34126101378809+34126101378909+221261013596709+221261013597209+34126101379409+23126101378309+321261013576009</t>
+        </is>
+      </c>
+      <c r="B34" s="23" t="inlineStr">
+        <is>
+          <t>PNCINFRA</t>
+        </is>
+      </c>
+      <c r="C34" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D34" s="24" t="n">
+        <v>46308</v>
+      </c>
+      <c r="E34" s="25" t="n">
+        <v>156.7238</v>
+      </c>
+      <c r="F34" s="26" t="n">
+        <v>1086</v>
+      </c>
+      <c r="G34" s="24" t="inlineStr"/>
+      <c r="H34" s="25" t="inlineStr"/>
       <c r="I34" s="21">
         <f>IF(OR($B34="",$H34=""),"",IF($C34="LONG",($H34-$E34)*$F34,($E34-$H34)*$F34))</f>
         <v/>
@@ -2683,7 +2865,9 @@
         <f>IF(OR($B34="",$I34="",$E34=0,$F34=0),"",$I34/($E34*$F34))</f>
         <v/>
       </c>
-      <c r="K34" s="4" t="n"/>
+      <c r="K34" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($K34="",0,$K34))</f>
         <v/>
@@ -2696,17 +2880,39 @@
         <f>IF($B34="","",IF($H34="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O34" s="23" t="n"/>
+      <c r="O34" s="23" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="23" t="n"/>
-      <c r="B35" s="23" t="n"/>
-      <c r="C35" s="23" t="n"/>
-      <c r="D35" s="24" t="n"/>
-      <c r="E35" s="25" t="n"/>
-      <c r="F35" s="26" t="n"/>
-      <c r="G35" s="24" t="n"/>
-      <c r="H35" s="25" t="n"/>
+      <c r="A35" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261013592909+23126101376109+321261013572209+23126101376609+321261013572609+321261013573209+321261013573809+221261013596209+34126101379109+34126101379209+221261013597909</t>
+        </is>
+      </c>
+      <c r="B35" s="23" t="inlineStr">
+        <is>
+          <t>SHRINGARMS</t>
+        </is>
+      </c>
+      <c r="C35" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D35" s="24" t="n">
+        <v>46308</v>
+      </c>
+      <c r="E35" s="25" t="n">
+        <v>311.7565</v>
+      </c>
+      <c r="F35" s="26" t="n">
+        <v>549</v>
+      </c>
+      <c r="G35" s="24" t="inlineStr"/>
+      <c r="H35" s="25" t="inlineStr"/>
       <c r="I35" s="21">
         <f>IF(OR($B35="",$H35=""),"",IF($C35="LONG",($H35-$E35)*$F35,($E35-$H35)*$F35))</f>
         <v/>
@@ -2715,7 +2921,9 @@
         <f>IF(OR($B35="",$I35="",$E35=0,$F35=0),"",$I35/($E35*$F35))</f>
         <v/>
       </c>
-      <c r="K35" s="4" t="n"/>
+      <c r="K35" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L35" s="21">
         <f>IF(OR($B35="",$I35=""),"",$I35-IF($K35="",0,$K35))</f>
         <v/>
@@ -2728,7 +2936,11 @@
         <f>IF($B35="","",IF($H35="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O35" s="23" t="n"/>
+      <c r="O35" s="23" t="inlineStr">
+        <is>
+          <t>15-20</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="23" t="n"/>
@@ -30381,7 +30593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30551,7 +30763,7 @@
     <row r="6">
       <c r="A6" s="27" t="inlineStr">
         <is>
-          <t>DELTACORP</t>
+          <t>CMLL</t>
         </is>
       </c>
       <c r="B6" s="20">
@@ -30594,7 +30806,7 @@
     <row r="7">
       <c r="A7" s="27" t="inlineStr">
         <is>
-          <t>DPABHUSHAN</t>
+          <t>DELTACORP</t>
         </is>
       </c>
       <c r="B7" s="20">
@@ -30637,7 +30849,7 @@
     <row r="8">
       <c r="A8" s="27" t="inlineStr">
         <is>
-          <t>GOODLUCK</t>
+          <t>DPABHUSHAN</t>
         </is>
       </c>
       <c r="B8" s="20">
@@ -30680,7 +30892,7 @@
     <row r="9">
       <c r="A9" s="27" t="inlineStr">
         <is>
-          <t>GPTINFRA</t>
+          <t>GOODLUCK</t>
         </is>
       </c>
       <c r="B9" s="20">
@@ -30723,7 +30935,7 @@
     <row r="10">
       <c r="A10" s="27" t="inlineStr">
         <is>
-          <t>INOXGREEN</t>
+          <t>GPTINFRA</t>
         </is>
       </c>
       <c r="B10" s="20">
@@ -30766,7 +30978,7 @@
     <row r="11">
       <c r="A11" s="27" t="inlineStr">
         <is>
-          <t>KOTIC</t>
+          <t>HATHWAY</t>
         </is>
       </c>
       <c r="B11" s="20">
@@ -30809,7 +31021,7 @@
     <row r="12">
       <c r="A12" s="27" t="inlineStr">
         <is>
-          <t>KRISHNADEF</t>
+          <t>INDIAGLYCO</t>
         </is>
       </c>
       <c r="B12" s="20">
@@ -30852,7 +31064,7 @@
     <row r="13">
       <c r="A13" s="27" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>INDOKEM</t>
         </is>
       </c>
       <c r="B13" s="20">
@@ -30895,7 +31107,7 @@
     <row r="14">
       <c r="A14" s="27" t="inlineStr">
         <is>
-          <t>MOBIKWIK</t>
+          <t>INOXGREEN</t>
         </is>
       </c>
       <c r="B14" s="20">
@@ -30938,7 +31150,7 @@
     <row r="15">
       <c r="A15" s="27" t="inlineStr">
         <is>
-          <t>PNGSREVA</t>
+          <t>KOTIC</t>
         </is>
       </c>
       <c r="B15" s="20">
@@ -30981,7 +31193,7 @@
     <row r="16">
       <c r="A16" s="27" t="inlineStr">
         <is>
-          <t>PRINCEPIPE</t>
+          <t>KRISHNADEF</t>
         </is>
       </c>
       <c r="B16" s="20">
@@ -31024,7 +31236,7 @@
     <row r="17">
       <c r="A17" s="27" t="inlineStr">
         <is>
-          <t>RSYSTEMS</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="B17" s="20">
@@ -31067,7 +31279,7 @@
     <row r="18">
       <c r="A18" s="27" t="inlineStr">
         <is>
-          <t>SAKSOFT</t>
+          <t>MOBIKWIK</t>
         </is>
       </c>
       <c r="B18" s="20">
@@ -31110,7 +31322,7 @@
     <row r="19">
       <c r="A19" s="27" t="inlineStr">
         <is>
-          <t>SATIN</t>
+          <t>PIXTRANS</t>
         </is>
       </c>
       <c r="B19" s="20">
@@ -31153,7 +31365,7 @@
     <row r="20">
       <c r="A20" s="27" t="inlineStr">
         <is>
-          <t>SGFIN</t>
+          <t>PNCINFRA</t>
         </is>
       </c>
       <c r="B20" s="20">
@@ -31196,7 +31408,7 @@
     <row r="21">
       <c r="A21" s="27" t="inlineStr">
         <is>
-          <t>SMCGLOBAL</t>
+          <t>PNGSREVA</t>
         </is>
       </c>
       <c r="B21" s="20">
@@ -31239,7 +31451,7 @@
     <row r="22">
       <c r="A22" s="27" t="inlineStr">
         <is>
-          <t>SUNCLAY</t>
+          <t>PRINCEPIPE</t>
         </is>
       </c>
       <c r="B22" s="20">
@@ -31282,7 +31494,7 @@
     <row r="23">
       <c r="A23" s="27" t="inlineStr">
         <is>
-          <t>SWARAJENG</t>
+          <t>RSYSTEMS</t>
         </is>
       </c>
       <c r="B23" s="20">
@@ -31325,7 +31537,7 @@
     <row r="24">
       <c r="A24" s="27" t="inlineStr">
         <is>
-          <t>YUKEN</t>
+          <t>SAKSOFT</t>
         </is>
       </c>
       <c r="B24" s="20">
@@ -31366,37 +31578,338 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="A25" s="27" t="inlineStr">
+        <is>
+          <t>SATIN</t>
+        </is>
+      </c>
+      <c r="B25" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A25)</f>
+        <v/>
+      </c>
+      <c r="C25" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A25,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D25" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A25,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E25" s="22">
+        <f>IFERROR($C25/$B25,"")</f>
+        <v/>
+      </c>
+      <c r="F25" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A25,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G25" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A25,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H25" s="21">
+        <f>IFERROR($G25/$B25,"")</f>
+        <v/>
+      </c>
+      <c r="I25" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A25),"")</f>
+        <v/>
+      </c>
+      <c r="J25" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A25),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="27" t="inlineStr">
+        <is>
+          <t>SGFIN</t>
+        </is>
+      </c>
+      <c r="B26" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A26)</f>
+        <v/>
+      </c>
+      <c r="C26" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A26,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D26" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A26,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E26" s="22">
+        <f>IFERROR($C26/$B26,"")</f>
+        <v/>
+      </c>
+      <c r="F26" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A26,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G26" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A26,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H26" s="21">
+        <f>IFERROR($G26/$B26,"")</f>
+        <v/>
+      </c>
+      <c r="I26" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A26),"")</f>
+        <v/>
+      </c>
+      <c r="J26" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A26),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="27" t="inlineStr">
+        <is>
+          <t>SHRINGARMS</t>
+        </is>
+      </c>
+      <c r="B27" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A27)</f>
+        <v/>
+      </c>
+      <c r="C27" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A27,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D27" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A27,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E27" s="22">
+        <f>IFERROR($C27/$B27,"")</f>
+        <v/>
+      </c>
+      <c r="F27" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A27,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G27" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A27,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H27" s="21">
+        <f>IFERROR($G27/$B27,"")</f>
+        <v/>
+      </c>
+      <c r="I27" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A27),"")</f>
+        <v/>
+      </c>
+      <c r="J27" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A27),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="27" t="inlineStr">
+        <is>
+          <t>SMCGLOBAL</t>
+        </is>
+      </c>
+      <c r="B28" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A28)</f>
+        <v/>
+      </c>
+      <c r="C28" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A28,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D28" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A28,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E28" s="22">
+        <f>IFERROR($C28/$B28,"")</f>
+        <v/>
+      </c>
+      <c r="F28" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A28,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G28" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A28,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H28" s="21">
+        <f>IFERROR($G28/$B28,"")</f>
+        <v/>
+      </c>
+      <c r="I28" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A28),"")</f>
+        <v/>
+      </c>
+      <c r="J28" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A28),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="27" t="inlineStr">
+        <is>
+          <t>SUNCLAY</t>
+        </is>
+      </c>
+      <c r="B29" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A29)</f>
+        <v/>
+      </c>
+      <c r="C29" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A29,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D29" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A29,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E29" s="22">
+        <f>IFERROR($C29/$B29,"")</f>
+        <v/>
+      </c>
+      <c r="F29" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A29,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G29" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A29,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H29" s="21">
+        <f>IFERROR($G29/$B29,"")</f>
+        <v/>
+      </c>
+      <c r="I29" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A29),"")</f>
+        <v/>
+      </c>
+      <c r="J29" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A29),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="27" t="inlineStr">
+        <is>
+          <t>SWARAJENG</t>
+        </is>
+      </c>
+      <c r="B30" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A30)</f>
+        <v/>
+      </c>
+      <c r="C30" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A30,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D30" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A30,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E30" s="22">
+        <f>IFERROR($C30/$B30,"")</f>
+        <v/>
+      </c>
+      <c r="F30" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A30,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G30" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A30,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H30" s="21">
+        <f>IFERROR($G30/$B30,"")</f>
+        <v/>
+      </c>
+      <c r="I30" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A30),"")</f>
+        <v/>
+      </c>
+      <c r="J30" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A30),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="27" t="inlineStr">
+        <is>
+          <t>YUKEN</t>
+        </is>
+      </c>
+      <c r="B31" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A31)</f>
+        <v/>
+      </c>
+      <c r="C31" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A31,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D31" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A31,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E31" s="22">
+        <f>IFERROR($C31/$B31,"")</f>
+        <v/>
+      </c>
+      <c r="F31" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A31,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G31" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A31,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H31" s="21">
+        <f>IFERROR($G31/$B31,"")</f>
+        <v/>
+      </c>
+      <c r="I31" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A31),"")</f>
+        <v/>
+      </c>
+      <c r="J31" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A31),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B25" s="30">
-        <f>SUM(B4:B24)</f>
-        <v/>
-      </c>
-      <c r="C25" s="30">
-        <f>SUM(C4:C24)</f>
-        <v/>
-      </c>
-      <c r="D25" s="30">
-        <f>SUM(D4:D24)</f>
-        <v/>
-      </c>
-      <c r="E25" s="31">
-        <f>IFERROR(C25/B25,"")</f>
-        <v/>
-      </c>
-      <c r="F25" s="32">
-        <f>SUM(F4:F24)</f>
-        <v/>
-      </c>
-      <c r="G25" s="32">
-        <f>SUM(G4:G24)</f>
-        <v/>
-      </c>
-      <c r="H25" s="32">
-        <f>IFERROR(G25/B25,"")</f>
+      <c r="B32" s="30">
+        <f>SUM(B4:B31)</f>
+        <v/>
+      </c>
+      <c r="C32" s="30">
+        <f>SUM(C4:C31)</f>
+        <v/>
+      </c>
+      <c r="D32" s="30">
+        <f>SUM(D4:D31)</f>
+        <v/>
+      </c>
+      <c r="E32" s="31">
+        <f>IFERROR(C32/B32,"")</f>
+        <v/>
+      </c>
+      <c r="F32" s="32">
+        <f>SUM(F4:F31)</f>
+        <v/>
+      </c>
+      <c r="G32" s="32">
+        <f>SUM(G4:G31)</f>
+        <v/>
+      </c>
+      <c r="H32" s="32">
+        <f>IFERROR(G32/B32,"")</f>
         <v/>
       </c>
     </row>
@@ -31415,7 +31928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N28"/>
+  <dimension ref="A1:N36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -31666,7 +32179,7 @@
         <v>35.4</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>123.79</v>
+        <v>125.76</v>
       </c>
       <c r="N6" s="21">
         <f>SUM(E6:M6)</f>
@@ -31717,7 +32230,7 @@
         <v>35.4</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>74.02</v>
+        <v>75.19</v>
       </c>
       <c r="N7" s="21">
         <f>SUM(E7:M7)</f>
@@ -31768,7 +32281,7 @@
         <v>35.4</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>74.16</v>
+        <v>75.34</v>
       </c>
       <c r="N8" s="21">
         <f>SUM(E8:M8)</f>
@@ -31819,7 +32332,7 @@
         <v>35.4</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>123.45</v>
+        <v>125.41</v>
       </c>
       <c r="N9" s="21">
         <f>SUM(E9:M9)</f>
@@ -31870,7 +32383,7 @@
         <v>35.4</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>103.01</v>
+        <v>104.65</v>
       </c>
       <c r="N10" s="21">
         <f>SUM(E10:M10)</f>
@@ -31921,7 +32434,7 @@
         <v>35.4</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>41.29</v>
+        <v>41.95</v>
       </c>
       <c r="N11" s="21">
         <f>SUM(E11:M11)</f>
@@ -31972,7 +32485,7 @@
         <v>35.4</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>49.49</v>
+        <v>50.27</v>
       </c>
       <c r="N12" s="21">
         <f>SUM(E12:M12)</f>
@@ -32023,7 +32536,7 @@
         <v>35.4</v>
       </c>
       <c r="M13" s="4" t="n">
-        <v>29.77</v>
+        <v>30.24</v>
       </c>
       <c r="N13" s="21">
         <f>SUM(E13:M13)</f>
@@ -32074,7 +32587,7 @@
         <v>35.4</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>41.17</v>
+        <v>30.11</v>
       </c>
       <c r="N14" s="21">
         <f>SUM(E14:M14)</f>
@@ -32203,22 +32716,22 @@
         <v>46307</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>60.1</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>200.23</v>
+        <v>388.39</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>6.15</v>
+        <v>11.92</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>0.2</v>
+        <v>0.39</v>
       </c>
       <c r="I17" s="4" t="n">
         <v>30.04</v>
       </c>
       <c r="J17" s="4" t="n">
-        <v>11.96</v>
+        <v>16.63</v>
       </c>
       <c r="K17" s="4" t="n">
         <v>14.75</v>
@@ -32227,7 +32740,7 @@
         <v>35.4</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>123.27</v>
+        <v>73.95999999999999</v>
       </c>
       <c r="N17" s="21">
         <f>SUM(E17:M17)</f>
@@ -32254,22 +32767,22 @@
         <v>46307</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>75.33</v>
+        <v>95.28</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>2.31</v>
+        <v>4.69</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>0.08</v>
+        <v>0.15</v>
       </c>
       <c r="I18" s="4" t="n">
         <v>11.3</v>
       </c>
       <c r="J18" s="4" t="n">
-        <v>0.43</v>
+        <v>4.47</v>
       </c>
       <c r="K18" s="4" t="n">
         <v>14.75</v>
@@ -32305,22 +32818,22 @@
         <v>46307</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>59.98</v>
+        <v>79.98</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>199.85</v>
+        <v>391.05</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>6.14</v>
+        <v>12.01</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>0.2</v>
+        <v>0.39</v>
       </c>
       <c r="I19" s="4" t="n">
         <v>29.98</v>
       </c>
       <c r="J19" s="4" t="n">
-        <v>11.94</v>
+        <v>16.63</v>
       </c>
       <c r="K19" s="4" t="n">
         <v>14.75</v>
@@ -32329,7 +32842,7 @@
         <v>35.4</v>
       </c>
       <c r="M19" s="4" t="n">
-        <v>127.52</v>
+        <v>127.32</v>
       </c>
       <c r="N19" s="21">
         <f>SUM(E19:M19)</f>
@@ -32356,22 +32869,22 @@
         <v>46307</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>60.11</v>
+        <v>80.11</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>200.46</v>
+        <v>403.61</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>6.15</v>
+        <v>12.39</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="I20" s="4" t="n">
         <v>30.07</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>11.96</v>
+        <v>16.72</v>
       </c>
       <c r="K20" s="4" t="n">
         <v>14.75</v>
@@ -32410,19 +32923,19 @@
         <v>0</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>99.53</v>
+        <v>199.48</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>3.06</v>
+        <v>6.12</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I21" s="4" t="n">
         <v>14.93</v>
       </c>
       <c r="J21" s="4" t="n">
-        <v>0.57</v>
+        <v>1.14</v>
       </c>
       <c r="K21" s="4" t="n">
         <v>14.75</v>
@@ -32458,22 +32971,22 @@
         <v>46307</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>49.11</v>
+        <v>69.11</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>201.41</v>
+        <v>397.41</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>6.18</v>
+        <v>12.2</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="I22" s="4" t="n">
         <v>30.68</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>9.99</v>
+        <v>14.71</v>
       </c>
       <c r="K22" s="4" t="n">
         <v>14.75</v>
@@ -32505,24 +33018,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D23" s="24" t="inlineStr"/>
+      <c r="D23" s="24" t="n">
+        <v>46308</v>
+      </c>
       <c r="E23" s="4" t="n">
-        <v>0</v>
+        <v>51.61</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>0</v>
+        <v>172.14</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>0</v>
+        <v>5.28</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>0</v>
+        <v>0.17</v>
       </c>
       <c r="I23" s="4" t="n">
-        <v>0</v>
+        <v>25.82</v>
       </c>
       <c r="J23" s="4" t="n">
-        <v>0</v>
+        <v>10.27</v>
       </c>
       <c r="K23" s="4" t="n">
         <v>14.75</v>
@@ -32531,7 +33046,7 @@
         <v>35.4</v>
       </c>
       <c r="M23" s="4" t="n">
-        <v>0</v>
+        <v>29.44</v>
       </c>
       <c r="N23" s="21">
         <f>SUM(E23:M23)</f>
@@ -32541,20 +33056,22 @@
     <row r="24">
       <c r="A24" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261012636709+221261012637509+321261012626709+221261012638409+23126101284609+34126101276109+221261012640409+34126101277309+34126101277409+221261012641109+321261012630109</t>
+          <t>DHAN-321261013231409</t>
         </is>
       </c>
       <c r="B24" s="23" t="inlineStr">
         <is>
-          <t>GOODLUCK</t>
+          <t>BLUSPRING</t>
         </is>
       </c>
       <c r="C24" s="23" t="inlineStr">
         <is>
-          <t>LONG</t>
-        </is>
-      </c>
-      <c r="D24" s="24" t="inlineStr"/>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D24" s="24" t="n">
+        <v>46308</v>
+      </c>
       <c r="E24" s="4" t="n">
         <v>0</v>
       </c>
@@ -32574,10 +33091,10 @@
         <v>0</v>
       </c>
       <c r="K24" s="4" t="n">
-        <v>14.75</v>
+        <v>0</v>
       </c>
       <c r="L24" s="4" t="n">
-        <v>35.4</v>
+        <v>0</v>
       </c>
       <c r="M24" s="4" t="n">
         <v>0</v>
@@ -32590,12 +33107,12 @@
     <row r="25">
       <c r="A25" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261012625809+321261012626209+23126101284209+23126101284309+321261012626909+34126101276209+34126101277109+321261012628809+221261012640809+23126101286309+34126101278009+321261012630809+221261012643209</t>
+          <t>DHAN-221261012636709+221261012637509+321261012626709+221261012638409+23126101284609+34126101276109+221261012640409+34126101277309+34126101277409+221261012641109+321261012630109</t>
         </is>
       </c>
       <c r="B25" s="23" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>GOODLUCK</t>
         </is>
       </c>
       <c r="C25" s="23" t="inlineStr">
@@ -32603,33 +33120,35 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D25" s="24" t="inlineStr"/>
+      <c r="D25" s="24" t="n">
+        <v>46308</v>
+      </c>
       <c r="E25" s="4" t="n">
-        <v>0</v>
+        <v>51.35</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>0</v>
+        <v>171.15</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>0</v>
+        <v>5.25</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>0</v>
+        <v>0.17</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>0</v>
+        <v>25.67</v>
       </c>
       <c r="J25" s="4" t="n">
-        <v>0</v>
+        <v>10.22</v>
       </c>
       <c r="K25" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L25" s="4" t="n">
-        <v>0</v>
+        <v>35.4</v>
       </c>
       <c r="M25" s="4" t="n">
-        <v>0</v>
+        <v>36.56</v>
       </c>
       <c r="N25" s="21">
         <f>SUM(E25:M25)</f>
@@ -32652,24 +33171,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D26" s="24" t="inlineStr"/>
+      <c r="D26" s="24" t="n">
+        <v>46308</v>
+      </c>
       <c r="E26" s="4" t="n">
-        <v>0</v>
+        <v>51.44</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>0</v>
+        <v>171.54</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>0</v>
+        <v>5.27</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>0</v>
+        <v>0.17</v>
       </c>
       <c r="I26" s="4" t="n">
-        <v>0</v>
+        <v>25.26</v>
       </c>
       <c r="J26" s="4" t="n">
-        <v>0</v>
+        <v>10.24</v>
       </c>
       <c r="K26" s="4" t="n">
         <v>14.75</v>
@@ -32678,7 +33199,7 @@
         <v>35.4</v>
       </c>
       <c r="M26" s="4" t="n">
-        <v>0</v>
+        <v>35.2</v>
       </c>
       <c r="N26" s="21">
         <f>SUM(E26:M26)</f>
@@ -32701,24 +33222,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D27" s="24" t="inlineStr"/>
+      <c r="D27" s="24" t="n">
+        <v>46308</v>
+      </c>
       <c r="E27" s="4" t="n">
-        <v>0</v>
+        <v>50.51</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>0</v>
+        <v>168.36</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>0</v>
+        <v>5.17</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>0</v>
+        <v>0.17</v>
       </c>
       <c r="I27" s="4" t="n">
-        <v>0</v>
+        <v>25.25</v>
       </c>
       <c r="J27" s="4" t="n">
-        <v>0</v>
+        <v>10.05</v>
       </c>
       <c r="K27" s="4" t="n">
         <v>14.75</v>
@@ -32727,7 +33250,7 @@
         <v>35.4</v>
       </c>
       <c r="M27" s="4" t="n">
-        <v>0</v>
+        <v>40.31</v>
       </c>
       <c r="N27" s="21">
         <f>SUM(E27:M27)</f>
@@ -32735,54 +33258,446 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="inlineStr">
+      <c r="A28" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126101377709+221261013593709+321261013572009+23126101376509+221261013594809+34126101378609+221261013595609+23126101377609+321261013574409+321261013575009+23126101378109+23126101378209</t>
+        </is>
+      </c>
+      <c r="B28" s="23" t="inlineStr">
+        <is>
+          <t>CMLL</t>
+        </is>
+      </c>
+      <c r="C28" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D28" s="24" t="inlineStr"/>
+      <c r="E28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L28" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" s="21">
+        <f>SUM(E28:M28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261013592809+34126101377809+321261013572109+23126101376309+34126101378309+321261013573109+34126101378709+221261013596309+23126101377709+221261013597309+321261013575409+321261013575609</t>
+        </is>
+      </c>
+      <c r="B29" s="23" t="inlineStr">
+        <is>
+          <t>HATHWAY</t>
+        </is>
+      </c>
+      <c r="C29" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D29" s="24" t="inlineStr"/>
+      <c r="E29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L29" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" s="21">
+        <f>SUM(E29:M29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126101375909+221261013593509+221261013594309+34126101378209+321261013572509+23126101377109+321261013573709+23126101377509+34126101379009+321261013575109+221261013597709+221261013598409+34126101379609</t>
+        </is>
+      </c>
+      <c r="B30" s="23" t="inlineStr">
+        <is>
+          <t>INDIAGLYCO</t>
+        </is>
+      </c>
+      <c r="C30" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D30" s="24" t="inlineStr"/>
+      <c r="E30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" s="21">
+        <f>SUM(E30:M30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126101377609+221261013593609+34126101378109+23126101376709+34126101378409+23126101377009+221261013595709+221261013596109+221261013596609+23126101377809+34126101379309+34126101379709+23126101378409+34126101379809+221261013599309+321261013576809</t>
+        </is>
+      </c>
+      <c r="B31" s="23" t="inlineStr">
+        <is>
+          <t>INDOKEM</t>
+        </is>
+      </c>
+      <c r="C31" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D31" s="24" t="inlineStr"/>
+      <c r="E31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" s="21">
+        <f>SUM(E31:M31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261012625809+321261012626209+23126101284209+23126101284309+321261012626909+34126101276209+34126101277109+321261012628809+221261012640809+23126101286309+34126101278009+321261012630809+221261012643209</t>
+        </is>
+      </c>
+      <c r="B32" s="23" t="inlineStr">
+        <is>
+          <t>MMWL</t>
+        </is>
+      </c>
+      <c r="C32" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D32" s="24" t="inlineStr"/>
+      <c r="E32" s="4" t="n">
+        <v>24.76</v>
+      </c>
+      <c r="F32" s="4" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="G32" s="4" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="H32" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="I32" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J32" s="4" t="n">
+        <v>4.95</v>
+      </c>
+      <c r="K32" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N32" s="21">
+        <f>SUM(E32:M32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261013593009+23126101376209+34126101378009+221261013594409+23126101376909+23126101377209+23126101377309+321261013574209+321261013574509+23126101377909+34126101379509+321261013575709</t>
+        </is>
+      </c>
+      <c r="B33" s="23" t="inlineStr">
+        <is>
+          <t>PIXTRANS</t>
+        </is>
+      </c>
+      <c r="C33" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D33" s="24" t="inlineStr"/>
+      <c r="E33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L33" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N33" s="21">
+        <f>SUM(E33:M33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261013571309+221261013593809+221261013594209+23126101376409+34126101378509+321261013573309+34126101378809+34126101378909+221261013596709+221261013597209+34126101379409+23126101378309+321261013576009</t>
+        </is>
+      </c>
+      <c r="B34" s="23" t="inlineStr">
+        <is>
+          <t>PNCINFRA</t>
+        </is>
+      </c>
+      <c r="C34" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D34" s="24" t="inlineStr"/>
+      <c r="E34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L34" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N34" s="21">
+        <f>SUM(E34:M34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261013592909+23126101376109+321261013572209+23126101376609+321261013572609+321261013573209+321261013573809+221261013596209+34126101379109+34126101379209+221261013597909</t>
+        </is>
+      </c>
+      <c r="B35" s="23" t="inlineStr">
+        <is>
+          <t>SHRINGARMS</t>
+        </is>
+      </c>
+      <c r="C35" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D35" s="24" t="inlineStr"/>
+      <c r="E35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L35" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N35" s="21">
+        <f>SUM(E35:M35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E28" s="32">
-        <f>SUM(E4:E27)</f>
-        <v/>
-      </c>
-      <c r="F28" s="32">
-        <f>SUM(F4:F27)</f>
-        <v/>
-      </c>
-      <c r="G28" s="32">
-        <f>SUM(G4:G27)</f>
-        <v/>
-      </c>
-      <c r="H28" s="32">
-        <f>SUM(H4:H27)</f>
-        <v/>
-      </c>
-      <c r="I28" s="32">
-        <f>SUM(I4:I27)</f>
-        <v/>
-      </c>
-      <c r="J28" s="32">
-        <f>SUM(J4:J27)</f>
-        <v/>
-      </c>
-      <c r="K28" s="32">
-        <f>SUM(K4:K27)</f>
-        <v/>
-      </c>
-      <c r="L28" s="32">
-        <f>SUM(L4:L27)</f>
-        <v/>
-      </c>
-      <c r="M28" s="32">
-        <f>SUM(M4:M27)</f>
-        <v/>
-      </c>
-      <c r="N28" s="32">
-        <f>SUM(N4:N27)</f>
+      <c r="E36" s="32">
+        <f>SUM(E4:E35)</f>
+        <v/>
+      </c>
+      <c r="F36" s="32">
+        <f>SUM(F4:F35)</f>
+        <v/>
+      </c>
+      <c r="G36" s="32">
+        <f>SUM(G4:G35)</f>
+        <v/>
+      </c>
+      <c r="H36" s="32">
+        <f>SUM(H4:H35)</f>
+        <v/>
+      </c>
+      <c r="I36" s="32">
+        <f>SUM(I4:I35)</f>
+        <v/>
+      </c>
+      <c r="J36" s="32">
+        <f>SUM(J4:J35)</f>
+        <v/>
+      </c>
+      <c r="K36" s="32">
+        <f>SUM(K4:K35)</f>
+        <v/>
+      </c>
+      <c r="L36" s="32">
+        <f>SUM(L4:L35)</f>
+        <v/>
+      </c>
+      <c r="M36" s="32">
+        <f>SUM(M4:M35)</f>
+        <v/>
+      </c>
+      <c r="N36" s="32">
+        <f>SUM(N4:N35)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:N27"/>
+  <autoFilter ref="A3:N35"/>
   <mergeCells count="2">
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>

</xml_diff>

<commit_message>
Data update — 2026-10-14 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_oct2026.xlsx
+++ b/results/strategy_pnl_oct2026.xlsx
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trade Log'!$A$3:$O$503</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1994,7 +1994,7 @@
         <v/>
       </c>
       <c r="K19" s="4" t="n">
-        <v>707.5</v>
+        <v>707.6</v>
       </c>
       <c r="L19" s="21">
         <f>IF(OR($B19="",$I19=""),"",$I19-IF($K19="",0,$K19))</f>
@@ -2234,7 +2234,7 @@
         <v/>
       </c>
       <c r="K23" s="4" t="n">
-        <v>344.89</v>
+        <v>419.24</v>
       </c>
       <c r="L23" s="21">
         <f>IF(OR($B23="",$I23=""),"",$I23-IF($K23="",0,$K23))</f>
@@ -2294,7 +2294,7 @@
         <v/>
       </c>
       <c r="K24" s="4" t="n">
-        <v>0</v>
+        <v>218.69</v>
       </c>
       <c r="L24" s="21">
         <f>IF(OR($B24="",$I24=""),"",$I24-IF($K24="",0,$K24))</f>
@@ -2354,7 +2354,7 @@
         <v/>
       </c>
       <c r="K25" s="4" t="n">
-        <v>350.52</v>
+        <v>556.79</v>
       </c>
       <c r="L25" s="21">
         <f>IF(OR($B25="",$I25=""),"",$I25-IF($K25="",0,$K25))</f>
@@ -2414,7 +2414,7 @@
         <v/>
       </c>
       <c r="K26" s="4" t="n">
-        <v>349.27</v>
+        <v>547.09</v>
       </c>
       <c r="L26" s="21">
         <f>IF(OR($B26="",$I26=""),"",$I26-IF($K26="",0,$K26))</f>
@@ -2474,7 +2474,7 @@
         <v/>
       </c>
       <c r="K27" s="4" t="n">
-        <v>349.97</v>
+        <v>547.28</v>
       </c>
       <c r="L27" s="21">
         <f>IF(OR($B27="",$I27=""),"",$I27-IF($K27="",0,$K27))</f>
@@ -2519,8 +2519,12 @@
       <c r="F28" s="26" t="n">
         <v>277</v>
       </c>
-      <c r="G28" s="24" t="inlineStr"/>
-      <c r="H28" s="25" t="inlineStr"/>
+      <c r="G28" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H28" s="25" t="n">
+        <v>608.04</v>
+      </c>
       <c r="I28" s="21">
         <f>IF(OR($B28="",$H28=""),"",IF($C28="LONG",($H28-$E28)*$F28,($E28-$H28)*$F28))</f>
         <v/>
@@ -2530,7 +2534,7 @@
         <v/>
       </c>
       <c r="K28" s="4" t="n">
-        <v>50.15</v>
+        <v>356.25</v>
       </c>
       <c r="L28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($K28="",0,$K28))</f>
@@ -2575,8 +2579,12 @@
       <c r="F29" s="26" t="n">
         <v>15360</v>
       </c>
-      <c r="G29" s="24" t="inlineStr"/>
-      <c r="H29" s="25" t="inlineStr"/>
+      <c r="G29" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H29" s="25" t="n">
+        <v>11.14</v>
+      </c>
       <c r="I29" s="21">
         <f>IF(OR($B29="",$H29=""),"",IF($C29="LONG",($H29-$E29)*$F29,($E29-$H29)*$F29))</f>
         <v/>
@@ -2586,7 +2594,7 @@
         <v/>
       </c>
       <c r="K29" s="4" t="n">
-        <v>50.15</v>
+        <v>349.1</v>
       </c>
       <c r="L29" s="21">
         <f>IF(OR($B29="",$I29=""),"",$I29-IF($K29="",0,$K29))</f>
@@ -2631,8 +2639,12 @@
       <c r="F30" s="26" t="n">
         <v>243</v>
       </c>
-      <c r="G30" s="24" t="inlineStr"/>
-      <c r="H30" s="25" t="inlineStr"/>
+      <c r="G30" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H30" s="25" t="n">
+        <v>358.7</v>
+      </c>
       <c r="I30" s="21">
         <f>IF(OR($B30="",$H30=""),"",IF($C30="LONG",($H30-$E30)*$F30,($E30-$H30)*$F30))</f>
         <v/>
@@ -2642,7 +2654,7 @@
         <v/>
       </c>
       <c r="K30" s="4" t="n">
-        <v>14.75</v>
+        <v>116.58</v>
       </c>
       <c r="L30" s="21">
         <f>IF(OR($B30="",$I30=""),"",$I30-IF($K30="",0,$K30))</f>
@@ -2665,12 +2677,12 @@
     <row r="31">
       <c r="A31" s="23" t="inlineStr">
         <is>
-          <t>DHAN-34126101377609+221261013593609+34126101378109+23126101376709+34126101378409+23126101377009+221261013595709+221261013596109+221261013596609+23126101377809+34126101379309+34126101379709+23126101378409+34126101379809+221261013599309+321261013576809</t>
+          <t>DHAN-221261013593009+23126101376209+34126101378009+221261013594409+23126101376909+23126101377209+23126101377309+321261013574209+321261013574509+23126101377909+34126101379509+321261013575709</t>
         </is>
       </c>
       <c r="B31" s="23" t="inlineStr">
         <is>
-          <t>INDOKEM</t>
+          <t>PIXTRANS</t>
         </is>
       </c>
       <c r="C31" s="23" t="inlineStr">
@@ -2682,13 +2694,17 @@
         <v>46308</v>
       </c>
       <c r="E31" s="25" t="n">
-        <v>677.9853000000001</v>
+        <v>1889.5856</v>
       </c>
       <c r="F31" s="26" t="n">
-        <v>126</v>
-      </c>
-      <c r="G31" s="24" t="inlineStr"/>
-      <c r="H31" s="25" t="inlineStr"/>
+        <v>90</v>
+      </c>
+      <c r="G31" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H31" s="25" t="n">
+        <v>1923.39</v>
+      </c>
       <c r="I31" s="21">
         <f>IF(OR($B31="",$H31=""),"",IF($C31="LONG",($H31-$E31)*$F31,($E31-$H31)*$F31))</f>
         <v/>
@@ -2698,7 +2714,7 @@
         <v/>
       </c>
       <c r="K31" s="4" t="n">
-        <v>14.75</v>
+        <v>347.17</v>
       </c>
       <c r="L31" s="21">
         <f>IF(OR($B31="",$I31=""),"",$I31-IF($K31="",0,$K31))</f>
@@ -2714,19 +2730,19 @@
       </c>
       <c r="O31" s="23" t="inlineStr">
         <is>
-          <t>10-15</t>
+          <t>5-10</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261012625809+321261012626209+23126101284209+23126101284309+321261012626909+34126101276209+34126101277109+321261012628809+221261012640809+23126101286309+34126101278009+321261012630809+221261012643209</t>
+          <t>DHAN-321261013571309+221261013593809+221261013594209+23126101376409+34126101378509+321261013573309+34126101378809+34126101378909+221261013596709+221261013597209+34126101379409+23126101378309+321261013576009</t>
         </is>
       </c>
       <c r="B32" s="23" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>PNCINFRA</t>
         </is>
       </c>
       <c r="C32" s="23" t="inlineStr">
@@ -2735,16 +2751,20 @@
         </is>
       </c>
       <c r="D32" s="24" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="E32" s="25" t="n">
-        <v>22.8999</v>
+        <v>156.7238</v>
       </c>
       <c r="F32" s="26" t="n">
-        <v>3742</v>
-      </c>
-      <c r="G32" s="24" t="inlineStr"/>
-      <c r="H32" s="25" t="inlineStr"/>
+        <v>1086</v>
+      </c>
+      <c r="G32" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H32" s="25" t="n">
+        <v>169.79</v>
+      </c>
       <c r="I32" s="21">
         <f>IF(OR($B32="",$H32=""),"",IF($C32="LONG",($H32-$E32)*$F32,($E32-$H32)*$F32))</f>
         <v/>
@@ -2754,7 +2774,7 @@
         <v/>
       </c>
       <c r="K32" s="4" t="n">
-        <v>53.57</v>
+        <v>349.67</v>
       </c>
       <c r="L32" s="21">
         <f>IF(OR($B32="",$I32=""),"",$I32-IF($K32="",0,$K32))</f>
@@ -2770,37 +2790,41 @@
       </c>
       <c r="O32" s="23" t="inlineStr">
         <is>
-          <t>5-10</t>
+          <t>10-15</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261013593009+23126101376209+34126101378009+221261013594409+23126101376909+23126101377209+23126101377309+321261013574209+321261013574509+23126101377909+34126101379509+321261013575709</t>
+          <t>DHAN-34126101478009</t>
         </is>
       </c>
       <c r="B33" s="23" t="inlineStr">
         <is>
-          <t>PIXTRANS</t>
+          <t>PNCINFRA</t>
         </is>
       </c>
       <c r="C33" s="23" t="inlineStr">
         <is>
-          <t>LONG</t>
+          <t>SHORT</t>
         </is>
       </c>
       <c r="D33" s="24" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="E33" s="25" t="n">
-        <v>1889.5856</v>
+        <v>169.61</v>
       </c>
       <c r="F33" s="26" t="n">
-        <v>90</v>
-      </c>
-      <c r="G33" s="24" t="inlineStr"/>
-      <c r="H33" s="25" t="inlineStr"/>
+        <v>1086</v>
+      </c>
+      <c r="G33" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H33" s="25" t="n">
+        <v>161.13</v>
+      </c>
       <c r="I33" s="21">
         <f>IF(OR($B33="",$H33=""),"",IF($C33="LONG",($H33-$E33)*$F33,($E33-$H33)*$F33))</f>
         <v/>
@@ -2810,7 +2834,7 @@
         <v/>
       </c>
       <c r="K33" s="4" t="n">
-        <v>50.15</v>
+        <v>0</v>
       </c>
       <c r="L33" s="21">
         <f>IF(OR($B33="",$I33=""),"",$I33-IF($K33="",0,$K33))</f>
@@ -2826,19 +2850,19 @@
       </c>
       <c r="O33" s="23" t="inlineStr">
         <is>
-          <t>5-10</t>
+          <t>10-15</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261013571309+221261013593809+221261013594209+23126101376409+34126101378509+321261013573309+34126101378809+34126101378909+221261013596709+221261013597209+34126101379409+23126101378309+321261013576009</t>
+          <t>DHAN-221261013592909+23126101376109+321261013572209+23126101376609+321261013572609+321261013573209+321261013573809+221261013596209+34126101379109+34126101379209+221261013597909</t>
         </is>
       </c>
       <c r="B34" s="23" t="inlineStr">
         <is>
-          <t>PNCINFRA</t>
+          <t>SHRINGARMS</t>
         </is>
       </c>
       <c r="C34" s="23" t="inlineStr">
@@ -2850,13 +2874,17 @@
         <v>46308</v>
       </c>
       <c r="E34" s="25" t="n">
-        <v>156.7238</v>
+        <v>311.7565</v>
       </c>
       <c r="F34" s="26" t="n">
-        <v>1086</v>
-      </c>
-      <c r="G34" s="24" t="inlineStr"/>
-      <c r="H34" s="25" t="inlineStr"/>
+        <v>549</v>
+      </c>
+      <c r="G34" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H34" s="25" t="n">
+        <v>315.82</v>
+      </c>
       <c r="I34" s="21">
         <f>IF(OR($B34="",$H34=""),"",IF($C34="LONG",($H34-$E34)*$F34,($E34-$H34)*$F34))</f>
         <v/>
@@ -2866,7 +2894,7 @@
         <v/>
       </c>
       <c r="K34" s="4" t="n">
-        <v>50.15</v>
+        <v>349.07</v>
       </c>
       <c r="L34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($K34="",0,$K34))</f>
@@ -2882,19 +2910,19 @@
       </c>
       <c r="O34" s="23" t="inlineStr">
         <is>
-          <t>10-15</t>
+          <t>15-20</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261013592909+23126101376109+321261013572209+23126101376609+321261013572609+321261013573209+321261013573809+221261013596209+34126101379109+34126101379209+221261013597909</t>
+          <t>DHAN-34126101377609+221261013593609+34126101378109+23126101376709+34126101378409+23126101377009+221261013595709+221261013596109+221261013596609+23126101377809+34126101379309+34126101379709+23126101378409+34126101379809+221261013599309+321261013576809</t>
         </is>
       </c>
       <c r="B35" s="23" t="inlineStr">
         <is>
-          <t>SHRINGARMS</t>
+          <t>INDOKEM</t>
         </is>
       </c>
       <c r="C35" s="23" t="inlineStr">
@@ -2906,10 +2934,10 @@
         <v>46308</v>
       </c>
       <c r="E35" s="25" t="n">
-        <v>311.7565</v>
+        <v>677.9853000000001</v>
       </c>
       <c r="F35" s="26" t="n">
-        <v>549</v>
+        <v>126</v>
       </c>
       <c r="G35" s="24" t="inlineStr"/>
       <c r="H35" s="25" t="inlineStr"/>
@@ -2922,7 +2950,7 @@
         <v/>
       </c>
       <c r="K35" s="4" t="n">
-        <v>50.15</v>
+        <v>116.19</v>
       </c>
       <c r="L35" s="21">
         <f>IF(OR($B35="",$I35=""),"",$I35-IF($K35="",0,$K35))</f>
@@ -2938,19 +2966,37 @@
       </c>
       <c r="O35" s="23" t="inlineStr">
         <is>
-          <t>15-20</t>
+          <t>10-15</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="23" t="n"/>
-      <c r="B36" s="23" t="n"/>
-      <c r="C36" s="23" t="n"/>
-      <c r="D36" s="24" t="n"/>
-      <c r="E36" s="25" t="n"/>
-      <c r="F36" s="26" t="n"/>
-      <c r="G36" s="24" t="n"/>
-      <c r="H36" s="25" t="n"/>
+      <c r="A36" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261014662909+221261014671509+321261014664009+341261014129509+341261014129709+321261014665509+221261014673509+231261014126609+221261014673809+221261014674109+231261014126809+341261014131109+221261014675709+231261014127209+341261014131309+231261014127309</t>
+        </is>
+      </c>
+      <c r="B36" s="23" t="inlineStr">
+        <is>
+          <t>JINDALPOLY</t>
+        </is>
+      </c>
+      <c r="C36" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D36" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E36" s="25" t="n">
+        <v>726.3234</v>
+      </c>
+      <c r="F36" s="26" t="n">
+        <v>201</v>
+      </c>
+      <c r="G36" s="24" t="inlineStr"/>
+      <c r="H36" s="25" t="inlineStr"/>
       <c r="I36" s="21">
         <f>IF(OR($B36="",$H36=""),"",IF($C36="LONG",($H36-$E36)*$F36,($E36-$H36)*$F36))</f>
         <v/>
@@ -2959,7 +3005,9 @@
         <f>IF(OR($B36="",$I36="",$E36=0,$F36=0),"",$I36/($E36*$F36))</f>
         <v/>
       </c>
-      <c r="K36" s="4" t="n"/>
+      <c r="K36" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L36" s="21">
         <f>IF(OR($B36="",$I36=""),"",$I36-IF($K36="",0,$K36))</f>
         <v/>
@@ -2972,17 +3020,39 @@
         <f>IF($B36="","",IF($H36="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O36" s="23" t="n"/>
+      <c r="O36" s="23" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="23" t="n"/>
-      <c r="B37" s="23" t="n"/>
-      <c r="C37" s="23" t="n"/>
-      <c r="D37" s="24" t="n"/>
-      <c r="E37" s="25" t="n"/>
-      <c r="F37" s="26" t="n"/>
-      <c r="G37" s="24" t="n"/>
-      <c r="H37" s="25" t="n"/>
+      <c r="A37" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261014663009+221261014671609+341261014129309+221261014671909+341261014129609+341261014129809+231261014126309+321261014666109+231261014126509+341261014130409+231261014126709+231261014126909</t>
+        </is>
+      </c>
+      <c r="B37" s="23" t="inlineStr">
+        <is>
+          <t>KROSS</t>
+        </is>
+      </c>
+      <c r="C37" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D37" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E37" s="25" t="n">
+        <v>271.509</v>
+      </c>
+      <c r="F37" s="26" t="n">
+        <v>737</v>
+      </c>
+      <c r="G37" s="24" t="inlineStr"/>
+      <c r="H37" s="25" t="inlineStr"/>
       <c r="I37" s="21">
         <f>IF(OR($B37="",$H37=""),"",IF($C37="LONG",($H37-$E37)*$F37,($E37-$H37)*$F37))</f>
         <v/>
@@ -2991,7 +3061,9 @@
         <f>IF(OR($B37="",$I37="",$E37=0,$F37=0),"",$I37/($E37*$F37))</f>
         <v/>
       </c>
-      <c r="K37" s="4" t="n"/>
+      <c r="K37" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L37" s="21">
         <f>IF(OR($B37="",$I37=""),"",$I37-IF($K37="",0,$K37))</f>
         <v/>
@@ -3004,17 +3076,39 @@
         <f>IF($B37="","",IF($H37="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O37" s="23" t="n"/>
+      <c r="O37" s="23" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="23" t="n"/>
-      <c r="B38" s="23" t="n"/>
-      <c r="C38" s="23" t="n"/>
-      <c r="D38" s="24" t="n"/>
-      <c r="E38" s="25" t="n"/>
-      <c r="F38" s="26" t="n"/>
-      <c r="G38" s="24" t="n"/>
-      <c r="H38" s="25" t="n"/>
+      <c r="A38" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261012625809+321261012626209+23126101284209+23126101284309+321261012626909+34126101276209+34126101277109+321261012628809+221261012640809+23126101286309+34126101278009+321261012630809+221261012643209</t>
+        </is>
+      </c>
+      <c r="B38" s="23" t="inlineStr">
+        <is>
+          <t>MMWL</t>
+        </is>
+      </c>
+      <c r="C38" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D38" s="24" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E38" s="25" t="n">
+        <v>22.8999</v>
+      </c>
+      <c r="F38" s="26" t="n">
+        <v>3742</v>
+      </c>
+      <c r="G38" s="24" t="inlineStr"/>
+      <c r="H38" s="25" t="inlineStr"/>
       <c r="I38" s="21">
         <f>IF(OR($B38="",$H38=""),"",IF($C38="LONG",($H38-$E38)*$F38,($E38-$H38)*$F38))</f>
         <v/>
@@ -3023,7 +3117,9 @@
         <f>IF(OR($B38="",$I38="",$E38=0,$F38=0),"",$I38/($E38*$F38))</f>
         <v/>
       </c>
-      <c r="K38" s="4" t="n"/>
+      <c r="K38" s="4" t="n">
+        <v>53.57</v>
+      </c>
       <c r="L38" s="21">
         <f>IF(OR($B38="",$I38=""),"",$I38-IF($K38="",0,$K38))</f>
         <v/>
@@ -3036,17 +3132,39 @@
         <f>IF($B38="","",IF($H38="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O38" s="23" t="n"/>
+      <c r="O38" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="23" t="n"/>
-      <c r="B39" s="23" t="n"/>
-      <c r="C39" s="23" t="n"/>
-      <c r="D39" s="24" t="n"/>
-      <c r="E39" s="25" t="n"/>
-      <c r="F39" s="26" t="n"/>
-      <c r="G39" s="24" t="n"/>
-      <c r="H39" s="25" t="n"/>
+      <c r="A39" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-341261014128909+341261014129109+231261014125709+321261014664109+321261014664809+231261014126009+321261014665609+231261014126409+341261014130309+341261014130509+221261014673909+341261014130709+221261014674609+221261014675009+221261014675509</t>
+        </is>
+      </c>
+      <c r="B39" s="23" t="inlineStr">
+        <is>
+          <t>NIBE</t>
+        </is>
+      </c>
+      <c r="C39" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D39" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E39" s="25" t="n">
+        <v>1380.7368</v>
+      </c>
+      <c r="F39" s="26" t="n">
+        <v>144</v>
+      </c>
+      <c r="G39" s="24" t="inlineStr"/>
+      <c r="H39" s="25" t="inlineStr"/>
       <c r="I39" s="21">
         <f>IF(OR($B39="",$H39=""),"",IF($C39="LONG",($H39-$E39)*$F39,($E39-$H39)*$F39))</f>
         <v/>
@@ -3055,7 +3173,9 @@
         <f>IF(OR($B39="",$I39="",$E39=0,$F39=0),"",$I39/($E39*$F39))</f>
         <v/>
       </c>
-      <c r="K39" s="4" t="n"/>
+      <c r="K39" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L39" s="21">
         <f>IF(OR($B39="",$I39=""),"",$I39-IF($K39="",0,$K39))</f>
         <v/>
@@ -3068,17 +3188,39 @@
         <f>IF($B39="","",IF($H39="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O39" s="23" t="n"/>
+      <c r="O39" s="23" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" s="23" t="n"/>
-      <c r="B40" s="23" t="n"/>
-      <c r="C40" s="23" t="n"/>
-      <c r="D40" s="24" t="n"/>
-      <c r="E40" s="25" t="n"/>
-      <c r="F40" s="26" t="n"/>
-      <c r="G40" s="24" t="n"/>
-      <c r="H40" s="25" t="n"/>
+      <c r="A40" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261014671209+321261014663609+231261014125809+221261014672009+231261014125909+231261014126109+221261014673109+341261014130209+321261014666509+341261014130609+321261014667409+321261014667809+341261014131209+221261014676209+221261014676809</t>
+        </is>
+      </c>
+      <c r="B40" s="23" t="inlineStr">
+        <is>
+          <t>RUBYMILLS</t>
+        </is>
+      </c>
+      <c r="C40" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D40" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E40" s="25" t="n">
+        <v>541.4497</v>
+      </c>
+      <c r="F40" s="26" t="n">
+        <v>184</v>
+      </c>
+      <c r="G40" s="24" t="inlineStr"/>
+      <c r="H40" s="25" t="inlineStr"/>
       <c r="I40" s="21">
         <f>IF(OR($B40="",$H40=""),"",IF($C40="LONG",($H40-$E40)*$F40,($E40-$H40)*$F40))</f>
         <v/>
@@ -3087,7 +3229,9 @@
         <f>IF(OR($B40="",$I40="",$E40=0,$F40=0),"",$I40/($E40*$F40))</f>
         <v/>
       </c>
-      <c r="K40" s="4" t="n"/>
+      <c r="K40" s="4" t="n">
+        <v>14.75</v>
+      </c>
       <c r="L40" s="21">
         <f>IF(OR($B40="",$I40=""),"",$I40-IF($K40="",0,$K40))</f>
         <v/>
@@ -3100,17 +3244,39 @@
         <f>IF($B40="","",IF($H40="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O40" s="23" t="n"/>
+      <c r="O40" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" s="23" t="n"/>
-      <c r="B41" s="23" t="n"/>
-      <c r="C41" s="23" t="n"/>
-      <c r="D41" s="24" t="n"/>
-      <c r="E41" s="25" t="n"/>
-      <c r="F41" s="26" t="n"/>
-      <c r="G41" s="24" t="n"/>
-      <c r="H41" s="25" t="n"/>
+      <c r="A41" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-341261014128809+341261014129209+221261014671809+321261014664309+221261014672409+321261014664909+341261014130009+221261014673409+221261014673609+221261014673709+221261014674009+321261014667309+341261014130909</t>
+        </is>
+      </c>
+      <c r="B41" s="23" t="inlineStr">
+        <is>
+          <t>SIMPLEXINF</t>
+        </is>
+      </c>
+      <c r="C41" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D41" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E41" s="25" t="n">
+        <v>266.801</v>
+      </c>
+      <c r="F41" s="26" t="n">
+        <v>749</v>
+      </c>
+      <c r="G41" s="24" t="inlineStr"/>
+      <c r="H41" s="25" t="inlineStr"/>
       <c r="I41" s="21">
         <f>IF(OR($B41="",$H41=""),"",IF($C41="LONG",($H41-$E41)*$F41,($E41-$H41)*$F41))</f>
         <v/>
@@ -3119,7 +3285,9 @@
         <f>IF(OR($B41="",$I41="",$E41=0,$F41=0),"",$I41/($E41*$F41))</f>
         <v/>
       </c>
-      <c r="K41" s="4" t="n"/>
+      <c r="K41" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L41" s="21">
         <f>IF(OR($B41="",$I41=""),"",$I41-IF($K41="",0,$K41))</f>
         <v/>
@@ -3132,17 +3300,39 @@
         <f>IF($B41="","",IF($H41="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O41" s="23" t="n"/>
+      <c r="O41" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="23" t="n"/>
-      <c r="B42" s="23" t="n"/>
-      <c r="C42" s="23" t="n"/>
-      <c r="D42" s="24" t="n"/>
-      <c r="E42" s="25" t="n"/>
-      <c r="F42" s="26" t="n"/>
-      <c r="G42" s="24" t="n"/>
-      <c r="H42" s="25" t="n"/>
+      <c r="A42" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-231261014125609+321261014663509+321261014663909+321261014664209+221261014672509+231261014126209+341261014130109+321261014666209+321261014666609+321261014666709+321261014667009+341261014130809+231261014127009+341261014131009+221261014675609</t>
+        </is>
+      </c>
+      <c r="B42" s="23" t="inlineStr">
+        <is>
+          <t>SPORTKING</t>
+        </is>
+      </c>
+      <c r="C42" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D42" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E42" s="25" t="n">
+        <v>226.1107</v>
+      </c>
+      <c r="F42" s="26" t="n">
+        <v>885</v>
+      </c>
+      <c r="G42" s="24" t="inlineStr"/>
+      <c r="H42" s="25" t="inlineStr"/>
       <c r="I42" s="21">
         <f>IF(OR($B42="",$H42=""),"",IF($C42="LONG",($H42-$E42)*$F42,($E42-$H42)*$F42))</f>
         <v/>
@@ -3151,7 +3341,9 @@
         <f>IF(OR($B42="",$I42="",$E42=0,$F42=0),"",$I42/($E42*$F42))</f>
         <v/>
       </c>
-      <c r="K42" s="4" t="n"/>
+      <c r="K42" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L42" s="21">
         <f>IF(OR($B42="",$I42=""),"",$I42-IF($K42="",0,$K42))</f>
         <v/>
@@ -3164,7 +3356,11 @@
         <f>IF($B42="","",IF($H42="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O42" s="23" t="n"/>
+      <c r="O42" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="23" t="n"/>
@@ -30593,7 +30789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31150,7 +31346,7 @@
     <row r="15">
       <c r="A15" s="27" t="inlineStr">
         <is>
-          <t>KOTIC</t>
+          <t>JINDALPOLY</t>
         </is>
       </c>
       <c r="B15" s="20">
@@ -31193,7 +31389,7 @@
     <row r="16">
       <c r="A16" s="27" t="inlineStr">
         <is>
-          <t>KRISHNADEF</t>
+          <t>KOTIC</t>
         </is>
       </c>
       <c r="B16" s="20">
@@ -31236,7 +31432,7 @@
     <row r="17">
       <c r="A17" s="27" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>KRISHNADEF</t>
         </is>
       </c>
       <c r="B17" s="20">
@@ -31279,7 +31475,7 @@
     <row r="18">
       <c r="A18" s="27" t="inlineStr">
         <is>
-          <t>MOBIKWIK</t>
+          <t>KROSS</t>
         </is>
       </c>
       <c r="B18" s="20">
@@ -31322,7 +31518,7 @@
     <row r="19">
       <c r="A19" s="27" t="inlineStr">
         <is>
-          <t>PIXTRANS</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="B19" s="20">
@@ -31365,7 +31561,7 @@
     <row r="20">
       <c r="A20" s="27" t="inlineStr">
         <is>
-          <t>PNCINFRA</t>
+          <t>MOBIKWIK</t>
         </is>
       </c>
       <c r="B20" s="20">
@@ -31408,7 +31604,7 @@
     <row r="21">
       <c r="A21" s="27" t="inlineStr">
         <is>
-          <t>PNGSREVA</t>
+          <t>NIBE</t>
         </is>
       </c>
       <c r="B21" s="20">
@@ -31451,7 +31647,7 @@
     <row r="22">
       <c r="A22" s="27" t="inlineStr">
         <is>
-          <t>PRINCEPIPE</t>
+          <t>PIXTRANS</t>
         </is>
       </c>
       <c r="B22" s="20">
@@ -31494,7 +31690,7 @@
     <row r="23">
       <c r="A23" s="27" t="inlineStr">
         <is>
-          <t>RSYSTEMS</t>
+          <t>PNCINFRA</t>
         </is>
       </c>
       <c r="B23" s="20">
@@ -31537,7 +31733,7 @@
     <row r="24">
       <c r="A24" s="27" t="inlineStr">
         <is>
-          <t>SAKSOFT</t>
+          <t>PNGSREVA</t>
         </is>
       </c>
       <c r="B24" s="20">
@@ -31580,7 +31776,7 @@
     <row r="25">
       <c r="A25" s="27" t="inlineStr">
         <is>
-          <t>SATIN</t>
+          <t>PRINCEPIPE</t>
         </is>
       </c>
       <c r="B25" s="20">
@@ -31623,7 +31819,7 @@
     <row r="26">
       <c r="A26" s="27" t="inlineStr">
         <is>
-          <t>SGFIN</t>
+          <t>RSYSTEMS</t>
         </is>
       </c>
       <c r="B26" s="20">
@@ -31666,7 +31862,7 @@
     <row r="27">
       <c r="A27" s="27" t="inlineStr">
         <is>
-          <t>SHRINGARMS</t>
+          <t>RUBYMILLS</t>
         </is>
       </c>
       <c r="B27" s="20">
@@ -31709,7 +31905,7 @@
     <row r="28">
       <c r="A28" s="27" t="inlineStr">
         <is>
-          <t>SMCGLOBAL</t>
+          <t>SAKSOFT</t>
         </is>
       </c>
       <c r="B28" s="20">
@@ -31752,7 +31948,7 @@
     <row r="29">
       <c r="A29" s="27" t="inlineStr">
         <is>
-          <t>SUNCLAY</t>
+          <t>SATIN</t>
         </is>
       </c>
       <c r="B29" s="20">
@@ -31795,7 +31991,7 @@
     <row r="30">
       <c r="A30" s="27" t="inlineStr">
         <is>
-          <t>SWARAJENG</t>
+          <t>SGFIN</t>
         </is>
       </c>
       <c r="B30" s="20">
@@ -31838,7 +32034,7 @@
     <row r="31">
       <c r="A31" s="27" t="inlineStr">
         <is>
-          <t>YUKEN</t>
+          <t>SHRINGARMS</t>
         </is>
       </c>
       <c r="B31" s="20">
@@ -31879,37 +32075,295 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
+      <c r="A32" s="27" t="inlineStr">
+        <is>
+          <t>SIMPLEXINF</t>
+        </is>
+      </c>
+      <c r="B32" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A32)</f>
+        <v/>
+      </c>
+      <c r="C32" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A32,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D32" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A32,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E32" s="22">
+        <f>IFERROR($C32/$B32,"")</f>
+        <v/>
+      </c>
+      <c r="F32" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A32,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G32" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A32,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H32" s="21">
+        <f>IFERROR($G32/$B32,"")</f>
+        <v/>
+      </c>
+      <c r="I32" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A32),"")</f>
+        <v/>
+      </c>
+      <c r="J32" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A32),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="27" t="inlineStr">
+        <is>
+          <t>SMCGLOBAL</t>
+        </is>
+      </c>
+      <c r="B33" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A33)</f>
+        <v/>
+      </c>
+      <c r="C33" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A33,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D33" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A33,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E33" s="22">
+        <f>IFERROR($C33/$B33,"")</f>
+        <v/>
+      </c>
+      <c r="F33" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A33,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G33" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A33,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H33" s="21">
+        <f>IFERROR($G33/$B33,"")</f>
+        <v/>
+      </c>
+      <c r="I33" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A33),"")</f>
+        <v/>
+      </c>
+      <c r="J33" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A33),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="27" t="inlineStr">
+        <is>
+          <t>SPORTKING</t>
+        </is>
+      </c>
+      <c r="B34" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A34)</f>
+        <v/>
+      </c>
+      <c r="C34" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A34,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D34" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A34,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E34" s="22">
+        <f>IFERROR($C34/$B34,"")</f>
+        <v/>
+      </c>
+      <c r="F34" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A34,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G34" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A34,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H34" s="21">
+        <f>IFERROR($G34/$B34,"")</f>
+        <v/>
+      </c>
+      <c r="I34" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A34),"")</f>
+        <v/>
+      </c>
+      <c r="J34" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A34),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="27" t="inlineStr">
+        <is>
+          <t>SUNCLAY</t>
+        </is>
+      </c>
+      <c r="B35" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A35)</f>
+        <v/>
+      </c>
+      <c r="C35" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A35,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D35" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A35,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E35" s="22">
+        <f>IFERROR($C35/$B35,"")</f>
+        <v/>
+      </c>
+      <c r="F35" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A35,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G35" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A35,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H35" s="21">
+        <f>IFERROR($G35/$B35,"")</f>
+        <v/>
+      </c>
+      <c r="I35" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A35),"")</f>
+        <v/>
+      </c>
+      <c r="J35" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A35),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="27" t="inlineStr">
+        <is>
+          <t>SWARAJENG</t>
+        </is>
+      </c>
+      <c r="B36" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A36)</f>
+        <v/>
+      </c>
+      <c r="C36" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A36,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D36" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A36,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E36" s="22">
+        <f>IFERROR($C36/$B36,"")</f>
+        <v/>
+      </c>
+      <c r="F36" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A36,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G36" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A36,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H36" s="21">
+        <f>IFERROR($G36/$B36,"")</f>
+        <v/>
+      </c>
+      <c r="I36" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A36),"")</f>
+        <v/>
+      </c>
+      <c r="J36" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A36),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="27" t="inlineStr">
+        <is>
+          <t>YUKEN</t>
+        </is>
+      </c>
+      <c r="B37" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A37)</f>
+        <v/>
+      </c>
+      <c r="C37" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A37,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D37" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A37,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E37" s="22">
+        <f>IFERROR($C37/$B37,"")</f>
+        <v/>
+      </c>
+      <c r="F37" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A37,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G37" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A37,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H37" s="21">
+        <f>IFERROR($G37/$B37,"")</f>
+        <v/>
+      </c>
+      <c r="I37" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A37),"")</f>
+        <v/>
+      </c>
+      <c r="J37" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A37),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B32" s="30">
-        <f>SUM(B4:B31)</f>
-        <v/>
-      </c>
-      <c r="C32" s="30">
-        <f>SUM(C4:C31)</f>
-        <v/>
-      </c>
-      <c r="D32" s="30">
-        <f>SUM(D4:D31)</f>
-        <v/>
-      </c>
-      <c r="E32" s="31">
-        <f>IFERROR(C32/B32,"")</f>
-        <v/>
-      </c>
-      <c r="F32" s="32">
-        <f>SUM(F4:F31)</f>
-        <v/>
-      </c>
-      <c r="G32" s="32">
-        <f>SUM(G4:G31)</f>
-        <v/>
-      </c>
-      <c r="H32" s="32">
-        <f>IFERROR(G32/B32,"")</f>
+      <c r="B38" s="30">
+        <f>SUM(B4:B37)</f>
+        <v/>
+      </c>
+      <c r="C38" s="30">
+        <f>SUM(C4:C37)</f>
+        <v/>
+      </c>
+      <c r="D38" s="30">
+        <f>SUM(D4:D37)</f>
+        <v/>
+      </c>
+      <c r="E38" s="31">
+        <f>IFERROR(C38/B38,"")</f>
+        <v/>
+      </c>
+      <c r="F38" s="32">
+        <f>SUM(F4:F37)</f>
+        <v/>
+      </c>
+      <c r="G38" s="32">
+        <f>SUM(G4:G37)</f>
+        <v/>
+      </c>
+      <c r="H38" s="32">
+        <f>IFERROR(G38/B38,"")</f>
         <v/>
       </c>
     </row>
@@ -31928,7 +32382,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N36"/>
+  <dimension ref="A1:N43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -32842,7 +33296,7 @@
         <v>35.4</v>
       </c>
       <c r="M19" s="4" t="n">
-        <v>127.32</v>
+        <v>127.42</v>
       </c>
       <c r="N19" s="21">
         <f>SUM(E19:M19)</f>
@@ -33022,22 +33476,22 @@
         <v>46308</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>51.61</v>
+        <v>71.61</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>172.14</v>
+        <v>216.25</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>5.28</v>
+        <v>10.74</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>0.17</v>
+        <v>0.35</v>
       </c>
       <c r="I23" s="4" t="n">
         <v>25.82</v>
       </c>
       <c r="J23" s="4" t="n">
-        <v>10.27</v>
+        <v>14.89</v>
       </c>
       <c r="K23" s="4" t="n">
         <v>14.75</v>
@@ -33073,22 +33527,22 @@
         <v>46308</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>0</v>
+        <v>176.73</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>0</v>
+        <v>10.8</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>0</v>
+        <v>0.35</v>
       </c>
       <c r="I24" s="4" t="n">
-        <v>0</v>
+        <v>5.21</v>
       </c>
       <c r="J24" s="4" t="n">
-        <v>0</v>
+        <v>5.61</v>
       </c>
       <c r="K24" s="4" t="n">
         <v>0</v>
@@ -33124,22 +33578,22 @@
         <v>46308</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>51.35</v>
+        <v>71.34999999999999</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>171.15</v>
+        <v>347.2</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>5.25</v>
+        <v>10.66</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>0.17</v>
+        <v>0.35</v>
       </c>
       <c r="I25" s="4" t="n">
         <v>25.67</v>
       </c>
       <c r="J25" s="4" t="n">
-        <v>10.22</v>
+        <v>14.82</v>
       </c>
       <c r="K25" s="4" t="n">
         <v>14.75</v>
@@ -33148,7 +33602,7 @@
         <v>35.4</v>
       </c>
       <c r="M25" s="4" t="n">
-        <v>36.56</v>
+        <v>36.59</v>
       </c>
       <c r="N25" s="21">
         <f>SUM(E25:M25)</f>
@@ -33175,22 +33629,22 @@
         <v>46308</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>51.44</v>
+        <v>71.44</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>171.54</v>
+        <v>339.48</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>5.27</v>
+        <v>10.42</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>0.17</v>
+        <v>0.34</v>
       </c>
       <c r="I26" s="4" t="n">
         <v>25.26</v>
       </c>
       <c r="J26" s="4" t="n">
-        <v>10.24</v>
+        <v>14.8</v>
       </c>
       <c r="K26" s="4" t="n">
         <v>14.75</v>
@@ -33226,22 +33680,22 @@
         <v>46308</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>50.51</v>
+        <v>70.51000000000001</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>168.36</v>
+        <v>335.81</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>5.17</v>
+        <v>10.31</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>0.17</v>
+        <v>0.34</v>
       </c>
       <c r="I27" s="4" t="n">
         <v>25.25</v>
       </c>
       <c r="J27" s="4" t="n">
-        <v>10.05</v>
+        <v>14.61</v>
       </c>
       <c r="K27" s="4" t="n">
         <v>14.75</v>
@@ -33273,24 +33727,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D28" s="24" t="inlineStr"/>
+      <c r="D28" s="24" t="n">
+        <v>46309</v>
+      </c>
       <c r="E28" s="4" t="n">
-        <v>0</v>
+        <v>51.3</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>0</v>
+        <v>170.95</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>0</v>
+        <v>5.25</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>0</v>
+        <v>0.17</v>
       </c>
       <c r="I28" s="4" t="n">
-        <v>0</v>
+        <v>25.64</v>
       </c>
       <c r="J28" s="4" t="n">
-        <v>0</v>
+        <v>10.21</v>
       </c>
       <c r="K28" s="4" t="n">
         <v>14.75</v>
@@ -33299,7 +33755,7 @@
         <v>35.4</v>
       </c>
       <c r="M28" s="4" t="n">
-        <v>0</v>
+        <v>42.58</v>
       </c>
       <c r="N28" s="21">
         <f>SUM(E28:M28)</f>
@@ -33322,24 +33778,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D29" s="24" t="inlineStr"/>
+      <c r="D29" s="24" t="n">
+        <v>46309</v>
+      </c>
       <c r="E29" s="4" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>0</v>
+        <v>171.42</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>0</v>
+        <v>5.26</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>0</v>
+        <v>0.17</v>
       </c>
       <c r="I29" s="4" t="n">
-        <v>0</v>
+        <v>25.77</v>
       </c>
       <c r="J29" s="4" t="n">
-        <v>0</v>
+        <v>10.16</v>
       </c>
       <c r="K29" s="4" t="n">
         <v>14.75</v>
@@ -33348,7 +33806,7 @@
         <v>35.4</v>
       </c>
       <c r="M29" s="4" t="n">
-        <v>0</v>
+        <v>35.17</v>
       </c>
       <c r="N29" s="21">
         <f>SUM(E29:M29)</f>
@@ -33371,24 +33829,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D30" s="24" t="inlineStr"/>
+      <c r="D30" s="24" t="n">
+        <v>46309</v>
+      </c>
       <c r="E30" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>0</v>
+        <v>85.76000000000001</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>0</v>
+        <v>2.63</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>0</v>
+        <v>0.09</v>
       </c>
       <c r="I30" s="4" t="n">
-        <v>0</v>
+        <v>12.86</v>
       </c>
       <c r="J30" s="4" t="n">
-        <v>0</v>
+        <v>0.49</v>
       </c>
       <c r="K30" s="4" t="n">
         <v>14.75</v>
@@ -33407,12 +33867,12 @@
     <row r="31">
       <c r="A31" s="23" t="inlineStr">
         <is>
-          <t>DHAN-34126101377609+221261013593609+34126101378109+23126101376709+34126101378409+23126101377009+221261013595709+221261013596109+221261013596609+23126101377809+34126101379309+34126101379709+23126101378409+34126101379809+221261013599309+321261013576809</t>
+          <t>DHAN-221261013593009+23126101376209+34126101378009+221261013594409+23126101376909+23126101377209+23126101377309+321261013574209+321261013574509+23126101377909+34126101379509+321261013575709</t>
         </is>
       </c>
       <c r="B31" s="23" t="inlineStr">
         <is>
-          <t>INDOKEM</t>
+          <t>PIXTRANS</t>
         </is>
       </c>
       <c r="C31" s="23" t="inlineStr">
@@ -33420,33 +33880,35 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D31" s="24" t="inlineStr"/>
+      <c r="D31" s="24" t="n">
+        <v>46309</v>
+      </c>
       <c r="E31" s="4" t="n">
-        <v>0</v>
+        <v>51.01</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>0</v>
+        <v>170.06</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>0</v>
+        <v>5.22</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>0</v>
+        <v>0.17</v>
       </c>
       <c r="I31" s="4" t="n">
-        <v>0</v>
+        <v>25.51</v>
       </c>
       <c r="J31" s="4" t="n">
-        <v>0</v>
+        <v>10.15</v>
       </c>
       <c r="K31" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L31" s="4" t="n">
-        <v>0</v>
+        <v>35.4</v>
       </c>
       <c r="M31" s="4" t="n">
-        <v>0</v>
+        <v>34.9</v>
       </c>
       <c r="N31" s="21">
         <f>SUM(E31:M31)</f>
@@ -33456,12 +33918,12 @@
     <row r="32">
       <c r="A32" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261012625809+321261012626209+23126101284209+23126101284309+321261012626909+34126101276209+34126101277109+321261012628809+221261012640809+23126101286309+34126101278009+321261012630809+221261012643209</t>
+          <t>DHAN-321261013571309+221261013593809+221261013594209+23126101376409+34126101378509+321261013573309+34126101378809+34126101378909+221261013596709+221261013597209+34126101379409+23126101378309+321261013576009</t>
         </is>
       </c>
       <c r="B32" s="23" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>PNCINFRA</t>
         </is>
       </c>
       <c r="C32" s="23" t="inlineStr">
@@ -33469,33 +33931,35 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D32" s="24" t="inlineStr"/>
+      <c r="D32" s="24" t="n">
+        <v>46309</v>
+      </c>
       <c r="E32" s="4" t="n">
-        <v>24.76</v>
+        <v>51.07</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>3.4</v>
+        <v>170.2</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>2.63</v>
+        <v>5.22</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>0.09</v>
+        <v>0.17</v>
       </c>
       <c r="I32" s="4" t="n">
-        <v>3</v>
+        <v>25.53</v>
       </c>
       <c r="J32" s="4" t="n">
-        <v>4.95</v>
+        <v>10.16</v>
       </c>
       <c r="K32" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L32" s="4" t="n">
-        <v>0</v>
+        <v>35.4</v>
       </c>
       <c r="M32" s="4" t="n">
-        <v>0</v>
+        <v>37.16</v>
       </c>
       <c r="N32" s="21">
         <f>SUM(E32:M32)</f>
@@ -33505,20 +33969,22 @@
     <row r="33">
       <c r="A33" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261013593009+23126101376209+34126101378009+221261013594409+23126101376909+23126101377209+23126101377309+321261013574209+321261013574509+23126101377909+34126101379509+321261013575709</t>
+          <t>DHAN-34126101478009</t>
         </is>
       </c>
       <c r="B33" s="23" t="inlineStr">
         <is>
-          <t>PIXTRANS</t>
+          <t>PNCINFRA</t>
         </is>
       </c>
       <c r="C33" s="23" t="inlineStr">
         <is>
-          <t>LONG</t>
-        </is>
-      </c>
-      <c r="D33" s="24" t="inlineStr"/>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D33" s="24" t="n">
+        <v>46309</v>
+      </c>
       <c r="E33" s="4" t="n">
         <v>0</v>
       </c>
@@ -33538,10 +34004,10 @@
         <v>0</v>
       </c>
       <c r="K33" s="4" t="n">
-        <v>14.75</v>
+        <v>0</v>
       </c>
       <c r="L33" s="4" t="n">
-        <v>35.4</v>
+        <v>0</v>
       </c>
       <c r="M33" s="4" t="n">
         <v>0</v>
@@ -33554,12 +34020,12 @@
     <row r="34">
       <c r="A34" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261013571309+221261013593809+221261013594209+23126101376409+34126101378509+321261013573309+34126101378809+34126101378909+221261013596709+221261013597209+34126101379409+23126101378309+321261013576009</t>
+          <t>DHAN-221261013592909+23126101376109+321261013572209+23126101376609+321261013572609+321261013573209+321261013573809+221261013596209+34126101379109+34126101379209+221261013597909</t>
         </is>
       </c>
       <c r="B34" s="23" t="inlineStr">
         <is>
-          <t>PNCINFRA</t>
+          <t>SHRINGARMS</t>
         </is>
       </c>
       <c r="C34" s="23" t="inlineStr">
@@ -33567,24 +34033,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D34" s="24" t="inlineStr"/>
+      <c r="D34" s="24" t="n">
+        <v>46309</v>
+      </c>
       <c r="E34" s="4" t="n">
-        <v>0</v>
+        <v>51.33</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>0</v>
+        <v>171.16</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>0</v>
+        <v>5.25</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>0</v>
+        <v>0.17</v>
       </c>
       <c r="I34" s="4" t="n">
-        <v>0</v>
+        <v>25.67</v>
       </c>
       <c r="J34" s="4" t="n">
-        <v>0</v>
+        <v>10.22</v>
       </c>
       <c r="K34" s="4" t="n">
         <v>14.75</v>
@@ -33593,7 +34061,7 @@
         <v>35.4</v>
       </c>
       <c r="M34" s="4" t="n">
-        <v>0</v>
+        <v>35.12</v>
       </c>
       <c r="N34" s="21">
         <f>SUM(E34:M34)</f>
@@ -33603,12 +34071,12 @@
     <row r="35">
       <c r="A35" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261013592909+23126101376109+321261013572209+23126101376609+321261013572609+321261013573209+321261013573809+221261013596209+34126101379109+34126101379209+221261013597909</t>
+          <t>DHAN-34126101377609+221261013593609+34126101378109+23126101376709+34126101378409+23126101377009+221261013595709+221261013596109+221261013596609+23126101377809+34126101379309+34126101379709+23126101378409+34126101379809+221261013599309+321261013576809</t>
         </is>
       </c>
       <c r="B35" s="23" t="inlineStr">
         <is>
-          <t>SHRINGARMS</t>
+          <t>INDOKEM</t>
         </is>
       </c>
       <c r="C35" s="23" t="inlineStr">
@@ -33621,25 +34089,25 @@
         <v>0</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>0</v>
+        <v>85.43000000000001</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>0</v>
+        <v>2.62</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>0</v>
+        <v>0.09</v>
       </c>
       <c r="I35" s="4" t="n">
-        <v>0</v>
+        <v>12.81</v>
       </c>
       <c r="J35" s="4" t="n">
-        <v>0</v>
+        <v>0.49</v>
       </c>
       <c r="K35" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L35" s="4" t="n">
-        <v>35.4</v>
+        <v>0</v>
       </c>
       <c r="M35" s="4" t="n">
         <v>0</v>
@@ -33650,54 +34118,397 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="3" t="inlineStr">
+      <c r="A36" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261014662909+221261014671509+321261014664009+341261014129509+341261014129709+321261014665509+221261014673509+231261014126609+221261014673809+221261014674109+231261014126809+341261014131109+221261014675709+231261014127209+341261014131309+231261014127309</t>
+        </is>
+      </c>
+      <c r="B36" s="23" t="inlineStr">
+        <is>
+          <t>JINDALPOLY</t>
+        </is>
+      </c>
+      <c r="C36" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D36" s="24" t="inlineStr"/>
+      <c r="E36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L36" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N36" s="21">
+        <f>SUM(E36:M36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261014663009+221261014671609+341261014129309+221261014671909+341261014129609+341261014129809+231261014126309+321261014666109+231261014126509+341261014130409+231261014126709+231261014126909</t>
+        </is>
+      </c>
+      <c r="B37" s="23" t="inlineStr">
+        <is>
+          <t>KROSS</t>
+        </is>
+      </c>
+      <c r="C37" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D37" s="24" t="inlineStr"/>
+      <c r="E37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L37" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N37" s="21">
+        <f>SUM(E37:M37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261012625809+321261012626209+23126101284209+23126101284309+321261012626909+34126101276209+34126101277109+321261012628809+221261012640809+23126101286309+34126101278009+321261012630809+221261012643209</t>
+        </is>
+      </c>
+      <c r="B38" s="23" t="inlineStr">
+        <is>
+          <t>MMWL</t>
+        </is>
+      </c>
+      <c r="C38" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D38" s="24" t="inlineStr"/>
+      <c r="E38" s="4" t="n">
+        <v>24.76</v>
+      </c>
+      <c r="F38" s="4" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="G38" s="4" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="H38" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="I38" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J38" s="4" t="n">
+        <v>4.95</v>
+      </c>
+      <c r="K38" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N38" s="21">
+        <f>SUM(E38:M38)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-341261014128909+341261014129109+231261014125709+321261014664109+321261014664809+231261014126009+321261014665609+231261014126409+341261014130309+341261014130509+221261014673909+341261014130709+221261014674609+221261014675009+221261014675509</t>
+        </is>
+      </c>
+      <c r="B39" s="23" t="inlineStr">
+        <is>
+          <t>NIBE</t>
+        </is>
+      </c>
+      <c r="C39" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D39" s="24" t="inlineStr"/>
+      <c r="E39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K39" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L39" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N39" s="21">
+        <f>SUM(E39:M39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261014671209+321261014663609+231261014125809+221261014672009+231261014125909+231261014126109+221261014673109+341261014130209+321261014666509+341261014130609+321261014667409+321261014667809+341261014131209+221261014676209+221261014676809</t>
+        </is>
+      </c>
+      <c r="B40" s="23" t="inlineStr">
+        <is>
+          <t>RUBYMILLS</t>
+        </is>
+      </c>
+      <c r="C40" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D40" s="24" t="inlineStr"/>
+      <c r="E40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N40" s="21">
+        <f>SUM(E40:M40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-341261014128809+341261014129209+221261014671809+321261014664309+221261014672409+321261014664909+341261014130009+221261014673409+221261014673609+221261014673709+221261014674009+321261014667309+341261014130909</t>
+        </is>
+      </c>
+      <c r="B41" s="23" t="inlineStr">
+        <is>
+          <t>SIMPLEXINF</t>
+        </is>
+      </c>
+      <c r="C41" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D41" s="24" t="inlineStr"/>
+      <c r="E41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L41" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N41" s="21">
+        <f>SUM(E41:M41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-231261014125609+321261014663509+321261014663909+321261014664209+221261014672509+231261014126209+341261014130109+321261014666209+321261014666609+321261014666709+321261014667009+341261014130809+231261014127009+341261014131009+221261014675609</t>
+        </is>
+      </c>
+      <c r="B42" s="23" t="inlineStr">
+        <is>
+          <t>SPORTKING</t>
+        </is>
+      </c>
+      <c r="C42" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D42" s="24" t="inlineStr"/>
+      <c r="E42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K42" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L42" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N42" s="21">
+        <f>SUM(E42:M42)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E36" s="32">
-        <f>SUM(E4:E35)</f>
-        <v/>
-      </c>
-      <c r="F36" s="32">
-        <f>SUM(F4:F35)</f>
-        <v/>
-      </c>
-      <c r="G36" s="32">
-        <f>SUM(G4:G35)</f>
-        <v/>
-      </c>
-      <c r="H36" s="32">
-        <f>SUM(H4:H35)</f>
-        <v/>
-      </c>
-      <c r="I36" s="32">
-        <f>SUM(I4:I35)</f>
-        <v/>
-      </c>
-      <c r="J36" s="32">
-        <f>SUM(J4:J35)</f>
-        <v/>
-      </c>
-      <c r="K36" s="32">
-        <f>SUM(K4:K35)</f>
-        <v/>
-      </c>
-      <c r="L36" s="32">
-        <f>SUM(L4:L35)</f>
-        <v/>
-      </c>
-      <c r="M36" s="32">
-        <f>SUM(M4:M35)</f>
-        <v/>
-      </c>
-      <c r="N36" s="32">
-        <f>SUM(N4:N35)</f>
+      <c r="E43" s="32">
+        <f>SUM(E4:E42)</f>
+        <v/>
+      </c>
+      <c r="F43" s="32">
+        <f>SUM(F4:F42)</f>
+        <v/>
+      </c>
+      <c r="G43" s="32">
+        <f>SUM(G4:G42)</f>
+        <v/>
+      </c>
+      <c r="H43" s="32">
+        <f>SUM(H4:H42)</f>
+        <v/>
+      </c>
+      <c r="I43" s="32">
+        <f>SUM(I4:I42)</f>
+        <v/>
+      </c>
+      <c r="J43" s="32">
+        <f>SUM(J4:J42)</f>
+        <v/>
+      </c>
+      <c r="K43" s="32">
+        <f>SUM(K4:K42)</f>
+        <v/>
+      </c>
+      <c r="L43" s="32">
+        <f>SUM(L4:L42)</f>
+        <v/>
+      </c>
+      <c r="M43" s="32">
+        <f>SUM(M4:M42)</f>
+        <v/>
+      </c>
+      <c r="N43" s="32">
+        <f>SUM(N4:N42)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:N35"/>
+  <autoFilter ref="A3:N42"/>
   <mergeCells count="2">
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>

</xml_diff>

<commit_message>
Data update — 2026-10-15 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_oct2026.xlsx
+++ b/results/strategy_pnl_oct2026.xlsx
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trade Log'!$A$3:$O$503</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$46</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1994,7 +1994,7 @@
         <v/>
       </c>
       <c r="K19" s="4" t="n">
-        <v>707.6</v>
+        <v>707.7</v>
       </c>
       <c r="L19" s="21">
         <f>IF(OR($B19="",$I19=""),"",$I19-IF($K19="",0,$K19))</f>
@@ -2354,7 +2354,7 @@
         <v/>
       </c>
       <c r="K25" s="4" t="n">
-        <v>556.79</v>
+        <v>556.73</v>
       </c>
       <c r="L25" s="21">
         <f>IF(OR($B25="",$I25=""),"",$I25-IF($K25="",0,$K25))</f>
@@ -2534,7 +2534,7 @@
         <v/>
       </c>
       <c r="K28" s="4" t="n">
-        <v>356.25</v>
+        <v>554.42</v>
       </c>
       <c r="L28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($K28="",0,$K28))</f>
@@ -2594,7 +2594,7 @@
         <v/>
       </c>
       <c r="K29" s="4" t="n">
-        <v>349.1</v>
+        <v>550.21</v>
       </c>
       <c r="L29" s="21">
         <f>IF(OR($B29="",$I29=""),"",$I29-IF($K29="",0,$K29))</f>
@@ -2654,7 +2654,7 @@
         <v/>
       </c>
       <c r="K30" s="4" t="n">
-        <v>116.58</v>
+        <v>207</v>
       </c>
       <c r="L30" s="21">
         <f>IF(OR($B30="",$I30=""),"",$I30-IF($K30="",0,$K30))</f>
@@ -2714,7 +2714,7 @@
         <v/>
       </c>
       <c r="K31" s="4" t="n">
-        <v>347.17</v>
+        <v>550.35</v>
       </c>
       <c r="L31" s="21">
         <f>IF(OR($B31="",$I31=""),"",$I31-IF($K31="",0,$K31))</f>
@@ -2774,7 +2774,7 @@
         <v/>
       </c>
       <c r="K32" s="4" t="n">
-        <v>349.67</v>
+        <v>425.43</v>
       </c>
       <c r="L32" s="21">
         <f>IF(OR($B32="",$I32=""),"",$I32-IF($K32="",0,$K32))</f>
@@ -2834,7 +2834,7 @@
         <v/>
       </c>
       <c r="K33" s="4" t="n">
-        <v>0</v>
+        <v>223.78</v>
       </c>
       <c r="L33" s="21">
         <f>IF(OR($B33="",$I33=""),"",$I33-IF($K33="",0,$K33))</f>
@@ -2894,7 +2894,7 @@
         <v/>
       </c>
       <c r="K34" s="4" t="n">
-        <v>349.07</v>
+        <v>552.55</v>
       </c>
       <c r="L34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($K34="",0,$K34))</f>
@@ -2917,12 +2917,12 @@
     <row r="35">
       <c r="A35" s="23" t="inlineStr">
         <is>
-          <t>DHAN-34126101377609+221261013593609+34126101378109+23126101376709+34126101378409+23126101377009+221261013595709+221261013596109+221261013596609+23126101377809+34126101379309+34126101379709+23126101378409+34126101379809+221261013599309+321261013576809</t>
+          <t>DHAN-321261014662909+221261014671509+321261014664009+341261014129509+341261014129709+321261014665509+221261014673509+231261014126609+221261014673809+221261014674109+231261014126809+341261014131109+221261014675709+231261014127209+341261014131309+231261014127309</t>
         </is>
       </c>
       <c r="B35" s="23" t="inlineStr">
         <is>
-          <t>INDOKEM</t>
+          <t>JINDALPOLY</t>
         </is>
       </c>
       <c r="C35" s="23" t="inlineStr">
@@ -2931,16 +2931,20 @@
         </is>
       </c>
       <c r="D35" s="24" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="E35" s="25" t="n">
-        <v>677.9853000000001</v>
+        <v>726.3234</v>
       </c>
       <c r="F35" s="26" t="n">
-        <v>126</v>
-      </c>
-      <c r="G35" s="24" t="inlineStr"/>
-      <c r="H35" s="25" t="inlineStr"/>
+        <v>201</v>
+      </c>
+      <c r="G35" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H35" s="25" t="n">
+        <v>708.0599999999999</v>
+      </c>
       <c r="I35" s="21">
         <f>IF(OR($B35="",$H35=""),"",IF($C35="LONG",($H35-$E35)*$F35,($E35-$H35)*$F35))</f>
         <v/>
@@ -2950,7 +2954,7 @@
         <v/>
       </c>
       <c r="K35" s="4" t="n">
-        <v>116.19</v>
+        <v>306.62</v>
       </c>
       <c r="L35" s="21">
         <f>IF(OR($B35="",$I35=""),"",$I35-IF($K35="",0,$K35))</f>
@@ -2973,12 +2977,12 @@
     <row r="36">
       <c r="A36" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261014662909+221261014671509+321261014664009+341261014129509+341261014129709+321261014665509+221261014673509+231261014126609+221261014673809+221261014674109+231261014126809+341261014131109+221261014675709+231261014127209+341261014131309+231261014127309</t>
+          <t>DHAN-321261014663009+221261014671609+341261014129309+221261014671909+341261014129609+341261014129809+231261014126309+321261014666109+231261014126509+341261014130409+231261014126709+231261014126909</t>
         </is>
       </c>
       <c r="B36" s="23" t="inlineStr">
         <is>
-          <t>JINDALPOLY</t>
+          <t>KROSS</t>
         </is>
       </c>
       <c r="C36" s="23" t="inlineStr">
@@ -2990,13 +2994,17 @@
         <v>46309</v>
       </c>
       <c r="E36" s="25" t="n">
-        <v>726.3234</v>
+        <v>271.509</v>
       </c>
       <c r="F36" s="26" t="n">
-        <v>201</v>
-      </c>
-      <c r="G36" s="24" t="inlineStr"/>
-      <c r="H36" s="25" t="inlineStr"/>
+        <v>737</v>
+      </c>
+      <c r="G36" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H36" s="25" t="n">
+        <v>270.99</v>
+      </c>
       <c r="I36" s="21">
         <f>IF(OR($B36="",$H36=""),"",IF($C36="LONG",($H36-$E36)*$F36,($E36-$H36)*$F36))</f>
         <v/>
@@ -3006,7 +3014,7 @@
         <v/>
       </c>
       <c r="K36" s="4" t="n">
-        <v>50.15</v>
+        <v>392.78</v>
       </c>
       <c r="L36" s="21">
         <f>IF(OR($B36="",$I36=""),"",$I36-IF($K36="",0,$K36))</f>
@@ -3029,12 +3037,12 @@
     <row r="37">
       <c r="A37" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261014663009+221261014671609+341261014129309+221261014671909+341261014129609+341261014129809+231261014126309+321261014666109+231261014126509+341261014130409+231261014126709+231261014126909</t>
+          <t>DHAN-341261014128909+341261014129109+231261014125709+321261014664109+321261014664809+231261014126009+321261014665609+231261014126409+341261014130309+341261014130509+221261014673909+341261014130709+221261014674609+221261014675009+221261014675509</t>
         </is>
       </c>
       <c r="B37" s="23" t="inlineStr">
         <is>
-          <t>KROSS</t>
+          <t>NIBE</t>
         </is>
       </c>
       <c r="C37" s="23" t="inlineStr">
@@ -3046,13 +3054,17 @@
         <v>46309</v>
       </c>
       <c r="E37" s="25" t="n">
-        <v>271.509</v>
+        <v>1380.7368</v>
       </c>
       <c r="F37" s="26" t="n">
-        <v>737</v>
-      </c>
-      <c r="G37" s="24" t="inlineStr"/>
-      <c r="H37" s="25" t="inlineStr"/>
+        <v>144</v>
+      </c>
+      <c r="G37" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H37" s="25" t="n">
+        <v>1334.24</v>
+      </c>
       <c r="I37" s="21">
         <f>IF(OR($B37="",$H37=""),"",IF($C37="LONG",($H37-$E37)*$F37,($E37-$H37)*$F37))</f>
         <v/>
@@ -3062,7 +3074,7 @@
         <v/>
       </c>
       <c r="K37" s="4" t="n">
-        <v>50.15</v>
+        <v>390.61</v>
       </c>
       <c r="L37" s="21">
         <f>IF(OR($B37="",$I37=""),"",$I37-IF($K37="",0,$K37))</f>
@@ -3085,12 +3097,12 @@
     <row r="38">
       <c r="A38" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261012625809+321261012626209+23126101284209+23126101284309+321261012626909+34126101276209+34126101277109+321261012628809+221261012640809+23126101286309+34126101278009+321261012630809+221261012643209</t>
+          <t>DHAN-221261014671209+321261014663609+231261014125809+221261014672009+231261014125909+231261014126109+221261014673109+341261014130209+321261014666509+341261014130609+321261014667409+321261014667809+341261014131209+221261014676209+221261014676809</t>
         </is>
       </c>
       <c r="B38" s="23" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>RUBYMILLS</t>
         </is>
       </c>
       <c r="C38" s="23" t="inlineStr">
@@ -3099,16 +3111,20 @@
         </is>
       </c>
       <c r="D38" s="24" t="n">
-        <v>46307</v>
+        <v>46309</v>
       </c>
       <c r="E38" s="25" t="n">
-        <v>22.8999</v>
+        <v>541.4497</v>
       </c>
       <c r="F38" s="26" t="n">
-        <v>3742</v>
-      </c>
-      <c r="G38" s="24" t="inlineStr"/>
-      <c r="H38" s="25" t="inlineStr"/>
+        <v>184</v>
+      </c>
+      <c r="G38" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H38" s="25" t="n">
+        <v>554.2</v>
+      </c>
       <c r="I38" s="21">
         <f>IF(OR($B38="",$H38=""),"",IF($C38="LONG",($H38-$E38)*$F38,($E38-$H38)*$F38))</f>
         <v/>
@@ -3118,7 +3134,7 @@
         <v/>
       </c>
       <c r="K38" s="4" t="n">
-        <v>53.57</v>
+        <v>133.05</v>
       </c>
       <c r="L38" s="21">
         <f>IF(OR($B38="",$I38=""),"",$I38-IF($K38="",0,$K38))</f>
@@ -3141,12 +3157,12 @@
     <row r="39">
       <c r="A39" s="23" t="inlineStr">
         <is>
-          <t>DHAN-341261014128909+341261014129109+231261014125709+321261014664109+321261014664809+231261014126009+321261014665609+231261014126409+341261014130309+341261014130509+221261014673909+341261014130709+221261014674609+221261014675009+221261014675509</t>
+          <t>DHAN-231261014125609+321261014663509+321261014663909+321261014664209+221261014672509+231261014126209+341261014130109+321261014666209+321261014666609+321261014666709+321261014667009+341261014130809+231261014127009+341261014131009+221261014675609</t>
         </is>
       </c>
       <c r="B39" s="23" t="inlineStr">
         <is>
-          <t>NIBE</t>
+          <t>SPORTKING</t>
         </is>
       </c>
       <c r="C39" s="23" t="inlineStr">
@@ -3158,13 +3174,17 @@
         <v>46309</v>
       </c>
       <c r="E39" s="25" t="n">
-        <v>1380.7368</v>
+        <v>226.1107</v>
       </c>
       <c r="F39" s="26" t="n">
-        <v>144</v>
-      </c>
-      <c r="G39" s="24" t="inlineStr"/>
-      <c r="H39" s="25" t="inlineStr"/>
+        <v>885</v>
+      </c>
+      <c r="G39" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H39" s="25" t="n">
+        <v>226.89</v>
+      </c>
       <c r="I39" s="21">
         <f>IF(OR($B39="",$H39=""),"",IF($C39="LONG",($H39-$E39)*$F39,($E39-$H39)*$F39))</f>
         <v/>
@@ -3174,7 +3194,7 @@
         <v/>
       </c>
       <c r="K39" s="4" t="n">
-        <v>50.15</v>
+        <v>392.91</v>
       </c>
       <c r="L39" s="21">
         <f>IF(OR($B39="",$I39=""),"",$I39-IF($K39="",0,$K39))</f>
@@ -3190,19 +3210,19 @@
       </c>
       <c r="O39" s="23" t="inlineStr">
         <is>
-          <t>10-15</t>
+          <t>5-10</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261014671209+321261014663609+231261014125809+221261014672009+231261014125909+231261014126109+221261014673109+341261014130209+321261014666509+341261014130609+321261014667409+321261014667809+341261014131209+221261014676209+221261014676809</t>
+          <t>DHAN-34126101377609+221261013593609+34126101378109+23126101376709+34126101378409+23126101377009+221261013595709+221261013596109+221261013596609+23126101377809+34126101379309+34126101379709+23126101378409+34126101379809+221261013599309+321261013576809</t>
         </is>
       </c>
       <c r="B40" s="23" t="inlineStr">
         <is>
-          <t>RUBYMILLS</t>
+          <t>INDOKEM</t>
         </is>
       </c>
       <c r="C40" s="23" t="inlineStr">
@@ -3211,13 +3231,13 @@
         </is>
       </c>
       <c r="D40" s="24" t="n">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="E40" s="25" t="n">
-        <v>541.4497</v>
+        <v>677.9853000000001</v>
       </c>
       <c r="F40" s="26" t="n">
-        <v>184</v>
+        <v>126</v>
       </c>
       <c r="G40" s="24" t="inlineStr"/>
       <c r="H40" s="25" t="inlineStr"/>
@@ -3230,7 +3250,7 @@
         <v/>
       </c>
       <c r="K40" s="4" t="n">
-        <v>14.75</v>
+        <v>116.19</v>
       </c>
       <c r="L40" s="21">
         <f>IF(OR($B40="",$I40=""),"",$I40-IF($K40="",0,$K40))</f>
@@ -3246,19 +3266,19 @@
       </c>
       <c r="O40" s="23" t="inlineStr">
         <is>
-          <t>5-10</t>
+          <t>10-15</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="23" t="inlineStr">
         <is>
-          <t>DHAN-341261014128809+341261014129209+221261014671809+321261014664309+221261014672409+321261014664909+341261014130009+221261014673409+221261014673609+221261014673709+221261014674009+321261014667309+341261014130909</t>
+          <t>DHAN-321261015672409+231261015159509+341261015154309+321261015674209+231261015159809+321261015674909+341261015154809+221261015678909+321261015675709+221261015679609+231261015160509</t>
         </is>
       </c>
       <c r="B41" s="23" t="inlineStr">
         <is>
-          <t>SIMPLEXINF</t>
+          <t>JAICORPLTD</t>
         </is>
       </c>
       <c r="C41" s="23" t="inlineStr">
@@ -3267,13 +3287,13 @@
         </is>
       </c>
       <c r="D41" s="24" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="E41" s="25" t="n">
-        <v>266.801</v>
+        <v>95.05800000000001</v>
       </c>
       <c r="F41" s="26" t="n">
-        <v>749</v>
+        <v>3153</v>
       </c>
       <c r="G41" s="24" t="inlineStr"/>
       <c r="H41" s="25" t="inlineStr"/>
@@ -3309,12 +3329,12 @@
     <row r="42">
       <c r="A42" s="23" t="inlineStr">
         <is>
-          <t>DHAN-231261014125609+321261014663509+321261014663909+321261014664209+221261014672509+231261014126209+341261014130109+321261014666209+321261014666609+321261014666709+321261014667009+341261014130809+231261014127009+341261014131009+221261014675609</t>
+          <t>DHAN-321261012625809+321261012626209+23126101284209+23126101284309+321261012626909+34126101276209+34126101277109+321261012628809+221261012640809+23126101286309+34126101278009+321261012630809+221261012643209</t>
         </is>
       </c>
       <c r="B42" s="23" t="inlineStr">
         <is>
-          <t>SPORTKING</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="C42" s="23" t="inlineStr">
@@ -3323,13 +3343,13 @@
         </is>
       </c>
       <c r="D42" s="24" t="n">
-        <v>46309</v>
+        <v>46307</v>
       </c>
       <c r="E42" s="25" t="n">
-        <v>226.1107</v>
+        <v>22.8999</v>
       </c>
       <c r="F42" s="26" t="n">
-        <v>885</v>
+        <v>3742</v>
       </c>
       <c r="G42" s="24" t="inlineStr"/>
       <c r="H42" s="25" t="inlineStr"/>
@@ -3342,7 +3362,7 @@
         <v/>
       </c>
       <c r="K42" s="4" t="n">
-        <v>50.15</v>
+        <v>53.57</v>
       </c>
       <c r="L42" s="21">
         <f>IF(OR($B42="",$I42=""),"",$I42-IF($K42="",0,$K42))</f>
@@ -3363,14 +3383,32 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="23" t="n"/>
-      <c r="B43" s="23" t="n"/>
-      <c r="C43" s="23" t="n"/>
-      <c r="D43" s="24" t="n"/>
-      <c r="E43" s="25" t="n"/>
-      <c r="F43" s="26" t="n"/>
-      <c r="G43" s="24" t="n"/>
-      <c r="H43" s="25" t="n"/>
+      <c r="A43" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-341261015154009+321261015672609+221261015677509+321261015674109+321261015674709+341261015154709+231261015160109+341261015154909+221261015679409+341261015155209+321261015676109</t>
+        </is>
+      </c>
+      <c r="B43" s="23" t="inlineStr">
+        <is>
+          <t>OAL</t>
+        </is>
+      </c>
+      <c r="C43" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D43" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="E43" s="25" t="n">
+        <v>578.2952</v>
+      </c>
+      <c r="F43" s="26" t="n">
+        <v>258</v>
+      </c>
+      <c r="G43" s="24" t="inlineStr"/>
+      <c r="H43" s="25" t="inlineStr"/>
       <c r="I43" s="21">
         <f>IF(OR($B43="",$H43=""),"",IF($C43="LONG",($H43-$E43)*$F43,($E43-$H43)*$F43))</f>
         <v/>
@@ -3379,7 +3417,9 @@
         <f>IF(OR($B43="",$I43="",$E43=0,$F43=0),"",$I43/($E43*$F43))</f>
         <v/>
       </c>
-      <c r="K43" s="4" t="n"/>
+      <c r="K43" s="4" t="n">
+        <v>14.75</v>
+      </c>
       <c r="L43" s="21">
         <f>IF(OR($B43="",$I43=""),"",$I43-IF($K43="",0,$K43))</f>
         <v/>
@@ -3392,17 +3432,39 @@
         <f>IF($B43="","",IF($H43="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O43" s="23" t="n"/>
+      <c r="O43" s="23" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" s="23" t="n"/>
-      <c r="B44" s="23" t="n"/>
-      <c r="C44" s="23" t="n"/>
-      <c r="D44" s="24" t="n"/>
-      <c r="E44" s="25" t="n"/>
-      <c r="F44" s="26" t="n"/>
-      <c r="G44" s="24" t="n"/>
-      <c r="H44" s="25" t="n"/>
+      <c r="A44" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-341261015153909+221261015677009+321261015673209+231261015159709+231261015159909+231261015160009+221261015678509+321261015675509+231261015160209+231261015160409+341261015155309</t>
+        </is>
+      </c>
+      <c r="B44" s="23" t="inlineStr">
+        <is>
+          <t>ORIENTELEC</t>
+        </is>
+      </c>
+      <c r="C44" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D44" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="E44" s="25" t="n">
+        <v>201.1512</v>
+      </c>
+      <c r="F44" s="26" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G44" s="24" t="inlineStr"/>
+      <c r="H44" s="25" t="inlineStr"/>
       <c r="I44" s="21">
         <f>IF(OR($B44="",$H44=""),"",IF($C44="LONG",($H44-$E44)*$F44,($E44-$H44)*$F44))</f>
         <v/>
@@ -3411,7 +3473,9 @@
         <f>IF(OR($B44="",$I44="",$E44=0,$F44=0),"",$I44/($E44*$F44))</f>
         <v/>
       </c>
-      <c r="K44" s="4" t="n"/>
+      <c r="K44" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L44" s="21">
         <f>IF(OR($B44="",$I44=""),"",$I44-IF($K44="",0,$K44))</f>
         <v/>
@@ -3424,17 +3488,39 @@
         <f>IF($B44="","",IF($H44="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O44" s="23" t="n"/>
+      <c r="O44" s="23" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="23" t="n"/>
-      <c r="B45" s="23" t="n"/>
-      <c r="C45" s="23" t="n"/>
-      <c r="D45" s="24" t="n"/>
-      <c r="E45" s="25" t="n"/>
-      <c r="F45" s="26" t="n"/>
-      <c r="G45" s="24" t="n"/>
-      <c r="H45" s="25" t="n"/>
+      <c r="A45" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-341261014128809+341261014129209+221261014671809+321261014664309+221261014672409+321261014664909+341261014130009+221261014673409+221261014673609+221261014673709+221261014674009+321261014667309+341261014130909</t>
+        </is>
+      </c>
+      <c r="B45" s="23" t="inlineStr">
+        <is>
+          <t>SIMPLEXINF</t>
+        </is>
+      </c>
+      <c r="C45" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D45" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E45" s="25" t="n">
+        <v>266.801</v>
+      </c>
+      <c r="F45" s="26" t="n">
+        <v>749</v>
+      </c>
+      <c r="G45" s="24" t="inlineStr"/>
+      <c r="H45" s="25" t="inlineStr"/>
       <c r="I45" s="21">
         <f>IF(OR($B45="",$H45=""),"",IF($C45="LONG",($H45-$E45)*$F45,($E45-$H45)*$F45))</f>
         <v/>
@@ -3443,7 +3529,9 @@
         <f>IF(OR($B45="",$I45="",$E45=0,$F45=0),"",$I45/($E45*$F45))</f>
         <v/>
       </c>
-      <c r="K45" s="4" t="n"/>
+      <c r="K45" s="4" t="n">
+        <v>392.35</v>
+      </c>
       <c r="L45" s="21">
         <f>IF(OR($B45="",$I45=""),"",$I45-IF($K45="",0,$K45))</f>
         <v/>
@@ -3456,17 +3544,39 @@
         <f>IF($B45="","",IF($H45="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O45" s="23" t="n"/>
+      <c r="O45" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="23" t="n"/>
-      <c r="B46" s="23" t="n"/>
-      <c r="C46" s="23" t="n"/>
-      <c r="D46" s="24" t="n"/>
-      <c r="E46" s="25" t="n"/>
-      <c r="F46" s="26" t="n"/>
-      <c r="G46" s="24" t="n"/>
-      <c r="H46" s="25" t="n"/>
+      <c r="A46" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-231261015159409+321261015672709+321261015673309+221261015677909+221261015678309+341261015154609+321261015675209+221261015678809+341261015155009+341261015155109+231261015160609+231261015160709+341261015155509</t>
+        </is>
+      </c>
+      <c r="B46" s="23" t="inlineStr">
+        <is>
+          <t>TEAMLEASE</t>
+        </is>
+      </c>
+      <c r="C46" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D46" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="E46" s="25" t="n">
+        <v>1133.7498</v>
+      </c>
+      <c r="F46" s="26" t="n">
+        <v>263</v>
+      </c>
+      <c r="G46" s="24" t="inlineStr"/>
+      <c r="H46" s="25" t="inlineStr"/>
       <c r="I46" s="21">
         <f>IF(OR($B46="",$H46=""),"",IF($C46="LONG",($H46-$E46)*$F46,($E46-$H46)*$F46))</f>
         <v/>
@@ -3475,7 +3585,9 @@
         <f>IF(OR($B46="",$I46="",$E46=0,$F46=0),"",$I46/($E46*$F46))</f>
         <v/>
       </c>
-      <c r="K46" s="4" t="n"/>
+      <c r="K46" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L46" s="21">
         <f>IF(OR($B46="",$I46=""),"",$I46-IF($K46="",0,$K46))</f>
         <v/>
@@ -3488,7 +3600,11 @@
         <f>IF($B46="","",IF($H46="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O46" s="23" t="n"/>
+      <c r="O46" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="23" t="n"/>
@@ -30789,7 +30905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:J42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31346,7 +31462,7 @@
     <row r="15">
       <c r="A15" s="27" t="inlineStr">
         <is>
-          <t>JINDALPOLY</t>
+          <t>JAICORPLTD</t>
         </is>
       </c>
       <c r="B15" s="20">
@@ -31389,7 +31505,7 @@
     <row r="16">
       <c r="A16" s="27" t="inlineStr">
         <is>
-          <t>KOTIC</t>
+          <t>JINDALPOLY</t>
         </is>
       </c>
       <c r="B16" s="20">
@@ -31432,7 +31548,7 @@
     <row r="17">
       <c r="A17" s="27" t="inlineStr">
         <is>
-          <t>KRISHNADEF</t>
+          <t>KOTIC</t>
         </is>
       </c>
       <c r="B17" s="20">
@@ -31475,7 +31591,7 @@
     <row r="18">
       <c r="A18" s="27" t="inlineStr">
         <is>
-          <t>KROSS</t>
+          <t>KRISHNADEF</t>
         </is>
       </c>
       <c r="B18" s="20">
@@ -31518,7 +31634,7 @@
     <row r="19">
       <c r="A19" s="27" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>KROSS</t>
         </is>
       </c>
       <c r="B19" s="20">
@@ -31561,7 +31677,7 @@
     <row r="20">
       <c r="A20" s="27" t="inlineStr">
         <is>
-          <t>MOBIKWIK</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="B20" s="20">
@@ -31604,7 +31720,7 @@
     <row r="21">
       <c r="A21" s="27" t="inlineStr">
         <is>
-          <t>NIBE</t>
+          <t>MOBIKWIK</t>
         </is>
       </c>
       <c r="B21" s="20">
@@ -31647,7 +31763,7 @@
     <row r="22">
       <c r="A22" s="27" t="inlineStr">
         <is>
-          <t>PIXTRANS</t>
+          <t>NIBE</t>
         </is>
       </c>
       <c r="B22" s="20">
@@ -31690,7 +31806,7 @@
     <row r="23">
       <c r="A23" s="27" t="inlineStr">
         <is>
-          <t>PNCINFRA</t>
+          <t>OAL</t>
         </is>
       </c>
       <c r="B23" s="20">
@@ -31733,7 +31849,7 @@
     <row r="24">
       <c r="A24" s="27" t="inlineStr">
         <is>
-          <t>PNGSREVA</t>
+          <t>ORIENTELEC</t>
         </is>
       </c>
       <c r="B24" s="20">
@@ -31776,7 +31892,7 @@
     <row r="25">
       <c r="A25" s="27" t="inlineStr">
         <is>
-          <t>PRINCEPIPE</t>
+          <t>PIXTRANS</t>
         </is>
       </c>
       <c r="B25" s="20">
@@ -31819,7 +31935,7 @@
     <row r="26">
       <c r="A26" s="27" t="inlineStr">
         <is>
-          <t>RSYSTEMS</t>
+          <t>PNCINFRA</t>
         </is>
       </c>
       <c r="B26" s="20">
@@ -31862,7 +31978,7 @@
     <row r="27">
       <c r="A27" s="27" t="inlineStr">
         <is>
-          <t>RUBYMILLS</t>
+          <t>PNGSREVA</t>
         </is>
       </c>
       <c r="B27" s="20">
@@ -31905,7 +32021,7 @@
     <row r="28">
       <c r="A28" s="27" t="inlineStr">
         <is>
-          <t>SAKSOFT</t>
+          <t>PRINCEPIPE</t>
         </is>
       </c>
       <c r="B28" s="20">
@@ -31948,7 +32064,7 @@
     <row r="29">
       <c r="A29" s="27" t="inlineStr">
         <is>
-          <t>SATIN</t>
+          <t>RSYSTEMS</t>
         </is>
       </c>
       <c r="B29" s="20">
@@ -31991,7 +32107,7 @@
     <row r="30">
       <c r="A30" s="27" t="inlineStr">
         <is>
-          <t>SGFIN</t>
+          <t>RUBYMILLS</t>
         </is>
       </c>
       <c r="B30" s="20">
@@ -32034,7 +32150,7 @@
     <row r="31">
       <c r="A31" s="27" t="inlineStr">
         <is>
-          <t>SHRINGARMS</t>
+          <t>SAKSOFT</t>
         </is>
       </c>
       <c r="B31" s="20">
@@ -32077,7 +32193,7 @@
     <row r="32">
       <c r="A32" s="27" t="inlineStr">
         <is>
-          <t>SIMPLEXINF</t>
+          <t>SATIN</t>
         </is>
       </c>
       <c r="B32" s="20">
@@ -32120,7 +32236,7 @@
     <row r="33">
       <c r="A33" s="27" t="inlineStr">
         <is>
-          <t>SMCGLOBAL</t>
+          <t>SGFIN</t>
         </is>
       </c>
       <c r="B33" s="20">
@@ -32163,7 +32279,7 @@
     <row r="34">
       <c r="A34" s="27" t="inlineStr">
         <is>
-          <t>SPORTKING</t>
+          <t>SHRINGARMS</t>
         </is>
       </c>
       <c r="B34" s="20">
@@ -32206,7 +32322,7 @@
     <row r="35">
       <c r="A35" s="27" t="inlineStr">
         <is>
-          <t>SUNCLAY</t>
+          <t>SIMPLEXINF</t>
         </is>
       </c>
       <c r="B35" s="20">
@@ -32249,7 +32365,7 @@
     <row r="36">
       <c r="A36" s="27" t="inlineStr">
         <is>
-          <t>SWARAJENG</t>
+          <t>SMCGLOBAL</t>
         </is>
       </c>
       <c r="B36" s="20">
@@ -32292,7 +32408,7 @@
     <row r="37">
       <c r="A37" s="27" t="inlineStr">
         <is>
-          <t>YUKEN</t>
+          <t>SPORTKING</t>
         </is>
       </c>
       <c r="B37" s="20">
@@ -32333,37 +32449,209 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="3" t="inlineStr">
+      <c r="A38" s="27" t="inlineStr">
+        <is>
+          <t>SUNCLAY</t>
+        </is>
+      </c>
+      <c r="B38" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A38)</f>
+        <v/>
+      </c>
+      <c r="C38" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A38,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D38" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A38,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E38" s="22">
+        <f>IFERROR($C38/$B38,"")</f>
+        <v/>
+      </c>
+      <c r="F38" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A38,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G38" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A38,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H38" s="21">
+        <f>IFERROR($G38/$B38,"")</f>
+        <v/>
+      </c>
+      <c r="I38" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A38),"")</f>
+        <v/>
+      </c>
+      <c r="J38" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A38),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="27" t="inlineStr">
+        <is>
+          <t>SWARAJENG</t>
+        </is>
+      </c>
+      <c r="B39" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A39)</f>
+        <v/>
+      </c>
+      <c r="C39" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A39,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D39" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A39,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E39" s="22">
+        <f>IFERROR($C39/$B39,"")</f>
+        <v/>
+      </c>
+      <c r="F39" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A39,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G39" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A39,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H39" s="21">
+        <f>IFERROR($G39/$B39,"")</f>
+        <v/>
+      </c>
+      <c r="I39" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A39),"")</f>
+        <v/>
+      </c>
+      <c r="J39" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A39),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="27" t="inlineStr">
+        <is>
+          <t>TEAMLEASE</t>
+        </is>
+      </c>
+      <c r="B40" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A40)</f>
+        <v/>
+      </c>
+      <c r="C40" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A40,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D40" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A40,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E40" s="22">
+        <f>IFERROR($C40/$B40,"")</f>
+        <v/>
+      </c>
+      <c r="F40" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A40,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G40" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A40,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H40" s="21">
+        <f>IFERROR($G40/$B40,"")</f>
+        <v/>
+      </c>
+      <c r="I40" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A40),"")</f>
+        <v/>
+      </c>
+      <c r="J40" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A40),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="27" t="inlineStr">
+        <is>
+          <t>YUKEN</t>
+        </is>
+      </c>
+      <c r="B41" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A41)</f>
+        <v/>
+      </c>
+      <c r="C41" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A41,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D41" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A41,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E41" s="22">
+        <f>IFERROR($C41/$B41,"")</f>
+        <v/>
+      </c>
+      <c r="F41" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A41,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G41" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A41,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H41" s="21">
+        <f>IFERROR($G41/$B41,"")</f>
+        <v/>
+      </c>
+      <c r="I41" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A41),"")</f>
+        <v/>
+      </c>
+      <c r="J41" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A41),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B38" s="30">
-        <f>SUM(B4:B37)</f>
-        <v/>
-      </c>
-      <c r="C38" s="30">
-        <f>SUM(C4:C37)</f>
-        <v/>
-      </c>
-      <c r="D38" s="30">
-        <f>SUM(D4:D37)</f>
-        <v/>
-      </c>
-      <c r="E38" s="31">
-        <f>IFERROR(C38/B38,"")</f>
-        <v/>
-      </c>
-      <c r="F38" s="32">
-        <f>SUM(F4:F37)</f>
-        <v/>
-      </c>
-      <c r="G38" s="32">
-        <f>SUM(G4:G37)</f>
-        <v/>
-      </c>
-      <c r="H38" s="32">
-        <f>IFERROR(G38/B38,"")</f>
+      <c r="B42" s="30">
+        <f>SUM(B4:B41)</f>
+        <v/>
+      </c>
+      <c r="C42" s="30">
+        <f>SUM(C4:C41)</f>
+        <v/>
+      </c>
+      <c r="D42" s="30">
+        <f>SUM(D4:D41)</f>
+        <v/>
+      </c>
+      <c r="E42" s="31">
+        <f>IFERROR(C42/B42,"")</f>
+        <v/>
+      </c>
+      <c r="F42" s="32">
+        <f>SUM(F4:F41)</f>
+        <v/>
+      </c>
+      <c r="G42" s="32">
+        <f>SUM(G4:G41)</f>
+        <v/>
+      </c>
+      <c r="H42" s="32">
+        <f>IFERROR(G42/B42,"")</f>
         <v/>
       </c>
     </row>
@@ -32382,7 +32670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N43"/>
+  <dimension ref="A1:N47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -33296,7 +33584,7 @@
         <v>35.4</v>
       </c>
       <c r="M19" s="4" t="n">
-        <v>127.42</v>
+        <v>127.52</v>
       </c>
       <c r="N19" s="21">
         <f>SUM(E19:M19)</f>
@@ -33602,7 +33890,7 @@
         <v>35.4</v>
       </c>
       <c r="M25" s="4" t="n">
-        <v>36.59</v>
+        <v>36.53</v>
       </c>
       <c r="N25" s="21">
         <f>SUM(E25:M25)</f>
@@ -33731,22 +34019,22 @@
         <v>46309</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>51.3</v>
+        <v>71.3</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>170.95</v>
+        <v>339.38</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>5.25</v>
+        <v>10.42</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>0.17</v>
+        <v>0.34</v>
       </c>
       <c r="I28" s="4" t="n">
         <v>25.64</v>
       </c>
       <c r="J28" s="4" t="n">
-        <v>10.21</v>
+        <v>14.77</v>
       </c>
       <c r="K28" s="4" t="n">
         <v>14.75</v>
@@ -33755,7 +34043,7 @@
         <v>35.4</v>
       </c>
       <c r="M28" s="4" t="n">
-        <v>42.58</v>
+        <v>42.42</v>
       </c>
       <c r="N28" s="21">
         <f>SUM(E28:M28)</f>
@@ -33782,22 +34070,22 @@
         <v>46309</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>51</v>
+        <v>71</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>171.42</v>
+        <v>342.53</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>5.26</v>
+        <v>10.51</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>0.17</v>
+        <v>0.34</v>
       </c>
       <c r="I29" s="4" t="n">
         <v>25.77</v>
       </c>
       <c r="J29" s="4" t="n">
-        <v>10.16</v>
+        <v>14.73</v>
       </c>
       <c r="K29" s="4" t="n">
         <v>14.75</v>
@@ -33836,19 +34124,19 @@
         <v>0</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>85.76000000000001</v>
+        <v>172.92</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>2.63</v>
+        <v>5.31</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>0.09</v>
+        <v>0.17</v>
       </c>
       <c r="I30" s="4" t="n">
         <v>12.86</v>
       </c>
       <c r="J30" s="4" t="n">
-        <v>0.49</v>
+        <v>0.99</v>
       </c>
       <c r="K30" s="4" t="n">
         <v>14.75</v>
@@ -33884,22 +34172,22 @@
         <v>46309</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>51.01</v>
+        <v>71.01000000000001</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>170.06</v>
+        <v>343.17</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>5.22</v>
+        <v>10.53</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>0.17</v>
+        <v>0.34</v>
       </c>
       <c r="I31" s="4" t="n">
         <v>25.51</v>
       </c>
       <c r="J31" s="4" t="n">
-        <v>10.15</v>
+        <v>14.74</v>
       </c>
       <c r="K31" s="4" t="n">
         <v>14.75</v>
@@ -33935,22 +34223,22 @@
         <v>46309</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>51.07</v>
+        <v>71.06999999999999</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>170.2</v>
+        <v>215.5</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>5.22</v>
+        <v>10.89</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>0.17</v>
+        <v>0.35</v>
       </c>
       <c r="I32" s="4" t="n">
         <v>25.53</v>
       </c>
       <c r="J32" s="4" t="n">
-        <v>10.16</v>
+        <v>14.82</v>
       </c>
       <c r="K32" s="4" t="n">
         <v>14.75</v>
@@ -33959,7 +34247,7 @@
         <v>35.4</v>
       </c>
       <c r="M32" s="4" t="n">
-        <v>37.16</v>
+        <v>37.12</v>
       </c>
       <c r="N32" s="21">
         <f>SUM(E32:M32)</f>
@@ -33986,22 +34274,22 @@
         <v>46309</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>0</v>
+        <v>181.5</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>0</v>
+        <v>11.03</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>0</v>
+        <v>0.36</v>
       </c>
       <c r="I33" s="4" t="n">
-        <v>0</v>
+        <v>5.25</v>
       </c>
       <c r="J33" s="4" t="n">
-        <v>0</v>
+        <v>5.65</v>
       </c>
       <c r="K33" s="4" t="n">
         <v>0</v>
@@ -34037,22 +34325,22 @@
         <v>46309</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>51.33</v>
+        <v>71.33</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>171.16</v>
+        <v>344.55</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>5.25</v>
+        <v>10.58</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>0.17</v>
+        <v>0.34</v>
       </c>
       <c r="I34" s="4" t="n">
         <v>25.67</v>
       </c>
       <c r="J34" s="4" t="n">
-        <v>10.22</v>
+        <v>14.81</v>
       </c>
       <c r="K34" s="4" t="n">
         <v>14.75</v>
@@ -34071,12 +34359,12 @@
     <row r="35">
       <c r="A35" s="23" t="inlineStr">
         <is>
-          <t>DHAN-34126101377609+221261013593609+34126101378109+23126101376709+34126101378409+23126101377009+221261013595709+221261013596109+221261013596609+23126101377809+34126101379309+34126101379709+23126101378409+34126101379809+221261013599309+321261013576809</t>
+          <t>DHAN-321261014662909+221261014671509+321261014664009+341261014129509+341261014129709+321261014665509+221261014673509+231261014126609+221261014673809+221261014674109+231261014126809+341261014131109+221261014675709+231261014127209+341261014131309+231261014127309</t>
         </is>
       </c>
       <c r="B35" s="23" t="inlineStr">
         <is>
-          <t>INDOKEM</t>
+          <t>JINDALPOLY</t>
         </is>
       </c>
       <c r="C35" s="23" t="inlineStr">
@@ -34084,33 +34372,35 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D35" s="24" t="inlineStr"/>
+      <c r="D35" s="24" t="n">
+        <v>46310</v>
+      </c>
       <c r="E35" s="4" t="n">
-        <v>0</v>
+        <v>43.82</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>85.43000000000001</v>
+        <v>145.99</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>2.62</v>
+        <v>4.48</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>0.09</v>
+        <v>0.15</v>
       </c>
       <c r="I35" s="4" t="n">
-        <v>12.81</v>
+        <v>21.9</v>
       </c>
       <c r="J35" s="4" t="n">
-        <v>0.49</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="K35" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L35" s="4" t="n">
-        <v>0</v>
+        <v>35.4</v>
       </c>
       <c r="M35" s="4" t="n">
-        <v>0</v>
+        <v>31.42</v>
       </c>
       <c r="N35" s="21">
         <f>SUM(E35:M35)</f>
@@ -34120,12 +34410,12 @@
     <row r="36">
       <c r="A36" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261014662909+221261014671509+321261014664009+341261014129509+341261014129709+321261014665509+221261014673509+231261014126609+221261014673809+221261014674109+231261014126809+341261014131109+221261014675709+231261014127209+341261014131309+231261014127309</t>
+          <t>DHAN-321261014663009+221261014671609+341261014129309+221261014671909+341261014129609+341261014129809+231261014126309+321261014666109+231261014126509+341261014130409+231261014126709+231261014126909</t>
         </is>
       </c>
       <c r="B36" s="23" t="inlineStr">
         <is>
-          <t>JINDALPOLY</t>
+          <t>KROSS</t>
         </is>
       </c>
       <c r="C36" s="23" t="inlineStr">
@@ -34133,24 +34423,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D36" s="24" t="inlineStr"/>
+      <c r="D36" s="24" t="n">
+        <v>46310</v>
+      </c>
       <c r="E36" s="4" t="n">
-        <v>0</v>
+        <v>60.01</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>0</v>
+        <v>200.1</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>0</v>
+        <v>6.14</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="I36" s="4" t="n">
-        <v>0</v>
+        <v>30.02</v>
       </c>
       <c r="J36" s="4" t="n">
-        <v>0</v>
+        <v>11.94</v>
       </c>
       <c r="K36" s="4" t="n">
         <v>14.75</v>
@@ -34159,7 +34451,7 @@
         <v>35.4</v>
       </c>
       <c r="M36" s="4" t="n">
-        <v>0</v>
+        <v>34.22</v>
       </c>
       <c r="N36" s="21">
         <f>SUM(E36:M36)</f>
@@ -34169,12 +34461,12 @@
     <row r="37">
       <c r="A37" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261014663009+221261014671609+341261014129309+221261014671909+341261014129609+341261014129809+231261014126309+321261014666109+231261014126509+341261014130409+231261014126709+231261014126909</t>
+          <t>DHAN-341261014128909+341261014129109+231261014125709+321261014664109+321261014664809+231261014126009+321261014665609+231261014126409+341261014130309+341261014130509+221261014673909+341261014130709+221261014674609+221261014675009+221261014675509</t>
         </is>
       </c>
       <c r="B37" s="23" t="inlineStr">
         <is>
-          <t>KROSS</t>
+          <t>NIBE</t>
         </is>
       </c>
       <c r="C37" s="23" t="inlineStr">
@@ -34182,24 +34474,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D37" s="24" t="inlineStr"/>
+      <c r="D37" s="24" t="n">
+        <v>46310</v>
+      </c>
       <c r="E37" s="4" t="n">
-        <v>0</v>
+        <v>59.64</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>0</v>
+        <v>198.83</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>0</v>
+        <v>6.1</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>0</v>
+        <v>29.82</v>
       </c>
       <c r="J37" s="4" t="n">
-        <v>0</v>
+        <v>11.87</v>
       </c>
       <c r="K37" s="4" t="n">
         <v>14.75</v>
@@ -34208,7 +34502,7 @@
         <v>35.4</v>
       </c>
       <c r="M37" s="4" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="N37" s="21">
         <f>SUM(E37:M37)</f>
@@ -34218,12 +34512,12 @@
     <row r="38">
       <c r="A38" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261012625809+321261012626209+23126101284209+23126101284309+321261012626909+34126101276209+34126101277109+321261012628809+221261012640809+23126101286309+34126101278009+321261012630809+221261012643209</t>
+          <t>DHAN-221261014671209+321261014663609+231261014125809+221261014672009+231261014125909+231261014126109+221261014673109+341261014130209+321261014666509+341261014130609+321261014667409+321261014667809+341261014131209+221261014676209+221261014676809</t>
         </is>
       </c>
       <c r="B38" s="23" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>RUBYMILLS</t>
         </is>
       </c>
       <c r="C38" s="23" t="inlineStr">
@@ -34231,24 +34525,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D38" s="24" t="inlineStr"/>
+      <c r="D38" s="24" t="n">
+        <v>46310</v>
+      </c>
       <c r="E38" s="4" t="n">
-        <v>24.76</v>
+        <v>0</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>3.4</v>
+        <v>99.63</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>2.63</v>
+        <v>3.06</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>0.09</v>
+        <v>0.1</v>
       </c>
       <c r="I38" s="4" t="n">
-        <v>3</v>
+        <v>14.94</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>4.95</v>
+        <v>0.57</v>
       </c>
       <c r="K38" s="4" t="n">
         <v>14.75</v>
@@ -34267,12 +34563,12 @@
     <row r="39">
       <c r="A39" s="23" t="inlineStr">
         <is>
-          <t>DHAN-341261014128909+341261014129109+231261014125709+321261014664109+321261014664809+231261014126009+321261014665609+231261014126409+341261014130309+341261014130509+221261014673909+341261014130709+221261014674609+221261014675009+221261014675509</t>
+          <t>DHAN-231261014125609+321261014663509+321261014663909+321261014664209+221261014672509+231261014126209+341261014130109+321261014666209+321261014666609+321261014666709+321261014667009+341261014130809+231261014127009+341261014131009+221261014675609</t>
         </is>
       </c>
       <c r="B39" s="23" t="inlineStr">
         <is>
-          <t>NIBE</t>
+          <t>SPORTKING</t>
         </is>
       </c>
       <c r="C39" s="23" t="inlineStr">
@@ -34280,24 +34576,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D39" s="24" t="inlineStr"/>
+      <c r="D39" s="24" t="n">
+        <v>46310</v>
+      </c>
       <c r="E39" s="4" t="n">
-        <v>0</v>
+        <v>60.05</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>0</v>
+        <v>200.11</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>0</v>
+        <v>6.14</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="I39" s="4" t="n">
-        <v>0</v>
+        <v>30.09</v>
       </c>
       <c r="J39" s="4" t="n">
-        <v>0</v>
+        <v>11.95</v>
       </c>
       <c r="K39" s="4" t="n">
         <v>14.75</v>
@@ -34306,7 +34604,7 @@
         <v>35.4</v>
       </c>
       <c r="M39" s="4" t="n">
-        <v>0</v>
+        <v>34.22</v>
       </c>
       <c r="N39" s="21">
         <f>SUM(E39:M39)</f>
@@ -34316,12 +34614,12 @@
     <row r="40">
       <c r="A40" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261014671209+321261014663609+231261014125809+221261014672009+231261014125909+231261014126109+221261014673109+341261014130209+321261014666509+341261014130609+321261014667409+321261014667809+341261014131209+221261014676209+221261014676809</t>
+          <t>DHAN-34126101377609+221261013593609+34126101378109+23126101376709+34126101378409+23126101377009+221261013595709+221261013596109+221261013596609+23126101377809+34126101379309+34126101379709+23126101378409+34126101379809+221261013599309+321261013576809</t>
         </is>
       </c>
       <c r="B40" s="23" t="inlineStr">
         <is>
-          <t>RUBYMILLS</t>
+          <t>INDOKEM</t>
         </is>
       </c>
       <c r="C40" s="23" t="inlineStr">
@@ -34334,19 +34632,19 @@
         <v>0</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>0</v>
+        <v>85.43000000000001</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>0</v>
+        <v>2.62</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>0</v>
+        <v>0.09</v>
       </c>
       <c r="I40" s="4" t="n">
-        <v>0</v>
+        <v>12.81</v>
       </c>
       <c r="J40" s="4" t="n">
-        <v>0</v>
+        <v>0.49</v>
       </c>
       <c r="K40" s="4" t="n">
         <v>14.75</v>
@@ -34365,12 +34663,12 @@
     <row r="41">
       <c r="A41" s="23" t="inlineStr">
         <is>
-          <t>DHAN-341261014128809+341261014129209+221261014671809+321261014664309+221261014672409+321261014664909+341261014130009+221261014673409+221261014673609+221261014673709+221261014674009+321261014667309+341261014130909</t>
+          <t>DHAN-321261015672409+231261015159509+341261015154309+321261015674209+231261015159809+321261015674909+341261015154809+221261015678909+321261015675709+221261015679609+231261015160509</t>
         </is>
       </c>
       <c r="B41" s="23" t="inlineStr">
         <is>
-          <t>SIMPLEXINF</t>
+          <t>JAICORPLTD</t>
         </is>
       </c>
       <c r="C41" s="23" t="inlineStr">
@@ -34414,12 +34712,12 @@
     <row r="42">
       <c r="A42" s="23" t="inlineStr">
         <is>
-          <t>DHAN-231261014125609+321261014663509+321261014663909+321261014664209+221261014672509+231261014126209+341261014130109+321261014666209+321261014666609+321261014666709+321261014667009+341261014130809+231261014127009+341261014131009+221261014675609</t>
+          <t>DHAN-321261012625809+321261012626209+23126101284209+23126101284309+321261012626909+34126101276209+34126101277109+321261012628809+221261012640809+23126101286309+34126101278009+321261012630809+221261012643209</t>
         </is>
       </c>
       <c r="B42" s="23" t="inlineStr">
         <is>
-          <t>SPORTKING</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="C42" s="23" t="inlineStr">
@@ -34429,28 +34727,28 @@
       </c>
       <c r="D42" s="24" t="inlineStr"/>
       <c r="E42" s="4" t="n">
-        <v>0</v>
+        <v>24.76</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="G42" s="4" t="n">
-        <v>0</v>
+        <v>2.63</v>
       </c>
       <c r="H42" s="4" t="n">
-        <v>0</v>
+        <v>0.09</v>
       </c>
       <c r="I42" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J42" s="4" t="n">
-        <v>0</v>
+        <v>4.95</v>
       </c>
       <c r="K42" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L42" s="4" t="n">
-        <v>35.4</v>
+        <v>0</v>
       </c>
       <c r="M42" s="4" t="n">
         <v>0</v>
@@ -34461,54 +34759,250 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="3" t="inlineStr">
+      <c r="A43" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-341261015154009+321261015672609+221261015677509+321261015674109+321261015674709+341261015154709+231261015160109+341261015154909+221261015679409+341261015155209+321261015676109</t>
+        </is>
+      </c>
+      <c r="B43" s="23" t="inlineStr">
+        <is>
+          <t>OAL</t>
+        </is>
+      </c>
+      <c r="C43" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D43" s="24" t="inlineStr"/>
+      <c r="E43" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J43" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K43" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L43" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M43" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N43" s="21">
+        <f>SUM(E43:M43)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-341261015153909+221261015677009+321261015673209+231261015159709+231261015159909+231261015160009+221261015678509+321261015675509+231261015160209+231261015160409+341261015155309</t>
+        </is>
+      </c>
+      <c r="B44" s="23" t="inlineStr">
+        <is>
+          <t>ORIENTELEC</t>
+        </is>
+      </c>
+      <c r="C44" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D44" s="24" t="inlineStr"/>
+      <c r="E44" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L44" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M44" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N44" s="21">
+        <f>SUM(E44:M44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-341261014128809+341261014129209+221261014671809+321261014664309+221261014672409+321261014664909+341261014130009+221261014673409+221261014673609+221261014673709+221261014674009+321261014667309+341261014130909</t>
+        </is>
+      </c>
+      <c r="B45" s="23" t="inlineStr">
+        <is>
+          <t>SIMPLEXINF</t>
+        </is>
+      </c>
+      <c r="C45" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D45" s="24" t="inlineStr"/>
+      <c r="E45" s="4" t="n">
+        <v>59.95</v>
+      </c>
+      <c r="F45" s="4" t="n">
+        <v>199.83</v>
+      </c>
+      <c r="G45" s="4" t="n">
+        <v>6.13</v>
+      </c>
+      <c r="H45" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I45" s="4" t="n">
+        <v>29.98</v>
+      </c>
+      <c r="J45" s="4" t="n">
+        <v>11.93</v>
+      </c>
+      <c r="K45" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L45" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M45" s="4" t="n">
+        <v>34.17</v>
+      </c>
+      <c r="N45" s="21">
+        <f>SUM(E45:M45)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-231261015159409+321261015672709+321261015673309+221261015677909+221261015678309+341261015154609+321261015675209+221261015678809+341261015155009+341261015155109+231261015160609+231261015160709+341261015155509</t>
+        </is>
+      </c>
+      <c r="B46" s="23" t="inlineStr">
+        <is>
+          <t>TEAMLEASE</t>
+        </is>
+      </c>
+      <c r="C46" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D46" s="24" t="inlineStr"/>
+      <c r="E46" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J46" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L46" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M46" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N46" s="21">
+        <f>SUM(E46:M46)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E43" s="32">
-        <f>SUM(E4:E42)</f>
-        <v/>
-      </c>
-      <c r="F43" s="32">
-        <f>SUM(F4:F42)</f>
-        <v/>
-      </c>
-      <c r="G43" s="32">
-        <f>SUM(G4:G42)</f>
-        <v/>
-      </c>
-      <c r="H43" s="32">
-        <f>SUM(H4:H42)</f>
-        <v/>
-      </c>
-      <c r="I43" s="32">
-        <f>SUM(I4:I42)</f>
-        <v/>
-      </c>
-      <c r="J43" s="32">
-        <f>SUM(J4:J42)</f>
-        <v/>
-      </c>
-      <c r="K43" s="32">
-        <f>SUM(K4:K42)</f>
-        <v/>
-      </c>
-      <c r="L43" s="32">
-        <f>SUM(L4:L42)</f>
-        <v/>
-      </c>
-      <c r="M43" s="32">
-        <f>SUM(M4:M42)</f>
-        <v/>
-      </c>
-      <c r="N43" s="32">
-        <f>SUM(N4:N42)</f>
+      <c r="E47" s="32">
+        <f>SUM(E4:E46)</f>
+        <v/>
+      </c>
+      <c r="F47" s="32">
+        <f>SUM(F4:F46)</f>
+        <v/>
+      </c>
+      <c r="G47" s="32">
+        <f>SUM(G4:G46)</f>
+        <v/>
+      </c>
+      <c r="H47" s="32">
+        <f>SUM(H4:H46)</f>
+        <v/>
+      </c>
+      <c r="I47" s="32">
+        <f>SUM(I4:I46)</f>
+        <v/>
+      </c>
+      <c r="J47" s="32">
+        <f>SUM(J4:J46)</f>
+        <v/>
+      </c>
+      <c r="K47" s="32">
+        <f>SUM(K4:K46)</f>
+        <v/>
+      </c>
+      <c r="L47" s="32">
+        <f>SUM(L4:L46)</f>
+        <v/>
+      </c>
+      <c r="M47" s="32">
+        <f>SUM(M4:M46)</f>
+        <v/>
+      </c>
+      <c r="N47" s="32">
+        <f>SUM(N4:N46)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:N42"/>
+  <autoFilter ref="A3:N46"/>
   <mergeCells count="2">
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>

</xml_diff>

<commit_message>
Data update — 2026-10-16 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_oct2026.xlsx
+++ b/results/strategy_pnl_oct2026.xlsx
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trade Log'!$A$3:$O$503</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$50</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1214,7 +1214,7 @@
         <v/>
       </c>
       <c r="K6" s="4" t="n">
-        <v>964.78</v>
+        <v>959.98</v>
       </c>
       <c r="L6" s="21">
         <f>IF(OR($B6="",$I6=""),"",$I6-IF($K6="",0,$K6))</f>
@@ -1274,7 +1274,7 @@
         <v/>
       </c>
       <c r="K7" s="4" t="n">
-        <v>824.88</v>
+        <v>822.01</v>
       </c>
       <c r="L7" s="21">
         <f>IF(OR($B7="",$I7=""),"",$I7-IF($K7="",0,$K7))</f>
@@ -1334,7 +1334,7 @@
         <v/>
       </c>
       <c r="K8" s="4" t="n">
-        <v>836.1</v>
+        <v>861.4</v>
       </c>
       <c r="L8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($K8="",0,$K8))</f>
@@ -1394,7 +1394,7 @@
         <v/>
       </c>
       <c r="K9" s="4" t="n">
-        <v>979.22</v>
+        <v>974.4299999999999</v>
       </c>
       <c r="L9" s="21">
         <f>IF(OR($B9="",$I9=""),"",$I9-IF($K9="",0,$K9))</f>
@@ -1454,7 +1454,7 @@
         <v/>
       </c>
       <c r="K10" s="4" t="n">
-        <v>951.17</v>
+        <v>947.17</v>
       </c>
       <c r="L10" s="21">
         <f>IF(OR($B10="",$I10=""),"",$I10-IF($K10="",0,$K10))</f>
@@ -1514,7 +1514,7 @@
         <v/>
       </c>
       <c r="K11" s="4" t="n">
-        <v>673.6900000000001</v>
+        <v>694.14</v>
       </c>
       <c r="L11" s="21">
         <f>IF(OR($B11="",$I11=""),"",$I11-IF($K11="",0,$K11))</f>
@@ -1574,7 +1574,7 @@
         <v/>
       </c>
       <c r="K12" s="4" t="n">
-        <v>735.3200000000001</v>
+        <v>759.8200000000001</v>
       </c>
       <c r="L12" s="21">
         <f>IF(OR($B12="",$I12=""),"",$I12-IF($K12="",0,$K12))</f>
@@ -1634,7 +1634,7 @@
         <v/>
       </c>
       <c r="K13" s="4" t="n">
-        <v>645.21</v>
+        <v>659.95</v>
       </c>
       <c r="L13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($K13="",0,$K13))</f>
@@ -1694,7 +1694,7 @@
         <v/>
       </c>
       <c r="K14" s="4" t="n">
-        <v>654.64</v>
+        <v>669.3200000000001</v>
       </c>
       <c r="L14" s="21">
         <f>IF(OR($B14="",$I14=""),"",$I14-IF($K14="",0,$K14))</f>
@@ -1874,7 +1874,7 @@
         <v/>
       </c>
       <c r="K17" s="4" t="n">
-        <v>651.58</v>
+        <v>630.54</v>
       </c>
       <c r="L17" s="21">
         <f>IF(OR($B17="",$I17=""),"",$I17-IF($K17="",0,$K17))</f>
@@ -1994,7 +1994,7 @@
         <v/>
       </c>
       <c r="K19" s="4" t="n">
-        <v>707.7</v>
+        <v>671.47</v>
       </c>
       <c r="L19" s="21">
         <f>IF(OR($B19="",$I19=""),"",$I19-IF($K19="",0,$K19))</f>
@@ -2054,7 +2054,7 @@
         <v/>
       </c>
       <c r="K20" s="4" t="n">
-        <v>716.86</v>
+        <v>681.75</v>
       </c>
       <c r="L20" s="21">
         <f>IF(OR($B20="",$I20=""),"",$I20-IF($K20="",0,$K20))</f>
@@ -2174,7 +2174,7 @@
         <v/>
       </c>
       <c r="K22" s="4" t="n">
-        <v>698.64</v>
+        <v>663.37</v>
       </c>
       <c r="L22" s="21">
         <f>IF(OR($B22="",$I22=""),"",$I22-IF($K22="",0,$K22))</f>
@@ -2234,7 +2234,7 @@
         <v/>
       </c>
       <c r="K23" s="4" t="n">
-        <v>419.24</v>
+        <v>421.4</v>
       </c>
       <c r="L23" s="21">
         <f>IF(OR($B23="",$I23=""),"",$I23-IF($K23="",0,$K23))</f>
@@ -2354,7 +2354,7 @@
         <v/>
       </c>
       <c r="K25" s="4" t="n">
-        <v>556.73</v>
+        <v>559.4</v>
       </c>
       <c r="L25" s="21">
         <f>IF(OR($B25="",$I25=""),"",$I25-IF($K25="",0,$K25))</f>
@@ -2414,7 +2414,7 @@
         <v/>
       </c>
       <c r="K26" s="4" t="n">
-        <v>547.09</v>
+        <v>549.67</v>
       </c>
       <c r="L26" s="21">
         <f>IF(OR($B26="",$I26=""),"",$I26-IF($K26="",0,$K26))</f>
@@ -2474,7 +2474,7 @@
         <v/>
       </c>
       <c r="K27" s="4" t="n">
-        <v>547.28</v>
+        <v>550.23</v>
       </c>
       <c r="L27" s="21">
         <f>IF(OR($B27="",$I27=""),"",$I27-IF($K27="",0,$K27))</f>
@@ -2534,7 +2534,7 @@
         <v/>
       </c>
       <c r="K28" s="4" t="n">
-        <v>554.42</v>
+        <v>557.4</v>
       </c>
       <c r="L28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($K28="",0,$K28))</f>
@@ -2594,7 +2594,7 @@
         <v/>
       </c>
       <c r="K29" s="4" t="n">
-        <v>550.21</v>
+        <v>552.79</v>
       </c>
       <c r="L29" s="21">
         <f>IF(OR($B29="",$I29=""),"",$I29-IF($K29="",0,$K29))</f>
@@ -2714,7 +2714,7 @@
         <v/>
       </c>
       <c r="K31" s="4" t="n">
-        <v>550.35</v>
+        <v>552.91</v>
       </c>
       <c r="L31" s="21">
         <f>IF(OR($B31="",$I31=""),"",$I31-IF($K31="",0,$K31))</f>
@@ -2774,7 +2774,7 @@
         <v/>
       </c>
       <c r="K32" s="4" t="n">
-        <v>425.43</v>
+        <v>428.12</v>
       </c>
       <c r="L32" s="21">
         <f>IF(OR($B32="",$I32=""),"",$I32-IF($K32="",0,$K32))</f>
@@ -2894,7 +2894,7 @@
         <v/>
       </c>
       <c r="K34" s="4" t="n">
-        <v>552.55</v>
+        <v>540.04</v>
       </c>
       <c r="L34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($K34="",0,$K34))</f>
@@ -2954,7 +2954,7 @@
         <v/>
       </c>
       <c r="K35" s="4" t="n">
-        <v>306.62</v>
+        <v>480.15</v>
       </c>
       <c r="L35" s="21">
         <f>IF(OR($B35="",$I35=""),"",$I35-IF($K35="",0,$K35))</f>
@@ -3014,7 +3014,7 @@
         <v/>
       </c>
       <c r="K36" s="4" t="n">
-        <v>392.78</v>
+        <v>626.08</v>
       </c>
       <c r="L36" s="21">
         <f>IF(OR($B36="",$I36=""),"",$I36-IF($K36="",0,$K36))</f>
@@ -3074,7 +3074,7 @@
         <v/>
       </c>
       <c r="K37" s="4" t="n">
-        <v>390.61</v>
+        <v>616.02</v>
       </c>
       <c r="L37" s="21">
         <f>IF(OR($B37="",$I37=""),"",$I37-IF($K37="",0,$K37))</f>
@@ -3134,7 +3134,7 @@
         <v/>
       </c>
       <c r="K38" s="4" t="n">
-        <v>133.05</v>
+        <v>238.83</v>
       </c>
       <c r="L38" s="21">
         <f>IF(OR($B38="",$I38=""),"",$I38-IF($K38="",0,$K38))</f>
@@ -3194,7 +3194,7 @@
         <v/>
       </c>
       <c r="K39" s="4" t="n">
-        <v>392.91</v>
+        <v>627.33</v>
       </c>
       <c r="L39" s="21">
         <f>IF(OR($B39="",$I39=""),"",$I39-IF($K39="",0,$K39))</f>
@@ -3217,12 +3217,12 @@
     <row r="40">
       <c r="A40" s="23" t="inlineStr">
         <is>
-          <t>DHAN-34126101377609+221261013593609+34126101378109+23126101376709+34126101378409+23126101377009+221261013595709+221261013596109+221261013596609+23126101377809+34126101379309+34126101379709+23126101378409+34126101379809+221261013599309+321261013576809</t>
+          <t>DHAN-321261015672409+231261015159509+341261015154309+321261015674209+231261015159809+321261015674909+341261015154809+221261015678909+321261015675709+221261015679609+231261015160509</t>
         </is>
       </c>
       <c r="B40" s="23" t="inlineStr">
         <is>
-          <t>INDOKEM</t>
+          <t>JAICORPLTD</t>
         </is>
       </c>
       <c r="C40" s="23" t="inlineStr">
@@ -3231,16 +3231,20 @@
         </is>
       </c>
       <c r="D40" s="24" t="n">
-        <v>46308</v>
+        <v>46310</v>
       </c>
       <c r="E40" s="25" t="n">
-        <v>677.9853000000001</v>
+        <v>95.05800000000001</v>
       </c>
       <c r="F40" s="26" t="n">
-        <v>126</v>
-      </c>
-      <c r="G40" s="24" t="inlineStr"/>
-      <c r="H40" s="25" t="inlineStr"/>
+        <v>3153</v>
+      </c>
+      <c r="G40" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H40" s="25" t="n">
+        <v>94.26000000000001</v>
+      </c>
       <c r="I40" s="21">
         <f>IF(OR($B40="",$H40=""),"",IF($C40="LONG",($H40-$E40)*$F40,($E40-$H40)*$F40))</f>
         <v/>
@@ -3250,7 +3254,7 @@
         <v/>
       </c>
       <c r="K40" s="4" t="n">
-        <v>116.19</v>
+        <v>547.34</v>
       </c>
       <c r="L40" s="21">
         <f>IF(OR($B40="",$I40=""),"",$I40-IF($K40="",0,$K40))</f>
@@ -3266,19 +3270,19 @@
       </c>
       <c r="O40" s="23" t="inlineStr">
         <is>
-          <t>10-15</t>
+          <t>5-10</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261015672409+231261015159509+341261015154309+321261015674209+231261015159809+321261015674909+341261015154809+221261015678909+321261015675709+221261015679609+231261015160509</t>
+          <t>DHAN-341261015154009+321261015672609+221261015677509+321261015674109+321261015674709+341261015154709+231261015160109+341261015154909+221261015679409+341261015155209+321261015676109</t>
         </is>
       </c>
       <c r="B41" s="23" t="inlineStr">
         <is>
-          <t>JAICORPLTD</t>
+          <t>OAL</t>
         </is>
       </c>
       <c r="C41" s="23" t="inlineStr">
@@ -3290,13 +3294,17 @@
         <v>46310</v>
       </c>
       <c r="E41" s="25" t="n">
-        <v>95.05800000000001</v>
+        <v>578.2952</v>
       </c>
       <c r="F41" s="26" t="n">
-        <v>3153</v>
-      </c>
-      <c r="G41" s="24" t="inlineStr"/>
-      <c r="H41" s="25" t="inlineStr"/>
+        <v>258</v>
+      </c>
+      <c r="G41" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H41" s="25" t="n">
+        <v>585.09</v>
+      </c>
       <c r="I41" s="21">
         <f>IF(OR($B41="",$H41=""),"",IF($C41="LONG",($H41-$E41)*$F41,($E41-$H41)*$F41))</f>
         <v/>
@@ -3306,7 +3314,7 @@
         <v/>
       </c>
       <c r="K41" s="4" t="n">
-        <v>50.15</v>
+        <v>191.91</v>
       </c>
       <c r="L41" s="21">
         <f>IF(OR($B41="",$I41=""),"",$I41-IF($K41="",0,$K41))</f>
@@ -3322,19 +3330,19 @@
       </c>
       <c r="O41" s="23" t="inlineStr">
         <is>
-          <t>5-10</t>
+          <t>10-15</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261012625809+321261012626209+23126101284209+23126101284309+321261012626909+34126101276209+34126101277109+321261012628809+221261012640809+23126101286309+34126101278009+321261012630809+221261012643209</t>
+          <t>DHAN-341261015153909+221261015677009+321261015673209+231261015159709+231261015159909+231261015160009+221261015678509+321261015675509+231261015160209+231261015160409+341261015155309</t>
         </is>
       </c>
       <c r="B42" s="23" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>ORIENTELEC</t>
         </is>
       </c>
       <c r="C42" s="23" t="inlineStr">
@@ -3343,16 +3351,20 @@
         </is>
       </c>
       <c r="D42" s="24" t="n">
-        <v>46307</v>
+        <v>46310</v>
       </c>
       <c r="E42" s="25" t="n">
-        <v>22.8999</v>
+        <v>201.1512</v>
       </c>
       <c r="F42" s="26" t="n">
-        <v>3742</v>
-      </c>
-      <c r="G42" s="24" t="inlineStr"/>
-      <c r="H42" s="25" t="inlineStr"/>
+        <v>1500</v>
+      </c>
+      <c r="G42" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H42" s="25" t="n">
+        <v>206.72</v>
+      </c>
       <c r="I42" s="21">
         <f>IF(OR($B42="",$H42=""),"",IF($C42="LONG",($H42-$E42)*$F42,($E42-$H42)*$F42))</f>
         <v/>
@@ -3362,7 +3374,7 @@
         <v/>
       </c>
       <c r="K42" s="4" t="n">
-        <v>53.57</v>
+        <v>552.14</v>
       </c>
       <c r="L42" s="21">
         <f>IF(OR($B42="",$I42=""),"",$I42-IF($K42="",0,$K42))</f>
@@ -3378,19 +3390,19 @@
       </c>
       <c r="O42" s="23" t="inlineStr">
         <is>
-          <t>5-10</t>
+          <t>10-15</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="23" t="inlineStr">
         <is>
-          <t>DHAN-341261015154009+321261015672609+221261015677509+321261015674109+321261015674709+341261015154709+231261015160109+341261015154909+221261015679409+341261015155209+321261015676109</t>
+          <t>DHAN-231261015159409+321261015672709+321261015673309+221261015677909+221261015678309+341261015154609+321261015675209+221261015678809+341261015155009+341261015155109+231261015160609+231261015160709+341261015155509</t>
         </is>
       </c>
       <c r="B43" s="23" t="inlineStr">
         <is>
-          <t>OAL</t>
+          <t>TEAMLEASE</t>
         </is>
       </c>
       <c r="C43" s="23" t="inlineStr">
@@ -3402,13 +3414,17 @@
         <v>46310</v>
       </c>
       <c r="E43" s="25" t="n">
-        <v>578.2952</v>
+        <v>1133.7498</v>
       </c>
       <c r="F43" s="26" t="n">
-        <v>258</v>
-      </c>
-      <c r="G43" s="24" t="inlineStr"/>
-      <c r="H43" s="25" t="inlineStr"/>
+        <v>263</v>
+      </c>
+      <c r="G43" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H43" s="25" t="n">
+        <v>1124.65</v>
+      </c>
       <c r="I43" s="21">
         <f>IF(OR($B43="",$H43=""),"",IF($C43="LONG",($H43-$E43)*$F43,($E43-$H43)*$F43))</f>
         <v/>
@@ -3418,7 +3434,7 @@
         <v/>
       </c>
       <c r="K43" s="4" t="n">
-        <v>14.75</v>
+        <v>542.6</v>
       </c>
       <c r="L43" s="21">
         <f>IF(OR($B43="",$I43=""),"",$I43-IF($K43="",0,$K43))</f>
@@ -3434,19 +3450,19 @@
       </c>
       <c r="O43" s="23" t="inlineStr">
         <is>
-          <t>10-15</t>
+          <t>5-10</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="23" t="inlineStr">
         <is>
-          <t>DHAN-341261015153909+221261015677009+321261015673209+231261015159709+231261015159909+231261015160009+221261015678509+321261015675509+231261015160209+231261015160409+341261015155309</t>
+          <t>DHAN-321261016683609+23126101679509+23126101679909+321261016685009+221261016694409+221261016695109+34126101677409+321261016686809+23126101680709+321261016687809+23126101681009+34126101678009</t>
         </is>
       </c>
       <c r="B44" s="23" t="inlineStr">
         <is>
-          <t>ORIENTELEC</t>
+          <t>EUROPRATIK</t>
         </is>
       </c>
       <c r="C44" s="23" t="inlineStr">
@@ -3455,13 +3471,13 @@
         </is>
       </c>
       <c r="D44" s="24" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="E44" s="25" t="n">
-        <v>201.1512</v>
+        <v>182.5264</v>
       </c>
       <c r="F44" s="26" t="n">
-        <v>1500</v>
+        <v>1636</v>
       </c>
       <c r="G44" s="24" t="inlineStr"/>
       <c r="H44" s="25" t="inlineStr"/>
@@ -3497,12 +3513,12 @@
     <row r="45">
       <c r="A45" s="23" t="inlineStr">
         <is>
-          <t>DHAN-341261014128809+341261014129209+221261014671809+321261014664309+221261014672409+321261014664909+341261014130009+221261014673409+221261014673609+221261014673709+221261014674009+321261014667309+341261014130909</t>
+          <t>DHAN-34126101377609+221261013593609+34126101378109+23126101376709+34126101378409+23126101377009+221261013595709+221261013596109+221261013596609+23126101377809+34126101379309+34126101379709+23126101378409+34126101379809+221261013599309+321261013576809</t>
         </is>
       </c>
       <c r="B45" s="23" t="inlineStr">
         <is>
-          <t>SIMPLEXINF</t>
+          <t>INDOKEM</t>
         </is>
       </c>
       <c r="C45" s="23" t="inlineStr">
@@ -3511,13 +3527,13 @@
         </is>
       </c>
       <c r="D45" s="24" t="n">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="E45" s="25" t="n">
-        <v>266.801</v>
+        <v>677.9853000000001</v>
       </c>
       <c r="F45" s="26" t="n">
-        <v>749</v>
+        <v>126</v>
       </c>
       <c r="G45" s="24" t="inlineStr"/>
       <c r="H45" s="25" t="inlineStr"/>
@@ -3530,7 +3546,7 @@
         <v/>
       </c>
       <c r="K45" s="4" t="n">
-        <v>392.35</v>
+        <v>116.19</v>
       </c>
       <c r="L45" s="21">
         <f>IF(OR($B45="",$I45=""),"",$I45-IF($K45="",0,$K45))</f>
@@ -3546,19 +3562,19 @@
       </c>
       <c r="O45" s="23" t="inlineStr">
         <is>
-          <t>5-10</t>
+          <t>10-15</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="23" t="inlineStr">
         <is>
-          <t>DHAN-231261015159409+321261015672709+321261015673309+221261015677909+221261015678309+341261015154609+321261015675209+221261015678809+341261015155009+341261015155109+231261015160609+231261015160709+341261015155509</t>
+          <t>DHAN-221261016693009+23126101679709+23126101679809+23126101680009+321261016685409+221261016694909+34126101677509+321261016686909+34126101677709+321261016687909+34126101677909</t>
         </is>
       </c>
       <c r="B46" s="23" t="inlineStr">
         <is>
-          <t>TEAMLEASE</t>
+          <t>MBEL</t>
         </is>
       </c>
       <c r="C46" s="23" t="inlineStr">
@@ -3567,13 +3583,13 @@
         </is>
       </c>
       <c r="D46" s="24" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="E46" s="25" t="n">
-        <v>1133.7498</v>
+        <v>287.8416</v>
       </c>
       <c r="F46" s="26" t="n">
-        <v>263</v>
+        <v>1043</v>
       </c>
       <c r="G46" s="24" t="inlineStr"/>
       <c r="H46" s="25" t="inlineStr"/>
@@ -3607,14 +3623,32 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="23" t="n"/>
-      <c r="B47" s="23" t="n"/>
-      <c r="C47" s="23" t="n"/>
-      <c r="D47" s="24" t="n"/>
-      <c r="E47" s="25" t="n"/>
-      <c r="F47" s="26" t="n"/>
-      <c r="G47" s="24" t="n"/>
-      <c r="H47" s="25" t="n"/>
+      <c r="A47" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261012625809+321261012626209+23126101284209+23126101284309+321261012626909+34126101276209+34126101277109+321261012628809+221261012640809+23126101286309+34126101278009+321261012630809+221261012643209</t>
+        </is>
+      </c>
+      <c r="B47" s="23" t="inlineStr">
+        <is>
+          <t>MMWL</t>
+        </is>
+      </c>
+      <c r="C47" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D47" s="24" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E47" s="25" t="n">
+        <v>22.8999</v>
+      </c>
+      <c r="F47" s="26" t="n">
+        <v>3742</v>
+      </c>
+      <c r="G47" s="24" t="inlineStr"/>
+      <c r="H47" s="25" t="inlineStr"/>
       <c r="I47" s="21">
         <f>IF(OR($B47="",$H47=""),"",IF($C47="LONG",($H47-$E47)*$F47,($E47-$H47)*$F47))</f>
         <v/>
@@ -3623,7 +3657,9 @@
         <f>IF(OR($B47="",$I47="",$E47=0,$F47=0),"",$I47/($E47*$F47))</f>
         <v/>
       </c>
-      <c r="K47" s="4" t="n"/>
+      <c r="K47" s="4" t="n">
+        <v>53.57</v>
+      </c>
       <c r="L47" s="21">
         <f>IF(OR($B47="",$I47=""),"",$I47-IF($K47="",0,$K47))</f>
         <v/>
@@ -3636,17 +3672,39 @@
         <f>IF($B47="","",IF($H47="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O47" s="23" t="n"/>
+      <c r="O47" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="23" t="n"/>
-      <c r="B48" s="23" t="n"/>
-      <c r="C48" s="23" t="n"/>
-      <c r="D48" s="24" t="n"/>
-      <c r="E48" s="25" t="n"/>
-      <c r="F48" s="26" t="n"/>
-      <c r="G48" s="24" t="n"/>
-      <c r="H48" s="25" t="n"/>
+      <c r="A48" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261016683509+23126101679609+221261016693309+321261016685109+321261016685509+321261016685809+221261016695509+34126101677609+23126101680609+23126101680809+321261016688709+321261016689109+221261016697009+321261016690409</t>
+        </is>
+      </c>
+      <c r="B48" s="23" t="inlineStr">
+        <is>
+          <t>PARACABLES</t>
+        </is>
+      </c>
+      <c r="C48" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D48" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="E48" s="25" t="n">
+        <v>60.1311</v>
+      </c>
+      <c r="F48" s="26" t="n">
+        <v>4996</v>
+      </c>
+      <c r="G48" s="24" t="inlineStr"/>
+      <c r="H48" s="25" t="inlineStr"/>
       <c r="I48" s="21">
         <f>IF(OR($B48="",$H48=""),"",IF($C48="LONG",($H48-$E48)*$F48,($E48-$H48)*$F48))</f>
         <v/>
@@ -3655,7 +3713,9 @@
         <f>IF(OR($B48="",$I48="",$E48=0,$F48=0),"",$I48/($E48*$F48))</f>
         <v/>
       </c>
-      <c r="K48" s="4" t="n"/>
+      <c r="K48" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L48" s="21">
         <f>IF(OR($B48="",$I48=""),"",$I48-IF($K48="",0,$K48))</f>
         <v/>
@@ -3668,17 +3728,39 @@
         <f>IF($B48="","",IF($H48="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O48" s="23" t="n"/>
+      <c r="O48" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="23" t="n"/>
-      <c r="B49" s="23" t="n"/>
-      <c r="C49" s="23" t="n"/>
-      <c r="D49" s="24" t="n"/>
-      <c r="E49" s="25" t="n"/>
-      <c r="F49" s="26" t="n"/>
-      <c r="G49" s="24" t="n"/>
-      <c r="H49" s="25" t="n"/>
+      <c r="A49" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-341261014128809+341261014129209+221261014671809+321261014664309+221261014672409+321261014664909+341261014130009+221261014673409+221261014673609+221261014673709+221261014674009+321261014667309+341261014130909</t>
+        </is>
+      </c>
+      <c r="B49" s="23" t="inlineStr">
+        <is>
+          <t>SIMPLEXINF</t>
+        </is>
+      </c>
+      <c r="C49" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D49" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E49" s="25" t="n">
+        <v>266.801</v>
+      </c>
+      <c r="F49" s="26" t="n">
+        <v>749</v>
+      </c>
+      <c r="G49" s="24" t="inlineStr"/>
+      <c r="H49" s="25" t="inlineStr"/>
       <c r="I49" s="21">
         <f>IF(OR($B49="",$H49=""),"",IF($C49="LONG",($H49-$E49)*$F49,($E49-$H49)*$F49))</f>
         <v/>
@@ -3687,7 +3769,9 @@
         <f>IF(OR($B49="",$I49="",$E49=0,$F49=0),"",$I49/($E49*$F49))</f>
         <v/>
       </c>
-      <c r="K49" s="4" t="n"/>
+      <c r="K49" s="4" t="n">
+        <v>394.85</v>
+      </c>
       <c r="L49" s="21">
         <f>IF(OR($B49="",$I49=""),"",$I49-IF($K49="",0,$K49))</f>
         <v/>
@@ -3700,17 +3784,39 @@
         <f>IF($B49="","",IF($H49="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O49" s="23" t="n"/>
+      <c r="O49" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="50">
-      <c r="A50" s="23" t="n"/>
-      <c r="B50" s="23" t="n"/>
-      <c r="C50" s="23" t="n"/>
-      <c r="D50" s="24" t="n"/>
-      <c r="E50" s="25" t="n"/>
-      <c r="F50" s="26" t="n"/>
-      <c r="G50" s="24" t="n"/>
-      <c r="H50" s="25" t="n"/>
+      <c r="A50" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261016692909+321261016684009+321261016684509+221261016693809+23126101680109+221261016695009+321261016686109+23126101680509+221261016696009+23126101680909+34126101677809+23126101681109</t>
+        </is>
+      </c>
+      <c r="B50" s="23" t="inlineStr">
+        <is>
+          <t>SOLARA</t>
+        </is>
+      </c>
+      <c r="C50" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D50" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="E50" s="25" t="n">
+        <v>693.1007</v>
+      </c>
+      <c r="F50" s="26" t="n">
+        <v>434</v>
+      </c>
+      <c r="G50" s="24" t="inlineStr"/>
+      <c r="H50" s="25" t="inlineStr"/>
       <c r="I50" s="21">
         <f>IF(OR($B50="",$H50=""),"",IF($C50="LONG",($H50-$E50)*$F50,($E50-$H50)*$F50))</f>
         <v/>
@@ -3719,7 +3825,9 @@
         <f>IF(OR($B50="",$I50="",$E50=0,$F50=0),"",$I50/($E50*$F50))</f>
         <v/>
       </c>
-      <c r="K50" s="4" t="n"/>
+      <c r="K50" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L50" s="21">
         <f>IF(OR($B50="",$I50=""),"",$I50-IF($K50="",0,$K50))</f>
         <v/>
@@ -3732,7 +3840,11 @@
         <f>IF($B50="","",IF($H50="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O50" s="23" t="n"/>
+      <c r="O50" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="23" t="n"/>
@@ -30905,7 +31017,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J42"/>
+  <dimension ref="A1:J46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31204,7 +31316,7 @@
     <row r="9">
       <c r="A9" s="27" t="inlineStr">
         <is>
-          <t>GOODLUCK</t>
+          <t>EUROPRATIK</t>
         </is>
       </c>
       <c r="B9" s="20">
@@ -31247,7 +31359,7 @@
     <row r="10">
       <c r="A10" s="27" t="inlineStr">
         <is>
-          <t>GPTINFRA</t>
+          <t>GOODLUCK</t>
         </is>
       </c>
       <c r="B10" s="20">
@@ -31290,7 +31402,7 @@
     <row r="11">
       <c r="A11" s="27" t="inlineStr">
         <is>
-          <t>HATHWAY</t>
+          <t>GPTINFRA</t>
         </is>
       </c>
       <c r="B11" s="20">
@@ -31333,7 +31445,7 @@
     <row r="12">
       <c r="A12" s="27" t="inlineStr">
         <is>
-          <t>INDIAGLYCO</t>
+          <t>HATHWAY</t>
         </is>
       </c>
       <c r="B12" s="20">
@@ -31376,7 +31488,7 @@
     <row r="13">
       <c r="A13" s="27" t="inlineStr">
         <is>
-          <t>INDOKEM</t>
+          <t>INDIAGLYCO</t>
         </is>
       </c>
       <c r="B13" s="20">
@@ -31419,7 +31531,7 @@
     <row r="14">
       <c r="A14" s="27" t="inlineStr">
         <is>
-          <t>INOXGREEN</t>
+          <t>INDOKEM</t>
         </is>
       </c>
       <c r="B14" s="20">
@@ -31462,7 +31574,7 @@
     <row r="15">
       <c r="A15" s="27" t="inlineStr">
         <is>
-          <t>JAICORPLTD</t>
+          <t>INOXGREEN</t>
         </is>
       </c>
       <c r="B15" s="20">
@@ -31505,7 +31617,7 @@
     <row r="16">
       <c r="A16" s="27" t="inlineStr">
         <is>
-          <t>JINDALPOLY</t>
+          <t>JAICORPLTD</t>
         </is>
       </c>
       <c r="B16" s="20">
@@ -31548,7 +31660,7 @@
     <row r="17">
       <c r="A17" s="27" t="inlineStr">
         <is>
-          <t>KOTIC</t>
+          <t>JINDALPOLY</t>
         </is>
       </c>
       <c r="B17" s="20">
@@ -31591,7 +31703,7 @@
     <row r="18">
       <c r="A18" s="27" t="inlineStr">
         <is>
-          <t>KRISHNADEF</t>
+          <t>KOTIC</t>
         </is>
       </c>
       <c r="B18" s="20">
@@ -31634,7 +31746,7 @@
     <row r="19">
       <c r="A19" s="27" t="inlineStr">
         <is>
-          <t>KROSS</t>
+          <t>KRISHNADEF</t>
         </is>
       </c>
       <c r="B19" s="20">
@@ -31677,7 +31789,7 @@
     <row r="20">
       <c r="A20" s="27" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>KROSS</t>
         </is>
       </c>
       <c r="B20" s="20">
@@ -31720,7 +31832,7 @@
     <row r="21">
       <c r="A21" s="27" t="inlineStr">
         <is>
-          <t>MOBIKWIK</t>
+          <t>MBEL</t>
         </is>
       </c>
       <c r="B21" s="20">
@@ -31763,7 +31875,7 @@
     <row r="22">
       <c r="A22" s="27" t="inlineStr">
         <is>
-          <t>NIBE</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="B22" s="20">
@@ -31806,7 +31918,7 @@
     <row r="23">
       <c r="A23" s="27" t="inlineStr">
         <is>
-          <t>OAL</t>
+          <t>MOBIKWIK</t>
         </is>
       </c>
       <c r="B23" s="20">
@@ -31849,7 +31961,7 @@
     <row r="24">
       <c r="A24" s="27" t="inlineStr">
         <is>
-          <t>ORIENTELEC</t>
+          <t>NIBE</t>
         </is>
       </c>
       <c r="B24" s="20">
@@ -31892,7 +32004,7 @@
     <row r="25">
       <c r="A25" s="27" t="inlineStr">
         <is>
-          <t>PIXTRANS</t>
+          <t>OAL</t>
         </is>
       </c>
       <c r="B25" s="20">
@@ -31935,7 +32047,7 @@
     <row r="26">
       <c r="A26" s="27" t="inlineStr">
         <is>
-          <t>PNCINFRA</t>
+          <t>ORIENTELEC</t>
         </is>
       </c>
       <c r="B26" s="20">
@@ -31978,7 +32090,7 @@
     <row r="27">
       <c r="A27" s="27" t="inlineStr">
         <is>
-          <t>PNGSREVA</t>
+          <t>PARACABLES</t>
         </is>
       </c>
       <c r="B27" s="20">
@@ -32021,7 +32133,7 @@
     <row r="28">
       <c r="A28" s="27" t="inlineStr">
         <is>
-          <t>PRINCEPIPE</t>
+          <t>PIXTRANS</t>
         </is>
       </c>
       <c r="B28" s="20">
@@ -32064,7 +32176,7 @@
     <row r="29">
       <c r="A29" s="27" t="inlineStr">
         <is>
-          <t>RSYSTEMS</t>
+          <t>PNCINFRA</t>
         </is>
       </c>
       <c r="B29" s="20">
@@ -32107,7 +32219,7 @@
     <row r="30">
       <c r="A30" s="27" t="inlineStr">
         <is>
-          <t>RUBYMILLS</t>
+          <t>PNGSREVA</t>
         </is>
       </c>
       <c r="B30" s="20">
@@ -32150,7 +32262,7 @@
     <row r="31">
       <c r="A31" s="27" t="inlineStr">
         <is>
-          <t>SAKSOFT</t>
+          <t>PRINCEPIPE</t>
         </is>
       </c>
       <c r="B31" s="20">
@@ -32193,7 +32305,7 @@
     <row r="32">
       <c r="A32" s="27" t="inlineStr">
         <is>
-          <t>SATIN</t>
+          <t>RSYSTEMS</t>
         </is>
       </c>
       <c r="B32" s="20">
@@ -32236,7 +32348,7 @@
     <row r="33">
       <c r="A33" s="27" t="inlineStr">
         <is>
-          <t>SGFIN</t>
+          <t>RUBYMILLS</t>
         </is>
       </c>
       <c r="B33" s="20">
@@ -32279,7 +32391,7 @@
     <row r="34">
       <c r="A34" s="27" t="inlineStr">
         <is>
-          <t>SHRINGARMS</t>
+          <t>SAKSOFT</t>
         </is>
       </c>
       <c r="B34" s="20">
@@ -32322,7 +32434,7 @@
     <row r="35">
       <c r="A35" s="27" t="inlineStr">
         <is>
-          <t>SIMPLEXINF</t>
+          <t>SATIN</t>
         </is>
       </c>
       <c r="B35" s="20">
@@ -32365,7 +32477,7 @@
     <row r="36">
       <c r="A36" s="27" t="inlineStr">
         <is>
-          <t>SMCGLOBAL</t>
+          <t>SGFIN</t>
         </is>
       </c>
       <c r="B36" s="20">
@@ -32408,7 +32520,7 @@
     <row r="37">
       <c r="A37" s="27" t="inlineStr">
         <is>
-          <t>SPORTKING</t>
+          <t>SHRINGARMS</t>
         </is>
       </c>
       <c r="B37" s="20">
@@ -32451,7 +32563,7 @@
     <row r="38">
       <c r="A38" s="27" t="inlineStr">
         <is>
-          <t>SUNCLAY</t>
+          <t>SIMPLEXINF</t>
         </is>
       </c>
       <c r="B38" s="20">
@@ -32494,7 +32606,7 @@
     <row r="39">
       <c r="A39" s="27" t="inlineStr">
         <is>
-          <t>SWARAJENG</t>
+          <t>SMCGLOBAL</t>
         </is>
       </c>
       <c r="B39" s="20">
@@ -32537,7 +32649,7 @@
     <row r="40">
       <c r="A40" s="27" t="inlineStr">
         <is>
-          <t>TEAMLEASE</t>
+          <t>SOLARA</t>
         </is>
       </c>
       <c r="B40" s="20">
@@ -32580,7 +32692,7 @@
     <row r="41">
       <c r="A41" s="27" t="inlineStr">
         <is>
-          <t>YUKEN</t>
+          <t>SPORTKING</t>
         </is>
       </c>
       <c r="B41" s="20">
@@ -32621,37 +32733,209 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="3" t="inlineStr">
+      <c r="A42" s="27" t="inlineStr">
+        <is>
+          <t>SUNCLAY</t>
+        </is>
+      </c>
+      <c r="B42" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A42)</f>
+        <v/>
+      </c>
+      <c r="C42" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A42,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D42" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A42,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E42" s="22">
+        <f>IFERROR($C42/$B42,"")</f>
+        <v/>
+      </c>
+      <c r="F42" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A42,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G42" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A42,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H42" s="21">
+        <f>IFERROR($G42/$B42,"")</f>
+        <v/>
+      </c>
+      <c r="I42" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A42),"")</f>
+        <v/>
+      </c>
+      <c r="J42" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A42),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="27" t="inlineStr">
+        <is>
+          <t>SWARAJENG</t>
+        </is>
+      </c>
+      <c r="B43" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A43)</f>
+        <v/>
+      </c>
+      <c r="C43" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A43,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D43" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A43,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E43" s="22">
+        <f>IFERROR($C43/$B43,"")</f>
+        <v/>
+      </c>
+      <c r="F43" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A43,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G43" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A43,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H43" s="21">
+        <f>IFERROR($G43/$B43,"")</f>
+        <v/>
+      </c>
+      <c r="I43" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A43),"")</f>
+        <v/>
+      </c>
+      <c r="J43" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A43),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="27" t="inlineStr">
+        <is>
+          <t>TEAMLEASE</t>
+        </is>
+      </c>
+      <c r="B44" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A44)</f>
+        <v/>
+      </c>
+      <c r="C44" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A44,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D44" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A44,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E44" s="22">
+        <f>IFERROR($C44/$B44,"")</f>
+        <v/>
+      </c>
+      <c r="F44" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A44,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G44" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A44,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H44" s="21">
+        <f>IFERROR($G44/$B44,"")</f>
+        <v/>
+      </c>
+      <c r="I44" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A44),"")</f>
+        <v/>
+      </c>
+      <c r="J44" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A44),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="27" t="inlineStr">
+        <is>
+          <t>YUKEN</t>
+        </is>
+      </c>
+      <c r="B45" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A45)</f>
+        <v/>
+      </c>
+      <c r="C45" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A45,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D45" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A45,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E45" s="22">
+        <f>IFERROR($C45/$B45,"")</f>
+        <v/>
+      </c>
+      <c r="F45" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A45,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G45" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A45,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H45" s="21">
+        <f>IFERROR($G45/$B45,"")</f>
+        <v/>
+      </c>
+      <c r="I45" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A45),"")</f>
+        <v/>
+      </c>
+      <c r="J45" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A45),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B42" s="30">
-        <f>SUM(B4:B41)</f>
-        <v/>
-      </c>
-      <c r="C42" s="30">
-        <f>SUM(C4:C41)</f>
-        <v/>
-      </c>
-      <c r="D42" s="30">
-        <f>SUM(D4:D41)</f>
-        <v/>
-      </c>
-      <c r="E42" s="31">
-        <f>IFERROR(C42/B42,"")</f>
-        <v/>
-      </c>
-      <c r="F42" s="32">
-        <f>SUM(F4:F41)</f>
-        <v/>
-      </c>
-      <c r="G42" s="32">
-        <f>SUM(G4:G41)</f>
-        <v/>
-      </c>
-      <c r="H42" s="32">
-        <f>IFERROR(G42/B42,"")</f>
+      <c r="B46" s="30">
+        <f>SUM(B4:B45)</f>
+        <v/>
+      </c>
+      <c r="C46" s="30">
+        <f>SUM(C4:C45)</f>
+        <v/>
+      </c>
+      <c r="D46" s="30">
+        <f>SUM(D4:D45)</f>
+        <v/>
+      </c>
+      <c r="E46" s="31">
+        <f>IFERROR(C46/B46,"")</f>
+        <v/>
+      </c>
+      <c r="F46" s="32">
+        <f>SUM(F4:F45)</f>
+        <v/>
+      </c>
+      <c r="G46" s="32">
+        <f>SUM(G4:G45)</f>
+        <v/>
+      </c>
+      <c r="H46" s="32">
+        <f>IFERROR(G46/B46,"")</f>
         <v/>
       </c>
     </row>
@@ -32670,7 +32954,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N47"/>
+  <dimension ref="A1:N51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -32921,7 +33205,7 @@
         <v>35.4</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>125.76</v>
+        <v>120.95</v>
       </c>
       <c r="N6" s="21">
         <f>SUM(E6:M6)</f>
@@ -32972,7 +33256,7 @@
         <v>35.4</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>75.19</v>
+        <v>72.31999999999999</v>
       </c>
       <c r="N7" s="21">
         <f>SUM(E7:M7)</f>
@@ -33023,7 +33307,7 @@
         <v>35.4</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>75.34</v>
+        <v>100.64</v>
       </c>
       <c r="N8" s="21">
         <f>SUM(E8:M8)</f>
@@ -33074,7 +33358,7 @@
         <v>35.4</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>125.41</v>
+        <v>120.62</v>
       </c>
       <c r="N9" s="21">
         <f>SUM(E9:M9)</f>
@@ -33125,7 +33409,7 @@
         <v>35.4</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>104.65</v>
+        <v>100.65</v>
       </c>
       <c r="N10" s="21">
         <f>SUM(E10:M10)</f>
@@ -33176,7 +33460,7 @@
         <v>35.4</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>41.95</v>
+        <v>62.39</v>
       </c>
       <c r="N11" s="21">
         <f>SUM(E11:M11)</f>
@@ -33227,7 +33511,7 @@
         <v>35.4</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>50.27</v>
+        <v>74.78</v>
       </c>
       <c r="N12" s="21">
         <f>SUM(E12:M12)</f>
@@ -33278,7 +33562,7 @@
         <v>35.4</v>
       </c>
       <c r="M13" s="4" t="n">
-        <v>30.24</v>
+        <v>44.98</v>
       </c>
       <c r="N13" s="21">
         <f>SUM(E13:M13)</f>
@@ -33329,7 +33613,7 @@
         <v>35.4</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>30.11</v>
+        <v>44.78</v>
       </c>
       <c r="N14" s="21">
         <f>SUM(E14:M14)</f>
@@ -33482,7 +33766,7 @@
         <v>35.4</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>73.95999999999999</v>
+        <v>52.92</v>
       </c>
       <c r="N17" s="21">
         <f>SUM(E17:M17)</f>
@@ -33584,7 +33868,7 @@
         <v>35.4</v>
       </c>
       <c r="M19" s="4" t="n">
-        <v>127.52</v>
+        <v>91.29000000000001</v>
       </c>
       <c r="N19" s="21">
         <f>SUM(E19:M19)</f>
@@ -33635,7 +33919,7 @@
         <v>35.4</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>123.4</v>
+        <v>88.29000000000001</v>
       </c>
       <c r="N20" s="21">
         <f>SUM(E20:M20)</f>
@@ -33737,7 +34021,7 @@
         <v>35.4</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>123.99</v>
+        <v>88.70999999999999</v>
       </c>
       <c r="N22" s="21">
         <f>SUM(E22:M22)</f>
@@ -33788,7 +34072,7 @@
         <v>35.4</v>
       </c>
       <c r="M23" s="4" t="n">
-        <v>29.44</v>
+        <v>31.59</v>
       </c>
       <c r="N23" s="21">
         <f>SUM(E23:M23)</f>
@@ -33890,7 +34174,7 @@
         <v>35.4</v>
       </c>
       <c r="M25" s="4" t="n">
-        <v>36.53</v>
+        <v>39.2</v>
       </c>
       <c r="N25" s="21">
         <f>SUM(E25:M25)</f>
@@ -33941,7 +34225,7 @@
         <v>35.4</v>
       </c>
       <c r="M26" s="4" t="n">
-        <v>35.2</v>
+        <v>37.78</v>
       </c>
       <c r="N26" s="21">
         <f>SUM(E26:M26)</f>
@@ -33992,7 +34276,7 @@
         <v>35.4</v>
       </c>
       <c r="M27" s="4" t="n">
-        <v>40.31</v>
+        <v>43.26</v>
       </c>
       <c r="N27" s="21">
         <f>SUM(E27:M27)</f>
@@ -34043,7 +34327,7 @@
         <v>35.4</v>
       </c>
       <c r="M28" s="4" t="n">
-        <v>42.42</v>
+        <v>45.4</v>
       </c>
       <c r="N28" s="21">
         <f>SUM(E28:M28)</f>
@@ -34094,7 +34378,7 @@
         <v>35.4</v>
       </c>
       <c r="M29" s="4" t="n">
-        <v>35.17</v>
+        <v>37.74</v>
       </c>
       <c r="N29" s="21">
         <f>SUM(E29:M29)</f>
@@ -34196,7 +34480,7 @@
         <v>35.4</v>
       </c>
       <c r="M31" s="4" t="n">
-        <v>34.9</v>
+        <v>37.45</v>
       </c>
       <c r="N31" s="21">
         <f>SUM(E31:M31)</f>
@@ -34247,7 +34531,7 @@
         <v>35.4</v>
       </c>
       <c r="M32" s="4" t="n">
-        <v>37.12</v>
+        <v>39.81</v>
       </c>
       <c r="N32" s="21">
         <f>SUM(E32:M32)</f>
@@ -34349,7 +34633,7 @@
         <v>35.4</v>
       </c>
       <c r="M34" s="4" t="n">
-        <v>35.12</v>
+        <v>22.62</v>
       </c>
       <c r="N34" s="21">
         <f>SUM(E34:M34)</f>
@@ -34376,22 +34660,22 @@
         <v>46310</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>43.82</v>
+        <v>63.82</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>145.99</v>
+        <v>288.31</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>4.48</v>
+        <v>8.85</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>0.15</v>
+        <v>0.29</v>
       </c>
       <c r="I35" s="4" t="n">
         <v>21.9</v>
       </c>
       <c r="J35" s="4" t="n">
-        <v>8.720000000000001</v>
+        <v>13.13</v>
       </c>
       <c r="K35" s="4" t="n">
         <v>14.75</v>
@@ -34400,7 +34684,7 @@
         <v>35.4</v>
       </c>
       <c r="M35" s="4" t="n">
-        <v>31.42</v>
+        <v>33.7</v>
       </c>
       <c r="N35" s="21">
         <f>SUM(E35:M35)</f>
@@ -34427,22 +34711,22 @@
         <v>46310</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>60.01</v>
+        <v>80.01000000000001</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>200.1</v>
+        <v>399.82</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>6.14</v>
+        <v>12.27</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="I36" s="4" t="n">
         <v>30.02</v>
       </c>
       <c r="J36" s="4" t="n">
-        <v>11.94</v>
+        <v>16.68</v>
       </c>
       <c r="K36" s="4" t="n">
         <v>14.75</v>
@@ -34451,7 +34735,7 @@
         <v>35.4</v>
       </c>
       <c r="M36" s="4" t="n">
-        <v>34.22</v>
+        <v>36.72</v>
       </c>
       <c r="N36" s="21">
         <f>SUM(E36:M36)</f>
@@ -34478,22 +34762,22 @@
         <v>46310</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>59.64</v>
+        <v>79.64</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>198.83</v>
+        <v>390.96</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>6.1</v>
+        <v>12</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>0.2</v>
+        <v>0.39</v>
       </c>
       <c r="I37" s="4" t="n">
         <v>29.82</v>
       </c>
       <c r="J37" s="4" t="n">
-        <v>11.87</v>
+        <v>16.57</v>
       </c>
       <c r="K37" s="4" t="n">
         <v>14.75</v>
@@ -34502,7 +34786,7 @@
         <v>35.4</v>
       </c>
       <c r="M37" s="4" t="n">
-        <v>34</v>
+        <v>36.49</v>
       </c>
       <c r="N37" s="21">
         <f>SUM(E37:M37)</f>
@@ -34532,19 +34816,19 @@
         <v>0</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>99.63</v>
+        <v>201.6</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>3.06</v>
+        <v>6.19</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I38" s="4" t="n">
         <v>14.94</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>0.57</v>
+        <v>1.15</v>
       </c>
       <c r="K38" s="4" t="n">
         <v>14.75</v>
@@ -34580,22 +34864,22 @@
         <v>46310</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>60.05</v>
+        <v>80.05</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>200.11</v>
+        <v>400.91</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>6.14</v>
+        <v>12.31</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="I39" s="4" t="n">
         <v>30.09</v>
       </c>
       <c r="J39" s="4" t="n">
-        <v>11.95</v>
+        <v>16.7</v>
       </c>
       <c r="K39" s="4" t="n">
         <v>14.75</v>
@@ -34604,7 +34888,7 @@
         <v>35.4</v>
       </c>
       <c r="M39" s="4" t="n">
-        <v>34.22</v>
+        <v>36.73</v>
       </c>
       <c r="N39" s="21">
         <f>SUM(E39:M39)</f>
@@ -34614,12 +34898,12 @@
     <row r="40">
       <c r="A40" s="23" t="inlineStr">
         <is>
-          <t>DHAN-34126101377609+221261013593609+34126101378109+23126101376709+34126101378409+23126101377009+221261013595709+221261013596109+221261013596609+23126101377809+34126101379309+34126101379709+23126101378409+34126101379809+221261013599309+321261013576809</t>
+          <t>DHAN-321261015672409+231261015159509+341261015154309+321261015674209+231261015159809+321261015674909+341261015154809+221261015678909+321261015675709+221261015679609+231261015160509</t>
         </is>
       </c>
       <c r="B40" s="23" t="inlineStr">
         <is>
-          <t>INDOKEM</t>
+          <t>JAICORPLTD</t>
         </is>
       </c>
       <c r="C40" s="23" t="inlineStr">
@@ -34627,33 +34911,35 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D40" s="24" t="inlineStr"/>
+      <c r="D40" s="24" t="n">
+        <v>46311</v>
+      </c>
       <c r="E40" s="4" t="n">
-        <v>0</v>
+        <v>89.95</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>85.43000000000001</v>
+        <v>299.72</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>2.62</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>0.09</v>
+        <v>0.3</v>
       </c>
       <c r="I40" s="4" t="n">
-        <v>12.81</v>
+        <v>44.96</v>
       </c>
       <c r="J40" s="4" t="n">
-        <v>0.49</v>
+        <v>17.9</v>
       </c>
       <c r="K40" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L40" s="4" t="n">
-        <v>0</v>
+        <v>35.4</v>
       </c>
       <c r="M40" s="4" t="n">
-        <v>0</v>
+        <v>35.15</v>
       </c>
       <c r="N40" s="21">
         <f>SUM(E40:M40)</f>
@@ -34663,12 +34949,12 @@
     <row r="41">
       <c r="A41" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261015672409+231261015159509+341261015154309+321261015674209+231261015159809+321261015674909+341261015154809+221261015678909+321261015675709+221261015679609+231261015160509</t>
+          <t>DHAN-341261015154009+321261015672609+221261015677509+321261015674109+321261015674709+341261015154709+231261015160109+341261015154909+221261015679409+341261015155209+321261015676109</t>
         </is>
       </c>
       <c r="B41" s="23" t="inlineStr">
         <is>
-          <t>JAICORPLTD</t>
+          <t>OAL</t>
         </is>
       </c>
       <c r="C41" s="23" t="inlineStr">
@@ -34676,30 +34962,32 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D41" s="24" t="inlineStr"/>
+      <c r="D41" s="24" t="n">
+        <v>46311</v>
+      </c>
       <c r="E41" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>0</v>
+        <v>149.2</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>0</v>
+        <v>4.58</v>
       </c>
       <c r="H41" s="4" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="I41" s="4" t="n">
-        <v>0</v>
+        <v>22.38</v>
       </c>
       <c r="J41" s="4" t="n">
-        <v>0</v>
+        <v>0.85</v>
       </c>
       <c r="K41" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L41" s="4" t="n">
-        <v>35.4</v>
+        <v>0</v>
       </c>
       <c r="M41" s="4" t="n">
         <v>0</v>
@@ -34712,12 +35000,12 @@
     <row r="42">
       <c r="A42" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261012625809+321261012626209+23126101284209+23126101284309+321261012626909+34126101276209+34126101277109+321261012628809+221261012640809+23126101286309+34126101278009+321261012630809+221261012643209</t>
+          <t>DHAN-341261015153909+221261015677009+321261015673209+231261015159709+231261015159909+231261015160009+221261015678509+321261015675509+231261015160209+231261015160409+341261015155309</t>
         </is>
       </c>
       <c r="B42" s="23" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>ORIENTELEC</t>
         </is>
       </c>
       <c r="C42" s="23" t="inlineStr">
@@ -34725,33 +35013,35 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D42" s="24" t="inlineStr"/>
+      <c r="D42" s="24" t="n">
+        <v>46311</v>
+      </c>
       <c r="E42" s="4" t="n">
-        <v>24.76</v>
+        <v>90.56999999999999</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>3.4</v>
+        <v>301.73</v>
       </c>
       <c r="G42" s="4" t="n">
-        <v>2.63</v>
+        <v>9.26</v>
       </c>
       <c r="H42" s="4" t="n">
-        <v>0.09</v>
+        <v>0.3</v>
       </c>
       <c r="I42" s="4" t="n">
-        <v>3</v>
+        <v>44.93</v>
       </c>
       <c r="J42" s="4" t="n">
-        <v>4.95</v>
+        <v>18.02</v>
       </c>
       <c r="K42" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L42" s="4" t="n">
-        <v>0</v>
+        <v>35.4</v>
       </c>
       <c r="M42" s="4" t="n">
-        <v>0</v>
+        <v>37.17</v>
       </c>
       <c r="N42" s="21">
         <f>SUM(E42:M42)</f>
@@ -34761,12 +35051,12 @@
     <row r="43">
       <c r="A43" s="23" t="inlineStr">
         <is>
-          <t>DHAN-341261015154009+321261015672609+221261015677509+321261015674109+321261015674709+341261015154709+231261015160109+341261015154909+221261015679409+341261015155209+321261015676109</t>
+          <t>DHAN-231261015159409+321261015672709+321261015673309+221261015677909+221261015678309+341261015154609+321261015675209+221261015678809+341261015155009+341261015155109+231261015160609+231261015160709+341261015155509</t>
         </is>
       </c>
       <c r="B43" s="23" t="inlineStr">
         <is>
-          <t>OAL</t>
+          <t>TEAMLEASE</t>
         </is>
       </c>
       <c r="C43" s="23" t="inlineStr">
@@ -34774,33 +35064,35 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D43" s="24" t="inlineStr"/>
+      <c r="D43" s="24" t="n">
+        <v>46311</v>
+      </c>
       <c r="E43" s="4" t="n">
-        <v>0</v>
+        <v>89.45</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>0</v>
+        <v>298.18</v>
       </c>
       <c r="G43" s="4" t="n">
-        <v>0</v>
+        <v>9.15</v>
       </c>
       <c r="H43" s="4" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="I43" s="4" t="n">
-        <v>0</v>
+        <v>44.73</v>
       </c>
       <c r="J43" s="4" t="n">
-        <v>0</v>
+        <v>17.8</v>
       </c>
       <c r="K43" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L43" s="4" t="n">
-        <v>0</v>
+        <v>35.4</v>
       </c>
       <c r="M43" s="4" t="n">
-        <v>0</v>
+        <v>32.83</v>
       </c>
       <c r="N43" s="21">
         <f>SUM(E43:M43)</f>
@@ -34810,12 +35102,12 @@
     <row r="44">
       <c r="A44" s="23" t="inlineStr">
         <is>
-          <t>DHAN-341261015153909+221261015677009+321261015673209+231261015159709+231261015159909+231261015160009+221261015678509+321261015675509+231261015160209+231261015160409+341261015155309</t>
+          <t>DHAN-321261016683609+23126101679509+23126101679909+321261016685009+221261016694409+221261016695109+34126101677409+321261016686809+23126101680709+321261016687809+23126101681009+34126101678009</t>
         </is>
       </c>
       <c r="B44" s="23" t="inlineStr">
         <is>
-          <t>ORIENTELEC</t>
+          <t>EUROPRATIK</t>
         </is>
       </c>
       <c r="C44" s="23" t="inlineStr">
@@ -34859,12 +35151,12 @@
     <row r="45">
       <c r="A45" s="23" t="inlineStr">
         <is>
-          <t>DHAN-341261014128809+341261014129209+221261014671809+321261014664309+221261014672409+321261014664909+341261014130009+221261014673409+221261014673609+221261014673709+221261014674009+321261014667309+341261014130909</t>
+          <t>DHAN-34126101377609+221261013593609+34126101378109+23126101376709+34126101378409+23126101377009+221261013595709+221261013596109+221261013596609+23126101377809+34126101379309+34126101379709+23126101378409+34126101379809+221261013599309+321261013576809</t>
         </is>
       </c>
       <c r="B45" s="23" t="inlineStr">
         <is>
-          <t>SIMPLEXINF</t>
+          <t>INDOKEM</t>
         </is>
       </c>
       <c r="C45" s="23" t="inlineStr">
@@ -34874,31 +35166,31 @@
       </c>
       <c r="D45" s="24" t="inlineStr"/>
       <c r="E45" s="4" t="n">
-        <v>59.95</v>
+        <v>0</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>199.83</v>
+        <v>85.43000000000001</v>
       </c>
       <c r="G45" s="4" t="n">
-        <v>6.13</v>
+        <v>2.62</v>
       </c>
       <c r="H45" s="4" t="n">
-        <v>0.2</v>
+        <v>0.09</v>
       </c>
       <c r="I45" s="4" t="n">
-        <v>29.98</v>
+        <v>12.81</v>
       </c>
       <c r="J45" s="4" t="n">
-        <v>11.93</v>
+        <v>0.49</v>
       </c>
       <c r="K45" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L45" s="4" t="n">
-        <v>35.4</v>
+        <v>0</v>
       </c>
       <c r="M45" s="4" t="n">
-        <v>34.17</v>
+        <v>0</v>
       </c>
       <c r="N45" s="21">
         <f>SUM(E45:M45)</f>
@@ -34908,12 +35200,12 @@
     <row r="46">
       <c r="A46" s="23" t="inlineStr">
         <is>
-          <t>DHAN-231261015159409+321261015672709+321261015673309+221261015677909+221261015678309+341261015154609+321261015675209+221261015678809+341261015155009+341261015155109+231261015160609+231261015160709+341261015155509</t>
+          <t>DHAN-221261016693009+23126101679709+23126101679809+23126101680009+321261016685409+221261016694909+34126101677509+321261016686909+34126101677709+321261016687909+34126101677909</t>
         </is>
       </c>
       <c r="B46" s="23" t="inlineStr">
         <is>
-          <t>TEAMLEASE</t>
+          <t>MBEL</t>
         </is>
       </c>
       <c r="C46" s="23" t="inlineStr">
@@ -34955,54 +35247,250 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="3" t="inlineStr">
+      <c r="A47" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261012625809+321261012626209+23126101284209+23126101284309+321261012626909+34126101276209+34126101277109+321261012628809+221261012640809+23126101286309+34126101278009+321261012630809+221261012643209</t>
+        </is>
+      </c>
+      <c r="B47" s="23" t="inlineStr">
+        <is>
+          <t>MMWL</t>
+        </is>
+      </c>
+      <c r="C47" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D47" s="24" t="inlineStr"/>
+      <c r="E47" s="4" t="n">
+        <v>24.76</v>
+      </c>
+      <c r="F47" s="4" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="G47" s="4" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="H47" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="I47" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J47" s="4" t="n">
+        <v>4.95</v>
+      </c>
+      <c r="K47" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L47" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M47" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N47" s="21">
+        <f>SUM(E47:M47)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261016683509+23126101679609+221261016693309+321261016685109+321261016685509+321261016685809+221261016695509+34126101677609+23126101680609+23126101680809+321261016688709+321261016689109+221261016697009+321261016690409</t>
+        </is>
+      </c>
+      <c r="B48" s="23" t="inlineStr">
+        <is>
+          <t>PARACABLES</t>
+        </is>
+      </c>
+      <c r="C48" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D48" s="24" t="inlineStr"/>
+      <c r="E48" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J48" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K48" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L48" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M48" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N48" s="21">
+        <f>SUM(E48:M48)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-341261014128809+341261014129209+221261014671809+321261014664309+221261014672409+321261014664909+341261014130009+221261014673409+221261014673609+221261014673709+221261014674009+321261014667309+341261014130909</t>
+        </is>
+      </c>
+      <c r="B49" s="23" t="inlineStr">
+        <is>
+          <t>SIMPLEXINF</t>
+        </is>
+      </c>
+      <c r="C49" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D49" s="24" t="inlineStr"/>
+      <c r="E49" s="4" t="n">
+        <v>59.95</v>
+      </c>
+      <c r="F49" s="4" t="n">
+        <v>199.83</v>
+      </c>
+      <c r="G49" s="4" t="n">
+        <v>6.13</v>
+      </c>
+      <c r="H49" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I49" s="4" t="n">
+        <v>29.98</v>
+      </c>
+      <c r="J49" s="4" t="n">
+        <v>11.93</v>
+      </c>
+      <c r="K49" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L49" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M49" s="4" t="n">
+        <v>36.67</v>
+      </c>
+      <c r="N49" s="21">
+        <f>SUM(E49:M49)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261016692909+321261016684009+321261016684509+221261016693809+23126101680109+221261016695009+321261016686109+23126101680509+221261016696009+23126101680909+34126101677809+23126101681109</t>
+        </is>
+      </c>
+      <c r="B50" s="23" t="inlineStr">
+        <is>
+          <t>SOLARA</t>
+        </is>
+      </c>
+      <c r="C50" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D50" s="24" t="inlineStr"/>
+      <c r="E50" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I50" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J50" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K50" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L50" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M50" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N50" s="21">
+        <f>SUM(E50:M50)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E47" s="32">
-        <f>SUM(E4:E46)</f>
-        <v/>
-      </c>
-      <c r="F47" s="32">
-        <f>SUM(F4:F46)</f>
-        <v/>
-      </c>
-      <c r="G47" s="32">
-        <f>SUM(G4:G46)</f>
-        <v/>
-      </c>
-      <c r="H47" s="32">
-        <f>SUM(H4:H46)</f>
-        <v/>
-      </c>
-      <c r="I47" s="32">
-        <f>SUM(I4:I46)</f>
-        <v/>
-      </c>
-      <c r="J47" s="32">
-        <f>SUM(J4:J46)</f>
-        <v/>
-      </c>
-      <c r="K47" s="32">
-        <f>SUM(K4:K46)</f>
-        <v/>
-      </c>
-      <c r="L47" s="32">
-        <f>SUM(L4:L46)</f>
-        <v/>
-      </c>
-      <c r="M47" s="32">
-        <f>SUM(M4:M46)</f>
-        <v/>
-      </c>
-      <c r="N47" s="32">
-        <f>SUM(N4:N46)</f>
+      <c r="E51" s="32">
+        <f>SUM(E4:E50)</f>
+        <v/>
+      </c>
+      <c r="F51" s="32">
+        <f>SUM(F4:F50)</f>
+        <v/>
+      </c>
+      <c r="G51" s="32">
+        <f>SUM(G4:G50)</f>
+        <v/>
+      </c>
+      <c r="H51" s="32">
+        <f>SUM(H4:H50)</f>
+        <v/>
+      </c>
+      <c r="I51" s="32">
+        <f>SUM(I4:I50)</f>
+        <v/>
+      </c>
+      <c r="J51" s="32">
+        <f>SUM(J4:J50)</f>
+        <v/>
+      </c>
+      <c r="K51" s="32">
+        <f>SUM(K4:K50)</f>
+        <v/>
+      </c>
+      <c r="L51" s="32">
+        <f>SUM(L4:L50)</f>
+        <v/>
+      </c>
+      <c r="M51" s="32">
+        <f>SUM(M4:M50)</f>
+        <v/>
+      </c>
+      <c r="N51" s="32">
+        <f>SUM(N4:N50)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:N46"/>
+  <autoFilter ref="A3:N50"/>
   <mergeCells count="2">
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>

</xml_diff>

<commit_message>
Reconcile MMWL (10-12 entry), INDOKEM, and SIMPLEXINF stuck at status=open
Same recurring poll-timeout-then-late-fill bug as YUKEN/KOTIC/MMWL(10-09)/
SUNCLAY. INDOKEM and SIMPLEXINF were closed automatically via the new
--reconcile flag (dhan/run_trades.py, this same commit series). MMWL
(10-12 entry) needed a manual fix instead -- its lookup window overlapped
the already-fixed MMWL (10-09 entry)'s own sell trade, so --reconcile
correctly refused to guess (7331 sold vs 3742 expected) rather than compute
a wrong blended price:

- MMWL (entered 10-12): exited 10-13 09:17:55 @ 23.18, +1048.13
- INDOKEM (entered 10-13): exited 10-14 12:04:34 @ 654.81, -2919.65
- SIMPLEXINF (entered 10-14): exited 10-15 09:19:21 @ 265.57, -922.02

Workbooks regenerated via --sync-pnl to reflect the fix (also pushed to
Google Drive automatically, per the fold-in from the previous commit).
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_oct2026.xlsx
+++ b/results/strategy_pnl_oct2026.xlsx
@@ -1214,7 +1214,7 @@
         <v/>
       </c>
       <c r="K6" s="4" t="n">
-        <v>959.98</v>
+        <v>956.73</v>
       </c>
       <c r="L6" s="21">
         <f>IF(OR($B6="",$I6=""),"",$I6-IF($K6="",0,$K6))</f>
@@ -1274,7 +1274,7 @@
         <v/>
       </c>
       <c r="K7" s="4" t="n">
-        <v>822.01</v>
+        <v>820.0599999999999</v>
       </c>
       <c r="L7" s="21">
         <f>IF(OR($B7="",$I7=""),"",$I7-IF($K7="",0,$K7))</f>
@@ -1334,7 +1334,7 @@
         <v/>
       </c>
       <c r="K8" s="4" t="n">
-        <v>861.4</v>
+        <v>858.7</v>
       </c>
       <c r="L8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($K8="",0,$K8))</f>
@@ -1394,7 +1394,7 @@
         <v/>
       </c>
       <c r="K9" s="4" t="n">
-        <v>974.4299999999999</v>
+        <v>971.1900000000001</v>
       </c>
       <c r="L9" s="21">
         <f>IF(OR($B9="",$I9=""),"",$I9-IF($K9="",0,$K9))</f>
@@ -1454,7 +1454,7 @@
         <v/>
       </c>
       <c r="K10" s="4" t="n">
-        <v>947.17</v>
+        <v>944.47</v>
       </c>
       <c r="L10" s="21">
         <f>IF(OR($B10="",$I10=""),"",$I10-IF($K10="",0,$K10))</f>
@@ -1514,7 +1514,7 @@
         <v/>
       </c>
       <c r="K11" s="4" t="n">
-        <v>694.14</v>
+        <v>692.8099999999999</v>
       </c>
       <c r="L11" s="21">
         <f>IF(OR($B11="",$I11=""),"",$I11-IF($K11="",0,$K11))</f>
@@ -1574,7 +1574,7 @@
         <v/>
       </c>
       <c r="K12" s="4" t="n">
-        <v>759.8200000000001</v>
+        <v>758.24</v>
       </c>
       <c r="L12" s="21">
         <f>IF(OR($B12="",$I12=""),"",$I12-IF($K12="",0,$K12))</f>
@@ -1634,7 +1634,7 @@
         <v/>
       </c>
       <c r="K13" s="4" t="n">
-        <v>659.95</v>
+        <v>689.8</v>
       </c>
       <c r="L13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($K13="",0,$K13))</f>
@@ -1694,7 +1694,7 @@
         <v/>
       </c>
       <c r="K14" s="4" t="n">
-        <v>669.3200000000001</v>
+        <v>668.37</v>
       </c>
       <c r="L14" s="21">
         <f>IF(OR($B14="",$I14=""),"",$I14-IF($K14="",0,$K14))</f>
@@ -1874,7 +1874,7 @@
         <v/>
       </c>
       <c r="K17" s="4" t="n">
-        <v>630.54</v>
+        <v>629.97</v>
       </c>
       <c r="L17" s="21">
         <f>IF(OR($B17="",$I17=""),"",$I17-IF($K17="",0,$K17))</f>
@@ -1994,7 +1994,7 @@
         <v/>
       </c>
       <c r="K19" s="4" t="n">
-        <v>671.47</v>
+        <v>670.55</v>
       </c>
       <c r="L19" s="21">
         <f>IF(OR($B19="",$I19=""),"",$I19-IF($K19="",0,$K19))</f>
@@ -2054,7 +2054,7 @@
         <v/>
       </c>
       <c r="K20" s="4" t="n">
-        <v>681.75</v>
+        <v>680.79</v>
       </c>
       <c r="L20" s="21">
         <f>IF(OR($B20="",$I20=""),"",$I20-IF($K20="",0,$K20))</f>
@@ -2174,7 +2174,7 @@
         <v/>
       </c>
       <c r="K22" s="4" t="n">
-        <v>663.37</v>
+        <v>662.41</v>
       </c>
       <c r="L22" s="21">
         <f>IF(OR($B22="",$I22=""),"",$I22-IF($K22="",0,$K22))</f>
@@ -2234,7 +2234,7 @@
         <v/>
       </c>
       <c r="K23" s="4" t="n">
-        <v>421.4</v>
+        <v>421.06</v>
       </c>
       <c r="L23" s="21">
         <f>IF(OR($B23="",$I23=""),"",$I23-IF($K23="",0,$K23))</f>
@@ -2354,7 +2354,7 @@
         <v/>
       </c>
       <c r="K25" s="4" t="n">
-        <v>559.4</v>
+        <v>558.99</v>
       </c>
       <c r="L25" s="21">
         <f>IF(OR($B25="",$I25=""),"",$I25-IF($K25="",0,$K25))</f>
@@ -2377,12 +2377,12 @@
     <row r="26">
       <c r="A26" s="23" t="inlineStr">
         <is>
-          <t>DHAN-34126101275609+321261012626309+221261012637809+34126101275809+23126101284509+321261012627209+34126101277009+34126101277209+34126101277609+221261012641209+321261012630309+23126101287209+321261012631409+321261012631709+321261012632009</t>
+          <t>DHAN-321261012625809+321261012626209+23126101284209+23126101284309+321261012626909+34126101276209+34126101277109+321261012628809+221261012640809+23126101286309+34126101278009+321261012630809+221261012643209</t>
         </is>
       </c>
       <c r="B26" s="23" t="inlineStr">
         <is>
-          <t>PRINCEPIPE</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="C26" s="23" t="inlineStr">
@@ -2394,16 +2394,16 @@
         <v>46307</v>
       </c>
       <c r="E26" s="25" t="n">
-        <v>267.6149</v>
+        <v>22.8999</v>
       </c>
       <c r="F26" s="26" t="n">
-        <v>641</v>
+        <v>3742</v>
       </c>
       <c r="G26" s="24" t="n">
         <v>46308</v>
       </c>
       <c r="H26" s="25" t="n">
-        <v>262</v>
+        <v>23.18</v>
       </c>
       <c r="I26" s="21">
         <f>IF(OR($B26="",$H26=""),"",IF($C26="LONG",($H26-$E26)*$F26,($E26-$H26)*$F26))</f>
@@ -2414,7 +2414,7 @@
         <v/>
       </c>
       <c r="K26" s="4" t="n">
-        <v>549.67</v>
+        <v>143.56</v>
       </c>
       <c r="L26" s="21">
         <f>IF(OR($B26="",$I26=""),"",$I26-IF($K26="",0,$K26))</f>
@@ -2437,12 +2437,12 @@
     <row r="27">
       <c r="A27" s="23" t="inlineStr">
         <is>
-          <t>DHAN-23126101283509+23126101284109+34126101275709+221261012638509+34126101275909+23126101284809+321261012628509+321261012628709+23126101286109+321261012629509+221261012641909+221261012642709+23126101287309+221261012643409+34126101278409</t>
+          <t>DHAN-34126101275609+321261012626309+221261012637809+34126101275809+23126101284509+321261012627209+34126101277009+34126101277209+34126101277609+221261012641209+321261012630309+23126101287209+321261012631409+321261012631709+321261012632009</t>
         </is>
       </c>
       <c r="B27" s="23" t="inlineStr">
         <is>
-          <t>SWARAJENG</t>
+          <t>PRINCEPIPE</t>
         </is>
       </c>
       <c r="C27" s="23" t="inlineStr">
@@ -2454,16 +2454,16 @@
         <v>46307</v>
       </c>
       <c r="E27" s="25" t="n">
-        <v>3741.3844</v>
+        <v>267.6149</v>
       </c>
       <c r="F27" s="26" t="n">
-        <v>45</v>
+        <v>641</v>
       </c>
       <c r="G27" s="24" t="n">
         <v>46308</v>
       </c>
       <c r="H27" s="25" t="n">
-        <v>3721.09</v>
+        <v>262</v>
       </c>
       <c r="I27" s="21">
         <f>IF(OR($B27="",$H27=""),"",IF($C27="LONG",($H27-$E27)*$F27,($E27-$H27)*$F27))</f>
@@ -2474,7 +2474,7 @@
         <v/>
       </c>
       <c r="K27" s="4" t="n">
-        <v>550.23</v>
+        <v>549.26</v>
       </c>
       <c r="L27" s="21">
         <f>IF(OR($B27="",$I27=""),"",$I27-IF($K27="",0,$K27))</f>
@@ -2497,12 +2497,12 @@
     <row r="28">
       <c r="A28" s="23" t="inlineStr">
         <is>
-          <t>DHAN-34126101377709+221261013593709+321261013572009+23126101376509+221261013594809+34126101378609+221261013595609+23126101377609+321261013574409+321261013575009+23126101378109+23126101378209</t>
+          <t>DHAN-23126101283509+23126101284109+34126101275709+221261012638509+34126101275909+23126101284809+321261012628509+321261012628709+23126101286109+321261012629509+221261012641909+221261012642709+23126101287309+221261012643409+34126101278409</t>
         </is>
       </c>
       <c r="B28" s="23" t="inlineStr">
         <is>
-          <t>CMLL</t>
+          <t>SWARAJENG</t>
         </is>
       </c>
       <c r="C28" s="23" t="inlineStr">
@@ -2511,19 +2511,19 @@
         </is>
       </c>
       <c r="D28" s="24" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E28" s="25" t="n">
+        <v>3741.3844</v>
+      </c>
+      <c r="F28" s="26" t="n">
+        <v>45</v>
+      </c>
+      <c r="G28" s="24" t="n">
         <v>46308</v>
       </c>
-      <c r="E28" s="25" t="n">
-        <v>617.1578</v>
-      </c>
-      <c r="F28" s="26" t="n">
-        <v>277</v>
-      </c>
-      <c r="G28" s="24" t="n">
-        <v>46309</v>
-      </c>
       <c r="H28" s="25" t="n">
-        <v>608.04</v>
+        <v>3721.09</v>
       </c>
       <c r="I28" s="21">
         <f>IF(OR($B28="",$H28=""),"",IF($C28="LONG",($H28-$E28)*$F28,($E28-$H28)*$F28))</f>
@@ -2534,7 +2534,7 @@
         <v/>
       </c>
       <c r="K28" s="4" t="n">
-        <v>557.4</v>
+        <v>549.76</v>
       </c>
       <c r="L28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($K28="",0,$K28))</f>
@@ -2550,19 +2550,19 @@
       </c>
       <c r="O28" s="23" t="inlineStr">
         <is>
-          <t>10-15</t>
+          <t>5-10</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261013592809+34126101377809+321261013572109+23126101376309+34126101378309+321261013573109+34126101378709+221261013596309+23126101377709+221261013597309+321261013575409+321261013575609</t>
+          <t>DHAN-34126101377709+221261013593709+321261013572009+23126101376509+221261013594809+34126101378609+221261013595609+23126101377609+321261013574409+321261013575009+23126101378109+23126101378209</t>
         </is>
       </c>
       <c r="B29" s="23" t="inlineStr">
         <is>
-          <t>HATHWAY</t>
+          <t>CMLL</t>
         </is>
       </c>
       <c r="C29" s="23" t="inlineStr">
@@ -2574,16 +2574,16 @@
         <v>46308</v>
       </c>
       <c r="E29" s="25" t="n">
-        <v>11.158</v>
+        <v>617.1578</v>
       </c>
       <c r="F29" s="26" t="n">
-        <v>15360</v>
+        <v>277</v>
       </c>
       <c r="G29" s="24" t="n">
         <v>46309</v>
       </c>
       <c r="H29" s="25" t="n">
-        <v>11.14</v>
+        <v>608.04</v>
       </c>
       <c r="I29" s="21">
         <f>IF(OR($B29="",$H29=""),"",IF($C29="LONG",($H29-$E29)*$F29,($E29-$H29)*$F29))</f>
@@ -2594,7 +2594,7 @@
         <v/>
       </c>
       <c r="K29" s="4" t="n">
-        <v>552.79</v>
+        <v>556.86</v>
       </c>
       <c r="L29" s="21">
         <f>IF(OR($B29="",$I29=""),"",$I29-IF($K29="",0,$K29))</f>
@@ -2617,12 +2617,12 @@
     <row r="30">
       <c r="A30" s="23" t="inlineStr">
         <is>
-          <t>DHAN-23126101375909+221261013593509+221261013594309+34126101378209+321261013572509+23126101377109+321261013573709+23126101377509+34126101379009+321261013575109+221261013597709+221261013598409+34126101379609</t>
+          <t>DHAN-221261013592809+34126101377809+321261013572109+23126101376309+34126101378309+321261013573109+34126101378709+221261013596309+23126101377709+221261013597309+321261013575409+321261013575609</t>
         </is>
       </c>
       <c r="B30" s="23" t="inlineStr">
         <is>
-          <t>INDIAGLYCO</t>
+          <t>HATHWAY</t>
         </is>
       </c>
       <c r="C30" s="23" t="inlineStr">
@@ -2634,16 +2634,16 @@
         <v>46308</v>
       </c>
       <c r="E30" s="25" t="n">
-        <v>352.906</v>
+        <v>11.158</v>
       </c>
       <c r="F30" s="26" t="n">
-        <v>243</v>
+        <v>15360</v>
       </c>
       <c r="G30" s="24" t="n">
         <v>46309</v>
       </c>
       <c r="H30" s="25" t="n">
-        <v>358.7</v>
+        <v>11.14</v>
       </c>
       <c r="I30" s="21">
         <f>IF(OR($B30="",$H30=""),"",IF($C30="LONG",($H30-$E30)*$F30,($E30-$H30)*$F30))</f>
@@ -2654,7 +2654,7 @@
         <v/>
       </c>
       <c r="K30" s="4" t="n">
-        <v>207</v>
+        <v>552.38</v>
       </c>
       <c r="L30" s="21">
         <f>IF(OR($B30="",$I30=""),"",$I30-IF($K30="",0,$K30))</f>
@@ -2670,19 +2670,19 @@
       </c>
       <c r="O30" s="23" t="inlineStr">
         <is>
-          <t>5-10</t>
+          <t>10-15</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261013593009+23126101376209+34126101378009+221261013594409+23126101376909+23126101377209+23126101377309+321261013574209+321261013574509+23126101377909+34126101379509+321261013575709</t>
+          <t>DHAN-23126101375909+221261013593509+221261013594309+34126101378209+321261013572509+23126101377109+321261013573709+23126101377509+34126101379009+321261013575109+221261013597709+221261013598409+34126101379609</t>
         </is>
       </c>
       <c r="B31" s="23" t="inlineStr">
         <is>
-          <t>PIXTRANS</t>
+          <t>INDIAGLYCO</t>
         </is>
       </c>
       <c r="C31" s="23" t="inlineStr">
@@ -2694,16 +2694,16 @@
         <v>46308</v>
       </c>
       <c r="E31" s="25" t="n">
-        <v>1889.5856</v>
+        <v>352.906</v>
       </c>
       <c r="F31" s="26" t="n">
-        <v>90</v>
+        <v>243</v>
       </c>
       <c r="G31" s="24" t="n">
         <v>46309</v>
       </c>
       <c r="H31" s="25" t="n">
-        <v>1923.39</v>
+        <v>358.7</v>
       </c>
       <c r="I31" s="21">
         <f>IF(OR($B31="",$H31=""),"",IF($C31="LONG",($H31-$E31)*$F31,($E31-$H31)*$F31))</f>
@@ -2714,7 +2714,7 @@
         <v/>
       </c>
       <c r="K31" s="4" t="n">
-        <v>552.91</v>
+        <v>207</v>
       </c>
       <c r="L31" s="21">
         <f>IF(OR($B31="",$I31=""),"",$I31-IF($K31="",0,$K31))</f>
@@ -2737,12 +2737,12 @@
     <row r="32">
       <c r="A32" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261013571309+221261013593809+221261013594209+23126101376409+34126101378509+321261013573309+34126101378809+34126101378909+221261013596709+221261013597209+34126101379409+23126101378309+321261013576009</t>
+          <t>DHAN-34126101377609+221261013593609+34126101378109+23126101376709+34126101378409+23126101377009+221261013595709+221261013596109+221261013596609+23126101377809+34126101379309+34126101379709+23126101378409+34126101379809+221261013599309+321261013576809</t>
         </is>
       </c>
       <c r="B32" s="23" t="inlineStr">
         <is>
-          <t>PNCINFRA</t>
+          <t>INDOKEM</t>
         </is>
       </c>
       <c r="C32" s="23" t="inlineStr">
@@ -2754,16 +2754,16 @@
         <v>46308</v>
       </c>
       <c r="E32" s="25" t="n">
-        <v>156.7238</v>
+        <v>677.9853000000001</v>
       </c>
       <c r="F32" s="26" t="n">
-        <v>1086</v>
+        <v>126</v>
       </c>
       <c r="G32" s="24" t="n">
         <v>46309</v>
       </c>
       <c r="H32" s="25" t="n">
-        <v>169.79</v>
+        <v>654.8135</v>
       </c>
       <c r="I32" s="21">
         <f>IF(OR($B32="",$H32=""),"",IF($C32="LONG",($H32-$E32)*$F32,($E32-$H32)*$F32))</f>
@@ -2774,7 +2774,7 @@
         <v/>
       </c>
       <c r="K32" s="4" t="n">
-        <v>428.12</v>
+        <v>116.19</v>
       </c>
       <c r="L32" s="21">
         <f>IF(OR($B32="",$I32=""),"",$I32-IF($K32="",0,$K32))</f>
@@ -2797,33 +2797,33 @@
     <row r="33">
       <c r="A33" s="23" t="inlineStr">
         <is>
-          <t>DHAN-34126101478009</t>
+          <t>DHAN-221261013593009+23126101376209+34126101378009+221261013594409+23126101376909+23126101377209+23126101377309+321261013574209+321261013574509+23126101377909+34126101379509+321261013575709</t>
         </is>
       </c>
       <c r="B33" s="23" t="inlineStr">
         <is>
-          <t>PNCINFRA</t>
+          <t>PIXTRANS</t>
         </is>
       </c>
       <c r="C33" s="23" t="inlineStr">
         <is>
-          <t>SHORT</t>
+          <t>LONG</t>
         </is>
       </c>
       <c r="D33" s="24" t="n">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="E33" s="25" t="n">
-        <v>169.61</v>
+        <v>1889.5856</v>
       </c>
       <c r="F33" s="26" t="n">
-        <v>1086</v>
+        <v>90</v>
       </c>
       <c r="G33" s="24" t="n">
         <v>46309</v>
       </c>
       <c r="H33" s="25" t="n">
-        <v>161.13</v>
+        <v>1923.39</v>
       </c>
       <c r="I33" s="21">
         <f>IF(OR($B33="",$H33=""),"",IF($C33="LONG",($H33-$E33)*$F33,($E33-$H33)*$F33))</f>
@@ -2834,7 +2834,7 @@
         <v/>
       </c>
       <c r="K33" s="4" t="n">
-        <v>223.78</v>
+        <v>552.51</v>
       </c>
       <c r="L33" s="21">
         <f>IF(OR($B33="",$I33=""),"",$I33-IF($K33="",0,$K33))</f>
@@ -2850,19 +2850,19 @@
       </c>
       <c r="O33" s="23" t="inlineStr">
         <is>
-          <t>10-15</t>
+          <t>5-10</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261013592909+23126101376109+321261013572209+23126101376609+321261013572609+321261013573209+321261013573809+221261013596209+34126101379109+34126101379209+221261013597909</t>
+          <t>DHAN-321261013571309+221261013593809+221261013594209+23126101376409+34126101378509+321261013573309+34126101378809+34126101378909+221261013596709+221261013597209+34126101379409+23126101378309+321261013576009</t>
         </is>
       </c>
       <c r="B34" s="23" t="inlineStr">
         <is>
-          <t>SHRINGARMS</t>
+          <t>PNCINFRA</t>
         </is>
       </c>
       <c r="C34" s="23" t="inlineStr">
@@ -2874,16 +2874,16 @@
         <v>46308</v>
       </c>
       <c r="E34" s="25" t="n">
-        <v>311.7565</v>
+        <v>156.7238</v>
       </c>
       <c r="F34" s="26" t="n">
-        <v>549</v>
+        <v>1086</v>
       </c>
       <c r="G34" s="24" t="n">
         <v>46309</v>
       </c>
       <c r="H34" s="25" t="n">
-        <v>315.82</v>
+        <v>169.79</v>
       </c>
       <c r="I34" s="21">
         <f>IF(OR($B34="",$H34=""),"",IF($C34="LONG",($H34-$E34)*$F34,($E34-$H34)*$F34))</f>
@@ -2894,7 +2894,7 @@
         <v/>
       </c>
       <c r="K34" s="4" t="n">
-        <v>540.04</v>
+        <v>427.71</v>
       </c>
       <c r="L34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($K34="",0,$K34))</f>
@@ -2910,40 +2910,40 @@
       </c>
       <c r="O34" s="23" t="inlineStr">
         <is>
-          <t>15-20</t>
+          <t>10-15</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261014662909+221261014671509+321261014664009+341261014129509+341261014129709+321261014665509+221261014673509+231261014126609+221261014673809+221261014674109+231261014126809+341261014131109+221261014675709+231261014127209+341261014131309+231261014127309</t>
+          <t>DHAN-34126101478009</t>
         </is>
       </c>
       <c r="B35" s="23" t="inlineStr">
         <is>
-          <t>JINDALPOLY</t>
+          <t>PNCINFRA</t>
         </is>
       </c>
       <c r="C35" s="23" t="inlineStr">
         <is>
-          <t>LONG</t>
+          <t>SHORT</t>
         </is>
       </c>
       <c r="D35" s="24" t="n">
         <v>46309</v>
       </c>
       <c r="E35" s="25" t="n">
-        <v>726.3234</v>
+        <v>169.61</v>
       </c>
       <c r="F35" s="26" t="n">
-        <v>201</v>
+        <v>1086</v>
       </c>
       <c r="G35" s="24" t="n">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="H35" s="25" t="n">
-        <v>708.0599999999999</v>
+        <v>161.13</v>
       </c>
       <c r="I35" s="21">
         <f>IF(OR($B35="",$H35=""),"",IF($C35="LONG",($H35-$E35)*$F35,($E35-$H35)*$F35))</f>
@@ -2954,7 +2954,7 @@
         <v/>
       </c>
       <c r="K35" s="4" t="n">
-        <v>480.15</v>
+        <v>223.78</v>
       </c>
       <c r="L35" s="21">
         <f>IF(OR($B35="",$I35=""),"",$I35-IF($K35="",0,$K35))</f>
@@ -2977,12 +2977,12 @@
     <row r="36">
       <c r="A36" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261014663009+221261014671609+341261014129309+221261014671909+341261014129609+341261014129809+231261014126309+321261014666109+231261014126509+341261014130409+231261014126709+231261014126909</t>
+          <t>DHAN-221261013592909+23126101376109+321261013572209+23126101376609+321261013572609+321261013573209+321261013573809+221261013596209+34126101379109+34126101379209+221261013597909</t>
         </is>
       </c>
       <c r="B36" s="23" t="inlineStr">
         <is>
-          <t>KROSS</t>
+          <t>SHRINGARMS</t>
         </is>
       </c>
       <c r="C36" s="23" t="inlineStr">
@@ -2991,19 +2991,19 @@
         </is>
       </c>
       <c r="D36" s="24" t="n">
+        <v>46308</v>
+      </c>
+      <c r="E36" s="25" t="n">
+        <v>311.7565</v>
+      </c>
+      <c r="F36" s="26" t="n">
+        <v>549</v>
+      </c>
+      <c r="G36" s="24" t="n">
         <v>46309</v>
       </c>
-      <c r="E36" s="25" t="n">
-        <v>271.509</v>
-      </c>
-      <c r="F36" s="26" t="n">
-        <v>737</v>
-      </c>
-      <c r="G36" s="24" t="n">
-        <v>46310</v>
-      </c>
       <c r="H36" s="25" t="n">
-        <v>270.99</v>
+        <v>315.82</v>
       </c>
       <c r="I36" s="21">
         <f>IF(OR($B36="",$H36=""),"",IF($C36="LONG",($H36-$E36)*$F36,($E36-$H36)*$F36))</f>
@@ -3014,7 +3014,7 @@
         <v/>
       </c>
       <c r="K36" s="4" t="n">
-        <v>626.08</v>
+        <v>539.8</v>
       </c>
       <c r="L36" s="21">
         <f>IF(OR($B36="",$I36=""),"",$I36-IF($K36="",0,$K36))</f>
@@ -3030,19 +3030,19 @@
       </c>
       <c r="O36" s="23" t="inlineStr">
         <is>
-          <t>10-15</t>
+          <t>15-20</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="23" t="inlineStr">
         <is>
-          <t>DHAN-341261014128909+341261014129109+231261014125709+321261014664109+321261014664809+231261014126009+321261014665609+231261014126409+341261014130309+341261014130509+221261014673909+341261014130709+221261014674609+221261014675009+221261014675509</t>
+          <t>DHAN-321261014662909+221261014671509+321261014664009+341261014129509+341261014129709+321261014665509+221261014673509+231261014126609+221261014673809+221261014674109+231261014126809+341261014131109+221261014675709+231261014127209+341261014131309+231261014127309</t>
         </is>
       </c>
       <c r="B37" s="23" t="inlineStr">
         <is>
-          <t>NIBE</t>
+          <t>JINDALPOLY</t>
         </is>
       </c>
       <c r="C37" s="23" t="inlineStr">
@@ -3054,16 +3054,16 @@
         <v>46309</v>
       </c>
       <c r="E37" s="25" t="n">
-        <v>1380.7368</v>
+        <v>726.3234</v>
       </c>
       <c r="F37" s="26" t="n">
-        <v>144</v>
+        <v>201</v>
       </c>
       <c r="G37" s="24" t="n">
         <v>46310</v>
       </c>
       <c r="H37" s="25" t="n">
-        <v>1334.24</v>
+        <v>708.0599999999999</v>
       </c>
       <c r="I37" s="21">
         <f>IF(OR($B37="",$H37=""),"",IF($C37="LONG",($H37-$E37)*$F37,($E37-$H37)*$F37))</f>
@@ -3074,7 +3074,7 @@
         <v/>
       </c>
       <c r="K37" s="4" t="n">
-        <v>616.02</v>
+        <v>479.82</v>
       </c>
       <c r="L37" s="21">
         <f>IF(OR($B37="",$I37=""),"",$I37-IF($K37="",0,$K37))</f>
@@ -3097,12 +3097,12 @@
     <row r="38">
       <c r="A38" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261014671209+321261014663609+231261014125809+221261014672009+231261014125909+231261014126109+221261014673109+341261014130209+321261014666509+341261014130609+321261014667409+321261014667809+341261014131209+221261014676209+221261014676809</t>
+          <t>DHAN-321261014663009+221261014671609+341261014129309+221261014671909+341261014129609+341261014129809+231261014126309+321261014666109+231261014126509+341261014130409+231261014126709+231261014126909</t>
         </is>
       </c>
       <c r="B38" s="23" t="inlineStr">
         <is>
-          <t>RUBYMILLS</t>
+          <t>KROSS</t>
         </is>
       </c>
       <c r="C38" s="23" t="inlineStr">
@@ -3114,16 +3114,16 @@
         <v>46309</v>
       </c>
       <c r="E38" s="25" t="n">
-        <v>541.4497</v>
+        <v>271.509</v>
       </c>
       <c r="F38" s="26" t="n">
-        <v>184</v>
+        <v>737</v>
       </c>
       <c r="G38" s="24" t="n">
         <v>46310</v>
       </c>
       <c r="H38" s="25" t="n">
-        <v>554.2</v>
+        <v>270.99</v>
       </c>
       <c r="I38" s="21">
         <f>IF(OR($B38="",$H38=""),"",IF($C38="LONG",($H38-$E38)*$F38,($E38-$H38)*$F38))</f>
@@ -3134,7 +3134,7 @@
         <v/>
       </c>
       <c r="K38" s="4" t="n">
-        <v>238.83</v>
+        <v>625.6799999999999</v>
       </c>
       <c r="L38" s="21">
         <f>IF(OR($B38="",$I38=""),"",$I38-IF($K38="",0,$K38))</f>
@@ -3150,19 +3150,19 @@
       </c>
       <c r="O38" s="23" t="inlineStr">
         <is>
-          <t>5-10</t>
+          <t>10-15</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="23" t="inlineStr">
         <is>
-          <t>DHAN-231261014125609+321261014663509+321261014663909+321261014664209+221261014672509+231261014126209+341261014130109+321261014666209+321261014666609+321261014666709+321261014667009+341261014130809+231261014127009+341261014131009+221261014675609</t>
+          <t>DHAN-341261014128909+341261014129109+231261014125709+321261014664109+321261014664809+231261014126009+321261014665609+231261014126409+341261014130309+341261014130509+221261014673909+341261014130709+221261014674609+221261014675009+221261014675509</t>
         </is>
       </c>
       <c r="B39" s="23" t="inlineStr">
         <is>
-          <t>SPORTKING</t>
+          <t>NIBE</t>
         </is>
       </c>
       <c r="C39" s="23" t="inlineStr">
@@ -3174,16 +3174,16 @@
         <v>46309</v>
       </c>
       <c r="E39" s="25" t="n">
-        <v>226.1107</v>
+        <v>1380.7368</v>
       </c>
       <c r="F39" s="26" t="n">
-        <v>885</v>
+        <v>144</v>
       </c>
       <c r="G39" s="24" t="n">
         <v>46310</v>
       </c>
       <c r="H39" s="25" t="n">
-        <v>226.89</v>
+        <v>1334.24</v>
       </c>
       <c r="I39" s="21">
         <f>IF(OR($B39="",$H39=""),"",IF($C39="LONG",($H39-$E39)*$F39,($E39-$H39)*$F39))</f>
@@ -3194,7 +3194,7 @@
         <v/>
       </c>
       <c r="K39" s="4" t="n">
-        <v>627.33</v>
+        <v>615.62</v>
       </c>
       <c r="L39" s="21">
         <f>IF(OR($B39="",$I39=""),"",$I39-IF($K39="",0,$K39))</f>
@@ -3210,19 +3210,19 @@
       </c>
       <c r="O39" s="23" t="inlineStr">
         <is>
-          <t>5-10</t>
+          <t>10-15</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261015672409+231261015159509+341261015154309+321261015674209+231261015159809+321261015674909+341261015154809+221261015678909+321261015675709+221261015679609+231261015160509</t>
+          <t>DHAN-221261014671209+321261014663609+231261014125809+221261014672009+231261014125909+231261014126109+221261014673109+341261014130209+321261014666509+341261014130609+321261014667409+321261014667809+341261014131209+221261014676209+221261014676809</t>
         </is>
       </c>
       <c r="B40" s="23" t="inlineStr">
         <is>
-          <t>JAICORPLTD</t>
+          <t>RUBYMILLS</t>
         </is>
       </c>
       <c r="C40" s="23" t="inlineStr">
@@ -3231,19 +3231,19 @@
         </is>
       </c>
       <c r="D40" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E40" s="25" t="n">
+        <v>541.4497</v>
+      </c>
+      <c r="F40" s="26" t="n">
+        <v>184</v>
+      </c>
+      <c r="G40" s="24" t="n">
         <v>46310</v>
       </c>
-      <c r="E40" s="25" t="n">
-        <v>95.05800000000001</v>
-      </c>
-      <c r="F40" s="26" t="n">
-        <v>3153</v>
-      </c>
-      <c r="G40" s="24" t="n">
-        <v>46311</v>
-      </c>
       <c r="H40" s="25" t="n">
-        <v>94.26000000000001</v>
+        <v>554.2</v>
       </c>
       <c r="I40" s="21">
         <f>IF(OR($B40="",$H40=""),"",IF($C40="LONG",($H40-$E40)*$F40,($E40-$H40)*$F40))</f>
@@ -3254,7 +3254,7 @@
         <v/>
       </c>
       <c r="K40" s="4" t="n">
-        <v>547.34</v>
+        <v>238.83</v>
       </c>
       <c r="L40" s="21">
         <f>IF(OR($B40="",$I40=""),"",$I40-IF($K40="",0,$K40))</f>
@@ -3277,12 +3277,12 @@
     <row r="41">
       <c r="A41" s="23" t="inlineStr">
         <is>
-          <t>DHAN-341261015154009+321261015672609+221261015677509+321261015674109+321261015674709+341261015154709+231261015160109+341261015154909+221261015679409+341261015155209+321261015676109</t>
+          <t>DHAN-341261014128809+341261014129209+221261014671809+321261014664309+221261014672409+321261014664909+341261014130009+221261014673409+221261014673609+221261014673709+221261014674009+321261014667309+341261014130909</t>
         </is>
       </c>
       <c r="B41" s="23" t="inlineStr">
         <is>
-          <t>OAL</t>
+          <t>SIMPLEXINF</t>
         </is>
       </c>
       <c r="C41" s="23" t="inlineStr">
@@ -3291,19 +3291,19 @@
         </is>
       </c>
       <c r="D41" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E41" s="25" t="n">
+        <v>266.801</v>
+      </c>
+      <c r="F41" s="26" t="n">
+        <v>749</v>
+      </c>
+      <c r="G41" s="24" t="n">
         <v>46310</v>
       </c>
-      <c r="E41" s="25" t="n">
-        <v>578.2952</v>
-      </c>
-      <c r="F41" s="26" t="n">
-        <v>258</v>
-      </c>
-      <c r="G41" s="24" t="n">
-        <v>46311</v>
-      </c>
       <c r="H41" s="25" t="n">
-        <v>585.09</v>
+        <v>265.57</v>
       </c>
       <c r="I41" s="21">
         <f>IF(OR($B41="",$H41=""),"",IF($C41="LONG",($H41-$E41)*$F41,($E41-$H41)*$F41))</f>
@@ -3314,7 +3314,7 @@
         <v/>
       </c>
       <c r="K41" s="4" t="n">
-        <v>191.91</v>
+        <v>394.45</v>
       </c>
       <c r="L41" s="21">
         <f>IF(OR($B41="",$I41=""),"",$I41-IF($K41="",0,$K41))</f>
@@ -3330,19 +3330,19 @@
       </c>
       <c r="O41" s="23" t="inlineStr">
         <is>
-          <t>10-15</t>
+          <t>5-10</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="23" t="inlineStr">
         <is>
-          <t>DHAN-341261015153909+221261015677009+321261015673209+231261015159709+231261015159909+231261015160009+221261015678509+321261015675509+231261015160209+231261015160409+341261015155309</t>
+          <t>DHAN-231261014125609+321261014663509+321261014663909+321261014664209+221261014672509+231261014126209+341261014130109+321261014666209+321261014666609+321261014666709+321261014667009+341261014130809+231261014127009+341261014131009+221261014675609</t>
         </is>
       </c>
       <c r="B42" s="23" t="inlineStr">
         <is>
-          <t>ORIENTELEC</t>
+          <t>SPORTKING</t>
         </is>
       </c>
       <c r="C42" s="23" t="inlineStr">
@@ -3351,19 +3351,19 @@
         </is>
       </c>
       <c r="D42" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E42" s="25" t="n">
+        <v>226.1107</v>
+      </c>
+      <c r="F42" s="26" t="n">
+        <v>885</v>
+      </c>
+      <c r="G42" s="24" t="n">
         <v>46310</v>
       </c>
-      <c r="E42" s="25" t="n">
-        <v>201.1512</v>
-      </c>
-      <c r="F42" s="26" t="n">
-        <v>1500</v>
-      </c>
-      <c r="G42" s="24" t="n">
-        <v>46311</v>
-      </c>
       <c r="H42" s="25" t="n">
-        <v>206.72</v>
+        <v>226.89</v>
       </c>
       <c r="I42" s="21">
         <f>IF(OR($B42="",$H42=""),"",IF($C42="LONG",($H42-$E42)*$F42,($E42-$H42)*$F42))</f>
@@ -3374,7 +3374,7 @@
         <v/>
       </c>
       <c r="K42" s="4" t="n">
-        <v>552.14</v>
+        <v>626.9299999999999</v>
       </c>
       <c r="L42" s="21">
         <f>IF(OR($B42="",$I42=""),"",$I42-IF($K42="",0,$K42))</f>
@@ -3390,19 +3390,19 @@
       </c>
       <c r="O42" s="23" t="inlineStr">
         <is>
-          <t>10-15</t>
+          <t>5-10</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="23" t="inlineStr">
         <is>
-          <t>DHAN-231261015159409+321261015672709+321261015673309+221261015677909+221261015678309+341261015154609+321261015675209+221261015678809+341261015155009+341261015155109+231261015160609+231261015160709+341261015155509</t>
+          <t>DHAN-321261015672409+231261015159509+341261015154309+321261015674209+231261015159809+321261015674909+341261015154809+221261015678909+321261015675709+221261015679609+231261015160509</t>
         </is>
       </c>
       <c r="B43" s="23" t="inlineStr">
         <is>
-          <t>TEAMLEASE</t>
+          <t>JAICORPLTD</t>
         </is>
       </c>
       <c r="C43" s="23" t="inlineStr">
@@ -3414,16 +3414,16 @@
         <v>46310</v>
       </c>
       <c r="E43" s="25" t="n">
-        <v>1133.7498</v>
+        <v>95.05800000000001</v>
       </c>
       <c r="F43" s="26" t="n">
-        <v>263</v>
+        <v>3153</v>
       </c>
       <c r="G43" s="24" t="n">
         <v>46311</v>
       </c>
       <c r="H43" s="25" t="n">
-        <v>1124.65</v>
+        <v>94.26000000000001</v>
       </c>
       <c r="I43" s="21">
         <f>IF(OR($B43="",$H43=""),"",IF($C43="LONG",($H43-$E43)*$F43,($E43-$H43)*$F43))</f>
@@ -3434,7 +3434,7 @@
         <v/>
       </c>
       <c r="K43" s="4" t="n">
-        <v>542.6</v>
+        <v>878.86</v>
       </c>
       <c r="L43" s="21">
         <f>IF(OR($B43="",$I43=""),"",$I43-IF($K43="",0,$K43))</f>
@@ -3457,12 +3457,12 @@
     <row r="44">
       <c r="A44" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261016683609+23126101679509+23126101679909+321261016685009+221261016694409+221261016695109+34126101677409+321261016686809+23126101680709+321261016687809+23126101681009+34126101678009</t>
+          <t>DHAN-341261015154009+321261015672609+221261015677509+321261015674109+321261015674709+341261015154709+231261015160109+341261015154909+221261015679409+341261015155209+321261015676109</t>
         </is>
       </c>
       <c r="B44" s="23" t="inlineStr">
         <is>
-          <t>EUROPRATIK</t>
+          <t>OAL</t>
         </is>
       </c>
       <c r="C44" s="23" t="inlineStr">
@@ -3471,16 +3471,20 @@
         </is>
       </c>
       <c r="D44" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="E44" s="25" t="n">
+        <v>578.2952</v>
+      </c>
+      <c r="F44" s="26" t="n">
+        <v>258</v>
+      </c>
+      <c r="G44" s="24" t="n">
         <v>46311</v>
       </c>
-      <c r="E44" s="25" t="n">
-        <v>182.5264</v>
-      </c>
-      <c r="F44" s="26" t="n">
-        <v>1636</v>
-      </c>
-      <c r="G44" s="24" t="inlineStr"/>
-      <c r="H44" s="25" t="inlineStr"/>
+      <c r="H44" s="25" t="n">
+        <v>585.09</v>
+      </c>
       <c r="I44" s="21">
         <f>IF(OR($B44="",$H44=""),"",IF($C44="LONG",($H44-$E44)*$F44,($E44-$H44)*$F44))</f>
         <v/>
@@ -3490,7 +3494,7 @@
         <v/>
       </c>
       <c r="K44" s="4" t="n">
-        <v>50.15</v>
+        <v>348.51</v>
       </c>
       <c r="L44" s="21">
         <f>IF(OR($B44="",$I44=""),"",$I44-IF($K44="",0,$K44))</f>
@@ -3513,12 +3517,12 @@
     <row r="45">
       <c r="A45" s="23" t="inlineStr">
         <is>
-          <t>DHAN-34126101377609+221261013593609+34126101378109+23126101376709+34126101378409+23126101377009+221261013595709+221261013596109+221261013596609+23126101377809+34126101379309+34126101379709+23126101378409+34126101379809+221261013599309+321261013576809</t>
+          <t>DHAN-341261015153909+221261015677009+321261015673209+231261015159709+231261015159909+231261015160009+221261015678509+321261015675509+231261015160209+231261015160409+341261015155309</t>
         </is>
       </c>
       <c r="B45" s="23" t="inlineStr">
         <is>
-          <t>INDOKEM</t>
+          <t>ORIENTELEC</t>
         </is>
       </c>
       <c r="C45" s="23" t="inlineStr">
@@ -3527,16 +3531,20 @@
         </is>
       </c>
       <c r="D45" s="24" t="n">
-        <v>46308</v>
+        <v>46310</v>
       </c>
       <c r="E45" s="25" t="n">
-        <v>677.9853000000001</v>
+        <v>201.1512</v>
       </c>
       <c r="F45" s="26" t="n">
-        <v>126</v>
-      </c>
-      <c r="G45" s="24" t="inlineStr"/>
-      <c r="H45" s="25" t="inlineStr"/>
+        <v>1500</v>
+      </c>
+      <c r="G45" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H45" s="25" t="n">
+        <v>206.72</v>
+      </c>
       <c r="I45" s="21">
         <f>IF(OR($B45="",$H45=""),"",IF($C45="LONG",($H45-$E45)*$F45,($E45-$H45)*$F45))</f>
         <v/>
@@ -3546,7 +3554,7 @@
         <v/>
       </c>
       <c r="K45" s="4" t="n">
-        <v>116.19</v>
+        <v>896.95</v>
       </c>
       <c r="L45" s="21">
         <f>IF(OR($B45="",$I45=""),"",$I45-IF($K45="",0,$K45))</f>
@@ -3569,12 +3577,12 @@
     <row r="46">
       <c r="A46" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261016693009+23126101679709+23126101679809+23126101680009+321261016685409+221261016694909+34126101677509+321261016686909+34126101677709+321261016687909+34126101677909</t>
+          <t>DHAN-231261015159409+321261015672709+321261015673309+221261015677909+221261015678309+341261015154609+321261015675209+221261015678809+341261015155009+341261015155109+231261015160609+231261015160709+341261015155509</t>
         </is>
       </c>
       <c r="B46" s="23" t="inlineStr">
         <is>
-          <t>MBEL</t>
+          <t>TEAMLEASE</t>
         </is>
       </c>
       <c r="C46" s="23" t="inlineStr">
@@ -3583,16 +3591,20 @@
         </is>
       </c>
       <c r="D46" s="24" t="n">
+        <v>46310</v>
+      </c>
+      <c r="E46" s="25" t="n">
+        <v>1133.7498</v>
+      </c>
+      <c r="F46" s="26" t="n">
+        <v>263</v>
+      </c>
+      <c r="G46" s="24" t="n">
         <v>46311</v>
       </c>
-      <c r="E46" s="25" t="n">
-        <v>287.8416</v>
-      </c>
-      <c r="F46" s="26" t="n">
-        <v>1043</v>
-      </c>
-      <c r="G46" s="24" t="inlineStr"/>
-      <c r="H46" s="25" t="inlineStr"/>
+      <c r="H46" s="25" t="n">
+        <v>1124.65</v>
+      </c>
       <c r="I46" s="21">
         <f>IF(OR($B46="",$H46=""),"",IF($C46="LONG",($H46-$E46)*$F46,($E46-$H46)*$F46))</f>
         <v/>
@@ -3602,7 +3614,7 @@
         <v/>
       </c>
       <c r="K46" s="4" t="n">
-        <v>50.15</v>
+        <v>872.6900000000001</v>
       </c>
       <c r="L46" s="21">
         <f>IF(OR($B46="",$I46=""),"",$I46-IF($K46="",0,$K46))</f>
@@ -3625,12 +3637,12 @@
     <row r="47">
       <c r="A47" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261012625809+321261012626209+23126101284209+23126101284309+321261012626909+34126101276209+34126101277109+321261012628809+221261012640809+23126101286309+34126101278009+321261012630809+221261012643209</t>
+          <t>DHAN-321261016683609+23126101679509+23126101679909+321261016685009+221261016694409+221261016695109+34126101677409+321261016686809+23126101680709+321261016687809+23126101681009+34126101678009</t>
         </is>
       </c>
       <c r="B47" s="23" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>EUROPRATIK</t>
         </is>
       </c>
       <c r="C47" s="23" t="inlineStr">
@@ -3639,13 +3651,13 @@
         </is>
       </c>
       <c r="D47" s="24" t="n">
-        <v>46307</v>
+        <v>46311</v>
       </c>
       <c r="E47" s="25" t="n">
-        <v>22.8999</v>
+        <v>182.5264</v>
       </c>
       <c r="F47" s="26" t="n">
-        <v>3742</v>
+        <v>1636</v>
       </c>
       <c r="G47" s="24" t="inlineStr"/>
       <c r="H47" s="25" t="inlineStr"/>
@@ -3658,7 +3670,7 @@
         <v/>
       </c>
       <c r="K47" s="4" t="n">
-        <v>53.57</v>
+        <v>694.27</v>
       </c>
       <c r="L47" s="21">
         <f>IF(OR($B47="",$I47=""),"",$I47-IF($K47="",0,$K47))</f>
@@ -3674,19 +3686,19 @@
       </c>
       <c r="O47" s="23" t="inlineStr">
         <is>
-          <t>5-10</t>
+          <t>10-15</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261016683509+23126101679609+221261016693309+321261016685109+321261016685509+321261016685809+221261016695509+34126101677609+23126101680609+23126101680809+321261016688709+321261016689109+221261016697009+321261016690409</t>
+          <t>DHAN-221261016693009+23126101679709+23126101679809+23126101680009+321261016685409+221261016694909+34126101677509+321261016686909+34126101677709+321261016687909+34126101677909</t>
         </is>
       </c>
       <c r="B48" s="23" t="inlineStr">
         <is>
-          <t>PARACABLES</t>
+          <t>MBEL</t>
         </is>
       </c>
       <c r="C48" s="23" t="inlineStr">
@@ -3698,10 +3710,10 @@
         <v>46311</v>
       </c>
       <c r="E48" s="25" t="n">
-        <v>60.1311</v>
+        <v>287.8416</v>
       </c>
       <c r="F48" s="26" t="n">
-        <v>4996</v>
+        <v>1043</v>
       </c>
       <c r="G48" s="24" t="inlineStr"/>
       <c r="H48" s="25" t="inlineStr"/>
@@ -3714,7 +3726,7 @@
         <v/>
       </c>
       <c r="K48" s="4" t="n">
-        <v>50.15</v>
+        <v>697.77</v>
       </c>
       <c r="L48" s="21">
         <f>IF(OR($B48="",$I48=""),"",$I48-IF($K48="",0,$K48))</f>
@@ -3737,12 +3749,12 @@
     <row r="49">
       <c r="A49" s="23" t="inlineStr">
         <is>
-          <t>DHAN-341261014128809+341261014129209+221261014671809+321261014664309+221261014672409+321261014664909+341261014130009+221261014673409+221261014673609+221261014673709+221261014674009+321261014667309+341261014130909</t>
+          <t>DHAN-321261016683509+23126101679609+221261016693309+321261016685109+321261016685509+321261016685809+221261016695509+34126101677609+23126101680609+23126101680809+321261016688709+321261016689109+221261016697009+321261016690409</t>
         </is>
       </c>
       <c r="B49" s="23" t="inlineStr">
         <is>
-          <t>SIMPLEXINF</t>
+          <t>PARACABLES</t>
         </is>
       </c>
       <c r="C49" s="23" t="inlineStr">
@@ -3751,13 +3763,13 @@
         </is>
       </c>
       <c r="D49" s="24" t="n">
-        <v>46309</v>
+        <v>46311</v>
       </c>
       <c r="E49" s="25" t="n">
-        <v>266.801</v>
+        <v>60.1311</v>
       </c>
       <c r="F49" s="26" t="n">
-        <v>749</v>
+        <v>4996</v>
       </c>
       <c r="G49" s="24" t="inlineStr"/>
       <c r="H49" s="25" t="inlineStr"/>
@@ -3770,7 +3782,7 @@
         <v/>
       </c>
       <c r="K49" s="4" t="n">
-        <v>394.85</v>
+        <v>694.98</v>
       </c>
       <c r="L49" s="21">
         <f>IF(OR($B49="",$I49=""),"",$I49-IF($K49="",0,$K49))</f>
@@ -3826,7 +3838,7 @@
         <v/>
       </c>
       <c r="K50" s="4" t="n">
-        <v>50.15</v>
+        <v>699</v>
       </c>
       <c r="L50" s="21">
         <f>IF(OR($B50="",$I50=""),"",$I50-IF($K50="",0,$K50))</f>
@@ -33205,7 +33217,7 @@
         <v>35.4</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>120.95</v>
+        <v>117.71</v>
       </c>
       <c r="N6" s="21">
         <f>SUM(E6:M6)</f>
@@ -33256,7 +33268,7 @@
         <v>35.4</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>72.31999999999999</v>
+        <v>70.38</v>
       </c>
       <c r="N7" s="21">
         <f>SUM(E7:M7)</f>
@@ -33307,7 +33319,7 @@
         <v>35.4</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>100.64</v>
+        <v>97.94</v>
       </c>
       <c r="N8" s="21">
         <f>SUM(E8:M8)</f>
@@ -33358,7 +33370,7 @@
         <v>35.4</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>120.62</v>
+        <v>117.38</v>
       </c>
       <c r="N9" s="21">
         <f>SUM(E9:M9)</f>
@@ -33409,7 +33421,7 @@
         <v>35.4</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>100.65</v>
+        <v>97.95</v>
       </c>
       <c r="N10" s="21">
         <f>SUM(E10:M10)</f>
@@ -33460,7 +33472,7 @@
         <v>35.4</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>62.39</v>
+        <v>61.07</v>
       </c>
       <c r="N11" s="21">
         <f>SUM(E11:M11)</f>
@@ -33511,7 +33523,7 @@
         <v>35.4</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>74.78</v>
+        <v>73.19</v>
       </c>
       <c r="N12" s="21">
         <f>SUM(E12:M12)</f>
@@ -33562,7 +33574,7 @@
         <v>35.4</v>
       </c>
       <c r="M13" s="4" t="n">
-        <v>44.98</v>
+        <v>74.84</v>
       </c>
       <c r="N13" s="21">
         <f>SUM(E13:M13)</f>
@@ -33613,7 +33625,7 @@
         <v>35.4</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>44.78</v>
+        <v>43.83</v>
       </c>
       <c r="N14" s="21">
         <f>SUM(E14:M14)</f>
@@ -33766,7 +33778,7 @@
         <v>35.4</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>52.92</v>
+        <v>52.34</v>
       </c>
       <c r="N17" s="21">
         <f>SUM(E17:M17)</f>
@@ -33868,7 +33880,7 @@
         <v>35.4</v>
       </c>
       <c r="M19" s="4" t="n">
-        <v>91.29000000000001</v>
+        <v>90.37</v>
       </c>
       <c r="N19" s="21">
         <f>SUM(E19:M19)</f>
@@ -33919,7 +33931,7 @@
         <v>35.4</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>88.29000000000001</v>
+        <v>87.34</v>
       </c>
       <c r="N20" s="21">
         <f>SUM(E20:M20)</f>
@@ -34021,7 +34033,7 @@
         <v>35.4</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>88.70999999999999</v>
+        <v>87.75</v>
       </c>
       <c r="N22" s="21">
         <f>SUM(E22:M22)</f>
@@ -34072,7 +34084,7 @@
         <v>35.4</v>
       </c>
       <c r="M23" s="4" t="n">
-        <v>31.59</v>
+        <v>31.25</v>
       </c>
       <c r="N23" s="21">
         <f>SUM(E23:M23)</f>
@@ -34174,7 +34186,7 @@
         <v>35.4</v>
       </c>
       <c r="M25" s="4" t="n">
-        <v>39.2</v>
+        <v>38.79</v>
       </c>
       <c r="N25" s="21">
         <f>SUM(E25:M25)</f>
@@ -34184,12 +34196,12 @@
     <row r="26">
       <c r="A26" s="23" t="inlineStr">
         <is>
-          <t>DHAN-34126101275609+321261012626309+221261012637809+34126101275809+23126101284509+321261012627209+34126101277009+34126101277209+34126101277609+221261012641209+321261012630309+23126101287209+321261012631409+321261012631709+321261012632009</t>
+          <t>DHAN-321261012625809+321261012626209+23126101284209+23126101284309+321261012626909+34126101276209+34126101277109+321261012628809+221261012640809+23126101286309+34126101278009+321261012630809+221261012643209</t>
         </is>
       </c>
       <c r="B26" s="23" t="inlineStr">
         <is>
-          <t>PRINCEPIPE</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="C26" s="23" t="inlineStr">
@@ -34201,31 +34213,31 @@
         <v>46308</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>71.44</v>
+        <v>24.76</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>339.48</v>
+        <v>90.14</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>10.42</v>
+        <v>5.29</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>0.34</v>
+        <v>0.17</v>
       </c>
       <c r="I26" s="4" t="n">
-        <v>25.26</v>
+        <v>3</v>
       </c>
       <c r="J26" s="4" t="n">
-        <v>14.8</v>
+        <v>5.44</v>
       </c>
       <c r="K26" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L26" s="4" t="n">
-        <v>35.4</v>
+        <v>0</v>
       </c>
       <c r="M26" s="4" t="n">
-        <v>37.78</v>
+        <v>0</v>
       </c>
       <c r="N26" s="21">
         <f>SUM(E26:M26)</f>
@@ -34235,12 +34247,12 @@
     <row r="27">
       <c r="A27" s="23" t="inlineStr">
         <is>
-          <t>DHAN-23126101283509+23126101284109+34126101275709+221261012638509+34126101275909+23126101284809+321261012628509+321261012628709+23126101286109+321261012629509+221261012641909+221261012642709+23126101287309+221261012643409+34126101278409</t>
+          <t>DHAN-34126101275609+321261012626309+221261012637809+34126101275809+23126101284509+321261012627209+34126101277009+34126101277209+34126101277609+221261012641209+321261012630309+23126101287209+321261012631409+321261012631709+321261012632009</t>
         </is>
       </c>
       <c r="B27" s="23" t="inlineStr">
         <is>
-          <t>SWARAJENG</t>
+          <t>PRINCEPIPE</t>
         </is>
       </c>
       <c r="C27" s="23" t="inlineStr">
@@ -34252,22 +34264,22 @@
         <v>46308</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>70.51000000000001</v>
+        <v>71.44</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>335.81</v>
+        <v>339.48</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>10.31</v>
+        <v>10.42</v>
       </c>
       <c r="H27" s="4" t="n">
         <v>0.34</v>
       </c>
       <c r="I27" s="4" t="n">
-        <v>25.25</v>
+        <v>25.26</v>
       </c>
       <c r="J27" s="4" t="n">
-        <v>14.61</v>
+        <v>14.8</v>
       </c>
       <c r="K27" s="4" t="n">
         <v>14.75</v>
@@ -34276,7 +34288,7 @@
         <v>35.4</v>
       </c>
       <c r="M27" s="4" t="n">
-        <v>43.26</v>
+        <v>37.37</v>
       </c>
       <c r="N27" s="21">
         <f>SUM(E27:M27)</f>
@@ -34286,12 +34298,12 @@
     <row r="28">
       <c r="A28" s="23" t="inlineStr">
         <is>
-          <t>DHAN-34126101377709+221261013593709+321261013572009+23126101376509+221261013594809+34126101378609+221261013595609+23126101377609+321261013574409+321261013575009+23126101378109+23126101378209</t>
+          <t>DHAN-23126101283509+23126101284109+34126101275709+221261012638509+34126101275909+23126101284809+321261012628509+321261012628709+23126101286109+321261012629509+221261012641909+221261012642709+23126101287309+221261012643409+34126101278409</t>
         </is>
       </c>
       <c r="B28" s="23" t="inlineStr">
         <is>
-          <t>CMLL</t>
+          <t>SWARAJENG</t>
         </is>
       </c>
       <c r="C28" s="23" t="inlineStr">
@@ -34300,25 +34312,25 @@
         </is>
       </c>
       <c r="D28" s="24" t="n">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>71.3</v>
+        <v>70.51000000000001</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>339.38</v>
+        <v>335.81</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>10.42</v>
+        <v>10.31</v>
       </c>
       <c r="H28" s="4" t="n">
         <v>0.34</v>
       </c>
       <c r="I28" s="4" t="n">
-        <v>25.64</v>
+        <v>25.25</v>
       </c>
       <c r="J28" s="4" t="n">
-        <v>14.77</v>
+        <v>14.61</v>
       </c>
       <c r="K28" s="4" t="n">
         <v>14.75</v>
@@ -34327,7 +34339,7 @@
         <v>35.4</v>
       </c>
       <c r="M28" s="4" t="n">
-        <v>45.4</v>
+        <v>42.79</v>
       </c>
       <c r="N28" s="21">
         <f>SUM(E28:M28)</f>
@@ -34337,12 +34349,12 @@
     <row r="29">
       <c r="A29" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261013592809+34126101377809+321261013572109+23126101376309+34126101378309+321261013573109+34126101378709+221261013596309+23126101377709+221261013597309+321261013575409+321261013575609</t>
+          <t>DHAN-34126101377709+221261013593709+321261013572009+23126101376509+221261013594809+34126101378609+221261013595609+23126101377609+321261013574409+321261013575009+23126101378109+23126101378209</t>
         </is>
       </c>
       <c r="B29" s="23" t="inlineStr">
         <is>
-          <t>HATHWAY</t>
+          <t>CMLL</t>
         </is>
       </c>
       <c r="C29" s="23" t="inlineStr">
@@ -34354,22 +34366,22 @@
         <v>46309</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>71</v>
+        <v>71.3</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>342.53</v>
+        <v>339.38</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>10.51</v>
+        <v>10.42</v>
       </c>
       <c r="H29" s="4" t="n">
         <v>0.34</v>
       </c>
       <c r="I29" s="4" t="n">
-        <v>25.77</v>
+        <v>25.64</v>
       </c>
       <c r="J29" s="4" t="n">
-        <v>14.73</v>
+        <v>14.77</v>
       </c>
       <c r="K29" s="4" t="n">
         <v>14.75</v>
@@ -34378,7 +34390,7 @@
         <v>35.4</v>
       </c>
       <c r="M29" s="4" t="n">
-        <v>37.74</v>
+        <v>44.86</v>
       </c>
       <c r="N29" s="21">
         <f>SUM(E29:M29)</f>
@@ -34388,12 +34400,12 @@
     <row r="30">
       <c r="A30" s="23" t="inlineStr">
         <is>
-          <t>DHAN-23126101375909+221261013593509+221261013594309+34126101378209+321261013572509+23126101377109+321261013573709+23126101377509+34126101379009+321261013575109+221261013597709+221261013598409+34126101379609</t>
+          <t>DHAN-221261013592809+34126101377809+321261013572109+23126101376309+34126101378309+321261013573109+34126101378709+221261013596309+23126101377709+221261013597309+321261013575409+321261013575609</t>
         </is>
       </c>
       <c r="B30" s="23" t="inlineStr">
         <is>
-          <t>INDIAGLYCO</t>
+          <t>HATHWAY</t>
         </is>
       </c>
       <c r="C30" s="23" t="inlineStr">
@@ -34405,31 +34417,31 @@
         <v>46309</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>172.92</v>
+        <v>342.53</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>5.31</v>
+        <v>10.51</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>0.17</v>
+        <v>0.34</v>
       </c>
       <c r="I30" s="4" t="n">
-        <v>12.86</v>
+        <v>25.77</v>
       </c>
       <c r="J30" s="4" t="n">
-        <v>0.99</v>
+        <v>14.73</v>
       </c>
       <c r="K30" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L30" s="4" t="n">
-        <v>0</v>
+        <v>35.4</v>
       </c>
       <c r="M30" s="4" t="n">
-        <v>0</v>
+        <v>37.34</v>
       </c>
       <c r="N30" s="21">
         <f>SUM(E30:M30)</f>
@@ -34439,12 +34451,12 @@
     <row r="31">
       <c r="A31" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261013593009+23126101376209+34126101378009+221261013594409+23126101376909+23126101377209+23126101377309+321261013574209+321261013574509+23126101377909+34126101379509+321261013575709</t>
+          <t>DHAN-23126101375909+221261013593509+221261013594309+34126101378209+321261013572509+23126101377109+321261013573709+23126101377509+34126101379009+321261013575109+221261013597709+221261013598409+34126101379609</t>
         </is>
       </c>
       <c r="B31" s="23" t="inlineStr">
         <is>
-          <t>PIXTRANS</t>
+          <t>INDIAGLYCO</t>
         </is>
       </c>
       <c r="C31" s="23" t="inlineStr">
@@ -34456,31 +34468,31 @@
         <v>46309</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>71.01000000000001</v>
+        <v>0</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>343.17</v>
+        <v>172.92</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>10.53</v>
+        <v>5.31</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>0.34</v>
+        <v>0.17</v>
       </c>
       <c r="I31" s="4" t="n">
-        <v>25.51</v>
+        <v>12.86</v>
       </c>
       <c r="J31" s="4" t="n">
-        <v>14.74</v>
+        <v>0.99</v>
       </c>
       <c r="K31" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L31" s="4" t="n">
-        <v>35.4</v>
+        <v>0</v>
       </c>
       <c r="M31" s="4" t="n">
-        <v>37.45</v>
+        <v>0</v>
       </c>
       <c r="N31" s="21">
         <f>SUM(E31:M31)</f>
@@ -34490,12 +34502,12 @@
     <row r="32">
       <c r="A32" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261013571309+221261013593809+221261013594209+23126101376409+34126101378509+321261013573309+34126101378809+34126101378909+221261013596709+221261013597209+34126101379409+23126101378309+321261013576009</t>
+          <t>DHAN-34126101377609+221261013593609+34126101378109+23126101376709+34126101378409+23126101377009+221261013595709+221261013596109+221261013596609+23126101377809+34126101379309+34126101379709+23126101378409+34126101379809+221261013599309+321261013576809</t>
         </is>
       </c>
       <c r="B32" s="23" t="inlineStr">
         <is>
-          <t>PNCINFRA</t>
+          <t>INDOKEM</t>
         </is>
       </c>
       <c r="C32" s="23" t="inlineStr">
@@ -34507,31 +34519,31 @@
         <v>46309</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>71.06999999999999</v>
+        <v>0</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>215.5</v>
+        <v>85.43000000000001</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>10.89</v>
+        <v>2.62</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>0.35</v>
+        <v>0.09</v>
       </c>
       <c r="I32" s="4" t="n">
-        <v>25.53</v>
+        <v>12.81</v>
       </c>
       <c r="J32" s="4" t="n">
-        <v>14.82</v>
+        <v>0.49</v>
       </c>
       <c r="K32" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L32" s="4" t="n">
-        <v>35.4</v>
+        <v>0</v>
       </c>
       <c r="M32" s="4" t="n">
-        <v>39.81</v>
+        <v>0</v>
       </c>
       <c r="N32" s="21">
         <f>SUM(E32:M32)</f>
@@ -34541,48 +34553,48 @@
     <row r="33">
       <c r="A33" s="23" t="inlineStr">
         <is>
-          <t>DHAN-34126101478009</t>
+          <t>DHAN-221261013593009+23126101376209+34126101378009+221261013594409+23126101376909+23126101377209+23126101377309+321261013574209+321261013574509+23126101377909+34126101379509+321261013575709</t>
         </is>
       </c>
       <c r="B33" s="23" t="inlineStr">
         <is>
-          <t>PNCINFRA</t>
+          <t>PIXTRANS</t>
         </is>
       </c>
       <c r="C33" s="23" t="inlineStr">
         <is>
-          <t>SHORT</t>
+          <t>LONG</t>
         </is>
       </c>
       <c r="D33" s="24" t="n">
         <v>46309</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>20</v>
+        <v>71.01000000000001</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>181.5</v>
+        <v>343.17</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>11.03</v>
+        <v>10.53</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>0.36</v>
+        <v>0.34</v>
       </c>
       <c r="I33" s="4" t="n">
-        <v>5.25</v>
+        <v>25.51</v>
       </c>
       <c r="J33" s="4" t="n">
-        <v>5.65</v>
+        <v>14.74</v>
       </c>
       <c r="K33" s="4" t="n">
-        <v>0</v>
+        <v>14.75</v>
       </c>
       <c r="L33" s="4" t="n">
-        <v>0</v>
+        <v>35.4</v>
       </c>
       <c r="M33" s="4" t="n">
-        <v>0</v>
+        <v>37.05</v>
       </c>
       <c r="N33" s="21">
         <f>SUM(E33:M33)</f>
@@ -34592,12 +34604,12 @@
     <row r="34">
       <c r="A34" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261013592909+23126101376109+321261013572209+23126101376609+321261013572609+321261013573209+321261013573809+221261013596209+34126101379109+34126101379209+221261013597909</t>
+          <t>DHAN-321261013571309+221261013593809+221261013594209+23126101376409+34126101378509+321261013573309+34126101378809+34126101378909+221261013596709+221261013597209+34126101379409+23126101378309+321261013576009</t>
         </is>
       </c>
       <c r="B34" s="23" t="inlineStr">
         <is>
-          <t>SHRINGARMS</t>
+          <t>PNCINFRA</t>
         </is>
       </c>
       <c r="C34" s="23" t="inlineStr">
@@ -34609,22 +34621,22 @@
         <v>46309</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>71.33</v>
+        <v>71.06999999999999</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>344.55</v>
+        <v>215.5</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>10.58</v>
+        <v>10.89</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>0.34</v>
+        <v>0.35</v>
       </c>
       <c r="I34" s="4" t="n">
-        <v>25.67</v>
+        <v>25.53</v>
       </c>
       <c r="J34" s="4" t="n">
-        <v>14.81</v>
+        <v>14.82</v>
       </c>
       <c r="K34" s="4" t="n">
         <v>14.75</v>
@@ -34633,7 +34645,7 @@
         <v>35.4</v>
       </c>
       <c r="M34" s="4" t="n">
-        <v>22.62</v>
+        <v>39.41</v>
       </c>
       <c r="N34" s="21">
         <f>SUM(E34:M34)</f>
@@ -34643,48 +34655,48 @@
     <row r="35">
       <c r="A35" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261014662909+221261014671509+321261014664009+341261014129509+341261014129709+321261014665509+221261014673509+231261014126609+221261014673809+221261014674109+231261014126809+341261014131109+221261014675709+231261014127209+341261014131309+231261014127309</t>
+          <t>DHAN-34126101478009</t>
         </is>
       </c>
       <c r="B35" s="23" t="inlineStr">
         <is>
-          <t>JINDALPOLY</t>
+          <t>PNCINFRA</t>
         </is>
       </c>
       <c r="C35" s="23" t="inlineStr">
         <is>
-          <t>LONG</t>
+          <t>SHORT</t>
         </is>
       </c>
       <c r="D35" s="24" t="n">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>63.82</v>
+        <v>20</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>288.31</v>
+        <v>181.5</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>8.85</v>
+        <v>11.03</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>0.29</v>
+        <v>0.36</v>
       </c>
       <c r="I35" s="4" t="n">
-        <v>21.9</v>
+        <v>5.25</v>
       </c>
       <c r="J35" s="4" t="n">
-        <v>13.13</v>
+        <v>5.65</v>
       </c>
       <c r="K35" s="4" t="n">
-        <v>14.75</v>
+        <v>0</v>
       </c>
       <c r="L35" s="4" t="n">
-        <v>35.4</v>
+        <v>0</v>
       </c>
       <c r="M35" s="4" t="n">
-        <v>33.7</v>
+        <v>0</v>
       </c>
       <c r="N35" s="21">
         <f>SUM(E35:M35)</f>
@@ -34694,12 +34706,12 @@
     <row r="36">
       <c r="A36" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261014663009+221261014671609+341261014129309+221261014671909+341261014129609+341261014129809+231261014126309+321261014666109+231261014126509+341261014130409+231261014126709+231261014126909</t>
+          <t>DHAN-221261013592909+23126101376109+321261013572209+23126101376609+321261013572609+321261013573209+321261013573809+221261013596209+34126101379109+34126101379209+221261013597909</t>
         </is>
       </c>
       <c r="B36" s="23" t="inlineStr">
         <is>
-          <t>KROSS</t>
+          <t>SHRINGARMS</t>
         </is>
       </c>
       <c r="C36" s="23" t="inlineStr">
@@ -34708,25 +34720,25 @@
         </is>
       </c>
       <c r="D36" s="24" t="n">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>80.01000000000001</v>
+        <v>71.33</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>399.82</v>
+        <v>344.55</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>12.27</v>
+        <v>10.58</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>0.4</v>
+        <v>0.34</v>
       </c>
       <c r="I36" s="4" t="n">
-        <v>30.02</v>
+        <v>25.67</v>
       </c>
       <c r="J36" s="4" t="n">
-        <v>16.68</v>
+        <v>14.81</v>
       </c>
       <c r="K36" s="4" t="n">
         <v>14.75</v>
@@ -34735,7 +34747,7 @@
         <v>35.4</v>
       </c>
       <c r="M36" s="4" t="n">
-        <v>36.72</v>
+        <v>22.37</v>
       </c>
       <c r="N36" s="21">
         <f>SUM(E36:M36)</f>
@@ -34745,12 +34757,12 @@
     <row r="37">
       <c r="A37" s="23" t="inlineStr">
         <is>
-          <t>DHAN-341261014128909+341261014129109+231261014125709+321261014664109+321261014664809+231261014126009+321261014665609+231261014126409+341261014130309+341261014130509+221261014673909+341261014130709+221261014674609+221261014675009+221261014675509</t>
+          <t>DHAN-321261014662909+221261014671509+321261014664009+341261014129509+341261014129709+321261014665509+221261014673509+231261014126609+221261014673809+221261014674109+231261014126809+341261014131109+221261014675709+231261014127209+341261014131309+231261014127309</t>
         </is>
       </c>
       <c r="B37" s="23" t="inlineStr">
         <is>
-          <t>NIBE</t>
+          <t>JINDALPOLY</t>
         </is>
       </c>
       <c r="C37" s="23" t="inlineStr">
@@ -34762,22 +34774,22 @@
         <v>46310</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>79.64</v>
+        <v>63.82</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>390.96</v>
+        <v>288.31</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>12</v>
+        <v>8.85</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>0.39</v>
+        <v>0.29</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>29.82</v>
+        <v>21.9</v>
       </c>
       <c r="J37" s="4" t="n">
-        <v>16.57</v>
+        <v>13.13</v>
       </c>
       <c r="K37" s="4" t="n">
         <v>14.75</v>
@@ -34786,7 +34798,7 @@
         <v>35.4</v>
       </c>
       <c r="M37" s="4" t="n">
-        <v>36.49</v>
+        <v>33.37</v>
       </c>
       <c r="N37" s="21">
         <f>SUM(E37:M37)</f>
@@ -34796,12 +34808,12 @@
     <row r="38">
       <c r="A38" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261014671209+321261014663609+231261014125809+221261014672009+231261014125909+231261014126109+221261014673109+341261014130209+321261014666509+341261014130609+321261014667409+321261014667809+341261014131209+221261014676209+221261014676809</t>
+          <t>DHAN-321261014663009+221261014671609+341261014129309+221261014671909+341261014129609+341261014129809+231261014126309+321261014666109+231261014126509+341261014130409+231261014126709+231261014126909</t>
         </is>
       </c>
       <c r="B38" s="23" t="inlineStr">
         <is>
-          <t>RUBYMILLS</t>
+          <t>KROSS</t>
         </is>
       </c>
       <c r="C38" s="23" t="inlineStr">
@@ -34813,31 +34825,31 @@
         <v>46310</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>0</v>
+        <v>80.01000000000001</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>201.6</v>
+        <v>399.82</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>6.19</v>
+        <v>12.27</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="I38" s="4" t="n">
-        <v>14.94</v>
+        <v>30.02</v>
       </c>
       <c r="J38" s="4" t="n">
-        <v>1.15</v>
+        <v>16.68</v>
       </c>
       <c r="K38" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L38" s="4" t="n">
-        <v>0</v>
+        <v>35.4</v>
       </c>
       <c r="M38" s="4" t="n">
-        <v>0</v>
+        <v>36.33</v>
       </c>
       <c r="N38" s="21">
         <f>SUM(E38:M38)</f>
@@ -34847,12 +34859,12 @@
     <row r="39">
       <c r="A39" s="23" t="inlineStr">
         <is>
-          <t>DHAN-231261014125609+321261014663509+321261014663909+321261014664209+221261014672509+231261014126209+341261014130109+321261014666209+321261014666609+321261014666709+321261014667009+341261014130809+231261014127009+341261014131009+221261014675609</t>
+          <t>DHAN-341261014128909+341261014129109+231261014125709+321261014664109+321261014664809+231261014126009+321261014665609+231261014126409+341261014130309+341261014130509+221261014673909+341261014130709+221261014674609+221261014675009+221261014675509</t>
         </is>
       </c>
       <c r="B39" s="23" t="inlineStr">
         <is>
-          <t>SPORTKING</t>
+          <t>NIBE</t>
         </is>
       </c>
       <c r="C39" s="23" t="inlineStr">
@@ -34864,22 +34876,22 @@
         <v>46310</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>80.05</v>
+        <v>79.64</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>400.91</v>
+        <v>390.96</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>12.31</v>
+        <v>12</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>0.4</v>
+        <v>0.39</v>
       </c>
       <c r="I39" s="4" t="n">
-        <v>30.09</v>
+        <v>29.82</v>
       </c>
       <c r="J39" s="4" t="n">
-        <v>16.7</v>
+        <v>16.57</v>
       </c>
       <c r="K39" s="4" t="n">
         <v>14.75</v>
@@ -34888,7 +34900,7 @@
         <v>35.4</v>
       </c>
       <c r="M39" s="4" t="n">
-        <v>36.73</v>
+        <v>36.09</v>
       </c>
       <c r="N39" s="21">
         <f>SUM(E39:M39)</f>
@@ -34898,12 +34910,12 @@
     <row r="40">
       <c r="A40" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261015672409+231261015159509+341261015154309+321261015674209+231261015159809+321261015674909+341261015154809+221261015678909+321261015675709+221261015679609+231261015160509</t>
+          <t>DHAN-221261014671209+321261014663609+231261014125809+221261014672009+231261014125909+231261014126109+221261014673109+341261014130209+321261014666509+341261014130609+321261014667409+321261014667809+341261014131209+221261014676209+221261014676809</t>
         </is>
       </c>
       <c r="B40" s="23" t="inlineStr">
         <is>
-          <t>JAICORPLTD</t>
+          <t>RUBYMILLS</t>
         </is>
       </c>
       <c r="C40" s="23" t="inlineStr">
@@ -34912,34 +34924,34 @@
         </is>
       </c>
       <c r="D40" s="24" t="n">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>89.95</v>
+        <v>0</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>299.72</v>
+        <v>201.6</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>9.199999999999999</v>
+        <v>6.19</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="I40" s="4" t="n">
-        <v>44.96</v>
+        <v>14.94</v>
       </c>
       <c r="J40" s="4" t="n">
-        <v>17.9</v>
+        <v>1.15</v>
       </c>
       <c r="K40" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L40" s="4" t="n">
-        <v>35.4</v>
+        <v>0</v>
       </c>
       <c r="M40" s="4" t="n">
-        <v>35.15</v>
+        <v>0</v>
       </c>
       <c r="N40" s="21">
         <f>SUM(E40:M40)</f>
@@ -34949,12 +34961,12 @@
     <row r="41">
       <c r="A41" s="23" t="inlineStr">
         <is>
-          <t>DHAN-341261015154009+321261015672609+221261015677509+321261015674109+321261015674709+341261015154709+231261015160109+341261015154909+221261015679409+341261015155209+321261015676109</t>
+          <t>DHAN-341261014128809+341261014129209+221261014671809+321261014664309+221261014672409+321261014664909+341261014130009+221261014673409+221261014673609+221261014673709+221261014674009+321261014667309+341261014130909</t>
         </is>
       </c>
       <c r="B41" s="23" t="inlineStr">
         <is>
-          <t>OAL</t>
+          <t>SIMPLEXINF</t>
         </is>
       </c>
       <c r="C41" s="23" t="inlineStr">
@@ -34963,34 +34975,34 @@
         </is>
       </c>
       <c r="D41" s="24" t="n">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>0</v>
+        <v>59.95</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>149.2</v>
+        <v>199.83</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>4.58</v>
+        <v>6.13</v>
       </c>
       <c r="H41" s="4" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="I41" s="4" t="n">
-        <v>22.38</v>
+        <v>29.98</v>
       </c>
       <c r="J41" s="4" t="n">
-        <v>0.85</v>
+        <v>11.93</v>
       </c>
       <c r="K41" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L41" s="4" t="n">
-        <v>0</v>
+        <v>35.4</v>
       </c>
       <c r="M41" s="4" t="n">
-        <v>0</v>
+        <v>36.28</v>
       </c>
       <c r="N41" s="21">
         <f>SUM(E41:M41)</f>
@@ -35000,12 +35012,12 @@
     <row r="42">
       <c r="A42" s="23" t="inlineStr">
         <is>
-          <t>DHAN-341261015153909+221261015677009+321261015673209+231261015159709+231261015159909+231261015160009+221261015678509+321261015675509+231261015160209+231261015160409+341261015155309</t>
+          <t>DHAN-231261014125609+321261014663509+321261014663909+321261014664209+221261014672509+231261014126209+341261014130109+321261014666209+321261014666609+321261014666709+321261014667009+341261014130809+231261014127009+341261014131009+221261014675609</t>
         </is>
       </c>
       <c r="B42" s="23" t="inlineStr">
         <is>
-          <t>ORIENTELEC</t>
+          <t>SPORTKING</t>
         </is>
       </c>
       <c r="C42" s="23" t="inlineStr">
@@ -35014,25 +35026,25 @@
         </is>
       </c>
       <c r="D42" s="24" t="n">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>90.56999999999999</v>
+        <v>80.05</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>301.73</v>
+        <v>400.91</v>
       </c>
       <c r="G42" s="4" t="n">
-        <v>9.26</v>
+        <v>12.31</v>
       </c>
       <c r="H42" s="4" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="I42" s="4" t="n">
-        <v>44.93</v>
+        <v>30.09</v>
       </c>
       <c r="J42" s="4" t="n">
-        <v>18.02</v>
+        <v>16.7</v>
       </c>
       <c r="K42" s="4" t="n">
         <v>14.75</v>
@@ -35041,7 +35053,7 @@
         <v>35.4</v>
       </c>
       <c r="M42" s="4" t="n">
-        <v>37.17</v>
+        <v>36.33</v>
       </c>
       <c r="N42" s="21">
         <f>SUM(E42:M42)</f>
@@ -35051,12 +35063,12 @@
     <row r="43">
       <c r="A43" s="23" t="inlineStr">
         <is>
-          <t>DHAN-231261015159409+321261015672709+321261015673309+221261015677909+221261015678309+341261015154609+321261015675209+221261015678809+341261015155009+341261015155109+231261015160609+231261015160709+341261015155509</t>
+          <t>DHAN-321261015672409+231261015159509+341261015154309+321261015674209+231261015159809+321261015674909+341261015154809+221261015678909+321261015675709+221261015679609+231261015160509</t>
         </is>
       </c>
       <c r="B43" s="23" t="inlineStr">
         <is>
-          <t>TEAMLEASE</t>
+          <t>JAICORPLTD</t>
         </is>
       </c>
       <c r="C43" s="23" t="inlineStr">
@@ -35068,22 +35080,22 @@
         <v>46311</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>89.45</v>
+        <v>109.95</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>298.18</v>
+        <v>596.92</v>
       </c>
       <c r="G43" s="4" t="n">
-        <v>9.15</v>
+        <v>18.32</v>
       </c>
       <c r="H43" s="4" t="n">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="I43" s="4" t="n">
-        <v>44.73</v>
+        <v>44.96</v>
       </c>
       <c r="J43" s="4" t="n">
-        <v>17.8</v>
+        <v>23.2</v>
       </c>
       <c r="K43" s="4" t="n">
         <v>14.75</v>
@@ -35092,7 +35104,7 @@
         <v>35.4</v>
       </c>
       <c r="M43" s="4" t="n">
-        <v>32.83</v>
+        <v>34.76</v>
       </c>
       <c r="N43" s="21">
         <f>SUM(E43:M43)</f>
@@ -35102,12 +35114,12 @@
     <row r="44">
       <c r="A44" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261016683609+23126101679509+23126101679909+321261016685009+221261016694409+221261016695109+34126101677409+321261016686809+23126101680709+321261016687809+23126101681009+34126101678009</t>
+          <t>DHAN-341261015154009+321261015672609+221261015677509+321261015674109+321261015674709+341261015154709+231261015160109+341261015154909+221261015679409+341261015155209+321261015676109</t>
         </is>
       </c>
       <c r="B44" s="23" t="inlineStr">
         <is>
-          <t>EUROPRATIK</t>
+          <t>OAL</t>
         </is>
       </c>
       <c r="C44" s="23" t="inlineStr">
@@ -35115,30 +35127,32 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D44" s="24" t="inlineStr"/>
+      <c r="D44" s="24" t="n">
+        <v>46311</v>
+      </c>
       <c r="E44" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>0</v>
+        <v>300.15</v>
       </c>
       <c r="G44" s="4" t="n">
-        <v>0</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="H44" s="4" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="I44" s="4" t="n">
-        <v>0</v>
+        <v>22.38</v>
       </c>
       <c r="J44" s="4" t="n">
-        <v>0</v>
+        <v>1.71</v>
       </c>
       <c r="K44" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L44" s="4" t="n">
-        <v>35.4</v>
+        <v>0</v>
       </c>
       <c r="M44" s="4" t="n">
         <v>0</v>
@@ -35151,12 +35165,12 @@
     <row r="45">
       <c r="A45" s="23" t="inlineStr">
         <is>
-          <t>DHAN-34126101377609+221261013593609+34126101378109+23126101376709+34126101378409+23126101377009+221261013595709+221261013596109+221261013596609+23126101377809+34126101379309+34126101379709+23126101378409+34126101379809+221261013599309+321261013576809</t>
+          <t>DHAN-341261015153909+221261015677009+321261015673209+231261015159709+231261015159909+231261015160009+221261015678509+321261015675509+231261015160209+231261015160409+341261015155309</t>
         </is>
       </c>
       <c r="B45" s="23" t="inlineStr">
         <is>
-          <t>INDOKEM</t>
+          <t>ORIENTELEC</t>
         </is>
       </c>
       <c r="C45" s="23" t="inlineStr">
@@ -35164,33 +35178,35 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D45" s="24" t="inlineStr"/>
+      <c r="D45" s="24" t="n">
+        <v>46311</v>
+      </c>
       <c r="E45" s="4" t="n">
-        <v>0</v>
+        <v>110.57</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>85.43000000000001</v>
+        <v>611.74</v>
       </c>
       <c r="G45" s="4" t="n">
-        <v>2.62</v>
+        <v>18.78</v>
       </c>
       <c r="H45" s="4" t="n">
-        <v>0.09</v>
+        <v>0.61</v>
       </c>
       <c r="I45" s="4" t="n">
-        <v>12.81</v>
+        <v>44.93</v>
       </c>
       <c r="J45" s="4" t="n">
-        <v>0.49</v>
+        <v>23.39</v>
       </c>
       <c r="K45" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L45" s="4" t="n">
-        <v>0</v>
+        <v>35.4</v>
       </c>
       <c r="M45" s="4" t="n">
-        <v>0</v>
+        <v>36.78</v>
       </c>
       <c r="N45" s="21">
         <f>SUM(E45:M45)</f>
@@ -35200,12 +35216,12 @@
     <row r="46">
       <c r="A46" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261016693009+23126101679709+23126101679809+23126101680009+321261016685409+221261016694909+34126101677509+321261016686909+34126101677709+321261016687909+34126101677909</t>
+          <t>DHAN-231261015159409+321261015672709+321261015673309+221261015677909+221261015678309+341261015154609+321261015675209+221261015678809+341261015155009+341261015155109+231261015160609+231261015160709+341261015155509</t>
         </is>
       </c>
       <c r="B46" s="23" t="inlineStr">
         <is>
-          <t>MBEL</t>
+          <t>TEAMLEASE</t>
         </is>
       </c>
       <c r="C46" s="23" t="inlineStr">
@@ -35213,24 +35229,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D46" s="24" t="inlineStr"/>
+      <c r="D46" s="24" t="n">
+        <v>46311</v>
+      </c>
       <c r="E46" s="4" t="n">
-        <v>0</v>
+        <v>109.45</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>0</v>
+        <v>593.96</v>
       </c>
       <c r="G46" s="4" t="n">
-        <v>0</v>
+        <v>18.23</v>
       </c>
       <c r="H46" s="4" t="n">
-        <v>0</v>
+        <v>0.59</v>
       </c>
       <c r="I46" s="4" t="n">
-        <v>0</v>
+        <v>44.73</v>
       </c>
       <c r="J46" s="4" t="n">
-        <v>0</v>
+        <v>23.09</v>
       </c>
       <c r="K46" s="4" t="n">
         <v>14.75</v>
@@ -35239,7 +35257,7 @@
         <v>35.4</v>
       </c>
       <c r="M46" s="4" t="n">
-        <v>0</v>
+        <v>32.48</v>
       </c>
       <c r="N46" s="21">
         <f>SUM(E46:M46)</f>
@@ -35249,12 +35267,12 @@
     <row r="47">
       <c r="A47" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261012625809+321261012626209+23126101284209+23126101284309+321261012626909+34126101276209+34126101277109+321261012628809+221261012640809+23126101286309+34126101278009+321261012630809+221261012643209</t>
+          <t>DHAN-321261016683609+23126101679509+23126101679909+321261016685009+221261016694409+221261016695109+34126101677409+321261016686809+23126101680709+321261016687809+23126101681009+34126101678009</t>
         </is>
       </c>
       <c r="B47" s="23" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>EUROPRATIK</t>
         </is>
       </c>
       <c r="C47" s="23" t="inlineStr">
@@ -35264,31 +35282,31 @@
       </c>
       <c r="D47" s="24" t="inlineStr"/>
       <c r="E47" s="4" t="n">
-        <v>24.76</v>
+        <v>89.59</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>3.4</v>
+        <v>298.62</v>
       </c>
       <c r="G47" s="4" t="n">
-        <v>2.63</v>
+        <v>9.17</v>
       </c>
       <c r="H47" s="4" t="n">
-        <v>0.09</v>
+        <v>0.3</v>
       </c>
       <c r="I47" s="4" t="n">
-        <v>3</v>
+        <v>44.79</v>
       </c>
       <c r="J47" s="4" t="n">
-        <v>4.95</v>
+        <v>17.83</v>
       </c>
       <c r="K47" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L47" s="4" t="n">
-        <v>0</v>
+        <v>35.4</v>
       </c>
       <c r="M47" s="4" t="n">
-        <v>0</v>
+        <v>183.83</v>
       </c>
       <c r="N47" s="21">
         <f>SUM(E47:M47)</f>
@@ -35298,12 +35316,12 @@
     <row r="48">
       <c r="A48" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261016683509+23126101679609+221261016693309+321261016685109+321261016685509+321261016685809+221261016695509+34126101677609+23126101680609+23126101680809+321261016688709+321261016689109+221261016697009+321261016690409</t>
+          <t>DHAN-221261016693009+23126101679709+23126101679809+23126101680009+321261016685409+221261016694909+34126101677509+321261016686909+34126101677709+321261016687909+34126101677909</t>
         </is>
       </c>
       <c r="B48" s="23" t="inlineStr">
         <is>
-          <t>PARACABLES</t>
+          <t>MBEL</t>
         </is>
       </c>
       <c r="C48" s="23" t="inlineStr">
@@ -35313,22 +35331,22 @@
       </c>
       <c r="D48" s="24" t="inlineStr"/>
       <c r="E48" s="4" t="n">
-        <v>0</v>
+        <v>90.11</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>0</v>
+        <v>300.22</v>
       </c>
       <c r="G48" s="4" t="n">
-        <v>0</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="H48" s="4" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="I48" s="4" t="n">
-        <v>0</v>
+        <v>45.03</v>
       </c>
       <c r="J48" s="4" t="n">
-        <v>0</v>
+        <v>17.93</v>
       </c>
       <c r="K48" s="4" t="n">
         <v>14.75</v>
@@ -35337,7 +35355,7 @@
         <v>35.4</v>
       </c>
       <c r="M48" s="4" t="n">
-        <v>0</v>
+        <v>184.81</v>
       </c>
       <c r="N48" s="21">
         <f>SUM(E48:M48)</f>
@@ -35347,12 +35365,12 @@
     <row r="49">
       <c r="A49" s="23" t="inlineStr">
         <is>
-          <t>DHAN-341261014128809+341261014129209+221261014671809+321261014664309+221261014672409+321261014664909+341261014130009+221261014673409+221261014673609+221261014673709+221261014674009+321261014667309+341261014130909</t>
+          <t>DHAN-321261016683509+23126101679609+221261016693309+321261016685109+321261016685509+321261016685809+221261016695509+34126101677609+23126101680609+23126101680809+321261016688709+321261016689109+221261016697009+321261016690409</t>
         </is>
       </c>
       <c r="B49" s="23" t="inlineStr">
         <is>
-          <t>SIMPLEXINF</t>
+          <t>PARACABLES</t>
         </is>
       </c>
       <c r="C49" s="23" t="inlineStr">
@@ -35362,22 +35380,22 @@
       </c>
       <c r="D49" s="24" t="inlineStr"/>
       <c r="E49" s="4" t="n">
-        <v>59.95</v>
+        <v>90.06</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>199.83</v>
+        <v>300.41</v>
       </c>
       <c r="G49" s="4" t="n">
-        <v>6.13</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="H49" s="4" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="I49" s="4" t="n">
-        <v>29.98</v>
+        <v>45.06</v>
       </c>
       <c r="J49" s="4" t="n">
-        <v>11.93</v>
+        <v>17.92</v>
       </c>
       <c r="K49" s="4" t="n">
         <v>14.75</v>
@@ -35386,7 +35404,7 @@
         <v>35.4</v>
       </c>
       <c r="M49" s="4" t="n">
-        <v>36.67</v>
+        <v>181.85</v>
       </c>
       <c r="N49" s="21">
         <f>SUM(E49:M49)</f>
@@ -35411,22 +35429,22 @@
       </c>
       <c r="D50" s="24" t="inlineStr"/>
       <c r="E50" s="4" t="n">
-        <v>0</v>
+        <v>90.25</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>0</v>
+        <v>300.81</v>
       </c>
       <c r="G50" s="4" t="n">
-        <v>0</v>
+        <v>9.23</v>
       </c>
       <c r="H50" s="4" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="I50" s="4" t="n">
-        <v>0</v>
+        <v>45.12</v>
       </c>
       <c r="J50" s="4" t="n">
-        <v>0</v>
+        <v>17.96</v>
       </c>
       <c r="K50" s="4" t="n">
         <v>14.75</v>
@@ -35435,7 +35453,7 @@
         <v>35.4</v>
       </c>
       <c r="M50" s="4" t="n">
-        <v>0</v>
+        <v>185.18</v>
       </c>
       <c r="N50" s="21">
         <f>SUM(E50:M50)</f>

</xml_diff>

<commit_message>
Data update — 2026-10-19 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_oct2026.xlsx
+++ b/results/strategy_pnl_oct2026.xlsx
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trade Log'!$A$3:$O$503</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$53</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -3659,8 +3659,12 @@
       <c r="F47" s="26" t="n">
         <v>1636</v>
       </c>
-      <c r="G47" s="24" t="inlineStr"/>
-      <c r="H47" s="25" t="inlineStr"/>
+      <c r="G47" s="24" t="n">
+        <v>46314</v>
+      </c>
+      <c r="H47" s="25" t="n">
+        <v>185</v>
+      </c>
       <c r="I47" s="21">
         <f>IF(OR($B47="",$H47=""),"",IF($C47="LONG",($H47-$E47)*$F47,($E47-$H47)*$F47))</f>
         <v/>
@@ -3715,8 +3719,12 @@
       <c r="F48" s="26" t="n">
         <v>1043</v>
       </c>
-      <c r="G48" s="24" t="inlineStr"/>
-      <c r="H48" s="25" t="inlineStr"/>
+      <c r="G48" s="24" t="n">
+        <v>46314</v>
+      </c>
+      <c r="H48" s="25" t="n">
+        <v>288.54</v>
+      </c>
       <c r="I48" s="21">
         <f>IF(OR($B48="",$H48=""),"",IF($C48="LONG",($H48-$E48)*$F48,($E48-$H48)*$F48))</f>
         <v/>
@@ -3771,8 +3779,12 @@
       <c r="F49" s="26" t="n">
         <v>4996</v>
       </c>
-      <c r="G49" s="24" t="inlineStr"/>
-      <c r="H49" s="25" t="inlineStr"/>
+      <c r="G49" s="24" t="n">
+        <v>46314</v>
+      </c>
+      <c r="H49" s="25" t="n">
+        <v>61.08</v>
+      </c>
       <c r="I49" s="21">
         <f>IF(OR($B49="",$H49=""),"",IF($C49="LONG",($H49-$E49)*$F49,($E49-$H49)*$F49))</f>
         <v/>
@@ -3827,8 +3839,12 @@
       <c r="F50" s="26" t="n">
         <v>434</v>
       </c>
-      <c r="G50" s="24" t="inlineStr"/>
-      <c r="H50" s="25" t="inlineStr"/>
+      <c r="G50" s="24" t="n">
+        <v>46314</v>
+      </c>
+      <c r="H50" s="25" t="n">
+        <v>705.59</v>
+      </c>
       <c r="I50" s="21">
         <f>IF(OR($B50="",$H50=""),"",IF($C50="LONG",($H50-$E50)*$F50,($E50-$H50)*$F50))</f>
         <v/>
@@ -3859,14 +3875,32 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="23" t="n"/>
-      <c r="B51" s="23" t="n"/>
-      <c r="C51" s="23" t="n"/>
-      <c r="D51" s="24" t="n"/>
-      <c r="E51" s="25" t="n"/>
-      <c r="F51" s="26" t="n"/>
-      <c r="G51" s="24" t="n"/>
-      <c r="H51" s="25" t="n"/>
+      <c r="A51" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126101987109+23126101991809+34126101987209+221261019598509+221261019598809+34126101987509+221261019599809+34126101987609+23126101992109+23126101992209+34126101987809+221261019601409</t>
+        </is>
+      </c>
+      <c r="B51" s="23" t="inlineStr">
+        <is>
+          <t>JAICORPLTD</t>
+        </is>
+      </c>
+      <c r="C51" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D51" s="24" t="n">
+        <v>46314</v>
+      </c>
+      <c r="E51" s="25" t="n">
+        <v>98.7749</v>
+      </c>
+      <c r="F51" s="26" t="n">
+        <v>3036</v>
+      </c>
+      <c r="G51" s="24" t="inlineStr"/>
+      <c r="H51" s="25" t="inlineStr"/>
       <c r="I51" s="21">
         <f>IF(OR($B51="",$H51=""),"",IF($C51="LONG",($H51-$E51)*$F51,($E51-$H51)*$F51))</f>
         <v/>
@@ -3875,7 +3909,9 @@
         <f>IF(OR($B51="",$I51="",$E51=0,$F51=0),"",$I51/($E51*$F51))</f>
         <v/>
       </c>
-      <c r="K51" s="4" t="n"/>
+      <c r="K51" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L51" s="21">
         <f>IF(OR($B51="",$I51=""),"",$I51-IF($K51="",0,$K51))</f>
         <v/>
@@ -3888,17 +3924,39 @@
         <f>IF($B51="","",IF($H51="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O51" s="23" t="n"/>
+      <c r="O51" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" s="23" t="n"/>
-      <c r="B52" s="23" t="n"/>
-      <c r="C52" s="23" t="n"/>
-      <c r="D52" s="24" t="n"/>
-      <c r="E52" s="25" t="n"/>
-      <c r="F52" s="26" t="n"/>
-      <c r="G52" s="24" t="n"/>
-      <c r="H52" s="25" t="n"/>
+      <c r="A52" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261019580109+321261019580509+321261019580809+221261019598309+221261019598909+34126101987409+221261019599909+321261019582809+221261019600309+321261019583209</t>
+        </is>
+      </c>
+      <c r="B52" s="23" t="inlineStr">
+        <is>
+          <t>KROSS</t>
+        </is>
+      </c>
+      <c r="C52" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D52" s="24" t="n">
+        <v>46314</v>
+      </c>
+      <c r="E52" s="25" t="n">
+        <v>299.18</v>
+      </c>
+      <c r="F52" s="26" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G52" s="24" t="inlineStr"/>
+      <c r="H52" s="25" t="inlineStr"/>
       <c r="I52" s="21">
         <f>IF(OR($B52="",$H52=""),"",IF($C52="LONG",($H52-$E52)*$F52,($E52-$H52)*$F52))</f>
         <v/>
@@ -3907,7 +3965,9 @@
         <f>IF(OR($B52="",$I52="",$E52=0,$F52=0),"",$I52/($E52*$F52))</f>
         <v/>
       </c>
-      <c r="K52" s="4" t="n"/>
+      <c r="K52" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L52" s="21">
         <f>IF(OR($B52="",$I52=""),"",$I52-IF($K52="",0,$K52))</f>
         <v/>
@@ -3920,17 +3980,39 @@
         <f>IF($B52="","",IF($H52="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O52" s="23" t="n"/>
+      <c r="O52" s="23" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" s="23" t="n"/>
-      <c r="B53" s="23" t="n"/>
-      <c r="C53" s="23" t="n"/>
-      <c r="D53" s="24" t="n"/>
-      <c r="E53" s="25" t="n"/>
-      <c r="F53" s="26" t="n"/>
-      <c r="G53" s="24" t="n"/>
-      <c r="H53" s="25" t="n"/>
+      <c r="A53" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261019597209+321261019580609+23126101992009+221261019598409+34126101987309+221261019599309+221261019599709+221261019600109+221261019600409+23126101992309+221261019601009+23126101992409+23126101992509+221261019602009</t>
+        </is>
+      </c>
+      <c r="B53" s="23" t="inlineStr">
+        <is>
+          <t>PARACABLES</t>
+        </is>
+      </c>
+      <c r="C53" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D53" s="24" t="n">
+        <v>46314</v>
+      </c>
+      <c r="E53" s="25" t="n">
+        <v>66.7538</v>
+      </c>
+      <c r="F53" s="26" t="n">
+        <v>2246</v>
+      </c>
+      <c r="G53" s="24" t="inlineStr"/>
+      <c r="H53" s="25" t="inlineStr"/>
       <c r="I53" s="21">
         <f>IF(OR($B53="",$H53=""),"",IF($C53="LONG",($H53-$E53)*$F53,($E53-$H53)*$F53))</f>
         <v/>
@@ -3939,7 +4021,9 @@
         <f>IF(OR($B53="",$I53="",$E53=0,$F53=0),"",$I53/($E53*$F53))</f>
         <v/>
       </c>
-      <c r="K53" s="4" t="n"/>
+      <c r="K53" s="4" t="n">
+        <v>14.75</v>
+      </c>
       <c r="L53" s="21">
         <f>IF(OR($B53="",$I53=""),"",$I53-IF($K53="",0,$K53))</f>
         <v/>
@@ -3952,7 +4036,11 @@
         <f>IF($B53="","",IF($H53="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O53" s="23" t="n"/>
+      <c r="O53" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="23" t="n"/>
@@ -32966,7 +33054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N51"/>
+  <dimension ref="A1:N54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -35280,7 +35368,9 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D47" s="24" t="inlineStr"/>
+      <c r="D47" s="24" t="n">
+        <v>46314</v>
+      </c>
       <c r="E47" s="4" t="n">
         <v>89.59</v>
       </c>
@@ -35329,7 +35419,9 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D48" s="24" t="inlineStr"/>
+      <c r="D48" s="24" t="n">
+        <v>46314</v>
+      </c>
       <c r="E48" s="4" t="n">
         <v>90.11</v>
       </c>
@@ -35378,7 +35470,9 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D49" s="24" t="inlineStr"/>
+      <c r="D49" s="24" t="n">
+        <v>46314</v>
+      </c>
       <c r="E49" s="4" t="n">
         <v>90.06</v>
       </c>
@@ -35427,7 +35521,9 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D50" s="24" t="inlineStr"/>
+      <c r="D50" s="24" t="n">
+        <v>46314</v>
+      </c>
       <c r="E50" s="4" t="n">
         <v>90.25</v>
       </c>
@@ -35461,54 +35557,201 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="3" t="inlineStr">
+      <c r="A51" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126101987109+23126101991809+34126101987209+221261019598509+221261019598809+34126101987509+221261019599809+34126101987609+23126101992109+23126101992209+34126101987809+221261019601409</t>
+        </is>
+      </c>
+      <c r="B51" s="23" t="inlineStr">
+        <is>
+          <t>JAICORPLTD</t>
+        </is>
+      </c>
+      <c r="C51" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D51" s="24" t="inlineStr"/>
+      <c r="E51" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I51" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J51" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K51" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L51" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M51" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N51" s="21">
+        <f>SUM(E51:M51)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261019580109+321261019580509+321261019580809+221261019598309+221261019598909+34126101987409+221261019599909+321261019582809+221261019600309+321261019583209</t>
+        </is>
+      </c>
+      <c r="B52" s="23" t="inlineStr">
+        <is>
+          <t>KROSS</t>
+        </is>
+      </c>
+      <c r="C52" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D52" s="24" t="inlineStr"/>
+      <c r="E52" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H52" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I52" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J52" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K52" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L52" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M52" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N52" s="21">
+        <f>SUM(E52:M52)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261019597209+321261019580609+23126101992009+221261019598409+34126101987309+221261019599309+221261019599709+221261019600109+221261019600409+23126101992309+221261019601009+23126101992409+23126101992509+221261019602009</t>
+        </is>
+      </c>
+      <c r="B53" s="23" t="inlineStr">
+        <is>
+          <t>PARACABLES</t>
+        </is>
+      </c>
+      <c r="C53" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D53" s="24" t="inlineStr"/>
+      <c r="E53" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H53" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I53" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J53" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K53" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L53" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M53" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N53" s="21">
+        <f>SUM(E53:M53)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E51" s="32">
-        <f>SUM(E4:E50)</f>
-        <v/>
-      </c>
-      <c r="F51" s="32">
-        <f>SUM(F4:F50)</f>
-        <v/>
-      </c>
-      <c r="G51" s="32">
-        <f>SUM(G4:G50)</f>
-        <v/>
-      </c>
-      <c r="H51" s="32">
-        <f>SUM(H4:H50)</f>
-        <v/>
-      </c>
-      <c r="I51" s="32">
-        <f>SUM(I4:I50)</f>
-        <v/>
-      </c>
-      <c r="J51" s="32">
-        <f>SUM(J4:J50)</f>
-        <v/>
-      </c>
-      <c r="K51" s="32">
-        <f>SUM(K4:K50)</f>
-        <v/>
-      </c>
-      <c r="L51" s="32">
-        <f>SUM(L4:L50)</f>
-        <v/>
-      </c>
-      <c r="M51" s="32">
-        <f>SUM(M4:M50)</f>
-        <v/>
-      </c>
-      <c r="N51" s="32">
-        <f>SUM(N4:N50)</f>
+      <c r="E54" s="32">
+        <f>SUM(E4:E53)</f>
+        <v/>
+      </c>
+      <c r="F54" s="32">
+        <f>SUM(F4:F53)</f>
+        <v/>
+      </c>
+      <c r="G54" s="32">
+        <f>SUM(G4:G53)</f>
+        <v/>
+      </c>
+      <c r="H54" s="32">
+        <f>SUM(H4:H53)</f>
+        <v/>
+      </c>
+      <c r="I54" s="32">
+        <f>SUM(I4:I53)</f>
+        <v/>
+      </c>
+      <c r="J54" s="32">
+        <f>SUM(J4:J53)</f>
+        <v/>
+      </c>
+      <c r="K54" s="32">
+        <f>SUM(K4:K53)</f>
+        <v/>
+      </c>
+      <c r="L54" s="32">
+        <f>SUM(L4:L53)</f>
+        <v/>
+      </c>
+      <c r="M54" s="32">
+        <f>SUM(M4:M53)</f>
+        <v/>
+      </c>
+      <c r="N54" s="32">
+        <f>SUM(N4:N53)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:N50"/>
+  <autoFilter ref="A3:N53"/>
   <mergeCells count="2">
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>
@@ -35523,7 +35766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -35858,40 +36101,85 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="28" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B12" s="20">
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,19),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,26))</f>
+        <v/>
+      </c>
+      <c r="C12" s="20">
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,19),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,26),'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D12" s="20">
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,19),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,26),'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E12" s="22">
+        <f>IFERROR($C12/$B12,"")</f>
+        <v/>
+      </c>
+      <c r="F12" s="21">
+        <f>SUMIFS('Trade Log'!$I$4:$I$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,19),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,26))</f>
+        <v/>
+      </c>
+      <c r="G12" s="21">
+        <f>SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,19),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,26))</f>
+        <v/>
+      </c>
+      <c r="H12" s="21">
+        <f>IFERROR($G12/$B12,"")</f>
+        <v/>
+      </c>
+      <c r="I12" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,19),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,26)),"")</f>
+        <v/>
+      </c>
+      <c r="J12" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,19),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,26)),"")</f>
+        <v/>
+      </c>
+      <c r="K12" s="29">
+        <f>IFERROR(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,19),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,26),'Trade Log'!$L$4:$L$503,"&gt;0")/ABS(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,19),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,26),'Trade Log'!$L$4:$L$503,"&lt;0")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B12" s="30">
-        <f>SUM(B10:B11)</f>
-        <v/>
-      </c>
-      <c r="C12" s="30">
-        <f>SUM(C10:C11)</f>
-        <v/>
-      </c>
-      <c r="D12" s="30">
-        <f>SUM(D10:D11)</f>
-        <v/>
-      </c>
-      <c r="E12" s="31">
-        <f>IFERROR(C12/B12,"")</f>
-        <v/>
-      </c>
-      <c r="F12" s="32">
-        <f>SUM(F10:F11)</f>
-        <v/>
-      </c>
-      <c r="G12" s="32">
-        <f>SUM(G10:G11)</f>
-        <v/>
-      </c>
-      <c r="H12" s="32">
-        <f>IFERROR(G12/B12,"")</f>
-        <v/>
-      </c>
-      <c r="K12" s="33">
+      <c r="B13" s="30">
+        <f>SUM(B10:B12)</f>
+        <v/>
+      </c>
+      <c r="C13" s="30">
+        <f>SUM(C10:C12)</f>
+        <v/>
+      </c>
+      <c r="D13" s="30">
+        <f>SUM(D10:D12)</f>
+        <v/>
+      </c>
+      <c r="E13" s="31">
+        <f>IFERROR(C13/B13,"")</f>
+        <v/>
+      </c>
+      <c r="F13" s="32">
+        <f>SUM(F10:F12)</f>
+        <v/>
+      </c>
+      <c r="G13" s="32">
+        <f>SUM(G10:G12)</f>
+        <v/>
+      </c>
+      <c r="H13" s="32">
+        <f>IFERROR(G13/B13,"")</f>
+        <v/>
+      </c>
+      <c r="K13" s="33">
         <f>IFERROR(SUMIF('Trade Log'!$L$4:$L$503,"&gt;0")/ABS(SUMIF('Trade Log'!$L$4:$L$503,"&lt;0")),"")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Data update — 2026-10-21 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_oct2026.xlsx
+++ b/results/strategy_pnl_oct2026.xlsx
@@ -1214,7 +1214,7 @@
         <v/>
       </c>
       <c r="K6" s="4" t="n">
-        <v>956.73</v>
+        <v>955</v>
       </c>
       <c r="L6" s="21">
         <f>IF(OR($B6="",$I6=""),"",$I6-IF($K6="",0,$K6))</f>
@@ -1274,7 +1274,7 @@
         <v/>
       </c>
       <c r="K7" s="4" t="n">
-        <v>820.0599999999999</v>
+        <v>819.03</v>
       </c>
       <c r="L7" s="21">
         <f>IF(OR($B7="",$I7=""),"",$I7-IF($K7="",0,$K7))</f>
@@ -1334,7 +1334,7 @@
         <v/>
       </c>
       <c r="K8" s="4" t="n">
-        <v>858.7</v>
+        <v>857.26</v>
       </c>
       <c r="L8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($K8="",0,$K8))</f>
@@ -1394,7 +1394,7 @@
         <v/>
       </c>
       <c r="K9" s="4" t="n">
-        <v>971.1900000000001</v>
+        <v>969.47</v>
       </c>
       <c r="L9" s="21">
         <f>IF(OR($B9="",$I9=""),"",$I9-IF($K9="",0,$K9))</f>
@@ -1454,7 +1454,7 @@
         <v/>
       </c>
       <c r="K10" s="4" t="n">
-        <v>944.47</v>
+        <v>943.03</v>
       </c>
       <c r="L10" s="21">
         <f>IF(OR($B10="",$I10=""),"",$I10-IF($K10="",0,$K10))</f>
@@ -1514,7 +1514,7 @@
         <v/>
       </c>
       <c r="K11" s="4" t="n">
-        <v>692.8099999999999</v>
+        <v>691.4</v>
       </c>
       <c r="L11" s="21">
         <f>IF(OR($B11="",$I11=""),"",$I11-IF($K11="",0,$K11))</f>
@@ -1574,7 +1574,7 @@
         <v/>
       </c>
       <c r="K12" s="4" t="n">
-        <v>758.24</v>
+        <v>756.54</v>
       </c>
       <c r="L12" s="21">
         <f>IF(OR($B12="",$I12=""),"",$I12-IF($K12="",0,$K12))</f>
@@ -1634,7 +1634,7 @@
         <v/>
       </c>
       <c r="K13" s="4" t="n">
-        <v>689.8</v>
+        <v>688.12</v>
       </c>
       <c r="L13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($K13="",0,$K13))</f>
@@ -1694,7 +1694,7 @@
         <v/>
       </c>
       <c r="K14" s="4" t="n">
-        <v>668.37</v>
+        <v>684</v>
       </c>
       <c r="L14" s="21">
         <f>IF(OR($B14="",$I14=""),"",$I14-IF($K14="",0,$K14))</f>
@@ -1874,7 +1874,7 @@
         <v/>
       </c>
       <c r="K17" s="4" t="n">
-        <v>629.97</v>
+        <v>661.51</v>
       </c>
       <c r="L17" s="21">
         <f>IF(OR($B17="",$I17=""),"",$I17-IF($K17="",0,$K17))</f>
@@ -1994,7 +1994,7 @@
         <v/>
       </c>
       <c r="K19" s="4" t="n">
-        <v>670.55</v>
+        <v>667.13</v>
       </c>
       <c r="L19" s="21">
         <f>IF(OR($B19="",$I19=""),"",$I19-IF($K19="",0,$K19))</f>
@@ -2054,7 +2054,7 @@
         <v/>
       </c>
       <c r="K20" s="4" t="n">
-        <v>680.79</v>
+        <v>677.4299999999999</v>
       </c>
       <c r="L20" s="21">
         <f>IF(OR($B20="",$I20=""),"",$I20-IF($K20="",0,$K20))</f>
@@ -2174,7 +2174,7 @@
         <v/>
       </c>
       <c r="K22" s="4" t="n">
-        <v>662.41</v>
+        <v>659.03</v>
       </c>
       <c r="L22" s="21">
         <f>IF(OR($B22="",$I22=""),"",$I22-IF($K22="",0,$K22))</f>
@@ -2234,7 +2234,7 @@
         <v/>
       </c>
       <c r="K23" s="4" t="n">
-        <v>421.06</v>
+        <v>419.86</v>
       </c>
       <c r="L23" s="21">
         <f>IF(OR($B23="",$I23=""),"",$I23-IF($K23="",0,$K23))</f>
@@ -2354,7 +2354,7 @@
         <v/>
       </c>
       <c r="K25" s="4" t="n">
-        <v>558.99</v>
+        <v>557.52</v>
       </c>
       <c r="L25" s="21">
         <f>IF(OR($B25="",$I25=""),"",$I25-IF($K25="",0,$K25))</f>
@@ -2474,7 +2474,7 @@
         <v/>
       </c>
       <c r="K27" s="4" t="n">
-        <v>549.26</v>
+        <v>547.8200000000001</v>
       </c>
       <c r="L27" s="21">
         <f>IF(OR($B27="",$I27=""),"",$I27-IF($K27="",0,$K27))</f>
@@ -2534,7 +2534,7 @@
         <v/>
       </c>
       <c r="K28" s="4" t="n">
-        <v>549.76</v>
+        <v>548.12</v>
       </c>
       <c r="L28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($K28="",0,$K28))</f>
@@ -2594,7 +2594,7 @@
         <v/>
       </c>
       <c r="K29" s="4" t="n">
-        <v>556.86</v>
+        <v>555.04</v>
       </c>
       <c r="L29" s="21">
         <f>IF(OR($B29="",$I29=""),"",$I29-IF($K29="",0,$K29))</f>
@@ -2654,7 +2654,7 @@
         <v/>
       </c>
       <c r="K30" s="4" t="n">
-        <v>552.38</v>
+        <v>550.9400000000001</v>
       </c>
       <c r="L30" s="21">
         <f>IF(OR($B30="",$I30=""),"",$I30-IF($K30="",0,$K30))</f>
@@ -2834,7 +2834,7 @@
         <v/>
       </c>
       <c r="K33" s="4" t="n">
-        <v>552.51</v>
+        <v>551.08</v>
       </c>
       <c r="L33" s="21">
         <f>IF(OR($B33="",$I33=""),"",$I33-IF($K33="",0,$K33))</f>
@@ -2894,7 +2894,7 @@
         <v/>
       </c>
       <c r="K34" s="4" t="n">
-        <v>427.71</v>
+        <v>426.23</v>
       </c>
       <c r="L34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($K34="",0,$K34))</f>
@@ -3014,7 +3014,7 @@
         <v/>
       </c>
       <c r="K36" s="4" t="n">
-        <v>539.8</v>
+        <v>538.9400000000001</v>
       </c>
       <c r="L36" s="21">
         <f>IF(OR($B36="",$I36=""),"",$I36-IF($K36="",0,$K36))</f>
@@ -3074,7 +3074,7 @@
         <v/>
       </c>
       <c r="K37" s="4" t="n">
-        <v>479.82</v>
+        <v>478.55</v>
       </c>
       <c r="L37" s="21">
         <f>IF(OR($B37="",$I37=""),"",$I37-IF($K37="",0,$K37))</f>
@@ -3134,7 +3134,7 @@
         <v/>
       </c>
       <c r="K38" s="4" t="n">
-        <v>625.6799999999999</v>
+        <v>624.29</v>
       </c>
       <c r="L38" s="21">
         <f>IF(OR($B38="",$I38=""),"",$I38-IF($K38="",0,$K38))</f>
@@ -3194,7 +3194,7 @@
         <v/>
       </c>
       <c r="K39" s="4" t="n">
-        <v>615.62</v>
+        <v>614.23</v>
       </c>
       <c r="L39" s="21">
         <f>IF(OR($B39="",$I39=""),"",$I39-IF($K39="",0,$K39))</f>
@@ -3314,7 +3314,7 @@
         <v/>
       </c>
       <c r="K41" s="4" t="n">
-        <v>394.45</v>
+        <v>393.06</v>
       </c>
       <c r="L41" s="21">
         <f>IF(OR($B41="",$I41=""),"",$I41-IF($K41="",0,$K41))</f>
@@ -3374,7 +3374,7 @@
         <v/>
       </c>
       <c r="K42" s="4" t="n">
-        <v>626.9299999999999</v>
+        <v>625.53</v>
       </c>
       <c r="L42" s="21">
         <f>IF(OR($B42="",$I42=""),"",$I42-IF($K42="",0,$K42))</f>
@@ -3434,7 +3434,7 @@
         <v/>
       </c>
       <c r="K43" s="4" t="n">
-        <v>878.86</v>
+        <v>877.37</v>
       </c>
       <c r="L43" s="21">
         <f>IF(OR($B43="",$I43=""),"",$I43-IF($K43="",0,$K43))</f>
@@ -3554,7 +3554,7 @@
         <v/>
       </c>
       <c r="K45" s="4" t="n">
-        <v>896.95</v>
+        <v>895.52</v>
       </c>
       <c r="L45" s="21">
         <f>IF(OR($B45="",$I45=""),"",$I45-IF($K45="",0,$K45))</f>
@@ -3614,7 +3614,7 @@
         <v/>
       </c>
       <c r="K46" s="4" t="n">
-        <v>872.6900000000001</v>
+        <v>871.4400000000001</v>
       </c>
       <c r="L46" s="21">
         <f>IF(OR($B46="",$I46=""),"",$I46-IF($K46="",0,$K46))</f>
@@ -3674,7 +3674,7 @@
         <v/>
       </c>
       <c r="K47" s="4" t="n">
-        <v>694.27</v>
+        <v>1031.86</v>
       </c>
       <c r="L47" s="21">
         <f>IF(OR($B47="",$I47=""),"",$I47-IF($K47="",0,$K47))</f>
@@ -3734,7 +3734,7 @@
         <v/>
       </c>
       <c r="K48" s="4" t="n">
-        <v>697.77</v>
+        <v>1033.58</v>
       </c>
       <c r="L48" s="21">
         <f>IF(OR($B48="",$I48=""),"",$I48-IF($K48="",0,$K48))</f>
@@ -3794,7 +3794,7 @@
         <v/>
       </c>
       <c r="K49" s="4" t="n">
-        <v>694.98</v>
+        <v>960.61</v>
       </c>
       <c r="L49" s="21">
         <f>IF(OR($B49="",$I49=""),"",$I49-IF($K49="",0,$K49))</f>
@@ -3854,7 +3854,7 @@
         <v/>
       </c>
       <c r="K50" s="4" t="n">
-        <v>699</v>
+        <v>1040.29</v>
       </c>
       <c r="L50" s="21">
         <f>IF(OR($B50="",$I50=""),"",$I50-IF($K50="",0,$K50))</f>
@@ -3899,8 +3899,12 @@
       <c r="F51" s="26" t="n">
         <v>3036</v>
       </c>
-      <c r="G51" s="24" t="inlineStr"/>
-      <c r="H51" s="25" t="inlineStr"/>
+      <c r="G51" s="24" t="n">
+        <v>46316</v>
+      </c>
+      <c r="H51" s="25" t="n">
+        <v>97.3</v>
+      </c>
       <c r="I51" s="21">
         <f>IF(OR($B51="",$H51=""),"",IF($C51="LONG",($H51-$E51)*$F51,($E51-$H51)*$F51))</f>
         <v/>
@@ -3910,7 +3914,7 @@
         <v/>
       </c>
       <c r="K51" s="4" t="n">
-        <v>50.15</v>
+        <v>642.47</v>
       </c>
       <c r="L51" s="21">
         <f>IF(OR($B51="",$I51=""),"",$I51-IF($K51="",0,$K51))</f>
@@ -3955,8 +3959,12 @@
       <c r="F52" s="26" t="n">
         <v>1000</v>
       </c>
-      <c r="G52" s="24" t="inlineStr"/>
-      <c r="H52" s="25" t="inlineStr"/>
+      <c r="G52" s="24" t="n">
+        <v>46316</v>
+      </c>
+      <c r="H52" s="25" t="n">
+        <v>282.49</v>
+      </c>
       <c r="I52" s="21">
         <f>IF(OR($B52="",$H52=""),"",IF($C52="LONG",($H52-$E52)*$F52,($E52-$H52)*$F52))</f>
         <v/>
@@ -3966,7 +3974,7 @@
         <v/>
       </c>
       <c r="K52" s="4" t="n">
-        <v>50.15</v>
+        <v>613.63</v>
       </c>
       <c r="L52" s="21">
         <f>IF(OR($B52="",$I52=""),"",$I52-IF($K52="",0,$K52))</f>
@@ -4011,8 +4019,12 @@
       <c r="F53" s="26" t="n">
         <v>2246</v>
       </c>
-      <c r="G53" s="24" t="inlineStr"/>
-      <c r="H53" s="25" t="inlineStr"/>
+      <c r="G53" s="24" t="n">
+        <v>46316</v>
+      </c>
+      <c r="H53" s="25" t="n">
+        <v>66.8359</v>
+      </c>
       <c r="I53" s="21">
         <f>IF(OR($B53="",$H53=""),"",IF($C53="LONG",($H53-$E53)*$F53,($E53-$H53)*$F53))</f>
         <v/>
@@ -4022,7 +4034,7 @@
         <v/>
       </c>
       <c r="K53" s="4" t="n">
-        <v>14.75</v>
+        <v>77.89</v>
       </c>
       <c r="L53" s="21">
         <f>IF(OR($B53="",$I53=""),"",$I53-IF($K53="",0,$K53))</f>
@@ -33305,7 +33317,7 @@
         <v>35.4</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>117.71</v>
+        <v>115.98</v>
       </c>
       <c r="N6" s="21">
         <f>SUM(E6:M6)</f>
@@ -33356,7 +33368,7 @@
         <v>35.4</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>70.38</v>
+        <v>69.34999999999999</v>
       </c>
       <c r="N7" s="21">
         <f>SUM(E7:M7)</f>
@@ -33407,7 +33419,7 @@
         <v>35.4</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>97.94</v>
+        <v>96.5</v>
       </c>
       <c r="N8" s="21">
         <f>SUM(E8:M8)</f>
@@ -33458,7 +33470,7 @@
         <v>35.4</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>117.38</v>
+        <v>115.66</v>
       </c>
       <c r="N9" s="21">
         <f>SUM(E9:M9)</f>
@@ -33509,7 +33521,7 @@
         <v>35.4</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>97.95</v>
+        <v>96.51000000000001</v>
       </c>
       <c r="N10" s="21">
         <f>SUM(E10:M10)</f>
@@ -33560,7 +33572,7 @@
         <v>35.4</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>61.07</v>
+        <v>59.66</v>
       </c>
       <c r="N11" s="21">
         <f>SUM(E11:M11)</f>
@@ -33611,7 +33623,7 @@
         <v>35.4</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>73.19</v>
+        <v>71.48999999999999</v>
       </c>
       <c r="N12" s="21">
         <f>SUM(E12:M12)</f>
@@ -33662,7 +33674,7 @@
         <v>35.4</v>
       </c>
       <c r="M13" s="4" t="n">
-        <v>74.84</v>
+        <v>73.15000000000001</v>
       </c>
       <c r="N13" s="21">
         <f>SUM(E13:M13)</f>
@@ -33713,7 +33725,7 @@
         <v>35.4</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>43.83</v>
+        <v>59.47</v>
       </c>
       <c r="N14" s="21">
         <f>SUM(E14:M14)</f>
@@ -33866,7 +33878,7 @@
         <v>35.4</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>52.34</v>
+        <v>83.88</v>
       </c>
       <c r="N17" s="21">
         <f>SUM(E17:M17)</f>
@@ -33968,7 +33980,7 @@
         <v>35.4</v>
       </c>
       <c r="M19" s="4" t="n">
-        <v>90.37</v>
+        <v>86.95</v>
       </c>
       <c r="N19" s="21">
         <f>SUM(E19:M19)</f>
@@ -34019,7 +34031,7 @@
         <v>35.4</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>87.34</v>
+        <v>83.98</v>
       </c>
       <c r="N20" s="21">
         <f>SUM(E20:M20)</f>
@@ -34121,7 +34133,7 @@
         <v>35.4</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>87.75</v>
+        <v>84.38</v>
       </c>
       <c r="N22" s="21">
         <f>SUM(E22:M22)</f>
@@ -34172,7 +34184,7 @@
         <v>35.4</v>
       </c>
       <c r="M23" s="4" t="n">
-        <v>31.25</v>
+        <v>30.05</v>
       </c>
       <c r="N23" s="21">
         <f>SUM(E23:M23)</f>
@@ -34274,7 +34286,7 @@
         <v>35.4</v>
       </c>
       <c r="M25" s="4" t="n">
-        <v>38.79</v>
+        <v>37.32</v>
       </c>
       <c r="N25" s="21">
         <f>SUM(E25:M25)</f>
@@ -34376,7 +34388,7 @@
         <v>35.4</v>
       </c>
       <c r="M27" s="4" t="n">
-        <v>37.37</v>
+        <v>35.93</v>
       </c>
       <c r="N27" s="21">
         <f>SUM(E27:M27)</f>
@@ -34427,7 +34439,7 @@
         <v>35.4</v>
       </c>
       <c r="M28" s="4" t="n">
-        <v>42.79</v>
+        <v>41.14</v>
       </c>
       <c r="N28" s="21">
         <f>SUM(E28:M28)</f>
@@ -34478,7 +34490,7 @@
         <v>35.4</v>
       </c>
       <c r="M29" s="4" t="n">
-        <v>44.86</v>
+        <v>43.04</v>
       </c>
       <c r="N29" s="21">
         <f>SUM(E29:M29)</f>
@@ -34529,7 +34541,7 @@
         <v>35.4</v>
       </c>
       <c r="M30" s="4" t="n">
-        <v>37.34</v>
+        <v>35.9</v>
       </c>
       <c r="N30" s="21">
         <f>SUM(E30:M30)</f>
@@ -34682,7 +34694,7 @@
         <v>35.4</v>
       </c>
       <c r="M33" s="4" t="n">
-        <v>37.05</v>
+        <v>35.62</v>
       </c>
       <c r="N33" s="21">
         <f>SUM(E33:M33)</f>
@@ -34733,7 +34745,7 @@
         <v>35.4</v>
       </c>
       <c r="M34" s="4" t="n">
-        <v>39.41</v>
+        <v>37.92</v>
       </c>
       <c r="N34" s="21">
         <f>SUM(E34:M34)</f>
@@ -34835,7 +34847,7 @@
         <v>35.4</v>
       </c>
       <c r="M36" s="4" t="n">
-        <v>22.37</v>
+        <v>21.51</v>
       </c>
       <c r="N36" s="21">
         <f>SUM(E36:M36)</f>
@@ -34886,7 +34898,7 @@
         <v>35.4</v>
       </c>
       <c r="M37" s="4" t="n">
-        <v>33.37</v>
+        <v>32.1</v>
       </c>
       <c r="N37" s="21">
         <f>SUM(E37:M37)</f>
@@ -34937,7 +34949,7 @@
         <v>35.4</v>
       </c>
       <c r="M38" s="4" t="n">
-        <v>36.33</v>
+        <v>34.93</v>
       </c>
       <c r="N38" s="21">
         <f>SUM(E38:M38)</f>
@@ -34988,7 +35000,7 @@
         <v>35.4</v>
       </c>
       <c r="M39" s="4" t="n">
-        <v>36.09</v>
+        <v>34.71</v>
       </c>
       <c r="N39" s="21">
         <f>SUM(E39:M39)</f>
@@ -35090,7 +35102,7 @@
         <v>35.4</v>
       </c>
       <c r="M41" s="4" t="n">
-        <v>36.28</v>
+        <v>34.88</v>
       </c>
       <c r="N41" s="21">
         <f>SUM(E41:M41)</f>
@@ -35141,7 +35153,7 @@
         <v>35.4</v>
       </c>
       <c r="M42" s="4" t="n">
-        <v>36.33</v>
+        <v>34.93</v>
       </c>
       <c r="N42" s="21">
         <f>SUM(E42:M42)</f>
@@ -35192,7 +35204,7 @@
         <v>35.4</v>
       </c>
       <c r="M43" s="4" t="n">
-        <v>34.76</v>
+        <v>33.27</v>
       </c>
       <c r="N43" s="21">
         <f>SUM(E43:M43)</f>
@@ -35294,7 +35306,7 @@
         <v>35.4</v>
       </c>
       <c r="M45" s="4" t="n">
-        <v>36.78</v>
+        <v>35.35</v>
       </c>
       <c r="N45" s="21">
         <f>SUM(E45:M45)</f>
@@ -35345,7 +35357,7 @@
         <v>35.4</v>
       </c>
       <c r="M46" s="4" t="n">
-        <v>32.48</v>
+        <v>31.23</v>
       </c>
       <c r="N46" s="21">
         <f>SUM(E46:M46)</f>
@@ -35372,22 +35384,22 @@
         <v>46314</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>89.59</v>
+        <v>109.59</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>298.62</v>
+        <v>601.3</v>
       </c>
       <c r="G47" s="4" t="n">
-        <v>9.17</v>
+        <v>18.46</v>
       </c>
       <c r="H47" s="4" t="n">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="I47" s="4" t="n">
         <v>44.79</v>
       </c>
       <c r="J47" s="4" t="n">
-        <v>17.83</v>
+        <v>23.16</v>
       </c>
       <c r="K47" s="4" t="n">
         <v>14.75</v>
@@ -35423,22 +35435,22 @@
         <v>46314</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>90.11</v>
+        <v>110.11</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>300.22</v>
+        <v>601.17</v>
       </c>
       <c r="G48" s="4" t="n">
-        <v>9.220000000000001</v>
+        <v>18.46</v>
       </c>
       <c r="H48" s="4" t="n">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="I48" s="4" t="n">
         <v>45.03</v>
       </c>
       <c r="J48" s="4" t="n">
-        <v>17.93</v>
+        <v>23.25</v>
       </c>
       <c r="K48" s="4" t="n">
         <v>14.75</v>
@@ -35474,22 +35486,22 @@
         <v>46314</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>90.06</v>
+        <v>130.06</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>300.41</v>
+        <v>508.5</v>
       </c>
       <c r="G49" s="4" t="n">
-        <v>9.220000000000001</v>
+        <v>18.59</v>
       </c>
       <c r="H49" s="4" t="n">
-        <v>0.3</v>
+        <v>0.61</v>
       </c>
       <c r="I49" s="4" t="n">
         <v>45.06</v>
       </c>
       <c r="J49" s="4" t="n">
-        <v>17.92</v>
+        <v>26.87</v>
       </c>
       <c r="K49" s="4" t="n">
         <v>14.75</v>
@@ -35498,7 +35510,7 @@
         <v>35.4</v>
       </c>
       <c r="M49" s="4" t="n">
-        <v>181.85</v>
+        <v>180.77</v>
       </c>
       <c r="N49" s="21">
         <f>SUM(E49:M49)</f>
@@ -35525,22 +35537,22 @@
         <v>46314</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>90.25</v>
+        <v>110.25</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>300.81</v>
+        <v>607.04</v>
       </c>
       <c r="G50" s="4" t="n">
-        <v>9.23</v>
+        <v>18.64</v>
       </c>
       <c r="H50" s="4" t="n">
-        <v>0.3</v>
+        <v>0.61</v>
       </c>
       <c r="I50" s="4" t="n">
         <v>45.12</v>
       </c>
       <c r="J50" s="4" t="n">
-        <v>17.96</v>
+        <v>23.31</v>
       </c>
       <c r="K50" s="4" t="n">
         <v>14.75</v>
@@ -35572,24 +35584,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D51" s="24" t="inlineStr"/>
+      <c r="D51" s="24" t="n">
+        <v>46316</v>
+      </c>
       <c r="E51" s="4" t="n">
-        <v>0</v>
+        <v>89.95999999999999</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>0</v>
+        <v>299.87</v>
       </c>
       <c r="G51" s="4" t="n">
-        <v>0</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="H51" s="4" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="I51" s="4" t="n">
-        <v>0</v>
+        <v>44.62</v>
       </c>
       <c r="J51" s="4" t="n">
-        <v>0</v>
+        <v>17.9</v>
       </c>
       <c r="K51" s="4" t="n">
         <v>14.75</v>
@@ -35598,7 +35612,7 @@
         <v>35.4</v>
       </c>
       <c r="M51" s="4" t="n">
-        <v>0</v>
+        <v>130.46</v>
       </c>
       <c r="N51" s="21">
         <f>SUM(E51:M51)</f>
@@ -35621,24 +35635,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D52" s="24" t="inlineStr"/>
+      <c r="D52" s="24" t="n">
+        <v>46316</v>
+      </c>
       <c r="E52" s="4" t="n">
-        <v>0</v>
+        <v>89.75</v>
       </c>
       <c r="F52" s="4" t="n">
-        <v>0</v>
+        <v>299.18</v>
       </c>
       <c r="G52" s="4" t="n">
-        <v>0</v>
+        <v>9.18</v>
       </c>
       <c r="H52" s="4" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="I52" s="4" t="n">
-        <v>0</v>
+        <v>44.88</v>
       </c>
       <c r="J52" s="4" t="n">
-        <v>0</v>
+        <v>17.86</v>
       </c>
       <c r="K52" s="4" t="n">
         <v>14.75</v>
@@ -35647,7 +35663,7 @@
         <v>35.4</v>
       </c>
       <c r="M52" s="4" t="n">
-        <v>0</v>
+        <v>102.32</v>
       </c>
       <c r="N52" s="21">
         <f>SUM(E52:M52)</f>
@@ -35670,24 +35686,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D53" s="24" t="inlineStr"/>
+      <c r="D53" s="24" t="n">
+        <v>46316</v>
+      </c>
       <c r="E53" s="4" t="n">
-        <v>0</v>
+        <v>44.94</v>
       </c>
       <c r="F53" s="4" t="n">
         <v>0</v>
       </c>
       <c r="G53" s="4" t="n">
-        <v>0</v>
+        <v>4.6</v>
       </c>
       <c r="H53" s="4" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="I53" s="4" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="J53" s="4" t="n">
-        <v>0</v>
+        <v>8.94</v>
       </c>
       <c r="K53" s="4" t="n">
         <v>14.75</v>

</xml_diff>

<commit_message>
Data update — 2026-10-22 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_oct2026.xlsx
+++ b/results/strategy_pnl_oct2026.xlsx
@@ -1394,7 +1394,7 @@
         <v/>
       </c>
       <c r="K9" s="4" t="n">
-        <v>969.47</v>
+        <v>969.46</v>
       </c>
       <c r="L9" s="21">
         <f>IF(OR($B9="",$I9=""),"",$I9-IF($K9="",0,$K9))</f>
@@ -1454,7 +1454,7 @@
         <v/>
       </c>
       <c r="K10" s="4" t="n">
-        <v>943.03</v>
+        <v>943.02</v>
       </c>
       <c r="L10" s="21">
         <f>IF(OR($B10="",$I10=""),"",$I10-IF($K10="",0,$K10))</f>
@@ -1514,7 +1514,7 @@
         <v/>
       </c>
       <c r="K11" s="4" t="n">
-        <v>691.4</v>
+        <v>691.54</v>
       </c>
       <c r="L11" s="21">
         <f>IF(OR($B11="",$I11=""),"",$I11-IF($K11="",0,$K11))</f>
@@ -1574,7 +1574,7 @@
         <v/>
       </c>
       <c r="K12" s="4" t="n">
-        <v>756.54</v>
+        <v>756.71</v>
       </c>
       <c r="L12" s="21">
         <f>IF(OR($B12="",$I12=""),"",$I12-IF($K12="",0,$K12))</f>
@@ -1634,7 +1634,7 @@
         <v/>
       </c>
       <c r="K13" s="4" t="n">
-        <v>688.12</v>
+        <v>688.36</v>
       </c>
       <c r="L13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($K13="",0,$K13))</f>
@@ -1694,7 +1694,7 @@
         <v/>
       </c>
       <c r="K14" s="4" t="n">
-        <v>684</v>
+        <v>684.15</v>
       </c>
       <c r="L14" s="21">
         <f>IF(OR($B14="",$I14=""),"",$I14-IF($K14="",0,$K14))</f>
@@ -1874,7 +1874,7 @@
         <v/>
       </c>
       <c r="K17" s="4" t="n">
-        <v>661.51</v>
+        <v>662.09</v>
       </c>
       <c r="L17" s="21">
         <f>IF(OR($B17="",$I17=""),"",$I17-IF($K17="",0,$K17))</f>
@@ -1994,7 +1994,7 @@
         <v/>
       </c>
       <c r="K19" s="4" t="n">
-        <v>667.13</v>
+        <v>667.79</v>
       </c>
       <c r="L19" s="21">
         <f>IF(OR($B19="",$I19=""),"",$I19-IF($K19="",0,$K19))</f>
@@ -2054,7 +2054,7 @@
         <v/>
       </c>
       <c r="K20" s="4" t="n">
-        <v>677.4299999999999</v>
+        <v>678.01</v>
       </c>
       <c r="L20" s="21">
         <f>IF(OR($B20="",$I20=""),"",$I20-IF($K20="",0,$K20))</f>
@@ -2174,7 +2174,7 @@
         <v/>
       </c>
       <c r="K22" s="4" t="n">
-        <v>659.03</v>
+        <v>659.61</v>
       </c>
       <c r="L22" s="21">
         <f>IF(OR($B22="",$I22=""),"",$I22-IF($K22="",0,$K22))</f>
@@ -2234,7 +2234,7 @@
         <v/>
       </c>
       <c r="K23" s="4" t="n">
-        <v>419.86</v>
+        <v>420.06</v>
       </c>
       <c r="L23" s="21">
         <f>IF(OR($B23="",$I23=""),"",$I23-IF($K23="",0,$K23))</f>
@@ -2354,7 +2354,7 @@
         <v/>
       </c>
       <c r="K25" s="4" t="n">
-        <v>557.52</v>
+        <v>557.8099999999999</v>
       </c>
       <c r="L25" s="21">
         <f>IF(OR($B25="",$I25=""),"",$I25-IF($K25="",0,$K25))</f>
@@ -2474,7 +2474,7 @@
         <v/>
       </c>
       <c r="K27" s="4" t="n">
-        <v>547.8200000000001</v>
+        <v>548.0700000000001</v>
       </c>
       <c r="L27" s="21">
         <f>IF(OR($B27="",$I27=""),"",$I27-IF($K27="",0,$K27))</f>
@@ -2534,7 +2534,7 @@
         <v/>
       </c>
       <c r="K28" s="4" t="n">
-        <v>548.12</v>
+        <v>548.4</v>
       </c>
       <c r="L28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($K28="",0,$K28))</f>
@@ -2594,7 +2594,7 @@
         <v/>
       </c>
       <c r="K29" s="4" t="n">
-        <v>555.04</v>
+        <v>555.1900000000001</v>
       </c>
       <c r="L29" s="21">
         <f>IF(OR($B29="",$I29=""),"",$I29-IF($K29="",0,$K29))</f>
@@ -2654,7 +2654,7 @@
         <v/>
       </c>
       <c r="K30" s="4" t="n">
-        <v>550.9400000000001</v>
+        <v>551.1900000000001</v>
       </c>
       <c r="L30" s="21">
         <f>IF(OR($B30="",$I30=""),"",$I30-IF($K30="",0,$K30))</f>
@@ -2834,7 +2834,7 @@
         <v/>
       </c>
       <c r="K33" s="4" t="n">
-        <v>551.08</v>
+        <v>551.33</v>
       </c>
       <c r="L33" s="21">
         <f>IF(OR($B33="",$I33=""),"",$I33-IF($K33="",0,$K33))</f>
@@ -2894,7 +2894,7 @@
         <v/>
       </c>
       <c r="K34" s="4" t="n">
-        <v>426.23</v>
+        <v>426.49</v>
       </c>
       <c r="L34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($K34="",0,$K34))</f>
@@ -3014,7 +3014,7 @@
         <v/>
       </c>
       <c r="K36" s="4" t="n">
-        <v>538.9400000000001</v>
+        <v>539.09</v>
       </c>
       <c r="L36" s="21">
         <f>IF(OR($B36="",$I36=""),"",$I36-IF($K36="",0,$K36))</f>
@@ -3074,7 +3074,7 @@
         <v/>
       </c>
       <c r="K37" s="4" t="n">
-        <v>478.55</v>
+        <v>478.78</v>
       </c>
       <c r="L37" s="21">
         <f>IF(OR($B37="",$I37=""),"",$I37-IF($K37="",0,$K37))</f>
@@ -3134,7 +3134,7 @@
         <v/>
       </c>
       <c r="K38" s="4" t="n">
-        <v>624.29</v>
+        <v>624.53</v>
       </c>
       <c r="L38" s="21">
         <f>IF(OR($B38="",$I38=""),"",$I38-IF($K38="",0,$K38))</f>
@@ -3194,7 +3194,7 @@
         <v/>
       </c>
       <c r="K39" s="4" t="n">
-        <v>614.23</v>
+        <v>614.47</v>
       </c>
       <c r="L39" s="21">
         <f>IF(OR($B39="",$I39=""),"",$I39-IF($K39="",0,$K39))</f>
@@ -3314,7 +3314,7 @@
         <v/>
       </c>
       <c r="K41" s="4" t="n">
-        <v>393.06</v>
+        <v>393.3</v>
       </c>
       <c r="L41" s="21">
         <f>IF(OR($B41="",$I41=""),"",$I41-IF($K41="",0,$K41))</f>
@@ -3374,7 +3374,7 @@
         <v/>
       </c>
       <c r="K42" s="4" t="n">
-        <v>625.53</v>
+        <v>618.74</v>
       </c>
       <c r="L42" s="21">
         <f>IF(OR($B42="",$I42=""),"",$I42-IF($K42="",0,$K42))</f>
@@ -3434,7 +3434,7 @@
         <v/>
       </c>
       <c r="K43" s="4" t="n">
-        <v>877.37</v>
+        <v>877.63</v>
       </c>
       <c r="L43" s="21">
         <f>IF(OR($B43="",$I43=""),"",$I43-IF($K43="",0,$K43))</f>
@@ -3554,7 +3554,7 @@
         <v/>
       </c>
       <c r="K45" s="4" t="n">
-        <v>895.52</v>
+        <v>895.76</v>
       </c>
       <c r="L45" s="21">
         <f>IF(OR($B45="",$I45=""),"",$I45-IF($K45="",0,$K45))</f>
@@ -3614,7 +3614,7 @@
         <v/>
       </c>
       <c r="K46" s="4" t="n">
-        <v>871.4400000000001</v>
+        <v>871.65</v>
       </c>
       <c r="L46" s="21">
         <f>IF(OR($B46="",$I46=""),"",$I46-IF($K46="",0,$K46))</f>
@@ -3794,7 +3794,7 @@
         <v/>
       </c>
       <c r="K49" s="4" t="n">
-        <v>960.61</v>
+        <v>960.73</v>
       </c>
       <c r="L49" s="21">
         <f>IF(OR($B49="",$I49=""),"",$I49-IF($K49="",0,$K49))</f>
@@ -3914,7 +3914,7 @@
         <v/>
       </c>
       <c r="K51" s="4" t="n">
-        <v>642.47</v>
+        <v>972.61</v>
       </c>
       <c r="L51" s="21">
         <f>IF(OR($B51="",$I51=""),"",$I51-IF($K51="",0,$K51))</f>
@@ -3974,7 +3974,7 @@
         <v/>
       </c>
       <c r="K52" s="4" t="n">
-        <v>613.63</v>
+        <v>930.28</v>
       </c>
       <c r="L52" s="21">
         <f>IF(OR($B52="",$I52=""),"",$I52-IF($K52="",0,$K52))</f>
@@ -4034,7 +4034,7 @@
         <v/>
       </c>
       <c r="K53" s="4" t="n">
-        <v>77.89</v>
+        <v>257.22</v>
       </c>
       <c r="L53" s="21">
         <f>IF(OR($B53="",$I53=""),"",$I53-IF($K53="",0,$K53))</f>
@@ -33317,7 +33317,7 @@
         <v>35.4</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>115.98</v>
+        <v>115.97</v>
       </c>
       <c r="N6" s="21">
         <f>SUM(E6:M6)</f>
@@ -33368,7 +33368,7 @@
         <v>35.4</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>69.34999999999999</v>
+        <v>69.34</v>
       </c>
       <c r="N7" s="21">
         <f>SUM(E7:M7)</f>
@@ -33419,7 +33419,7 @@
         <v>35.4</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>96.5</v>
+        <v>96.48999999999999</v>
       </c>
       <c r="N8" s="21">
         <f>SUM(E8:M8)</f>
@@ -33470,7 +33470,7 @@
         <v>35.4</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>115.66</v>
+        <v>115.65</v>
       </c>
       <c r="N9" s="21">
         <f>SUM(E9:M9)</f>
@@ -33521,7 +33521,7 @@
         <v>35.4</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>96.51000000000001</v>
+        <v>96.5</v>
       </c>
       <c r="N10" s="21">
         <f>SUM(E10:M10)</f>
@@ -33572,7 +33572,7 @@
         <v>35.4</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>59.66</v>
+        <v>59.8</v>
       </c>
       <c r="N11" s="21">
         <f>SUM(E11:M11)</f>
@@ -33623,7 +33623,7 @@
         <v>35.4</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>71.48999999999999</v>
+        <v>71.67</v>
       </c>
       <c r="N12" s="21">
         <f>SUM(E12:M12)</f>
@@ -33674,7 +33674,7 @@
         <v>35.4</v>
       </c>
       <c r="M13" s="4" t="n">
-        <v>73.15000000000001</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="N13" s="21">
         <f>SUM(E13:M13)</f>
@@ -33725,7 +33725,7 @@
         <v>35.4</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>59.47</v>
+        <v>59.61</v>
       </c>
       <c r="N14" s="21">
         <f>SUM(E14:M14)</f>
@@ -33878,7 +33878,7 @@
         <v>35.4</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>83.88</v>
+        <v>84.45999999999999</v>
       </c>
       <c r="N17" s="21">
         <f>SUM(E17:M17)</f>
@@ -33980,7 +33980,7 @@
         <v>35.4</v>
       </c>
       <c r="M19" s="4" t="n">
-        <v>86.95</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="N19" s="21">
         <f>SUM(E19:M19)</f>
@@ -34031,7 +34031,7 @@
         <v>35.4</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>83.98</v>
+        <v>84.56</v>
       </c>
       <c r="N20" s="21">
         <f>SUM(E20:M20)</f>
@@ -34133,7 +34133,7 @@
         <v>35.4</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>84.38</v>
+        <v>84.95999999999999</v>
       </c>
       <c r="N22" s="21">
         <f>SUM(E22:M22)</f>
@@ -34184,7 +34184,7 @@
         <v>35.4</v>
       </c>
       <c r="M23" s="4" t="n">
-        <v>30.05</v>
+        <v>30.26</v>
       </c>
       <c r="N23" s="21">
         <f>SUM(E23:M23)</f>
@@ -34286,7 +34286,7 @@
         <v>35.4</v>
       </c>
       <c r="M25" s="4" t="n">
-        <v>37.32</v>
+        <v>37.61</v>
       </c>
       <c r="N25" s="21">
         <f>SUM(E25:M25)</f>
@@ -34388,7 +34388,7 @@
         <v>35.4</v>
       </c>
       <c r="M27" s="4" t="n">
-        <v>35.93</v>
+        <v>36.18</v>
       </c>
       <c r="N27" s="21">
         <f>SUM(E27:M27)</f>
@@ -34439,7 +34439,7 @@
         <v>35.4</v>
       </c>
       <c r="M28" s="4" t="n">
-        <v>41.14</v>
+        <v>41.43</v>
       </c>
       <c r="N28" s="21">
         <f>SUM(E28:M28)</f>
@@ -34490,7 +34490,7 @@
         <v>35.4</v>
       </c>
       <c r="M29" s="4" t="n">
-        <v>43.04</v>
+        <v>43.19</v>
       </c>
       <c r="N29" s="21">
         <f>SUM(E29:M29)</f>
@@ -34541,7 +34541,7 @@
         <v>35.4</v>
       </c>
       <c r="M30" s="4" t="n">
-        <v>35.9</v>
+        <v>36.15</v>
       </c>
       <c r="N30" s="21">
         <f>SUM(E30:M30)</f>
@@ -34694,7 +34694,7 @@
         <v>35.4</v>
       </c>
       <c r="M33" s="4" t="n">
-        <v>35.62</v>
+        <v>35.87</v>
       </c>
       <c r="N33" s="21">
         <f>SUM(E33:M33)</f>
@@ -34745,7 +34745,7 @@
         <v>35.4</v>
       </c>
       <c r="M34" s="4" t="n">
-        <v>37.92</v>
+        <v>38.18</v>
       </c>
       <c r="N34" s="21">
         <f>SUM(E34:M34)</f>
@@ -34847,7 +34847,7 @@
         <v>35.4</v>
       </c>
       <c r="M36" s="4" t="n">
-        <v>21.51</v>
+        <v>21.66</v>
       </c>
       <c r="N36" s="21">
         <f>SUM(E36:M36)</f>
@@ -34898,7 +34898,7 @@
         <v>35.4</v>
       </c>
       <c r="M37" s="4" t="n">
-        <v>32.1</v>
+        <v>32.33</v>
       </c>
       <c r="N37" s="21">
         <f>SUM(E37:M37)</f>
@@ -34949,7 +34949,7 @@
         <v>35.4</v>
       </c>
       <c r="M38" s="4" t="n">
-        <v>34.93</v>
+        <v>35.17</v>
       </c>
       <c r="N38" s="21">
         <f>SUM(E38:M38)</f>
@@ -35000,7 +35000,7 @@
         <v>35.4</v>
       </c>
       <c r="M39" s="4" t="n">
-        <v>34.71</v>
+        <v>34.95</v>
       </c>
       <c r="N39" s="21">
         <f>SUM(E39:M39)</f>
@@ -35102,7 +35102,7 @@
         <v>35.4</v>
       </c>
       <c r="M41" s="4" t="n">
-        <v>34.88</v>
+        <v>35.12</v>
       </c>
       <c r="N41" s="21">
         <f>SUM(E41:M41)</f>
@@ -35153,7 +35153,7 @@
         <v>35.4</v>
       </c>
       <c r="M42" s="4" t="n">
-        <v>34.93</v>
+        <v>28.14</v>
       </c>
       <c r="N42" s="21">
         <f>SUM(E42:M42)</f>
@@ -35204,7 +35204,7 @@
         <v>35.4</v>
       </c>
       <c r="M43" s="4" t="n">
-        <v>33.27</v>
+        <v>33.53</v>
       </c>
       <c r="N43" s="21">
         <f>SUM(E43:M43)</f>
@@ -35306,7 +35306,7 @@
         <v>35.4</v>
       </c>
       <c r="M45" s="4" t="n">
-        <v>35.35</v>
+        <v>35.58</v>
       </c>
       <c r="N45" s="21">
         <f>SUM(E45:M45)</f>
@@ -35357,7 +35357,7 @@
         <v>35.4</v>
       </c>
       <c r="M46" s="4" t="n">
-        <v>31.23</v>
+        <v>31.44</v>
       </c>
       <c r="N46" s="21">
         <f>SUM(E46:M46)</f>
@@ -35510,7 +35510,7 @@
         <v>35.4</v>
       </c>
       <c r="M49" s="4" t="n">
-        <v>180.77</v>
+        <v>180.9</v>
       </c>
       <c r="N49" s="21">
         <f>SUM(E49:M49)</f>
@@ -35588,22 +35588,22 @@
         <v>46316</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>89.95999999999999</v>
+        <v>109.96</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>299.87</v>
+        <v>595.26</v>
       </c>
       <c r="G51" s="4" t="n">
-        <v>9.210000000000001</v>
+        <v>18.28</v>
       </c>
       <c r="H51" s="4" t="n">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="I51" s="4" t="n">
         <v>44.62</v>
       </c>
       <c r="J51" s="4" t="n">
-        <v>17.9</v>
+        <v>23.19</v>
       </c>
       <c r="K51" s="4" t="n">
         <v>14.75</v>
@@ -35612,7 +35612,7 @@
         <v>35.4</v>
       </c>
       <c r="M51" s="4" t="n">
-        <v>130.46</v>
+        <v>130.56</v>
       </c>
       <c r="N51" s="21">
         <f>SUM(E51:M51)</f>
@@ -35639,22 +35639,22 @@
         <v>46316</v>
       </c>
       <c r="E52" s="4" t="n">
-        <v>89.75</v>
+        <v>109.75</v>
       </c>
       <c r="F52" s="4" t="n">
-        <v>299.18</v>
+        <v>581.67</v>
       </c>
       <c r="G52" s="4" t="n">
-        <v>9.18</v>
+        <v>17.86</v>
       </c>
       <c r="H52" s="4" t="n">
-        <v>0.3</v>
+        <v>0.58</v>
       </c>
       <c r="I52" s="4" t="n">
         <v>44.88</v>
       </c>
       <c r="J52" s="4" t="n">
-        <v>17.86</v>
+        <v>23.07</v>
       </c>
       <c r="K52" s="4" t="n">
         <v>14.75</v>
@@ -35690,22 +35690,22 @@
         <v>46316</v>
       </c>
       <c r="E53" s="4" t="n">
-        <v>44.94</v>
+        <v>64.94</v>
       </c>
       <c r="F53" s="4" t="n">
-        <v>0</v>
+        <v>150.12</v>
       </c>
       <c r="G53" s="4" t="n">
-        <v>4.6</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="H53" s="4" t="n">
-        <v>0.15</v>
+        <v>0.3</v>
       </c>
       <c r="I53" s="4" t="n">
         <v>4.5</v>
       </c>
       <c r="J53" s="4" t="n">
-        <v>8.94</v>
+        <v>13.4</v>
       </c>
       <c r="K53" s="4" t="n">
         <v>14.75</v>

</xml_diff>

<commit_message>
Data update — 2026-10-23 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_oct2026.xlsx
+++ b/results/strategy_pnl_oct2026.xlsx
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trade Log'!$A$3:$O$503</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$55</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1214,7 +1214,7 @@
         <v/>
       </c>
       <c r="K6" s="4" t="n">
-        <v>955</v>
+        <v>954.99</v>
       </c>
       <c r="L6" s="21">
         <f>IF(OR($B6="",$I6=""),"",$I6-IF($K6="",0,$K6))</f>
@@ -1274,7 +1274,7 @@
         <v/>
       </c>
       <c r="K7" s="4" t="n">
-        <v>819.03</v>
+        <v>819.02</v>
       </c>
       <c r="L7" s="21">
         <f>IF(OR($B7="",$I7=""),"",$I7-IF($K7="",0,$K7))</f>
@@ -1334,7 +1334,7 @@
         <v/>
       </c>
       <c r="K8" s="4" t="n">
-        <v>857.26</v>
+        <v>857.25</v>
       </c>
       <c r="L8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($K8="",0,$K8))</f>
@@ -1394,7 +1394,7 @@
         <v/>
       </c>
       <c r="K9" s="4" t="n">
-        <v>969.46</v>
+        <v>969.45</v>
       </c>
       <c r="L9" s="21">
         <f>IF(OR($B9="",$I9=""),"",$I9-IF($K9="",0,$K9))</f>
@@ -1634,7 +1634,7 @@
         <v/>
       </c>
       <c r="K13" s="4" t="n">
-        <v>688.36</v>
+        <v>688.42</v>
       </c>
       <c r="L13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($K13="",0,$K13))</f>
@@ -1694,7 +1694,7 @@
         <v/>
       </c>
       <c r="K14" s="4" t="n">
-        <v>684.15</v>
+        <v>684.14</v>
       </c>
       <c r="L14" s="21">
         <f>IF(OR($B14="",$I14=""),"",$I14-IF($K14="",0,$K14))</f>
@@ -1874,7 +1874,7 @@
         <v/>
       </c>
       <c r="K17" s="4" t="n">
-        <v>662.09</v>
+        <v>662.08</v>
       </c>
       <c r="L17" s="21">
         <f>IF(OR($B17="",$I17=""),"",$I17-IF($K17="",0,$K17))</f>
@@ -2054,7 +2054,7 @@
         <v/>
       </c>
       <c r="K20" s="4" t="n">
-        <v>678.01</v>
+        <v>678</v>
       </c>
       <c r="L20" s="21">
         <f>IF(OR($B20="",$I20=""),"",$I20-IF($K20="",0,$K20))</f>
@@ -2174,7 +2174,7 @@
         <v/>
       </c>
       <c r="K22" s="4" t="n">
-        <v>659.61</v>
+        <v>659.6</v>
       </c>
       <c r="L22" s="21">
         <f>IF(OR($B22="",$I22=""),"",$I22-IF($K22="",0,$K22))</f>
@@ -2474,7 +2474,7 @@
         <v/>
       </c>
       <c r="K27" s="4" t="n">
-        <v>548.0700000000001</v>
+        <v>548.0599999999999</v>
       </c>
       <c r="L27" s="21">
         <f>IF(OR($B27="",$I27=""),"",$I27-IF($K27="",0,$K27))</f>
@@ -2654,7 +2654,7 @@
         <v/>
       </c>
       <c r="K30" s="4" t="n">
-        <v>551.1900000000001</v>
+        <v>551.1799999999999</v>
       </c>
       <c r="L30" s="21">
         <f>IF(OR($B30="",$I30=""),"",$I30-IF($K30="",0,$K30))</f>
@@ -2834,7 +2834,7 @@
         <v/>
       </c>
       <c r="K33" s="4" t="n">
-        <v>551.33</v>
+        <v>551.3200000000001</v>
       </c>
       <c r="L33" s="21">
         <f>IF(OR($B33="",$I33=""),"",$I33-IF($K33="",0,$K33))</f>
@@ -2894,7 +2894,7 @@
         <v/>
       </c>
       <c r="K34" s="4" t="n">
-        <v>426.49</v>
+        <v>426.51</v>
       </c>
       <c r="L34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($K34="",0,$K34))</f>
@@ -3014,7 +3014,7 @@
         <v/>
       </c>
       <c r="K36" s="4" t="n">
-        <v>539.09</v>
+        <v>539.08</v>
       </c>
       <c r="L36" s="21">
         <f>IF(OR($B36="",$I36=""),"",$I36-IF($K36="",0,$K36))</f>
@@ -3074,7 +3074,7 @@
         <v/>
       </c>
       <c r="K37" s="4" t="n">
-        <v>478.78</v>
+        <v>478.8</v>
       </c>
       <c r="L37" s="21">
         <f>IF(OR($B37="",$I37=""),"",$I37-IF($K37="",0,$K37))</f>
@@ -3134,7 +3134,7 @@
         <v/>
       </c>
       <c r="K38" s="4" t="n">
-        <v>624.53</v>
+        <v>624.52</v>
       </c>
       <c r="L38" s="21">
         <f>IF(OR($B38="",$I38=""),"",$I38-IF($K38="",0,$K38))</f>
@@ -3314,7 +3314,7 @@
         <v/>
       </c>
       <c r="K41" s="4" t="n">
-        <v>393.3</v>
+        <v>393.29</v>
       </c>
       <c r="L41" s="21">
         <f>IF(OR($B41="",$I41=""),"",$I41-IF($K41="",0,$K41))</f>
@@ -3434,7 +3434,7 @@
         <v/>
       </c>
       <c r="K43" s="4" t="n">
-        <v>877.63</v>
+        <v>877.62</v>
       </c>
       <c r="L43" s="21">
         <f>IF(OR($B43="",$I43=""),"",$I43-IF($K43="",0,$K43))</f>
@@ -3554,7 +3554,7 @@
         <v/>
       </c>
       <c r="K45" s="4" t="n">
-        <v>895.76</v>
+        <v>895.78</v>
       </c>
       <c r="L45" s="21">
         <f>IF(OR($B45="",$I45=""),"",$I45-IF($K45="",0,$K45))</f>
@@ -3794,7 +3794,7 @@
         <v/>
       </c>
       <c r="K49" s="4" t="n">
-        <v>960.73</v>
+        <v>960.02</v>
       </c>
       <c r="L49" s="21">
         <f>IF(OR($B49="",$I49=""),"",$I49-IF($K49="",0,$K49))</f>
@@ -4055,14 +4055,32 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="23" t="n"/>
-      <c r="B54" s="23" t="n"/>
-      <c r="C54" s="23" t="n"/>
-      <c r="D54" s="24" t="n"/>
-      <c r="E54" s="25" t="n"/>
-      <c r="F54" s="26" t="n"/>
-      <c r="G54" s="24" t="n"/>
-      <c r="H54" s="25" t="n"/>
+      <c r="A54" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-341261023126009+321261023756709+231261023120709+221261023808609+341261023126109+231261023120809+231261023121009+321261023759509+321261023759709+221261023810109+341261023126409+321261023760109+341261023126709</t>
+        </is>
+      </c>
+      <c r="B54" s="23" t="inlineStr">
+        <is>
+          <t>FISCHER</t>
+        </is>
+      </c>
+      <c r="C54" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D54" s="24" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E54" s="25" t="n">
+        <v>24.9837</v>
+      </c>
+      <c r="F54" s="26" t="n">
+        <v>6007</v>
+      </c>
+      <c r="G54" s="24" t="inlineStr"/>
+      <c r="H54" s="25" t="inlineStr"/>
       <c r="I54" s="21">
         <f>IF(OR($B54="",$H54=""),"",IF($C54="LONG",($H54-$E54)*$F54,($E54-$H54)*$F54))</f>
         <v/>
@@ -4071,7 +4089,9 @@
         <f>IF(OR($B54="",$I54="",$E54=0,$F54=0),"",$I54/($E54*$F54))</f>
         <v/>
       </c>
-      <c r="K54" s="4" t="n"/>
+      <c r="K54" s="4" t="n">
+        <v>14.75</v>
+      </c>
       <c r="L54" s="21">
         <f>IF(OR($B54="",$I54=""),"",$I54-IF($K54="",0,$K54))</f>
         <v/>
@@ -4084,17 +4104,39 @@
         <f>IF($B54="","",IF($H54="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O54" s="23" t="n"/>
+      <c r="O54" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="55">
-      <c r="A55" s="23" t="n"/>
-      <c r="B55" s="23" t="n"/>
-      <c r="C55" s="23" t="n"/>
-      <c r="D55" s="24" t="n"/>
-      <c r="E55" s="25" t="n"/>
-      <c r="F55" s="26" t="n"/>
-      <c r="G55" s="24" t="n"/>
-      <c r="H55" s="25" t="n"/>
+      <c r="A55" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261023807609+321261023756809+231261023120609+221261023808709+221261023809309+231261023120909+221261023809609+231261023121109+341261023126209+341261023126309+341261023126509+341261023126609+321261023760409</t>
+        </is>
+      </c>
+      <c r="B55" s="23" t="inlineStr">
+        <is>
+          <t>JINDALPOLY</t>
+        </is>
+      </c>
+      <c r="C55" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D55" s="24" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E55" s="25" t="n">
+        <v>726.0981</v>
+      </c>
+      <c r="F55" s="26" t="n">
+        <v>410</v>
+      </c>
+      <c r="G55" s="24" t="inlineStr"/>
+      <c r="H55" s="25" t="inlineStr"/>
       <c r="I55" s="21">
         <f>IF(OR($B55="",$H55=""),"",IF($C55="LONG",($H55-$E55)*$F55,($E55-$H55)*$F55))</f>
         <v/>
@@ -4103,7 +4145,9 @@
         <f>IF(OR($B55="",$I55="",$E55=0,$F55=0),"",$I55/($E55*$F55))</f>
         <v/>
       </c>
-      <c r="K55" s="4" t="n"/>
+      <c r="K55" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L55" s="21">
         <f>IF(OR($B55="",$I55=""),"",$I55-IF($K55="",0,$K55))</f>
         <v/>
@@ -4116,7 +4160,11 @@
         <f>IF($B55="","",IF($H55="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O55" s="23" t="n"/>
+      <c r="O55" s="23" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="23" t="n"/>
@@ -31129,7 +31177,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J46"/>
+  <dimension ref="A1:J47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31471,7 +31519,7 @@
     <row r="10">
       <c r="A10" s="27" t="inlineStr">
         <is>
-          <t>GOODLUCK</t>
+          <t>FISCHER</t>
         </is>
       </c>
       <c r="B10" s="20">
@@ -31514,7 +31562,7 @@
     <row r="11">
       <c r="A11" s="27" t="inlineStr">
         <is>
-          <t>GPTINFRA</t>
+          <t>GOODLUCK</t>
         </is>
       </c>
       <c r="B11" s="20">
@@ -31557,7 +31605,7 @@
     <row r="12">
       <c r="A12" s="27" t="inlineStr">
         <is>
-          <t>HATHWAY</t>
+          <t>GPTINFRA</t>
         </is>
       </c>
       <c r="B12" s="20">
@@ -31600,7 +31648,7 @@
     <row r="13">
       <c r="A13" s="27" t="inlineStr">
         <is>
-          <t>INDIAGLYCO</t>
+          <t>HATHWAY</t>
         </is>
       </c>
       <c r="B13" s="20">
@@ -31643,7 +31691,7 @@
     <row r="14">
       <c r="A14" s="27" t="inlineStr">
         <is>
-          <t>INDOKEM</t>
+          <t>INDIAGLYCO</t>
         </is>
       </c>
       <c r="B14" s="20">
@@ -31686,7 +31734,7 @@
     <row r="15">
       <c r="A15" s="27" t="inlineStr">
         <is>
-          <t>INOXGREEN</t>
+          <t>INDOKEM</t>
         </is>
       </c>
       <c r="B15" s="20">
@@ -31729,7 +31777,7 @@
     <row r="16">
       <c r="A16" s="27" t="inlineStr">
         <is>
-          <t>JAICORPLTD</t>
+          <t>INOXGREEN</t>
         </is>
       </c>
       <c r="B16" s="20">
@@ -31772,7 +31820,7 @@
     <row r="17">
       <c r="A17" s="27" t="inlineStr">
         <is>
-          <t>JINDALPOLY</t>
+          <t>JAICORPLTD</t>
         </is>
       </c>
       <c r="B17" s="20">
@@ -31815,7 +31863,7 @@
     <row r="18">
       <c r="A18" s="27" t="inlineStr">
         <is>
-          <t>KOTIC</t>
+          <t>JINDALPOLY</t>
         </is>
       </c>
       <c r="B18" s="20">
@@ -31858,7 +31906,7 @@
     <row r="19">
       <c r="A19" s="27" t="inlineStr">
         <is>
-          <t>KRISHNADEF</t>
+          <t>KOTIC</t>
         </is>
       </c>
       <c r="B19" s="20">
@@ -31901,7 +31949,7 @@
     <row r="20">
       <c r="A20" s="27" t="inlineStr">
         <is>
-          <t>KROSS</t>
+          <t>KRISHNADEF</t>
         </is>
       </c>
       <c r="B20" s="20">
@@ -31944,7 +31992,7 @@
     <row r="21">
       <c r="A21" s="27" t="inlineStr">
         <is>
-          <t>MBEL</t>
+          <t>KROSS</t>
         </is>
       </c>
       <c r="B21" s="20">
@@ -31987,7 +32035,7 @@
     <row r="22">
       <c r="A22" s="27" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>MBEL</t>
         </is>
       </c>
       <c r="B22" s="20">
@@ -32030,7 +32078,7 @@
     <row r="23">
       <c r="A23" s="27" t="inlineStr">
         <is>
-          <t>MOBIKWIK</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="B23" s="20">
@@ -32073,7 +32121,7 @@
     <row r="24">
       <c r="A24" s="27" t="inlineStr">
         <is>
-          <t>NIBE</t>
+          <t>MOBIKWIK</t>
         </is>
       </c>
       <c r="B24" s="20">
@@ -32116,7 +32164,7 @@
     <row r="25">
       <c r="A25" s="27" t="inlineStr">
         <is>
-          <t>OAL</t>
+          <t>NIBE</t>
         </is>
       </c>
       <c r="B25" s="20">
@@ -32159,7 +32207,7 @@
     <row r="26">
       <c r="A26" s="27" t="inlineStr">
         <is>
-          <t>ORIENTELEC</t>
+          <t>OAL</t>
         </is>
       </c>
       <c r="B26" s="20">
@@ -32202,7 +32250,7 @@
     <row r="27">
       <c r="A27" s="27" t="inlineStr">
         <is>
-          <t>PARACABLES</t>
+          <t>ORIENTELEC</t>
         </is>
       </c>
       <c r="B27" s="20">
@@ -32245,7 +32293,7 @@
     <row r="28">
       <c r="A28" s="27" t="inlineStr">
         <is>
-          <t>PIXTRANS</t>
+          <t>PARACABLES</t>
         </is>
       </c>
       <c r="B28" s="20">
@@ -32288,7 +32336,7 @@
     <row r="29">
       <c r="A29" s="27" t="inlineStr">
         <is>
-          <t>PNCINFRA</t>
+          <t>PIXTRANS</t>
         </is>
       </c>
       <c r="B29" s="20">
@@ -32331,7 +32379,7 @@
     <row r="30">
       <c r="A30" s="27" t="inlineStr">
         <is>
-          <t>PNGSREVA</t>
+          <t>PNCINFRA</t>
         </is>
       </c>
       <c r="B30" s="20">
@@ -32374,7 +32422,7 @@
     <row r="31">
       <c r="A31" s="27" t="inlineStr">
         <is>
-          <t>PRINCEPIPE</t>
+          <t>PNGSREVA</t>
         </is>
       </c>
       <c r="B31" s="20">
@@ -32417,7 +32465,7 @@
     <row r="32">
       <c r="A32" s="27" t="inlineStr">
         <is>
-          <t>RSYSTEMS</t>
+          <t>PRINCEPIPE</t>
         </is>
       </c>
       <c r="B32" s="20">
@@ -32460,7 +32508,7 @@
     <row r="33">
       <c r="A33" s="27" t="inlineStr">
         <is>
-          <t>RUBYMILLS</t>
+          <t>RSYSTEMS</t>
         </is>
       </c>
       <c r="B33" s="20">
@@ -32503,7 +32551,7 @@
     <row r="34">
       <c r="A34" s="27" t="inlineStr">
         <is>
-          <t>SAKSOFT</t>
+          <t>RUBYMILLS</t>
         </is>
       </c>
       <c r="B34" s="20">
@@ -32546,7 +32594,7 @@
     <row r="35">
       <c r="A35" s="27" t="inlineStr">
         <is>
-          <t>SATIN</t>
+          <t>SAKSOFT</t>
         </is>
       </c>
       <c r="B35" s="20">
@@ -32589,7 +32637,7 @@
     <row r="36">
       <c r="A36" s="27" t="inlineStr">
         <is>
-          <t>SGFIN</t>
+          <t>SATIN</t>
         </is>
       </c>
       <c r="B36" s="20">
@@ -32632,7 +32680,7 @@
     <row r="37">
       <c r="A37" s="27" t="inlineStr">
         <is>
-          <t>SHRINGARMS</t>
+          <t>SGFIN</t>
         </is>
       </c>
       <c r="B37" s="20">
@@ -32675,7 +32723,7 @@
     <row r="38">
       <c r="A38" s="27" t="inlineStr">
         <is>
-          <t>SIMPLEXINF</t>
+          <t>SHRINGARMS</t>
         </is>
       </c>
       <c r="B38" s="20">
@@ -32718,7 +32766,7 @@
     <row r="39">
       <c r="A39" s="27" t="inlineStr">
         <is>
-          <t>SMCGLOBAL</t>
+          <t>SIMPLEXINF</t>
         </is>
       </c>
       <c r="B39" s="20">
@@ -32761,7 +32809,7 @@
     <row r="40">
       <c r="A40" s="27" t="inlineStr">
         <is>
-          <t>SOLARA</t>
+          <t>SMCGLOBAL</t>
         </is>
       </c>
       <c r="B40" s="20">
@@ -32804,7 +32852,7 @@
     <row r="41">
       <c r="A41" s="27" t="inlineStr">
         <is>
-          <t>SPORTKING</t>
+          <t>SOLARA</t>
         </is>
       </c>
       <c r="B41" s="20">
@@ -32847,7 +32895,7 @@
     <row r="42">
       <c r="A42" s="27" t="inlineStr">
         <is>
-          <t>SUNCLAY</t>
+          <t>SPORTKING</t>
         </is>
       </c>
       <c r="B42" s="20">
@@ -32890,7 +32938,7 @@
     <row r="43">
       <c r="A43" s="27" t="inlineStr">
         <is>
-          <t>SWARAJENG</t>
+          <t>SUNCLAY</t>
         </is>
       </c>
       <c r="B43" s="20">
@@ -32933,7 +32981,7 @@
     <row r="44">
       <c r="A44" s="27" t="inlineStr">
         <is>
-          <t>TEAMLEASE</t>
+          <t>SWARAJENG</t>
         </is>
       </c>
       <c r="B44" s="20">
@@ -32976,7 +33024,7 @@
     <row r="45">
       <c r="A45" s="27" t="inlineStr">
         <is>
-          <t>YUKEN</t>
+          <t>TEAMLEASE</t>
         </is>
       </c>
       <c r="B45" s="20">
@@ -33017,37 +33065,80 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="3" t="inlineStr">
+      <c r="A46" s="27" t="inlineStr">
+        <is>
+          <t>YUKEN</t>
+        </is>
+      </c>
+      <c r="B46" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A46)</f>
+        <v/>
+      </c>
+      <c r="C46" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A46,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D46" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A46,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E46" s="22">
+        <f>IFERROR($C46/$B46,"")</f>
+        <v/>
+      </c>
+      <c r="F46" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A46,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G46" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A46,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H46" s="21">
+        <f>IFERROR($G46/$B46,"")</f>
+        <v/>
+      </c>
+      <c r="I46" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A46),"")</f>
+        <v/>
+      </c>
+      <c r="J46" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A46),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B46" s="30">
-        <f>SUM(B4:B45)</f>
-        <v/>
-      </c>
-      <c r="C46" s="30">
-        <f>SUM(C4:C45)</f>
-        <v/>
-      </c>
-      <c r="D46" s="30">
-        <f>SUM(D4:D45)</f>
-        <v/>
-      </c>
-      <c r="E46" s="31">
-        <f>IFERROR(C46/B46,"")</f>
-        <v/>
-      </c>
-      <c r="F46" s="32">
-        <f>SUM(F4:F45)</f>
-        <v/>
-      </c>
-      <c r="G46" s="32">
-        <f>SUM(G4:G45)</f>
-        <v/>
-      </c>
-      <c r="H46" s="32">
-        <f>IFERROR(G46/B46,"")</f>
+      <c r="B47" s="30">
+        <f>SUM(B4:B46)</f>
+        <v/>
+      </c>
+      <c r="C47" s="30">
+        <f>SUM(C4:C46)</f>
+        <v/>
+      </c>
+      <c r="D47" s="30">
+        <f>SUM(D4:D46)</f>
+        <v/>
+      </c>
+      <c r="E47" s="31">
+        <f>IFERROR(C47/B47,"")</f>
+        <v/>
+      </c>
+      <c r="F47" s="32">
+        <f>SUM(F4:F46)</f>
+        <v/>
+      </c>
+      <c r="G47" s="32">
+        <f>SUM(G4:G46)</f>
+        <v/>
+      </c>
+      <c r="H47" s="32">
+        <f>IFERROR(G47/B47,"")</f>
         <v/>
       </c>
     </row>
@@ -33066,7 +33157,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N54"/>
+  <dimension ref="A1:N56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -33470,7 +33561,7 @@
         <v>35.4</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>115.65</v>
+        <v>115.64</v>
       </c>
       <c r="N9" s="21">
         <f>SUM(E9:M9)</f>
@@ -33623,7 +33714,7 @@
         <v>35.4</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>71.67</v>
+        <v>71.66</v>
       </c>
       <c r="N12" s="21">
         <f>SUM(E12:M12)</f>
@@ -33674,7 +33765,7 @@
         <v>35.4</v>
       </c>
       <c r="M13" s="4" t="n">
-        <v>73.40000000000001</v>
+        <v>73.45</v>
       </c>
       <c r="N13" s="21">
         <f>SUM(E13:M13)</f>
@@ -33878,7 +33969,7 @@
         <v>35.4</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>84.45999999999999</v>
+        <v>84.45</v>
       </c>
       <c r="N17" s="21">
         <f>SUM(E17:M17)</f>
@@ -33980,7 +34071,7 @@
         <v>35.4</v>
       </c>
       <c r="M19" s="4" t="n">
-        <v>87.59999999999999</v>
+        <v>87.61</v>
       </c>
       <c r="N19" s="21">
         <f>SUM(E19:M19)</f>
@@ -34031,7 +34122,7 @@
         <v>35.4</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>84.56</v>
+        <v>84.55</v>
       </c>
       <c r="N20" s="21">
         <f>SUM(E20:M20)</f>
@@ -34133,7 +34224,7 @@
         <v>35.4</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>84.95999999999999</v>
+        <v>84.95</v>
       </c>
       <c r="N22" s="21">
         <f>SUM(E22:M22)</f>
@@ -34184,7 +34275,7 @@
         <v>35.4</v>
       </c>
       <c r="M23" s="4" t="n">
-        <v>30.26</v>
+        <v>30.25</v>
       </c>
       <c r="N23" s="21">
         <f>SUM(E23:M23)</f>
@@ -34439,7 +34530,7 @@
         <v>35.4</v>
       </c>
       <c r="M28" s="4" t="n">
-        <v>41.43</v>
+        <v>41.42</v>
       </c>
       <c r="N28" s="21">
         <f>SUM(E28:M28)</f>
@@ -34541,7 +34632,7 @@
         <v>35.4</v>
       </c>
       <c r="M30" s="4" t="n">
-        <v>36.15</v>
+        <v>36.14</v>
       </c>
       <c r="N30" s="21">
         <f>SUM(E30:M30)</f>
@@ -34694,7 +34785,7 @@
         <v>35.4</v>
       </c>
       <c r="M33" s="4" t="n">
-        <v>35.87</v>
+        <v>35.86</v>
       </c>
       <c r="N33" s="21">
         <f>SUM(E33:M33)</f>
@@ -34745,7 +34836,7 @@
         <v>35.4</v>
       </c>
       <c r="M34" s="4" t="n">
-        <v>38.18</v>
+        <v>38.2</v>
       </c>
       <c r="N34" s="21">
         <f>SUM(E34:M34)</f>
@@ -34898,7 +34989,7 @@
         <v>35.4</v>
       </c>
       <c r="M37" s="4" t="n">
-        <v>32.33</v>
+        <v>32.35</v>
       </c>
       <c r="N37" s="21">
         <f>SUM(E37:M37)</f>
@@ -35000,7 +35091,7 @@
         <v>35.4</v>
       </c>
       <c r="M39" s="4" t="n">
-        <v>34.95</v>
+        <v>34.94</v>
       </c>
       <c r="N39" s="21">
         <f>SUM(E39:M39)</f>
@@ -35153,7 +35244,7 @@
         <v>35.4</v>
       </c>
       <c r="M42" s="4" t="n">
-        <v>28.14</v>
+        <v>28.13</v>
       </c>
       <c r="N42" s="21">
         <f>SUM(E42:M42)</f>
@@ -35306,7 +35397,7 @@
         <v>35.4</v>
       </c>
       <c r="M45" s="4" t="n">
-        <v>35.58</v>
+        <v>35.6</v>
       </c>
       <c r="N45" s="21">
         <f>SUM(E45:M45)</f>
@@ -35510,7 +35601,7 @@
         <v>35.4</v>
       </c>
       <c r="M49" s="4" t="n">
-        <v>180.9</v>
+        <v>180.19</v>
       </c>
       <c r="N49" s="21">
         <f>SUM(E49:M49)</f>
@@ -35722,54 +35813,152 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="3" t="inlineStr">
+      <c r="A54" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-341261023126009+321261023756709+231261023120709+221261023808609+341261023126109+231261023120809+231261023121009+321261023759509+321261023759709+221261023810109+341261023126409+321261023760109+341261023126709</t>
+        </is>
+      </c>
+      <c r="B54" s="23" t="inlineStr">
+        <is>
+          <t>FISCHER</t>
+        </is>
+      </c>
+      <c r="C54" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D54" s="24" t="inlineStr"/>
+      <c r="E54" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J54" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K54" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L54" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M54" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N54" s="21">
+        <f>SUM(E54:M54)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261023807609+321261023756809+231261023120609+221261023808709+221261023809309+231261023120909+221261023809609+231261023121109+341261023126209+341261023126309+341261023126509+341261023126609+321261023760409</t>
+        </is>
+      </c>
+      <c r="B55" s="23" t="inlineStr">
+        <is>
+          <t>JINDALPOLY</t>
+        </is>
+      </c>
+      <c r="C55" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D55" s="24" t="inlineStr"/>
+      <c r="E55" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J55" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K55" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L55" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M55" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N55" s="21">
+        <f>SUM(E55:M55)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E54" s="32">
-        <f>SUM(E4:E53)</f>
-        <v/>
-      </c>
-      <c r="F54" s="32">
-        <f>SUM(F4:F53)</f>
-        <v/>
-      </c>
-      <c r="G54" s="32">
-        <f>SUM(G4:G53)</f>
-        <v/>
-      </c>
-      <c r="H54" s="32">
-        <f>SUM(H4:H53)</f>
-        <v/>
-      </c>
-      <c r="I54" s="32">
-        <f>SUM(I4:I53)</f>
-        <v/>
-      </c>
-      <c r="J54" s="32">
-        <f>SUM(J4:J53)</f>
-        <v/>
-      </c>
-      <c r="K54" s="32">
-        <f>SUM(K4:K53)</f>
-        <v/>
-      </c>
-      <c r="L54" s="32">
-        <f>SUM(L4:L53)</f>
-        <v/>
-      </c>
-      <c r="M54" s="32">
-        <f>SUM(M4:M53)</f>
-        <v/>
-      </c>
-      <c r="N54" s="32">
-        <f>SUM(N4:N53)</f>
+      <c r="E56" s="32">
+        <f>SUM(E4:E55)</f>
+        <v/>
+      </c>
+      <c r="F56" s="32">
+        <f>SUM(F4:F55)</f>
+        <v/>
+      </c>
+      <c r="G56" s="32">
+        <f>SUM(G4:G55)</f>
+        <v/>
+      </c>
+      <c r="H56" s="32">
+        <f>SUM(H4:H55)</f>
+        <v/>
+      </c>
+      <c r="I56" s="32">
+        <f>SUM(I4:I55)</f>
+        <v/>
+      </c>
+      <c r="J56" s="32">
+        <f>SUM(J4:J55)</f>
+        <v/>
+      </c>
+      <c r="K56" s="32">
+        <f>SUM(K4:K55)</f>
+        <v/>
+      </c>
+      <c r="L56" s="32">
+        <f>SUM(L4:L55)</f>
+        <v/>
+      </c>
+      <c r="M56" s="32">
+        <f>SUM(M4:M55)</f>
+        <v/>
+      </c>
+      <c r="N56" s="32">
+        <f>SUM(N4:N55)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:N53"/>
+  <autoFilter ref="A3:N55"/>
   <mergeCells count="2">
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>

</xml_diff>

<commit_message>
Data update — 2026-10-26 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_oct2026.xlsx
+++ b/results/strategy_pnl_oct2026.xlsx
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trade Log'!$A$3:$O$503</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$56</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1214,7 +1214,7 @@
         <v/>
       </c>
       <c r="K6" s="4" t="n">
-        <v>954.99</v>
+        <v>955.01</v>
       </c>
       <c r="L6" s="21">
         <f>IF(OR($B6="",$I6=""),"",$I6-IF($K6="",0,$K6))</f>
@@ -1274,7 +1274,7 @@
         <v/>
       </c>
       <c r="K7" s="4" t="n">
-        <v>819.02</v>
+        <v>819.04</v>
       </c>
       <c r="L7" s="21">
         <f>IF(OR($B7="",$I7=""),"",$I7-IF($K7="",0,$K7))</f>
@@ -1334,7 +1334,7 @@
         <v/>
       </c>
       <c r="K8" s="4" t="n">
-        <v>857.25</v>
+        <v>857.27</v>
       </c>
       <c r="L8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($K8="",0,$K8))</f>
@@ -1394,7 +1394,7 @@
         <v/>
       </c>
       <c r="K9" s="4" t="n">
-        <v>969.45</v>
+        <v>969.48</v>
       </c>
       <c r="L9" s="21">
         <f>IF(OR($B9="",$I9=""),"",$I9-IF($K9="",0,$K9))</f>
@@ -1454,7 +1454,7 @@
         <v/>
       </c>
       <c r="K10" s="4" t="n">
-        <v>943.02</v>
+        <v>943.04</v>
       </c>
       <c r="L10" s="21">
         <f>IF(OR($B10="",$I10=""),"",$I10-IF($K10="",0,$K10))</f>
@@ -1514,7 +1514,7 @@
         <v/>
       </c>
       <c r="K11" s="4" t="n">
-        <v>691.54</v>
+        <v>691.26</v>
       </c>
       <c r="L11" s="21">
         <f>IF(OR($B11="",$I11=""),"",$I11-IF($K11="",0,$K11))</f>
@@ -1574,7 +1574,7 @@
         <v/>
       </c>
       <c r="K12" s="4" t="n">
-        <v>756.71</v>
+        <v>756.38</v>
       </c>
       <c r="L12" s="21">
         <f>IF(OR($B12="",$I12=""),"",$I12-IF($K12="",0,$K12))</f>
@@ -1634,7 +1634,7 @@
         <v/>
       </c>
       <c r="K13" s="4" t="n">
-        <v>688.42</v>
+        <v>687.86</v>
       </c>
       <c r="L13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($K13="",0,$K13))</f>
@@ -1694,7 +1694,7 @@
         <v/>
       </c>
       <c r="K14" s="4" t="n">
-        <v>684.14</v>
+        <v>683.87</v>
       </c>
       <c r="L14" s="21">
         <f>IF(OR($B14="",$I14=""),"",$I14-IF($K14="",0,$K14))</f>
@@ -1874,7 +1874,7 @@
         <v/>
       </c>
       <c r="K17" s="4" t="n">
-        <v>662.08</v>
+        <v>660.9400000000001</v>
       </c>
       <c r="L17" s="21">
         <f>IF(OR($B17="",$I17=""),"",$I17-IF($K17="",0,$K17))</f>
@@ -1994,7 +1994,7 @@
         <v/>
       </c>
       <c r="K19" s="4" t="n">
-        <v>667.79</v>
+        <v>666.67</v>
       </c>
       <c r="L19" s="21">
         <f>IF(OR($B19="",$I19=""),"",$I19-IF($K19="",0,$K19))</f>
@@ -2054,7 +2054,7 @@
         <v/>
       </c>
       <c r="K20" s="4" t="n">
-        <v>678</v>
+        <v>676.87</v>
       </c>
       <c r="L20" s="21">
         <f>IF(OR($B20="",$I20=""),"",$I20-IF($K20="",0,$K20))</f>
@@ -2174,7 +2174,7 @@
         <v/>
       </c>
       <c r="K22" s="4" t="n">
-        <v>659.6</v>
+        <v>658.46</v>
       </c>
       <c r="L22" s="21">
         <f>IF(OR($B22="",$I22=""),"",$I22-IF($K22="",0,$K22))</f>
@@ -2234,7 +2234,7 @@
         <v/>
       </c>
       <c r="K23" s="4" t="n">
-        <v>420.06</v>
+        <v>419.65</v>
       </c>
       <c r="L23" s="21">
         <f>IF(OR($B23="",$I23=""),"",$I23-IF($K23="",0,$K23))</f>
@@ -2354,7 +2354,7 @@
         <v/>
       </c>
       <c r="K25" s="4" t="n">
-        <v>557.8099999999999</v>
+        <v>557.29</v>
       </c>
       <c r="L25" s="21">
         <f>IF(OR($B25="",$I25=""),"",$I25-IF($K25="",0,$K25))</f>
@@ -2474,7 +2474,7 @@
         <v/>
       </c>
       <c r="K27" s="4" t="n">
-        <v>548.0599999999999</v>
+        <v>547.58</v>
       </c>
       <c r="L27" s="21">
         <f>IF(OR($B27="",$I27=""),"",$I27-IF($K27="",0,$K27))</f>
@@ -2534,7 +2534,7 @@
         <v/>
       </c>
       <c r="K28" s="4" t="n">
-        <v>548.4</v>
+        <v>547.84</v>
       </c>
       <c r="L28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($K28="",0,$K28))</f>
@@ -2594,7 +2594,7 @@
         <v/>
       </c>
       <c r="K29" s="4" t="n">
-        <v>555.1900000000001</v>
+        <v>554.59</v>
       </c>
       <c r="L29" s="21">
         <f>IF(OR($B29="",$I29=""),"",$I29-IF($K29="",0,$K29))</f>
@@ -2654,7 +2654,7 @@
         <v/>
       </c>
       <c r="K30" s="4" t="n">
-        <v>551.1799999999999</v>
+        <v>550.7</v>
       </c>
       <c r="L30" s="21">
         <f>IF(OR($B30="",$I30=""),"",$I30-IF($K30="",0,$K30))</f>
@@ -2834,7 +2834,7 @@
         <v/>
       </c>
       <c r="K33" s="4" t="n">
-        <v>551.3200000000001</v>
+        <v>550.84</v>
       </c>
       <c r="L33" s="21">
         <f>IF(OR($B33="",$I33=""),"",$I33-IF($K33="",0,$K33))</f>
@@ -2894,7 +2894,7 @@
         <v/>
       </c>
       <c r="K34" s="4" t="n">
-        <v>426.51</v>
+        <v>425.96</v>
       </c>
       <c r="L34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($K34="",0,$K34))</f>
@@ -3014,7 +3014,7 @@
         <v/>
       </c>
       <c r="K36" s="4" t="n">
-        <v>539.08</v>
+        <v>553.04</v>
       </c>
       <c r="L36" s="21">
         <f>IF(OR($B36="",$I36=""),"",$I36-IF($K36="",0,$K36))</f>
@@ -3074,7 +3074,7 @@
         <v/>
       </c>
       <c r="K37" s="4" t="n">
-        <v>478.8</v>
+        <v>478.05</v>
       </c>
       <c r="L37" s="21">
         <f>IF(OR($B37="",$I37=""),"",$I37-IF($K37="",0,$K37))</f>
@@ -3134,7 +3134,7 @@
         <v/>
       </c>
       <c r="K38" s="4" t="n">
-        <v>624.52</v>
+        <v>624.05</v>
       </c>
       <c r="L38" s="21">
         <f>IF(OR($B38="",$I38=""),"",$I38-IF($K38="",0,$K38))</f>
@@ -3194,7 +3194,7 @@
         <v/>
       </c>
       <c r="K39" s="4" t="n">
-        <v>614.47</v>
+        <v>614</v>
       </c>
       <c r="L39" s="21">
         <f>IF(OR($B39="",$I39=""),"",$I39-IF($K39="",0,$K39))</f>
@@ -3314,7 +3314,7 @@
         <v/>
       </c>
       <c r="K41" s="4" t="n">
-        <v>393.29</v>
+        <v>592.26</v>
       </c>
       <c r="L41" s="21">
         <f>IF(OR($B41="",$I41=""),"",$I41-IF($K41="",0,$K41))</f>
@@ -3374,7 +3374,7 @@
         <v/>
       </c>
       <c r="K42" s="4" t="n">
-        <v>618.74</v>
+        <v>618.36</v>
       </c>
       <c r="L42" s="21">
         <f>IF(OR($B42="",$I42=""),"",$I42-IF($K42="",0,$K42))</f>
@@ -3434,7 +3434,7 @@
         <v/>
       </c>
       <c r="K43" s="4" t="n">
-        <v>877.62</v>
+        <v>924.52</v>
       </c>
       <c r="L43" s="21">
         <f>IF(OR($B43="",$I43=""),"",$I43-IF($K43="",0,$K43))</f>
@@ -3554,7 +3554,7 @@
         <v/>
       </c>
       <c r="K45" s="4" t="n">
-        <v>895.78</v>
+        <v>945.8200000000001</v>
       </c>
       <c r="L45" s="21">
         <f>IF(OR($B45="",$I45=""),"",$I45-IF($K45="",0,$K45))</f>
@@ -3614,7 +3614,7 @@
         <v/>
       </c>
       <c r="K46" s="4" t="n">
-        <v>871.65</v>
+        <v>915.86</v>
       </c>
       <c r="L46" s="21">
         <f>IF(OR($B46="",$I46=""),"",$I46-IF($K46="",0,$K46))</f>
@@ -3674,7 +3674,7 @@
         <v/>
       </c>
       <c r="K47" s="4" t="n">
-        <v>1031.86</v>
+        <v>1026.85</v>
       </c>
       <c r="L47" s="21">
         <f>IF(OR($B47="",$I47=""),"",$I47-IF($K47="",0,$K47))</f>
@@ -3734,7 +3734,7 @@
         <v/>
       </c>
       <c r="K48" s="4" t="n">
-        <v>1033.58</v>
+        <v>1028.54</v>
       </c>
       <c r="L48" s="21">
         <f>IF(OR($B48="",$I48=""),"",$I48-IF($K48="",0,$K48))</f>
@@ -3794,7 +3794,7 @@
         <v/>
       </c>
       <c r="K49" s="4" t="n">
-        <v>960.02</v>
+        <v>955.05</v>
       </c>
       <c r="L49" s="21">
         <f>IF(OR($B49="",$I49=""),"",$I49-IF($K49="",0,$K49))</f>
@@ -3854,7 +3854,7 @@
         <v/>
       </c>
       <c r="K50" s="4" t="n">
-        <v>1040.29</v>
+        <v>1035.24</v>
       </c>
       <c r="L50" s="21">
         <f>IF(OR($B50="",$I50=""),"",$I50-IF($K50="",0,$K50))</f>
@@ -3914,7 +3914,7 @@
         <v/>
       </c>
       <c r="K51" s="4" t="n">
-        <v>972.61</v>
+        <v>984.48</v>
       </c>
       <c r="L51" s="21">
         <f>IF(OR($B51="",$I51=""),"",$I51-IF($K51="",0,$K51))</f>
@@ -3974,7 +3974,7 @@
         <v/>
       </c>
       <c r="K52" s="4" t="n">
-        <v>930.28</v>
+        <v>939.9299999999999</v>
       </c>
       <c r="L52" s="21">
         <f>IF(OR($B52="",$I52=""),"",$I52-IF($K52="",0,$K52))</f>
@@ -4079,8 +4079,12 @@
       <c r="F54" s="26" t="n">
         <v>6007</v>
       </c>
-      <c r="G54" s="24" t="inlineStr"/>
-      <c r="H54" s="25" t="inlineStr"/>
+      <c r="G54" s="24" t="n">
+        <v>46321</v>
+      </c>
+      <c r="H54" s="25" t="n">
+        <v>25.7571</v>
+      </c>
       <c r="I54" s="21">
         <f>IF(OR($B54="",$H54=""),"",IF($C54="LONG",($H54-$E54)*$F54,($E54-$H54)*$F54))</f>
         <v/>
@@ -4090,7 +4094,7 @@
         <v/>
       </c>
       <c r="K54" s="4" t="n">
-        <v>14.75</v>
+        <v>192.92</v>
       </c>
       <c r="L54" s="21">
         <f>IF(OR($B54="",$I54=""),"",$I54-IF($K54="",0,$K54))</f>
@@ -4135,8 +4139,12 @@
       <c r="F55" s="26" t="n">
         <v>410</v>
       </c>
-      <c r="G55" s="24" t="inlineStr"/>
-      <c r="H55" s="25" t="inlineStr"/>
+      <c r="G55" s="24" t="n">
+        <v>46321</v>
+      </c>
+      <c r="H55" s="25" t="n">
+        <v>696</v>
+      </c>
       <c r="I55" s="21">
         <f>IF(OR($B55="",$H55=""),"",IF($C55="LONG",($H55-$E55)*$F55,($E55-$H55)*$F55))</f>
         <v/>
@@ -4146,7 +4154,7 @@
         <v/>
       </c>
       <c r="K55" s="4" t="n">
-        <v>50.15</v>
+        <v>555.48</v>
       </c>
       <c r="L55" s="21">
         <f>IF(OR($B55="",$I55=""),"",$I55-IF($K55="",0,$K55))</f>
@@ -4167,14 +4175,32 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="23" t="n"/>
-      <c r="B56" s="23" t="n"/>
-      <c r="C56" s="23" t="n"/>
-      <c r="D56" s="24" t="n"/>
-      <c r="E56" s="25" t="n"/>
-      <c r="F56" s="26" t="n"/>
-      <c r="G56" s="24" t="n"/>
-      <c r="H56" s="25" t="n"/>
+      <c r="A56" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126102699709+221261026669809+321261026636409+321261026636909+23126102699809+34126102699309+221261026670609+221261026671109+231261026100009+231261026100109+34126102699609+34126102699709</t>
+        </is>
+      </c>
+      <c r="B56" s="23" t="inlineStr">
+        <is>
+          <t>INDOSTAR</t>
+        </is>
+      </c>
+      <c r="C56" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D56" s="24" t="n">
+        <v>46321</v>
+      </c>
+      <c r="E56" s="25" t="n">
+        <v>183.525</v>
+      </c>
+      <c r="F56" s="26" t="n">
+        <v>1635</v>
+      </c>
+      <c r="G56" s="24" t="inlineStr"/>
+      <c r="H56" s="25" t="inlineStr"/>
       <c r="I56" s="21">
         <f>IF(OR($B56="",$H56=""),"",IF($C56="LONG",($H56-$E56)*$F56,($E56-$H56)*$F56))</f>
         <v/>
@@ -4183,7 +4209,9 @@
         <f>IF(OR($B56="",$I56="",$E56=0,$F56=0),"",$I56/($E56*$F56))</f>
         <v/>
       </c>
-      <c r="K56" s="4" t="n"/>
+      <c r="K56" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L56" s="21">
         <f>IF(OR($B56="",$I56=""),"",$I56-IF($K56="",0,$K56))</f>
         <v/>
@@ -4196,7 +4224,11 @@
         <f>IF($B56="","",IF($H56="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O56" s="23" t="n"/>
+      <c r="O56" s="23" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="23" t="n"/>
@@ -31177,7 +31209,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J47"/>
+  <dimension ref="A1:J48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31777,7 +31809,7 @@
     <row r="16">
       <c r="A16" s="27" t="inlineStr">
         <is>
-          <t>INOXGREEN</t>
+          <t>INDOSTAR</t>
         </is>
       </c>
       <c r="B16" s="20">
@@ -31820,7 +31852,7 @@
     <row r="17">
       <c r="A17" s="27" t="inlineStr">
         <is>
-          <t>JAICORPLTD</t>
+          <t>INOXGREEN</t>
         </is>
       </c>
       <c r="B17" s="20">
@@ -31863,7 +31895,7 @@
     <row r="18">
       <c r="A18" s="27" t="inlineStr">
         <is>
-          <t>JINDALPOLY</t>
+          <t>JAICORPLTD</t>
         </is>
       </c>
       <c r="B18" s="20">
@@ -31906,7 +31938,7 @@
     <row r="19">
       <c r="A19" s="27" t="inlineStr">
         <is>
-          <t>KOTIC</t>
+          <t>JINDALPOLY</t>
         </is>
       </c>
       <c r="B19" s="20">
@@ -31949,7 +31981,7 @@
     <row r="20">
       <c r="A20" s="27" t="inlineStr">
         <is>
-          <t>KRISHNADEF</t>
+          <t>KOTIC</t>
         </is>
       </c>
       <c r="B20" s="20">
@@ -31992,7 +32024,7 @@
     <row r="21">
       <c r="A21" s="27" t="inlineStr">
         <is>
-          <t>KROSS</t>
+          <t>KRISHNADEF</t>
         </is>
       </c>
       <c r="B21" s="20">
@@ -32035,7 +32067,7 @@
     <row r="22">
       <c r="A22" s="27" t="inlineStr">
         <is>
-          <t>MBEL</t>
+          <t>KROSS</t>
         </is>
       </c>
       <c r="B22" s="20">
@@ -32078,7 +32110,7 @@
     <row r="23">
       <c r="A23" s="27" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>MBEL</t>
         </is>
       </c>
       <c r="B23" s="20">
@@ -32121,7 +32153,7 @@
     <row r="24">
       <c r="A24" s="27" t="inlineStr">
         <is>
-          <t>MOBIKWIK</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="B24" s="20">
@@ -32164,7 +32196,7 @@
     <row r="25">
       <c r="A25" s="27" t="inlineStr">
         <is>
-          <t>NIBE</t>
+          <t>MOBIKWIK</t>
         </is>
       </c>
       <c r="B25" s="20">
@@ -32207,7 +32239,7 @@
     <row r="26">
       <c r="A26" s="27" t="inlineStr">
         <is>
-          <t>OAL</t>
+          <t>NIBE</t>
         </is>
       </c>
       <c r="B26" s="20">
@@ -32250,7 +32282,7 @@
     <row r="27">
       <c r="A27" s="27" t="inlineStr">
         <is>
-          <t>ORIENTELEC</t>
+          <t>OAL</t>
         </is>
       </c>
       <c r="B27" s="20">
@@ -32293,7 +32325,7 @@
     <row r="28">
       <c r="A28" s="27" t="inlineStr">
         <is>
-          <t>PARACABLES</t>
+          <t>ORIENTELEC</t>
         </is>
       </c>
       <c r="B28" s="20">
@@ -32336,7 +32368,7 @@
     <row r="29">
       <c r="A29" s="27" t="inlineStr">
         <is>
-          <t>PIXTRANS</t>
+          <t>PARACABLES</t>
         </is>
       </c>
       <c r="B29" s="20">
@@ -32379,7 +32411,7 @@
     <row r="30">
       <c r="A30" s="27" t="inlineStr">
         <is>
-          <t>PNCINFRA</t>
+          <t>PIXTRANS</t>
         </is>
       </c>
       <c r="B30" s="20">
@@ -32422,7 +32454,7 @@
     <row r="31">
       <c r="A31" s="27" t="inlineStr">
         <is>
-          <t>PNGSREVA</t>
+          <t>PNCINFRA</t>
         </is>
       </c>
       <c r="B31" s="20">
@@ -32465,7 +32497,7 @@
     <row r="32">
       <c r="A32" s="27" t="inlineStr">
         <is>
-          <t>PRINCEPIPE</t>
+          <t>PNGSREVA</t>
         </is>
       </c>
       <c r="B32" s="20">
@@ -32508,7 +32540,7 @@
     <row r="33">
       <c r="A33" s="27" t="inlineStr">
         <is>
-          <t>RSYSTEMS</t>
+          <t>PRINCEPIPE</t>
         </is>
       </c>
       <c r="B33" s="20">
@@ -32551,7 +32583,7 @@
     <row r="34">
       <c r="A34" s="27" t="inlineStr">
         <is>
-          <t>RUBYMILLS</t>
+          <t>RSYSTEMS</t>
         </is>
       </c>
       <c r="B34" s="20">
@@ -32594,7 +32626,7 @@
     <row r="35">
       <c r="A35" s="27" t="inlineStr">
         <is>
-          <t>SAKSOFT</t>
+          <t>RUBYMILLS</t>
         </is>
       </c>
       <c r="B35" s="20">
@@ -32637,7 +32669,7 @@
     <row r="36">
       <c r="A36" s="27" t="inlineStr">
         <is>
-          <t>SATIN</t>
+          <t>SAKSOFT</t>
         </is>
       </c>
       <c r="B36" s="20">
@@ -32680,7 +32712,7 @@
     <row r="37">
       <c r="A37" s="27" t="inlineStr">
         <is>
-          <t>SGFIN</t>
+          <t>SATIN</t>
         </is>
       </c>
       <c r="B37" s="20">
@@ -32723,7 +32755,7 @@
     <row r="38">
       <c r="A38" s="27" t="inlineStr">
         <is>
-          <t>SHRINGARMS</t>
+          <t>SGFIN</t>
         </is>
       </c>
       <c r="B38" s="20">
@@ -32766,7 +32798,7 @@
     <row r="39">
       <c r="A39" s="27" t="inlineStr">
         <is>
-          <t>SIMPLEXINF</t>
+          <t>SHRINGARMS</t>
         </is>
       </c>
       <c r="B39" s="20">
@@ -32809,7 +32841,7 @@
     <row r="40">
       <c r="A40" s="27" t="inlineStr">
         <is>
-          <t>SMCGLOBAL</t>
+          <t>SIMPLEXINF</t>
         </is>
       </c>
       <c r="B40" s="20">
@@ -32852,7 +32884,7 @@
     <row r="41">
       <c r="A41" s="27" t="inlineStr">
         <is>
-          <t>SOLARA</t>
+          <t>SMCGLOBAL</t>
         </is>
       </c>
       <c r="B41" s="20">
@@ -32895,7 +32927,7 @@
     <row r="42">
       <c r="A42" s="27" t="inlineStr">
         <is>
-          <t>SPORTKING</t>
+          <t>SOLARA</t>
         </is>
       </c>
       <c r="B42" s="20">
@@ -32938,7 +32970,7 @@
     <row r="43">
       <c r="A43" s="27" t="inlineStr">
         <is>
-          <t>SUNCLAY</t>
+          <t>SPORTKING</t>
         </is>
       </c>
       <c r="B43" s="20">
@@ -32981,7 +33013,7 @@
     <row r="44">
       <c r="A44" s="27" t="inlineStr">
         <is>
-          <t>SWARAJENG</t>
+          <t>SUNCLAY</t>
         </is>
       </c>
       <c r="B44" s="20">
@@ -33024,7 +33056,7 @@
     <row r="45">
       <c r="A45" s="27" t="inlineStr">
         <is>
-          <t>TEAMLEASE</t>
+          <t>SWARAJENG</t>
         </is>
       </c>
       <c r="B45" s="20">
@@ -33067,7 +33099,7 @@
     <row r="46">
       <c r="A46" s="27" t="inlineStr">
         <is>
-          <t>YUKEN</t>
+          <t>TEAMLEASE</t>
         </is>
       </c>
       <c r="B46" s="20">
@@ -33108,37 +33140,80 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="3" t="inlineStr">
+      <c r="A47" s="27" t="inlineStr">
+        <is>
+          <t>YUKEN</t>
+        </is>
+      </c>
+      <c r="B47" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A47)</f>
+        <v/>
+      </c>
+      <c r="C47" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A47,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D47" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A47,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E47" s="22">
+        <f>IFERROR($C47/$B47,"")</f>
+        <v/>
+      </c>
+      <c r="F47" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A47,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G47" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A47,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H47" s="21">
+        <f>IFERROR($G47/$B47,"")</f>
+        <v/>
+      </c>
+      <c r="I47" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A47),"")</f>
+        <v/>
+      </c>
+      <c r="J47" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A47),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B47" s="30">
-        <f>SUM(B4:B46)</f>
-        <v/>
-      </c>
-      <c r="C47" s="30">
-        <f>SUM(C4:C46)</f>
-        <v/>
-      </c>
-      <c r="D47" s="30">
-        <f>SUM(D4:D46)</f>
-        <v/>
-      </c>
-      <c r="E47" s="31">
-        <f>IFERROR(C47/B47,"")</f>
-        <v/>
-      </c>
-      <c r="F47" s="32">
-        <f>SUM(F4:F46)</f>
-        <v/>
-      </c>
-      <c r="G47" s="32">
-        <f>SUM(G4:G46)</f>
-        <v/>
-      </c>
-      <c r="H47" s="32">
-        <f>IFERROR(G47/B47,"")</f>
+      <c r="B48" s="30">
+        <f>SUM(B4:B47)</f>
+        <v/>
+      </c>
+      <c r="C48" s="30">
+        <f>SUM(C4:C47)</f>
+        <v/>
+      </c>
+      <c r="D48" s="30">
+        <f>SUM(D4:D47)</f>
+        <v/>
+      </c>
+      <c r="E48" s="31">
+        <f>IFERROR(C48/B48,"")</f>
+        <v/>
+      </c>
+      <c r="F48" s="32">
+        <f>SUM(F4:F47)</f>
+        <v/>
+      </c>
+      <c r="G48" s="32">
+        <f>SUM(G4:G47)</f>
+        <v/>
+      </c>
+      <c r="H48" s="32">
+        <f>IFERROR(G48/B48,"")</f>
         <v/>
       </c>
     </row>
@@ -33157,7 +33232,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N56"/>
+  <dimension ref="A1:N57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -33408,7 +33483,7 @@
         <v>35.4</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>115.97</v>
+        <v>115.99</v>
       </c>
       <c r="N6" s="21">
         <f>SUM(E6:M6)</f>
@@ -33459,7 +33534,7 @@
         <v>35.4</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>69.34</v>
+        <v>69.34999999999999</v>
       </c>
       <c r="N7" s="21">
         <f>SUM(E7:M7)</f>
@@ -33510,7 +33585,7 @@
         <v>35.4</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>96.48999999999999</v>
+        <v>96.51000000000001</v>
       </c>
       <c r="N8" s="21">
         <f>SUM(E8:M8)</f>
@@ -33561,7 +33636,7 @@
         <v>35.4</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>115.64</v>
+        <v>115.66</v>
       </c>
       <c r="N9" s="21">
         <f>SUM(E9:M9)</f>
@@ -33612,7 +33687,7 @@
         <v>35.4</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>96.5</v>
+        <v>96.52</v>
       </c>
       <c r="N10" s="21">
         <f>SUM(E10:M10)</f>
@@ -33663,7 +33738,7 @@
         <v>35.4</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>59.8</v>
+        <v>59.52</v>
       </c>
       <c r="N11" s="21">
         <f>SUM(E11:M11)</f>
@@ -33714,7 +33789,7 @@
         <v>35.4</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>71.66</v>
+        <v>71.33</v>
       </c>
       <c r="N12" s="21">
         <f>SUM(E12:M12)</f>
@@ -33765,7 +33840,7 @@
         <v>35.4</v>
       </c>
       <c r="M13" s="4" t="n">
-        <v>73.45</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="N13" s="21">
         <f>SUM(E13:M13)</f>
@@ -33816,7 +33891,7 @@
         <v>35.4</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>59.61</v>
+        <v>59.33</v>
       </c>
       <c r="N14" s="21">
         <f>SUM(E14:M14)</f>
@@ -33969,7 +34044,7 @@
         <v>35.4</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>84.45</v>
+        <v>83.31999999999999</v>
       </c>
       <c r="N17" s="21">
         <f>SUM(E17:M17)</f>
@@ -34071,7 +34146,7 @@
         <v>35.4</v>
       </c>
       <c r="M19" s="4" t="n">
-        <v>87.61</v>
+        <v>86.48999999999999</v>
       </c>
       <c r="N19" s="21">
         <f>SUM(E19:M19)</f>
@@ -34122,7 +34197,7 @@
         <v>35.4</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>84.55</v>
+        <v>83.41</v>
       </c>
       <c r="N20" s="21">
         <f>SUM(E20:M20)</f>
@@ -34224,7 +34299,7 @@
         <v>35.4</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>84.95</v>
+        <v>83.81</v>
       </c>
       <c r="N22" s="21">
         <f>SUM(E22:M22)</f>
@@ -34275,7 +34350,7 @@
         <v>35.4</v>
       </c>
       <c r="M23" s="4" t="n">
-        <v>30.25</v>
+        <v>29.85</v>
       </c>
       <c r="N23" s="21">
         <f>SUM(E23:M23)</f>
@@ -34377,7 +34452,7 @@
         <v>35.4</v>
       </c>
       <c r="M25" s="4" t="n">
-        <v>37.61</v>
+        <v>37.09</v>
       </c>
       <c r="N25" s="21">
         <f>SUM(E25:M25)</f>
@@ -34479,7 +34554,7 @@
         <v>35.4</v>
       </c>
       <c r="M27" s="4" t="n">
-        <v>36.18</v>
+        <v>35.69</v>
       </c>
       <c r="N27" s="21">
         <f>SUM(E27:M27)</f>
@@ -34530,7 +34605,7 @@
         <v>35.4</v>
       </c>
       <c r="M28" s="4" t="n">
-        <v>41.42</v>
+        <v>40.87</v>
       </c>
       <c r="N28" s="21">
         <f>SUM(E28:M28)</f>
@@ -34581,7 +34656,7 @@
         <v>35.4</v>
       </c>
       <c r="M29" s="4" t="n">
-        <v>43.19</v>
+        <v>42.59</v>
       </c>
       <c r="N29" s="21">
         <f>SUM(E29:M29)</f>
@@ -34632,7 +34707,7 @@
         <v>35.4</v>
       </c>
       <c r="M30" s="4" t="n">
-        <v>36.14</v>
+        <v>35.66</v>
       </c>
       <c r="N30" s="21">
         <f>SUM(E30:M30)</f>
@@ -34785,7 +34860,7 @@
         <v>35.4</v>
       </c>
       <c r="M33" s="4" t="n">
-        <v>35.86</v>
+        <v>35.38</v>
       </c>
       <c r="N33" s="21">
         <f>SUM(E33:M33)</f>
@@ -34836,7 +34911,7 @@
         <v>35.4</v>
       </c>
       <c r="M34" s="4" t="n">
-        <v>38.2</v>
+        <v>37.65</v>
       </c>
       <c r="N34" s="21">
         <f>SUM(E34:M34)</f>
@@ -34938,7 +35013,7 @@
         <v>35.4</v>
       </c>
       <c r="M36" s="4" t="n">
-        <v>21.66</v>
+        <v>35.61</v>
       </c>
       <c r="N36" s="21">
         <f>SUM(E36:M36)</f>
@@ -34989,7 +35064,7 @@
         <v>35.4</v>
       </c>
       <c r="M37" s="4" t="n">
-        <v>32.35</v>
+        <v>31.6</v>
       </c>
       <c r="N37" s="21">
         <f>SUM(E37:M37)</f>
@@ -35040,7 +35115,7 @@
         <v>35.4</v>
       </c>
       <c r="M38" s="4" t="n">
-        <v>35.17</v>
+        <v>34.69</v>
       </c>
       <c r="N38" s="21">
         <f>SUM(E38:M38)</f>
@@ -35091,7 +35166,7 @@
         <v>35.4</v>
       </c>
       <c r="M39" s="4" t="n">
-        <v>34.94</v>
+        <v>34.47</v>
       </c>
       <c r="N39" s="21">
         <f>SUM(E39:M39)</f>
@@ -35193,7 +35268,7 @@
         <v>35.4</v>
       </c>
       <c r="M41" s="4" t="n">
-        <v>35.12</v>
+        <v>234.08</v>
       </c>
       <c r="N41" s="21">
         <f>SUM(E41:M41)</f>
@@ -35244,7 +35319,7 @@
         <v>35.4</v>
       </c>
       <c r="M42" s="4" t="n">
-        <v>28.13</v>
+        <v>27.76</v>
       </c>
       <c r="N42" s="21">
         <f>SUM(E42:M42)</f>
@@ -35295,7 +35370,7 @@
         <v>35.4</v>
       </c>
       <c r="M43" s="4" t="n">
-        <v>33.53</v>
+        <v>80.42</v>
       </c>
       <c r="N43" s="21">
         <f>SUM(E43:M43)</f>
@@ -35397,7 +35472,7 @@
         <v>35.4</v>
       </c>
       <c r="M45" s="4" t="n">
-        <v>35.6</v>
+        <v>85.64</v>
       </c>
       <c r="N45" s="21">
         <f>SUM(E45:M45)</f>
@@ -35448,7 +35523,7 @@
         <v>35.4</v>
       </c>
       <c r="M46" s="4" t="n">
-        <v>31.44</v>
+        <v>75.66</v>
       </c>
       <c r="N46" s="21">
         <f>SUM(E46:M46)</f>
@@ -35499,7 +35574,7 @@
         <v>35.4</v>
       </c>
       <c r="M47" s="4" t="n">
-        <v>183.83</v>
+        <v>178.81</v>
       </c>
       <c r="N47" s="21">
         <f>SUM(E47:M47)</f>
@@ -35550,7 +35625,7 @@
         <v>35.4</v>
       </c>
       <c r="M48" s="4" t="n">
-        <v>184.81</v>
+        <v>179.77</v>
       </c>
       <c r="N48" s="21">
         <f>SUM(E48:M48)</f>
@@ -35601,7 +35676,7 @@
         <v>35.4</v>
       </c>
       <c r="M49" s="4" t="n">
-        <v>180.19</v>
+        <v>175.22</v>
       </c>
       <c r="N49" s="21">
         <f>SUM(E49:M49)</f>
@@ -35652,7 +35727,7 @@
         <v>35.4</v>
       </c>
       <c r="M50" s="4" t="n">
-        <v>185.18</v>
+        <v>180.13</v>
       </c>
       <c r="N50" s="21">
         <f>SUM(E50:M50)</f>
@@ -35703,7 +35778,7 @@
         <v>35.4</v>
       </c>
       <c r="M51" s="4" t="n">
-        <v>130.56</v>
+        <v>142.42</v>
       </c>
       <c r="N51" s="21">
         <f>SUM(E51:M51)</f>
@@ -35754,7 +35829,7 @@
         <v>35.4</v>
       </c>
       <c r="M52" s="4" t="n">
-        <v>102.32</v>
+        <v>111.97</v>
       </c>
       <c r="N52" s="21">
         <f>SUM(E52:M52)</f>
@@ -35828,24 +35903,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D54" s="24" t="inlineStr"/>
+      <c r="D54" s="24" t="n">
+        <v>46321</v>
+      </c>
       <c r="E54" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F54" s="4" t="n">
-        <v>0</v>
+        <v>150.05</v>
       </c>
       <c r="G54" s="4" t="n">
-        <v>0</v>
+        <v>4.61</v>
       </c>
       <c r="H54" s="4" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="I54" s="4" t="n">
-        <v>0</v>
+        <v>22.51</v>
       </c>
       <c r="J54" s="4" t="n">
-        <v>0</v>
+        <v>0.86</v>
       </c>
       <c r="K54" s="4" t="n">
         <v>14.75</v>
@@ -35877,24 +35954,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D55" s="24" t="inlineStr"/>
+      <c r="D55" s="24" t="n">
+        <v>46321</v>
+      </c>
       <c r="E55" s="4" t="n">
-        <v>0</v>
+        <v>89.3</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>0</v>
+        <v>297.95</v>
       </c>
       <c r="G55" s="4" t="n">
-        <v>0</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="H55" s="4" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="I55" s="4" t="n">
-        <v>0</v>
+        <v>44.49</v>
       </c>
       <c r="J55" s="4" t="n">
-        <v>0</v>
+        <v>17.77</v>
       </c>
       <c r="K55" s="4" t="n">
         <v>14.75</v>
@@ -35903,7 +35982,7 @@
         <v>35.4</v>
       </c>
       <c r="M55" s="4" t="n">
-        <v>0</v>
+        <v>46.37</v>
       </c>
       <c r="N55" s="21">
         <f>SUM(E55:M55)</f>
@@ -35911,54 +35990,103 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="3" t="inlineStr">
+      <c r="A56" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126102699709+221261026669809+321261026636409+321261026636909+23126102699809+34126102699309+221261026670609+221261026671109+231261026100009+231261026100109+34126102699609+34126102699709</t>
+        </is>
+      </c>
+      <c r="B56" s="23" t="inlineStr">
+        <is>
+          <t>INDOSTAR</t>
+        </is>
+      </c>
+      <c r="C56" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D56" s="24" t="inlineStr"/>
+      <c r="E56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K56" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L56" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N56" s="21">
+        <f>SUM(E56:M56)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E56" s="32">
-        <f>SUM(E4:E55)</f>
-        <v/>
-      </c>
-      <c r="F56" s="32">
-        <f>SUM(F4:F55)</f>
-        <v/>
-      </c>
-      <c r="G56" s="32">
-        <f>SUM(G4:G55)</f>
-        <v/>
-      </c>
-      <c r="H56" s="32">
-        <f>SUM(H4:H55)</f>
-        <v/>
-      </c>
-      <c r="I56" s="32">
-        <f>SUM(I4:I55)</f>
-        <v/>
-      </c>
-      <c r="J56" s="32">
-        <f>SUM(J4:J55)</f>
-        <v/>
-      </c>
-      <c r="K56" s="32">
-        <f>SUM(K4:K55)</f>
-        <v/>
-      </c>
-      <c r="L56" s="32">
-        <f>SUM(L4:L55)</f>
-        <v/>
-      </c>
-      <c r="M56" s="32">
-        <f>SUM(M4:M55)</f>
-        <v/>
-      </c>
-      <c r="N56" s="32">
-        <f>SUM(N4:N55)</f>
+      <c r="E57" s="32">
+        <f>SUM(E4:E56)</f>
+        <v/>
+      </c>
+      <c r="F57" s="32">
+        <f>SUM(F4:F56)</f>
+        <v/>
+      </c>
+      <c r="G57" s="32">
+        <f>SUM(G4:G56)</f>
+        <v/>
+      </c>
+      <c r="H57" s="32">
+        <f>SUM(H4:H56)</f>
+        <v/>
+      </c>
+      <c r="I57" s="32">
+        <f>SUM(I4:I56)</f>
+        <v/>
+      </c>
+      <c r="J57" s="32">
+        <f>SUM(J4:J56)</f>
+        <v/>
+      </c>
+      <c r="K57" s="32">
+        <f>SUM(K4:K56)</f>
+        <v/>
+      </c>
+      <c r="L57" s="32">
+        <f>SUM(L4:L56)</f>
+        <v/>
+      </c>
+      <c r="M57" s="32">
+        <f>SUM(M4:M56)</f>
+        <v/>
+      </c>
+      <c r="N57" s="32">
+        <f>SUM(N4:N56)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:N55"/>
+  <autoFilter ref="A3:N56"/>
   <mergeCells count="2">
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>
@@ -35973,7 +36101,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -36353,40 +36481,85 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="28" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B13" s="20">
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,26),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,11,2))</f>
+        <v/>
+      </c>
+      <c r="C13" s="20">
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,26),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,11,2),'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D13" s="20">
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,26),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,11,2),'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E13" s="22">
+        <f>IFERROR($C13/$B13,"")</f>
+        <v/>
+      </c>
+      <c r="F13" s="21">
+        <f>SUMIFS('Trade Log'!$I$4:$I$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,26),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,11,2))</f>
+        <v/>
+      </c>
+      <c r="G13" s="21">
+        <f>SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,26),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,11,2))</f>
+        <v/>
+      </c>
+      <c r="H13" s="21">
+        <f>IFERROR($G13/$B13,"")</f>
+        <v/>
+      </c>
+      <c r="I13" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,26),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,11,2)),"")</f>
+        <v/>
+      </c>
+      <c r="J13" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,26),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,11,2)),"")</f>
+        <v/>
+      </c>
+      <c r="K13" s="29">
+        <f>IFERROR(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,26),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,11,2),'Trade Log'!$L$4:$L$503,"&gt;0")/ABS(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,26),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,11,2),'Trade Log'!$L$4:$L$503,"&lt;0")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B13" s="30">
-        <f>SUM(B10:B12)</f>
-        <v/>
-      </c>
-      <c r="C13" s="30">
-        <f>SUM(C10:C12)</f>
-        <v/>
-      </c>
-      <c r="D13" s="30">
-        <f>SUM(D10:D12)</f>
-        <v/>
-      </c>
-      <c r="E13" s="31">
-        <f>IFERROR(C13/B13,"")</f>
-        <v/>
-      </c>
-      <c r="F13" s="32">
-        <f>SUM(F10:F12)</f>
-        <v/>
-      </c>
-      <c r="G13" s="32">
-        <f>SUM(G10:G12)</f>
-        <v/>
-      </c>
-      <c r="H13" s="32">
-        <f>IFERROR(G13/B13,"")</f>
-        <v/>
-      </c>
-      <c r="K13" s="33">
+      <c r="B14" s="30">
+        <f>SUM(B10:B13)</f>
+        <v/>
+      </c>
+      <c r="C14" s="30">
+        <f>SUM(C10:C13)</f>
+        <v/>
+      </c>
+      <c r="D14" s="30">
+        <f>SUM(D10:D13)</f>
+        <v/>
+      </c>
+      <c r="E14" s="31">
+        <f>IFERROR(C14/B14,"")</f>
+        <v/>
+      </c>
+      <c r="F14" s="32">
+        <f>SUM(F10:F13)</f>
+        <v/>
+      </c>
+      <c r="G14" s="32">
+        <f>SUM(G10:G13)</f>
+        <v/>
+      </c>
+      <c r="H14" s="32">
+        <f>IFERROR(G14/B14,"")</f>
+        <v/>
+      </c>
+      <c r="K14" s="33">
         <f>IFERROR(SUMIF('Trade Log'!$L$4:$L$503,"&gt;0")/ABS(SUMIF('Trade Log'!$L$4:$L$503,"&lt;0")),"")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Data update — 2026-10-27 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_oct2026.xlsx
+++ b/results/strategy_pnl_oct2026.xlsx
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trade Log'!$A$3:$O$503</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$64</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1274,7 +1274,7 @@
         <v/>
       </c>
       <c r="K7" s="4" t="n">
-        <v>819.04</v>
+        <v>819.03</v>
       </c>
       <c r="L7" s="21">
         <f>IF(OR($B7="",$I7=""),"",$I7-IF($K7="",0,$K7))</f>
@@ -1334,7 +1334,7 @@
         <v/>
       </c>
       <c r="K8" s="4" t="n">
-        <v>857.27</v>
+        <v>857.26</v>
       </c>
       <c r="L8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($K8="",0,$K8))</f>
@@ -1394,7 +1394,7 @@
         <v/>
       </c>
       <c r="K9" s="4" t="n">
-        <v>969.48</v>
+        <v>969.47</v>
       </c>
       <c r="L9" s="21">
         <f>IF(OR($B9="",$I9=""),"",$I9-IF($K9="",0,$K9))</f>
@@ -1454,7 +1454,7 @@
         <v/>
       </c>
       <c r="K10" s="4" t="n">
-        <v>943.04</v>
+        <v>943.03</v>
       </c>
       <c r="L10" s="21">
         <f>IF(OR($B10="",$I10=""),"",$I10-IF($K10="",0,$K10))</f>
@@ -1574,7 +1574,7 @@
         <v/>
       </c>
       <c r="K12" s="4" t="n">
-        <v>756.38</v>
+        <v>756.37</v>
       </c>
       <c r="L12" s="21">
         <f>IF(OR($B12="",$I12=""),"",$I12-IF($K12="",0,$K12))</f>
@@ -1634,7 +1634,7 @@
         <v/>
       </c>
       <c r="K13" s="4" t="n">
-        <v>687.86</v>
+        <v>687.9299999999999</v>
       </c>
       <c r="L13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($K13="",0,$K13))</f>
@@ -1694,7 +1694,7 @@
         <v/>
       </c>
       <c r="K14" s="4" t="n">
-        <v>683.87</v>
+        <v>683.86</v>
       </c>
       <c r="L14" s="21">
         <f>IF(OR($B14="",$I14=""),"",$I14-IF($K14="",0,$K14))</f>
@@ -1874,7 +1874,7 @@
         <v/>
       </c>
       <c r="K17" s="4" t="n">
-        <v>660.9400000000001</v>
+        <v>660.95</v>
       </c>
       <c r="L17" s="21">
         <f>IF(OR($B17="",$I17=""),"",$I17-IF($K17="",0,$K17))</f>
@@ -1994,7 +1994,7 @@
         <v/>
       </c>
       <c r="K19" s="4" t="n">
-        <v>666.67</v>
+        <v>666.74</v>
       </c>
       <c r="L19" s="21">
         <f>IF(OR($B19="",$I19=""),"",$I19-IF($K19="",0,$K19))</f>
@@ -2354,7 +2354,7 @@
         <v/>
       </c>
       <c r="K25" s="4" t="n">
-        <v>557.29</v>
+        <v>557.3</v>
       </c>
       <c r="L25" s="21">
         <f>IF(OR($B25="",$I25=""),"",$I25-IF($K25="",0,$K25))</f>
@@ -2594,7 +2594,7 @@
         <v/>
       </c>
       <c r="K29" s="4" t="n">
-        <v>554.59</v>
+        <v>554.6</v>
       </c>
       <c r="L29" s="21">
         <f>IF(OR($B29="",$I29=""),"",$I29-IF($K29="",0,$K29))</f>
@@ -2894,7 +2894,7 @@
         <v/>
       </c>
       <c r="K34" s="4" t="n">
-        <v>425.96</v>
+        <v>425.99</v>
       </c>
       <c r="L34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($K34="",0,$K34))</f>
@@ -3074,7 +3074,7 @@
         <v/>
       </c>
       <c r="K37" s="4" t="n">
-        <v>478.05</v>
+        <v>477.87</v>
       </c>
       <c r="L37" s="21">
         <f>IF(OR($B37="",$I37=""),"",$I37-IF($K37="",0,$K37))</f>
@@ -3314,7 +3314,7 @@
         <v/>
       </c>
       <c r="K41" s="4" t="n">
-        <v>592.26</v>
+        <v>592.28</v>
       </c>
       <c r="L41" s="21">
         <f>IF(OR($B41="",$I41=""),"",$I41-IF($K41="",0,$K41))</f>
@@ -3434,7 +3434,7 @@
         <v/>
       </c>
       <c r="K43" s="4" t="n">
-        <v>924.52</v>
+        <v>924.55</v>
       </c>
       <c r="L43" s="21">
         <f>IF(OR($B43="",$I43=""),"",$I43-IF($K43="",0,$K43))</f>
@@ -3554,7 +3554,7 @@
         <v/>
       </c>
       <c r="K45" s="4" t="n">
-        <v>945.8200000000001</v>
+        <v>945.87</v>
       </c>
       <c r="L45" s="21">
         <f>IF(OR($B45="",$I45=""),"",$I45-IF($K45="",0,$K45))</f>
@@ -3614,7 +3614,7 @@
         <v/>
       </c>
       <c r="K46" s="4" t="n">
-        <v>915.86</v>
+        <v>915.87</v>
       </c>
       <c r="L46" s="21">
         <f>IF(OR($B46="",$I46=""),"",$I46-IF($K46="",0,$K46))</f>
@@ -3674,7 +3674,7 @@
         <v/>
       </c>
       <c r="K47" s="4" t="n">
-        <v>1026.85</v>
+        <v>1026.87</v>
       </c>
       <c r="L47" s="21">
         <f>IF(OR($B47="",$I47=""),"",$I47-IF($K47="",0,$K47))</f>
@@ -3734,7 +3734,7 @@
         <v/>
       </c>
       <c r="K48" s="4" t="n">
-        <v>1028.54</v>
+        <v>1028.56</v>
       </c>
       <c r="L48" s="21">
         <f>IF(OR($B48="",$I48=""),"",$I48-IF($K48="",0,$K48))</f>
@@ -3794,7 +3794,7 @@
         <v/>
       </c>
       <c r="K49" s="4" t="n">
-        <v>955.05</v>
+        <v>955.1</v>
       </c>
       <c r="L49" s="21">
         <f>IF(OR($B49="",$I49=""),"",$I49-IF($K49="",0,$K49))</f>
@@ -3854,7 +3854,7 @@
         <v/>
       </c>
       <c r="K50" s="4" t="n">
-        <v>1035.24</v>
+        <v>1035.26</v>
       </c>
       <c r="L50" s="21">
         <f>IF(OR($B50="",$I50=""),"",$I50-IF($K50="",0,$K50))</f>
@@ -3914,7 +3914,7 @@
         <v/>
       </c>
       <c r="K51" s="4" t="n">
-        <v>984.48</v>
+        <v>984.54</v>
       </c>
       <c r="L51" s="21">
         <f>IF(OR($B51="",$I51=""),"",$I51-IF($K51="",0,$K51))</f>
@@ -3974,7 +3974,7 @@
         <v/>
       </c>
       <c r="K52" s="4" t="n">
-        <v>939.9299999999999</v>
+        <v>939.9400000000001</v>
       </c>
       <c r="L52" s="21">
         <f>IF(OR($B52="",$I52=""),"",$I52-IF($K52="",0,$K52))</f>
@@ -4094,7 +4094,7 @@
         <v/>
       </c>
       <c r="K54" s="4" t="n">
-        <v>192.92</v>
+        <v>222.31</v>
       </c>
       <c r="L54" s="21">
         <f>IF(OR($B54="",$I54=""),"",$I54-IF($K54="",0,$K54))</f>
@@ -4117,33 +4117,33 @@
     <row r="55">
       <c r="A55" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261023807609+321261023756809+231261023120609+221261023808709+221261023809309+231261023120909+221261023809609+231261023121109+341261023126209+341261023126309+341261023126509+341261023126609+321261023760409</t>
+          <t>DHAN-23126102637609</t>
         </is>
       </c>
       <c r="B55" s="23" t="inlineStr">
         <is>
-          <t>JINDALPOLY</t>
+          <t>FISCHER</t>
         </is>
       </c>
       <c r="C55" s="23" t="inlineStr">
         <is>
-          <t>LONG</t>
+          <t>SHORT</t>
         </is>
       </c>
       <c r="D55" s="24" t="n">
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="E55" s="25" t="n">
-        <v>726.0981</v>
+        <v>25.7414</v>
       </c>
       <c r="F55" s="26" t="n">
-        <v>410</v>
+        <v>6007</v>
       </c>
       <c r="G55" s="24" t="n">
         <v>46321</v>
       </c>
       <c r="H55" s="25" t="n">
-        <v>696</v>
+        <v>26.5045</v>
       </c>
       <c r="I55" s="21">
         <f>IF(OR($B55="",$H55=""),"",IF($C55="LONG",($H55-$E55)*$F55,($E55-$H55)*$F55))</f>
@@ -4154,7 +4154,7 @@
         <v/>
       </c>
       <c r="K55" s="4" t="n">
-        <v>555.48</v>
+        <v>161.96</v>
       </c>
       <c r="L55" s="21">
         <f>IF(OR($B55="",$I55=""),"",$I55-IF($K55="",0,$K55))</f>
@@ -4170,19 +4170,19 @@
       </c>
       <c r="O55" s="23" t="inlineStr">
         <is>
-          <t>10-15</t>
+          <t>5-10</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="23" t="inlineStr">
         <is>
-          <t>DHAN-23126102699709+221261026669809+321261026636409+321261026636909+23126102699809+34126102699309+221261026670609+221261026671109+231261026100009+231261026100109+34126102699609+34126102699709</t>
+          <t>DHAN-221261023807609+321261023756809+231261023120609+221261023808709+221261023809309+231261023120909+221261023809609+231261023121109+341261023126209+341261023126309+341261023126509+341261023126609+321261023760409</t>
         </is>
       </c>
       <c r="B56" s="23" t="inlineStr">
         <is>
-          <t>INDOSTAR</t>
+          <t>JINDALPOLY</t>
         </is>
       </c>
       <c r="C56" s="23" t="inlineStr">
@@ -4191,16 +4191,20 @@
         </is>
       </c>
       <c r="D56" s="24" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E56" s="25" t="n">
+        <v>726.0981</v>
+      </c>
+      <c r="F56" s="26" t="n">
+        <v>410</v>
+      </c>
+      <c r="G56" s="24" t="n">
         <v>46321</v>
       </c>
-      <c r="E56" s="25" t="n">
-        <v>183.525</v>
-      </c>
-      <c r="F56" s="26" t="n">
-        <v>1635</v>
-      </c>
-      <c r="G56" s="24" t="inlineStr"/>
-      <c r="H56" s="25" t="inlineStr"/>
+      <c r="H56" s="25" t="n">
+        <v>696</v>
+      </c>
       <c r="I56" s="21">
         <f>IF(OR($B56="",$H56=""),"",IF($C56="LONG",($H56-$E56)*$F56,($E56-$H56)*$F56))</f>
         <v/>
@@ -4210,7 +4214,7 @@
         <v/>
       </c>
       <c r="K56" s="4" t="n">
-        <v>50.15</v>
+        <v>875.1900000000001</v>
       </c>
       <c r="L56" s="21">
         <f>IF(OR($B56="",$I56=""),"",$I56-IF($K56="",0,$K56))</f>
@@ -4231,14 +4235,36 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="23" t="n"/>
-      <c r="B57" s="23" t="n"/>
-      <c r="C57" s="23" t="n"/>
-      <c r="D57" s="24" t="n"/>
-      <c r="E57" s="25" t="n"/>
-      <c r="F57" s="26" t="n"/>
-      <c r="G57" s="24" t="n"/>
-      <c r="H57" s="25" t="n"/>
+      <c r="A57" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126102699709+221261026669809+321261026636409+321261026636909+23126102699809+34126102699309+221261026670609+221261026671109+231261026100009+231261026100109+34126102699609+34126102699709</t>
+        </is>
+      </c>
+      <c r="B57" s="23" t="inlineStr">
+        <is>
+          <t>INDOSTAR</t>
+        </is>
+      </c>
+      <c r="C57" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D57" s="24" t="n">
+        <v>46321</v>
+      </c>
+      <c r="E57" s="25" t="n">
+        <v>183.525</v>
+      </c>
+      <c r="F57" s="26" t="n">
+        <v>1635</v>
+      </c>
+      <c r="G57" s="24" t="n">
+        <v>46322</v>
+      </c>
+      <c r="H57" s="25" t="n">
+        <v>192.4</v>
+      </c>
       <c r="I57" s="21">
         <f>IF(OR($B57="",$H57=""),"",IF($C57="LONG",($H57-$E57)*$F57,($E57-$H57)*$F57))</f>
         <v/>
@@ -4247,7 +4273,9 @@
         <f>IF(OR($B57="",$I57="",$E57=0,$F57=0),"",$I57/($E57*$F57))</f>
         <v/>
       </c>
-      <c r="K57" s="4" t="n"/>
+      <c r="K57" s="4" t="n">
+        <v>574.5</v>
+      </c>
       <c r="L57" s="21">
         <f>IF(OR($B57="",$I57=""),"",$I57-IF($K57="",0,$K57))</f>
         <v/>
@@ -4260,17 +4288,39 @@
         <f>IF($B57="","",IF($H57="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O57" s="23" t="n"/>
+      <c r="O57" s="23" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
     </row>
     <row r="58">
-      <c r="A58" s="23" t="n"/>
-      <c r="B58" s="23" t="n"/>
-      <c r="C58" s="23" t="n"/>
-      <c r="D58" s="24" t="n"/>
-      <c r="E58" s="25" t="n"/>
-      <c r="F58" s="26" t="n"/>
-      <c r="G58" s="24" t="n"/>
-      <c r="H58" s="25" t="n"/>
+      <c r="A58" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126102781109+34126102781509+23126102780909+34126102781709+321261027587409+23126102781709+321261027588509+221261027607309+23126102782009+34126102783009+23126102782409+221261027608709+23126102782709+321261027592209</t>
+        </is>
+      </c>
+      <c r="B58" s="23" t="inlineStr">
+        <is>
+          <t>AGIIL</t>
+        </is>
+      </c>
+      <c r="C58" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D58" s="24" t="n">
+        <v>46322</v>
+      </c>
+      <c r="E58" s="25" t="n">
+        <v>233.1162</v>
+      </c>
+      <c r="F58" s="26" t="n">
+        <v>737</v>
+      </c>
+      <c r="G58" s="24" t="inlineStr"/>
+      <c r="H58" s="25" t="inlineStr"/>
       <c r="I58" s="21">
         <f>IF(OR($B58="",$H58=""),"",IF($C58="LONG",($H58-$E58)*$F58,($E58-$H58)*$F58))</f>
         <v/>
@@ -4279,7 +4329,9 @@
         <f>IF(OR($B58="",$I58="",$E58=0,$F58=0),"",$I58/($E58*$F58))</f>
         <v/>
       </c>
-      <c r="K58" s="4" t="n"/>
+      <c r="K58" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L58" s="21">
         <f>IF(OR($B58="",$I58=""),"",$I58-IF($K58="",0,$K58))</f>
         <v/>
@@ -4292,17 +4344,39 @@
         <f>IF($B58="","",IF($H58="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O58" s="23" t="n"/>
+      <c r="O58" s="23" t="inlineStr">
+        <is>
+          <t>15-20</t>
+        </is>
+      </c>
     </row>
     <row r="59">
-      <c r="A59" s="23" t="n"/>
-      <c r="B59" s="23" t="n"/>
-      <c r="C59" s="23" t="n"/>
-      <c r="D59" s="24" t="n"/>
-      <c r="E59" s="25" t="n"/>
-      <c r="F59" s="26" t="n"/>
-      <c r="G59" s="24" t="n"/>
-      <c r="H59" s="25" t="n"/>
+      <c r="A59" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126102780509+34126102781309+23126102781009+23126102781209+221261027605909+34126102781909+321261027588609+23126102781809+321261027589309+23126102782209+321261027590909+23126102782809+34126102783609</t>
+        </is>
+      </c>
+      <c r="B59" s="23" t="inlineStr">
+        <is>
+          <t>BAJEL</t>
+        </is>
+      </c>
+      <c r="C59" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D59" s="24" t="n">
+        <v>46322</v>
+      </c>
+      <c r="E59" s="25" t="n">
+        <v>168.7027</v>
+      </c>
+      <c r="F59" s="26" t="n">
+        <v>507</v>
+      </c>
+      <c r="G59" s="24" t="inlineStr"/>
+      <c r="H59" s="25" t="inlineStr"/>
       <c r="I59" s="21">
         <f>IF(OR($B59="",$H59=""),"",IF($C59="LONG",($H59-$E59)*$F59,($E59-$H59)*$F59))</f>
         <v/>
@@ -4311,7 +4385,9 @@
         <f>IF(OR($B59="",$I59="",$E59=0,$F59=0),"",$I59/($E59*$F59))</f>
         <v/>
       </c>
-      <c r="K59" s="4" t="n"/>
+      <c r="K59" s="4" t="n">
+        <v>14.75</v>
+      </c>
       <c r="L59" s="21">
         <f>IF(OR($B59="",$I59=""),"",$I59-IF($K59="",0,$K59))</f>
         <v/>
@@ -4324,17 +4400,39 @@
         <f>IF($B59="","",IF($H59="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O59" s="23" t="n"/>
+      <c r="O59" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="60">
-      <c r="A60" s="23" t="n"/>
-      <c r="B60" s="23" t="n"/>
-      <c r="C60" s="23" t="n"/>
-      <c r="D60" s="24" t="n"/>
-      <c r="E60" s="25" t="n"/>
-      <c r="F60" s="26" t="n"/>
-      <c r="G60" s="24" t="n"/>
-      <c r="H60" s="25" t="n"/>
+      <c r="A60" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261027603909+23126102780809+34126102781609+221261027605309+34126102781809+221261027606409+34126102782209+34126102782709+221261027607909+34126102782909+34126102783209+34126102783409+321261027591809+23126102783009</t>
+        </is>
+      </c>
+      <c r="B60" s="23" t="inlineStr">
+        <is>
+          <t>BBL</t>
+        </is>
+      </c>
+      <c r="C60" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D60" s="24" t="n">
+        <v>46322</v>
+      </c>
+      <c r="E60" s="25" t="n">
+        <v>2588.2151</v>
+      </c>
+      <c r="F60" s="26" t="n">
+        <v>66</v>
+      </c>
+      <c r="G60" s="24" t="inlineStr"/>
+      <c r="H60" s="25" t="inlineStr"/>
       <c r="I60" s="21">
         <f>IF(OR($B60="",$H60=""),"",IF($C60="LONG",($H60-$E60)*$F60,($E60-$H60)*$F60))</f>
         <v/>
@@ -4343,7 +4441,9 @@
         <f>IF(OR($B60="",$I60="",$E60=0,$F60=0),"",$I60/($E60*$F60))</f>
         <v/>
       </c>
-      <c r="K60" s="4" t="n"/>
+      <c r="K60" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L60" s="21">
         <f>IF(OR($B60="",$I60=""),"",$I60-IF($K60="",0,$K60))</f>
         <v/>
@@ -4356,17 +4456,39 @@
         <f>IF($B60="","",IF($H60="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O60" s="23" t="n"/>
+      <c r="O60" s="23" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
     </row>
     <row r="61">
-      <c r="A61" s="23" t="n"/>
-      <c r="B61" s="23" t="n"/>
-      <c r="C61" s="23" t="n"/>
-      <c r="D61" s="24" t="n"/>
-      <c r="E61" s="25" t="n"/>
-      <c r="F61" s="26" t="n"/>
-      <c r="G61" s="24" t="n"/>
-      <c r="H61" s="25" t="n"/>
+      <c r="A61" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261027586409+221261027604309+221261027604909+221261027605409+221261027606009+221261027606309+221261027606809+23126102781909+321261027589409+321261027590009+221261027608409</t>
+        </is>
+      </c>
+      <c r="B61" s="23" t="inlineStr">
+        <is>
+          <t>JISLJALEQS</t>
+        </is>
+      </c>
+      <c r="C61" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D61" s="24" t="n">
+        <v>46322</v>
+      </c>
+      <c r="E61" s="25" t="n">
+        <v>24.9779</v>
+      </c>
+      <c r="F61" s="26" t="n">
+        <v>6857</v>
+      </c>
+      <c r="G61" s="24" t="inlineStr"/>
+      <c r="H61" s="25" t="inlineStr"/>
       <c r="I61" s="21">
         <f>IF(OR($B61="",$H61=""),"",IF($C61="LONG",($H61-$E61)*$F61,($E61-$H61)*$F61))</f>
         <v/>
@@ -4375,7 +4497,9 @@
         <f>IF(OR($B61="",$I61="",$E61=0,$F61=0),"",$I61/($E61*$F61))</f>
         <v/>
       </c>
-      <c r="K61" s="4" t="n"/>
+      <c r="K61" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L61" s="21">
         <f>IF(OR($B61="",$I61=""),"",$I61-IF($K61="",0,$K61))</f>
         <v/>
@@ -4388,17 +4512,39 @@
         <f>IF($B61="","",IF($H61="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O61" s="23" t="n"/>
+      <c r="O61" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="62">
-      <c r="A62" s="23" t="n"/>
-      <c r="B62" s="23" t="n"/>
-      <c r="C62" s="23" t="n"/>
-      <c r="D62" s="24" t="n"/>
-      <c r="E62" s="25" t="n"/>
-      <c r="F62" s="26" t="n"/>
-      <c r="G62" s="24" t="n"/>
-      <c r="H62" s="25" t="n"/>
+      <c r="A62" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261027603809+34126102781409+221261027604809+321261027587109+23126102781309+23126102781609+34126102782109+34126102782609+321261027589509+321261027590209+34126102783109+23126102782509</t>
+        </is>
+      </c>
+      <c r="B62" s="23" t="inlineStr">
+        <is>
+          <t>MAHLOG</t>
+        </is>
+      </c>
+      <c r="C62" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D62" s="24" t="n">
+        <v>46322</v>
+      </c>
+      <c r="E62" s="25" t="n">
+        <v>434.8638</v>
+      </c>
+      <c r="F62" s="26" t="n">
+        <v>394</v>
+      </c>
+      <c r="G62" s="24" t="inlineStr"/>
+      <c r="H62" s="25" t="inlineStr"/>
       <c r="I62" s="21">
         <f>IF(OR($B62="",$H62=""),"",IF($C62="LONG",($H62-$E62)*$F62,($E62-$H62)*$F62))</f>
         <v/>
@@ -4407,7 +4553,9 @@
         <f>IF(OR($B62="",$I62="",$E62=0,$F62=0),"",$I62/($E62*$F62))</f>
         <v/>
       </c>
-      <c r="K62" s="4" t="n"/>
+      <c r="K62" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L62" s="21">
         <f>IF(OR($B62="",$I62=""),"",$I62-IF($K62="",0,$K62))</f>
         <v/>
@@ -4420,17 +4568,39 @@
         <f>IF($B62="","",IF($H62="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O62" s="23" t="n"/>
+      <c r="O62" s="23" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
     </row>
     <row r="63">
-      <c r="A63" s="23" t="n"/>
-      <c r="B63" s="23" t="n"/>
-      <c r="C63" s="23" t="n"/>
-      <c r="D63" s="24" t="n"/>
-      <c r="E63" s="25" t="n"/>
-      <c r="F63" s="26" t="n"/>
-      <c r="G63" s="24" t="n"/>
-      <c r="H63" s="25" t="n"/>
+      <c r="A63" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126102780609+321261027586709+221261027605009+221261027605509+321261027587309+321261027587809+221261027606909+321261027588809+34126102782809+321261027590109+23126102782309+23126102782609</t>
+        </is>
+      </c>
+      <c r="B63" s="23" t="inlineStr">
+        <is>
+          <t>PARACABLES</t>
+        </is>
+      </c>
+      <c r="C63" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D63" s="24" t="n">
+        <v>46322</v>
+      </c>
+      <c r="E63" s="25" t="n">
+        <v>65.38590000000001</v>
+      </c>
+      <c r="F63" s="26" t="n">
+        <v>2614</v>
+      </c>
+      <c r="G63" s="24" t="inlineStr"/>
+      <c r="H63" s="25" t="inlineStr"/>
       <c r="I63" s="21">
         <f>IF(OR($B63="",$H63=""),"",IF($C63="LONG",($H63-$E63)*$F63,($E63-$H63)*$F63))</f>
         <v/>
@@ -4439,7 +4609,9 @@
         <f>IF(OR($B63="",$I63="",$E63=0,$F63=0),"",$I63/($E63*$F63))</f>
         <v/>
       </c>
-      <c r="K63" s="4" t="n"/>
+      <c r="K63" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L63" s="21">
         <f>IF(OR($B63="",$I63=""),"",$I63-IF($K63="",0,$K63))</f>
         <v/>
@@ -4452,17 +4624,39 @@
         <f>IF($B63="","",IF($H63="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O63" s="23" t="n"/>
+      <c r="O63" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="64">
-      <c r="A64" s="23" t="n"/>
-      <c r="B64" s="23" t="n"/>
-      <c r="C64" s="23" t="n"/>
-      <c r="D64" s="24" t="n"/>
-      <c r="E64" s="25" t="n"/>
-      <c r="F64" s="26" t="n"/>
-      <c r="G64" s="24" t="n"/>
-      <c r="H64" s="25" t="n"/>
+      <c r="A64" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261027604009+34126102781209+321261027587009+221261027605609+23126102781409+321261027587709+34126102782009+34126102782509+23126102782109+321261027590309+34126102783309+321261027591009+321261027591709</t>
+        </is>
+      </c>
+      <c r="B64" s="23" t="inlineStr">
+        <is>
+          <t>ZAGGLE</t>
+        </is>
+      </c>
+      <c r="C64" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D64" s="24" t="n">
+        <v>46322</v>
+      </c>
+      <c r="E64" s="25" t="n">
+        <v>164.4613</v>
+      </c>
+      <c r="F64" s="26" t="n">
+        <v>1041</v>
+      </c>
+      <c r="G64" s="24" t="inlineStr"/>
+      <c r="H64" s="25" t="inlineStr"/>
       <c r="I64" s="21">
         <f>IF(OR($B64="",$H64=""),"",IF($C64="LONG",($H64-$E64)*$F64,($E64-$H64)*$F64))</f>
         <v/>
@@ -4471,7 +4665,9 @@
         <f>IF(OR($B64="",$I64="",$E64=0,$F64=0),"",$I64/($E64*$F64))</f>
         <v/>
       </c>
-      <c r="K64" s="4" t="n"/>
+      <c r="K64" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L64" s="21">
         <f>IF(OR($B64="",$I64=""),"",$I64-IF($K64="",0,$K64))</f>
         <v/>
@@ -4484,7 +4680,11 @@
         <f>IF($B64="","",IF($H64="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O64" s="23" t="n"/>
+      <c r="O64" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="23" t="n"/>
@@ -31209,7 +31409,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J48"/>
+  <dimension ref="A1:J54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31293,7 +31493,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>ARFIN</t>
+          <t>AGIIL</t>
         </is>
       </c>
       <c r="B4" s="20">
@@ -31336,7 +31536,7 @@
     <row r="5">
       <c r="A5" s="27" t="inlineStr">
         <is>
-          <t>BLUSPRING</t>
+          <t>ARFIN</t>
         </is>
       </c>
       <c r="B5" s="20">
@@ -31379,7 +31579,7 @@
     <row r="6">
       <c r="A6" s="27" t="inlineStr">
         <is>
-          <t>CMLL</t>
+          <t>BAJEL</t>
         </is>
       </c>
       <c r="B6" s="20">
@@ -31422,7 +31622,7 @@
     <row r="7">
       <c r="A7" s="27" t="inlineStr">
         <is>
-          <t>DELTACORP</t>
+          <t>BBL</t>
         </is>
       </c>
       <c r="B7" s="20">
@@ -31465,7 +31665,7 @@
     <row r="8">
       <c r="A8" s="27" t="inlineStr">
         <is>
-          <t>DPABHUSHAN</t>
+          <t>BLUSPRING</t>
         </is>
       </c>
       <c r="B8" s="20">
@@ -31508,7 +31708,7 @@
     <row r="9">
       <c r="A9" s="27" t="inlineStr">
         <is>
-          <t>EUROPRATIK</t>
+          <t>CMLL</t>
         </is>
       </c>
       <c r="B9" s="20">
@@ -31551,7 +31751,7 @@
     <row r="10">
       <c r="A10" s="27" t="inlineStr">
         <is>
-          <t>FISCHER</t>
+          <t>DELTACORP</t>
         </is>
       </c>
       <c r="B10" s="20">
@@ -31594,7 +31794,7 @@
     <row r="11">
       <c r="A11" s="27" t="inlineStr">
         <is>
-          <t>GOODLUCK</t>
+          <t>DPABHUSHAN</t>
         </is>
       </c>
       <c r="B11" s="20">
@@ -31637,7 +31837,7 @@
     <row r="12">
       <c r="A12" s="27" t="inlineStr">
         <is>
-          <t>GPTINFRA</t>
+          <t>EUROPRATIK</t>
         </is>
       </c>
       <c r="B12" s="20">
@@ -31680,7 +31880,7 @@
     <row r="13">
       <c r="A13" s="27" t="inlineStr">
         <is>
-          <t>HATHWAY</t>
+          <t>FISCHER</t>
         </is>
       </c>
       <c r="B13" s="20">
@@ -31723,7 +31923,7 @@
     <row r="14">
       <c r="A14" s="27" t="inlineStr">
         <is>
-          <t>INDIAGLYCO</t>
+          <t>GOODLUCK</t>
         </is>
       </c>
       <c r="B14" s="20">
@@ -31766,7 +31966,7 @@
     <row r="15">
       <c r="A15" s="27" t="inlineStr">
         <is>
-          <t>INDOKEM</t>
+          <t>GPTINFRA</t>
         </is>
       </c>
       <c r="B15" s="20">
@@ -31809,7 +32009,7 @@
     <row r="16">
       <c r="A16" s="27" t="inlineStr">
         <is>
-          <t>INDOSTAR</t>
+          <t>HATHWAY</t>
         </is>
       </c>
       <c r="B16" s="20">
@@ -31852,7 +32052,7 @@
     <row r="17">
       <c r="A17" s="27" t="inlineStr">
         <is>
-          <t>INOXGREEN</t>
+          <t>INDIAGLYCO</t>
         </is>
       </c>
       <c r="B17" s="20">
@@ -31895,7 +32095,7 @@
     <row r="18">
       <c r="A18" s="27" t="inlineStr">
         <is>
-          <t>JAICORPLTD</t>
+          <t>INDOKEM</t>
         </is>
       </c>
       <c r="B18" s="20">
@@ -31938,7 +32138,7 @@
     <row r="19">
       <c r="A19" s="27" t="inlineStr">
         <is>
-          <t>JINDALPOLY</t>
+          <t>INDOSTAR</t>
         </is>
       </c>
       <c r="B19" s="20">
@@ -31981,7 +32181,7 @@
     <row r="20">
       <c r="A20" s="27" t="inlineStr">
         <is>
-          <t>KOTIC</t>
+          <t>INOXGREEN</t>
         </is>
       </c>
       <c r="B20" s="20">
@@ -32024,7 +32224,7 @@
     <row r="21">
       <c r="A21" s="27" t="inlineStr">
         <is>
-          <t>KRISHNADEF</t>
+          <t>JAICORPLTD</t>
         </is>
       </c>
       <c r="B21" s="20">
@@ -32067,7 +32267,7 @@
     <row r="22">
       <c r="A22" s="27" t="inlineStr">
         <is>
-          <t>KROSS</t>
+          <t>JINDALPOLY</t>
         </is>
       </c>
       <c r="B22" s="20">
@@ -32110,7 +32310,7 @@
     <row r="23">
       <c r="A23" s="27" t="inlineStr">
         <is>
-          <t>MBEL</t>
+          <t>JISLJALEQS</t>
         </is>
       </c>
       <c r="B23" s="20">
@@ -32153,7 +32353,7 @@
     <row r="24">
       <c r="A24" s="27" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>KOTIC</t>
         </is>
       </c>
       <c r="B24" s="20">
@@ -32196,7 +32396,7 @@
     <row r="25">
       <c r="A25" s="27" t="inlineStr">
         <is>
-          <t>MOBIKWIK</t>
+          <t>KRISHNADEF</t>
         </is>
       </c>
       <c r="B25" s="20">
@@ -32239,7 +32439,7 @@
     <row r="26">
       <c r="A26" s="27" t="inlineStr">
         <is>
-          <t>NIBE</t>
+          <t>KROSS</t>
         </is>
       </c>
       <c r="B26" s="20">
@@ -32282,7 +32482,7 @@
     <row r="27">
       <c r="A27" s="27" t="inlineStr">
         <is>
-          <t>OAL</t>
+          <t>MAHLOG</t>
         </is>
       </c>
       <c r="B27" s="20">
@@ -32325,7 +32525,7 @@
     <row r="28">
       <c r="A28" s="27" t="inlineStr">
         <is>
-          <t>ORIENTELEC</t>
+          <t>MBEL</t>
         </is>
       </c>
       <c r="B28" s="20">
@@ -32368,7 +32568,7 @@
     <row r="29">
       <c r="A29" s="27" t="inlineStr">
         <is>
-          <t>PARACABLES</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="B29" s="20">
@@ -32411,7 +32611,7 @@
     <row r="30">
       <c r="A30" s="27" t="inlineStr">
         <is>
-          <t>PIXTRANS</t>
+          <t>MOBIKWIK</t>
         </is>
       </c>
       <c r="B30" s="20">
@@ -32454,7 +32654,7 @@
     <row r="31">
       <c r="A31" s="27" t="inlineStr">
         <is>
-          <t>PNCINFRA</t>
+          <t>NIBE</t>
         </is>
       </c>
       <c r="B31" s="20">
@@ -32497,7 +32697,7 @@
     <row r="32">
       <c r="A32" s="27" t="inlineStr">
         <is>
-          <t>PNGSREVA</t>
+          <t>OAL</t>
         </is>
       </c>
       <c r="B32" s="20">
@@ -32540,7 +32740,7 @@
     <row r="33">
       <c r="A33" s="27" t="inlineStr">
         <is>
-          <t>PRINCEPIPE</t>
+          <t>ORIENTELEC</t>
         </is>
       </c>
       <c r="B33" s="20">
@@ -32583,7 +32783,7 @@
     <row r="34">
       <c r="A34" s="27" t="inlineStr">
         <is>
-          <t>RSYSTEMS</t>
+          <t>PARACABLES</t>
         </is>
       </c>
       <c r="B34" s="20">
@@ -32626,7 +32826,7 @@
     <row r="35">
       <c r="A35" s="27" t="inlineStr">
         <is>
-          <t>RUBYMILLS</t>
+          <t>PIXTRANS</t>
         </is>
       </c>
       <c r="B35" s="20">
@@ -32669,7 +32869,7 @@
     <row r="36">
       <c r="A36" s="27" t="inlineStr">
         <is>
-          <t>SAKSOFT</t>
+          <t>PNCINFRA</t>
         </is>
       </c>
       <c r="B36" s="20">
@@ -32712,7 +32912,7 @@
     <row r="37">
       <c r="A37" s="27" t="inlineStr">
         <is>
-          <t>SATIN</t>
+          <t>PNGSREVA</t>
         </is>
       </c>
       <c r="B37" s="20">
@@ -32755,7 +32955,7 @@
     <row r="38">
       <c r="A38" s="27" t="inlineStr">
         <is>
-          <t>SGFIN</t>
+          <t>PRINCEPIPE</t>
         </is>
       </c>
       <c r="B38" s="20">
@@ -32798,7 +32998,7 @@
     <row r="39">
       <c r="A39" s="27" t="inlineStr">
         <is>
-          <t>SHRINGARMS</t>
+          <t>RSYSTEMS</t>
         </is>
       </c>
       <c r="B39" s="20">
@@ -32841,7 +33041,7 @@
     <row r="40">
       <c r="A40" s="27" t="inlineStr">
         <is>
-          <t>SIMPLEXINF</t>
+          <t>RUBYMILLS</t>
         </is>
       </c>
       <c r="B40" s="20">
@@ -32884,7 +33084,7 @@
     <row r="41">
       <c r="A41" s="27" t="inlineStr">
         <is>
-          <t>SMCGLOBAL</t>
+          <t>SAKSOFT</t>
         </is>
       </c>
       <c r="B41" s="20">
@@ -32927,7 +33127,7 @@
     <row r="42">
       <c r="A42" s="27" t="inlineStr">
         <is>
-          <t>SOLARA</t>
+          <t>SATIN</t>
         </is>
       </c>
       <c r="B42" s="20">
@@ -32970,7 +33170,7 @@
     <row r="43">
       <c r="A43" s="27" t="inlineStr">
         <is>
-          <t>SPORTKING</t>
+          <t>SGFIN</t>
         </is>
       </c>
       <c r="B43" s="20">
@@ -33013,7 +33213,7 @@
     <row r="44">
       <c r="A44" s="27" t="inlineStr">
         <is>
-          <t>SUNCLAY</t>
+          <t>SHRINGARMS</t>
         </is>
       </c>
       <c r="B44" s="20">
@@ -33056,7 +33256,7 @@
     <row r="45">
       <c r="A45" s="27" t="inlineStr">
         <is>
-          <t>SWARAJENG</t>
+          <t>SIMPLEXINF</t>
         </is>
       </c>
       <c r="B45" s="20">
@@ -33099,7 +33299,7 @@
     <row r="46">
       <c r="A46" s="27" t="inlineStr">
         <is>
-          <t>TEAMLEASE</t>
+          <t>SMCGLOBAL</t>
         </is>
       </c>
       <c r="B46" s="20">
@@ -33142,7 +33342,7 @@
     <row r="47">
       <c r="A47" s="27" t="inlineStr">
         <is>
-          <t>YUKEN</t>
+          <t>SOLARA</t>
         </is>
       </c>
       <c r="B47" s="20">
@@ -33183,37 +33383,295 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="3" t="inlineStr">
+      <c r="A48" s="27" t="inlineStr">
+        <is>
+          <t>SPORTKING</t>
+        </is>
+      </c>
+      <c r="B48" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A48)</f>
+        <v/>
+      </c>
+      <c r="C48" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A48,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D48" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A48,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E48" s="22">
+        <f>IFERROR($C48/$B48,"")</f>
+        <v/>
+      </c>
+      <c r="F48" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A48,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G48" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A48,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H48" s="21">
+        <f>IFERROR($G48/$B48,"")</f>
+        <v/>
+      </c>
+      <c r="I48" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A48),"")</f>
+        <v/>
+      </c>
+      <c r="J48" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A48),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="27" t="inlineStr">
+        <is>
+          <t>SUNCLAY</t>
+        </is>
+      </c>
+      <c r="B49" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A49)</f>
+        <v/>
+      </c>
+      <c r="C49" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A49,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D49" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A49,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E49" s="22">
+        <f>IFERROR($C49/$B49,"")</f>
+        <v/>
+      </c>
+      <c r="F49" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A49,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G49" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A49,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H49" s="21">
+        <f>IFERROR($G49/$B49,"")</f>
+        <v/>
+      </c>
+      <c r="I49" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A49),"")</f>
+        <v/>
+      </c>
+      <c r="J49" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A49),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="27" t="inlineStr">
+        <is>
+          <t>SWARAJENG</t>
+        </is>
+      </c>
+      <c r="B50" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A50)</f>
+        <v/>
+      </c>
+      <c r="C50" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A50,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D50" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A50,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E50" s="22">
+        <f>IFERROR($C50/$B50,"")</f>
+        <v/>
+      </c>
+      <c r="F50" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A50,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G50" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A50,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H50" s="21">
+        <f>IFERROR($G50/$B50,"")</f>
+        <v/>
+      </c>
+      <c r="I50" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A50),"")</f>
+        <v/>
+      </c>
+      <c r="J50" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A50),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="27" t="inlineStr">
+        <is>
+          <t>TEAMLEASE</t>
+        </is>
+      </c>
+      <c r="B51" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A51)</f>
+        <v/>
+      </c>
+      <c r="C51" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A51,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D51" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A51,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E51" s="22">
+        <f>IFERROR($C51/$B51,"")</f>
+        <v/>
+      </c>
+      <c r="F51" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A51,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G51" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A51,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H51" s="21">
+        <f>IFERROR($G51/$B51,"")</f>
+        <v/>
+      </c>
+      <c r="I51" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A51),"")</f>
+        <v/>
+      </c>
+      <c r="J51" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A51),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="27" t="inlineStr">
+        <is>
+          <t>YUKEN</t>
+        </is>
+      </c>
+      <c r="B52" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A52)</f>
+        <v/>
+      </c>
+      <c r="C52" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A52,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D52" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A52,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E52" s="22">
+        <f>IFERROR($C52/$B52,"")</f>
+        <v/>
+      </c>
+      <c r="F52" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A52,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G52" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A52,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H52" s="21">
+        <f>IFERROR($G52/$B52,"")</f>
+        <v/>
+      </c>
+      <c r="I52" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A52),"")</f>
+        <v/>
+      </c>
+      <c r="J52" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A52),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="27" t="inlineStr">
+        <is>
+          <t>ZAGGLE</t>
+        </is>
+      </c>
+      <c r="B53" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A53)</f>
+        <v/>
+      </c>
+      <c r="C53" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A53,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D53" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A53,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E53" s="22">
+        <f>IFERROR($C53/$B53,"")</f>
+        <v/>
+      </c>
+      <c r="F53" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A53,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G53" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A53,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H53" s="21">
+        <f>IFERROR($G53/$B53,"")</f>
+        <v/>
+      </c>
+      <c r="I53" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A53),"")</f>
+        <v/>
+      </c>
+      <c r="J53" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A53),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B48" s="30">
-        <f>SUM(B4:B47)</f>
-        <v/>
-      </c>
-      <c r="C48" s="30">
-        <f>SUM(C4:C47)</f>
-        <v/>
-      </c>
-      <c r="D48" s="30">
-        <f>SUM(D4:D47)</f>
-        <v/>
-      </c>
-      <c r="E48" s="31">
-        <f>IFERROR(C48/B48,"")</f>
-        <v/>
-      </c>
-      <c r="F48" s="32">
-        <f>SUM(F4:F47)</f>
-        <v/>
-      </c>
-      <c r="G48" s="32">
-        <f>SUM(G4:G47)</f>
-        <v/>
-      </c>
-      <c r="H48" s="32">
-        <f>IFERROR(G48/B48,"")</f>
+      <c r="B54" s="30">
+        <f>SUM(B4:B53)</f>
+        <v/>
+      </c>
+      <c r="C54" s="30">
+        <f>SUM(C4:C53)</f>
+        <v/>
+      </c>
+      <c r="D54" s="30">
+        <f>SUM(D4:D53)</f>
+        <v/>
+      </c>
+      <c r="E54" s="31">
+        <f>IFERROR(C54/B54,"")</f>
+        <v/>
+      </c>
+      <c r="F54" s="32">
+        <f>SUM(F4:F53)</f>
+        <v/>
+      </c>
+      <c r="G54" s="32">
+        <f>SUM(G4:G53)</f>
+        <v/>
+      </c>
+      <c r="H54" s="32">
+        <f>IFERROR(G54/B54,"")</f>
         <v/>
       </c>
     </row>
@@ -33232,7 +33690,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N57"/>
+  <dimension ref="A1:N65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -33483,7 +33941,7 @@
         <v>35.4</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>115.99</v>
+        <v>115.98</v>
       </c>
       <c r="N6" s="21">
         <f>SUM(E6:M6)</f>
@@ -33585,7 +34043,7 @@
         <v>35.4</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>96.51000000000001</v>
+        <v>96.5</v>
       </c>
       <c r="N8" s="21">
         <f>SUM(E8:M8)</f>
@@ -33687,7 +34145,7 @@
         <v>35.4</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>96.52</v>
+        <v>96.51000000000001</v>
       </c>
       <c r="N10" s="21">
         <f>SUM(E10:M10)</f>
@@ -33840,7 +34298,7 @@
         <v>35.4</v>
       </c>
       <c r="M13" s="4" t="n">
-        <v>72.90000000000001</v>
+        <v>72.97</v>
       </c>
       <c r="N13" s="21">
         <f>SUM(E13:M13)</f>
@@ -34146,7 +34604,7 @@
         <v>35.4</v>
       </c>
       <c r="M19" s="4" t="n">
-        <v>86.48999999999999</v>
+        <v>86.56</v>
       </c>
       <c r="N19" s="21">
         <f>SUM(E19:M19)</f>
@@ -34452,7 +34910,7 @@
         <v>35.4</v>
       </c>
       <c r="M25" s="4" t="n">
-        <v>37.09</v>
+        <v>37.1</v>
       </c>
       <c r="N25" s="21">
         <f>SUM(E25:M25)</f>
@@ -34656,7 +35114,7 @@
         <v>35.4</v>
       </c>
       <c r="M29" s="4" t="n">
-        <v>42.59</v>
+        <v>42.6</v>
       </c>
       <c r="N29" s="21">
         <f>SUM(E29:M29)</f>
@@ -34911,7 +35369,7 @@
         <v>35.4</v>
       </c>
       <c r="M34" s="4" t="n">
-        <v>37.65</v>
+        <v>37.68</v>
       </c>
       <c r="N34" s="21">
         <f>SUM(E34:M34)</f>
@@ -35064,7 +35522,7 @@
         <v>35.4</v>
       </c>
       <c r="M37" s="4" t="n">
-        <v>31.6</v>
+        <v>31.42</v>
       </c>
       <c r="N37" s="21">
         <f>SUM(E37:M37)</f>
@@ -35268,7 +35726,7 @@
         <v>35.4</v>
       </c>
       <c r="M41" s="4" t="n">
-        <v>234.08</v>
+        <v>234.11</v>
       </c>
       <c r="N41" s="21">
         <f>SUM(E41:M41)</f>
@@ -35370,7 +35828,7 @@
         <v>35.4</v>
       </c>
       <c r="M43" s="4" t="n">
-        <v>80.42</v>
+        <v>80.45</v>
       </c>
       <c r="N43" s="21">
         <f>SUM(E43:M43)</f>
@@ -35472,7 +35930,7 @@
         <v>35.4</v>
       </c>
       <c r="M45" s="4" t="n">
-        <v>85.64</v>
+        <v>85.7</v>
       </c>
       <c r="N45" s="21">
         <f>SUM(E45:M45)</f>
@@ -35574,7 +36032,7 @@
         <v>35.4</v>
       </c>
       <c r="M47" s="4" t="n">
-        <v>178.81</v>
+        <v>178.83</v>
       </c>
       <c r="N47" s="21">
         <f>SUM(E47:M47)</f>
@@ -35625,7 +36083,7 @@
         <v>35.4</v>
       </c>
       <c r="M48" s="4" t="n">
-        <v>179.77</v>
+        <v>179.79</v>
       </c>
       <c r="N48" s="21">
         <f>SUM(E48:M48)</f>
@@ -35676,7 +36134,7 @@
         <v>35.4</v>
       </c>
       <c r="M49" s="4" t="n">
-        <v>175.22</v>
+        <v>175.26</v>
       </c>
       <c r="N49" s="21">
         <f>SUM(E49:M49)</f>
@@ -35727,7 +36185,7 @@
         <v>35.4</v>
       </c>
       <c r="M50" s="4" t="n">
-        <v>180.13</v>
+        <v>180.15</v>
       </c>
       <c r="N50" s="21">
         <f>SUM(E50:M50)</f>
@@ -35778,7 +36236,7 @@
         <v>35.4</v>
       </c>
       <c r="M51" s="4" t="n">
-        <v>142.42</v>
+        <v>142.48</v>
       </c>
       <c r="N51" s="21">
         <f>SUM(E51:M51)</f>
@@ -35829,7 +36287,7 @@
         <v>35.4</v>
       </c>
       <c r="M52" s="4" t="n">
-        <v>111.97</v>
+        <v>111.98</v>
       </c>
       <c r="N52" s="21">
         <f>SUM(E52:M52)</f>
@@ -35907,22 +36365,22 @@
         <v>46321</v>
       </c>
       <c r="E54" s="4" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F54" s="4" t="n">
         <v>150.05</v>
       </c>
       <c r="G54" s="4" t="n">
-        <v>4.61</v>
+        <v>9.359999999999999</v>
       </c>
       <c r="H54" s="4" t="n">
-        <v>0.15</v>
+        <v>0.31</v>
       </c>
       <c r="I54" s="4" t="n">
         <v>22.51</v>
       </c>
       <c r="J54" s="4" t="n">
-        <v>0.86</v>
+        <v>5.34</v>
       </c>
       <c r="K54" s="4" t="n">
         <v>14.75</v>
@@ -35941,48 +36399,48 @@
     <row r="55">
       <c r="A55" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261023807609+321261023756809+231261023120609+221261023808709+221261023809309+231261023120909+221261023809609+231261023121109+341261023126209+341261023126309+341261023126509+341261023126609+321261023760409</t>
+          <t>DHAN-23126102637609</t>
         </is>
       </c>
       <c r="B55" s="23" t="inlineStr">
         <is>
-          <t>JINDALPOLY</t>
+          <t>FISCHER</t>
         </is>
       </c>
       <c r="C55" s="23" t="inlineStr">
         <is>
-          <t>LONG</t>
+          <t>SHORT</t>
         </is>
       </c>
       <c r="D55" s="24" t="n">
         <v>46321</v>
       </c>
       <c r="E55" s="4" t="n">
-        <v>89.3</v>
+        <v>0</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>297.95</v>
+        <v>156.18</v>
       </c>
       <c r="G55" s="4" t="n">
-        <v>9.140000000000001</v>
+        <v>4.75</v>
       </c>
       <c r="H55" s="4" t="n">
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="I55" s="4" t="n">
-        <v>44.49</v>
+        <v>0</v>
       </c>
       <c r="J55" s="4" t="n">
-        <v>17.77</v>
+        <v>0.88</v>
       </c>
       <c r="K55" s="4" t="n">
-        <v>14.75</v>
+        <v>0</v>
       </c>
       <c r="L55" s="4" t="n">
-        <v>35.4</v>
+        <v>0</v>
       </c>
       <c r="M55" s="4" t="n">
-        <v>46.37</v>
+        <v>0</v>
       </c>
       <c r="N55" s="21">
         <f>SUM(E55:M55)</f>
@@ -35992,12 +36450,12 @@
     <row r="56">
       <c r="A56" s="23" t="inlineStr">
         <is>
-          <t>DHAN-23126102699709+221261026669809+321261026636409+321261026636909+23126102699809+34126102699309+221261026670609+221261026671109+231261026100009+231261026100109+34126102699609+34126102699709</t>
+          <t>DHAN-221261023807609+321261023756809+231261023120609+221261023808709+221261023809309+231261023120909+221261023809609+231261023121109+341261023126209+341261023126309+341261023126509+341261023126609+321261023760409</t>
         </is>
       </c>
       <c r="B56" s="23" t="inlineStr">
         <is>
-          <t>INDOSTAR</t>
+          <t>JINDALPOLY</t>
         </is>
       </c>
       <c r="C56" s="23" t="inlineStr">
@@ -36005,24 +36463,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D56" s="24" t="inlineStr"/>
+      <c r="D56" s="24" t="n">
+        <v>46321</v>
+      </c>
       <c r="E56" s="4" t="n">
-        <v>0</v>
+        <v>109.3</v>
       </c>
       <c r="F56" s="4" t="n">
-        <v>0</v>
+        <v>583.65</v>
       </c>
       <c r="G56" s="4" t="n">
-        <v>0</v>
+        <v>17.91</v>
       </c>
       <c r="H56" s="4" t="n">
-        <v>0</v>
+        <v>0.58</v>
       </c>
       <c r="I56" s="4" t="n">
-        <v>0</v>
+        <v>44.49</v>
       </c>
       <c r="J56" s="4" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="K56" s="4" t="n">
         <v>14.75</v>
@@ -36031,7 +36491,7 @@
         <v>35.4</v>
       </c>
       <c r="M56" s="4" t="n">
-        <v>0</v>
+        <v>46.11</v>
       </c>
       <c r="N56" s="21">
         <f>SUM(E56:M56)</f>
@@ -36039,54 +36499,448 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="3" t="inlineStr">
+      <c r="A57" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126102699709+221261026669809+321261026636409+321261026636909+23126102699809+34126102699309+221261026670609+221261026671109+231261026100009+231261026100109+34126102699609+34126102699709</t>
+        </is>
+      </c>
+      <c r="B57" s="23" t="inlineStr">
+        <is>
+          <t>INDOSTAR</t>
+        </is>
+      </c>
+      <c r="C57" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D57" s="24" t="n">
+        <v>46322</v>
+      </c>
+      <c r="E57" s="4" t="n">
+        <v>90.05</v>
+      </c>
+      <c r="F57" s="4" t="n">
+        <v>300.07</v>
+      </c>
+      <c r="G57" s="4" t="n">
+        <v>9.210000000000001</v>
+      </c>
+      <c r="H57" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="I57" s="4" t="n">
+        <v>45.22</v>
+      </c>
+      <c r="J57" s="4" t="n">
+        <v>17.92</v>
+      </c>
+      <c r="K57" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L57" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M57" s="4" t="n">
+        <v>61.57</v>
+      </c>
+      <c r="N57" s="21">
+        <f>SUM(E57:M57)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126102781109+34126102781509+23126102780909+34126102781709+321261027587409+23126102781709+321261027588509+221261027607309+23126102782009+34126102783009+23126102782409+221261027608709+23126102782709+321261027592209</t>
+        </is>
+      </c>
+      <c r="B58" s="23" t="inlineStr">
+        <is>
+          <t>AGIIL</t>
+        </is>
+      </c>
+      <c r="C58" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D58" s="24" t="inlineStr"/>
+      <c r="E58" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F58" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I58" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J58" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K58" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L58" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M58" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N58" s="21">
+        <f>SUM(E58:M58)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126102780509+34126102781309+23126102781009+23126102781209+221261027605909+34126102781909+321261027588609+23126102781809+321261027589309+23126102782209+321261027590909+23126102782809+34126102783609</t>
+        </is>
+      </c>
+      <c r="B59" s="23" t="inlineStr">
+        <is>
+          <t>BAJEL</t>
+        </is>
+      </c>
+      <c r="C59" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D59" s="24" t="inlineStr"/>
+      <c r="E59" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I59" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J59" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K59" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L59" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M59" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N59" s="21">
+        <f>SUM(E59:M59)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261027603909+23126102780809+34126102781609+221261027605309+34126102781809+221261027606409+34126102782209+34126102782709+221261027607909+34126102782909+34126102783209+34126102783409+321261027591809+23126102783009</t>
+        </is>
+      </c>
+      <c r="B60" s="23" t="inlineStr">
+        <is>
+          <t>BBL</t>
+        </is>
+      </c>
+      <c r="C60" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D60" s="24" t="inlineStr"/>
+      <c r="E60" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F60" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G60" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I60" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J60" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K60" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L60" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M60" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N60" s="21">
+        <f>SUM(E60:M60)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261027586409+221261027604309+221261027604909+221261027605409+221261027606009+221261027606309+221261027606809+23126102781909+321261027589409+321261027590009+221261027608409</t>
+        </is>
+      </c>
+      <c r="B61" s="23" t="inlineStr">
+        <is>
+          <t>JISLJALEQS</t>
+        </is>
+      </c>
+      <c r="C61" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D61" s="24" t="inlineStr"/>
+      <c r="E61" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F61" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G61" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I61" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J61" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K61" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L61" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M61" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N61" s="21">
+        <f>SUM(E61:M61)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261027603809+34126102781409+221261027604809+321261027587109+23126102781309+23126102781609+34126102782109+34126102782609+321261027589509+321261027590209+34126102783109+23126102782509</t>
+        </is>
+      </c>
+      <c r="B62" s="23" t="inlineStr">
+        <is>
+          <t>MAHLOG</t>
+        </is>
+      </c>
+      <c r="C62" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D62" s="24" t="inlineStr"/>
+      <c r="E62" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F62" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G62" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H62" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I62" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J62" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K62" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L62" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M62" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N62" s="21">
+        <f>SUM(E62:M62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126102780609+321261027586709+221261027605009+221261027605509+321261027587309+321261027587809+221261027606909+321261027588809+34126102782809+321261027590109+23126102782309+23126102782609</t>
+        </is>
+      </c>
+      <c r="B63" s="23" t="inlineStr">
+        <is>
+          <t>PARACABLES</t>
+        </is>
+      </c>
+      <c r="C63" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D63" s="24" t="inlineStr"/>
+      <c r="E63" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F63" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H63" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I63" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J63" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K63" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L63" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M63" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N63" s="21">
+        <f>SUM(E63:M63)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261027604009+34126102781209+321261027587009+221261027605609+23126102781409+321261027587709+34126102782009+34126102782509+23126102782109+321261027590309+34126102783309+321261027591009+321261027591709</t>
+        </is>
+      </c>
+      <c r="B64" s="23" t="inlineStr">
+        <is>
+          <t>ZAGGLE</t>
+        </is>
+      </c>
+      <c r="C64" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D64" s="24" t="inlineStr"/>
+      <c r="E64" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F64" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G64" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H64" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I64" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J64" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K64" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L64" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M64" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N64" s="21">
+        <f>SUM(E64:M64)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E57" s="32">
-        <f>SUM(E4:E56)</f>
-        <v/>
-      </c>
-      <c r="F57" s="32">
-        <f>SUM(F4:F56)</f>
-        <v/>
-      </c>
-      <c r="G57" s="32">
-        <f>SUM(G4:G56)</f>
-        <v/>
-      </c>
-      <c r="H57" s="32">
-        <f>SUM(H4:H56)</f>
-        <v/>
-      </c>
-      <c r="I57" s="32">
-        <f>SUM(I4:I56)</f>
-        <v/>
-      </c>
-      <c r="J57" s="32">
-        <f>SUM(J4:J56)</f>
-        <v/>
-      </c>
-      <c r="K57" s="32">
-        <f>SUM(K4:K56)</f>
-        <v/>
-      </c>
-      <c r="L57" s="32">
-        <f>SUM(L4:L56)</f>
-        <v/>
-      </c>
-      <c r="M57" s="32">
-        <f>SUM(M4:M56)</f>
-        <v/>
-      </c>
-      <c r="N57" s="32">
-        <f>SUM(N4:N56)</f>
+      <c r="E65" s="32">
+        <f>SUM(E4:E64)</f>
+        <v/>
+      </c>
+      <c r="F65" s="32">
+        <f>SUM(F4:F64)</f>
+        <v/>
+      </c>
+      <c r="G65" s="32">
+        <f>SUM(G4:G64)</f>
+        <v/>
+      </c>
+      <c r="H65" s="32">
+        <f>SUM(H4:H64)</f>
+        <v/>
+      </c>
+      <c r="I65" s="32">
+        <f>SUM(I4:I64)</f>
+        <v/>
+      </c>
+      <c r="J65" s="32">
+        <f>SUM(J4:J64)</f>
+        <v/>
+      </c>
+      <c r="K65" s="32">
+        <f>SUM(K4:K64)</f>
+        <v/>
+      </c>
+      <c r="L65" s="32">
+        <f>SUM(L4:L64)</f>
+        <v/>
+      </c>
+      <c r="M65" s="32">
+        <f>SUM(M4:M64)</f>
+        <v/>
+      </c>
+      <c r="N65" s="32">
+        <f>SUM(N4:N64)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:N56"/>
+  <autoFilter ref="A3:N64"/>
   <mergeCells count="2">
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>

</xml_diff>

<commit_message>
Data update — 2026-10-28 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_oct2026.xlsx
+++ b/results/strategy_pnl_oct2026.xlsx
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trade Log'!$A$3:$O$503</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$66</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1214,7 +1214,7 @@
         <v/>
       </c>
       <c r="K6" s="4" t="n">
-        <v>955.01</v>
+        <v>955</v>
       </c>
       <c r="L6" s="21">
         <f>IF(OR($B6="",$I6=""),"",$I6-IF($K6="",0,$K6))</f>
@@ -1394,7 +1394,7 @@
         <v/>
       </c>
       <c r="K9" s="4" t="n">
-        <v>969.47</v>
+        <v>969.46</v>
       </c>
       <c r="L9" s="21">
         <f>IF(OR($B9="",$I9=""),"",$I9-IF($K9="",0,$K9))</f>
@@ -1514,7 +1514,7 @@
         <v/>
       </c>
       <c r="K11" s="4" t="n">
-        <v>691.26</v>
+        <v>691.25</v>
       </c>
       <c r="L11" s="21">
         <f>IF(OR($B11="",$I11=""),"",$I11-IF($K11="",0,$K11))</f>
@@ -1634,7 +1634,7 @@
         <v/>
       </c>
       <c r="K13" s="4" t="n">
-        <v>687.9299999999999</v>
+        <v>687.97</v>
       </c>
       <c r="L13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($K13="",0,$K13))</f>
@@ -1874,7 +1874,7 @@
         <v/>
       </c>
       <c r="K17" s="4" t="n">
-        <v>660.95</v>
+        <v>660.9299999999999</v>
       </c>
       <c r="L17" s="21">
         <f>IF(OR($B17="",$I17=""),"",$I17-IF($K17="",0,$K17))</f>
@@ -1994,7 +1994,7 @@
         <v/>
       </c>
       <c r="K19" s="4" t="n">
-        <v>666.74</v>
+        <v>666.78</v>
       </c>
       <c r="L19" s="21">
         <f>IF(OR($B19="",$I19=""),"",$I19-IF($K19="",0,$K19))</f>
@@ -2054,7 +2054,7 @@
         <v/>
       </c>
       <c r="K20" s="4" t="n">
-        <v>676.87</v>
+        <v>676.85</v>
       </c>
       <c r="L20" s="21">
         <f>IF(OR($B20="",$I20=""),"",$I20-IF($K20="",0,$K20))</f>
@@ -2174,7 +2174,7 @@
         <v/>
       </c>
       <c r="K22" s="4" t="n">
-        <v>658.46</v>
+        <v>658.45</v>
       </c>
       <c r="L22" s="21">
         <f>IF(OR($B22="",$I22=""),"",$I22-IF($K22="",0,$K22))</f>
@@ -2354,7 +2354,7 @@
         <v/>
       </c>
       <c r="K25" s="4" t="n">
-        <v>557.3</v>
+        <v>557.26</v>
       </c>
       <c r="L25" s="21">
         <f>IF(OR($B25="",$I25=""),"",$I25-IF($K25="",0,$K25))</f>
@@ -2474,7 +2474,7 @@
         <v/>
       </c>
       <c r="K27" s="4" t="n">
-        <v>547.58</v>
+        <v>547.5700000000001</v>
       </c>
       <c r="L27" s="21">
         <f>IF(OR($B27="",$I27=""),"",$I27-IF($K27="",0,$K27))</f>
@@ -2534,7 +2534,7 @@
         <v/>
       </c>
       <c r="K28" s="4" t="n">
-        <v>547.84</v>
+        <v>547.83</v>
       </c>
       <c r="L28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($K28="",0,$K28))</f>
@@ -2594,7 +2594,7 @@
         <v/>
       </c>
       <c r="K29" s="4" t="n">
-        <v>554.6</v>
+        <v>554.61</v>
       </c>
       <c r="L29" s="21">
         <f>IF(OR($B29="",$I29=""),"",$I29-IF($K29="",0,$K29))</f>
@@ -2654,7 +2654,7 @@
         <v/>
       </c>
       <c r="K30" s="4" t="n">
-        <v>550.7</v>
+        <v>550.6900000000001</v>
       </c>
       <c r="L30" s="21">
         <f>IF(OR($B30="",$I30=""),"",$I30-IF($K30="",0,$K30))</f>
@@ -2894,7 +2894,7 @@
         <v/>
       </c>
       <c r="K34" s="4" t="n">
-        <v>425.99</v>
+        <v>426.01</v>
       </c>
       <c r="L34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($K34="",0,$K34))</f>
@@ -3014,7 +3014,7 @@
         <v/>
       </c>
       <c r="K36" s="4" t="n">
-        <v>553.04</v>
+        <v>553.03</v>
       </c>
       <c r="L36" s="21">
         <f>IF(OR($B36="",$I36=""),"",$I36-IF($K36="",0,$K36))</f>
@@ -3074,7 +3074,7 @@
         <v/>
       </c>
       <c r="K37" s="4" t="n">
-        <v>477.87</v>
+        <v>477.89</v>
       </c>
       <c r="L37" s="21">
         <f>IF(OR($B37="",$I37=""),"",$I37-IF($K37="",0,$K37))</f>
@@ -3314,7 +3314,7 @@
         <v/>
       </c>
       <c r="K41" s="4" t="n">
-        <v>592.28</v>
+        <v>592.42</v>
       </c>
       <c r="L41" s="21">
         <f>IF(OR($B41="",$I41=""),"",$I41-IF($K41="",0,$K41))</f>
@@ -3434,7 +3434,7 @@
         <v/>
       </c>
       <c r="K43" s="4" t="n">
-        <v>924.55</v>
+        <v>924.64</v>
       </c>
       <c r="L43" s="21">
         <f>IF(OR($B43="",$I43=""),"",$I43-IF($K43="",0,$K43))</f>
@@ -3554,7 +3554,7 @@
         <v/>
       </c>
       <c r="K45" s="4" t="n">
-        <v>945.87</v>
+        <v>945.9299999999999</v>
       </c>
       <c r="L45" s="21">
         <f>IF(OR($B45="",$I45=""),"",$I45-IF($K45="",0,$K45))</f>
@@ -3614,7 +3614,7 @@
         <v/>
       </c>
       <c r="K46" s="4" t="n">
-        <v>915.87</v>
+        <v>915.9</v>
       </c>
       <c r="L46" s="21">
         <f>IF(OR($B46="",$I46=""),"",$I46-IF($K46="",0,$K46))</f>
@@ -3674,7 +3674,7 @@
         <v/>
       </c>
       <c r="K47" s="4" t="n">
-        <v>1026.87</v>
+        <v>1027</v>
       </c>
       <c r="L47" s="21">
         <f>IF(OR($B47="",$I47=""),"",$I47-IF($K47="",0,$K47))</f>
@@ -3734,7 +3734,7 @@
         <v/>
       </c>
       <c r="K48" s="4" t="n">
-        <v>1028.56</v>
+        <v>1028.69</v>
       </c>
       <c r="L48" s="21">
         <f>IF(OR($B48="",$I48=""),"",$I48-IF($K48="",0,$K48))</f>
@@ -3794,7 +3794,7 @@
         <v/>
       </c>
       <c r="K49" s="4" t="n">
-        <v>955.1</v>
+        <v>954.05</v>
       </c>
       <c r="L49" s="21">
         <f>IF(OR($B49="",$I49=""),"",$I49-IF($K49="",0,$K49))</f>
@@ -3854,7 +3854,7 @@
         <v/>
       </c>
       <c r="K50" s="4" t="n">
-        <v>1035.26</v>
+        <v>1035.39</v>
       </c>
       <c r="L50" s="21">
         <f>IF(OR($B50="",$I50=""),"",$I50-IF($K50="",0,$K50))</f>
@@ -3914,7 +3914,7 @@
         <v/>
       </c>
       <c r="K51" s="4" t="n">
-        <v>984.54</v>
+        <v>984.75</v>
       </c>
       <c r="L51" s="21">
         <f>IF(OR($B51="",$I51=""),"",$I51-IF($K51="",0,$K51))</f>
@@ -3974,7 +3974,7 @@
         <v/>
       </c>
       <c r="K52" s="4" t="n">
-        <v>939.9400000000001</v>
+        <v>940.02</v>
       </c>
       <c r="L52" s="21">
         <f>IF(OR($B52="",$I52=""),"",$I52-IF($K52="",0,$K52))</f>
@@ -4214,7 +4214,7 @@
         <v/>
       </c>
       <c r="K56" s="4" t="n">
-        <v>875.1900000000001</v>
+        <v>875.26</v>
       </c>
       <c r="L56" s="21">
         <f>IF(OR($B56="",$I56=""),"",$I56-IF($K56="",0,$K56))</f>
@@ -4274,7 +4274,7 @@
         <v/>
       </c>
       <c r="K57" s="4" t="n">
-        <v>574.5</v>
+        <v>933.5</v>
       </c>
       <c r="L57" s="21">
         <f>IF(OR($B57="",$I57=""),"",$I57-IF($K57="",0,$K57))</f>
@@ -4319,8 +4319,12 @@
       <c r="F58" s="26" t="n">
         <v>737</v>
       </c>
-      <c r="G58" s="24" t="inlineStr"/>
-      <c r="H58" s="25" t="inlineStr"/>
+      <c r="G58" s="24" t="n">
+        <v>46323</v>
+      </c>
+      <c r="H58" s="25" t="n">
+        <v>222.59</v>
+      </c>
       <c r="I58" s="21">
         <f>IF(OR($B58="",$H58=""),"",IF($C58="LONG",($H58-$E58)*$F58,($E58-$H58)*$F58))</f>
         <v/>
@@ -4330,7 +4334,7 @@
         <v/>
       </c>
       <c r="K58" s="4" t="n">
-        <v>50.15</v>
+        <v>351.43</v>
       </c>
       <c r="L58" s="21">
         <f>IF(OR($B58="",$I58=""),"",$I58-IF($K58="",0,$K58))</f>
@@ -4353,12 +4357,12 @@
     <row r="59">
       <c r="A59" s="23" t="inlineStr">
         <is>
-          <t>DHAN-23126102780509+34126102781309+23126102781009+23126102781209+221261027605909+34126102781909+321261027588609+23126102781809+321261027589309+23126102782209+321261027590909+23126102782809+34126102783609</t>
+          <t>DHAN-221261027603909+23126102780809+34126102781609+221261027605309+34126102781809+221261027606409+34126102782209+34126102782709+221261027607909+34126102782909+34126102783209+34126102783409+321261027591809+23126102783009</t>
         </is>
       </c>
       <c r="B59" s="23" t="inlineStr">
         <is>
-          <t>BAJEL</t>
+          <t>BBL</t>
         </is>
       </c>
       <c r="C59" s="23" t="inlineStr">
@@ -4370,13 +4374,17 @@
         <v>46322</v>
       </c>
       <c r="E59" s="25" t="n">
-        <v>168.7027</v>
+        <v>2588.2151</v>
       </c>
       <c r="F59" s="26" t="n">
-        <v>507</v>
-      </c>
-      <c r="G59" s="24" t="inlineStr"/>
-      <c r="H59" s="25" t="inlineStr"/>
+        <v>66</v>
+      </c>
+      <c r="G59" s="24" t="n">
+        <v>46323</v>
+      </c>
+      <c r="H59" s="25" t="n">
+        <v>2586.23</v>
+      </c>
       <c r="I59" s="21">
         <f>IF(OR($B59="",$H59=""),"",IF($C59="LONG",($H59-$E59)*$F59,($E59-$H59)*$F59))</f>
         <v/>
@@ -4386,7 +4394,7 @@
         <v/>
       </c>
       <c r="K59" s="4" t="n">
-        <v>14.75</v>
+        <v>351.37</v>
       </c>
       <c r="L59" s="21">
         <f>IF(OR($B59="",$I59=""),"",$I59-IF($K59="",0,$K59))</f>
@@ -4402,19 +4410,19 @@
       </c>
       <c r="O59" s="23" t="inlineStr">
         <is>
-          <t>5-10</t>
+          <t>10-15</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261027603909+23126102780809+34126102781609+221261027605309+34126102781809+221261027606409+34126102782209+34126102782709+221261027607909+34126102782909+34126102783209+34126102783409+321261027591809+23126102783009</t>
+          <t>DHAN-321261027586409+221261027604309+221261027604909+221261027605409+221261027606009+221261027606309+221261027606809+23126102781909+321261027589409+321261027590009+221261027608409</t>
         </is>
       </c>
       <c r="B60" s="23" t="inlineStr">
         <is>
-          <t>BBL</t>
+          <t>JISLJALEQS</t>
         </is>
       </c>
       <c r="C60" s="23" t="inlineStr">
@@ -4426,13 +4434,17 @@
         <v>46322</v>
       </c>
       <c r="E60" s="25" t="n">
-        <v>2588.2151</v>
+        <v>24.9779</v>
       </c>
       <c r="F60" s="26" t="n">
-        <v>66</v>
-      </c>
-      <c r="G60" s="24" t="inlineStr"/>
-      <c r="H60" s="25" t="inlineStr"/>
+        <v>6857</v>
+      </c>
+      <c r="G60" s="24" t="n">
+        <v>46323</v>
+      </c>
+      <c r="H60" s="25" t="n">
+        <v>24.5</v>
+      </c>
       <c r="I60" s="21">
         <f>IF(OR($B60="",$H60=""),"",IF($C60="LONG",($H60-$E60)*$F60,($E60-$H60)*$F60))</f>
         <v/>
@@ -4442,7 +4454,7 @@
         <v/>
       </c>
       <c r="K60" s="4" t="n">
-        <v>50.15</v>
+        <v>350.53</v>
       </c>
       <c r="L60" s="21">
         <f>IF(OR($B60="",$I60=""),"",$I60-IF($K60="",0,$K60))</f>
@@ -4458,19 +4470,19 @@
       </c>
       <c r="O60" s="23" t="inlineStr">
         <is>
-          <t>10-15</t>
+          <t>5-10</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261027586409+221261027604309+221261027604909+221261027605409+221261027606009+221261027606309+221261027606809+23126102781909+321261027589409+321261027590009+221261027608409</t>
+          <t>DHAN-221261027603809+34126102781409+221261027604809+321261027587109+23126102781309+23126102781609+34126102782109+34126102782609+321261027589509+321261027590209+34126102783109+23126102782509</t>
         </is>
       </c>
       <c r="B61" s="23" t="inlineStr">
         <is>
-          <t>JISLJALEQS</t>
+          <t>MAHLOG</t>
         </is>
       </c>
       <c r="C61" s="23" t="inlineStr">
@@ -4482,13 +4494,17 @@
         <v>46322</v>
       </c>
       <c r="E61" s="25" t="n">
-        <v>24.9779</v>
+        <v>434.8638</v>
       </c>
       <c r="F61" s="26" t="n">
-        <v>6857</v>
-      </c>
-      <c r="G61" s="24" t="inlineStr"/>
-      <c r="H61" s="25" t="inlineStr"/>
+        <v>394</v>
+      </c>
+      <c r="G61" s="24" t="n">
+        <v>46323</v>
+      </c>
+      <c r="H61" s="25" t="n">
+        <v>426.03</v>
+      </c>
       <c r="I61" s="21">
         <f>IF(OR($B61="",$H61=""),"",IF($C61="LONG",($H61-$E61)*$F61,($E61-$H61)*$F61))</f>
         <v/>
@@ -4498,7 +4514,7 @@
         <v/>
       </c>
       <c r="K61" s="4" t="n">
-        <v>50.15</v>
+        <v>353.48</v>
       </c>
       <c r="L61" s="21">
         <f>IF(OR($B61="",$I61=""),"",$I61-IF($K61="",0,$K61))</f>
@@ -4514,19 +4530,19 @@
       </c>
       <c r="O61" s="23" t="inlineStr">
         <is>
-          <t>5-10</t>
+          <t>10-15</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261027603809+34126102781409+221261027604809+321261027587109+23126102781309+23126102781609+34126102782109+34126102782609+321261027589509+321261027590209+34126102783109+23126102782509</t>
+          <t>DHAN-23126102780609+321261027586709+221261027605009+221261027605509+321261027587309+321261027587809+221261027606909+321261027588809+34126102782809+321261027590109+23126102782309+23126102782609</t>
         </is>
       </c>
       <c r="B62" s="23" t="inlineStr">
         <is>
-          <t>MAHLOG</t>
+          <t>PARACABLES</t>
         </is>
       </c>
       <c r="C62" s="23" t="inlineStr">
@@ -4538,13 +4554,17 @@
         <v>46322</v>
       </c>
       <c r="E62" s="25" t="n">
-        <v>434.8638</v>
+        <v>65.38590000000001</v>
       </c>
       <c r="F62" s="26" t="n">
-        <v>394</v>
-      </c>
-      <c r="G62" s="24" t="inlineStr"/>
-      <c r="H62" s="25" t="inlineStr"/>
+        <v>2614</v>
+      </c>
+      <c r="G62" s="24" t="n">
+        <v>46323</v>
+      </c>
+      <c r="H62" s="25" t="n">
+        <v>64.59999999999999</v>
+      </c>
       <c r="I62" s="21">
         <f>IF(OR($B62="",$H62=""),"",IF($C62="LONG",($H62-$E62)*$F62,($E62-$H62)*$F62))</f>
         <v/>
@@ -4554,7 +4574,7 @@
         <v/>
       </c>
       <c r="K62" s="4" t="n">
-        <v>50.15</v>
+        <v>347.56</v>
       </c>
       <c r="L62" s="21">
         <f>IF(OR($B62="",$I62=""),"",$I62-IF($K62="",0,$K62))</f>
@@ -4570,19 +4590,19 @@
       </c>
       <c r="O62" s="23" t="inlineStr">
         <is>
-          <t>10-15</t>
+          <t>5-10</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="23" t="inlineStr">
         <is>
-          <t>DHAN-23126102780609+321261027586709+221261027605009+221261027605509+321261027587309+321261027587809+221261027606909+321261027588809+34126102782809+321261027590109+23126102782309+23126102782609</t>
+          <t>DHAN-221261027604009+34126102781209+321261027587009+221261027605609+23126102781409+321261027587709+34126102782009+34126102782509+23126102782109+321261027590309+34126102783309+321261027591009+321261027591709</t>
         </is>
       </c>
       <c r="B63" s="23" t="inlineStr">
         <is>
-          <t>PARACABLES</t>
+          <t>ZAGGLE</t>
         </is>
       </c>
       <c r="C63" s="23" t="inlineStr">
@@ -4594,13 +4614,17 @@
         <v>46322</v>
       </c>
       <c r="E63" s="25" t="n">
-        <v>65.38590000000001</v>
+        <v>164.4613</v>
       </c>
       <c r="F63" s="26" t="n">
-        <v>2614</v>
-      </c>
-      <c r="G63" s="24" t="inlineStr"/>
-      <c r="H63" s="25" t="inlineStr"/>
+        <v>1041</v>
+      </c>
+      <c r="G63" s="24" t="n">
+        <v>46323</v>
+      </c>
+      <c r="H63" s="25" t="n">
+        <v>159.81</v>
+      </c>
       <c r="I63" s="21">
         <f>IF(OR($B63="",$H63=""),"",IF($C63="LONG",($H63-$E63)*$F63,($E63-$H63)*$F63))</f>
         <v/>
@@ -4610,7 +4634,7 @@
         <v/>
       </c>
       <c r="K63" s="4" t="n">
-        <v>50.15</v>
+        <v>348.6</v>
       </c>
       <c r="L63" s="21">
         <f>IF(OR($B63="",$I63=""),"",$I63-IF($K63="",0,$K63))</f>
@@ -4633,12 +4657,12 @@
     <row r="64">
       <c r="A64" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261027604009+34126102781209+321261027587009+221261027605609+23126102781409+321261027587709+34126102782009+34126102782509+23126102782109+321261027590309+34126102783309+321261027591009+321261027591709</t>
+          <t>DHAN-341261028101109+231261028103509+3212610281010209+341261028101309+3212610281010909+341261028101509+3212610281011309+3212610281011409+231261028104009+231261028104109+341261028102109+341261028102309</t>
         </is>
       </c>
       <c r="B64" s="23" t="inlineStr">
         <is>
-          <t>ZAGGLE</t>
+          <t>AARTIDRUGS</t>
         </is>
       </c>
       <c r="C64" s="23" t="inlineStr">
@@ -4647,13 +4671,13 @@
         </is>
       </c>
       <c r="D64" s="24" t="n">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="E64" s="25" t="n">
-        <v>164.4613</v>
+        <v>449.1103</v>
       </c>
       <c r="F64" s="26" t="n">
-        <v>1041</v>
+        <v>668</v>
       </c>
       <c r="G64" s="24" t="inlineStr"/>
       <c r="H64" s="25" t="inlineStr"/>
@@ -4682,19 +4706,37 @@
       </c>
       <c r="O64" s="23" t="inlineStr">
         <is>
-          <t>5-10</t>
+          <t>10-15</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="23" t="n"/>
-      <c r="B65" s="23" t="n"/>
-      <c r="C65" s="23" t="n"/>
-      <c r="D65" s="24" t="n"/>
-      <c r="E65" s="25" t="n"/>
-      <c r="F65" s="26" t="n"/>
-      <c r="G65" s="24" t="n"/>
-      <c r="H65" s="25" t="n"/>
+      <c r="A65" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126102780509+34126102781309+23126102781009+23126102781209+221261027605909+34126102781909+321261027588609+23126102781809+321261027589309+23126102782209+321261027590909+23126102782809+34126102783609</t>
+        </is>
+      </c>
+      <c r="B65" s="23" t="inlineStr">
+        <is>
+          <t>BAJEL</t>
+        </is>
+      </c>
+      <c r="C65" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D65" s="24" t="n">
+        <v>46322</v>
+      </c>
+      <c r="E65" s="25" t="n">
+        <v>168.7027</v>
+      </c>
+      <c r="F65" s="26" t="n">
+        <v>507</v>
+      </c>
+      <c r="G65" s="24" t="inlineStr"/>
+      <c r="H65" s="25" t="inlineStr"/>
       <c r="I65" s="21">
         <f>IF(OR($B65="",$H65=""),"",IF($C65="LONG",($H65-$E65)*$F65,($E65-$H65)*$F65))</f>
         <v/>
@@ -4703,7 +4745,9 @@
         <f>IF(OR($B65="",$I65="",$E65=0,$F65=0),"",$I65/($E65*$F65))</f>
         <v/>
       </c>
-      <c r="K65" s="4" t="n"/>
+      <c r="K65" s="4" t="n">
+        <v>122.32</v>
+      </c>
       <c r="L65" s="21">
         <f>IF(OR($B65="",$I65=""),"",$I65-IF($K65="",0,$K65))</f>
         <v/>
@@ -4716,17 +4760,39 @@
         <f>IF($B65="","",IF($H65="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O65" s="23" t="n"/>
+      <c r="O65" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="66">
-      <c r="A66" s="23" t="n"/>
-      <c r="B66" s="23" t="n"/>
-      <c r="C66" s="23" t="n"/>
-      <c r="D66" s="24" t="n"/>
-      <c r="E66" s="25" t="n"/>
-      <c r="F66" s="26" t="n"/>
-      <c r="G66" s="24" t="n"/>
-      <c r="H66" s="25" t="n"/>
+      <c r="A66" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-2212610281025009+3212610281009509+3212610281010309+231261028103709+2212610281026009+2212610281026209+2212610281026509+341261028101709+231261028103909+341261028101809+341261028102009+341261028102209+231261028104209+231261028104309+231261028104409+3212610281012909</t>
+        </is>
+      </c>
+      <c r="B66" s="23" t="inlineStr">
+        <is>
+          <t>PNGSREVA</t>
+        </is>
+      </c>
+      <c r="C66" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D66" s="24" t="n">
+        <v>46323</v>
+      </c>
+      <c r="E66" s="25" t="n">
+        <v>646.7184</v>
+      </c>
+      <c r="F66" s="26" t="n">
+        <v>465</v>
+      </c>
+      <c r="G66" s="24" t="inlineStr"/>
+      <c r="H66" s="25" t="inlineStr"/>
       <c r="I66" s="21">
         <f>IF(OR($B66="",$H66=""),"",IF($C66="LONG",($H66-$E66)*$F66,($E66-$H66)*$F66))</f>
         <v/>
@@ -4735,7 +4801,9 @@
         <f>IF(OR($B66="",$I66="",$E66=0,$F66=0),"",$I66/($E66*$F66))</f>
         <v/>
       </c>
-      <c r="K66" s="4" t="n"/>
+      <c r="K66" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L66" s="21">
         <f>IF(OR($B66="",$I66=""),"",$I66-IF($K66="",0,$K66))</f>
         <v/>
@@ -4748,7 +4816,11 @@
         <f>IF($B66="","",IF($H66="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O66" s="23" t="n"/>
+      <c r="O66" s="23" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="23" t="n"/>
@@ -31409,7 +31481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:J55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31493,7 +31565,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>AGIIL</t>
+          <t>AARTIDRUGS</t>
         </is>
       </c>
       <c r="B4" s="20">
@@ -31536,7 +31608,7 @@
     <row r="5">
       <c r="A5" s="27" t="inlineStr">
         <is>
-          <t>ARFIN</t>
+          <t>AGIIL</t>
         </is>
       </c>
       <c r="B5" s="20">
@@ -31579,7 +31651,7 @@
     <row r="6">
       <c r="A6" s="27" t="inlineStr">
         <is>
-          <t>BAJEL</t>
+          <t>ARFIN</t>
         </is>
       </c>
       <c r="B6" s="20">
@@ -31622,7 +31694,7 @@
     <row r="7">
       <c r="A7" s="27" t="inlineStr">
         <is>
-          <t>BBL</t>
+          <t>BAJEL</t>
         </is>
       </c>
       <c r="B7" s="20">
@@ -31665,7 +31737,7 @@
     <row r="8">
       <c r="A8" s="27" t="inlineStr">
         <is>
-          <t>BLUSPRING</t>
+          <t>BBL</t>
         </is>
       </c>
       <c r="B8" s="20">
@@ -31708,7 +31780,7 @@
     <row r="9">
       <c r="A9" s="27" t="inlineStr">
         <is>
-          <t>CMLL</t>
+          <t>BLUSPRING</t>
         </is>
       </c>
       <c r="B9" s="20">
@@ -31751,7 +31823,7 @@
     <row r="10">
       <c r="A10" s="27" t="inlineStr">
         <is>
-          <t>DELTACORP</t>
+          <t>CMLL</t>
         </is>
       </c>
       <c r="B10" s="20">
@@ -31794,7 +31866,7 @@
     <row r="11">
       <c r="A11" s="27" t="inlineStr">
         <is>
-          <t>DPABHUSHAN</t>
+          <t>DELTACORP</t>
         </is>
       </c>
       <c r="B11" s="20">
@@ -31837,7 +31909,7 @@
     <row r="12">
       <c r="A12" s="27" t="inlineStr">
         <is>
-          <t>EUROPRATIK</t>
+          <t>DPABHUSHAN</t>
         </is>
       </c>
       <c r="B12" s="20">
@@ -31880,7 +31952,7 @@
     <row r="13">
       <c r="A13" s="27" t="inlineStr">
         <is>
-          <t>FISCHER</t>
+          <t>EUROPRATIK</t>
         </is>
       </c>
       <c r="B13" s="20">
@@ -31923,7 +31995,7 @@
     <row r="14">
       <c r="A14" s="27" t="inlineStr">
         <is>
-          <t>GOODLUCK</t>
+          <t>FISCHER</t>
         </is>
       </c>
       <c r="B14" s="20">
@@ -31966,7 +32038,7 @@
     <row r="15">
       <c r="A15" s="27" t="inlineStr">
         <is>
-          <t>GPTINFRA</t>
+          <t>GOODLUCK</t>
         </is>
       </c>
       <c r="B15" s="20">
@@ -32009,7 +32081,7 @@
     <row r="16">
       <c r="A16" s="27" t="inlineStr">
         <is>
-          <t>HATHWAY</t>
+          <t>GPTINFRA</t>
         </is>
       </c>
       <c r="B16" s="20">
@@ -32052,7 +32124,7 @@
     <row r="17">
       <c r="A17" s="27" t="inlineStr">
         <is>
-          <t>INDIAGLYCO</t>
+          <t>HATHWAY</t>
         </is>
       </c>
       <c r="B17" s="20">
@@ -32095,7 +32167,7 @@
     <row r="18">
       <c r="A18" s="27" t="inlineStr">
         <is>
-          <t>INDOKEM</t>
+          <t>INDIAGLYCO</t>
         </is>
       </c>
       <c r="B18" s="20">
@@ -32138,7 +32210,7 @@
     <row r="19">
       <c r="A19" s="27" t="inlineStr">
         <is>
-          <t>INDOSTAR</t>
+          <t>INDOKEM</t>
         </is>
       </c>
       <c r="B19" s="20">
@@ -32181,7 +32253,7 @@
     <row r="20">
       <c r="A20" s="27" t="inlineStr">
         <is>
-          <t>INOXGREEN</t>
+          <t>INDOSTAR</t>
         </is>
       </c>
       <c r="B20" s="20">
@@ -32224,7 +32296,7 @@
     <row r="21">
       <c r="A21" s="27" t="inlineStr">
         <is>
-          <t>JAICORPLTD</t>
+          <t>INOXGREEN</t>
         </is>
       </c>
       <c r="B21" s="20">
@@ -32267,7 +32339,7 @@
     <row r="22">
       <c r="A22" s="27" t="inlineStr">
         <is>
-          <t>JINDALPOLY</t>
+          <t>JAICORPLTD</t>
         </is>
       </c>
       <c r="B22" s="20">
@@ -32310,7 +32382,7 @@
     <row r="23">
       <c r="A23" s="27" t="inlineStr">
         <is>
-          <t>JISLJALEQS</t>
+          <t>JINDALPOLY</t>
         </is>
       </c>
       <c r="B23" s="20">
@@ -32353,7 +32425,7 @@
     <row r="24">
       <c r="A24" s="27" t="inlineStr">
         <is>
-          <t>KOTIC</t>
+          <t>JISLJALEQS</t>
         </is>
       </c>
       <c r="B24" s="20">
@@ -32396,7 +32468,7 @@
     <row r="25">
       <c r="A25" s="27" t="inlineStr">
         <is>
-          <t>KRISHNADEF</t>
+          <t>KOTIC</t>
         </is>
       </c>
       <c r="B25" s="20">
@@ -32439,7 +32511,7 @@
     <row r="26">
       <c r="A26" s="27" t="inlineStr">
         <is>
-          <t>KROSS</t>
+          <t>KRISHNADEF</t>
         </is>
       </c>
       <c r="B26" s="20">
@@ -32482,7 +32554,7 @@
     <row r="27">
       <c r="A27" s="27" t="inlineStr">
         <is>
-          <t>MAHLOG</t>
+          <t>KROSS</t>
         </is>
       </c>
       <c r="B27" s="20">
@@ -32525,7 +32597,7 @@
     <row r="28">
       <c r="A28" s="27" t="inlineStr">
         <is>
-          <t>MBEL</t>
+          <t>MAHLOG</t>
         </is>
       </c>
       <c r="B28" s="20">
@@ -32568,7 +32640,7 @@
     <row r="29">
       <c r="A29" s="27" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>MBEL</t>
         </is>
       </c>
       <c r="B29" s="20">
@@ -32611,7 +32683,7 @@
     <row r="30">
       <c r="A30" s="27" t="inlineStr">
         <is>
-          <t>MOBIKWIK</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="B30" s="20">
@@ -32654,7 +32726,7 @@
     <row r="31">
       <c r="A31" s="27" t="inlineStr">
         <is>
-          <t>NIBE</t>
+          <t>MOBIKWIK</t>
         </is>
       </c>
       <c r="B31" s="20">
@@ -32697,7 +32769,7 @@
     <row r="32">
       <c r="A32" s="27" t="inlineStr">
         <is>
-          <t>OAL</t>
+          <t>NIBE</t>
         </is>
       </c>
       <c r="B32" s="20">
@@ -32740,7 +32812,7 @@
     <row r="33">
       <c r="A33" s="27" t="inlineStr">
         <is>
-          <t>ORIENTELEC</t>
+          <t>OAL</t>
         </is>
       </c>
       <c r="B33" s="20">
@@ -32783,7 +32855,7 @@
     <row r="34">
       <c r="A34" s="27" t="inlineStr">
         <is>
-          <t>PARACABLES</t>
+          <t>ORIENTELEC</t>
         </is>
       </c>
       <c r="B34" s="20">
@@ -32826,7 +32898,7 @@
     <row r="35">
       <c r="A35" s="27" t="inlineStr">
         <is>
-          <t>PIXTRANS</t>
+          <t>PARACABLES</t>
         </is>
       </c>
       <c r="B35" s="20">
@@ -32869,7 +32941,7 @@
     <row r="36">
       <c r="A36" s="27" t="inlineStr">
         <is>
-          <t>PNCINFRA</t>
+          <t>PIXTRANS</t>
         </is>
       </c>
       <c r="B36" s="20">
@@ -32912,7 +32984,7 @@
     <row r="37">
       <c r="A37" s="27" t="inlineStr">
         <is>
-          <t>PNGSREVA</t>
+          <t>PNCINFRA</t>
         </is>
       </c>
       <c r="B37" s="20">
@@ -32955,7 +33027,7 @@
     <row r="38">
       <c r="A38" s="27" t="inlineStr">
         <is>
-          <t>PRINCEPIPE</t>
+          <t>PNGSREVA</t>
         </is>
       </c>
       <c r="B38" s="20">
@@ -32998,7 +33070,7 @@
     <row r="39">
       <c r="A39" s="27" t="inlineStr">
         <is>
-          <t>RSYSTEMS</t>
+          <t>PRINCEPIPE</t>
         </is>
       </c>
       <c r="B39" s="20">
@@ -33041,7 +33113,7 @@
     <row r="40">
       <c r="A40" s="27" t="inlineStr">
         <is>
-          <t>RUBYMILLS</t>
+          <t>RSYSTEMS</t>
         </is>
       </c>
       <c r="B40" s="20">
@@ -33084,7 +33156,7 @@
     <row r="41">
       <c r="A41" s="27" t="inlineStr">
         <is>
-          <t>SAKSOFT</t>
+          <t>RUBYMILLS</t>
         </is>
       </c>
       <c r="B41" s="20">
@@ -33127,7 +33199,7 @@
     <row r="42">
       <c r="A42" s="27" t="inlineStr">
         <is>
-          <t>SATIN</t>
+          <t>SAKSOFT</t>
         </is>
       </c>
       <c r="B42" s="20">
@@ -33170,7 +33242,7 @@
     <row r="43">
       <c r="A43" s="27" t="inlineStr">
         <is>
-          <t>SGFIN</t>
+          <t>SATIN</t>
         </is>
       </c>
       <c r="B43" s="20">
@@ -33213,7 +33285,7 @@
     <row r="44">
       <c r="A44" s="27" t="inlineStr">
         <is>
-          <t>SHRINGARMS</t>
+          <t>SGFIN</t>
         </is>
       </c>
       <c r="B44" s="20">
@@ -33256,7 +33328,7 @@
     <row r="45">
       <c r="A45" s="27" t="inlineStr">
         <is>
-          <t>SIMPLEXINF</t>
+          <t>SHRINGARMS</t>
         </is>
       </c>
       <c r="B45" s="20">
@@ -33299,7 +33371,7 @@
     <row r="46">
       <c r="A46" s="27" t="inlineStr">
         <is>
-          <t>SMCGLOBAL</t>
+          <t>SIMPLEXINF</t>
         </is>
       </c>
       <c r="B46" s="20">
@@ -33342,7 +33414,7 @@
     <row r="47">
       <c r="A47" s="27" t="inlineStr">
         <is>
-          <t>SOLARA</t>
+          <t>SMCGLOBAL</t>
         </is>
       </c>
       <c r="B47" s="20">
@@ -33385,7 +33457,7 @@
     <row r="48">
       <c r="A48" s="27" t="inlineStr">
         <is>
-          <t>SPORTKING</t>
+          <t>SOLARA</t>
         </is>
       </c>
       <c r="B48" s="20">
@@ -33428,7 +33500,7 @@
     <row r="49">
       <c r="A49" s="27" t="inlineStr">
         <is>
-          <t>SUNCLAY</t>
+          <t>SPORTKING</t>
         </is>
       </c>
       <c r="B49" s="20">
@@ -33471,7 +33543,7 @@
     <row r="50">
       <c r="A50" s="27" t="inlineStr">
         <is>
-          <t>SWARAJENG</t>
+          <t>SUNCLAY</t>
         </is>
       </c>
       <c r="B50" s="20">
@@ -33514,7 +33586,7 @@
     <row r="51">
       <c r="A51" s="27" t="inlineStr">
         <is>
-          <t>TEAMLEASE</t>
+          <t>SWARAJENG</t>
         </is>
       </c>
       <c r="B51" s="20">
@@ -33557,7 +33629,7 @@
     <row r="52">
       <c r="A52" s="27" t="inlineStr">
         <is>
-          <t>YUKEN</t>
+          <t>TEAMLEASE</t>
         </is>
       </c>
       <c r="B52" s="20">
@@ -33600,7 +33672,7 @@
     <row r="53">
       <c r="A53" s="27" t="inlineStr">
         <is>
-          <t>ZAGGLE</t>
+          <t>YUKEN</t>
         </is>
       </c>
       <c r="B53" s="20">
@@ -33641,37 +33713,80 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="3" t="inlineStr">
+      <c r="A54" s="27" t="inlineStr">
+        <is>
+          <t>ZAGGLE</t>
+        </is>
+      </c>
+      <c r="B54" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A54)</f>
+        <v/>
+      </c>
+      <c r="C54" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A54,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D54" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A54,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E54" s="22">
+        <f>IFERROR($C54/$B54,"")</f>
+        <v/>
+      </c>
+      <c r="F54" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A54,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G54" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A54,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H54" s="21">
+        <f>IFERROR($G54/$B54,"")</f>
+        <v/>
+      </c>
+      <c r="I54" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A54),"")</f>
+        <v/>
+      </c>
+      <c r="J54" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A54),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B54" s="30">
-        <f>SUM(B4:B53)</f>
-        <v/>
-      </c>
-      <c r="C54" s="30">
-        <f>SUM(C4:C53)</f>
-        <v/>
-      </c>
-      <c r="D54" s="30">
-        <f>SUM(D4:D53)</f>
-        <v/>
-      </c>
-      <c r="E54" s="31">
-        <f>IFERROR(C54/B54,"")</f>
-        <v/>
-      </c>
-      <c r="F54" s="32">
-        <f>SUM(F4:F53)</f>
-        <v/>
-      </c>
-      <c r="G54" s="32">
-        <f>SUM(G4:G53)</f>
-        <v/>
-      </c>
-      <c r="H54" s="32">
-        <f>IFERROR(G54/B54,"")</f>
+      <c r="B55" s="30">
+        <f>SUM(B4:B54)</f>
+        <v/>
+      </c>
+      <c r="C55" s="30">
+        <f>SUM(C4:C54)</f>
+        <v/>
+      </c>
+      <c r="D55" s="30">
+        <f>SUM(D4:D54)</f>
+        <v/>
+      </c>
+      <c r="E55" s="31">
+        <f>IFERROR(C55/B55,"")</f>
+        <v/>
+      </c>
+      <c r="F55" s="32">
+        <f>SUM(F4:F54)</f>
+        <v/>
+      </c>
+      <c r="G55" s="32">
+        <f>SUM(G4:G54)</f>
+        <v/>
+      </c>
+      <c r="H55" s="32">
+        <f>IFERROR(G55/B55,"")</f>
         <v/>
       </c>
     </row>
@@ -33690,7 +33805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N65"/>
+  <dimension ref="A1:N67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -34094,7 +34209,7 @@
         <v>35.4</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>115.66</v>
+        <v>115.65</v>
       </c>
       <c r="N9" s="21">
         <f>SUM(E9:M9)</f>
@@ -34196,7 +34311,7 @@
         <v>35.4</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>59.52</v>
+        <v>59.51</v>
       </c>
       <c r="N11" s="21">
         <f>SUM(E11:M11)</f>
@@ -34247,7 +34362,7 @@
         <v>35.4</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>71.33</v>
+        <v>71.31999999999999</v>
       </c>
       <c r="N12" s="21">
         <f>SUM(E12:M12)</f>
@@ -34298,7 +34413,7 @@
         <v>35.4</v>
       </c>
       <c r="M13" s="4" t="n">
-        <v>72.97</v>
+        <v>73.01000000000001</v>
       </c>
       <c r="N13" s="21">
         <f>SUM(E13:M13)</f>
@@ -34502,7 +34617,7 @@
         <v>35.4</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>83.31999999999999</v>
+        <v>83.31</v>
       </c>
       <c r="N17" s="21">
         <f>SUM(E17:M17)</f>
@@ -34604,7 +34719,7 @@
         <v>35.4</v>
       </c>
       <c r="M19" s="4" t="n">
-        <v>86.56</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="N19" s="21">
         <f>SUM(E19:M19)</f>
@@ -34655,7 +34770,7 @@
         <v>35.4</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>83.41</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="N20" s="21">
         <f>SUM(E20:M20)</f>
@@ -34757,7 +34872,7 @@
         <v>35.4</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>83.81</v>
+        <v>83.8</v>
       </c>
       <c r="N22" s="21">
         <f>SUM(E22:M22)</f>
@@ -34808,7 +34923,7 @@
         <v>35.4</v>
       </c>
       <c r="M23" s="4" t="n">
-        <v>29.85</v>
+        <v>29.84</v>
       </c>
       <c r="N23" s="21">
         <f>SUM(E23:M23)</f>
@@ -34910,7 +35025,7 @@
         <v>35.4</v>
       </c>
       <c r="M25" s="4" t="n">
-        <v>37.1</v>
+        <v>37.06</v>
       </c>
       <c r="N25" s="21">
         <f>SUM(E25:M25)</f>
@@ -35012,7 +35127,7 @@
         <v>35.4</v>
       </c>
       <c r="M27" s="4" t="n">
-        <v>35.69</v>
+        <v>35.68</v>
       </c>
       <c r="N27" s="21">
         <f>SUM(E27:M27)</f>
@@ -35063,7 +35178,7 @@
         <v>35.4</v>
       </c>
       <c r="M28" s="4" t="n">
-        <v>40.87</v>
+        <v>40.86</v>
       </c>
       <c r="N28" s="21">
         <f>SUM(E28:M28)</f>
@@ -35114,7 +35229,7 @@
         <v>35.4</v>
       </c>
       <c r="M29" s="4" t="n">
-        <v>42.6</v>
+        <v>42.61</v>
       </c>
       <c r="N29" s="21">
         <f>SUM(E29:M29)</f>
@@ -35165,7 +35280,7 @@
         <v>35.4</v>
       </c>
       <c r="M30" s="4" t="n">
-        <v>35.66</v>
+        <v>35.65</v>
       </c>
       <c r="N30" s="21">
         <f>SUM(E30:M30)</f>
@@ -35369,7 +35484,7 @@
         <v>35.4</v>
       </c>
       <c r="M34" s="4" t="n">
-        <v>37.68</v>
+        <v>37.7</v>
       </c>
       <c r="N34" s="21">
         <f>SUM(E34:M34)</f>
@@ -35471,7 +35586,7 @@
         <v>35.4</v>
       </c>
       <c r="M36" s="4" t="n">
-        <v>35.61</v>
+        <v>35.6</v>
       </c>
       <c r="N36" s="21">
         <f>SUM(E36:M36)</f>
@@ -35522,7 +35637,7 @@
         <v>35.4</v>
       </c>
       <c r="M37" s="4" t="n">
-        <v>31.42</v>
+        <v>31.44</v>
       </c>
       <c r="N37" s="21">
         <f>SUM(E37:M37)</f>
@@ -35726,7 +35841,7 @@
         <v>35.4</v>
       </c>
       <c r="M41" s="4" t="n">
-        <v>234.11</v>
+        <v>234.24</v>
       </c>
       <c r="N41" s="21">
         <f>SUM(E41:M41)</f>
@@ -35777,7 +35892,7 @@
         <v>35.4</v>
       </c>
       <c r="M42" s="4" t="n">
-        <v>27.76</v>
+        <v>27.75</v>
       </c>
       <c r="N42" s="21">
         <f>SUM(E42:M42)</f>
@@ -35828,7 +35943,7 @@
         <v>35.4</v>
       </c>
       <c r="M43" s="4" t="n">
-        <v>80.45</v>
+        <v>80.54000000000001</v>
       </c>
       <c r="N43" s="21">
         <f>SUM(E43:M43)</f>
@@ -35930,7 +36045,7 @@
         <v>35.4</v>
       </c>
       <c r="M45" s="4" t="n">
-        <v>85.7</v>
+        <v>85.76000000000001</v>
       </c>
       <c r="N45" s="21">
         <f>SUM(E45:M45)</f>
@@ -35981,7 +36096,7 @@
         <v>35.4</v>
       </c>
       <c r="M46" s="4" t="n">
-        <v>75.66</v>
+        <v>75.69</v>
       </c>
       <c r="N46" s="21">
         <f>SUM(E46:M46)</f>
@@ -36032,7 +36147,7 @@
         <v>35.4</v>
       </c>
       <c r="M47" s="4" t="n">
-        <v>178.83</v>
+        <v>178.96</v>
       </c>
       <c r="N47" s="21">
         <f>SUM(E47:M47)</f>
@@ -36083,7 +36198,7 @@
         <v>35.4</v>
       </c>
       <c r="M48" s="4" t="n">
-        <v>179.79</v>
+        <v>179.92</v>
       </c>
       <c r="N48" s="21">
         <f>SUM(E48:M48)</f>
@@ -36134,7 +36249,7 @@
         <v>35.4</v>
       </c>
       <c r="M49" s="4" t="n">
-        <v>175.26</v>
+        <v>174.22</v>
       </c>
       <c r="N49" s="21">
         <f>SUM(E49:M49)</f>
@@ -36185,7 +36300,7 @@
         <v>35.4</v>
       </c>
       <c r="M50" s="4" t="n">
-        <v>180.15</v>
+        <v>180.27</v>
       </c>
       <c r="N50" s="21">
         <f>SUM(E50:M50)</f>
@@ -36236,7 +36351,7 @@
         <v>35.4</v>
       </c>
       <c r="M51" s="4" t="n">
-        <v>142.48</v>
+        <v>142.7</v>
       </c>
       <c r="N51" s="21">
         <f>SUM(E51:M51)</f>
@@ -36287,7 +36402,7 @@
         <v>35.4</v>
       </c>
       <c r="M52" s="4" t="n">
-        <v>111.98</v>
+        <v>112.06</v>
       </c>
       <c r="N52" s="21">
         <f>SUM(E52:M52)</f>
@@ -36491,7 +36606,7 @@
         <v>35.4</v>
       </c>
       <c r="M56" s="4" t="n">
-        <v>46.11</v>
+        <v>46.18</v>
       </c>
       <c r="N56" s="21">
         <f>SUM(E56:M56)</f>
@@ -36518,22 +36633,22 @@
         <v>46322</v>
       </c>
       <c r="E57" s="4" t="n">
-        <v>90.05</v>
+        <v>117.55</v>
       </c>
       <c r="F57" s="4" t="n">
-        <v>300.07</v>
+        <v>614.85</v>
       </c>
       <c r="G57" s="4" t="n">
-        <v>9.210000000000001</v>
+        <v>18.87</v>
       </c>
       <c r="H57" s="4" t="n">
-        <v>0.3</v>
+        <v>0.61</v>
       </c>
       <c r="I57" s="4" t="n">
         <v>45.22</v>
       </c>
       <c r="J57" s="4" t="n">
-        <v>17.92</v>
+        <v>24.67</v>
       </c>
       <c r="K57" s="4" t="n">
         <v>14.75</v>
@@ -36565,24 +36680,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D58" s="24" t="inlineStr"/>
+      <c r="D58" s="24" t="n">
+        <v>46323</v>
+      </c>
       <c r="E58" s="4" t="n">
-        <v>0</v>
+        <v>51.55</v>
       </c>
       <c r="F58" s="4" t="n">
-        <v>0</v>
+        <v>171.81</v>
       </c>
       <c r="G58" s="4" t="n">
-        <v>0</v>
+        <v>5.27</v>
       </c>
       <c r="H58" s="4" t="n">
-        <v>0</v>
+        <v>0.17</v>
       </c>
       <c r="I58" s="4" t="n">
-        <v>0</v>
+        <v>25.77</v>
       </c>
       <c r="J58" s="4" t="n">
-        <v>0</v>
+        <v>10.26</v>
       </c>
       <c r="K58" s="4" t="n">
         <v>14.75</v>
@@ -36591,7 +36708,7 @@
         <v>35.4</v>
       </c>
       <c r="M58" s="4" t="n">
-        <v>0</v>
+        <v>36.45</v>
       </c>
       <c r="N58" s="21">
         <f>SUM(E58:M58)</f>
@@ -36601,12 +36718,12 @@
     <row r="59">
       <c r="A59" s="23" t="inlineStr">
         <is>
-          <t>DHAN-23126102780509+34126102781309+23126102781009+23126102781209+221261027605909+34126102781909+321261027588609+23126102781809+321261027589309+23126102782209+321261027590909+23126102782809+34126102783609</t>
+          <t>DHAN-221261027603909+23126102780809+34126102781609+221261027605309+34126102781809+221261027606409+34126102782209+34126102782709+221261027607909+34126102782909+34126102783209+34126102783409+321261027591809+23126102783009</t>
         </is>
       </c>
       <c r="B59" s="23" t="inlineStr">
         <is>
-          <t>BAJEL</t>
+          <t>BBL</t>
         </is>
       </c>
       <c r="C59" s="23" t="inlineStr">
@@ -36614,33 +36731,35 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D59" s="24" t="inlineStr"/>
+      <c r="D59" s="24" t="n">
+        <v>46323</v>
+      </c>
       <c r="E59" s="4" t="n">
-        <v>0</v>
+        <v>51.24</v>
       </c>
       <c r="F59" s="4" t="n">
-        <v>0</v>
+        <v>170.82</v>
       </c>
       <c r="G59" s="4" t="n">
-        <v>0</v>
+        <v>5.24</v>
       </c>
       <c r="H59" s="4" t="n">
-        <v>0</v>
+        <v>0.17</v>
       </c>
       <c r="I59" s="4" t="n">
-        <v>0</v>
+        <v>25.62</v>
       </c>
       <c r="J59" s="4" t="n">
-        <v>0</v>
+        <v>10.2</v>
       </c>
       <c r="K59" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L59" s="4" t="n">
-        <v>0</v>
+        <v>35.4</v>
       </c>
       <c r="M59" s="4" t="n">
-        <v>0</v>
+        <v>37.93</v>
       </c>
       <c r="N59" s="21">
         <f>SUM(E59:M59)</f>
@@ -36650,12 +36769,12 @@
     <row r="60">
       <c r="A60" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261027603909+23126102780809+34126102781609+221261027605309+34126102781809+221261027606409+34126102782209+34126102782709+221261027607909+34126102782909+34126102783209+34126102783409+321261027591809+23126102783009</t>
+          <t>DHAN-321261027586409+221261027604309+221261027604909+221261027605409+221261027606009+221261027606309+221261027606809+23126102781909+321261027589409+321261027590009+221261027608409</t>
         </is>
       </c>
       <c r="B60" s="23" t="inlineStr">
         <is>
-          <t>BBL</t>
+          <t>JISLJALEQS</t>
         </is>
       </c>
       <c r="C60" s="23" t="inlineStr">
@@ -36663,24 +36782,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D60" s="24" t="inlineStr"/>
+      <c r="D60" s="24" t="n">
+        <v>46323</v>
+      </c>
       <c r="E60" s="4" t="n">
-        <v>0</v>
+        <v>51.45</v>
       </c>
       <c r="F60" s="4" t="n">
-        <v>0</v>
+        <v>171.29</v>
       </c>
       <c r="G60" s="4" t="n">
-        <v>0</v>
+        <v>5.26</v>
       </c>
       <c r="H60" s="4" t="n">
-        <v>0</v>
+        <v>0.17</v>
       </c>
       <c r="I60" s="4" t="n">
-        <v>0</v>
+        <v>25.26</v>
       </c>
       <c r="J60" s="4" t="n">
-        <v>0</v>
+        <v>10.24</v>
       </c>
       <c r="K60" s="4" t="n">
         <v>14.75</v>
@@ -36689,7 +36810,7 @@
         <v>35.4</v>
       </c>
       <c r="M60" s="4" t="n">
-        <v>0</v>
+        <v>36.72</v>
       </c>
       <c r="N60" s="21">
         <f>SUM(E60:M60)</f>
@@ -36699,12 +36820,12 @@
     <row r="61">
       <c r="A61" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261027586409+221261027604309+221261027604909+221261027605409+221261027606009+221261027606309+221261027606809+23126102781909+321261027589409+321261027590009+221261027608409</t>
+          <t>DHAN-221261027603809+34126102781409+221261027604809+321261027587109+23126102781309+23126102781609+34126102782109+34126102782609+321261027589509+321261027590209+34126102783109+23126102782509</t>
         </is>
       </c>
       <c r="B61" s="23" t="inlineStr">
         <is>
-          <t>JISLJALEQS</t>
+          <t>MAHLOG</t>
         </is>
       </c>
       <c r="C61" s="23" t="inlineStr">
@@ -36712,24 +36833,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D61" s="24" t="inlineStr"/>
+      <c r="D61" s="24" t="n">
+        <v>46323</v>
+      </c>
       <c r="E61" s="4" t="n">
-        <v>0</v>
+        <v>51.41</v>
       </c>
       <c r="F61" s="4" t="n">
-        <v>0</v>
+        <v>171.33</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>0</v>
+        <v>5.26</v>
       </c>
       <c r="H61" s="4" t="n">
-        <v>0</v>
+        <v>0.17</v>
       </c>
       <c r="I61" s="4" t="n">
-        <v>0</v>
+        <v>25.7</v>
       </c>
       <c r="J61" s="4" t="n">
-        <v>0</v>
+        <v>10.23</v>
       </c>
       <c r="K61" s="4" t="n">
         <v>14.75</v>
@@ -36738,7 +36861,7 @@
         <v>35.4</v>
       </c>
       <c r="M61" s="4" t="n">
-        <v>0</v>
+        <v>39.22</v>
       </c>
       <c r="N61" s="21">
         <f>SUM(E61:M61)</f>
@@ -36748,12 +36871,12 @@
     <row r="62">
       <c r="A62" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261027603809+34126102781409+221261027604809+321261027587109+23126102781309+23126102781609+34126102782109+34126102782609+321261027589509+321261027590209+34126102783109+23126102782509</t>
+          <t>DHAN-23126102780609+321261027586709+221261027605009+221261027605509+321261027587309+321261027587809+221261027606909+321261027588809+34126102782809+321261027590109+23126102782309+23126102782609</t>
         </is>
       </c>
       <c r="B62" s="23" t="inlineStr">
         <is>
-          <t>MAHLOG</t>
+          <t>PARACABLES</t>
         </is>
       </c>
       <c r="C62" s="23" t="inlineStr">
@@ -36761,24 +36884,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D62" s="24" t="inlineStr"/>
+      <c r="D62" s="24" t="n">
+        <v>46323</v>
+      </c>
       <c r="E62" s="4" t="n">
-        <v>0</v>
+        <v>51.28</v>
       </c>
       <c r="F62" s="4" t="n">
-        <v>0</v>
+        <v>170.93</v>
       </c>
       <c r="G62" s="4" t="n">
-        <v>0</v>
+        <v>5.25</v>
       </c>
       <c r="H62" s="4" t="n">
-        <v>0</v>
+        <v>0.17</v>
       </c>
       <c r="I62" s="4" t="n">
-        <v>0</v>
+        <v>25.64</v>
       </c>
       <c r="J62" s="4" t="n">
-        <v>0</v>
+        <v>10.21</v>
       </c>
       <c r="K62" s="4" t="n">
         <v>14.75</v>
@@ -36787,7 +36912,7 @@
         <v>35.4</v>
       </c>
       <c r="M62" s="4" t="n">
-        <v>0</v>
+        <v>33.94</v>
       </c>
       <c r="N62" s="21">
         <f>SUM(E62:M62)</f>
@@ -36797,12 +36922,12 @@
     <row r="63">
       <c r="A63" s="23" t="inlineStr">
         <is>
-          <t>DHAN-23126102780609+321261027586709+221261027605009+221261027605509+321261027587309+321261027587809+221261027606909+321261027588809+34126102782809+321261027590109+23126102782309+23126102782609</t>
+          <t>DHAN-221261027604009+34126102781209+321261027587009+221261027605609+23126102781409+321261027587709+34126102782009+34126102782509+23126102782109+321261027590309+34126102783309+321261027591009+321261027591709</t>
         </is>
       </c>
       <c r="B63" s="23" t="inlineStr">
         <is>
-          <t>PARACABLES</t>
+          <t>ZAGGLE</t>
         </is>
       </c>
       <c r="C63" s="23" t="inlineStr">
@@ -36810,24 +36935,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D63" s="24" t="inlineStr"/>
+      <c r="D63" s="24" t="n">
+        <v>46323</v>
+      </c>
       <c r="E63" s="4" t="n">
-        <v>0</v>
+        <v>51.38</v>
       </c>
       <c r="F63" s="4" t="n">
-        <v>0</v>
+        <v>171.2</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>0</v>
+        <v>5.26</v>
       </c>
       <c r="H63" s="4" t="n">
-        <v>0</v>
+        <v>0.17</v>
       </c>
       <c r="I63" s="4" t="n">
-        <v>0</v>
+        <v>25.68</v>
       </c>
       <c r="J63" s="4" t="n">
-        <v>0</v>
+        <v>10.23</v>
       </c>
       <c r="K63" s="4" t="n">
         <v>14.75</v>
@@ -36836,7 +36963,7 @@
         <v>35.4</v>
       </c>
       <c r="M63" s="4" t="n">
-        <v>0</v>
+        <v>34.53</v>
       </c>
       <c r="N63" s="21">
         <f>SUM(E63:M63)</f>
@@ -36846,12 +36973,12 @@
     <row r="64">
       <c r="A64" s="23" t="inlineStr">
         <is>
-          <t>DHAN-221261027604009+34126102781209+321261027587009+221261027605609+23126102781409+321261027587709+34126102782009+34126102782509+23126102782109+321261027590309+34126102783309+321261027591009+321261027591709</t>
+          <t>DHAN-341261028101109+231261028103509+3212610281010209+341261028101309+3212610281010909+341261028101509+3212610281011309+3212610281011409+231261028104009+231261028104109+341261028102109+341261028102309</t>
         </is>
       </c>
       <c r="B64" s="23" t="inlineStr">
         <is>
-          <t>ZAGGLE</t>
+          <t>AARTIDRUGS</t>
         </is>
       </c>
       <c r="C64" s="23" t="inlineStr">
@@ -36893,54 +37020,152 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="3" t="inlineStr">
+      <c r="A65" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126102780509+34126102781309+23126102781009+23126102781209+221261027605909+34126102781909+321261027588609+23126102781809+321261027589309+23126102782209+321261027590909+23126102782809+34126102783609</t>
+        </is>
+      </c>
+      <c r="B65" s="23" t="inlineStr">
+        <is>
+          <t>BAJEL</t>
+        </is>
+      </c>
+      <c r="C65" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D65" s="24" t="inlineStr"/>
+      <c r="E65" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F65" s="4" t="n">
+        <v>90.59</v>
+      </c>
+      <c r="G65" s="4" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="H65" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="I65" s="4" t="n">
+        <v>13.59</v>
+      </c>
+      <c r="J65" s="4" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="K65" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L65" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M65" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N65" s="21">
+        <f>SUM(E65:M65)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-2212610281025009+3212610281009509+3212610281010309+231261028103709+2212610281026009+2212610281026209+2212610281026509+341261028101709+231261028103909+341261028101809+341261028102009+341261028102209+231261028104209+231261028104309+231261028104409+3212610281012909</t>
+        </is>
+      </c>
+      <c r="B66" s="23" t="inlineStr">
+        <is>
+          <t>PNGSREVA</t>
+        </is>
+      </c>
+      <c r="C66" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D66" s="24" t="inlineStr"/>
+      <c r="E66" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F66" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G66" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H66" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I66" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J66" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K66" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L66" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M66" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N66" s="21">
+        <f>SUM(E66:M66)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E65" s="32">
-        <f>SUM(E4:E64)</f>
-        <v/>
-      </c>
-      <c r="F65" s="32">
-        <f>SUM(F4:F64)</f>
-        <v/>
-      </c>
-      <c r="G65" s="32">
-        <f>SUM(G4:G64)</f>
-        <v/>
-      </c>
-      <c r="H65" s="32">
-        <f>SUM(H4:H64)</f>
-        <v/>
-      </c>
-      <c r="I65" s="32">
-        <f>SUM(I4:I64)</f>
-        <v/>
-      </c>
-      <c r="J65" s="32">
-        <f>SUM(J4:J64)</f>
-        <v/>
-      </c>
-      <c r="K65" s="32">
-        <f>SUM(K4:K64)</f>
-        <v/>
-      </c>
-      <c r="L65" s="32">
-        <f>SUM(L4:L64)</f>
-        <v/>
-      </c>
-      <c r="M65" s="32">
-        <f>SUM(M4:M64)</f>
-        <v/>
-      </c>
-      <c r="N65" s="32">
-        <f>SUM(N4:N64)</f>
+      <c r="E67" s="32">
+        <f>SUM(E4:E66)</f>
+        <v/>
+      </c>
+      <c r="F67" s="32">
+        <f>SUM(F4:F66)</f>
+        <v/>
+      </c>
+      <c r="G67" s="32">
+        <f>SUM(G4:G66)</f>
+        <v/>
+      </c>
+      <c r="H67" s="32">
+        <f>SUM(H4:H66)</f>
+        <v/>
+      </c>
+      <c r="I67" s="32">
+        <f>SUM(I4:I66)</f>
+        <v/>
+      </c>
+      <c r="J67" s="32">
+        <f>SUM(J4:J66)</f>
+        <v/>
+      </c>
+      <c r="K67" s="32">
+        <f>SUM(K4:K66)</f>
+        <v/>
+      </c>
+      <c r="L67" s="32">
+        <f>SUM(L4:L66)</f>
+        <v/>
+      </c>
+      <c r="M67" s="32">
+        <f>SUM(M4:M66)</f>
+        <v/>
+      </c>
+      <c r="N67" s="32">
+        <f>SUM(N4:N66)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:N64"/>
+  <autoFilter ref="A3:N66"/>
   <mergeCells count="2">
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>

</xml_diff>

<commit_message>
Data update — 2026-10-29 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_oct2026.xlsx
+++ b/results/strategy_pnl_oct2026.xlsx
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trade Log'!$A$3:$O$503</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$71</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1214,7 +1214,7 @@
         <v/>
       </c>
       <c r="K6" s="4" t="n">
-        <v>955</v>
+        <v>954.99</v>
       </c>
       <c r="L6" s="21">
         <f>IF(OR($B6="",$I6=""),"",$I6-IF($K6="",0,$K6))</f>
@@ -1274,7 +1274,7 @@
         <v/>
       </c>
       <c r="K7" s="4" t="n">
-        <v>819.03</v>
+        <v>819.02</v>
       </c>
       <c r="L7" s="21">
         <f>IF(OR($B7="",$I7=""),"",$I7-IF($K7="",0,$K7))</f>
@@ -1334,7 +1334,7 @@
         <v/>
       </c>
       <c r="K8" s="4" t="n">
-        <v>857.26</v>
+        <v>857.25</v>
       </c>
       <c r="L8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($K8="",0,$K8))</f>
@@ -1454,7 +1454,7 @@
         <v/>
       </c>
       <c r="K10" s="4" t="n">
-        <v>943.03</v>
+        <v>943.02</v>
       </c>
       <c r="L10" s="21">
         <f>IF(OR($B10="",$I10=""),"",$I10-IF($K10="",0,$K10))</f>
@@ -1514,7 +1514,7 @@
         <v/>
       </c>
       <c r="K11" s="4" t="n">
-        <v>691.25</v>
+        <v>691.24</v>
       </c>
       <c r="L11" s="21">
         <f>IF(OR($B11="",$I11=""),"",$I11-IF($K11="",0,$K11))</f>
@@ -1574,7 +1574,7 @@
         <v/>
       </c>
       <c r="K12" s="4" t="n">
-        <v>756.37</v>
+        <v>756.36</v>
       </c>
       <c r="L12" s="21">
         <f>IF(OR($B12="",$I12=""),"",$I12-IF($K12="",0,$K12))</f>
@@ -1634,7 +1634,7 @@
         <v/>
       </c>
       <c r="K13" s="4" t="n">
-        <v>687.97</v>
+        <v>688.04</v>
       </c>
       <c r="L13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($K13="",0,$K13))</f>
@@ -1694,7 +1694,7 @@
         <v/>
       </c>
       <c r="K14" s="4" t="n">
-        <v>683.86</v>
+        <v>683.85</v>
       </c>
       <c r="L14" s="21">
         <f>IF(OR($B14="",$I14=""),"",$I14-IF($K14="",0,$K14))</f>
@@ -1874,7 +1874,7 @@
         <v/>
       </c>
       <c r="K17" s="4" t="n">
-        <v>660.9299999999999</v>
+        <v>660.91</v>
       </c>
       <c r="L17" s="21">
         <f>IF(OR($B17="",$I17=""),"",$I17-IF($K17="",0,$K17))</f>
@@ -1994,7 +1994,7 @@
         <v/>
       </c>
       <c r="K19" s="4" t="n">
-        <v>666.78</v>
+        <v>666.85</v>
       </c>
       <c r="L19" s="21">
         <f>IF(OR($B19="",$I19=""),"",$I19-IF($K19="",0,$K19))</f>
@@ -2054,7 +2054,7 @@
         <v/>
       </c>
       <c r="K20" s="4" t="n">
-        <v>676.85</v>
+        <v>676.83</v>
       </c>
       <c r="L20" s="21">
         <f>IF(OR($B20="",$I20=""),"",$I20-IF($K20="",0,$K20))</f>
@@ -2174,7 +2174,7 @@
         <v/>
       </c>
       <c r="K22" s="4" t="n">
-        <v>658.45</v>
+        <v>658.4299999999999</v>
       </c>
       <c r="L22" s="21">
         <f>IF(OR($B22="",$I22=""),"",$I22-IF($K22="",0,$K22))</f>
@@ -2234,7 +2234,7 @@
         <v/>
       </c>
       <c r="K23" s="4" t="n">
-        <v>419.65</v>
+        <v>419.64</v>
       </c>
       <c r="L23" s="21">
         <f>IF(OR($B23="",$I23=""),"",$I23-IF($K23="",0,$K23))</f>
@@ -2354,7 +2354,7 @@
         <v/>
       </c>
       <c r="K25" s="4" t="n">
-        <v>557.26</v>
+        <v>557.28</v>
       </c>
       <c r="L25" s="21">
         <f>IF(OR($B25="",$I25=""),"",$I25-IF($K25="",0,$K25))</f>
@@ -2474,7 +2474,7 @@
         <v/>
       </c>
       <c r="K27" s="4" t="n">
-        <v>547.5700000000001</v>
+        <v>547.5599999999999</v>
       </c>
       <c r="L27" s="21">
         <f>IF(OR($B27="",$I27=""),"",$I27-IF($K27="",0,$K27))</f>
@@ -2534,7 +2534,7 @@
         <v/>
       </c>
       <c r="K28" s="4" t="n">
-        <v>547.83</v>
+        <v>547.8200000000001</v>
       </c>
       <c r="L28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($K28="",0,$K28))</f>
@@ -2594,7 +2594,7 @@
         <v/>
       </c>
       <c r="K29" s="4" t="n">
-        <v>554.61</v>
+        <v>554.62</v>
       </c>
       <c r="L29" s="21">
         <f>IF(OR($B29="",$I29=""),"",$I29-IF($K29="",0,$K29))</f>
@@ -2654,7 +2654,7 @@
         <v/>
       </c>
       <c r="K30" s="4" t="n">
-        <v>550.6900000000001</v>
+        <v>550.6799999999999</v>
       </c>
       <c r="L30" s="21">
         <f>IF(OR($B30="",$I30=""),"",$I30-IF($K30="",0,$K30))</f>
@@ -2834,7 +2834,7 @@
         <v/>
       </c>
       <c r="K33" s="4" t="n">
-        <v>550.84</v>
+        <v>550.83</v>
       </c>
       <c r="L33" s="21">
         <f>IF(OR($B33="",$I33=""),"",$I33-IF($K33="",0,$K33))</f>
@@ -2894,7 +2894,7 @@
         <v/>
       </c>
       <c r="K34" s="4" t="n">
-        <v>426.01</v>
+        <v>426.03</v>
       </c>
       <c r="L34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($K34="",0,$K34))</f>
@@ -3014,7 +3014,7 @@
         <v/>
       </c>
       <c r="K36" s="4" t="n">
-        <v>553.03</v>
+        <v>553.02</v>
       </c>
       <c r="L36" s="21">
         <f>IF(OR($B36="",$I36=""),"",$I36-IF($K36="",0,$K36))</f>
@@ -3074,7 +3074,7 @@
         <v/>
       </c>
       <c r="K37" s="4" t="n">
-        <v>477.89</v>
+        <v>477.9</v>
       </c>
       <c r="L37" s="21">
         <f>IF(OR($B37="",$I37=""),"",$I37-IF($K37="",0,$K37))</f>
@@ -3134,7 +3134,7 @@
         <v/>
       </c>
       <c r="K38" s="4" t="n">
-        <v>624.05</v>
+        <v>624.04</v>
       </c>
       <c r="L38" s="21">
         <f>IF(OR($B38="",$I38=""),"",$I38-IF($K38="",0,$K38))</f>
@@ -3194,7 +3194,7 @@
         <v/>
       </c>
       <c r="K39" s="4" t="n">
-        <v>614</v>
+        <v>613.99</v>
       </c>
       <c r="L39" s="21">
         <f>IF(OR($B39="",$I39=""),"",$I39-IF($K39="",0,$K39))</f>
@@ -3314,7 +3314,7 @@
         <v/>
       </c>
       <c r="K41" s="4" t="n">
-        <v>592.42</v>
+        <v>592.37</v>
       </c>
       <c r="L41" s="21">
         <f>IF(OR($B41="",$I41=""),"",$I41-IF($K41="",0,$K41))</f>
@@ -3374,7 +3374,7 @@
         <v/>
       </c>
       <c r="K42" s="4" t="n">
-        <v>618.36</v>
+        <v>618.35</v>
       </c>
       <c r="L42" s="21">
         <f>IF(OR($B42="",$I42=""),"",$I42-IF($K42="",0,$K42))</f>
@@ -3434,7 +3434,7 @@
         <v/>
       </c>
       <c r="K43" s="4" t="n">
-        <v>924.64</v>
+        <v>924.6900000000001</v>
       </c>
       <c r="L43" s="21">
         <f>IF(OR($B43="",$I43=""),"",$I43-IF($K43="",0,$K43))</f>
@@ -3554,7 +3554,7 @@
         <v/>
       </c>
       <c r="K45" s="4" t="n">
-        <v>945.9299999999999</v>
+        <v>945.96</v>
       </c>
       <c r="L45" s="21">
         <f>IF(OR($B45="",$I45=""),"",$I45-IF($K45="",0,$K45))</f>
@@ -3614,7 +3614,7 @@
         <v/>
       </c>
       <c r="K46" s="4" t="n">
-        <v>915.9</v>
+        <v>915.88</v>
       </c>
       <c r="L46" s="21">
         <f>IF(OR($B46="",$I46=""),"",$I46-IF($K46="",0,$K46))</f>
@@ -3674,7 +3674,7 @@
         <v/>
       </c>
       <c r="K47" s="4" t="n">
-        <v>1027</v>
+        <v>1026.96</v>
       </c>
       <c r="L47" s="21">
         <f>IF(OR($B47="",$I47=""),"",$I47-IF($K47="",0,$K47))</f>
@@ -3734,7 +3734,7 @@
         <v/>
       </c>
       <c r="K48" s="4" t="n">
-        <v>1028.69</v>
+        <v>1028.65</v>
       </c>
       <c r="L48" s="21">
         <f>IF(OR($B48="",$I48=""),"",$I48-IF($K48="",0,$K48))</f>
@@ -3794,7 +3794,7 @@
         <v/>
       </c>
       <c r="K49" s="4" t="n">
-        <v>954.05</v>
+        <v>954.08</v>
       </c>
       <c r="L49" s="21">
         <f>IF(OR($B49="",$I49=""),"",$I49-IF($K49="",0,$K49))</f>
@@ -3854,7 +3854,7 @@
         <v/>
       </c>
       <c r="K50" s="4" t="n">
-        <v>1035.39</v>
+        <v>1035.35</v>
       </c>
       <c r="L50" s="21">
         <f>IF(OR($B50="",$I50=""),"",$I50-IF($K50="",0,$K50))</f>
@@ -3914,7 +3914,7 @@
         <v/>
       </c>
       <c r="K51" s="4" t="n">
-        <v>984.75</v>
+        <v>984.84</v>
       </c>
       <c r="L51" s="21">
         <f>IF(OR($B51="",$I51=""),"",$I51-IF($K51="",0,$K51))</f>
@@ -3974,7 +3974,7 @@
         <v/>
       </c>
       <c r="K52" s="4" t="n">
-        <v>940.02</v>
+        <v>940</v>
       </c>
       <c r="L52" s="21">
         <f>IF(OR($B52="",$I52=""),"",$I52-IF($K52="",0,$K52))</f>
@@ -4214,7 +4214,7 @@
         <v/>
       </c>
       <c r="K56" s="4" t="n">
-        <v>875.26</v>
+        <v>875.27</v>
       </c>
       <c r="L56" s="21">
         <f>IF(OR($B56="",$I56=""),"",$I56-IF($K56="",0,$K56))</f>
@@ -4334,7 +4334,7 @@
         <v/>
       </c>
       <c r="K58" s="4" t="n">
-        <v>351.43</v>
+        <v>545.2</v>
       </c>
       <c r="L58" s="21">
         <f>IF(OR($B58="",$I58=""),"",$I58-IF($K58="",0,$K58))</f>
@@ -4394,7 +4394,7 @@
         <v/>
       </c>
       <c r="K59" s="4" t="n">
-        <v>351.37</v>
+        <v>552.04</v>
       </c>
       <c r="L59" s="21">
         <f>IF(OR($B59="",$I59=""),"",$I59-IF($K59="",0,$K59))</f>
@@ -4454,7 +4454,7 @@
         <v/>
       </c>
       <c r="K60" s="4" t="n">
-        <v>350.53</v>
+        <v>548.4299999999999</v>
       </c>
       <c r="L60" s="21">
         <f>IF(OR($B60="",$I60=""),"",$I60-IF($K60="",0,$K60))</f>
@@ -4514,7 +4514,7 @@
         <v/>
       </c>
       <c r="K61" s="4" t="n">
-        <v>353.48</v>
+        <v>551.7</v>
       </c>
       <c r="L61" s="21">
         <f>IF(OR($B61="",$I61=""),"",$I61-IF($K61="",0,$K61))</f>
@@ -4574,7 +4574,7 @@
         <v/>
       </c>
       <c r="K62" s="4" t="n">
-        <v>347.56</v>
+        <v>546.35</v>
       </c>
       <c r="L62" s="21">
         <f>IF(OR($B62="",$I62=""),"",$I62-IF($K62="",0,$K62))</f>
@@ -4634,7 +4634,7 @@
         <v/>
       </c>
       <c r="K63" s="4" t="n">
-        <v>348.6</v>
+        <v>544.8</v>
       </c>
       <c r="L63" s="21">
         <f>IF(OR($B63="",$I63=""),"",$I63-IF($K63="",0,$K63))</f>
@@ -4679,8 +4679,12 @@
       <c r="F64" s="26" t="n">
         <v>668</v>
       </c>
-      <c r="G64" s="24" t="inlineStr"/>
-      <c r="H64" s="25" t="inlineStr"/>
+      <c r="G64" s="24" t="n">
+        <v>46324</v>
+      </c>
+      <c r="H64" s="25" t="n">
+        <v>449.8</v>
+      </c>
       <c r="I64" s="21">
         <f>IF(OR($B64="",$H64=""),"",IF($C64="LONG",($H64-$E64)*$F64,($E64-$H64)*$F64))</f>
         <v/>
@@ -4690,7 +4694,7 @@
         <v/>
       </c>
       <c r="K64" s="4" t="n">
-        <v>50.15</v>
+        <v>582.64</v>
       </c>
       <c r="L64" s="21">
         <f>IF(OR($B64="",$I64=""),"",$I64-IF($K64="",0,$K64))</f>
@@ -4713,12 +4717,12 @@
     <row r="65">
       <c r="A65" s="23" t="inlineStr">
         <is>
-          <t>DHAN-23126102780509+34126102781309+23126102781009+23126102781209+221261027605909+34126102781909+321261027588609+23126102781809+321261027589309+23126102782209+321261027590909+23126102782809+34126102783609</t>
+          <t>DHAN-2212610281025009+3212610281009509+3212610281010309+231261028103709+2212610281026009+2212610281026209+2212610281026509+341261028101709+231261028103909+341261028101809+341261028102009+341261028102209+231261028104209+231261028104309+231261028104409+3212610281012909</t>
         </is>
       </c>
       <c r="B65" s="23" t="inlineStr">
         <is>
-          <t>BAJEL</t>
+          <t>PNGSREVA</t>
         </is>
       </c>
       <c r="C65" s="23" t="inlineStr">
@@ -4727,16 +4731,20 @@
         </is>
       </c>
       <c r="D65" s="24" t="n">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="E65" s="25" t="n">
-        <v>168.7027</v>
+        <v>646.7184</v>
       </c>
       <c r="F65" s="26" t="n">
-        <v>507</v>
-      </c>
-      <c r="G65" s="24" t="inlineStr"/>
-      <c r="H65" s="25" t="inlineStr"/>
+        <v>465</v>
+      </c>
+      <c r="G65" s="24" t="n">
+        <v>46324</v>
+      </c>
+      <c r="H65" s="25" t="n">
+        <v>658.02</v>
+      </c>
       <c r="I65" s="21">
         <f>IF(OR($B65="",$H65=""),"",IF($C65="LONG",($H65-$E65)*$F65,($E65-$H65)*$F65))</f>
         <v/>
@@ -4746,7 +4754,7 @@
         <v/>
       </c>
       <c r="K65" s="4" t="n">
-        <v>122.32</v>
+        <v>565.01</v>
       </c>
       <c r="L65" s="21">
         <f>IF(OR($B65="",$I65=""),"",$I65-IF($K65="",0,$K65))</f>
@@ -4762,19 +4770,19 @@
       </c>
       <c r="O65" s="23" t="inlineStr">
         <is>
-          <t>5-10</t>
+          <t>10-15</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="23" t="inlineStr">
         <is>
-          <t>DHAN-2212610281025009+3212610281009509+3212610281010309+231261028103709+2212610281026009+2212610281026209+2212610281026509+341261028101709+231261028103909+341261028101809+341261028102009+341261028102209+231261028104209+231261028104309+231261028104409+3212610281012909</t>
+          <t>DHAN-231261029107209+321261029713609+221261029729709+341261029101609+221261029730509+231261029108709+341261029101909+231261029109909+321261029716309+341261029102509+221261029732909+231261029110409+231261029110609</t>
         </is>
       </c>
       <c r="B66" s="23" t="inlineStr">
         <is>
-          <t>PNGSREVA</t>
+          <t>APOLLOPIPE</t>
         </is>
       </c>
       <c r="C66" s="23" t="inlineStr">
@@ -4783,13 +4791,13 @@
         </is>
       </c>
       <c r="D66" s="24" t="n">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="E66" s="25" t="n">
-        <v>646.7184</v>
+        <v>551.2455</v>
       </c>
       <c r="F66" s="26" t="n">
-        <v>465</v>
+        <v>435</v>
       </c>
       <c r="G66" s="24" t="inlineStr"/>
       <c r="H66" s="25" t="inlineStr"/>
@@ -4823,14 +4831,32 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="23" t="n"/>
-      <c r="B67" s="23" t="n"/>
-      <c r="C67" s="23" t="n"/>
-      <c r="D67" s="24" t="n"/>
-      <c r="E67" s="25" t="n"/>
-      <c r="F67" s="26" t="n"/>
-      <c r="G67" s="24" t="n"/>
-      <c r="H67" s="25" t="n"/>
+      <c r="A67" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126102780509+34126102781309+23126102781009+23126102781209+221261027605909+34126102781909+321261027588609+23126102781809+321261027589309+23126102782209+321261027590909+23126102782809+34126102783609</t>
+        </is>
+      </c>
+      <c r="B67" s="23" t="inlineStr">
+        <is>
+          <t>BAJEL</t>
+        </is>
+      </c>
+      <c r="C67" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D67" s="24" t="n">
+        <v>46322</v>
+      </c>
+      <c r="E67" s="25" t="n">
+        <v>168.7027</v>
+      </c>
+      <c r="F67" s="26" t="n">
+        <v>507</v>
+      </c>
+      <c r="G67" s="24" t="inlineStr"/>
+      <c r="H67" s="25" t="inlineStr"/>
       <c r="I67" s="21">
         <f>IF(OR($B67="",$H67=""),"",IF($C67="LONG",($H67-$E67)*$F67,($E67-$H67)*$F67))</f>
         <v/>
@@ -4839,7 +4865,9 @@
         <f>IF(OR($B67="",$I67="",$E67=0,$F67=0),"",$I67/($E67*$F67))</f>
         <v/>
       </c>
-      <c r="K67" s="4" t="n"/>
+      <c r="K67" s="4" t="n">
+        <v>122.32</v>
+      </c>
       <c r="L67" s="21">
         <f>IF(OR($B67="",$I67=""),"",$I67-IF($K67="",0,$K67))</f>
         <v/>
@@ -4852,17 +4880,39 @@
         <f>IF($B67="","",IF($H67="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O67" s="23" t="n"/>
+      <c r="O67" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="68">
-      <c r="A68" s="23" t="n"/>
-      <c r="B68" s="23" t="n"/>
-      <c r="C68" s="23" t="n"/>
-      <c r="D68" s="24" t="n"/>
-      <c r="E68" s="25" t="n"/>
-      <c r="F68" s="26" t="n"/>
-      <c r="G68" s="24" t="n"/>
-      <c r="H68" s="25" t="n"/>
+      <c r="A68" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261029713009+221261029729209+231261029107809+231261029108409+231261029108509+221261029730909+231261029109609+231261029109809+221261029731809+341261029102409+221261029733009+341261029103009</t>
+        </is>
+      </c>
+      <c r="B68" s="23" t="inlineStr">
+        <is>
+          <t>CNL</t>
+        </is>
+      </c>
+      <c r="C68" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D68" s="24" t="n">
+        <v>46324</v>
+      </c>
+      <c r="E68" s="25" t="n">
+        <v>1214.5775</v>
+      </c>
+      <c r="F68" s="26" t="n">
+        <v>98</v>
+      </c>
+      <c r="G68" s="24" t="inlineStr"/>
+      <c r="H68" s="25" t="inlineStr"/>
       <c r="I68" s="21">
         <f>IF(OR($B68="",$H68=""),"",IF($C68="LONG",($H68-$E68)*$F68,($E68-$H68)*$F68))</f>
         <v/>
@@ -4871,7 +4921,9 @@
         <f>IF(OR($B68="",$I68="",$E68=0,$F68=0),"",$I68/($E68*$F68))</f>
         <v/>
       </c>
-      <c r="K68" s="4" t="n"/>
+      <c r="K68" s="4" t="n">
+        <v>14.75</v>
+      </c>
       <c r="L68" s="21">
         <f>IF(OR($B68="",$I68=""),"",$I68-IF($K68="",0,$K68))</f>
         <v/>
@@ -4884,17 +4936,39 @@
         <f>IF($B68="","",IF($H68="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O68" s="23" t="n"/>
+      <c r="O68" s="23" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
     </row>
     <row r="69">
-      <c r="A69" s="23" t="n"/>
-      <c r="B69" s="23" t="n"/>
-      <c r="C69" s="23" t="n"/>
-      <c r="D69" s="24" t="n"/>
-      <c r="E69" s="25" t="n"/>
-      <c r="F69" s="26" t="n"/>
-      <c r="G69" s="24" t="n"/>
-      <c r="H69" s="25" t="n"/>
+      <c r="A69" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-341261029101409+221261029729309+221261029729809+231261029108209+221261029730609+221261029731009+231261029109509+341261029102109+221261029731909+321261029716409+341261029102909+341261029103109</t>
+        </is>
+      </c>
+      <c r="B69" s="23" t="inlineStr">
+        <is>
+          <t>HUBTOWN</t>
+        </is>
+      </c>
+      <c r="C69" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D69" s="24" t="n">
+        <v>46324</v>
+      </c>
+      <c r="E69" s="25" t="n">
+        <v>182.3842</v>
+      </c>
+      <c r="F69" s="26" t="n">
+        <v>1322</v>
+      </c>
+      <c r="G69" s="24" t="inlineStr"/>
+      <c r="H69" s="25" t="inlineStr"/>
       <c r="I69" s="21">
         <f>IF(OR($B69="",$H69=""),"",IF($C69="LONG",($H69-$E69)*$F69,($E69-$H69)*$F69))</f>
         <v/>
@@ -4903,7 +4977,9 @@
         <f>IF(OR($B69="",$I69="",$E69=0,$F69=0),"",$I69/($E69*$F69))</f>
         <v/>
       </c>
-      <c r="K69" s="4" t="n"/>
+      <c r="K69" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L69" s="21">
         <f>IF(OR($B69="",$I69=""),"",$I69-IF($K69="",0,$K69))</f>
         <v/>
@@ -4916,17 +4992,39 @@
         <f>IF($B69="","",IF($H69="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O69" s="23" t="n"/>
+      <c r="O69" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="70">
-      <c r="A70" s="23" t="n"/>
-      <c r="B70" s="23" t="n"/>
-      <c r="C70" s="23" t="n"/>
-      <c r="D70" s="24" t="n"/>
-      <c r="E70" s="25" t="n"/>
-      <c r="F70" s="26" t="n"/>
-      <c r="G70" s="24" t="n"/>
-      <c r="H70" s="25" t="n"/>
+      <c r="A70" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261029729009+231261029107609+341261029101509+321261029714509+321261029714609+341261029101709+321261029715509+341261029102209+221261029732009+231261029110109+231261029110309+321261029716709</t>
+        </is>
+      </c>
+      <c r="B70" s="23" t="inlineStr">
+        <is>
+          <t>NILKAMAL</t>
+        </is>
+      </c>
+      <c r="C70" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D70" s="24" t="n">
+        <v>46324</v>
+      </c>
+      <c r="E70" s="25" t="n">
+        <v>2005.5798</v>
+      </c>
+      <c r="F70" s="26" t="n">
+        <v>119</v>
+      </c>
+      <c r="G70" s="24" t="inlineStr"/>
+      <c r="H70" s="25" t="inlineStr"/>
       <c r="I70" s="21">
         <f>IF(OR($B70="",$H70=""),"",IF($C70="LONG",($H70-$E70)*$F70,($E70-$H70)*$F70))</f>
         <v/>
@@ -4935,7 +5033,9 @@
         <f>IF(OR($B70="",$I70="",$E70=0,$F70=0),"",$I70/($E70*$F70))</f>
         <v/>
       </c>
-      <c r="K70" s="4" t="n"/>
+      <c r="K70" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L70" s="21">
         <f>IF(OR($B70="",$I70=""),"",$I70-IF($K70="",0,$K70))</f>
         <v/>
@@ -4948,17 +5048,39 @@
         <f>IF($B70="","",IF($H70="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O70" s="23" t="n"/>
+      <c r="O70" s="23" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
     </row>
     <row r="71">
-      <c r="A71" s="23" t="n"/>
-      <c r="B71" s="23" t="n"/>
-      <c r="C71" s="23" t="n"/>
-      <c r="D71" s="24" t="n"/>
-      <c r="E71" s="25" t="n"/>
-      <c r="F71" s="26" t="n"/>
-      <c r="G71" s="24" t="n"/>
-      <c r="H71" s="25" t="n"/>
+      <c r="A71" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-231261029107309+321261029713509+221261029729909+231261029108309+231261029108609+321261029714809+341261029101809+321261029716109+341261029102309+231261029110209+341261029102809+231261029110509+321261029716909</t>
+        </is>
+      </c>
+      <c r="B71" s="23" t="inlineStr">
+        <is>
+          <t>SATIN</t>
+        </is>
+      </c>
+      <c r="C71" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D71" s="24" t="n">
+        <v>46324</v>
+      </c>
+      <c r="E71" s="25" t="n">
+        <v>250.8632</v>
+      </c>
+      <c r="F71" s="26" t="n">
+        <v>956</v>
+      </c>
+      <c r="G71" s="24" t="inlineStr"/>
+      <c r="H71" s="25" t="inlineStr"/>
       <c r="I71" s="21">
         <f>IF(OR($B71="",$H71=""),"",IF($C71="LONG",($H71-$E71)*$F71,($E71-$H71)*$F71))</f>
         <v/>
@@ -4967,7 +5089,9 @@
         <f>IF(OR($B71="",$I71="",$E71=0,$F71=0),"",$I71/($E71*$F71))</f>
         <v/>
       </c>
-      <c r="K71" s="4" t="n"/>
+      <c r="K71" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L71" s="21">
         <f>IF(OR($B71="",$I71=""),"",$I71-IF($K71="",0,$K71))</f>
         <v/>
@@ -4980,7 +5104,11 @@
         <f>IF($B71="","",IF($H71="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O71" s="23" t="n"/>
+      <c r="O71" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="23" t="n"/>
@@ -31481,7 +31609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J55"/>
+  <dimension ref="A1:J59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31651,7 +31779,7 @@
     <row r="6">
       <c r="A6" s="27" t="inlineStr">
         <is>
-          <t>ARFIN</t>
+          <t>APOLLOPIPE</t>
         </is>
       </c>
       <c r="B6" s="20">
@@ -31694,7 +31822,7 @@
     <row r="7">
       <c r="A7" s="27" t="inlineStr">
         <is>
-          <t>BAJEL</t>
+          <t>ARFIN</t>
         </is>
       </c>
       <c r="B7" s="20">
@@ -31737,7 +31865,7 @@
     <row r="8">
       <c r="A8" s="27" t="inlineStr">
         <is>
-          <t>BBL</t>
+          <t>BAJEL</t>
         </is>
       </c>
       <c r="B8" s="20">
@@ -31780,7 +31908,7 @@
     <row r="9">
       <c r="A9" s="27" t="inlineStr">
         <is>
-          <t>BLUSPRING</t>
+          <t>BBL</t>
         </is>
       </c>
       <c r="B9" s="20">
@@ -31823,7 +31951,7 @@
     <row r="10">
       <c r="A10" s="27" t="inlineStr">
         <is>
-          <t>CMLL</t>
+          <t>BLUSPRING</t>
         </is>
       </c>
       <c r="B10" s="20">
@@ -31866,7 +31994,7 @@
     <row r="11">
       <c r="A11" s="27" t="inlineStr">
         <is>
-          <t>DELTACORP</t>
+          <t>CMLL</t>
         </is>
       </c>
       <c r="B11" s="20">
@@ -31909,7 +32037,7 @@
     <row r="12">
       <c r="A12" s="27" t="inlineStr">
         <is>
-          <t>DPABHUSHAN</t>
+          <t>CNL</t>
         </is>
       </c>
       <c r="B12" s="20">
@@ -31952,7 +32080,7 @@
     <row r="13">
       <c r="A13" s="27" t="inlineStr">
         <is>
-          <t>EUROPRATIK</t>
+          <t>DELTACORP</t>
         </is>
       </c>
       <c r="B13" s="20">
@@ -31995,7 +32123,7 @@
     <row r="14">
       <c r="A14" s="27" t="inlineStr">
         <is>
-          <t>FISCHER</t>
+          <t>DPABHUSHAN</t>
         </is>
       </c>
       <c r="B14" s="20">
@@ -32038,7 +32166,7 @@
     <row r="15">
       <c r="A15" s="27" t="inlineStr">
         <is>
-          <t>GOODLUCK</t>
+          <t>EUROPRATIK</t>
         </is>
       </c>
       <c r="B15" s="20">
@@ -32081,7 +32209,7 @@
     <row r="16">
       <c r="A16" s="27" t="inlineStr">
         <is>
-          <t>GPTINFRA</t>
+          <t>FISCHER</t>
         </is>
       </c>
       <c r="B16" s="20">
@@ -32124,7 +32252,7 @@
     <row r="17">
       <c r="A17" s="27" t="inlineStr">
         <is>
-          <t>HATHWAY</t>
+          <t>GOODLUCK</t>
         </is>
       </c>
       <c r="B17" s="20">
@@ -32167,7 +32295,7 @@
     <row r="18">
       <c r="A18" s="27" t="inlineStr">
         <is>
-          <t>INDIAGLYCO</t>
+          <t>GPTINFRA</t>
         </is>
       </c>
       <c r="B18" s="20">
@@ -32210,7 +32338,7 @@
     <row r="19">
       <c r="A19" s="27" t="inlineStr">
         <is>
-          <t>INDOKEM</t>
+          <t>HATHWAY</t>
         </is>
       </c>
       <c r="B19" s="20">
@@ -32253,7 +32381,7 @@
     <row r="20">
       <c r="A20" s="27" t="inlineStr">
         <is>
-          <t>INDOSTAR</t>
+          <t>HUBTOWN</t>
         </is>
       </c>
       <c r="B20" s="20">
@@ -32296,7 +32424,7 @@
     <row r="21">
       <c r="A21" s="27" t="inlineStr">
         <is>
-          <t>INOXGREEN</t>
+          <t>INDIAGLYCO</t>
         </is>
       </c>
       <c r="B21" s="20">
@@ -32339,7 +32467,7 @@
     <row r="22">
       <c r="A22" s="27" t="inlineStr">
         <is>
-          <t>JAICORPLTD</t>
+          <t>INDOKEM</t>
         </is>
       </c>
       <c r="B22" s="20">
@@ -32382,7 +32510,7 @@
     <row r="23">
       <c r="A23" s="27" t="inlineStr">
         <is>
-          <t>JINDALPOLY</t>
+          <t>INDOSTAR</t>
         </is>
       </c>
       <c r="B23" s="20">
@@ -32425,7 +32553,7 @@
     <row r="24">
       <c r="A24" s="27" t="inlineStr">
         <is>
-          <t>JISLJALEQS</t>
+          <t>INOXGREEN</t>
         </is>
       </c>
       <c r="B24" s="20">
@@ -32468,7 +32596,7 @@
     <row r="25">
       <c r="A25" s="27" t="inlineStr">
         <is>
-          <t>KOTIC</t>
+          <t>JAICORPLTD</t>
         </is>
       </c>
       <c r="B25" s="20">
@@ -32511,7 +32639,7 @@
     <row r="26">
       <c r="A26" s="27" t="inlineStr">
         <is>
-          <t>KRISHNADEF</t>
+          <t>JINDALPOLY</t>
         </is>
       </c>
       <c r="B26" s="20">
@@ -32554,7 +32682,7 @@
     <row r="27">
       <c r="A27" s="27" t="inlineStr">
         <is>
-          <t>KROSS</t>
+          <t>JISLJALEQS</t>
         </is>
       </c>
       <c r="B27" s="20">
@@ -32597,7 +32725,7 @@
     <row r="28">
       <c r="A28" s="27" t="inlineStr">
         <is>
-          <t>MAHLOG</t>
+          <t>KOTIC</t>
         </is>
       </c>
       <c r="B28" s="20">
@@ -32640,7 +32768,7 @@
     <row r="29">
       <c r="A29" s="27" t="inlineStr">
         <is>
-          <t>MBEL</t>
+          <t>KRISHNADEF</t>
         </is>
       </c>
       <c r="B29" s="20">
@@ -32683,7 +32811,7 @@
     <row r="30">
       <c r="A30" s="27" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>KROSS</t>
         </is>
       </c>
       <c r="B30" s="20">
@@ -32726,7 +32854,7 @@
     <row r="31">
       <c r="A31" s="27" t="inlineStr">
         <is>
-          <t>MOBIKWIK</t>
+          <t>MAHLOG</t>
         </is>
       </c>
       <c r="B31" s="20">
@@ -32769,7 +32897,7 @@
     <row r="32">
       <c r="A32" s="27" t="inlineStr">
         <is>
-          <t>NIBE</t>
+          <t>MBEL</t>
         </is>
       </c>
       <c r="B32" s="20">
@@ -32812,7 +32940,7 @@
     <row r="33">
       <c r="A33" s="27" t="inlineStr">
         <is>
-          <t>OAL</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="B33" s="20">
@@ -32855,7 +32983,7 @@
     <row r="34">
       <c r="A34" s="27" t="inlineStr">
         <is>
-          <t>ORIENTELEC</t>
+          <t>MOBIKWIK</t>
         </is>
       </c>
       <c r="B34" s="20">
@@ -32898,7 +33026,7 @@
     <row r="35">
       <c r="A35" s="27" t="inlineStr">
         <is>
-          <t>PARACABLES</t>
+          <t>NIBE</t>
         </is>
       </c>
       <c r="B35" s="20">
@@ -32941,7 +33069,7 @@
     <row r="36">
       <c r="A36" s="27" t="inlineStr">
         <is>
-          <t>PIXTRANS</t>
+          <t>NILKAMAL</t>
         </is>
       </c>
       <c r="B36" s="20">
@@ -32984,7 +33112,7 @@
     <row r="37">
       <c r="A37" s="27" t="inlineStr">
         <is>
-          <t>PNCINFRA</t>
+          <t>OAL</t>
         </is>
       </c>
       <c r="B37" s="20">
@@ -33027,7 +33155,7 @@
     <row r="38">
       <c r="A38" s="27" t="inlineStr">
         <is>
-          <t>PNGSREVA</t>
+          <t>ORIENTELEC</t>
         </is>
       </c>
       <c r="B38" s="20">
@@ -33070,7 +33198,7 @@
     <row r="39">
       <c r="A39" s="27" t="inlineStr">
         <is>
-          <t>PRINCEPIPE</t>
+          <t>PARACABLES</t>
         </is>
       </c>
       <c r="B39" s="20">
@@ -33113,7 +33241,7 @@
     <row r="40">
       <c r="A40" s="27" t="inlineStr">
         <is>
-          <t>RSYSTEMS</t>
+          <t>PIXTRANS</t>
         </is>
       </c>
       <c r="B40" s="20">
@@ -33156,7 +33284,7 @@
     <row r="41">
       <c r="A41" s="27" t="inlineStr">
         <is>
-          <t>RUBYMILLS</t>
+          <t>PNCINFRA</t>
         </is>
       </c>
       <c r="B41" s="20">
@@ -33199,7 +33327,7 @@
     <row r="42">
       <c r="A42" s="27" t="inlineStr">
         <is>
-          <t>SAKSOFT</t>
+          <t>PNGSREVA</t>
         </is>
       </c>
       <c r="B42" s="20">
@@ -33242,7 +33370,7 @@
     <row r="43">
       <c r="A43" s="27" t="inlineStr">
         <is>
-          <t>SATIN</t>
+          <t>PRINCEPIPE</t>
         </is>
       </c>
       <c r="B43" s="20">
@@ -33285,7 +33413,7 @@
     <row r="44">
       <c r="A44" s="27" t="inlineStr">
         <is>
-          <t>SGFIN</t>
+          <t>RSYSTEMS</t>
         </is>
       </c>
       <c r="B44" s="20">
@@ -33328,7 +33456,7 @@
     <row r="45">
       <c r="A45" s="27" t="inlineStr">
         <is>
-          <t>SHRINGARMS</t>
+          <t>RUBYMILLS</t>
         </is>
       </c>
       <c r="B45" s="20">
@@ -33371,7 +33499,7 @@
     <row r="46">
       <c r="A46" s="27" t="inlineStr">
         <is>
-          <t>SIMPLEXINF</t>
+          <t>SAKSOFT</t>
         </is>
       </c>
       <c r="B46" s="20">
@@ -33414,7 +33542,7 @@
     <row r="47">
       <c r="A47" s="27" t="inlineStr">
         <is>
-          <t>SMCGLOBAL</t>
+          <t>SATIN</t>
         </is>
       </c>
       <c r="B47" s="20">
@@ -33457,7 +33585,7 @@
     <row r="48">
       <c r="A48" s="27" t="inlineStr">
         <is>
-          <t>SOLARA</t>
+          <t>SGFIN</t>
         </is>
       </c>
       <c r="B48" s="20">
@@ -33500,7 +33628,7 @@
     <row r="49">
       <c r="A49" s="27" t="inlineStr">
         <is>
-          <t>SPORTKING</t>
+          <t>SHRINGARMS</t>
         </is>
       </c>
       <c r="B49" s="20">
@@ -33543,7 +33671,7 @@
     <row r="50">
       <c r="A50" s="27" t="inlineStr">
         <is>
-          <t>SUNCLAY</t>
+          <t>SIMPLEXINF</t>
         </is>
       </c>
       <c r="B50" s="20">
@@ -33586,7 +33714,7 @@
     <row r="51">
       <c r="A51" s="27" t="inlineStr">
         <is>
-          <t>SWARAJENG</t>
+          <t>SMCGLOBAL</t>
         </is>
       </c>
       <c r="B51" s="20">
@@ -33629,7 +33757,7 @@
     <row r="52">
       <c r="A52" s="27" t="inlineStr">
         <is>
-          <t>TEAMLEASE</t>
+          <t>SOLARA</t>
         </is>
       </c>
       <c r="B52" s="20">
@@ -33672,7 +33800,7 @@
     <row r="53">
       <c r="A53" s="27" t="inlineStr">
         <is>
-          <t>YUKEN</t>
+          <t>SPORTKING</t>
         </is>
       </c>
       <c r="B53" s="20">
@@ -33715,7 +33843,7 @@
     <row r="54">
       <c r="A54" s="27" t="inlineStr">
         <is>
-          <t>ZAGGLE</t>
+          <t>SUNCLAY</t>
         </is>
       </c>
       <c r="B54" s="20">
@@ -33756,37 +33884,209 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="3" t="inlineStr">
+      <c r="A55" s="27" t="inlineStr">
+        <is>
+          <t>SWARAJENG</t>
+        </is>
+      </c>
+      <c r="B55" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A55)</f>
+        <v/>
+      </c>
+      <c r="C55" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A55,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D55" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A55,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E55" s="22">
+        <f>IFERROR($C55/$B55,"")</f>
+        <v/>
+      </c>
+      <c r="F55" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A55,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G55" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A55,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H55" s="21">
+        <f>IFERROR($G55/$B55,"")</f>
+        <v/>
+      </c>
+      <c r="I55" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A55),"")</f>
+        <v/>
+      </c>
+      <c r="J55" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A55),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="27" t="inlineStr">
+        <is>
+          <t>TEAMLEASE</t>
+        </is>
+      </c>
+      <c r="B56" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A56)</f>
+        <v/>
+      </c>
+      <c r="C56" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A56,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D56" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A56,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E56" s="22">
+        <f>IFERROR($C56/$B56,"")</f>
+        <v/>
+      </c>
+      <c r="F56" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A56,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G56" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A56,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H56" s="21">
+        <f>IFERROR($G56/$B56,"")</f>
+        <v/>
+      </c>
+      <c r="I56" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A56),"")</f>
+        <v/>
+      </c>
+      <c r="J56" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A56),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="27" t="inlineStr">
+        <is>
+          <t>YUKEN</t>
+        </is>
+      </c>
+      <c r="B57" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A57)</f>
+        <v/>
+      </c>
+      <c r="C57" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A57,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D57" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A57,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E57" s="22">
+        <f>IFERROR($C57/$B57,"")</f>
+        <v/>
+      </c>
+      <c r="F57" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A57,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G57" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A57,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H57" s="21">
+        <f>IFERROR($G57/$B57,"")</f>
+        <v/>
+      </c>
+      <c r="I57" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A57),"")</f>
+        <v/>
+      </c>
+      <c r="J57" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A57),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="27" t="inlineStr">
+        <is>
+          <t>ZAGGLE</t>
+        </is>
+      </c>
+      <c r="B58" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A58)</f>
+        <v/>
+      </c>
+      <c r="C58" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A58,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D58" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A58,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E58" s="22">
+        <f>IFERROR($C58/$B58,"")</f>
+        <v/>
+      </c>
+      <c r="F58" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A58,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G58" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A58,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H58" s="21">
+        <f>IFERROR($G58/$B58,"")</f>
+        <v/>
+      </c>
+      <c r="I58" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A58),"")</f>
+        <v/>
+      </c>
+      <c r="J58" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A58),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B55" s="30">
-        <f>SUM(B4:B54)</f>
-        <v/>
-      </c>
-      <c r="C55" s="30">
-        <f>SUM(C4:C54)</f>
-        <v/>
-      </c>
-      <c r="D55" s="30">
-        <f>SUM(D4:D54)</f>
-        <v/>
-      </c>
-      <c r="E55" s="31">
-        <f>IFERROR(C55/B55,"")</f>
-        <v/>
-      </c>
-      <c r="F55" s="32">
-        <f>SUM(F4:F54)</f>
-        <v/>
-      </c>
-      <c r="G55" s="32">
-        <f>SUM(G4:G54)</f>
-        <v/>
-      </c>
-      <c r="H55" s="32">
-        <f>IFERROR(G55/B55,"")</f>
+      <c r="B59" s="30">
+        <f>SUM(B4:B58)</f>
+        <v/>
+      </c>
+      <c r="C59" s="30">
+        <f>SUM(C4:C58)</f>
+        <v/>
+      </c>
+      <c r="D59" s="30">
+        <f>SUM(D4:D58)</f>
+        <v/>
+      </c>
+      <c r="E59" s="31">
+        <f>IFERROR(C59/B59,"")</f>
+        <v/>
+      </c>
+      <c r="F59" s="32">
+        <f>SUM(F4:F58)</f>
+        <v/>
+      </c>
+      <c r="G59" s="32">
+        <f>SUM(G4:G58)</f>
+        <v/>
+      </c>
+      <c r="H59" s="32">
+        <f>IFERROR(G59/B59,"")</f>
         <v/>
       </c>
     </row>
@@ -33805,7 +34105,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N67"/>
+  <dimension ref="A1:N72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -34056,7 +34356,7 @@
         <v>35.4</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>115.98</v>
+        <v>115.97</v>
       </c>
       <c r="N6" s="21">
         <f>SUM(E6:M6)</f>
@@ -34107,7 +34407,7 @@
         <v>35.4</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>69.34999999999999</v>
+        <v>69.34</v>
       </c>
       <c r="N7" s="21">
         <f>SUM(E7:M7)</f>
@@ -34158,7 +34458,7 @@
         <v>35.4</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>96.5</v>
+        <v>96.48999999999999</v>
       </c>
       <c r="N8" s="21">
         <f>SUM(E8:M8)</f>
@@ -34260,7 +34560,7 @@
         <v>35.4</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>96.51000000000001</v>
+        <v>96.5</v>
       </c>
       <c r="N10" s="21">
         <f>SUM(E10:M10)</f>
@@ -34311,7 +34611,7 @@
         <v>35.4</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>59.51</v>
+        <v>59.5</v>
       </c>
       <c r="N11" s="21">
         <f>SUM(E11:M11)</f>
@@ -34362,7 +34662,7 @@
         <v>35.4</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>71.31999999999999</v>
+        <v>71.31</v>
       </c>
       <c r="N12" s="21">
         <f>SUM(E12:M12)</f>
@@ -34413,7 +34713,7 @@
         <v>35.4</v>
       </c>
       <c r="M13" s="4" t="n">
-        <v>73.01000000000001</v>
+        <v>73.06999999999999</v>
       </c>
       <c r="N13" s="21">
         <f>SUM(E13:M13)</f>
@@ -34464,7 +34764,7 @@
         <v>35.4</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>59.33</v>
+        <v>59.32</v>
       </c>
       <c r="N14" s="21">
         <f>SUM(E14:M14)</f>
@@ -34617,7 +34917,7 @@
         <v>35.4</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>83.31</v>
+        <v>83.29000000000001</v>
       </c>
       <c r="N17" s="21">
         <f>SUM(E17:M17)</f>
@@ -34719,7 +35019,7 @@
         <v>35.4</v>
       </c>
       <c r="M19" s="4" t="n">
-        <v>86.59999999999999</v>
+        <v>86.66</v>
       </c>
       <c r="N19" s="21">
         <f>SUM(E19:M19)</f>
@@ -34770,7 +35070,7 @@
         <v>35.4</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>83.40000000000001</v>
+        <v>83.38</v>
       </c>
       <c r="N20" s="21">
         <f>SUM(E20:M20)</f>
@@ -34872,7 +35172,7 @@
         <v>35.4</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>83.8</v>
+        <v>83.77</v>
       </c>
       <c r="N22" s="21">
         <f>SUM(E22:M22)</f>
@@ -35025,7 +35325,7 @@
         <v>35.4</v>
       </c>
       <c r="M25" s="4" t="n">
-        <v>37.06</v>
+        <v>37.08</v>
       </c>
       <c r="N25" s="21">
         <f>SUM(E25:M25)</f>
@@ -35178,7 +35478,7 @@
         <v>35.4</v>
       </c>
       <c r="M28" s="4" t="n">
-        <v>40.86</v>
+        <v>40.85</v>
       </c>
       <c r="N28" s="21">
         <f>SUM(E28:M28)</f>
@@ -35229,7 +35529,7 @@
         <v>35.4</v>
       </c>
       <c r="M29" s="4" t="n">
-        <v>42.61</v>
+        <v>42.62</v>
       </c>
       <c r="N29" s="21">
         <f>SUM(E29:M29)</f>
@@ -35280,7 +35580,7 @@
         <v>35.4</v>
       </c>
       <c r="M30" s="4" t="n">
-        <v>35.65</v>
+        <v>35.64</v>
       </c>
       <c r="N30" s="21">
         <f>SUM(E30:M30)</f>
@@ -35433,7 +35733,7 @@
         <v>35.4</v>
       </c>
       <c r="M33" s="4" t="n">
-        <v>35.38</v>
+        <v>35.37</v>
       </c>
       <c r="N33" s="21">
         <f>SUM(E33:M33)</f>
@@ -35484,7 +35784,7 @@
         <v>35.4</v>
       </c>
       <c r="M34" s="4" t="n">
-        <v>37.7</v>
+        <v>37.72</v>
       </c>
       <c r="N34" s="21">
         <f>SUM(E34:M34)</f>
@@ -35637,7 +35937,7 @@
         <v>35.4</v>
       </c>
       <c r="M37" s="4" t="n">
-        <v>31.44</v>
+        <v>31.45</v>
       </c>
       <c r="N37" s="21">
         <f>SUM(E37:M37)</f>
@@ -35688,7 +35988,7 @@
         <v>35.4</v>
       </c>
       <c r="M38" s="4" t="n">
-        <v>34.69</v>
+        <v>34.68</v>
       </c>
       <c r="N38" s="21">
         <f>SUM(E38:M38)</f>
@@ -35739,7 +36039,7 @@
         <v>35.4</v>
       </c>
       <c r="M39" s="4" t="n">
-        <v>34.47</v>
+        <v>34.46</v>
       </c>
       <c r="N39" s="21">
         <f>SUM(E39:M39)</f>
@@ -35841,7 +36141,7 @@
         <v>35.4</v>
       </c>
       <c r="M41" s="4" t="n">
-        <v>234.24</v>
+        <v>234.2</v>
       </c>
       <c r="N41" s="21">
         <f>SUM(E41:M41)</f>
@@ -35892,7 +36192,7 @@
         <v>35.4</v>
       </c>
       <c r="M42" s="4" t="n">
-        <v>27.75</v>
+        <v>27.74</v>
       </c>
       <c r="N42" s="21">
         <f>SUM(E42:M42)</f>
@@ -35943,7 +36243,7 @@
         <v>35.4</v>
       </c>
       <c r="M43" s="4" t="n">
-        <v>80.54000000000001</v>
+        <v>80.59</v>
       </c>
       <c r="N43" s="21">
         <f>SUM(E43:M43)</f>
@@ -36045,7 +36345,7 @@
         <v>35.4</v>
       </c>
       <c r="M45" s="4" t="n">
-        <v>85.76000000000001</v>
+        <v>85.79000000000001</v>
       </c>
       <c r="N45" s="21">
         <f>SUM(E45:M45)</f>
@@ -36096,7 +36396,7 @@
         <v>35.4</v>
       </c>
       <c r="M46" s="4" t="n">
-        <v>75.69</v>
+        <v>75.67</v>
       </c>
       <c r="N46" s="21">
         <f>SUM(E46:M46)</f>
@@ -36147,7 +36447,7 @@
         <v>35.4</v>
       </c>
       <c r="M47" s="4" t="n">
-        <v>178.96</v>
+        <v>178.93</v>
       </c>
       <c r="N47" s="21">
         <f>SUM(E47:M47)</f>
@@ -36198,7 +36498,7 @@
         <v>35.4</v>
       </c>
       <c r="M48" s="4" t="n">
-        <v>179.92</v>
+        <v>179.89</v>
       </c>
       <c r="N48" s="21">
         <f>SUM(E48:M48)</f>
@@ -36249,7 +36549,7 @@
         <v>35.4</v>
       </c>
       <c r="M49" s="4" t="n">
-        <v>174.22</v>
+        <v>174.25</v>
       </c>
       <c r="N49" s="21">
         <f>SUM(E49:M49)</f>
@@ -36300,7 +36600,7 @@
         <v>35.4</v>
       </c>
       <c r="M50" s="4" t="n">
-        <v>180.27</v>
+        <v>180.24</v>
       </c>
       <c r="N50" s="21">
         <f>SUM(E50:M50)</f>
@@ -36351,7 +36651,7 @@
         <v>35.4</v>
       </c>
       <c r="M51" s="4" t="n">
-        <v>142.7</v>
+        <v>142.78</v>
       </c>
       <c r="N51" s="21">
         <f>SUM(E51:M51)</f>
@@ -36402,7 +36702,7 @@
         <v>35.4</v>
       </c>
       <c r="M52" s="4" t="n">
-        <v>112.06</v>
+        <v>112.04</v>
       </c>
       <c r="N52" s="21">
         <f>SUM(E52:M52)</f>
@@ -36606,7 +36906,7 @@
         <v>35.4</v>
       </c>
       <c r="M56" s="4" t="n">
-        <v>46.18</v>
+        <v>46.19</v>
       </c>
       <c r="N56" s="21">
         <f>SUM(E56:M56)</f>
@@ -36684,22 +36984,22 @@
         <v>46323</v>
       </c>
       <c r="E58" s="4" t="n">
-        <v>51.55</v>
+        <v>71.55</v>
       </c>
       <c r="F58" s="4" t="n">
-        <v>171.81</v>
+        <v>335.86</v>
       </c>
       <c r="G58" s="4" t="n">
-        <v>5.27</v>
+        <v>10.31</v>
       </c>
       <c r="H58" s="4" t="n">
-        <v>0.17</v>
+        <v>0.34</v>
       </c>
       <c r="I58" s="4" t="n">
         <v>25.77</v>
       </c>
       <c r="J58" s="4" t="n">
-        <v>10.26</v>
+        <v>14.8</v>
       </c>
       <c r="K58" s="4" t="n">
         <v>14.75</v>
@@ -36708,7 +37008,7 @@
         <v>35.4</v>
       </c>
       <c r="M58" s="4" t="n">
-        <v>36.45</v>
+        <v>36.42</v>
       </c>
       <c r="N58" s="21">
         <f>SUM(E58:M58)</f>
@@ -36735,22 +37035,22 @@
         <v>46323</v>
       </c>
       <c r="E59" s="4" t="n">
-        <v>51.24</v>
+        <v>71.23999999999999</v>
       </c>
       <c r="F59" s="4" t="n">
-        <v>170.82</v>
+        <v>341.51</v>
       </c>
       <c r="G59" s="4" t="n">
-        <v>5.24</v>
+        <v>10.48</v>
       </c>
       <c r="H59" s="4" t="n">
-        <v>0.17</v>
+        <v>0.34</v>
       </c>
       <c r="I59" s="4" t="n">
         <v>25.62</v>
       </c>
       <c r="J59" s="4" t="n">
-        <v>10.2</v>
+        <v>14.77</v>
       </c>
       <c r="K59" s="4" t="n">
         <v>14.75</v>
@@ -36759,7 +37059,7 @@
         <v>35.4</v>
       </c>
       <c r="M59" s="4" t="n">
-        <v>37.93</v>
+        <v>37.92</v>
       </c>
       <c r="N59" s="21">
         <f>SUM(E59:M59)</f>
@@ -36786,22 +37086,22 @@
         <v>46323</v>
       </c>
       <c r="E60" s="4" t="n">
-        <v>51.45</v>
+        <v>71.45</v>
       </c>
       <c r="F60" s="4" t="n">
-        <v>171.29</v>
+        <v>339.29</v>
       </c>
       <c r="G60" s="4" t="n">
-        <v>5.26</v>
+        <v>10.41</v>
       </c>
       <c r="H60" s="4" t="n">
-        <v>0.17</v>
+        <v>0.34</v>
       </c>
       <c r="I60" s="4" t="n">
         <v>25.26</v>
       </c>
       <c r="J60" s="4" t="n">
-        <v>10.24</v>
+        <v>14.8</v>
       </c>
       <c r="K60" s="4" t="n">
         <v>14.75</v>
@@ -36810,7 +37110,7 @@
         <v>35.4</v>
       </c>
       <c r="M60" s="4" t="n">
-        <v>36.72</v>
+        <v>36.73</v>
       </c>
       <c r="N60" s="21">
         <f>SUM(E60:M60)</f>
@@ -36837,22 +37137,22 @@
         <v>46323</v>
       </c>
       <c r="E61" s="4" t="n">
-        <v>51.41</v>
+        <v>71.41</v>
       </c>
       <c r="F61" s="4" t="n">
-        <v>171.33</v>
+        <v>339.64</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>5.26</v>
+        <v>10.41</v>
       </c>
       <c r="H61" s="4" t="n">
-        <v>0.17</v>
+        <v>0.34</v>
       </c>
       <c r="I61" s="4" t="n">
         <v>25.7</v>
       </c>
       <c r="J61" s="4" t="n">
-        <v>10.23</v>
+        <v>14.79</v>
       </c>
       <c r="K61" s="4" t="n">
         <v>14.75</v>
@@ -36861,7 +37161,7 @@
         <v>35.4</v>
       </c>
       <c r="M61" s="4" t="n">
-        <v>39.22</v>
+        <v>39.25</v>
       </c>
       <c r="N61" s="21">
         <f>SUM(E61:M61)</f>
@@ -36888,22 +37188,22 @@
         <v>46323</v>
       </c>
       <c r="E62" s="4" t="n">
-        <v>51.28</v>
+        <v>71.28</v>
       </c>
       <c r="F62" s="4" t="n">
-        <v>170.93</v>
+        <v>339.79</v>
       </c>
       <c r="G62" s="4" t="n">
-        <v>5.25</v>
+        <v>10.43</v>
       </c>
       <c r="H62" s="4" t="n">
-        <v>0.17</v>
+        <v>0.34</v>
       </c>
       <c r="I62" s="4" t="n">
         <v>25.64</v>
       </c>
       <c r="J62" s="4" t="n">
-        <v>10.21</v>
+        <v>14.77</v>
       </c>
       <c r="K62" s="4" t="n">
         <v>14.75</v>
@@ -36912,7 +37212,7 @@
         <v>35.4</v>
       </c>
       <c r="M62" s="4" t="n">
-        <v>33.94</v>
+        <v>33.95</v>
       </c>
       <c r="N62" s="21">
         <f>SUM(E62:M62)</f>
@@ -36939,22 +37239,22 @@
         <v>46323</v>
       </c>
       <c r="E63" s="4" t="n">
-        <v>51.38</v>
+        <v>71.38</v>
       </c>
       <c r="F63" s="4" t="n">
-        <v>171.2</v>
+        <v>337.56</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>5.26</v>
+        <v>10.36</v>
       </c>
       <c r="H63" s="4" t="n">
-        <v>0.17</v>
+        <v>0.34</v>
       </c>
       <c r="I63" s="4" t="n">
         <v>25.68</v>
       </c>
       <c r="J63" s="4" t="n">
-        <v>10.23</v>
+        <v>14.77</v>
       </c>
       <c r="K63" s="4" t="n">
         <v>14.75</v>
@@ -36963,7 +37263,7 @@
         <v>35.4</v>
       </c>
       <c r="M63" s="4" t="n">
-        <v>34.53</v>
+        <v>34.56</v>
       </c>
       <c r="N63" s="21">
         <f>SUM(E63:M63)</f>
@@ -36986,24 +37286,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D64" s="24" t="inlineStr"/>
+      <c r="D64" s="24" t="n">
+        <v>46324</v>
+      </c>
       <c r="E64" s="4" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="F64" s="4" t="n">
-        <v>0</v>
+        <v>300.01</v>
       </c>
       <c r="G64" s="4" t="n">
-        <v>0</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="H64" s="4" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="I64" s="4" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="J64" s="4" t="n">
-        <v>0</v>
+        <v>17.91</v>
       </c>
       <c r="K64" s="4" t="n">
         <v>14.75</v>
@@ -37012,7 +37314,7 @@
         <v>35.4</v>
       </c>
       <c r="M64" s="4" t="n">
-        <v>0</v>
+        <v>70.06</v>
       </c>
       <c r="N64" s="21">
         <f>SUM(E64:M64)</f>
@@ -37022,12 +37324,12 @@
     <row r="65">
       <c r="A65" s="23" t="inlineStr">
         <is>
-          <t>DHAN-23126102780509+34126102781309+23126102781009+23126102781209+221261027605909+34126102781909+321261027588609+23126102781809+321261027589309+23126102782209+321261027590909+23126102782809+34126102783609</t>
+          <t>DHAN-2212610281025009+3212610281009509+3212610281010309+231261028103709+2212610281026009+2212610281026209+2212610281026509+341261028101709+231261028103909+341261028101809+341261028102009+341261028102209+231261028104209+231261028104309+231261028104409+3212610281012909</t>
         </is>
       </c>
       <c r="B65" s="23" t="inlineStr">
         <is>
-          <t>BAJEL</t>
+          <t>PNGSREVA</t>
         </is>
       </c>
       <c r="C65" s="23" t="inlineStr">
@@ -37035,33 +37337,35 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D65" s="24" t="inlineStr"/>
+      <c r="D65" s="24" t="n">
+        <v>46324</v>
+      </c>
       <c r="E65" s="4" t="n">
-        <v>0</v>
+        <v>90.23</v>
       </c>
       <c r="F65" s="4" t="n">
-        <v>90.59</v>
+        <v>300.72</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>2.78</v>
+        <v>9.23</v>
       </c>
       <c r="H65" s="4" t="n">
-        <v>0.09</v>
+        <v>0.3</v>
       </c>
       <c r="I65" s="4" t="n">
-        <v>13.59</v>
+        <v>45</v>
       </c>
       <c r="J65" s="4" t="n">
-        <v>0.52</v>
+        <v>17.96</v>
       </c>
       <c r="K65" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L65" s="4" t="n">
-        <v>0</v>
+        <v>35.4</v>
       </c>
       <c r="M65" s="4" t="n">
-        <v>0</v>
+        <v>51.42</v>
       </c>
       <c r="N65" s="21">
         <f>SUM(E65:M65)</f>
@@ -37071,12 +37375,12 @@
     <row r="66">
       <c r="A66" s="23" t="inlineStr">
         <is>
-          <t>DHAN-2212610281025009+3212610281009509+3212610281010309+231261028103709+2212610281026009+2212610281026209+2212610281026509+341261028101709+231261028103909+341261028101809+341261028102009+341261028102209+231261028104209+231261028104309+231261028104409+3212610281012909</t>
+          <t>DHAN-231261029107209+321261029713609+221261029729709+341261029101609+221261029730509+231261029108709+341261029101909+231261029109909+321261029716309+341261029102509+221261029732909+231261029110409+231261029110609</t>
         </is>
       </c>
       <c r="B66" s="23" t="inlineStr">
         <is>
-          <t>PNGSREVA</t>
+          <t>APOLLOPIPE</t>
         </is>
       </c>
       <c r="C66" s="23" t="inlineStr">
@@ -37118,54 +37422,299 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="3" t="inlineStr">
+      <c r="A67" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126102780509+34126102781309+23126102781009+23126102781209+221261027605909+34126102781909+321261027588609+23126102781809+321261027589309+23126102782209+321261027590909+23126102782809+34126102783609</t>
+        </is>
+      </c>
+      <c r="B67" s="23" t="inlineStr">
+        <is>
+          <t>BAJEL</t>
+        </is>
+      </c>
+      <c r="C67" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D67" s="24" t="inlineStr"/>
+      <c r="E67" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F67" s="4" t="n">
+        <v>90.59</v>
+      </c>
+      <c r="G67" s="4" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="H67" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="I67" s="4" t="n">
+        <v>13.59</v>
+      </c>
+      <c r="J67" s="4" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="K67" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L67" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M67" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N67" s="21">
+        <f>SUM(E67:M67)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261029713009+221261029729209+231261029107809+231261029108409+231261029108509+221261029730909+231261029109609+231261029109809+221261029731809+341261029102409+221261029733009+341261029103009</t>
+        </is>
+      </c>
+      <c r="B68" s="23" t="inlineStr">
+        <is>
+          <t>CNL</t>
+        </is>
+      </c>
+      <c r="C68" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D68" s="24" t="inlineStr"/>
+      <c r="E68" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F68" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I68" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J68" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K68" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L68" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M68" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N68" s="21">
+        <f>SUM(E68:M68)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-341261029101409+221261029729309+221261029729809+231261029108209+221261029730609+221261029731009+231261029109509+341261029102109+221261029731909+321261029716409+341261029102909+341261029103109</t>
+        </is>
+      </c>
+      <c r="B69" s="23" t="inlineStr">
+        <is>
+          <t>HUBTOWN</t>
+        </is>
+      </c>
+      <c r="C69" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D69" s="24" t="inlineStr"/>
+      <c r="E69" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G69" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H69" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I69" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J69" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K69" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L69" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M69" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N69" s="21">
+        <f>SUM(E69:M69)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261029729009+231261029107609+341261029101509+321261029714509+321261029714609+341261029101709+321261029715509+341261029102209+221261029732009+231261029110109+231261029110309+321261029716709</t>
+        </is>
+      </c>
+      <c r="B70" s="23" t="inlineStr">
+        <is>
+          <t>NILKAMAL</t>
+        </is>
+      </c>
+      <c r="C70" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D70" s="24" t="inlineStr"/>
+      <c r="E70" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F70" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G70" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I70" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J70" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K70" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L70" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M70" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N70" s="21">
+        <f>SUM(E70:M70)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-231261029107309+321261029713509+221261029729909+231261029108309+231261029108609+321261029714809+341261029101809+321261029716109+341261029102309+231261029110209+341261029102809+231261029110509+321261029716909</t>
+        </is>
+      </c>
+      <c r="B71" s="23" t="inlineStr">
+        <is>
+          <t>SATIN</t>
+        </is>
+      </c>
+      <c r="C71" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D71" s="24" t="inlineStr"/>
+      <c r="E71" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F71" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G71" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H71" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I71" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J71" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K71" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L71" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M71" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N71" s="21">
+        <f>SUM(E71:M71)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E67" s="32">
-        <f>SUM(E4:E66)</f>
-        <v/>
-      </c>
-      <c r="F67" s="32">
-        <f>SUM(F4:F66)</f>
-        <v/>
-      </c>
-      <c r="G67" s="32">
-        <f>SUM(G4:G66)</f>
-        <v/>
-      </c>
-      <c r="H67" s="32">
-        <f>SUM(H4:H66)</f>
-        <v/>
-      </c>
-      <c r="I67" s="32">
-        <f>SUM(I4:I66)</f>
-        <v/>
-      </c>
-      <c r="J67" s="32">
-        <f>SUM(J4:J66)</f>
-        <v/>
-      </c>
-      <c r="K67" s="32">
-        <f>SUM(K4:K66)</f>
-        <v/>
-      </c>
-      <c r="L67" s="32">
-        <f>SUM(L4:L66)</f>
-        <v/>
-      </c>
-      <c r="M67" s="32">
-        <f>SUM(M4:M66)</f>
-        <v/>
-      </c>
-      <c r="N67" s="32">
-        <f>SUM(N4:N66)</f>
+      <c r="E72" s="32">
+        <f>SUM(E4:E71)</f>
+        <v/>
+      </c>
+      <c r="F72" s="32">
+        <f>SUM(F4:F71)</f>
+        <v/>
+      </c>
+      <c r="G72" s="32">
+        <f>SUM(G4:G71)</f>
+        <v/>
+      </c>
+      <c r="H72" s="32">
+        <f>SUM(H4:H71)</f>
+        <v/>
+      </c>
+      <c r="I72" s="32">
+        <f>SUM(I4:I71)</f>
+        <v/>
+      </c>
+      <c r="J72" s="32">
+        <f>SUM(J4:J71)</f>
+        <v/>
+      </c>
+      <c r="K72" s="32">
+        <f>SUM(K4:K71)</f>
+        <v/>
+      </c>
+      <c r="L72" s="32">
+        <f>SUM(L4:L71)</f>
+        <v/>
+      </c>
+      <c r="M72" s="32">
+        <f>SUM(M4:M71)</f>
+        <v/>
+      </c>
+      <c r="N72" s="32">
+        <f>SUM(N4:N71)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:N66"/>
+  <autoFilter ref="A3:N71"/>
   <mergeCells count="2">
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>

</xml_diff>

<commit_message>
Data update — 2026-10-30 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_oct2026.xlsx
+++ b/results/strategy_pnl_oct2026.xlsx
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trade Log'!$A$3:$O$503</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$76</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1394,7 +1394,7 @@
         <v/>
       </c>
       <c r="K9" s="4" t="n">
-        <v>969.46</v>
+        <v>969.45</v>
       </c>
       <c r="L9" s="21">
         <f>IF(OR($B9="",$I9=""),"",$I9-IF($K9="",0,$K9))</f>
@@ -1634,7 +1634,7 @@
         <v/>
       </c>
       <c r="K13" s="4" t="n">
-        <v>688.04</v>
+        <v>688.09</v>
       </c>
       <c r="L13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($K13="",0,$K13))</f>
@@ -1994,7 +1994,7 @@
         <v/>
       </c>
       <c r="K19" s="4" t="n">
-        <v>666.85</v>
+        <v>666.92</v>
       </c>
       <c r="L19" s="21">
         <f>IF(OR($B19="",$I19=""),"",$I19-IF($K19="",0,$K19))</f>
@@ -2054,7 +2054,7 @@
         <v/>
       </c>
       <c r="K20" s="4" t="n">
-        <v>676.83</v>
+        <v>676.84</v>
       </c>
       <c r="L20" s="21">
         <f>IF(OR($B20="",$I20=""),"",$I20-IF($K20="",0,$K20))</f>
@@ -2354,7 +2354,7 @@
         <v/>
       </c>
       <c r="K25" s="4" t="n">
-        <v>557.28</v>
+        <v>557.09</v>
       </c>
       <c r="L25" s="21">
         <f>IF(OR($B25="",$I25=""),"",$I25-IF($K25="",0,$K25))</f>
@@ -2594,7 +2594,7 @@
         <v/>
       </c>
       <c r="K29" s="4" t="n">
-        <v>554.62</v>
+        <v>554.63</v>
       </c>
       <c r="L29" s="21">
         <f>IF(OR($B29="",$I29=""),"",$I29-IF($K29="",0,$K29))</f>
@@ -2654,7 +2654,7 @@
         <v/>
       </c>
       <c r="K30" s="4" t="n">
-        <v>550.6799999999999</v>
+        <v>550.6900000000001</v>
       </c>
       <c r="L30" s="21">
         <f>IF(OR($B30="",$I30=""),"",$I30-IF($K30="",0,$K30))</f>
@@ -2894,7 +2894,7 @@
         <v/>
       </c>
       <c r="K34" s="4" t="n">
-        <v>426.03</v>
+        <v>426.06</v>
       </c>
       <c r="L34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($K34="",0,$K34))</f>
@@ -3074,7 +3074,7 @@
         <v/>
       </c>
       <c r="K37" s="4" t="n">
-        <v>477.9</v>
+        <v>477.93</v>
       </c>
       <c r="L37" s="21">
         <f>IF(OR($B37="",$I37=""),"",$I37-IF($K37="",0,$K37))</f>
@@ -3314,7 +3314,7 @@
         <v/>
       </c>
       <c r="K41" s="4" t="n">
-        <v>592.37</v>
+        <v>592.35</v>
       </c>
       <c r="L41" s="21">
         <f>IF(OR($B41="",$I41=""),"",$I41-IF($K41="",0,$K41))</f>
@@ -3434,7 +3434,7 @@
         <v/>
       </c>
       <c r="K43" s="4" t="n">
-        <v>924.6900000000001</v>
+        <v>924.72</v>
       </c>
       <c r="L43" s="21">
         <f>IF(OR($B43="",$I43=""),"",$I43-IF($K43="",0,$K43))</f>
@@ -3554,7 +3554,7 @@
         <v/>
       </c>
       <c r="K45" s="4" t="n">
-        <v>945.96</v>
+        <v>945.98</v>
       </c>
       <c r="L45" s="21">
         <f>IF(OR($B45="",$I45=""),"",$I45-IF($K45="",0,$K45))</f>
@@ -3614,7 +3614,7 @@
         <v/>
       </c>
       <c r="K46" s="4" t="n">
-        <v>915.88</v>
+        <v>915.87</v>
       </c>
       <c r="L46" s="21">
         <f>IF(OR($B46="",$I46=""),"",$I46-IF($K46="",0,$K46))</f>
@@ -3674,7 +3674,7 @@
         <v/>
       </c>
       <c r="K47" s="4" t="n">
-        <v>1026.96</v>
+        <v>1026.94</v>
       </c>
       <c r="L47" s="21">
         <f>IF(OR($B47="",$I47=""),"",$I47-IF($K47="",0,$K47))</f>
@@ -3734,7 +3734,7 @@
         <v/>
       </c>
       <c r="K48" s="4" t="n">
-        <v>1028.65</v>
+        <v>1028.63</v>
       </c>
       <c r="L48" s="21">
         <f>IF(OR($B48="",$I48=""),"",$I48-IF($K48="",0,$K48))</f>
@@ -3854,7 +3854,7 @@
         <v/>
       </c>
       <c r="K50" s="4" t="n">
-        <v>1035.35</v>
+        <v>1035.33</v>
       </c>
       <c r="L50" s="21">
         <f>IF(OR($B50="",$I50=""),"",$I50-IF($K50="",0,$K50))</f>
@@ -3914,7 +3914,7 @@
         <v/>
       </c>
       <c r="K51" s="4" t="n">
-        <v>984.84</v>
+        <v>984.88</v>
       </c>
       <c r="L51" s="21">
         <f>IF(OR($B51="",$I51=""),"",$I51-IF($K51="",0,$K51))</f>
@@ -3974,7 +3974,7 @@
         <v/>
       </c>
       <c r="K52" s="4" t="n">
-        <v>940</v>
+        <v>939.99</v>
       </c>
       <c r="L52" s="21">
         <f>IF(OR($B52="",$I52=""),"",$I52-IF($K52="",0,$K52))</f>
@@ -4214,7 +4214,7 @@
         <v/>
       </c>
       <c r="K56" s="4" t="n">
-        <v>875.27</v>
+        <v>875.3099999999999</v>
       </c>
       <c r="L56" s="21">
         <f>IF(OR($B56="",$I56=""),"",$I56-IF($K56="",0,$K56))</f>
@@ -4334,7 +4334,7 @@
         <v/>
       </c>
       <c r="K58" s="4" t="n">
-        <v>545.2</v>
+        <v>545.0599999999999</v>
       </c>
       <c r="L58" s="21">
         <f>IF(OR($B58="",$I58=""),"",$I58-IF($K58="",0,$K58))</f>
@@ -4514,7 +4514,7 @@
         <v/>
       </c>
       <c r="K61" s="4" t="n">
-        <v>551.7</v>
+        <v>551.71</v>
       </c>
       <c r="L61" s="21">
         <f>IF(OR($B61="",$I61=""),"",$I61-IF($K61="",0,$K61))</f>
@@ -4574,7 +4574,7 @@
         <v/>
       </c>
       <c r="K62" s="4" t="n">
-        <v>546.35</v>
+        <v>546.36</v>
       </c>
       <c r="L62" s="21">
         <f>IF(OR($B62="",$I62=""),"",$I62-IF($K62="",0,$K62))</f>
@@ -4634,7 +4634,7 @@
         <v/>
       </c>
       <c r="K63" s="4" t="n">
-        <v>544.8</v>
+        <v>544.84</v>
       </c>
       <c r="L63" s="21">
         <f>IF(OR($B63="",$I63=""),"",$I63-IF($K63="",0,$K63))</f>
@@ -4694,7 +4694,7 @@
         <v/>
       </c>
       <c r="K64" s="4" t="n">
-        <v>582.64</v>
+        <v>917.89</v>
       </c>
       <c r="L64" s="21">
         <f>IF(OR($B64="",$I64=""),"",$I64-IF($K64="",0,$K64))</f>
@@ -4754,7 +4754,7 @@
         <v/>
       </c>
       <c r="K65" s="4" t="n">
-        <v>565.01</v>
+        <v>906.04</v>
       </c>
       <c r="L65" s="21">
         <f>IF(OR($B65="",$I65=""),"",$I65-IF($K65="",0,$K65))</f>
@@ -4799,8 +4799,12 @@
       <c r="F66" s="26" t="n">
         <v>435</v>
       </c>
-      <c r="G66" s="24" t="inlineStr"/>
-      <c r="H66" s="25" t="inlineStr"/>
+      <c r="G66" s="24" t="n">
+        <v>46325</v>
+      </c>
+      <c r="H66" s="25" t="n">
+        <v>516.63</v>
+      </c>
       <c r="I66" s="21">
         <f>IF(OR($B66="",$H66=""),"",IF($C66="LONG",($H66-$E66)*$F66,($E66-$H66)*$F66))</f>
         <v/>
@@ -4810,7 +4814,7 @@
         <v/>
       </c>
       <c r="K66" s="4" t="n">
-        <v>50.15</v>
+        <v>468.99</v>
       </c>
       <c r="L66" s="21">
         <f>IF(OR($B66="",$I66=""),"",$I66-IF($K66="",0,$K66))</f>
@@ -4833,12 +4837,12 @@
     <row r="67">
       <c r="A67" s="23" t="inlineStr">
         <is>
-          <t>DHAN-23126102780509+34126102781309+23126102781009+23126102781209+221261027605909+34126102781909+321261027588609+23126102781809+321261027589309+23126102782209+321261027590909+23126102782809+34126102783609</t>
+          <t>DHAN-321261029713009+221261029729209+231261029107809+231261029108409+231261029108509+221261029730909+231261029109609+231261029109809+221261029731809+341261029102409+221261029733009+341261029103009</t>
         </is>
       </c>
       <c r="B67" s="23" t="inlineStr">
         <is>
-          <t>BAJEL</t>
+          <t>CNL</t>
         </is>
       </c>
       <c r="C67" s="23" t="inlineStr">
@@ -4847,16 +4851,20 @@
         </is>
       </c>
       <c r="D67" s="24" t="n">
-        <v>46322</v>
+        <v>46324</v>
       </c>
       <c r="E67" s="25" t="n">
-        <v>168.7027</v>
+        <v>1214.5775</v>
       </c>
       <c r="F67" s="26" t="n">
-        <v>507</v>
-      </c>
-      <c r="G67" s="24" t="inlineStr"/>
-      <c r="H67" s="25" t="inlineStr"/>
+        <v>98</v>
+      </c>
+      <c r="G67" s="24" t="n">
+        <v>46325</v>
+      </c>
+      <c r="H67" s="25" t="n">
+        <v>1231.05</v>
+      </c>
       <c r="I67" s="21">
         <f>IF(OR($B67="",$H67=""),"",IF($C67="LONG",($H67-$E67)*$F67,($E67-$H67)*$F67))</f>
         <v/>
@@ -4866,7 +4874,7 @@
         <v/>
       </c>
       <c r="K67" s="4" t="n">
-        <v>122.32</v>
+        <v>156.08</v>
       </c>
       <c r="L67" s="21">
         <f>IF(OR($B67="",$I67=""),"",$I67-IF($K67="",0,$K67))</f>
@@ -4882,19 +4890,19 @@
       </c>
       <c r="O67" s="23" t="inlineStr">
         <is>
-          <t>5-10</t>
+          <t>10-15</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261029713009+221261029729209+231261029107809+231261029108409+231261029108509+221261029730909+231261029109609+231261029109809+221261029731809+341261029102409+221261029733009+341261029103009</t>
+          <t>DHAN-341261029101409+221261029729309+221261029729809+231261029108209+221261029730609+221261029731009+231261029109509+341261029102109+221261029731909+321261029716409+341261029102909+341261029103109</t>
         </is>
       </c>
       <c r="B68" s="23" t="inlineStr">
         <is>
-          <t>CNL</t>
+          <t>HUBTOWN</t>
         </is>
       </c>
       <c r="C68" s="23" t="inlineStr">
@@ -4906,13 +4914,17 @@
         <v>46324</v>
       </c>
       <c r="E68" s="25" t="n">
-        <v>1214.5775</v>
+        <v>182.3842</v>
       </c>
       <c r="F68" s="26" t="n">
-        <v>98</v>
-      </c>
-      <c r="G68" s="24" t="inlineStr"/>
-      <c r="H68" s="25" t="inlineStr"/>
+        <v>1322</v>
+      </c>
+      <c r="G68" s="24" t="n">
+        <v>46325</v>
+      </c>
+      <c r="H68" s="25" t="n">
+        <v>188.42</v>
+      </c>
       <c r="I68" s="21">
         <f>IF(OR($B68="",$H68=""),"",IF($C68="LONG",($H68-$E68)*$F68,($E68-$H68)*$F68))</f>
         <v/>
@@ -4922,7 +4934,7 @@
         <v/>
       </c>
       <c r="K68" s="4" t="n">
-        <v>14.75</v>
+        <v>471.51</v>
       </c>
       <c r="L68" s="21">
         <f>IF(OR($B68="",$I68=""),"",$I68-IF($K68="",0,$K68))</f>
@@ -4938,14 +4950,14 @@
       </c>
       <c r="O68" s="23" t="inlineStr">
         <is>
-          <t>10-15</t>
+          <t>5-10</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="23" t="inlineStr">
         <is>
-          <t>DHAN-341261029101409+221261029729309+221261029729809+231261029108209+221261029730609+221261029731009+231261029109509+341261029102109+221261029731909+321261029716409+341261029102909+341261029103109</t>
+          <t>DHAN-23126103014009</t>
         </is>
       </c>
       <c r="B69" s="23" t="inlineStr">
@@ -4955,20 +4967,24 @@
       </c>
       <c r="C69" s="23" t="inlineStr">
         <is>
-          <t>LONG</t>
+          <t>SHORT</t>
         </is>
       </c>
       <c r="D69" s="24" t="n">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="E69" s="25" t="n">
-        <v>182.3842</v>
+        <v>188.42</v>
       </c>
       <c r="F69" s="26" t="n">
         <v>1322</v>
       </c>
-      <c r="G69" s="24" t="inlineStr"/>
-      <c r="H69" s="25" t="inlineStr"/>
+      <c r="G69" s="24" t="n">
+        <v>46325</v>
+      </c>
+      <c r="H69" s="25" t="n">
+        <v>179</v>
+      </c>
       <c r="I69" s="21">
         <f>IF(OR($B69="",$H69=""),"",IF($C69="LONG",($H69-$E69)*$F69,($E69-$H69)*$F69))</f>
         <v/>
@@ -4978,7 +4994,7 @@
         <v/>
       </c>
       <c r="K69" s="4" t="n">
-        <v>50.15</v>
+        <v>0</v>
       </c>
       <c r="L69" s="21">
         <f>IF(OR($B69="",$I69=""),"",$I69-IF($K69="",0,$K69))</f>
@@ -5023,8 +5039,12 @@
       <c r="F70" s="26" t="n">
         <v>119</v>
       </c>
-      <c r="G70" s="24" t="inlineStr"/>
-      <c r="H70" s="25" t="inlineStr"/>
+      <c r="G70" s="24" t="n">
+        <v>46325</v>
+      </c>
+      <c r="H70" s="25" t="n">
+        <v>1955.18</v>
+      </c>
       <c r="I70" s="21">
         <f>IF(OR($B70="",$H70=""),"",IF($C70="LONG",($H70-$E70)*$F70,($E70-$H70)*$F70))</f>
         <v/>
@@ -5034,7 +5054,7 @@
         <v/>
       </c>
       <c r="K70" s="4" t="n">
-        <v>50.15</v>
+        <v>458.81</v>
       </c>
       <c r="L70" s="21">
         <f>IF(OR($B70="",$I70=""),"",$I70-IF($K70="",0,$K70))</f>
@@ -5079,8 +5099,12 @@
       <c r="F71" s="26" t="n">
         <v>956</v>
       </c>
-      <c r="G71" s="24" t="inlineStr"/>
-      <c r="H71" s="25" t="inlineStr"/>
+      <c r="G71" s="24" t="n">
+        <v>46325</v>
+      </c>
+      <c r="H71" s="25" t="n">
+        <v>237.47</v>
+      </c>
       <c r="I71" s="21">
         <f>IF(OR($B71="",$H71=""),"",IF($C71="LONG",($H71-$E71)*$F71,($E71-$H71)*$F71))</f>
         <v/>
@@ -5090,7 +5114,7 @@
         <v/>
       </c>
       <c r="K71" s="4" t="n">
-        <v>50.15</v>
+        <v>468.98</v>
       </c>
       <c r="L71" s="21">
         <f>IF(OR($B71="",$I71=""),"",$I71-IF($K71="",0,$K71))</f>
@@ -5111,14 +5135,32 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="23" t="n"/>
-      <c r="B72" s="23" t="n"/>
-      <c r="C72" s="23" t="n"/>
-      <c r="D72" s="24" t="n"/>
-      <c r="E72" s="25" t="n"/>
-      <c r="F72" s="26" t="n"/>
-      <c r="G72" s="24" t="n"/>
-      <c r="H72" s="25" t="n"/>
+      <c r="A72" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126102780509+34126102781309+23126102781009+23126102781209+221261027605909+34126102781909+321261027588609+23126102781809+321261027589309+23126102782209+321261027590909+23126102782809+34126102783609</t>
+        </is>
+      </c>
+      <c r="B72" s="23" t="inlineStr">
+        <is>
+          <t>BAJEL</t>
+        </is>
+      </c>
+      <c r="C72" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D72" s="24" t="n">
+        <v>46322</v>
+      </c>
+      <c r="E72" s="25" t="n">
+        <v>168.7027</v>
+      </c>
+      <c r="F72" s="26" t="n">
+        <v>507</v>
+      </c>
+      <c r="G72" s="24" t="inlineStr"/>
+      <c r="H72" s="25" t="inlineStr"/>
       <c r="I72" s="21">
         <f>IF(OR($B72="",$H72=""),"",IF($C72="LONG",($H72-$E72)*$F72,($E72-$H72)*$F72))</f>
         <v/>
@@ -5127,7 +5169,9 @@
         <f>IF(OR($B72="",$I72="",$E72=0,$F72=0),"",$I72/($E72*$F72))</f>
         <v/>
       </c>
-      <c r="K72" s="4" t="n"/>
+      <c r="K72" s="4" t="n">
+        <v>122.32</v>
+      </c>
       <c r="L72" s="21">
         <f>IF(OR($B72="",$I72=""),"",$I72-IF($K72="",0,$K72))</f>
         <v/>
@@ -5140,17 +5184,39 @@
         <f>IF($B72="","",IF($H72="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O72" s="23" t="n"/>
+      <c r="O72" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="73">
-      <c r="A73" s="23" t="n"/>
-      <c r="B73" s="23" t="n"/>
-      <c r="C73" s="23" t="n"/>
-      <c r="D73" s="24" t="n"/>
-      <c r="E73" s="25" t="n"/>
-      <c r="F73" s="26" t="n"/>
-      <c r="G73" s="24" t="n"/>
-      <c r="H73" s="25" t="n"/>
+      <c r="A73" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261030639109+231261030110409+321261030624409+221261030640409+341261030103309+341261030103509+321261030625509+221261030641609+231261030111009+221261030642209+341261030103909+341261030104009</t>
+        </is>
+      </c>
+      <c r="B73" s="23" t="inlineStr">
+        <is>
+          <t>DHANUKA</t>
+        </is>
+      </c>
+      <c r="C73" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D73" s="24" t="n">
+        <v>46325</v>
+      </c>
+      <c r="E73" s="25" t="n">
+        <v>974.2136</v>
+      </c>
+      <c r="F73" s="26" t="n">
+        <v>246</v>
+      </c>
+      <c r="G73" s="24" t="inlineStr"/>
+      <c r="H73" s="25" t="inlineStr"/>
       <c r="I73" s="21">
         <f>IF(OR($B73="",$H73=""),"",IF($C73="LONG",($H73-$E73)*$F73,($E73-$H73)*$F73))</f>
         <v/>
@@ -5159,7 +5225,9 @@
         <f>IF(OR($B73="",$I73="",$E73=0,$F73=0),"",$I73/($E73*$F73))</f>
         <v/>
       </c>
-      <c r="K73" s="4" t="n"/>
+      <c r="K73" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L73" s="21">
         <f>IF(OR($B73="",$I73=""),"",$I73-IF($K73="",0,$K73))</f>
         <v/>
@@ -5172,17 +5240,39 @@
         <f>IF($B73="","",IF($H73="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O73" s="23" t="n"/>
+      <c r="O73" s="23" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
     </row>
     <row r="74">
-      <c r="A74" s="23" t="n"/>
-      <c r="B74" s="23" t="n"/>
-      <c r="C74" s="23" t="n"/>
-      <c r="D74" s="24" t="n"/>
-      <c r="E74" s="25" t="n"/>
-      <c r="F74" s="26" t="n"/>
-      <c r="G74" s="24" t="n"/>
-      <c r="H74" s="25" t="n"/>
+      <c r="A74" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-231261030110209+221261030639609+231261030110509+221261030640509+231261030110709+231261030110809+231261030110909+221261030641709+341261030103709+321261030626409+221261030643009</t>
+        </is>
+      </c>
+      <c r="B74" s="23" t="inlineStr">
+        <is>
+          <t>GREAVESCOT</t>
+        </is>
+      </c>
+      <c r="C74" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D74" s="24" t="n">
+        <v>46325</v>
+      </c>
+      <c r="E74" s="25" t="n">
+        <v>199.451</v>
+      </c>
+      <c r="F74" s="26" t="n">
+        <v>1201</v>
+      </c>
+      <c r="G74" s="24" t="inlineStr"/>
+      <c r="H74" s="25" t="inlineStr"/>
       <c r="I74" s="21">
         <f>IF(OR($B74="",$H74=""),"",IF($C74="LONG",($H74-$E74)*$F74,($E74-$H74)*$F74))</f>
         <v/>
@@ -5191,7 +5281,9 @@
         <f>IF(OR($B74="",$I74="",$E74=0,$F74=0),"",$I74/($E74*$F74))</f>
         <v/>
       </c>
-      <c r="K74" s="4" t="n"/>
+      <c r="K74" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L74" s="21">
         <f>IF(OR($B74="",$I74=""),"",$I74-IF($K74="",0,$K74))</f>
         <v/>
@@ -5204,17 +5296,39 @@
         <f>IF($B74="","",IF($H74="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O74" s="23" t="n"/>
+      <c r="O74" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="75">
-      <c r="A75" s="23" t="n"/>
-      <c r="B75" s="23" t="n"/>
-      <c r="C75" s="23" t="n"/>
-      <c r="D75" s="24" t="n"/>
-      <c r="E75" s="25" t="n"/>
-      <c r="F75" s="26" t="n"/>
-      <c r="G75" s="24" t="n"/>
-      <c r="H75" s="25" t="n"/>
+      <c r="A75" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261030639209+341261030103109+221261030639909+231261030110609+341261030103409+321261030625109+341261030103609+231261030111109+231261030111209+221261030643109+221261030643409+221261030643809+321261030628009+221261030644509</t>
+        </is>
+      </c>
+      <c r="B75" s="23" t="inlineStr">
+        <is>
+          <t>JISLJALEQS</t>
+        </is>
+      </c>
+      <c r="C75" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D75" s="24" t="n">
+        <v>46325</v>
+      </c>
+      <c r="E75" s="25" t="n">
+        <v>28.4477</v>
+      </c>
+      <c r="F75" s="26" t="n">
+        <v>8421</v>
+      </c>
+      <c r="G75" s="24" t="inlineStr"/>
+      <c r="H75" s="25" t="inlineStr"/>
       <c r="I75" s="21">
         <f>IF(OR($B75="",$H75=""),"",IF($C75="LONG",($H75-$E75)*$F75,($E75-$H75)*$F75))</f>
         <v/>
@@ -5223,7 +5337,9 @@
         <f>IF(OR($B75="",$I75="",$E75=0,$F75=0),"",$I75/($E75*$F75))</f>
         <v/>
       </c>
-      <c r="K75" s="4" t="n"/>
+      <c r="K75" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L75" s="21">
         <f>IF(OR($B75="",$I75=""),"",$I75-IF($K75="",0,$K75))</f>
         <v/>
@@ -5236,17 +5352,39 @@
         <f>IF($B75="","",IF($H75="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O75" s="23" t="n"/>
+      <c r="O75" s="23" t="inlineStr">
+        <is>
+          <t>15-20</t>
+        </is>
+      </c>
     </row>
     <row r="76">
-      <c r="A76" s="23" t="n"/>
-      <c r="B76" s="23" t="n"/>
-      <c r="C76" s="23" t="n"/>
-      <c r="D76" s="24" t="n"/>
-      <c r="E76" s="25" t="n"/>
-      <c r="F76" s="26" t="n"/>
-      <c r="G76" s="24" t="n"/>
-      <c r="H76" s="25" t="n"/>
+      <c r="A76" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261030623709+341261030104109</t>
+        </is>
+      </c>
+      <c r="B76" s="23" t="inlineStr">
+        <is>
+          <t>MARSONS</t>
+        </is>
+      </c>
+      <c r="C76" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D76" s="24" t="n">
+        <v>46325</v>
+      </c>
+      <c r="E76" s="25" t="n">
+        <v>148.86</v>
+      </c>
+      <c r="F76" s="26" t="n">
+        <v>1612</v>
+      </c>
+      <c r="G76" s="24" t="inlineStr"/>
+      <c r="H76" s="25" t="inlineStr"/>
       <c r="I76" s="21">
         <f>IF(OR($B76="",$H76=""),"",IF($C76="LONG",($H76-$E76)*$F76,($E76-$H76)*$F76))</f>
         <v/>
@@ -5255,7 +5393,9 @@
         <f>IF(OR($B76="",$I76="",$E76=0,$F76=0),"",$I76/($E76*$F76))</f>
         <v/>
       </c>
-      <c r="K76" s="4" t="n"/>
+      <c r="K76" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L76" s="21">
         <f>IF(OR($B76="",$I76=""),"",$I76-IF($K76="",0,$K76))</f>
         <v/>
@@ -5268,7 +5408,11 @@
         <f>IF($B76="","",IF($H76="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O76" s="23" t="n"/>
+      <c r="O76" s="23" t="inlineStr">
+        <is>
+          <t>15-20</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="23" t="n"/>
@@ -31609,7 +31753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J59"/>
+  <dimension ref="A1:J62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -32123,7 +32267,7 @@
     <row r="14">
       <c r="A14" s="27" t="inlineStr">
         <is>
-          <t>DPABHUSHAN</t>
+          <t>DHANUKA</t>
         </is>
       </c>
       <c r="B14" s="20">
@@ -32166,7 +32310,7 @@
     <row r="15">
       <c r="A15" s="27" t="inlineStr">
         <is>
-          <t>EUROPRATIK</t>
+          <t>DPABHUSHAN</t>
         </is>
       </c>
       <c r="B15" s="20">
@@ -32209,7 +32353,7 @@
     <row r="16">
       <c r="A16" s="27" t="inlineStr">
         <is>
-          <t>FISCHER</t>
+          <t>EUROPRATIK</t>
         </is>
       </c>
       <c r="B16" s="20">
@@ -32252,7 +32396,7 @@
     <row r="17">
       <c r="A17" s="27" t="inlineStr">
         <is>
-          <t>GOODLUCK</t>
+          <t>FISCHER</t>
         </is>
       </c>
       <c r="B17" s="20">
@@ -32295,7 +32439,7 @@
     <row r="18">
       <c r="A18" s="27" t="inlineStr">
         <is>
-          <t>GPTINFRA</t>
+          <t>GOODLUCK</t>
         </is>
       </c>
       <c r="B18" s="20">
@@ -32338,7 +32482,7 @@
     <row r="19">
       <c r="A19" s="27" t="inlineStr">
         <is>
-          <t>HATHWAY</t>
+          <t>GPTINFRA</t>
         </is>
       </c>
       <c r="B19" s="20">
@@ -32381,7 +32525,7 @@
     <row r="20">
       <c r="A20" s="27" t="inlineStr">
         <is>
-          <t>HUBTOWN</t>
+          <t>GREAVESCOT</t>
         </is>
       </c>
       <c r="B20" s="20">
@@ -32424,7 +32568,7 @@
     <row r="21">
       <c r="A21" s="27" t="inlineStr">
         <is>
-          <t>INDIAGLYCO</t>
+          <t>HATHWAY</t>
         </is>
       </c>
       <c r="B21" s="20">
@@ -32467,7 +32611,7 @@
     <row r="22">
       <c r="A22" s="27" t="inlineStr">
         <is>
-          <t>INDOKEM</t>
+          <t>HUBTOWN</t>
         </is>
       </c>
       <c r="B22" s="20">
@@ -32510,7 +32654,7 @@
     <row r="23">
       <c r="A23" s="27" t="inlineStr">
         <is>
-          <t>INDOSTAR</t>
+          <t>INDIAGLYCO</t>
         </is>
       </c>
       <c r="B23" s="20">
@@ -32553,7 +32697,7 @@
     <row r="24">
       <c r="A24" s="27" t="inlineStr">
         <is>
-          <t>INOXGREEN</t>
+          <t>INDOKEM</t>
         </is>
       </c>
       <c r="B24" s="20">
@@ -32596,7 +32740,7 @@
     <row r="25">
       <c r="A25" s="27" t="inlineStr">
         <is>
-          <t>JAICORPLTD</t>
+          <t>INDOSTAR</t>
         </is>
       </c>
       <c r="B25" s="20">
@@ -32639,7 +32783,7 @@
     <row r="26">
       <c r="A26" s="27" t="inlineStr">
         <is>
-          <t>JINDALPOLY</t>
+          <t>INOXGREEN</t>
         </is>
       </c>
       <c r="B26" s="20">
@@ -32682,7 +32826,7 @@
     <row r="27">
       <c r="A27" s="27" t="inlineStr">
         <is>
-          <t>JISLJALEQS</t>
+          <t>JAICORPLTD</t>
         </is>
       </c>
       <c r="B27" s="20">
@@ -32725,7 +32869,7 @@
     <row r="28">
       <c r="A28" s="27" t="inlineStr">
         <is>
-          <t>KOTIC</t>
+          <t>JINDALPOLY</t>
         </is>
       </c>
       <c r="B28" s="20">
@@ -32768,7 +32912,7 @@
     <row r="29">
       <c r="A29" s="27" t="inlineStr">
         <is>
-          <t>KRISHNADEF</t>
+          <t>JISLJALEQS</t>
         </is>
       </c>
       <c r="B29" s="20">
@@ -32811,7 +32955,7 @@
     <row r="30">
       <c r="A30" s="27" t="inlineStr">
         <is>
-          <t>KROSS</t>
+          <t>KOTIC</t>
         </is>
       </c>
       <c r="B30" s="20">
@@ -32854,7 +32998,7 @@
     <row r="31">
       <c r="A31" s="27" t="inlineStr">
         <is>
-          <t>MAHLOG</t>
+          <t>KRISHNADEF</t>
         </is>
       </c>
       <c r="B31" s="20">
@@ -32897,7 +33041,7 @@
     <row r="32">
       <c r="A32" s="27" t="inlineStr">
         <is>
-          <t>MBEL</t>
+          <t>KROSS</t>
         </is>
       </c>
       <c r="B32" s="20">
@@ -32940,7 +33084,7 @@
     <row r="33">
       <c r="A33" s="27" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>MAHLOG</t>
         </is>
       </c>
       <c r="B33" s="20">
@@ -32983,7 +33127,7 @@
     <row r="34">
       <c r="A34" s="27" t="inlineStr">
         <is>
-          <t>MOBIKWIK</t>
+          <t>MARSONS</t>
         </is>
       </c>
       <c r="B34" s="20">
@@ -33026,7 +33170,7 @@
     <row r="35">
       <c r="A35" s="27" t="inlineStr">
         <is>
-          <t>NIBE</t>
+          <t>MBEL</t>
         </is>
       </c>
       <c r="B35" s="20">
@@ -33069,7 +33213,7 @@
     <row r="36">
       <c r="A36" s="27" t="inlineStr">
         <is>
-          <t>NILKAMAL</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="B36" s="20">
@@ -33112,7 +33256,7 @@
     <row r="37">
       <c r="A37" s="27" t="inlineStr">
         <is>
-          <t>OAL</t>
+          <t>MOBIKWIK</t>
         </is>
       </c>
       <c r="B37" s="20">
@@ -33155,7 +33299,7 @@
     <row r="38">
       <c r="A38" s="27" t="inlineStr">
         <is>
-          <t>ORIENTELEC</t>
+          <t>NIBE</t>
         </is>
       </c>
       <c r="B38" s="20">
@@ -33198,7 +33342,7 @@
     <row r="39">
       <c r="A39" s="27" t="inlineStr">
         <is>
-          <t>PARACABLES</t>
+          <t>NILKAMAL</t>
         </is>
       </c>
       <c r="B39" s="20">
@@ -33241,7 +33385,7 @@
     <row r="40">
       <c r="A40" s="27" t="inlineStr">
         <is>
-          <t>PIXTRANS</t>
+          <t>OAL</t>
         </is>
       </c>
       <c r="B40" s="20">
@@ -33284,7 +33428,7 @@
     <row r="41">
       <c r="A41" s="27" t="inlineStr">
         <is>
-          <t>PNCINFRA</t>
+          <t>ORIENTELEC</t>
         </is>
       </c>
       <c r="B41" s="20">
@@ -33327,7 +33471,7 @@
     <row r="42">
       <c r="A42" s="27" t="inlineStr">
         <is>
-          <t>PNGSREVA</t>
+          <t>PARACABLES</t>
         </is>
       </c>
       <c r="B42" s="20">
@@ -33370,7 +33514,7 @@
     <row r="43">
       <c r="A43" s="27" t="inlineStr">
         <is>
-          <t>PRINCEPIPE</t>
+          <t>PIXTRANS</t>
         </is>
       </c>
       <c r="B43" s="20">
@@ -33413,7 +33557,7 @@
     <row r="44">
       <c r="A44" s="27" t="inlineStr">
         <is>
-          <t>RSYSTEMS</t>
+          <t>PNCINFRA</t>
         </is>
       </c>
       <c r="B44" s="20">
@@ -33456,7 +33600,7 @@
     <row r="45">
       <c r="A45" s="27" t="inlineStr">
         <is>
-          <t>RUBYMILLS</t>
+          <t>PNGSREVA</t>
         </is>
       </c>
       <c r="B45" s="20">
@@ -33499,7 +33643,7 @@
     <row r="46">
       <c r="A46" s="27" t="inlineStr">
         <is>
-          <t>SAKSOFT</t>
+          <t>PRINCEPIPE</t>
         </is>
       </c>
       <c r="B46" s="20">
@@ -33542,7 +33686,7 @@
     <row r="47">
       <c r="A47" s="27" t="inlineStr">
         <is>
-          <t>SATIN</t>
+          <t>RSYSTEMS</t>
         </is>
       </c>
       <c r="B47" s="20">
@@ -33585,7 +33729,7 @@
     <row r="48">
       <c r="A48" s="27" t="inlineStr">
         <is>
-          <t>SGFIN</t>
+          <t>RUBYMILLS</t>
         </is>
       </c>
       <c r="B48" s="20">
@@ -33628,7 +33772,7 @@
     <row r="49">
       <c r="A49" s="27" t="inlineStr">
         <is>
-          <t>SHRINGARMS</t>
+          <t>SAKSOFT</t>
         </is>
       </c>
       <c r="B49" s="20">
@@ -33671,7 +33815,7 @@
     <row r="50">
       <c r="A50" s="27" t="inlineStr">
         <is>
-          <t>SIMPLEXINF</t>
+          <t>SATIN</t>
         </is>
       </c>
       <c r="B50" s="20">
@@ -33714,7 +33858,7 @@
     <row r="51">
       <c r="A51" s="27" t="inlineStr">
         <is>
-          <t>SMCGLOBAL</t>
+          <t>SGFIN</t>
         </is>
       </c>
       <c r="B51" s="20">
@@ -33757,7 +33901,7 @@
     <row r="52">
       <c r="A52" s="27" t="inlineStr">
         <is>
-          <t>SOLARA</t>
+          <t>SHRINGARMS</t>
         </is>
       </c>
       <c r="B52" s="20">
@@ -33800,7 +33944,7 @@
     <row r="53">
       <c r="A53" s="27" t="inlineStr">
         <is>
-          <t>SPORTKING</t>
+          <t>SIMPLEXINF</t>
         </is>
       </c>
       <c r="B53" s="20">
@@ -33843,7 +33987,7 @@
     <row r="54">
       <c r="A54" s="27" t="inlineStr">
         <is>
-          <t>SUNCLAY</t>
+          <t>SMCGLOBAL</t>
         </is>
       </c>
       <c r="B54" s="20">
@@ -33886,7 +34030,7 @@
     <row r="55">
       <c r="A55" s="27" t="inlineStr">
         <is>
-          <t>SWARAJENG</t>
+          <t>SOLARA</t>
         </is>
       </c>
       <c r="B55" s="20">
@@ -33929,7 +34073,7 @@
     <row r="56">
       <c r="A56" s="27" t="inlineStr">
         <is>
-          <t>TEAMLEASE</t>
+          <t>SPORTKING</t>
         </is>
       </c>
       <c r="B56" s="20">
@@ -33972,7 +34116,7 @@
     <row r="57">
       <c r="A57" s="27" t="inlineStr">
         <is>
-          <t>YUKEN</t>
+          <t>SUNCLAY</t>
         </is>
       </c>
       <c r="B57" s="20">
@@ -34015,7 +34159,7 @@
     <row r="58">
       <c r="A58" s="27" t="inlineStr">
         <is>
-          <t>ZAGGLE</t>
+          <t>SWARAJENG</t>
         </is>
       </c>
       <c r="B58" s="20">
@@ -34056,37 +34200,166 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="3" t="inlineStr">
+      <c r="A59" s="27" t="inlineStr">
+        <is>
+          <t>TEAMLEASE</t>
+        </is>
+      </c>
+      <c r="B59" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A59)</f>
+        <v/>
+      </c>
+      <c r="C59" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A59,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D59" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A59,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E59" s="22">
+        <f>IFERROR($C59/$B59,"")</f>
+        <v/>
+      </c>
+      <c r="F59" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A59,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G59" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A59,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H59" s="21">
+        <f>IFERROR($G59/$B59,"")</f>
+        <v/>
+      </c>
+      <c r="I59" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A59),"")</f>
+        <v/>
+      </c>
+      <c r="J59" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A59),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="27" t="inlineStr">
+        <is>
+          <t>YUKEN</t>
+        </is>
+      </c>
+      <c r="B60" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A60)</f>
+        <v/>
+      </c>
+      <c r="C60" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A60,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D60" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A60,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E60" s="22">
+        <f>IFERROR($C60/$B60,"")</f>
+        <v/>
+      </c>
+      <c r="F60" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A60,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G60" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A60,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H60" s="21">
+        <f>IFERROR($G60/$B60,"")</f>
+        <v/>
+      </c>
+      <c r="I60" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A60),"")</f>
+        <v/>
+      </c>
+      <c r="J60" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A60),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="27" t="inlineStr">
+        <is>
+          <t>ZAGGLE</t>
+        </is>
+      </c>
+      <c r="B61" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A61)</f>
+        <v/>
+      </c>
+      <c r="C61" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A61,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D61" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A61,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E61" s="22">
+        <f>IFERROR($C61/$B61,"")</f>
+        <v/>
+      </c>
+      <c r="F61" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A61,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G61" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A61,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H61" s="21">
+        <f>IFERROR($G61/$B61,"")</f>
+        <v/>
+      </c>
+      <c r="I61" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A61),"")</f>
+        <v/>
+      </c>
+      <c r="J61" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A61),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B59" s="30">
-        <f>SUM(B4:B58)</f>
-        <v/>
-      </c>
-      <c r="C59" s="30">
-        <f>SUM(C4:C58)</f>
-        <v/>
-      </c>
-      <c r="D59" s="30">
-        <f>SUM(D4:D58)</f>
-        <v/>
-      </c>
-      <c r="E59" s="31">
-        <f>IFERROR(C59/B59,"")</f>
-        <v/>
-      </c>
-      <c r="F59" s="32">
-        <f>SUM(F4:F58)</f>
-        <v/>
-      </c>
-      <c r="G59" s="32">
-        <f>SUM(G4:G58)</f>
-        <v/>
-      </c>
-      <c r="H59" s="32">
-        <f>IFERROR(G59/B59,"")</f>
+      <c r="B62" s="30">
+        <f>SUM(B4:B61)</f>
+        <v/>
+      </c>
+      <c r="C62" s="30">
+        <f>SUM(C4:C61)</f>
+        <v/>
+      </c>
+      <c r="D62" s="30">
+        <f>SUM(D4:D61)</f>
+        <v/>
+      </c>
+      <c r="E62" s="31">
+        <f>IFERROR(C62/B62,"")</f>
+        <v/>
+      </c>
+      <c r="F62" s="32">
+        <f>SUM(F4:F61)</f>
+        <v/>
+      </c>
+      <c r="G62" s="32">
+        <f>SUM(G4:G61)</f>
+        <v/>
+      </c>
+      <c r="H62" s="32">
+        <f>IFERROR(G62/B62,"")</f>
         <v/>
       </c>
     </row>
@@ -34105,7 +34378,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N72"/>
+  <dimension ref="A1:N77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -34356,7 +34629,7 @@
         <v>35.4</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>115.97</v>
+        <v>115.96</v>
       </c>
       <c r="N6" s="21">
         <f>SUM(E6:M6)</f>
@@ -34509,7 +34782,7 @@
         <v>35.4</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>115.65</v>
+        <v>115.64</v>
       </c>
       <c r="N9" s="21">
         <f>SUM(E9:M9)</f>
@@ -34713,7 +34986,7 @@
         <v>35.4</v>
       </c>
       <c r="M13" s="4" t="n">
-        <v>73.06999999999999</v>
+        <v>73.13</v>
       </c>
       <c r="N13" s="21">
         <f>SUM(E13:M13)</f>
@@ -35019,7 +35292,7 @@
         <v>35.4</v>
       </c>
       <c r="M19" s="4" t="n">
-        <v>86.66</v>
+        <v>86.73</v>
       </c>
       <c r="N19" s="21">
         <f>SUM(E19:M19)</f>
@@ -35172,7 +35445,7 @@
         <v>35.4</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>83.77</v>
+        <v>83.78</v>
       </c>
       <c r="N22" s="21">
         <f>SUM(E22:M22)</f>
@@ -35325,7 +35598,7 @@
         <v>35.4</v>
       </c>
       <c r="M25" s="4" t="n">
-        <v>37.08</v>
+        <v>36.89</v>
       </c>
       <c r="N25" s="21">
         <f>SUM(E25:M25)</f>
@@ -35529,7 +35802,7 @@
         <v>35.4</v>
       </c>
       <c r="M29" s="4" t="n">
-        <v>42.62</v>
+        <v>42.63</v>
       </c>
       <c r="N29" s="21">
         <f>SUM(E29:M29)</f>
@@ -35784,7 +36057,7 @@
         <v>35.4</v>
       </c>
       <c r="M34" s="4" t="n">
-        <v>37.72</v>
+        <v>37.75</v>
       </c>
       <c r="N34" s="21">
         <f>SUM(E34:M34)</f>
@@ -35937,7 +36210,7 @@
         <v>35.4</v>
       </c>
       <c r="M37" s="4" t="n">
-        <v>31.45</v>
+        <v>31.48</v>
       </c>
       <c r="N37" s="21">
         <f>SUM(E37:M37)</f>
@@ -36141,7 +36414,7 @@
         <v>35.4</v>
       </c>
       <c r="M41" s="4" t="n">
-        <v>234.2</v>
+        <v>234.17</v>
       </c>
       <c r="N41" s="21">
         <f>SUM(E41:M41)</f>
@@ -36192,7 +36465,7 @@
         <v>35.4</v>
       </c>
       <c r="M42" s="4" t="n">
-        <v>27.74</v>
+        <v>27.75</v>
       </c>
       <c r="N42" s="21">
         <f>SUM(E42:M42)</f>
@@ -36243,7 +36516,7 @@
         <v>35.4</v>
       </c>
       <c r="M43" s="4" t="n">
-        <v>80.59</v>
+        <v>80.62</v>
       </c>
       <c r="N43" s="21">
         <f>SUM(E43:M43)</f>
@@ -36345,7 +36618,7 @@
         <v>35.4</v>
       </c>
       <c r="M45" s="4" t="n">
-        <v>85.79000000000001</v>
+        <v>85.81</v>
       </c>
       <c r="N45" s="21">
         <f>SUM(E45:M45)</f>
@@ -36447,7 +36720,7 @@
         <v>35.4</v>
       </c>
       <c r="M47" s="4" t="n">
-        <v>178.93</v>
+        <v>178.9</v>
       </c>
       <c r="N47" s="21">
         <f>SUM(E47:M47)</f>
@@ -36498,7 +36771,7 @@
         <v>35.4</v>
       </c>
       <c r="M48" s="4" t="n">
-        <v>179.89</v>
+        <v>179.86</v>
       </c>
       <c r="N48" s="21">
         <f>SUM(E48:M48)</f>
@@ -36600,7 +36873,7 @@
         <v>35.4</v>
       </c>
       <c r="M50" s="4" t="n">
-        <v>180.24</v>
+        <v>180.22</v>
       </c>
       <c r="N50" s="21">
         <f>SUM(E50:M50)</f>
@@ -36651,7 +36924,7 @@
         <v>35.4</v>
       </c>
       <c r="M51" s="4" t="n">
-        <v>142.78</v>
+        <v>142.83</v>
       </c>
       <c r="N51" s="21">
         <f>SUM(E51:M51)</f>
@@ -36702,7 +36975,7 @@
         <v>35.4</v>
       </c>
       <c r="M52" s="4" t="n">
-        <v>112.04</v>
+        <v>112.03</v>
       </c>
       <c r="N52" s="21">
         <f>SUM(E52:M52)</f>
@@ -36906,7 +37179,7 @@
         <v>35.4</v>
       </c>
       <c r="M56" s="4" t="n">
-        <v>46.19</v>
+        <v>46.23</v>
       </c>
       <c r="N56" s="21">
         <f>SUM(E56:M56)</f>
@@ -37008,7 +37281,7 @@
         <v>35.4</v>
       </c>
       <c r="M58" s="4" t="n">
-        <v>36.42</v>
+        <v>36.29</v>
       </c>
       <c r="N58" s="21">
         <f>SUM(E58:M58)</f>
@@ -37059,7 +37332,7 @@
         <v>35.4</v>
       </c>
       <c r="M59" s="4" t="n">
-        <v>37.92</v>
+        <v>37.93</v>
       </c>
       <c r="N59" s="21">
         <f>SUM(E59:M59)</f>
@@ -37161,7 +37434,7 @@
         <v>35.4</v>
       </c>
       <c r="M61" s="4" t="n">
-        <v>39.25</v>
+        <v>39.27</v>
       </c>
       <c r="N61" s="21">
         <f>SUM(E61:M61)</f>
@@ -37212,7 +37485,7 @@
         <v>35.4</v>
       </c>
       <c r="M62" s="4" t="n">
-        <v>33.95</v>
+        <v>33.96</v>
       </c>
       <c r="N62" s="21">
         <f>SUM(E62:M62)</f>
@@ -37263,7 +37536,7 @@
         <v>35.4</v>
       </c>
       <c r="M63" s="4" t="n">
-        <v>34.56</v>
+        <v>34.59</v>
       </c>
       <c r="N63" s="21">
         <f>SUM(E63:M63)</f>
@@ -37290,22 +37563,22 @@
         <v>46324</v>
       </c>
       <c r="E64" s="4" t="n">
-        <v>90</v>
+        <v>110</v>
       </c>
       <c r="F64" s="4" t="n">
-        <v>300.01</v>
+        <v>600.39</v>
       </c>
       <c r="G64" s="4" t="n">
-        <v>9.210000000000001</v>
+        <v>18.43</v>
       </c>
       <c r="H64" s="4" t="n">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="I64" s="4" t="n">
         <v>45</v>
       </c>
       <c r="J64" s="4" t="n">
-        <v>17.91</v>
+        <v>23.23</v>
       </c>
       <c r="K64" s="4" t="n">
         <v>14.75</v>
@@ -37314,7 +37587,7 @@
         <v>35.4</v>
       </c>
       <c r="M64" s="4" t="n">
-        <v>70.06</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="N64" s="21">
         <f>SUM(E64:M64)</f>
@@ -37341,22 +37614,22 @@
         <v>46324</v>
       </c>
       <c r="E65" s="4" t="n">
-        <v>90.23</v>
+        <v>110.23</v>
       </c>
       <c r="F65" s="4" t="n">
-        <v>300.72</v>
+        <v>606.7</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>9.23</v>
+        <v>18.63</v>
       </c>
       <c r="H65" s="4" t="n">
-        <v>0.3</v>
+        <v>0.61</v>
       </c>
       <c r="I65" s="4" t="n">
         <v>45</v>
       </c>
       <c r="J65" s="4" t="n">
-        <v>17.96</v>
+        <v>23.3</v>
       </c>
       <c r="K65" s="4" t="n">
         <v>14.75</v>
@@ -37388,24 +37661,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D66" s="24" t="inlineStr"/>
+      <c r="D66" s="24" t="n">
+        <v>46325</v>
+      </c>
       <c r="E66" s="4" t="n">
-        <v>0</v>
+        <v>71.95</v>
       </c>
       <c r="F66" s="4" t="n">
-        <v>0</v>
+        <v>239.79</v>
       </c>
       <c r="G66" s="4" t="n">
-        <v>0</v>
+        <v>7.36</v>
       </c>
       <c r="H66" s="4" t="n">
-        <v>0</v>
+        <v>0.24</v>
       </c>
       <c r="I66" s="4" t="n">
-        <v>0</v>
+        <v>35.97</v>
       </c>
       <c r="J66" s="4" t="n">
-        <v>0</v>
+        <v>14.32</v>
       </c>
       <c r="K66" s="4" t="n">
         <v>14.75</v>
@@ -37414,7 +37689,7 @@
         <v>35.4</v>
       </c>
       <c r="M66" s="4" t="n">
-        <v>0</v>
+        <v>49.21</v>
       </c>
       <c r="N66" s="21">
         <f>SUM(E66:M66)</f>
@@ -37424,12 +37699,12 @@
     <row r="67">
       <c r="A67" s="23" t="inlineStr">
         <is>
-          <t>DHAN-23126102780509+34126102781309+23126102781009+23126102781209+221261027605909+34126102781909+321261027588609+23126102781809+321261027589309+23126102782209+321261027590909+23126102782809+34126102783609</t>
+          <t>DHAN-321261029713009+221261029729209+231261029107809+231261029108409+231261029108509+221261029730909+231261029109609+231261029109809+221261029731809+341261029102409+221261029733009+341261029103009</t>
         </is>
       </c>
       <c r="B67" s="23" t="inlineStr">
         <is>
-          <t>BAJEL</t>
+          <t>CNL</t>
         </is>
       </c>
       <c r="C67" s="23" t="inlineStr">
@@ -37437,24 +37712,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D67" s="24" t="inlineStr"/>
+      <c r="D67" s="24" t="n">
+        <v>46325</v>
+      </c>
       <c r="E67" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F67" s="4" t="n">
-        <v>90.59</v>
+        <v>119.03</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>2.78</v>
+        <v>3.65</v>
       </c>
       <c r="H67" s="4" t="n">
-        <v>0.09</v>
+        <v>0.12</v>
       </c>
       <c r="I67" s="4" t="n">
-        <v>13.59</v>
+        <v>17.85</v>
       </c>
       <c r="J67" s="4" t="n">
-        <v>0.52</v>
+        <v>0.68</v>
       </c>
       <c r="K67" s="4" t="n">
         <v>14.75</v>
@@ -37473,12 +37750,12 @@
     <row r="68">
       <c r="A68" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321261029713009+221261029729209+231261029107809+231261029108409+231261029108509+221261029730909+231261029109609+231261029109809+221261029731809+341261029102409+221261029733009+341261029103009</t>
+          <t>DHAN-341261029101409+221261029729309+221261029729809+231261029108209+221261029730609+221261029731009+231261029109509+341261029102109+221261029731909+321261029716409+341261029102909+341261029103109</t>
         </is>
       </c>
       <c r="B68" s="23" t="inlineStr">
         <is>
-          <t>CNL</t>
+          <t>HUBTOWN</t>
         </is>
       </c>
       <c r="C68" s="23" t="inlineStr">
@@ -37486,33 +37763,35 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D68" s="24" t="inlineStr"/>
+      <c r="D68" s="24" t="n">
+        <v>46325</v>
+      </c>
       <c r="E68" s="4" t="n">
-        <v>0</v>
+        <v>72.33</v>
       </c>
       <c r="F68" s="4" t="n">
-        <v>0</v>
+        <v>241.11</v>
       </c>
       <c r="G68" s="4" t="n">
-        <v>0</v>
+        <v>7.4</v>
       </c>
       <c r="H68" s="4" t="n">
-        <v>0</v>
+        <v>0.24</v>
       </c>
       <c r="I68" s="4" t="n">
-        <v>0</v>
+        <v>36.41</v>
       </c>
       <c r="J68" s="4" t="n">
-        <v>0</v>
+        <v>14.4</v>
       </c>
       <c r="K68" s="4" t="n">
         <v>14.75</v>
       </c>
       <c r="L68" s="4" t="n">
-        <v>0</v>
+        <v>35.4</v>
       </c>
       <c r="M68" s="4" t="n">
-        <v>0</v>
+        <v>49.48</v>
       </c>
       <c r="N68" s="21">
         <f>SUM(E68:M68)</f>
@@ -37522,7 +37801,7 @@
     <row r="69">
       <c r="A69" s="23" t="inlineStr">
         <is>
-          <t>DHAN-341261029101409+221261029729309+221261029729809+231261029108209+221261029730609+221261029731009+231261029109509+341261029102109+221261029731909+321261029716409+341261029102909+341261029103109</t>
+          <t>DHAN-23126103014009</t>
         </is>
       </c>
       <c r="B69" s="23" t="inlineStr">
@@ -37532,10 +37811,12 @@
       </c>
       <c r="C69" s="23" t="inlineStr">
         <is>
-          <t>LONG</t>
-        </is>
-      </c>
-      <c r="D69" s="24" t="inlineStr"/>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D69" s="24" t="n">
+        <v>46325</v>
+      </c>
       <c r="E69" s="4" t="n">
         <v>0</v>
       </c>
@@ -37555,10 +37836,10 @@
         <v>0</v>
       </c>
       <c r="K69" s="4" t="n">
-        <v>14.75</v>
+        <v>0</v>
       </c>
       <c r="L69" s="4" t="n">
-        <v>35.4</v>
+        <v>0</v>
       </c>
       <c r="M69" s="4" t="n">
         <v>0</v>
@@ -37584,24 +37865,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D70" s="24" t="inlineStr"/>
+      <c r="D70" s="24" t="n">
+        <v>46325</v>
+      </c>
       <c r="E70" s="4" t="n">
-        <v>0</v>
+        <v>71.58</v>
       </c>
       <c r="F70" s="4" t="n">
-        <v>0</v>
+        <v>238.66</v>
       </c>
       <c r="G70" s="4" t="n">
-        <v>0</v>
+        <v>7.33</v>
       </c>
       <c r="H70" s="4" t="n">
-        <v>0</v>
+        <v>0.24</v>
       </c>
       <c r="I70" s="4" t="n">
-        <v>0</v>
+        <v>35.8</v>
       </c>
       <c r="J70" s="4" t="n">
-        <v>0</v>
+        <v>14.25</v>
       </c>
       <c r="K70" s="4" t="n">
         <v>14.75</v>
@@ -37610,7 +37893,7 @@
         <v>35.4</v>
       </c>
       <c r="M70" s="4" t="n">
-        <v>0</v>
+        <v>40.81</v>
       </c>
       <c r="N70" s="21">
         <f>SUM(E70:M70)</f>
@@ -37633,24 +37916,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D71" s="24" t="inlineStr"/>
+      <c r="D71" s="24" t="n">
+        <v>46325</v>
+      </c>
       <c r="E71" s="4" t="n">
-        <v>0</v>
+        <v>71.91</v>
       </c>
       <c r="F71" s="4" t="n">
-        <v>0</v>
+        <v>239.82</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>0</v>
+        <v>7.36</v>
       </c>
       <c r="H71" s="4" t="n">
-        <v>0</v>
+        <v>0.24</v>
       </c>
       <c r="I71" s="4" t="n">
-        <v>0</v>
+        <v>35.97</v>
       </c>
       <c r="J71" s="4" t="n">
-        <v>0</v>
+        <v>14.31</v>
       </c>
       <c r="K71" s="4" t="n">
         <v>14.75</v>
@@ -37659,7 +37944,7 @@
         <v>35.4</v>
       </c>
       <c r="M71" s="4" t="n">
-        <v>0</v>
+        <v>49.21</v>
       </c>
       <c r="N71" s="21">
         <f>SUM(E71:M71)</f>
@@ -37667,54 +37952,299 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="3" t="inlineStr">
+      <c r="A72" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126102780509+34126102781309+23126102781009+23126102781209+221261027605909+34126102781909+321261027588609+23126102781809+321261027589309+23126102782209+321261027590909+23126102782809+34126102783609</t>
+        </is>
+      </c>
+      <c r="B72" s="23" t="inlineStr">
+        <is>
+          <t>BAJEL</t>
+        </is>
+      </c>
+      <c r="C72" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D72" s="24" t="inlineStr"/>
+      <c r="E72" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F72" s="4" t="n">
+        <v>90.59</v>
+      </c>
+      <c r="G72" s="4" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="H72" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="I72" s="4" t="n">
+        <v>13.59</v>
+      </c>
+      <c r="J72" s="4" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="K72" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L72" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M72" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N72" s="21">
+        <f>SUM(E72:M72)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261030639109+231261030110409+321261030624409+221261030640409+341261030103309+341261030103509+321261030625509+221261030641609+231261030111009+221261030642209+341261030103909+341261030104009</t>
+        </is>
+      </c>
+      <c r="B73" s="23" t="inlineStr">
+        <is>
+          <t>DHANUKA</t>
+        </is>
+      </c>
+      <c r="C73" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D73" s="24" t="inlineStr"/>
+      <c r="E73" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F73" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G73" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H73" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I73" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J73" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K73" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L73" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M73" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N73" s="21">
+        <f>SUM(E73:M73)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-231261030110209+221261030639609+231261030110509+221261030640509+231261030110709+231261030110809+231261030110909+221261030641709+341261030103709+321261030626409+221261030643009</t>
+        </is>
+      </c>
+      <c r="B74" s="23" t="inlineStr">
+        <is>
+          <t>GREAVESCOT</t>
+        </is>
+      </c>
+      <c r="C74" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D74" s="24" t="inlineStr"/>
+      <c r="E74" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F74" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G74" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H74" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I74" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J74" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K74" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L74" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M74" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N74" s="21">
+        <f>SUM(E74:M74)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221261030639209+341261030103109+221261030639909+231261030110609+341261030103409+321261030625109+341261030103609+231261030111109+231261030111209+221261030643109+221261030643409+221261030643809+321261030628009+221261030644509</t>
+        </is>
+      </c>
+      <c r="B75" s="23" t="inlineStr">
+        <is>
+          <t>JISLJALEQS</t>
+        </is>
+      </c>
+      <c r="C75" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D75" s="24" t="inlineStr"/>
+      <c r="E75" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F75" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G75" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H75" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I75" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J75" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K75" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L75" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M75" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N75" s="21">
+        <f>SUM(E75:M75)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321261030623709+341261030104109</t>
+        </is>
+      </c>
+      <c r="B76" s="23" t="inlineStr">
+        <is>
+          <t>MARSONS</t>
+        </is>
+      </c>
+      <c r="C76" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D76" s="24" t="inlineStr"/>
+      <c r="E76" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F76" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G76" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H76" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I76" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J76" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K76" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L76" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M76" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N76" s="21">
+        <f>SUM(E76:M76)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E72" s="32">
-        <f>SUM(E4:E71)</f>
-        <v/>
-      </c>
-      <c r="F72" s="32">
-        <f>SUM(F4:F71)</f>
-        <v/>
-      </c>
-      <c r="G72" s="32">
-        <f>SUM(G4:G71)</f>
-        <v/>
-      </c>
-      <c r="H72" s="32">
-        <f>SUM(H4:H71)</f>
-        <v/>
-      </c>
-      <c r="I72" s="32">
-        <f>SUM(I4:I71)</f>
-        <v/>
-      </c>
-      <c r="J72" s="32">
-        <f>SUM(J4:J71)</f>
-        <v/>
-      </c>
-      <c r="K72" s="32">
-        <f>SUM(K4:K71)</f>
-        <v/>
-      </c>
-      <c r="L72" s="32">
-        <f>SUM(L4:L71)</f>
-        <v/>
-      </c>
-      <c r="M72" s="32">
-        <f>SUM(M4:M71)</f>
-        <v/>
-      </c>
-      <c r="N72" s="32">
-        <f>SUM(N4:N71)</f>
+      <c r="E77" s="32">
+        <f>SUM(E4:E76)</f>
+        <v/>
+      </c>
+      <c r="F77" s="32">
+        <f>SUM(F4:F76)</f>
+        <v/>
+      </c>
+      <c r="G77" s="32">
+        <f>SUM(G4:G76)</f>
+        <v/>
+      </c>
+      <c r="H77" s="32">
+        <f>SUM(H4:H76)</f>
+        <v/>
+      </c>
+      <c r="I77" s="32">
+        <f>SUM(I4:I76)</f>
+        <v/>
+      </c>
+      <c r="J77" s="32">
+        <f>SUM(J4:J76)</f>
+        <v/>
+      </c>
+      <c r="K77" s="32">
+        <f>SUM(K4:K76)</f>
+        <v/>
+      </c>
+      <c r="L77" s="32">
+        <f>SUM(L4:L76)</f>
+        <v/>
+      </c>
+      <c r="M77" s="32">
+        <f>SUM(M4:M76)</f>
+        <v/>
+      </c>
+      <c r="N77" s="32">
+        <f>SUM(N4:N76)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:N71"/>
+  <autoFilter ref="A3:N76"/>
   <mergeCells count="2">
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>

</xml_diff>